<commit_message>
chore: update jobs data [2026-06-17 07:55 UTC]
</commit_message>
<xml_diff>
--- a/mimu_jobs.xlsx
+++ b/mimu_jobs.xlsx
@@ -624,11 +624,14 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Ward (1),
-Bahan Township, Yangon, Myanmar</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr"/>
+          <t>Ward (1),, Bahan Township, Yangon, Myanmar</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>As a global leader, CARE is shaping the future of the humanitarian and development sector. Each year, we deliver support and services to millions of people in over a hundred countries. We do this by focusing on our mission and living the values that drive our organization. A career at CARE is an opportunity to be part of a movement that brings communities together to solve complex problems and foster lasting change throughout the world. We seek individuals who are passionate about humanitarian and development work, collaborate well with others, embrace learning and innovation, and deliver results. What it’s like to work at CARE? CARE is a mission-driven international humanitarian aid and development organization that offers an opportunity to work with people across the world. Not a day will go by that you won’t learn something profound, meet an expert, or write a sentence that can change a life. We are committed to an environment where everyone can succeed. CARE in Myanmar is looking f</t>
+        </is>
+      </c>
       <c r="T2" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -711,8 +714,16 @@
         </is>
       </c>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>No. 69 (A), Kanbawza Street</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>SOLIDARITES INTERNATIONAL (SI) is an international humanitarian NGO which, for more than 40 years, has been providing assistance to populations affected by armed conflicts and natural disasters by meeting their vital needs for food, water and shelter. Particularly involved in the fight against diseases linked to unsafe water, the first cause of death in the world, SI's interventions provide expertise in the field of access to drinking water, sanitation and hygiene promotion, but also in the essential area of food security and livelihoods. Present in around twenty countries, SI's teams - 2000 people in total made up of expatriates, national staff, permanent staff at headquarters, and a few volunteers - work with professionalism and commitment while respecting cultures. Solidarités International (SI) is determined to prevent and fight all type of abuse – all act of exploitation, abuse and/or sexual harassment (SEAH) against members of beneficiary communities or collaborators, fraud, corr</t>
+        </is>
+      </c>
       <c r="T3" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -796,7 +807,11 @@
       </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Capacity building / Awareness raising on response activities • Contribute to the design and planning of relevant training and awareness raising sessions for IDPs, Protection Focal Points and delivering at field level. • Conduct in delivery of awareness sessions to conflict affected people as required. Data / information management • Ensure accurate data records and appropriate management of project documentation or otherwise manage and maintain the case management database, including confidential handling of individual case files and databases. • Track the processes of internal or external referral or transfer, including maintaining contact with the focal point at respective agencies and coordinating the flow of information from cases to service providers. Coordination / referral / service mapping • Coordinate with other protection colleagues and protection focal point on case identifying, implementing and referral • Maintain the good relationship between the community / the beneficiar</t>
+        </is>
+      </c>
       <c r="T4" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -880,7 +895,11 @@
       </c>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>ADRA Myanmar is an ‘implementing office’ within the ADRA network and a recognized NGO in Myanmar. Established in 1984, ADRA Myanmar is one of the oldest country offices in ADRA providing development and relief assistance opportunities throughout the country. ADRA Myanmar operates under multi sectors that cater to Education, Food Security &amp; Livelihoods, Health, Nutrition, WASH and Humanitarian actions. Position Summary: ADRA Myanmar implements a diverse range of infrastructure interventions as part of its humanitarian and development programming. These interventions include water supply systems, sanitation facilities, shelters, community infrastructure, and productive assets that contribute to livelihoods, resilience, disaster preparedness, and sustainable development. The Civil Engineering Specialist (WASH &amp; Infrastructure) is responsible for providing technical leadership in the design, implementation, supervision, monitoring, and quality assurance of infrastructure projects and suppo</t>
+        </is>
+      </c>
       <c r="T5" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -960,7 +979,11 @@
       </c>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Myanmar is facing a complex humanitarian crisis driven by conflict, displacement, and recent natural disasters, resulting in widespread psychological distress and limited access to mental health and psychosocial support (MHPSS), particularly in rural and conflict-affected areas. Frontline responders and local humanitarian staff are especially affected, experiencing high levels of stress, burnout, and trauma. Despite growing recognition of these needs, there remains a lack of structured, scalable approaches to staff wellbeing and duty of care across organisations. In response, Christian Aid and Tearfund are implementing a Collective Initiative to scale the Community Resilience Model (CRM), an evidence- based, peer-to-peer approach to strengthening resilience among staff and communities. As the project expands to community-level delivery, a Training Coordinator is required to support the effective coordination, delivery, and documentation of CRM trainings across participating organisatio</t>
+        </is>
+      </c>
       <c r="T6" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -1039,13 +1062,12 @@
         </is>
       </c>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>2026
-Parent Sector: UNESCO Project Antenna Office in Yangon</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Under the Global Partnership for Education (GPE) System Capacity Grant (SCG) for Myanmar, the United Nations Educational, Scientific and Cultural Organization (UNESCO) Myanmar Project Antenna Office is implementing a multi-year programme to strengthen the resilience and effectiveness of Myanmar’s education sector through improved planning, coordination, financing, monitoring, and evidence generation. The SCG contributes to strengthening evidence-based decision-making, sector coordination, and strategic planning in Myanmar’s education sector. In a complex and evolving operating context, timely and reliable data analysis is essential to support education programming, coordination, policy dialogue, resource mobilization, and monitoring of sector progress. UNESCO requires technical support to process, analyze, and present quantitative and secondary data relevant to education sector planning, coordination, monitoring, and evidence generation. This includes support to review and organize lar</t>
+        </is>
+      </c>
       <c r="T7" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -1126,10 +1148,14 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Ward 6, Yankin Township, Yangon, Myanmar</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr"/>
+          <t>No.10 (B-1), Thukhawaddy Street</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>products and information more available, accessible, and affordable to people in 90 developing countries worldwide. Through innovative social marketing DKT aims to give Myanmar's people greater knowledge and a wider range of choices for reproductive health. DKT International Myanmar invites applications for the following position in Yangon, Myanmar. Position: Demand Generator Report To: Clinical Service Coordinator Duty Station: Magway (Part Time) Closing Date: as soon as possible About the Job: We are seeking a reliable and detail-oriented Demand Generator who conducts outreach to identify women in need of family planning services, provides key information using job aids, distributes promotional pamphlets to vulnerable women, and refers them to designated private clinics. The ideal candidate is self-motivated, approachable, and adaptable, with the ability to work effectively in various field conditions while ensuring the integrity and confidentiality of collected data. Responsibilitie</t>
+        </is>
+      </c>
       <c r="T8" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -1210,10 +1236,14 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Ward 6, Yankin Township, Yangon, Myanmar</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr"/>
+          <t>No.10 (B-1), Thukhawaddy Street</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>products and information more available, accessible, and affordable to people in 90 developing countries worldwide. Through innovative social marketing DKT aims to give Myanmar's people greater knowledge and a wider range of choices for reproductive health. DKT International Myanmar invites applications for the following position in Yangon, Myanmar. Position: Demand Generator Report To: Clinical Service Coordinator Duty Station: Mon State (Part Time) Closing Date: as soon as possible About the Job: We are seeking a reliable and detail-oriented Demand Generator who conducts outreach to identify women in need of family planning services, provides key information using job aids, distributes promotional pamphlets to vulnerable women, and refers them to designated private clinics. The ideal candidate is self-motivated, approachable, and adaptable, with the ability to work effectively in various field conditions while ensuring the integrity and confidentiality of collected data. Responsibili</t>
+        </is>
+      </c>
       <c r="T9" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -1294,10 +1324,14 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Ward 6, Yankin Township, Yangon, Myanmar</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr"/>
+          <t>No.10 (B-1), Thukhawaddy Street</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>products and information more available, accessible, and affordable to people in 90 developing countries worldwide. Through innovative social marketing DKT aims to give Myanmar's people greater knowledge and a wider range of choices for reproductive health. DKT International Myanmar invites applications for the following position in Yangon, Myanmar. Position: Demand Generator Report To: Clinical Service Coordinator Duty Station: Mandalay (Part Time) Closing Date: as soon as possible About the Job: We are seeking a reliable and detail-oriented Demand Generator who conducts outreach to identify women in need of family planning services, provides key information using job aids, distributes promotional pamphlets to vulnerable women, and refers them to designated private clinics. The ideal candidate is self-motivated, approachable, and adaptable, with the ability to work effectively in various field conditions while ensuring the integrity and confidentiality of collected data. Responsibilit</t>
+        </is>
+      </c>
       <c r="T10" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -1377,7 +1411,11 @@
           <t>No. (47), Shwe Taung Kyar Street</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>World Vision is a Christian, relief, development and advocacy organization working for/ with communities</t>
+        </is>
+      </c>
       <c r="T11" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -1465,7 +1503,11 @@
           <t>No. (14), Hnin Si Street</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Please refer to our website: https://myinttasaytaman.org/ Job Summary MTSTM Organization is seeking a highly organized, detail-oriented, and proactive Admin and Finance Assistant to support the implementation of the TB/HIV Prevention Project. The position will play a key role in ensuring efficient financial management, administrative coordination, HR-related support, documentation, and operational support for the project. The Admin and Finance Assistant will work closely with the Admin and Finance Officer, coordinate with project staff and field teams, and contribute to accurate financial reporting, compliance, and smooth day-to-day office operations. Key Responsibilities Financial Recordkeeping &amp; Reporting: Assist the Admin and Finance Officer in maintaining accurate records of project expenditure. Systematically review and prepare detailed weekly, monthly, quarterly, and annual budget reports, ensuring accuracy, transparency, and timely submission. Support budget monitoring and repor</t>
+        </is>
+      </c>
       <c r="T12" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -1549,7 +1591,11 @@
       </c>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>training to CBPG on protection risk analysis, developing and implementation of Community Action Plan (CAP) in accordance with CBP approaches and CBP SoP. • Support capacity development through training and coaching CBPG members in supporting the community in the identification and understanding of protection risks and problems and prioritizing key protection risks in addressing through CAP as per SoP and guidance. • Support protection assistants to be friendly with CBP tools and carry out the activities per CBP SoP and data protection guidelines. • Submit internal bi-weekly protection reports/trackers in English to Protection Team Leader; these reports should summarize activities carried out by the Protection teams and underline key weekly findings. • Regularly liaise with the DRC IM and MEAL Office based staff, ensure the accurate management of data records and trackers. • Support DRC Protection team and CSO partners in adapting a systematic application of participatory, community, ri</t>
+        </is>
+      </c>
       <c r="T13" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -1629,7 +1675,11 @@
       </c>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Mercy Corps is a leading global development agency and social enterprise improving lives all around the world. With a network of experienced professionals, we partner with local communities to put bold ideas into action to help people recover, overcome hardship, and build better lives – now, and for the future. Mercy Corps in Myanmar focuses on agriculture and livelihoods, income generation, market development and energy access. In Myanmar, Mercy Corps leads a dynamic and impactful portfolio of development programs that strengthen community resilience, foster inclusive growth, and advance economic wellbeing nationwide. Grounded in a systems- based approach, our work prioritizes livelihoods, climate resilience, environmental sustainability, and inclusive market systems development. The country team collaborates across sectors to expand economic opportunities, promote equitable natural resource management, and support community-driven governance. Our programs are intentionally designed t</t>
+        </is>
+      </c>
       <c r="T14" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -1709,7 +1759,11 @@
           <t>No. 27, Thuta 1st Street</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>KKEC is currently seeking a motivated, dedicated and qualified candidate to fill the following position. Title of the position: HR &amp; Admin Coordinator Department: HR &amp; Admin Department Job location: Yangon, Myanmar Reports to: Assistant Director of Finance and Administration</t>
+        </is>
+      </c>
       <c r="T15" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -1780,11 +1834,7 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>1 for Kalemyo and another 1 for Mandalay</t>
-        </is>
-      </c>
+      <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
@@ -1869,7 +1919,11 @@
       </c>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Applications will be reviewed on a rolling basis, and interviews will be conducted accordingly. Vacancy Announcement / WASH Expert SG 07</t>
+        </is>
+      </c>
       <c r="T17" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -1953,7 +2007,11 @@
       </c>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>ADRA Myanmar is an ‘implementing office’ within the ADRA network and a recognized NGO in Myanmar. Established in 1984, ADRA Myanmar is one of the oldest country offices in ADRA providing development and relief assistance opportunities throughout the country. ADRA Myanmar operates under multi sectors that cater to Education, Food Security &amp; Livelihoods, Health, Nutrition, WASH and Humanitarian actions. Job Summary: The Health and Nutrition Specialist will provide technical leadership and support ADRA Myanmar’s Health &amp; Nutrition Programming, Research, M&amp;E strategies and program development. This will include research &amp; analysis; producing reports and visual representations; provision of technical advice; presenting and sharing learnings, conducting Program Management and Business Development. The Health and Nutrition Specialist will support institutional development of ADRA Myanmar in health sector that includes participation in the Health &amp; Nutrition Clusters and Coordination activitit</t>
+        </is>
+      </c>
       <c r="T18" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -2078,7 +2136,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Volunteer</t>
+          <t>Full-time</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -2141,7 +2199,11 @@
           <t>No.42, Strand Road</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr"/>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Plan, MRCS Health Strategy and policy. The goal of the program is to reduce mortality and morbidity related to priority communicable diseases and the impact of public health in emergencies and WASH in emergency by improving the capacity of communities and Red Cross branches. MRCS continues to engage several community-based programmes with the support from Red Cross movement partners and the interventions undertaken are aimed at improving the resilience of vulnerable communities towards occurring risks (health risks and future disasters). Project/Program Background: The Earthquake Operation under the Myanmar Red Cross Society (MRCS) is a dedicated emergency response initiative designed to address the urgent humanitarian needs resulting from the recent earthquake that has impacted multiple regions across Myanmar. Coordinated with support from both domestic and international partners, the operation aims to provide timely and effective assistance in key sectors such as shelter, health, wat</t>
+        </is>
+      </c>
       <c r="T20" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -2213,7 +2275,11 @@
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>(သို့ ိုြဟတို ်) mrcshrrecruitment@redcross.org.mm သို့ ို လ ြ် ြူ ာ ခ ်း ိုို့ရြည်။ အခသ်းစ တအ် ြေျြအ် လြ်ြျာ်းအာ်း www. redcross.org.mm တွင ် ၀ငခ် ရာြက်ြည် ရှုနင ို ် ါ သည်။ လူခတွွဲ့စစခ် ြ်းမြေင်း် ခ ်းွ ြေျယ်ြေံ သူြ ိုသာ အခကြာင်း် ကြာ်းြည်မဖစပ် သည်။ "Person with disability are encouraged to apply this post as they will be given equal opportunity" "Our recruitment and selection procedures reflect our commitment to the safety and protection of children, and prevention of violence among</t>
+        </is>
+      </c>
       <c r="T21" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -2393,12 +2459,12 @@
         </is>
       </c>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>16, Kantkawmyaing 1st Street</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>be based on the results and satisfactory references. • MPG has the right to cancel or defer the recruitment process at any stage, including after completion of the employment contractual agreement, if it is impacted by donor funding constraints or decisions that are beyond its control. • By applying, the job applicant acknowledges that they understand these recruitment procedures. Interested candidates are requested to enter the below link or scan the QR code by filling necessary information for the application submission as soon as possible. Please ensure that all required details are completed in the form. Incomplete submissions will not be considered. MPG VACANCY ANNOUNCEMENT 3 Click Here for Job Application Submission for this position! Myanmar Positive Group, Head Office No 3/16, Kantkawmyaing 1st Street, 8 Ward, Yankin Township, Yangon Region, Myanmar. For detailed information, please contact recruitment@myanmarpositivegroup.org OR (HP + 95 9 987 608 567, + 95 9 797 212 020) with</t>
+        </is>
+      </c>
       <c r="T23" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -2478,7 +2544,11 @@
       </c>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>operational in 30 developing countries around the world. Our vision is a just world in which all men and</t>
+        </is>
+      </c>
       <c r="T24" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -2567,10 +2637,14 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>18 regions across Myanmar in 2012 and has</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr"/>
+          <t>No. 7, Room No.202, Moe Kaung Condo, Moe Kaung Road</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Myanmar Youth Stars (MYS) is an organization, formed by a group of Young people form key population that function as a network to respond to HIV in Myanmar and established in early 2013 in order to response to the inequality, stigma and discrimination towards young people who are marginalized and higher risk of getting HIV infection. Myanmar Youth Stars Network is currently working with 18 regions across Myanmar in 2012 and has started developing the capacity of individuals in network. The network targeted members young</t>
+        </is>
+      </c>
       <c r="T25" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -2645,12 +2719,12 @@
         </is>
       </c>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>94 townships of Myanmar in the areas of disease control</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Myanmar Health Assistant Association (MHAA), TB Hospital Road, Aung San, Insein Township, Yangon, Myanmar. Specific Duties and Responsibilities ❖ Ensure to get good quality X Rays in accordance with national quality standards. ❖ Take main responsibility for maintenance of X Ray machines and accessories and also assist to Medical Doctor (X Ray).</t>
+        </is>
+      </c>
       <c r="T26" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -2721,12 +2795,12 @@
         </is>
       </c>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>94 townships of Myanmar in the areas of disease control</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>MHAA. 1 Myanmar Health Assistant Association (MHAA), TB Hospital Road, Aung San, Insein Township, Yangon, Myanmar. Position Summary Under the direct supervision of the Project Coordinator, the Project Supporting Staff will provide day-to-day support to project implementation. The role includes administrative, financial, logistics, coordination, and basic health support activities, particularly related to TB projects. The staff will assist the Project Coordinator, Finance Assistant, and project team to ensure smooth project operations in accordance with MHAA policies and project guidelines. Key Responsibilities Project &amp; Patient Support ❖ Receive and greet visitors and ensure proper reception services. ❖ Support the distribution of transportation allowance (TA), project support packages to TB patients, and incentives to volunteers in accordance with project guidelines. ❖ Maintain accurate and up-to-date distribution records and submit reports to supervisors. ❖ Support the Project Coordi</t>
+        </is>
+      </c>
       <c r="T27" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -2797,12 +2871,12 @@
         </is>
       </c>
       <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>94 townships of Myanmar in the areas of disease control</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>MHAA. 1 Myanmar Health Assistant Association (MHAA), TB Hospital Road, Aung San, Insein Township, Yangon, Myanmar. Position Summary Under the overall guidance of the Project Manager, and in close consultation with the Project Officers, the PC will: Strengthening the referral mechanism ❖ Conduct regular supervision and monitoring visits to CBTBC volunteers/ Field Agents in the respective townships. ❖ Coordinate between TB volunteers and THD/TB teams/ GP/ Pharmacies for the referral of presumptive TB cases for diagnosis and treatment. ❖ Lead and coordinate teleconsultation services in collaboration with private X- ray centers and project medical officers to provide TB services to patients at the office. (PSA) ❖ Ensure that teleconsultation sites are operated in accordance with TB infection control measures. (PSA) ❖ Facilitate laboratory investigations for sputum samples collected and referred from sputum collection centers. (PSA) ❖ Arrange the provision of performance-based incentives fo</t>
+        </is>
+      </c>
       <c r="T28" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -2873,12 +2947,12 @@
         </is>
       </c>
       <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>94 townships of Myanmar in the areas of disease control</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>MHAA. 1 Myanmar Health Assistant Association (MHAA), TB Hospital Road, Aung San, Insein Township, Yangon, Myanmar. Position Summary Under the direct supervision of the Project Manager and with the guidance of Technical Leads from MHAA Head Quarter, the Project Officer is responsible for effective and client-centered management within the Project Area. Key Responsibilities ❖ Manage and lead the integrated MNCH project implementation together with Township Project Team. ❖ Assist the design of activities that promote equitable access to the services for marginalized people in the township. ❖ Develop a strategic work plan to implement progressive activities for the effective project implementation in the township. ❖ Organize, support and facilitate regular stakeholder coordination meetings, community meetings and CSO/CBO coordination meetings. ❖ Provide technical support on supervision visits, meetings, training, and action planning for the project staff and volunteers. ❖ Support and assis</t>
+        </is>
+      </c>
       <c r="T29" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -2953,12 +3027,12 @@
         </is>
       </c>
       <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>94 townships of Myanmar in the areas of disease control</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Myanmar Health Assistant Association (MHAA), TB Hospital Road, Aung San, Insein Township, Yangon, Myanmar. Summary of the Position Under the direct supervision of Head of M&amp;E, the post holder has overall responsibility for successfully management and implementation of monitoring and evaluation activities for TB, Malaria and other disease control programs. He/she is responsible for designing, implementing and supervising project M&amp;E activities,</t>
+        </is>
+      </c>
       <c r="T30" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -3045,13 +3119,12 @@
         </is>
       </c>
       <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>70
-branches in Yangon</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>BRAC is an international development organisation working across Asia and Africa to alleviate poverty by empowering people and creating opportunities. Our mission is to support communities facing poverty, illiteracy, and disease through large-scale economic and social programmes that help individuals realise their potential. Since 2014, BRAC Myanmar has provided pro-poor and pro-rural services through 500+ staff across 70 branches in Yangon, Bago, Mandalay, Sagaing, Mon, Shan, Kayin, and Nay Pyi Taw. Using a microfinance-</t>
+        </is>
+      </c>
       <c r="T31" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -3139,7 +3212,11 @@
       </c>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Founded in 1956, DRC Danish Refugee Council is Denmark’s largest, and a leading international NGO. We have continuously been ranked as one of the best NGOs in the world - and are one of the few with a specific expertise in forced displacement. In over 40 countries, we protect, advocate and build sustainable futures for refugees and other displacement-affected people and communities. To support and strengthen the DRC programme in Myanmar, we are looking for highly motivated and capable candidates to fill the position of</t>
+        </is>
+      </c>
       <c r="T32" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -3223,7 +3300,11 @@
       </c>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>BRAC is an international development organisation working across Asia and Africa to alleviate poverty by empowering people and creating opportunities. Our mission is to support communities facing poverty, illiteracy, and disease through large-scale economic and social programmes that help individuals realise their potential. Since 2014, BRAC Myanmar has provided pro-poor and pro-rural services through 500+ staff across 70+ branches in Yangon, Bago, Mandalay, Sagaing, Mon, Shan, Kayin, and Nay Pyi</t>
+        </is>
+      </c>
       <c r="T33" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -3311,7 +3392,11 @@
       </c>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>The Myanmar Heart Development Organization (MHDO) is a national non-governmental organization established in 2006, with a strong mandate to deliver community-based humanitarian and development program across Myanmar. MHDO works primarily in the thematic areas of food security and livelihoods, WASH, health and nutrition, disaster risk reduction, and emergency response, with a consistent focus on vulnerable and hard-to-reach communities. The organization applies participatory approaches and aligns its programming with humanitarian standards, donor requirements, and national priorities. MHDO has successfully designed, implemented, and monitored multi-sector projects in partnership with INGOs and other donors. Key achievements include effective field-level implementation of livelihood and agricultural support, WASH infrastructure and hygiene promotion, community health and nutrition activities, and timely emergency response and early recovery interventions. MHDO has demonstrated strong cap</t>
+        </is>
+      </c>
       <c r="T34" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -3458,8 +3543,16 @@
         </is>
       </c>
       <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>No.125 (B5+B6)), Bo Saw Aung Street</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Program Coordinator; • To assist various tasks like interpretation (i.e., Myanmar to Local Language/English or vice versa), arranging/compiling relevant data, data analysis and periodical reports etc.; • To document of Case Management activities of Drop In Centre/Outreach Project Office related activities. Nursing support Tasks • To get blood testing related technical support from Nurse-in-charge or Lab technician; • To assist the Medical Coordinator in giving appropriate medical interventions and nursing care to the clients; • To dispense medicines correctly and appropriate information is given to the clients; • To perform laboratory HIV testing as written in the AHRN laboratory protocols manual at mobile setting; • To maintain laboratory equipment in a clean and operable condition to perform the Quality control of HIV testing where no lab facility is existing; • To participate in the Health Education sessions and provide relevant information when required; • To ensure proper cleaning</t>
+        </is>
+      </c>
       <c r="T36" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -3542,13 +3635,12 @@
         </is>
       </c>
       <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>9
-Duty Based: Yangon</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>in 2006. Inspired by His Majesty’s vision of heritage-led regeneration, we support artisans and their communities with everything they need to sustain themselves and revitalize their heritage, in Afghanistan, Myanmar, and across the Middle East. Turquoise Mountain Myanmar was established in 2016, promoting traditional textile weaving, goldsmithing, and lacquerware production, and the rebuilding of historic buildings. Turquoise Mountain supports the sales of traditional Myanmar crafts to international markets and showcases the artisans’ work on a global stage through exhibitions, creative and commercial partnerships, and bespoke commissions. We have also established a hub for design, and craft in Yangon, Myanmar with a strong focus on public outreach and crafts education. The hub also has a boutique that brings the best of Myanmar craftmanship to market. Purpose of the Position: The Programme Manager is responsible for overseeing all aspects of the programme’s administration and impleme</t>
+        </is>
+      </c>
       <c r="T37" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -3629,10 +3721,14 @@
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1, Kant Kaw Myaing Street</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr"/>
+          <t>Ward 8, Yankin Township, Yangon</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Sun Community Health (“SCH”) is a non-profit, non-political and non-sectarian organization. It is a local non- governmental organization in Myanmar and is established in particular to advance socially beneficial purposes in Myanmar by promoting and providing information, services and products related to the prevention, promotion, curation and rehabilitation of the major health services including but not limited to HIV/AIDS, malaria, tuberculosis, maternal and child health, reproductive health and non-communicable diseases with the aim of furthering good health, prosperity and the relief of poverty, distress and sickness. This also includes state-</t>
+        </is>
+      </c>
       <c r="T38" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -3717,10 +3813,14 @@
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1, Kant Kaw Myaing Street</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr"/>
+          <t>Ward 8, Yankin Township, Yangon</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Sun Community Health (“SCH”) is a non-profit, non-political and non-sectarian organization. It is a local non- governmental organization in Myanmar and is established in particular to advance socially beneficial purposes in Myanmar by promoting and providing information, services and products related to the prevention, promotion, curation and rehabilitation of the major health services including but not limited to HIV/AIDS, malaria, tuberculosis, maternal and child health, reproductive health and non-communicable diseases with the aim of furthering good health, prosperity and the relief of poverty, distress and sickness. This also includes state-</t>
+        </is>
+      </c>
       <c r="T39" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -3801,10 +3901,14 @@
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1, Kant Kaw Myaing Street</t>
-        </is>
-      </c>
-      <c r="S40" t="inlineStr"/>
+          <t>Ward 8, Yankin Township, Yangon</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Sun Community Health (“SCH”) is a non-profit, non-political and non-sectarian organization. It is a local non- governmental organization in Myanmar and is established in particular to advance socially beneficial purposes in Myanmar by promoting and providing information, services and products related to the prevention, promotion, curation and rehabilitation of the major health services including but not limited to HIV/AIDS, malaria, tuberculosis, maternal and child health, reproductive health and non-communicable diseases with the aim of furthering good health, prosperity and the relief of poverty, distress and sickness. This also includes state-</t>
+        </is>
+      </c>
       <c r="T40" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -3885,10 +3989,14 @@
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1, Kant Kaw Myaing Street</t>
-        </is>
-      </c>
-      <c r="S41" t="inlineStr"/>
+          <t>Ward 8, Yankin Township, Yangon</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Sun Community Health (“SCH”) is a non-profit, non-political and non-sectarian organization. It is a local non governmental organization in Myanmar and is established in particular to advance socially beneficial purposes in Myanmar by promoting and providing information, services and products related to the prevention, promotion, curation and rehabilitation of the major health services including but not limited to HIV/AIDS, malaria, tuberculosis, maternal and child health, reproductive health and non-communicable diseases with the aim of furthering good health, prosperity and the relief of poverty, distress and sickness. This also includes state</t>
+        </is>
+      </c>
       <c r="T41" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -3969,10 +4077,14 @@
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1, Kant Kaw Myaing Street</t>
-        </is>
-      </c>
-      <c r="S42" t="inlineStr"/>
+          <t>Ward 8, Yankin Township, Yangon</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Sun Community Health (“SCH”) is a non-profit, non-political and non-sectarian organization. It is a local non- governmental organization in Myanmar and is established in particular to advance socially beneficial purposes in Myanmar by promoting and providing information, services and products related to the prevention, promotion, curation and rehabilitation of the major health services including but not limited to HIV/AIDS, malaria, tuberculosis, maternal and child health, reproductive health and non-communicable diseases with the aim of furthering good health, prosperity and the relief of poverty, distress and sickness. This also includes state-</t>
+        </is>
+      </c>
       <c r="T42" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -4057,10 +4169,14 @@
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1, Kant Kaw Myaing Street</t>
-        </is>
-      </c>
-      <c r="S43" t="inlineStr"/>
+          <t>Ward 8, Yankin Township, Yangon</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Sun Community Health (“SCH”) is a non-profit, non-political and non-sectarian organization. It is a local non- governmental organization in Myanmar and is established in particular to advance socially beneficial purposes in Myanmar by promoting and providing information, services and products related to the prevention, promotion, curation and rehabilitation of the major health services including but not limited to HIV/AIDS, malaria, tuberculosis, maternal and child health, reproductive health and non-communicable diseases with the aim of furthering good health, prosperity and the relief of poverty, distress and sickness. This also includes state-</t>
+        </is>
+      </c>
       <c r="T43" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -4143,8 +4259,16 @@
         </is>
       </c>
       <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>No. (B 36), 65th B Street, between 65th * 66th Street, 103rd * 104th Street</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Sun Community Health (“SCH”) is a non-profit, non-political and non-sectarian organization. It is a local non- governmental organization in Myanmar and is established in particular to advance socially beneficial purposes in Myanmar by promoting and providing information, services and products related to the prevention, promotion, curation and rehabilitation of the major health services including but not limited to HIV/AIDS, malaria, tuberculosis, maternal and child health, reproductive health and non-communicable diseases with the aim of furthering good health, prosperity and the relief of poverty, distress and sickness. This also includes state-</t>
+        </is>
+      </c>
       <c r="T44" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -4224,7 +4348,11 @@
       </c>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>religion, age, gender, sexual orientation, or disability. Lan Pya Kyel is committed to maintaining a workplace free from fraud, corruption, sexual exploitation, harassment, and abuse. Our employees are expected to adhere to the highest standards of integrity and professionalism, as outlined in the Code of Conduct. “Lan Pya Kyel internal staff are encouraged to apply, and will be given equal treatment to external candidates”</t>
+        </is>
+      </c>
       <c r="T45" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -4308,7 +4436,11 @@
       </c>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr"/>
-      <c r="S46" t="inlineStr"/>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>reflects our commitment to the protection of children from abuse. All staff has an obligation and a responsibility to: • Ensure they fully understand the provisions of the Child Safeguarding Policy, the Code of Conduct and Local/Country Procedures. • Conduct themselves in accordance with the rules of the Child Safeguarding Policy, in their personal and professional lives – which includes reporting suspicions of child abuse. • Ensure the way they are carrying out their work is not putting children at risk (or further risk) – this means constantly scrutinizing their work through a child safeguarding lens and talking to children about possible design/implementation “flaws”. • Promote the message of child safeguarding to colleagues in other organizations and government ministries, children in their own and beneficiary families, and community members in general. • Be vigilant about observing possible child abuse/harm in their personal and professional lives. All managers have the above resp</t>
+        </is>
+      </c>
       <c r="T46" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -4392,7 +4524,11 @@
       </c>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>the content or location of the role changes, in which case the Child Safeguarding level will be reviewed.</t>
+        </is>
+      </c>
       <c r="T47" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -4468,7 +4604,11 @@
       </c>
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Mercy Corps Myanmar, through the Climate Resilience of Mangrove-Dependent Agri-Food Systems through Market, Household and Community Transformations (CRAFT) programme, invites private sector agricultural actors to submit Request for Application (RFA) to participate in a Partnership Facility designed to expand climate- resilient, inclusive, and sustainable agricultural services in the Ayeyarwady Delta. This RFA is the first step in identifying private sector partners who are committed to introducing or scaling innovative, climate-smart, and gender-responsive market solutions that benefit smallholder farmers and mangrove-dependent households in Bogale and Laputta Townships. Selected applicants will be invited to a co-design process with Mercy Corps to develop a detailed intervention model and partnership agreement. Programme Background: Through this activity, the CRAFT programme aims to support target households and communities in Bogale and Laputta townships to improve climate resilience</t>
+        </is>
+      </c>
       <c r="T48" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -4557,7 +4697,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Volunteer</t>
+          <t>Full-time</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -4620,7 +4760,11 @@
           <t>No.42, Strand Road</t>
         </is>
       </c>
-      <c r="S50" t="inlineStr"/>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">terms of relief distribution, transport activity, local purchase of relief items, support to health and care activities, support to disaster management programmes (such as purchase of disaster preparedness stocks), carrying out custom clearance of the imported suppliers, dissemination of procedures and guidelines, training of staffs and volunteers. Since early 2013, the Logistics and Supply Chain Management Department has been supporting MRCS develop a common community- based approach to build community resilience. Technical assistance and support on strengthening disaster preparedness and response systems is also included in the operational plan. Logistics and Supply Chain Management Team is supporting to those programme as well as other projects and programme which MRCS is implementing in country with the bilateral supports of Partner National Societies (PNSs) in Myanmar. Purpose of the Position: The purpose of the Logistics Officer is to initiate and implement logistics activities, </t>
+        </is>
+      </c>
       <c r="T50" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>
@@ -4641,7 +4785,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Volunteer</t>
+          <t>Full-time</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -4704,7 +4848,11 @@
           <t>No.42, Strand Road</t>
         </is>
       </c>
-      <c r="S51" t="inlineStr"/>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Society (MRCS) is a dedicated emergency response initiative designed to address the urgent humanitarian needs resulting from the recent earthquake that has impacted multiple regions across Myanmar. Coordinated with support from both domestic and international partners, the operation aims to provide timely and effective assistance in key sectors such as shelter, health, water and sanitation, livelihood recovery, and protection services. The Earthquake Operation is managed under the Mandalay Earthquake Relief and Recovery Operation (ERRO) Team, working in close collaboration with MRCS Internal Departments, Branches, Volunteers, and Communities to ensure a well-coordinated, people-centered response aligned with MRCS’s strategic priorities and operational guidelines. Purpose of the Position: Field Officer will ensure all activities are implemented in line with the project goal, objectives and output indicators. Field Officer will be based in Sagaing and will work under the direct supervisi</t>
+        </is>
+      </c>
       <c r="T51" t="inlineStr">
         <is>
           <t>https://themimu.info/jobs-for-myanmar-nationals</t>

</xml_diff>

<commit_message>
chore: update jobs data [2026-06-17 08:10 UTC]
</commit_message>
<xml_diff>
--- a/mimu_jobs.xlsx
+++ b/mimu_jobs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MIMU Jobs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="MIMU Jobs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -701,7 +701,11 @@
           <t>Solidarites International</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAVUAAAEXCAYAAAAdnNdJAAAACXBIWXMAAA7EAAAOxAGVKw4bAAALP0lEQVR4nO3dy47b5hnHYW08dnxK4tz/DeQCegldddFFgbZBATdJbc9IM4HvQBWNGFAYSiJ14P/Tq2fxDBAgQ/00BF5TPHxaLBaLNQBnEw8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPIAb9vnbb9dP3323/u2HH3ZaN9AJE8QDuCG/ff/93gE6ZNe2Nj/Wj72B3P13+j1y8+IB3IDHzRHp1GG62vzO0LZWBwbz6t27+PvlpsUDKGx14KN939CR5mriQH54/jz+vrlp8QAKWr55M3oIdv9v//d/2Zg6jNe9bTy+fTt8JLs50k3/fSgtHkAhyx2DrO9px0f7pwnnXIeOah8mHBmn/1aUFQ+ggIfXr48eZlPOtz4ODOND51jHbgfOJB7AlXuaMBS/fvS+f/Fi0jD8cHf3h9fc/DhqmHbWDfzNKC0ewBU7ZqiN9fT27Z9er38L1dhTDeuB9u5c7vZgdjsWZxIP4EpdapiuB15r6lHpro/3DyOOqtN/V65ePIArdIlh+r73GlNOK3R23tfaOyLdO4wdrXK6eABX5hID9eu21xO3P3R7VLeNY863Ll284jziAVyRS33knzwAB+5tnXpk23l6/Tr+N6WceABXIj1IO/e9o8mx98X+YZAOPCiwy8Nm+/cGL9PEA7gC6WH6ufc8/9Tf79YDuH/2bNR73fUkVnofcDXiATTumMVQzuWpd+HoXHcBDBlz+iC9L7gK8QAaduwN9ufwr+2OiR/z7wfucR3y8OLFtCNedwdwWDyARn28u4sN1M77TcNy4lD/z8j3dso/Fr82sG9oWjyARiUH6lTrEe9necZ/JNL7hqbFA2hQekiOMnIJv/sLnBO2fCB7xANozDH3e85p17KBfVPPw051/+pVfF/RpHgAjUkPzb2DbET//2Y8F5zeVzQpHkBDdt2jmTbm4/Y/Nrr7UefsWjoNwJ/FA2hIengeczT48Ztvmu7j5sQDaMR/F20N1V9GfIFfurHjohU98QAakR5OX415Cir5UMKQ9L6jKfEAGrD5ER9MnU8Dq09t+9ToOV/rsLIlHkAD0kNpzNFeuu/Ufm5GPIAGtDyQWr9v1lClJx5A2OZHbBAdOn+aHpRTuGDF7+IBhB3zDaXn8OOepms5Ou1L70uaEA8grKUjuk/Pn8cHo6HKieIBhLUyUJcvX8aH4qnWDexP4uIBBH1YzDdU9w3UVh+PPed75GbEAwiac+DsarjW86dT3yc3Ix5AUHrQPIUukhmqXFA8gKA5hkz3tSxDr33O9U67OxiWmyPe5Zs3X7abuqPBUGXRQABBlx4wu84x/vrs2emDdOSX+83xPrc9vHwZ369ExQMISh21Hbu9sav+J97rMcOekuIBhKxmWId06HV/O2KFqXMMqtVMF8TGrLJFafEAQh7evLnocHnYseLUpAF15tWfDFVmEA8g5NJrkg695odXr0b97vLAEoB9T1tfo7LvXtE5hurUdsqJBxDyeOGPw0OveWiQTzkyXR24wj/0O3MMVReqbl48gJBL33Y09JrLHUN1yjAde2/r6vXrP/3uHEN13cC+JSoeQMihI71LDNUvr/v7YO2u5P97Qu/UBwV+6v3+XF8QmN6vxMUDCHm88IWqc3Vufpzl9ef6Xqv0fiUuHkDIcvPxuPXhstq6ADXFh4FtzTFQDVUWDQQQsvlx0eFyyo36pzzCOnT1f457cg1VfhcPIOjSA2bqUnjnWAIw8T4NVbbEAwiaa9Cs9zSsznhud3D7My8tmN6nxMUDCJpz2CSG2fu7u1kblmd+AoyrFA8gqMoC0bve39wd6wb2KXHxAMLSA/EU6UdSxw53bko8gLD0YDx6oO75qJ1YpPqUux0oJR5A2NwXcs7hw57n6y/9pNgu6wb2JU2IB9CA9JCcYt/78DUqNCAeQAPSg3KMQ/e8zvUY6qAG9iHNiAfQgEuvA3CqQ6tYpfvS+4+mxANoRHowHTuw0n37Lphxk+IBNOLSi1ZPHlYHPu7/vMgP1DFDn5sTD6Ah6QH11fpKOg1VBsQDaEh6QB06d3p/4eUKzz38uUnxABryyyIzWA8N03Woax83+7NDPIDGzDmYxlzkWTZ2rver9H6iWfEAGvP3xeUH6+OIr3H+NEPH0f8YOEplt3gADbrEjfSPEwZR9EZ+R6mcJh5Ao841gJYDXxW98zUbH6YGKiPEA2jY0UelE2+If5oyTLfuXzVQaVA8gMYdM+zG+HXiqvyr3nnYuR+tXTewL7gK8QCuwK5B8+n580nbWS6mryR139tG4nzrzw3sA65GPIAr0X1tdDcQ30/4nZ8Wxy3H17+6/hC86f9zA397rko8gGK6j+nHHk12g3t7W+kLVx9fvIj/Pbk68QCu3DkWhl5unS/96+K4j/jn/gaDpYHKceIBXLFjHxTohubT1lHp5sdxg3Tr4tiPR7YMbnfEwwmwQzyAKzf6yG8zRNe93z12ucH+c/fnvHi17J2CgIniAVy5XeuadqcF+kd8p6wy1Q3O9da21jte9xSPEx5UgB3iARS3+XHaR/He/a9/OXF7u6wb+FtRQjyAwo4epJuP9//sbWs58YLY07t3o//f9N+JUuIBFLWa+FG/OyJ9ePbsD9tYTnxqanspwc2PyUfBcAbxAIp6XBweat3R57r3e8dcdPrbEdtYOX/KZcQDKO6pd4V/aLGV7qb/qYP0sXeV/svTWyOG6dTFXmCieAA3bMoQ3XWr09hvBpiyBCGcIB7AjRrzBNTQCvvd6lT9o9997g1T5hUP4IYNDdZdH8+nPIb6OHCuFmYSD4DR9g3Sj3d38T5YNBAAk3Vfpd2/jxUaEQ8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAlcQDACqJBwBUEg8AqCQeAFBJPACgkngAQCXxAIBK4gEAZfwf+VfpLwPNMBEAAAAASUVORK5CYII=</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
           <t>Human Resources</t>
@@ -877,7 +881,11 @@
           <t>ADRA Myanmar</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAZ4AAABuCAIAAACY++L1AAAACXBIWXMAAA7EAAAOxAGVKw4bAAAYS0lEQVR4nO1dW2/cthLW/+lj/4AfDgoURYv2YXGaNIm5TmGgBYLaib0rabeAfvqhpPV6Tc2Nw6EkH/MDURjNijeRn4bDuVTVa8fuY9Vuq2Zbta5q3PDf674cbuDS//j69OODGx7c9n8UFBQULINv76v2+kRkGHOlF1/5SJGPbukBFxQU/F9iv6kOA5e1ObmMLrWnuZueUrtfl56OgoKC14vNZiCU5biMkelcT3OecwsKCgp47D8tKZopy3VVf1p64goKClaIGtf3v6LSDtcRBQUFbx13vw4XlEtTUo5SLh8KCt4idp96GSc7xQwWHp49m6cDY7fpLwT6f8rfeq+MKwfVgoK3gC757EmYqj1zyrYnNQmaG55hW5fKg76GLuu0FhQULAglLww2H56DRvgzLP1jz32xaDizkvr90xBGe2DVRYfvWGc1lQUFBWtArTJJ81zw99WLejyvEfX4VjZaa4yu6s+PBGM+/PDi9/cbpWGKl+AKCgpePRoXfVHgeeRvhKGIw2N7Az8ShfoTxbMgPMfFsvZoE1dQUPAq0b6Pc4Tyu/3LH2SFuFS1s9PWP3ykekigl+NijPL85NTOrNsFBQXZ4a5ipJhtdfyTr/NAnEOdcf/3G/SuQ6LIO3yOIDhPl866/wUFBfZo5WKak9bZ4JLU8T3/uAIUk4olxCiCKygoWCl6rZPQMiNyJ2MckfVAd8DHch9zWeEFQNHBfNtfkhQUFKwL7Qd+9/YmaS66ZsymrM3v0oTdWiiErMO16DqlLSa+BQXrgURYO6puMA/YlaUzHgIGjN32qiPkccsTXF28UAsKFsftrUBYSzDLAI+iM18sYsdhNSTiW1fCJRUULIUdS2qu+vKjvv4jpqKaV+m+Q5hI4fZwxl8/8R5jj3luSAoKCijwzu3JByvQAmOR8xp27ZtaLXe9UJeb04KCOcEeqfYfUpvA9HcpYqAa2Lk73WijY53zLbwsCgoKeDDymouzjcAAVn5cTsV+zCO4VUOodNoY0H9IVg56Sdx+P3d/6s/Vvzdh6b/HW7wMv5nzw9m+48492tIOnnz9FdynXu9hsh/VoCP9rOjL3eJeliOv2bSSjUfU6LDIJUZsy3ww1n1tOiaywEr6tU8mCmDLZVgHc+SjNphErpeJAt2RvklrMVanNd8pavUAcP1OVdXg11kPYZGa4SvRh6L8XVPVHhq+oXkdzW4rdzil4qC41MqXojbgdQ/5G03kID21OaD0gblkkRDb4Zdzyqd0f5Y3BqB5zTDvyeN7uIlY7DkrWQVXgvXobNxA7G7IqE0r+cRBoJdv8y6p8vbmlCkxjgK2Tw+OZftces/li3JwT2EBxQQx2p/XCTplL860T0QTNS4WDz/IMltuq8dZaIXphpujDygIZwM/g9/SFm7YlsX4hcHUYs1TYMYxdSHwk0k4ZqXfz+QAall9sYussN9K/ZQT4ReGJJP3+PlUBwo84/BZGiknCuxc5Q4gSITSOW2fZT/Y2AT59xrEaEwEdhd5K146t9+L1sdl8bMvB1hDFz9SAl5EJw6ndOinRSAJBGDc4gf+mt64RcdoDDwx7ZIbvSe1lupx0XPld/ftz6k9xyAKErGUCSf6Ll0cKUgAX1PE8Hosr42LMqJ+aJWYf/o8QWPLcYX5ACWTnOPjTG+bHPCnSFDl+rwStv3nORE0E+nA5vfokrsNtytYG8tcJmCKAP8KH/8b/th/cwKh2r+kqA8CvCvEm1mdn0XOF7tf4NmQw5909i/76ZlxKot9w9XMK7oy9xMiUxXlsLWmtVRZQbNPoo6CPuDr+8zpDcyxZzUVs7wsAJgxF9gb4lQv3Pmb75KG7TlUx2uxkwsKC0IQ3/zmpp+BSzzgK2M9VwpEbLsZlu+Cu+WOjHaTKIlkGhd9GWguPclvSGYI5PMC6Kdp8lHifYYEXQd1GfIx0ycFvogbAtW9kjMp+9n05f7l3GJh4wxNbRIR9IoanbNvvcalp3lA5NPwH3ssyweLTNRG1+zL0fROLNjItPnufECjlU06IckNehAEIwOXqdxuQMlo54actCFQ18tS8D9iO6bAfJ/QCSyO6YmD0LXn0BISa282EPTa72ddOK9sFEBfWRq6vgRE1lxzXiv/MWuaQoePP9CdydVbrFyT8iIbwdUSW+QAdxSNCOF8IpFhG/ivpaODBINyV9Xud2poj9bCJrH85sSePLVoYpdmo7YKOXaci5VxeHCSG0G1O8+nmlCcXYL2sJkW4rsNHtbkN48HznxGxCniyQW/P494b7/8GNeTwN79+Ccyn+L5yQRwbdhucqYD66C2ShALJwpW9YCoueVngssKz7Q1Q7sU9uJ1yYc2CopDGwW10Y0g2dWpJ4mKtnGAcnUbeHbGH69JWQboyWSiMCPknbX9jRzBJJxjjtJCgS3WQ20VN/Co71DuCaRNea+uUusPxdgztZHq5uwJyNFdNJlW3gw96Dr+YkCy+Ci2B1ZkpwdKlIFbzLITqiOfi5OOcUEH46A/3dP17vek1bQulDyGVVFbxa3DvVhJT1RiAsbzIfky4QCdRkcQlwl5HaUPyBkTlGgMuSPxLcqTBOq6B7QIbSrM4UZuIXGabWjsaCULJYu57ENwY0tQue2XeW3UVhmdudJrYOqn1W3J38sXFb6sjWb/dJc1FNii5AcgKQ6upwPvHJEfg6gRp/qoEgVwU2HuGdEnd6Qz2Md2fgT6muC0VSPKwbF0DqxSgxVSGyuhS2C1SjEwrp1pGv1glQZSEe1MlpJKhUHUUGO3K6aNAq2WY2/NYzsTlFhbCpBlsM+dxDdQ8oIxirxzcZ1PR7CBga7OonFbIbVV3BliJ4ipNcfUEZ10STU3+Gn09IMMnmQMsJ0T+3usYMYKIE10V3Gdj+rJtMRSG+j8gEmasTekxJybdD4R4XCg1um1YYV1UhtznyA47s0xddmojd0RTGiDHCZN4CvZ49vmW+QxEEOK69IZiY5WikN+1BijbhII8+Y1hCAOaAsUxh25fK2iM62T2iruQ8vG+FNsIsMepuhDJR3uOiVRWHbrwDljy7cr8bGasrhucmO19anNxbyVllQ/yV8tJhHsZgx2FDSNZT+gLhOMxMzVUhsttOrM123HRa3AhLcTGKj6LxyIWaO2EAuxuelv9OEukk7CzwUZ4QigRe3kathN2xb4eojo0kILFWLsRA2znUmb3160SxiR0+cOk8jRq6U28GZMuE6qpaktxaJIuCazhk4JwUamxaRowkNYyFOGk7uJZDc/arWBIlwn+VZY7SR2FK2vGQ3ObAZugcsk7RpMddhil66W2irOjJy24M1NbV/+oJq406oLAiqghVOKamy/07Rf/pmkwI8tlumqj9FODs8/iF01pphrCT1bUySdxuGO6yTLKI5pQl+LeRA06q6oH9PfS4POrJnauE8sgdxvOZNxWeCEsCfrmc9rRbJ5xnJ08OBb9xRLfnvKHUVAlJli+LZ/VRHQjksUojvz+gM4EenhXPrf0MO/Oc3V6QVj5jUxd9DH/ILb18BkyTG/p7+X6VGa10xtDz9wiwQXjnLv+Uy08mJtcPuLPu2ZxVvdxduU9lFK4gXX7p3WKcopo181A8ucaU43ZX0SEFW3+9QhYk/YM/yeVzTHho1KR+BfLPEcova2S+3Pmqmt4sSFXaRzjuG4cnBKE5gBC0QHil6szqQp7uV+E3p5gfgC+zPs47WRm2eGHFoE6vfSPEOSbu8+UJlBOtcb0yS9iPz7OWhRkhk+65l05dTGZIpx6IP5ZqzKdnMdVHUUiOTMRZPTd+aiDYvIGTMXL6TUkdn2JPBE7GecTZi0wpI74tVjYM4mO/9iEZlOL9EldWnl1MbeaGHXxMQj6aCEDO0SCnLRCSmSsW02Wc/CxJ3rLOfkuGqx5bA9JZ20Ei2XKlkRSJQR0fSId5eYQ2Dd1IYlnzwXzAQk3yumcpi4hGqDFyGuit7XBgCXCB07dOXFz3VzQVhevqufkoS3gyGFwmV9PSUqioEVgrbkms8jOdUpcvfaqY3LiosJJsQjKWjIKPbqTA7VRBKUhxGk18a/6ew2lVbG40Z3tfw2LuWy+M0wqjXBf82H6X2WHHR0gCT9zrqpreJuEjAdAvGIGrRb5L8Jd1B/T96vHDTDGERwA7fQGXtBsu5S5igX6w/U4+RDICd+jdwJxKDeMrVh/Yz9PQvaYqlJu1sPNBWxOt+8TldApdNw4dve48p8u4Kk2R8e8xGESdmiyyWLwm6y+GamtuCVxYK++VU71qyf2lhLeBCxv6exJ3htaxD9MbgNIJKEgKDD66cmAAEqRfS7e2ezdUdGq7gtelgZx41qO2rehs731stGci4m1MxJbUGKeJ3unx6mDuunNl06GKuJ8q1j3NpsbQJ23/1qMPPEoTD13h8cOdsbDcdNXK+EW7Qevu0m6V1iiz+LHa/hbxG7+Jotn0AInCXs0yJv2hAzXLno8AqoTeVulThRNbc3DXOhqcPtyEtSGprpREg0IHtx8FiCKBXSR+/cO7hzWdnTTkvPode861LU4uvPBbIOS/J1qte9ArnX7kGrMH6D1LaHyrgdjuLtcGU3wBnWRlKqIHCJsJBTGwFQIohF+ylJsmhHj6h4X67YwQq5eFXUNo9CQHnIfXvUZlKsckexfrJWRQ/QZJeFDbXZ6Yzmn7vYql4jtc1m3qjAK6A2a10bWxqZ8blJPo3ZjEPv1VHFF5TadE3DVc27r7AWCVhRG2gplsnRap61exB7br3o2yunNkznRTzSbeByP/7RnWpgLVJNsibOZhOmWBsnwBzPbRUbaoNuBnRImTsFgnizY6FFfStqAyO16F8/jil3NJ+SCrV8nUH3EpeQOZh3ndNklxWpEp00byavL3Ft0LZldFxiFDsoLyG7VfIdSGtBQrMporgsfSfAS4dcLlbUBja9d5pRMA0F1pjJ2Ybo8Fmx9b92asPGa7VQ6dYTnTSDO7F0b/Y96XKrT1EK1DULtYVhnhKWZhSXpTcHWqLUpPecFbXBPqSfNaOgkYMvDDM8rJzaWB/SDnnQaqHuSGvYvjj96AJqMwFt3aWtNF6db0Jt4OvXfU9i6Sxx1kBLDvpUZUVt82xmSVI+TbXkJEhiwJ2xcmpT57UyXKjsfYIuF9pdnrVBhyCSXK8BgA+GjnrEhNoqlcAorEdeNM1BC5cOim1CbeCbypHRqrFwQpjiTrvhp1g7tZGve4930nahMiHLnKbO0HnLaG08IGc4xdp4BvyFIevKSG2qMehIzXbF0DChNng/Z6C2fGRhFXp35dRG7VLyfdkuVEzncy51PDE1GU6jYM02rzW2Litqm7Lqq6A2RT021AY+4jRDIBC8FFvLEvqq9Iv4iLRmaqMVbXQ+OvO9zeYPiorW7V7WZntiYC52Y/r5DFB5RAiBVtQGWsecLXQi+v8GqA27IDdH8FKO1jlliOHLt8qaqY02ZaBhu1BP/aH1ADGCW2CwZa4MIfqp9KMA790IAcrsQApNuiLWSiydpawYTO5gnkqmNvD3Zul/ntBN3og5aMFNiDVTGzE69lBiuFAldQp79VyVs+kShiz3pPCYkeqsqG0HjUSR6EDYGZP5gieKO0klUhv2eHcb3X8awaEgR2p6evlK8iFVK6a225+TFpv9xh7A3NjKheWLpxR6Or6f5NrQXibETKgVtVXQu1RIuVFclrhiYKNZTtLMQm05nBCCJmZ34RLaZ66W2ggSkXyzDRfqJbqOWXiSTRec7dRhRGlQa0O3GlG2gqrLSm2KtxjFZYltgR8WFinUhiXISIz+PMVfkyD6mZCeq22d1LbB94VQ4jBcqAF2H1L3QrDynWxEsWDM8XTshlU6TQ9sSG0gU9z+J67nciJLXzG6SlKoDTY8zCBPBaE+zBV5ZxxIdRt9h3iqYZXURkTlu/lFVkM2aqsERryEbWYQl8EwpGWAHbk2lPekR+SgOxWkDantCLYY6TkUS2fqFQOvXYkwr6U2dLdkOA7MSROJKT9WSG2Eb1MrTmFntVAxsBE7sEu84Gf5qG3als087GXsZkht36AMibHygrAz6TMFaiQ7wYM6asOkmxzy1O6PsJUoz6dY0GGHWY3bCqkNU4HHWVdkprYvPzIrEDs4B4q2TuWkJQSWbFe4NmDcf0ZrvNSUG1JbZaFukxNZYkPTSRdeeiiorcO/sTnUHGGK+Ax3FJeg7VpZI6a1URsmhMZOo9VCpbrKCW7TQ1/gBZUpPuBzc3T6Wr0VCPaSLvOTmlIb6HzTvIvp8yzUhiUMlkBBbdi3a57AkzlcUwOkGDGtitqwl6uJQ5ef2iouOemUPoIB6slFDKs9GwLbVOdzkLHUBh27oqxm5ESWMk3gdsoktWE/yKTan3Yv62l0BK1uo68U10NtVvLaiCz7Gew2x24Pl1m9X/5TbCIR++45bb1Ttcvz1hqm2JbaquQzqbAzia2k5KmJorYWvyTKpL4NmCKrkvhFu/hU0CS+EmrDchir7XJMFmp6W6dR/Lf/WcAG86yNm1/Mtm0IIpuRl6fMqQ08k+qMpGOLHLHb7xJyaiMOC1bpiAJMVcsm4fMlYLYWThAEtdHRpQxheA49g5iN+oNZz0dIslKN+d5e/M/8mooRdMd0web4qrGLVDVxgKtELtILO5PSQ5Dr5VwjpDaC1/LRzTRJRe47hOemuX2leDCfOd4ZxB3IMYGA/iFNunJoPw8TI21+ic715aC7kfqWNVniVcSBjaS70j9r20PwslKO9JzQmYQRMDtvJvFwCnZaWkRwox7JzMvYgca3m+jSSyuYMr0UMDsKURpr4RED35OUFy0/eCYSR4XcXaS7p5j0ED7+xOhTEqktk4KDCAyZyY3mEve03fk4cOjjzGYe+JacpAaEX43sDZsaHW539bwd8rA2pjGEyywHUjo8zLkk+bHSPjEmxDHiHpGNRZ3M3EPwwV2MGJVCbZl4jYkGITNFVsPL42yUxNPwJ/uZPUz4HxhG6Ow21Fz57nXJN4a3PzOmMM9DcwbNTeGni7UIyb0gz+iqXqEv3SApdJ+SKToK6vgW6u5JegjmS40VhtXUluND7T+80hS5eaI7CLfx5V56fB/97D6NBf5511MkMVFe5sXOy1GgHTOwCWkzHAzBpQ4vSydVFsVCrse/XKX36qRuQvlwWtJbEcWBUPVN2ENs28QNTUVtVlcHt7d9+JD+E6VYN8Me9hJW+1mv7/MP9qeeLXXznrFsTyRFGGT5Hh4/DNmCb3j2bKGYEXL419GMpJkgNIzFf2J7U6GPZqrYqC75FdUOy+PrNi4Q+Rl+HjyXHYeqFBQfvOV+NhSrVLcrYoHNoOIpkx6CEqtCIFdQm+GNWOL+CcpdzPBtm1629Iq2ZCG6hZymzYrFmrndJHBujPSU9WXFQcFuscA+mPnmSFGzQmccS22251DbRfPWqK2/PdhG57fHsH5qG9F8FGstLssrpbZqUDfmbQBTEsenekrvIahY1QlTcmrz9ZvHL223luU2RoFl2/Q8pRkMpzPZxz38lrPneTI30qE4zmU8D8qR9SVqsL/NS21gBLcD6bmWg9owEt+reEdObfVPmvoLCrJis6keN6E6rL3pdbj3m95USJGIbo1gDYtSqK1C7GOJiBc5qA37UilHJKA2/5v7/I7HBQUFDCRH8VbsUXCJGrFxw+4TzKmtxWKpq+6hRLaByNAKCgoWgFTR6KKD5KA1O+DHttSGpVmJ1dF6GV5oBjmbY1NBQYEUXiiTKpIi7bYxU+Hd7+EvDakNizfpi7zzG9J+/bJkMi4vKCiwARFibLqZv8rEnwPuuBvcxFtRmxctsaOo0P3gTpAS7VShmy92UEFBgR69qCK+B+zviQVkQVTY/Pb8MxNq8+In5i4u4aDeMltu9zdX0KuCggIbHH6P9NXYMvuciE5xlt3Sqe3Rodo9moLbD3EOIr1niTOY54KCggVwEJv5nct+i/q4UnEX3Km5FGpr8JMvZvt356KjBvgJUeYZKygoWBVaXBQiSu3CVNt3v1In0zot7BJhmeEbffjhRU/uN2GKdUlhJdOCgoLXh9gINs9ijntmhPSgmIry7Slh4Eisck3iZTm6hea9oKBgBqgJ7iT4zM5rjTyoGV4KCgreBPbXBnyx8tKWi4KCgreJ0QVVd75bc/GC3myZ4goKCtaLGs+j8YrKeHQtKCgoCHH/vrdfS89oN1sZY2p36ojsBQUFbw3NGFRvnSq5oWOxrv4FBQUFL3Bwp2wOS3HZaJI2Wzb1goKCN4er0U9zPLTmkenqwbO1Hur/8uPSAy4oKHiz2HxXHbentN7n8PCnvyfy1/kHh7MJ7kCRBQUF/1/4HxADTQoqcV4QAAAAAElFTkSuQmCC</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>Engineering &amp; Construction</t>
@@ -1133,7 +1141,11 @@
           <t>DKT Myanmar</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAWYAAAErCAYAAADt4CmkAAAACXBIWXMAAA7EAAAOxAGVKw4bAAAjzklEQVR4nO2dTW/cOBKGeciX7QWC+cX+BXuYY4ABAszeDGQyiRO7u9UdDDDX/Cdtl9SK3W0VRYofRRbfw5OdTWw1VSw+TZEUaYwxPaiDjXnX781V311Af7ermPE+3onHFyzTnXJQOmdi5t6+zNwTLwBwpDPX/Q/zH5UcjvcmHV+wzOEoMulcic3e3IjHdQbxAgBH9orFvIeYq0BjDhbaKRAvAHBEY6OAmOtCYw5CzCAIjY0CYq4LjTkIMYMgNDYKiLkuNOYgxAyC0NgoIOa60JiDEDMIQmOjgJjrQmMOQswgCI2NAmKuC405CDGDIDQ2Coi5LjTmIMQMgtDYKCDmutCYgxAzCEJjo4CY60JjDkLMIAiNjQJirguNOQgxgyA0NgqIuS405iDEDILQ2Cgg5rrQmIMQMwhCY6OAmOtCYw5CzCAIjY0CYq4LjTkIMYMgNDYKiLkuNOYgxAyC0NgoIOa60JiDEDMIQmOjgJjrQmMOQswgCI2NAmKuC405CDGDIDQ2Coi5LjTmIMQMgtDYKCDmutCYgxAzCEJjo4CY62Kv8JRsiBkEATEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpOoVi3psb8bjOIF4A4AjErIedeXuU3PVw35ccCqQ7cVCYg4dT3J/fY0rGz7payhH5JAVuQMw66I5Spl6adMyBZL4v9tLlE1WC4x/91yNb8/rI22MP5t0wfkb/O/Zkrgbov8d/uz7+HP37VX9/+v3cZYaY62dzzDfN9Qjc6JbzXT5ZU3JnSL6TdOlR4ub0OBHWY6Hr7E+QrB+ODa5PfC+aG3QLYu6GOkRPGTTYY/57aADvno3X5WsI0/gR9bD/THBvEHO9/Gveq64/4Id6MR//OIr41TCYHqMnHC/w9KUwDn3EulfNDVuzmD8qrzvgj1oxP5o3g4xLEbGNw2kWtoeYLYmqV8ya6w2sQ5WYb435NRFXg5BfcjNMNKKBzyWqTjFrrjOwHhVi/mBMNb1jF6gHfY9GfpGo+sS8U/gyBohD1WK+M+MroDkn8PJVDPX630HMz+IhnW8x2SvqSID4VCvm3WkyTzqAqaEvnQ8QsyoxPw7DbZAy4KlOzLTWswUhn3PjNLQBMZfPN/NGdT2BOFQl5mmfAOmgSVUUrTSBmOvlk/I6AvGoQsy0+L5DQg9fSjuLnDU3+trFTC82aZwLAWkoXsy0V0WrveQ5DkPPeX5JHcRcJj8NXrUGfhQtZq0rLsIr7br/DDFXwfEPlXsUg7QUK+bc+1jUxn7mVW6IuTwgZbCGIsWsWTAx2V3ISnPcahSz5voAaSlKzLemxaVw6zkMr3C/bkIEtYl5a97giQ+sphgxfxikLB+Q2uiOFXgLMRfFj9P2rtIxA/VShJjvlEslNdPWoZpjWIuYv+BYKBABcTH3RueR5zkZtw39DWIW5i/lX44gH+Jixqx1rIrU/fhcupj/CymDiIiKGVKOxwFiFqOHlEFkxMR8wFgc8KBkMWO7ABAbETHfY4ct4EmpYqYTc6RjA/SRXcx0OjSkDHwpUcybo5SxVhmkILuYMXwB1lCamLfY7B4kJKuYOzz2gZWUJOY9huJAYrKJ+Zt5j9etwWpKEfPfBk99ID1ZxNwbzFyDMEoQ8/8gZZCJLGLGm30gFGkxY7N7kJPkYn5EQoMISIq5Rw6DzCQXM3rLIAaSYkYOg9wkFTMSGsRCSsyYsAYSJBPz7wYvkoB4SIi5G/YfwRAGyE8yMWPNMohJbjE/mFfoLQMxkoj5Mx4BQWRyivlfrLkHwiQR867hsWXaO4Gg8fX98amBnhx25m2/PbI5sjv9HW15Ov4cHpVdyCXmr+hUgAKILua/Gkzs/UmwJFzqbfk9MtO+C1ena7QVN78YpxczjjgDpXCILeaWVmKMvePr/tG8iSoGyOElqcV8p7xDsR/y9PXxie1N//1Id4TydnNid8HDKl6rzF3Ki83x3h5m4pSCxyGWiznrntx/NNTjoPucDkFNIYkdBP0i3inFrHnLADp9vk8Yu/OOmb44dgVsBxAk5lbGlump4C5D8LdKE31dzNM1Ds1SpiGyPzMK46DQAYeaxdzC+Nw4jpy/kvanMWjp+5eNfZq47xRvdk9C+ZY5VyHmwsTcwsGqNLknVRHbQSC6v/hspBBzZ94qlvLNkDO581TjHFPVYtbeo+uWZ0mT8+UoEs2P3TZii3mrdKJqYpto/gNiLgaXJNd94jVVTI4xZRdoOZ5moXDEFPO90d2RwIZPcalWzJqHMcblcOKVcMad0gZgI5ZsOvOb6qcOytefgrmpMS+rFbPm3kehS2WGxtfSmHMMMWufoKZ8+CqclxBzIWLeK96siBpxL18BLB+Ui+ayLkJiRfWouadM8fluXovnJMRcjJj1JvujeSsd/EVaGdYIFbPmGE17s0jnotY4Vydmza+xSp8x54P2R/TQ+tAoi+eUNNymMQ+rE/NO9TBGGT0QV0Y56x3rXytm7S/nlDbcBjFng/9Hrb3lQ2HJ3nKjmFgj5u2wtarmmOR93brVHKxOzBoroeCKWES3hPzqZDOsrdcbD6rrroCca8EJhfpg/h9oCzzpgKWphJsqJv3m0L7qwDUOD0oF8RSLG9HtAWxojHtVYtY6vlzTpF8LjcK3Xn4qj0PpOaox9lWJWetj877QnkirjeKpXpYbR688Bq5xkM1BfStgqhHz2CvROdN9H+k0EplGoVdKLkLSfP8ECeK2gDyz1wHEnIm54L8VD1YKSu+NtCympbrRPL4+3f+mgBxbzkGIORNzjUBf8AuuAI9GoVdONjHTvsNan+Cme38s4HVrtxzU54ZCvfDyL7WOL3eVvVTyslHorBeCE/NO+ZazRKqzJdPkIMScifO/GHc109cQ6J6+mffSwQ5sFG2JeX/sRWrtJDzPyxLXK/M5CDFn4vwv9C6Tkz+hJLxR6JXUpZhpvFVjB2GOmp7kIOZsnP+F1kmW2if+xkahs24u6+ez8nu9hMRQ2qvXfA5CzJloo/HvKl6/rL1uiEnMvxu9cxz2+6+j1wwxi4lZ5+PjpuL1y091o1dYk5g136ONrpKNtQ4Qcy6e/g+dfScdpBSUtnXiWjRLa9wMXu/9ubCtYA8XiFlAzDu1GxcVGXiIGZxRwwQ1xCwgZq0TfzXNetuAmHVDTw3fCx9yg5gFxKy14de0gB9ibpuSjpGaQ+NbwcWLWets+LbwXgjEDCb2wwb5v4nnGsQszvgfvdG8IqP8SRWIGUyUPPQGMWcWM72uLB2gFNCXzZ18kCFm4JGz18XmLMScWcw7tVt9lj/TDTGDS0rtNeMFk8xi1vhNWHDQIWZgpdRJQIg5s5i1ji8XGnSIGVih9vhQ4B7NEHNmMR8KCFCaBC8y6BAzWKTE4QyIObOYtTZ6iBnUSokT1xBzdjHrHMrYlRl0iBk4UVrHAmLOKOY71WIu73EQYgau0GvaPwvIPYhZSMzSwUnFo4J9mCHmtilpL3GNq7eKFTOd0CsdnFR8L3BmG2IGPpQ0nAExZxSz1nP+iG/yAYaYQTDbQobkIOasYtYX7Im/5AMMMYNgSuk1Q8wZxay5wX+UDzDEDIKhScD7InJQ3yKBYsWs8VuQoCTq5QMMMYMolPDCCcScUcxaG/xB0QZGmusJuEH1/1E8ByHmbGLW22MuMuAQM1iN9OZGEHNWMets8BAz0Ib0NrYQc0Yxa23wEDPQSCd4Ig/EnFHMeocyMMYM9CE5nAExZxSzxvffCYgZaIQmtekoOIkc7CDmnGLWF2wCYgZakRqmg5gh5gjJCzEDnVAu/AExRwFiRsAhZhANiS1tIeaMYj4oHWMuNOAQM4iCxHCGxqW1hXpC7+RfoQGHmEE0cp/QAzFnFPNBYbALDjjEDKKRex4FYs4oZq0NvtCAQ8wgGiTmnXkDMQdQqCf0jjHjzT/QAjnFojEHixWzxm/BMeDY9hPoh8RyhxwMip90254Vs9bJP3rM+10+wGgUIDldpgNbNeZgsWLuFJ/5l6sngUYBJKFOyC1ycBXFinmrtMdMPAruxIVGAXKS48BWjTlYrJg1H8a6Na+lA4xGAbKQQzAac7BYMdNOVdLBScUePWbQEI+JOyIaFwoUK+afRvN+Gf+RDjDEnBGKET3Stxqr1C+caBRzoZud6W70JZwsDDHngXo+D78Eond4zh6Dm/4LxOxF4WLW2WOGmNuAhPR8ovezMcPfSZdLgpQvVmnMwcLFrC/gqZMUYi4DalibmbmEVuOVcv2+xpgWLWaNjyjEAT1m1dDwxTdmr4hHxevzl9gleuFEYw4WLmadY3KFBh2NIgIk5W5hFUK7MUuT9xp3oizUEZOY34oHKAWFLoWBmIMb07XT0rBdw73mFK9pQ8yZxfyoVMwUdC2vZUPMIyQH12OVfpp2JwFTLBWFmDOLuVecwFre/oOYRynvPXuCrcaNhNMhB53iJN22WTEb1WLWMQGosVH4NqDdijc5vyrO7SViLxfVmIMViFnnBKCWcWaNjcK9Dm+OX7DrT+rQurWtS+7/RA5aKV7MWpMXYq6b8ZE8rOd3b16rfYlqOX7xes0ac7B4MW+UzmBreclEY6NwaTT/mDiTWBonrlygdxR65KA1x6TbtlXMH4zOsTgtKzM0Ngob4/BFvCVfWl+icmsDcXZZ1JiDxYvZKBUzsWbSqDQ0NgqOUcrxn3Ra7TXHGs44FHAv8WNTgZi19ipijrNBzOkbSqrNpzQfCmGDvui+B0yeQszCYtb6ptShzOBDzDOk3BHwrqE4XhJjrgViFhIz7WcrHagUjNtCigcbYl6gyzBRq/WpcIn9sLfIb4Fi1he7KsSsNfhE7Xszaxdzrvp5NHr3H08dY41uKHQ5bRvBJ2pfNqdZzLnrRnMsl+IcskJJoxsK9cLLv9wqnSChXtJ9hAkQKTTLJL+Ydc6luBDSa9aYg9WI+V/zXu2jXs2rMzQ2CsnG0SnN8SVCxvE15mA1QxlaK4Cg+/pTPuhoFDP1kjueXaO9ZpoIf1i546LGHKR4fCigfTuJWfPMda2TgBobxYSEmH83mAREDo4UuDXw/D/Q6RDSwUoFfUP+Vz7waBTPyLFMrrWY2li7TYHWeBXYWWuvEsaKSHNYZSq+GZ0z4k/1ISPmL6bdXvOapxStOVjgODP/j1oPaJ2S8pN88J24M7qHlggpMWvPcxv05Oi7V7NWMdOXc2E+4P9xZ16JByx1ZRRQAVb+p7gxPEdSzDS+qHXzriV2nk+OmnOxsOEM+w9oHs5Ye1RRLsZli3rjf14Xso+SrcQ5NO6an9zGQ36Lec9hKWF1P+ZRT+mrfCXMNIC2ZCEt5o3yPLfhcyamZjETJOdCfGD/AdoqUPvkCFXGrXxF/II2h9ce80ukxUzj+Jof02PFXruYp3gU0HNe/qEWem4kwl5YyL0Z30ZrcbxTWsxjnrfZax6H9Nxi1MqXF8WEcjLliycLyxWXL9DCt+RYGdfDSwcSUugaSnou9tJipi0xW+iEzMffbTijtfgcToJ+CMythyG/3g7XOgzcLC0+WL7onw1VSIw9a33ozbhcq2UpT3GXFnOL4nke/4+ID8skaPoCozH5R/PmRW+a2jKNT9PLed0wHHl1+p35J+BgMbdWIVMFpD7AdfwGbW/Ygou5tJSJzbFOWhxKIlyWLLbkgeWcvfk15GETsO33g8VMk4CtJew4CfDOexG+DZL99vRNKn1/JVGKmFuWj8u6/lbH4QXi7Z6wrT5uH4bDQW+GgzzX9qI78+o0ZNHWl5srJYl5e+w1S8dDim5hXX+rDkhBNDG3vLn4UzCvT2NHV0M8SNbfzPvhdc6/zDjIvzGvh17x7vSIg2R2i6u0kCf6hgW0tGcEeszxiCbmsWLaTFiQlpLETLSyEukSeqLbWnrNaP/xiCrmXcOPeSAdpYn5Y8MSstVFq19YaeIcUcz41gQpKE3MYyekzcd224GtO7T9iHGOLOYdxppBZEoU89/GNDtZy71wslF8gEb+GEcW89hrbrM3AdJQopiNaXcSkKuPj6bdgwXixziBmDcNbG4E8lGqmLXvSW6vk/mNfFr9sorNIYWYx14zKgjEoVQxt5znXI+u1XjEJpmYH0y7Y3AgLiWL+VBAfCSgtv1tptcMMceLbxIxE/8UcIOgfkoW861pd1x1rl46TP5HIamY8Q0KYlCymEcZtZnjNJ5MR5w9jwVtIi9dLg0kF/Mj5AwCKV3MLZ2/eMlh5sDWVp8g4sY1sZjHHgUeb8B6ShezabjzMXe6D+aWwskiZnyLghBqEHPLS0S7ixdO8B5DONnE/EfDvQoQRg1iJrpGxXxZPy0fXhuLbGImHszrZnsVYD21iLnlTby6Y9s+/5JCrzmErGIeK+wd5Ay8qEXMxz+a7SlevnDS8luRMcguZnybpuRG5XBRLWImWh1fJTF/eRELfbmYCxEx96bdtZ+poIYxnsCrTww1iZnOgGy313xeT5uGh3ZCERHzlMD4Ro3HdIoxxCxPq71mksnvL2KBNr42liJiJr6i4qLwfPPyg0Ip1Cbmz6bdtby7ixdOvmPCfxWiYibGzY4g57WQtB6exRM95jJotcMxt+ucxpxMjbiYiUfzttlEDoFi9tjAMqUaxdzq0VPE9qLXPK5rRq/ZhyLEPMkZPWe/inuc2acAYi6HVjsbc/X1gM6XF8WImfhkMKzhAj0ubphj5CHmcmj1/MsxP+dy8y16zo4UJWbiL9NuT8MFis2BkTLEXBbjyqM2RcQd2EovmEHOyxQnZuIj5DwLxeRywxiIuWxaXa9PT74fmJjs8PavQ/wKFPNTUuPbdYLktLX0lCHmMmn7CZCvN+pRY9iSp2gxE1t8uw4JfOcYL4i5PFoVEN13b81VrHHmY1e4mIlpwX5rvefxfv2kBDGXx0PTezXbn/K+Giylm6MKMU9shwRvo/dB98mtvLCh8XXg2sU81kub8uEmAS/BuPM5VYmZuDPjmJ1WQdN97RYeAW2gx1wmXaMb+pBs748dKpcYPTTU8VqiOjFPfDLjjLeWx6DDsGXn1fGefguKC/bKKJPjH81Kx7f+NLXrtVQr5on9KeFrnWA5DL3/qxd72a5F4/IsDWImWn1N+3Cxn4sLP820KktfPrvFrHIxT/xtxt5iLd+0h2FN8rthYjN2HP4174dXYDm+MGwW2B0fNX34fqSLwLcC8isGxz+GuDw0Bt2z66qiS6ahy1raNcRs4ftpw/jSHh0PpxdEaAlgX0CcAKiJzbC8Tu/65/3pBKLxRTLrU6J8ZYSyG3pdV6chg7wV+jzQdFDnzwLiAYAGtsNk6vWv9lXLio4nJ1wN8qXhrd3pSfbW/f7lKyAm9FhEJ3XvTt9IMVd3jJN3E1dRx40BAHZoPXQ37GB3dSbrnEMg4+dd/+KpLG+H5YCdMauHdC6QD3hq+lOwOvNq+PbqziqW/v/NRUVf//qZSfAk+z8KuBcAwDm3hrYUHt8ypJ4pzetsT73V/bMn6cthhO6iNz71cA+//ED/+27YUOzH8PPRpOuCfGABAACcIV4AAAAA54gXAAAAwDniBQAAAHCOeAEAAACcI14AAAAA54gXAAAAwDniBQAAAHCOeAEAAACcI14AAAAA54gXAAAAwDniBQAAAHCOeAEAAACcI14AAAAA54gXAAAAwDniBQAAAHCOeAEAAImgg3tpE3k6aJcOvM240TsIY/yP7bDz//UL6CQA2wU2w6GoL3+PThLwKUg3HMvi/tn7mZ+Px2+zn/mP+U+Cz3pnjcsXpl5s0GkM3a/zxq6PDfPd6tNXdqfrXPLocY3x9Ji5sr4OTuCOKd9uIW9fXsc/zq5smbbAtbmHgLjcDXX29lceXJ6TN53iQXHbeLbRl7kx3wYfPK5Bp73Pxyw8N/ZMfYTeN0H3+Hi8ziURT3ufEvPd7BlXdCO2C/zDno937XPw4OypuHvLZ6c8dJVLLErm2J91WIjvZjjWJs55hYcVCc/Fee8hvk9H5nPL/qW0xGYo3/x5bwtHw8/k33z+x6BjYtUxsd2tiMvtKT99TpeeJH2/Mv57pj3Y2u0l35jcWOoQLvHdvLG2hZBrj/myrj17MCVJXDH7JhjEzMknjpjPG6N7j4EX882xUb13ukYqMXM5+1SP7vdZs5g/Wa7llhPUi/QXCidmEp9rrzmVmG1+8MldPl/WtWcP7EkeImYKTu98oxDzHLHFPDWc7bFHEZrgB8fGk07M9hxYyt3z/KtTzJ8itYXDMPzlJxVOzD6xlxCzb4zn82Vde/ZgSpL4Yh4D7BYAiHmeFGKeGqLLRFCMnkcKMf8ccsZ+bL3PI3WNYr6L3A72nnK2iZmu5TJEkkLM95FzYz5f1rVnD6YkSSNmCoCLACDmeVKJeYzvsgCW4sxJ5zkpxGyTwnM5bJwbWn1idonBU57ZRfUUM/fJu6XPd5F8CjG7tFPKjb9XXn/Ml3Xt2YPpZtKI2bUB+ov5avh3Dq5yDpbfmeAqjLvm0vVs/FgpZu564/2NKxUOvz5jfRItiXk/DIvYx3LTiNlVNG4N/Id55Vhf/nX/yNxniJgpL2wxIBHTihxanUIdo+MvDRLcntrNkpzd6sAuQJdecwoxu06AhuSfCjG79Jp9xeySuLEDx4l5EzgelvI+xsSfb8DUcL4s/L7Lk8lSrzm2mH86lsslf32YE2FYPq0Xs00+LkNMFHuuF30YJoiXc9rtqcUen9hipuV3rl/aJNe1dadCzC6NEGJOdx90Da4RLq3QcBEgNQTbuubYYuafIubEeRNtbWkpYr5nyjK1GdeXSPbD8jr+Oi6/75IbO8s1Yot5z3hsLl4+sbpEjZgPC0GAmNPeB9fDWpKAa8/U1sOKLea5Mh1Oa3LnPydO/ZQiZu4+x2VqfuvUubyge/24GA+3MW5bO44v5jmP3LCxXvs5asS8lHAQc9r74KUVR8yHodc83/uOLea5Xt5hGE+df6kgdAb+KRZli3nNF9AdE0+33HAT88Ey0RZTzOO9zH1pX1vnatbloCIx2x4dIOa098E1Zqq/Nb/nk+QxxfzA1MHu9Nlcj+lrhLooQcx3TDnWyozge832e/NZFcJ5JKaYufZJ1+LmJejef18Vs0rFzI+BzScdxJz2PrjGt7TOnBMdV+dz47kxxXxgZcCLebzP8AZTgpi5dkq90n71ffHXtP/ey7qw5cbcPERMMc+PIz+9hcg/afjXYcVi5sbB5t8GhJjT3cfDsBRsfmKM27DpKdnn66VjH39fliummLnx5SmntpaJwdC6KEHMPyztam05Hi0xs80LzYnZtkRzroyxxHxrOIc81TvvOP/2W7GYX7NjV3O9tJrFPK0Z9sXl/kLvY2PesA3FbeZ9vl527Jpukv35NWKJ+fGYU0sNi3tkpXJ9DmwsJYiZz8H1nYOeuTfC9hIGJ+adZWXEp4trxBLzgf1yeboOt5SOyvzTM2bVinnHNJCpYfcvbrReMa/F5RGKv49pa89Lxhnop5dN+DWda9/8m+qPWx99GeNYYnad9OLHTMP2RyhBzHx9hr5izMWWX+XBibm31tV5OeOJ2W3VBV8uv61AqxazbaJic5F8ELPffYSy9JhqS+SpXraOveZYYp77Ipi7D34cNqzRlCBm7ndClwTyX2a8sDgx27xwua48hph7M7+yZK4DyPXm/edsKhazrcIvx5ohZr/7CIFi4Lolpk3MvbG/6DBdI4aYO+az5saOuX2aXb+M+FjIi5mPt9tugT71PJaFv65NzLa2v3v2MzHEvLFsP3r5s9w+zb65Ub2Yvxh+neTzBISY/e5jLXT/3z0asU3MY/n4lx2mDYTiiJlbJjffgHnRxN2fI7eY+SGHsFM51qxYWBKzbb/mqdccQ8zc53DX4Ffu+OwfX7mYuYS+bOAQs999+DJtbuTbY1wSc+9QvzHEzK3G4F5q4Seg1td/CWLmYh06lMHPB60byli+7vhzccQ8P9nL7ZLn4qMlVIh5a/he87SRSM1ipkez+Yk4O5fj7D734S7km6DlfEtiHuPC95ppJUSomL8yjcmWH4+WtwDXDmeUIGZ+jDl0YnP+utzOeOPvLIuZ35Fx3EArVMzfmHq21Ytt1UjvGC8VYuYq8fmN1CxmmXXMtKXim2EM8PF0+KbtDa6lrTl9GuxcvdjmEkLFbLsv6hVx8D2jtfswyIt57Vt6a2NsO7jURcy2+6S/DxUzd21bbvxtuV/XQ3zViNl2BM64yxXEHHofD9Zd5Ogw1jgvdMzVC79PxY1l/XGYmNeydivQEsTMt6H1L9BQz5W75poXTF7mBj/W3JlXQWJ2PQDAFdc4qhHz+Bn2zetdBOBKi2ImtpZ9dsdN2/0+36de+De+OEEui9m2yc76xrduf4QSxMzFMqytxNsrYy4ePRM7W264iPmz5bprca1PVWJ+sDZevzHE5WRrU8xcg3Gtz5fXchfzlh3vW7d7ma0BhGJbBsbHQl7M95YY+5wKvlTHLvfmKmZbTvJvB8fZqH8Njw5bp6oS83hD7sGEmNfdh+0LcEz6eMvlXH6ew0XMPtfzYc04cwli7plyrL2n341tfsB+PR8x28o9n6MuYk6TGy4rXNSJ+atHQCHm9ffBzTxPdXrr+Pm+Yu48VpEsiTn2KdCX9+Aag6dYyIt5LAd/9qTvihPbEtDNwhe4j5ht5Z5jScx/MfURKzeW4qZOzD4VBDGvvw9bT8gntmvG/l0n65bEbFuR4rdhFPeCk9+jfyli5nbQm8rTe+QWv8pjeRLMV8y9cZ8vWBKzbYmm30Zi8+W5XxjOUClm114zxBx2H9w+u1MCu0yArRHzzrHXvCTmWGt2Q3bXO79OGWLuF9pP5yDnbuEaLpsi+YrZ1oZ8xRzrzU7+OkudD4Vi5iq1VjHTInx6hAwhxX30xt5DcTsJed1qGZcvXptge8M/qvpO3HG57bs/QiliJnYL8R3Xrr/s9d2a6YRs29PU8nl/XBteisdSTrqImXth7bDipJq1G17xK42uYjnAXsBUYnbpNdci5lBsDTH0PmxjvpTI/11sfOvEbHvcdhHzNuIr1Z8NLwOfrUBLEjM1ZG7b1eeCnbaHHbeB5U8Yca2X83j4i5ng1jW7ipnbtGhNbnwz79ky2PaUib1aiOrl9vwzpiTJK+bxM+0VBDHHuQ/bSpilXnPI+vKlL16bAGLsZ+ByPZ/lgyWJmdhaDqNYLwifeKwT8/GPfulLxSZmfiOndXVhe2uV/x3FYv7LEpSQRkhAzE/Qukx+gf9N/8Ha+NaLeWmfD7uYuR3A1q3Vte3Z0DteozQxT+021uoEyoU/PMq/Vszc757X87yYuZOwiQeH9cc+ZbFNgKoW83iDtt4cxBzvMFbbSyd+gvTbhcs2STX/uQ/MK9xr39gj7g3fa3Z9/bdEMY/X4d/2dOWwYq/qEDEf/+htvWauTlKc6chtGcAdIDvmtXIxj5uax9+YBWI+Z2dsO/xd93+yjS9MzNxBn2Nuzd93inwwlvt3fTGjVDGPcX63as33tLxszY57IWK23T/hu5fy2mEMomfq1paj2cS8PT0SvWT5tcy533MVM7FjrhESbBLC3DV/BHyzdkw5Q7Ft0M3fh39suLoa4RLw2jsn5hrTfI7Mf+YPpoxLS5hcRHA4TYid47o/wvrf5eIyd02fDdufc2fG1RrTpN+SkMc9i9c9/o/xuJotv+vv92xM+a1q98zPh57g0jE5yjloG9kFdFbn7flnrL8ZAGqjZ0j9uz7XjHGftE6ZvvhILE9M+4C/DTpiy1b+1DFIFa/S+D/hEd3YFPsptAAAAABJRU5ErkJggg==</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr">
         <is>
           <t>Healthcare &amp; Medicine</t>
@@ -1221,7 +1233,11 @@
           <t>DKT Myanmar</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAWYAAAErCAYAAADt4CmkAAAACXBIWXMAAA7EAAAOxAGVKw4bAAAjzklEQVR4nO2dTW/cOBKGeciX7QWC+cX+BXuYY4ABAszeDGQyiRO7u9UdDDDX/Cdtl9SK3W0VRYofRRbfw5OdTWw1VSw+TZEUaYwxPaiDjXnX781V311Af7ermPE+3onHFyzTnXJQOmdi5t6+zNwTLwBwpDPX/Q/zH5UcjvcmHV+wzOEoMulcic3e3IjHdQbxAgBH9orFvIeYq0BjDhbaKRAvAHBEY6OAmOtCYw5CzCAIjY0CYq4LjTkIMYMgNDYKiLkuNOYgxAyC0NgoIOa60JiDEDMIQmOjgJjrQmMOQswgCI2NAmKuC405CDGDIDQ2Coi5LjTmIMQMgtDYKCDmutCYgxAzCEJjo4CY60JjDkLMIAiNjQJirguNOQgxgyA0NgqIuS405iDEDILQ2Cgg5rrQmIMQMwhCY6OAmOtCYw5CzCAIjY0CYq4LjTkIMYMgNDYKiLkuNOYgxAyC0NgoIOa60JiDEDMIQmOjgJjrQmMOQswgCI2NAmKuC405CDGDIDQ2Coi5LjTmIMQMgtDYKCDmutCYgxAzCEJjo4CY62Kv8JRsiBkEATEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpOoVi3psb8bjOIF4A4AjErIedeXuU3PVw35ccCqQ7cVCYg4dT3J/fY0rGz7payhH5JAVuQMw66I5Spl6adMyBZL4v9tLlE1WC4x/91yNb8/rI22MP5t0wfkb/O/Zkrgbov8d/uz7+HP37VX9/+v3cZYaY62dzzDfN9Qjc6JbzXT5ZU3JnSL6TdOlR4ub0OBHWY6Hr7E+QrB+ODa5PfC+aG3QLYu6GOkRPGTTYY/57aADvno3X5WsI0/gR9bD/THBvEHO9/Gveq64/4Id6MR//OIr41TCYHqMnHC/w9KUwDn3EulfNDVuzmD8qrzvgj1oxP5o3g4xLEbGNw2kWtoeYLYmqV8ya6w2sQ5WYb435NRFXg5BfcjNMNKKBzyWqTjFrrjOwHhVi/mBMNb1jF6gHfY9GfpGo+sS8U/gyBohD1WK+M+MroDkn8PJVDPX630HMz+IhnW8x2SvqSID4VCvm3WkyTzqAqaEvnQ8QsyoxPw7DbZAy4KlOzLTWswUhn3PjNLQBMZfPN/NGdT2BOFQl5mmfAOmgSVUUrTSBmOvlk/I6AvGoQsy0+L5DQg9fSjuLnDU3+trFTC82aZwLAWkoXsy0V0WrveQ5DkPPeX5JHcRcJj8NXrUGfhQtZq0rLsIr7br/DDFXwfEPlXsUg7QUK+bc+1jUxn7mVW6IuTwgZbCGIsWsWTAx2V3ISnPcahSz5voAaSlKzLemxaVw6zkMr3C/bkIEtYl5a97giQ+sphgxfxikLB+Q2uiOFXgLMRfFj9P2rtIxA/VShJjvlEslNdPWoZpjWIuYv+BYKBABcTH3RueR5zkZtw39DWIW5i/lX44gH+Jixqx1rIrU/fhcupj/CymDiIiKGVKOxwFiFqOHlEFkxMR8wFgc8KBkMWO7ABAbETHfY4ct4EmpYqYTc6RjA/SRXcx0OjSkDHwpUcybo5SxVhmkILuYMXwB1lCamLfY7B4kJKuYOzz2gZWUJOY9huJAYrKJ+Zt5j9etwWpKEfPfBk99ID1ZxNwbzFyDMEoQ8/8gZZCJLGLGm30gFGkxY7N7kJPkYn5EQoMISIq5Rw6DzCQXM3rLIAaSYkYOg9wkFTMSGsRCSsyYsAYSJBPz7wYvkoB4SIi5G/YfwRAGyE8yMWPNMohJbjE/mFfoLQMxkoj5Mx4BQWRyivlfrLkHwiQR867hsWXaO4Gg8fX98amBnhx25m2/PbI5sjv9HW15Ov4cHpVdyCXmr+hUgAKILua/Gkzs/UmwJFzqbfk9MtO+C1ena7QVN78YpxczjjgDpXCILeaWVmKMvePr/tG8iSoGyOElqcV8p7xDsR/y9PXxie1N//1Id4TydnNid8HDKl6rzF3Ki83x3h5m4pSCxyGWiznrntx/NNTjoPucDkFNIYkdBP0i3inFrHnLADp9vk8Yu/OOmb44dgVsBxAk5lbGlump4C5D8LdKE31dzNM1Ds1SpiGyPzMK46DQAYeaxdzC+Nw4jpy/kvanMWjp+5eNfZq47xRvdk9C+ZY5VyHmwsTcwsGqNLknVRHbQSC6v/hspBBzZ94qlvLNkDO581TjHFPVYtbeo+uWZ0mT8+UoEs2P3TZii3mrdKJqYpto/gNiLgaXJNd94jVVTI4xZRdoOZ5moXDEFPO90d2RwIZPcalWzJqHMcblcOKVcMad0gZgI5ZsOvOb6qcOytefgrmpMS+rFbPm3kehS2WGxtfSmHMMMWufoKZ8+CqclxBzIWLeK96siBpxL18BLB+Ui+ayLkJiRfWouadM8fluXovnJMRcjJj1JvujeSsd/EVaGdYIFbPmGE17s0jnotY4Vydmza+xSp8x54P2R/TQ+tAoi+eUNNymMQ+rE/NO9TBGGT0QV0Y56x3rXytm7S/nlDbcBjFng/9Hrb3lQ2HJ3nKjmFgj5u2wtarmmOR93brVHKxOzBoroeCKWES3hPzqZDOsrdcbD6rrroCca8EJhfpg/h9oCzzpgKWphJsqJv3m0L7qwDUOD0oF8RSLG9HtAWxojHtVYtY6vlzTpF8LjcK3Xn4qj0PpOaox9lWJWetj877QnkirjeKpXpYbR688Bq5xkM1BfStgqhHz2CvROdN9H+k0EplGoVdKLkLSfP8ECeK2gDyz1wHEnIm54L8VD1YKSu+NtCympbrRPL4+3f+mgBxbzkGIORNzjUBf8AuuAI9GoVdONjHTvsNan+Cme38s4HVrtxzU54ZCvfDyL7WOL3eVvVTyslHorBeCE/NO+ZazRKqzJdPkIMScifO/GHc109cQ6J6+mffSwQ5sFG2JeX/sRWrtJDzPyxLXK/M5CDFn4vwv9C6Tkz+hJLxR6JXUpZhpvFVjB2GOmp7kIOZsnP+F1kmW2if+xkahs24u6+ez8nu9hMRQ2qvXfA5CzJloo/HvKl6/rL1uiEnMvxu9cxz2+6+j1wwxi4lZ5+PjpuL1y091o1dYk5g136ONrpKNtQ4Qcy6e/g+dfScdpBSUtnXiWjRLa9wMXu/9ubCtYA8XiFlAzDu1GxcVGXiIGZxRwwQ1xCwgZq0TfzXNetuAmHVDTw3fCx9yg5gFxKy14de0gB9ibpuSjpGaQ+NbwcWLWets+LbwXgjEDCb2wwb5v4nnGsQszvgfvdG8IqP8SRWIGUyUPPQGMWcWM72uLB2gFNCXzZ18kCFm4JGz18XmLMScWcw7tVt9lj/TDTGDS0rtNeMFk8xi1vhNWHDQIWZgpdRJQIg5s5i1ji8XGnSIGVih9vhQ4B7NEHNmMR8KCFCaBC8y6BAzWKTE4QyIObOYtTZ6iBnUSokT1xBzdjHrHMrYlRl0iBk4UVrHAmLOKOY71WIu73EQYgau0GvaPwvIPYhZSMzSwUnFo4J9mCHmtilpL3GNq7eKFTOd0CsdnFR8L3BmG2IGPpQ0nAExZxSz1nP+iG/yAYaYQTDbQobkIOasYtYX7Im/5AMMMYNgSuk1Q8wZxay5wX+UDzDEDIKhScD7InJQ3yKBYsWs8VuQoCTq5QMMMYMolPDCCcScUcxaG/xB0QZGmusJuEH1/1E8ByHmbGLW22MuMuAQM1iN9OZGEHNWMets8BAz0Ib0NrYQc0Yxa23wEDPQSCd4Ig/EnFHMeocyMMYM9CE5nAExZxSzxvffCYgZaIQmtekoOIkc7CDmnGLWF2wCYgZakRqmg5gh5gjJCzEDnVAu/AExRwFiRsAhZhANiS1tIeaMYj4oHWMuNOAQM4iCxHCGxqW1hXpC7+RfoQGHmEE0cp/QAzFnFPNBYbALDjjEDKKRex4FYs4oZq0NvtCAQ8wgGiTmnXkDMQdQqCf0jjHjzT/QAjnFojEHixWzxm/BMeDY9hPoh8RyhxwMip90254Vs9bJP3rM+10+wGgUIDldpgNbNeZgsWLuFJ/5l6sngUYBJKFOyC1ycBXFinmrtMdMPAruxIVGAXKS48BWjTlYrJg1H8a6Na+lA4xGAbKQQzAac7BYMdNOVdLBScUePWbQEI+JOyIaFwoUK+afRvN+Gf+RDjDEnBGKET3Stxqr1C+caBRzoZud6W70JZwsDDHngXo+D78Eond4zh6Dm/4LxOxF4WLW2WOGmNuAhPR8ovezMcPfSZdLgpQvVmnMwcLFrC/gqZMUYi4DalibmbmEVuOVcv2+xpgWLWaNjyjEAT1m1dDwxTdmr4hHxevzl9gleuFEYw4WLmadY3KFBh2NIgIk5W5hFUK7MUuT9xp3oizUEZOY34oHKAWFLoWBmIMb07XT0rBdw73mFK9pQ8yZxfyoVMwUdC2vZUPMIyQH12OVfpp2JwFTLBWFmDOLuVecwFre/oOYRynvPXuCrcaNhNMhB53iJN22WTEb1WLWMQGosVH4NqDdijc5vyrO7SViLxfVmIMViFnnBKCWcWaNjcK9Dm+OX7DrT+rQurWtS+7/RA5aKV7MWpMXYq6b8ZE8rOd3b16rfYlqOX7xes0ac7B4MW+UzmBreclEY6NwaTT/mDiTWBonrlygdxR65KA1x6TbtlXMH4zOsTgtKzM0Ngob4/BFvCVfWl+icmsDcXZZ1JiDxYvZKBUzsWbSqDQ0NgqOUcrxn3Ra7TXHGs44FHAv8WNTgZi19ipijrNBzOkbSqrNpzQfCmGDvui+B0yeQszCYtb6ptShzOBDzDOk3BHwrqE4XhJjrgViFhIz7WcrHagUjNtCigcbYl6gyzBRq/WpcIn9sLfIb4Fi1he7KsSsNfhE7Xszaxdzrvp5NHr3H08dY41uKHQ5bRvBJ2pfNqdZzLnrRnMsl+IcskJJoxsK9cLLv9wqnSChXtJ9hAkQKTTLJL+Ydc6luBDSa9aYg9WI+V/zXu2jXs2rMzQ2CsnG0SnN8SVCxvE15mA1QxlaK4Cg+/pTPuhoFDP1kjueXaO9ZpoIf1i546LGHKR4fCigfTuJWfPMda2TgBobxYSEmH83mAREDo4UuDXw/D/Q6RDSwUoFfUP+Vz7waBTPyLFMrrWY2li7TYHWeBXYWWuvEsaKSHNYZSq+GZ0z4k/1ISPmL6bdXvOapxStOVjgODP/j1oPaJ2S8pN88J24M7qHlggpMWvPcxv05Oi7V7NWMdOXc2E+4P9xZ16JByx1ZRRQAVb+p7gxPEdSzDS+qHXzriV2nk+OmnOxsOEM+w9oHs5Ye1RRLsZli3rjf14Xso+SrcQ5NO6an9zGQ36Lec9hKWF1P+ZRT+mrfCXMNIC2ZCEt5o3yPLfhcyamZjETJOdCfGD/AdoqUPvkCFXGrXxF/II2h9ce80ukxUzj+Jof02PFXruYp3gU0HNe/qEWem4kwl5YyL0Z30ZrcbxTWsxjnrfZax6H9Nxi1MqXF8WEcjLliycLyxWXL9DCt+RYGdfDSwcSUugaSnou9tJipi0xW+iEzMffbTijtfgcToJ+CMythyG/3g7XOgzcLC0+WL7onw1VSIw9a33ozbhcq2UpT3GXFnOL4nke/4+ID8skaPoCozH5R/PmRW+a2jKNT9PLed0wHHl1+p35J+BgMbdWIVMFpD7AdfwGbW/Ygou5tJSJzbFOWhxKIlyWLLbkgeWcvfk15GETsO33g8VMk4CtJew4CfDOexG+DZL99vRNKn1/JVGKmFuWj8u6/lbH4QXi7Z6wrT5uH4bDQW+GgzzX9qI78+o0ZNHWl5srJYl5e+w1S8dDim5hXX+rDkhBNDG3vLn4UzCvT2NHV0M8SNbfzPvhdc6/zDjIvzGvh17x7vSIg2R2i6u0kCf6hgW0tGcEeszxiCbmsWLaTFiQlpLETLSyEukSeqLbWnrNaP/xiCrmXcOPeSAdpYn5Y8MSstVFq19YaeIcUcz41gQpKE3MYyekzcd224GtO7T9iHGOLOYdxppBZEoU89/GNDtZy71wslF8gEb+GEcW89hrbrM3AdJQopiNaXcSkKuPj6bdgwXixziBmDcNbG4E8lGqmLXvSW6vk/mNfFr9sorNIYWYx14zKgjEoVQxt5znXI+u1XjEJpmYH0y7Y3AgLiWL+VBAfCSgtv1tptcMMceLbxIxE/8UcIOgfkoW861pd1x1rl46TP5HIamY8Q0KYlCymEcZtZnjNJ5MR5w9jwVtIi9dLg0kF/Mj5AwCKV3MLZ2/eMlh5sDWVp8g4sY1sZjHHgUeb8B6ShezabjzMXe6D+aWwskiZnyLghBqEHPLS0S7ixdO8B5DONnE/EfDvQoQRg1iJrpGxXxZPy0fXhuLbGImHszrZnsVYD21iLnlTby6Y9s+/5JCrzmErGIeK+wd5Ay8qEXMxz+a7SlevnDS8luRMcguZnybpuRG5XBRLWImWh1fJTF/eRELfbmYCxEx96bdtZ+poIYxnsCrTww1iZnOgGy313xeT5uGh3ZCERHzlMD4Ro3HdIoxxCxPq71mksnvL2KBNr42liJiJr6i4qLwfPPyg0Ip1Cbmz6bdtby7ixdOvmPCfxWiYibGzY4g57WQtB6exRM95jJotcMxt+ucxpxMjbiYiUfzttlEDoFi9tjAMqUaxdzq0VPE9qLXPK5rRq/ZhyLEPMkZPWe/inuc2acAYi6HVjsbc/X1gM6XF8WImfhkMKzhAj0ubphj5CHmcmj1/MsxP+dy8y16zo4UJWbiL9NuT8MFis2BkTLEXBbjyqM2RcQd2EovmEHOyxQnZuIj5DwLxeRywxiIuWxaXa9PT74fmJjs8PavQ/wKFPNTUuPbdYLktLX0lCHmMmn7CZCvN+pRY9iSp2gxE1t8uw4JfOcYL4i5PFoVEN13b81VrHHmY1e4mIlpwX5rvefxfv2kBDGXx0PTezXbn/K+Giylm6MKMU9shwRvo/dB98mtvLCh8XXg2sU81kub8uEmAS/BuPM5VYmZuDPjmJ1WQdN97RYeAW2gx1wmXaMb+pBs748dKpcYPTTU8VqiOjFPfDLjjLeWx6DDsGXn1fGefguKC/bKKJPjH81Kx7f+NLXrtVQr5on9KeFrnWA5DL3/qxd72a5F4/IsDWImWn1N+3Cxn4sLP820KktfPrvFrHIxT/xtxt5iLd+0h2FN8rthYjN2HP4174dXYDm+MGwW2B0fNX34fqSLwLcC8isGxz+GuDw0Bt2z66qiS6ahy1raNcRs4ftpw/jSHh0PpxdEaAlgX0CcAKiJzbC8Tu/65/3pBKLxRTLrU6J8ZYSyG3pdV6chg7wV+jzQdFDnzwLiAYAGtsNk6vWv9lXLio4nJ1wN8qXhrd3pSfbW/f7lKyAm9FhEJ3XvTt9IMVd3jJN3E1dRx40BAHZoPXQ37GB3dSbrnEMg4+dd/+KpLG+H5YCdMauHdC6QD3hq+lOwOvNq+PbqziqW/v/NRUVf//qZSfAk+z8KuBcAwDm3hrYUHt8ypJ4pzetsT73V/bMn6cthhO6iNz71cA+//ED/+27YUOzH8PPRpOuCfGABAACcIV4AAAAA54gXAAAAwDniBQAAAHCOeAEAAACcI14AAAAA54gXAAAAwDniBQAAAHCOeAEAAACcI14AAAAA54gXAAAAwDniBQAAAHCOeAEAAACcI14AAAAA54gXAAAAwDniBQAAAHCOeAEAAImgg3tpE3k6aJcOvM240TsIY/yP7bDz//UL6CQA2wU2w6GoL3+PThLwKUg3HMvi/tn7mZ+Px2+zn/mP+U+Cz3pnjcsXpl5s0GkM3a/zxq6PDfPd6tNXdqfrXPLocY3x9Ji5sr4OTuCOKd9uIW9fXsc/zq5smbbAtbmHgLjcDXX29lceXJ6TN53iQXHbeLbRl7kx3wYfPK5Bp73Pxyw8N/ZMfYTeN0H3+Hi8ziURT3ufEvPd7BlXdCO2C/zDno937XPw4OypuHvLZ6c8dJVLLErm2J91WIjvZjjWJs55hYcVCc/Fee8hvk9H5nPL/qW0xGYo3/x5bwtHw8/k33z+x6BjYtUxsd2tiMvtKT99TpeeJH2/Mv57pj3Y2u0l35jcWOoQLvHdvLG2hZBrj/myrj17MCVJXDH7JhjEzMknjpjPG6N7j4EX882xUb13ukYqMXM5+1SP7vdZs5g/Wa7llhPUi/QXCidmEp9rrzmVmG1+8MldPl/WtWcP7EkeImYKTu98oxDzHLHFPDWc7bFHEZrgB8fGk07M9hxYyt3z/KtTzJ8itYXDMPzlJxVOzD6xlxCzb4zn82Vde/ZgSpL4Yh4D7BYAiHmeFGKeGqLLRFCMnkcKMf8ccsZ+bL3PI3WNYr6L3A72nnK2iZmu5TJEkkLM95FzYz5f1rVnD6YkSSNmCoCLACDmeVKJeYzvsgCW4sxJ5zkpxGyTwnM5bJwbWn1idonBU57ZRfUUM/fJu6XPd5F8CjG7tFPKjb9XXn/Ml3Xt2YPpZtKI2bUB+ov5avh3Dq5yDpbfmeAqjLvm0vVs/FgpZu564/2NKxUOvz5jfRItiXk/DIvYx3LTiNlVNG4N/Id55Vhf/nX/yNxniJgpL2wxIBHTihxanUIdo+MvDRLcntrNkpzd6sAuQJdecwoxu06AhuSfCjG79Jp9xeySuLEDx4l5EzgelvI+xsSfb8DUcL4s/L7Lk8lSrzm2mH86lsslf32YE2FYPq0Xs00+LkNMFHuuF30YJoiXc9rtqcUen9hipuV3rl/aJNe1dadCzC6NEGJOdx90Da4RLq3QcBEgNQTbuubYYuafIubEeRNtbWkpYr5nyjK1GdeXSPbD8jr+Oi6/75IbO8s1Yot5z3hsLl4+sbpEjZgPC0GAmNPeB9fDWpKAa8/U1sOKLea5Mh1Oa3LnPydO/ZQiZu4+x2VqfuvUubyge/24GA+3MW5bO44v5jmP3LCxXvs5asS8lHAQc9r74KUVR8yHodc83/uOLea5Xt5hGE+df6kgdAb+KRZli3nNF9AdE0+33HAT88Ey0RZTzOO9zH1pX1vnatbloCIx2x4dIOa098E1Zqq/Nb/nk+QxxfzA1MHu9Nlcj+lrhLooQcx3TDnWyozge832e/NZFcJ5JKaYufZJ1+LmJejef18Vs0rFzI+BzScdxJz2PrjGt7TOnBMdV+dz47kxxXxgZcCLebzP8AZTgpi5dkq90n71ffHXtP/ey7qw5cbcPERMMc+PIz+9hcg/afjXYcVi5sbB5t8GhJjT3cfDsBRsfmKM27DpKdnn66VjH39fliummLnx5SmntpaJwdC6KEHMPyztam05Hi0xs80LzYnZtkRzroyxxHxrOIc81TvvOP/2W7GYX7NjV3O9tJrFPK0Z9sXl/kLvY2PesA3FbeZ9vl527Jpukv35NWKJ+fGYU0sNi3tkpXJ9DmwsJYiZz8H1nYOeuTfC9hIGJ+adZWXEp4trxBLzgf1yeboOt5SOyvzTM2bVinnHNJCpYfcvbrReMa/F5RGKv49pa89Lxhnop5dN+DWda9/8m+qPWx99GeNYYnad9OLHTMP2RyhBzHx9hr5izMWWX+XBibm31tV5OeOJ2W3VBV8uv61AqxazbaJic5F8ELPffYSy9JhqS+SpXraOveZYYp77Ipi7D34cNqzRlCBm7ndClwTyX2a8sDgx27xwua48hph7M7+yZK4DyPXm/edsKhazrcIvx5ohZr/7CIFi4Lolpk3MvbG/6DBdI4aYO+az5saOuX2aXb+M+FjIi5mPt9tugT71PJaFv65NzLa2v3v2MzHEvLFsP3r5s9w+zb65Ub2Yvxh+neTzBISY/e5jLXT/3z0asU3MY/n4lx2mDYTiiJlbJjffgHnRxN2fI7eY+SGHsFM51qxYWBKzbb/mqdccQ8zc53DX4Ffu+OwfX7mYuYS+bOAQs999+DJtbuTbY1wSc+9QvzHEzK3G4F5q4Seg1td/CWLmYh06lMHPB60byli+7vhzccQ8P9nL7ZLn4qMlVIh5a/he87SRSM1ipkez+Yk4O5fj7D734S7km6DlfEtiHuPC95ppJUSomL8yjcmWH4+WtwDXDmeUIGZ+jDl0YnP+utzOeOPvLIuZ35Fx3EArVMzfmHq21Ytt1UjvGC8VYuYq8fmN1CxmmXXMtKXim2EM8PF0+KbtDa6lrTl9GuxcvdjmEkLFbLsv6hVx8D2jtfswyIt57Vt6a2NsO7jURcy2+6S/DxUzd21bbvxtuV/XQ3zViNl2BM64yxXEHHofD9Zd5Ogw1jgvdMzVC79PxY1l/XGYmNeydivQEsTMt6H1L9BQz5W75poXTF7mBj/W3JlXQWJ2PQDAFdc4qhHz+Bn2zetdBOBKi2ImtpZ9dsdN2/0+36de+De+OEEui9m2yc76xrduf4QSxMzFMqytxNsrYy4ePRM7W264iPmz5bprca1PVWJ+sDZevzHE5WRrU8xcg3Gtz5fXchfzlh3vW7d7ma0BhGJbBsbHQl7M95YY+5wKvlTHLvfmKmZbTvJvB8fZqH8Njw5bp6oS83hD7sGEmNfdh+0LcEz6eMvlXH6ew0XMPtfzYc04cwli7plyrL2n341tfsB+PR8x28o9n6MuYk6TGy4rXNSJ+atHQCHm9ffBzTxPdXrr+Pm+Yu48VpEsiTn2KdCX9+Aag6dYyIt5LAd/9qTvihPbEtDNwhe4j5ht5Z5jScx/MfURKzeW4qZOzD4VBDGvvw9bT8gntmvG/l0n65bEbFuR4rdhFPeCk9+jfyli5nbQm8rTe+QWv8pjeRLMV8y9cZ8vWBKzbYmm30Zi8+W5XxjOUClm114zxBx2H9w+u1MCu0yArRHzzrHXvCTmWGt2Q3bXO79OGWLuF9pP5yDnbuEaLpsi+YrZ1oZ8xRzrzU7+OkudD4Vi5iq1VjHTInx6hAwhxX30xt5DcTsJed1qGZcvXptge8M/qvpO3HG57bs/QiliJnYL8R3Xrr/s9d2a6YRs29PU8nl/XBteisdSTrqImXth7bDipJq1G17xK42uYjnAXsBUYnbpNdci5lBsDTH0PmxjvpTI/11sfOvEbHvcdhHzNuIr1Z8NLwOfrUBLEjM1ZG7b1eeCnbaHHbeB5U8Yca2X83j4i5ng1jW7ipnbtGhNbnwz79ky2PaUib1aiOrl9vwzpiTJK+bxM+0VBDHHuQ/bSpilXnPI+vKlL16bAGLsZ+ByPZ/lgyWJmdhaDqNYLwifeKwT8/GPfulLxSZmfiOndXVhe2uV/x3FYv7LEpSQRkhAzE/Qukx+gf9N/8Ha+NaLeWmfD7uYuR3A1q3Vte3Z0DteozQxT+021uoEyoU/PMq/Vszc757X87yYuZOwiQeH9cc+ZbFNgKoW83iDtt4cxBzvMFbbSyd+gvTbhcs2STX/uQ/MK9xr39gj7g3fa3Z9/bdEMY/X4d/2dOWwYq/qEDEf/+htvWauTlKc6chtGcAdIDvmtXIxj5uax9+YBWI+Z2dsO/xd93+yjS9MzNxBn2Nuzd93inwwlvt3fTGjVDGPcX63as33tLxszY57IWK23T/hu5fy2mEMomfq1paj2cS8PT0SvWT5tcy533MVM7FjrhESbBLC3DV/BHyzdkw5Q7Ft0M3fh39suLoa4RLw2jsn5hrTfI7Mf+YPpoxLS5hcRHA4TYid47o/wvrf5eIyd02fDdufc2fG1RrTpN+SkMc9i9c9/o/xuJotv+vv92xM+a1q98zPh57g0jE5yjloG9kFdFbn7flnrL8ZAGqjZ0j9uz7XjHGftE6ZvvhILE9M+4C/DTpiy1b+1DFIFa/S+D/hEd3YFPsptAAAAABJRU5ErkJggg==</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr">
         <is>
           <t>Healthcare &amp; Medicine</t>
@@ -1309,7 +1325,11 @@
           <t>DKT Myanmar</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAWYAAAErCAYAAADt4CmkAAAACXBIWXMAAA7EAAAOxAGVKw4bAAAjzklEQVR4nO2dTW/cOBKGeciX7QWC+cX+BXuYY4ABAszeDGQyiRO7u9UdDDDX/Cdtl9SK3W0VRYofRRbfw5OdTWw1VSw+TZEUaYwxPaiDjXnX781V311Af7ermPE+3onHFyzTnXJQOmdi5t6+zNwTLwBwpDPX/Q/zH5UcjvcmHV+wzOEoMulcic3e3IjHdQbxAgBH9orFvIeYq0BjDhbaKRAvAHBEY6OAmOtCYw5CzCAIjY0CYq4LjTkIMYMgNDYKiLkuNOYgxAyC0NgoIOa60JiDEDMIQmOjgJjrQmMOQswgCI2NAmKuC405CDGDIDQ2Coi5LjTmIMQMgtDYKCDmutCYgxAzCEJjo4CY60JjDkLMIAiNjQJirguNOQgxgyA0NgqIuS405iDEDILQ2Cgg5rrQmIMQMwhCY6OAmOtCYw5CzCAIjY0CYq4LjTkIMYMgNDYKiLkuNOYgxAyC0NgoIOa60JiDEDMIQmOjgJjrQmMOQswgCI2NAmKuC405CDGDIDQ2Coi5LjTmIMQMgtDYKCDmutCYgxAzCEJjo4CY62Kv8JRsiBkEATEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpIOZsiBcAOAIxA2kg5myIFwA4AjEDaSDmbIgXADgCMQNpOoVi3psb8bjOIF4A4AjErIedeXuU3PVw35ccCqQ7cVCYg4dT3J/fY0rGz7payhH5JAVuQMw66I5Spl6adMyBZL4v9tLlE1WC4x/91yNb8/rI22MP5t0wfkb/O/Zkrgbov8d/uz7+HP37VX9/+v3cZYaY62dzzDfN9Qjc6JbzXT5ZU3JnSL6TdOlR4ub0OBHWY6Hr7E+QrB+ODa5PfC+aG3QLYu6GOkRPGTTYY/57aADvno3X5WsI0/gR9bD/THBvEHO9/Gveq64/4Id6MR//OIr41TCYHqMnHC/w9KUwDn3EulfNDVuzmD8qrzvgj1oxP5o3g4xLEbGNw2kWtoeYLYmqV8ya6w2sQ5WYb435NRFXg5BfcjNMNKKBzyWqTjFrrjOwHhVi/mBMNb1jF6gHfY9GfpGo+sS8U/gyBohD1WK+M+MroDkn8PJVDPX630HMz+IhnW8x2SvqSID4VCvm3WkyTzqAqaEvnQ8QsyoxPw7DbZAy4KlOzLTWswUhn3PjNLQBMZfPN/NGdT2BOFQl5mmfAOmgSVUUrTSBmOvlk/I6AvGoQsy0+L5DQg9fSjuLnDU3+trFTC82aZwLAWkoXsy0V0WrveQ5DkPPeX5JHcRcJj8NXrUGfhQtZq0rLsIr7br/DDFXwfEPlXsUg7QUK+bc+1jUxn7mVW6IuTwgZbCGIsWsWTAx2V3ISnPcahSz5voAaSlKzLemxaVw6zkMr3C/bkIEtYl5a97giQ+sphgxfxikLB+Q2uiOFXgLMRfFj9P2rtIxA/VShJjvlEslNdPWoZpjWIuYv+BYKBABcTH3RueR5zkZtw39DWIW5i/lX44gH+Jixqx1rIrU/fhcupj/CymDiIiKGVKOxwFiFqOHlEFkxMR8wFgc8KBkMWO7ABAbETHfY4ct4EmpYqYTc6RjA/SRXcx0OjSkDHwpUcybo5SxVhmkILuYMXwB1lCamLfY7B4kJKuYOzz2gZWUJOY9huJAYrKJ+Zt5j9etwWpKEfPfBk99ID1ZxNwbzFyDMEoQ8/8gZZCJLGLGm30gFGkxY7N7kJPkYn5EQoMISIq5Rw6DzCQXM3rLIAaSYkYOg9wkFTMSGsRCSsyYsAYSJBPz7wYvkoB4SIi5G/YfwRAGyE8yMWPNMohJbjE/mFfoLQMxkoj5Mx4BQWRyivlfrLkHwiQR867hsWXaO4Gg8fX98amBnhx25m2/PbI5sjv9HW15Ov4cHpVdyCXmr+hUgAKILua/Gkzs/UmwJFzqbfk9MtO+C1ena7QVN78YpxczjjgDpXCILeaWVmKMvePr/tG8iSoGyOElqcV8p7xDsR/y9PXxie1N//1Id4TydnNid8HDKl6rzF3Ki83x3h5m4pSCxyGWiznrntx/NNTjoPucDkFNIYkdBP0i3inFrHnLADp9vk8Yu/OOmb44dgVsBxAk5lbGlump4C5D8LdKE31dzNM1Ds1SpiGyPzMK46DQAYeaxdzC+Nw4jpy/kvanMWjp+5eNfZq47xRvdk9C+ZY5VyHmwsTcwsGqNLknVRHbQSC6v/hspBBzZ94qlvLNkDO581TjHFPVYtbeo+uWZ0mT8+UoEs2P3TZii3mrdKJqYpto/gNiLgaXJNd94jVVTI4xZRdoOZ5moXDEFPO90d2RwIZPcalWzJqHMcblcOKVcMad0gZgI5ZsOvOb6qcOytefgrmpMS+rFbPm3kehS2WGxtfSmHMMMWufoKZ8+CqclxBzIWLeK96siBpxL18BLB+Ui+ayLkJiRfWouadM8fluXovnJMRcjJj1JvujeSsd/EVaGdYIFbPmGE17s0jnotY4Vydmza+xSp8x54P2R/TQ+tAoi+eUNNymMQ+rE/NO9TBGGT0QV0Y56x3rXytm7S/nlDbcBjFng/9Hrb3lQ2HJ3nKjmFgj5u2wtarmmOR93brVHKxOzBoroeCKWES3hPzqZDOsrdcbD6rrroCca8EJhfpg/h9oCzzpgKWphJsqJv3m0L7qwDUOD0oF8RSLG9HtAWxojHtVYtY6vlzTpF8LjcK3Xn4qj0PpOaox9lWJWetj877QnkirjeKpXpYbR688Bq5xkM1BfStgqhHz2CvROdN9H+k0EplGoVdKLkLSfP8ECeK2gDyz1wHEnIm54L8VD1YKSu+NtCympbrRPL4+3f+mgBxbzkGIORNzjUBf8AuuAI9GoVdONjHTvsNan+Cme38s4HVrtxzU54ZCvfDyL7WOL3eVvVTyslHorBeCE/NO+ZazRKqzJdPkIMScifO/GHc109cQ6J6+mffSwQ5sFG2JeX/sRWrtJDzPyxLXK/M5CDFn4vwv9C6Tkz+hJLxR6JXUpZhpvFVjB2GOmp7kIOZsnP+F1kmW2if+xkahs24u6+ez8nu9hMRQ2qvXfA5CzJloo/HvKl6/rL1uiEnMvxu9cxz2+6+j1wwxi4lZ5+PjpuL1y091o1dYk5g136ONrpKNtQ4Qcy6e/g+dfScdpBSUtnXiWjRLa9wMXu/9ubCtYA8XiFlAzDu1GxcVGXiIGZxRwwQ1xCwgZq0TfzXNetuAmHVDTw3fCx9yg5gFxKy14de0gB9ibpuSjpGaQ+NbwcWLWets+LbwXgjEDCb2wwb5v4nnGsQszvgfvdG8IqP8SRWIGUyUPPQGMWcWM72uLB2gFNCXzZ18kCFm4JGz18XmLMScWcw7tVt9lj/TDTGDS0rtNeMFk8xi1vhNWHDQIWZgpdRJQIg5s5i1ji8XGnSIGVih9vhQ4B7NEHNmMR8KCFCaBC8y6BAzWKTE4QyIObOYtTZ6iBnUSokT1xBzdjHrHMrYlRl0iBk4UVrHAmLOKOY71WIu73EQYgau0GvaPwvIPYhZSMzSwUnFo4J9mCHmtilpL3GNq7eKFTOd0CsdnFR8L3BmG2IGPpQ0nAExZxSz1nP+iG/yAYaYQTDbQobkIOasYtYX7Im/5AMMMYNgSuk1Q8wZxay5wX+UDzDEDIKhScD7InJQ3yKBYsWs8VuQoCTq5QMMMYMolPDCCcScUcxaG/xB0QZGmusJuEH1/1E8ByHmbGLW22MuMuAQM1iN9OZGEHNWMets8BAz0Ib0NrYQc0Yxa23wEDPQSCd4Ig/EnFHMeocyMMYM9CE5nAExZxSzxvffCYgZaIQmtekoOIkc7CDmnGLWF2wCYgZakRqmg5gh5gjJCzEDnVAu/AExRwFiRsAhZhANiS1tIeaMYj4oHWMuNOAQM4iCxHCGxqW1hXpC7+RfoQGHmEE0cp/QAzFnFPNBYbALDjjEDKKRex4FYs4oZq0NvtCAQ8wgGiTmnXkDMQdQqCf0jjHjzT/QAjnFojEHixWzxm/BMeDY9hPoh8RyhxwMip90254Vs9bJP3rM+10+wGgUIDldpgNbNeZgsWLuFJ/5l6sngUYBJKFOyC1ycBXFinmrtMdMPAruxIVGAXKS48BWjTlYrJg1H8a6Na+lA4xGAbKQQzAac7BYMdNOVdLBScUePWbQEI+JOyIaFwoUK+afRvN+Gf+RDjDEnBGKET3Stxqr1C+caBRzoZud6W70JZwsDDHngXo+D78Eond4zh6Dm/4LxOxF4WLW2WOGmNuAhPR8ovezMcPfSZdLgpQvVmnMwcLFrC/gqZMUYi4DalibmbmEVuOVcv2+xpgWLWaNjyjEAT1m1dDwxTdmr4hHxevzl9gleuFEYw4WLmadY3KFBh2NIgIk5W5hFUK7MUuT9xp3oizUEZOY34oHKAWFLoWBmIMb07XT0rBdw73mFK9pQ8yZxfyoVMwUdC2vZUPMIyQH12OVfpp2JwFTLBWFmDOLuVecwFre/oOYRynvPXuCrcaNhNMhB53iJN22WTEb1WLWMQGosVH4NqDdijc5vyrO7SViLxfVmIMViFnnBKCWcWaNjcK9Dm+OX7DrT+rQurWtS+7/RA5aKV7MWpMXYq6b8ZE8rOd3b16rfYlqOX7xes0ac7B4MW+UzmBreclEY6NwaTT/mDiTWBonrlygdxR65KA1x6TbtlXMH4zOsTgtKzM0Ngob4/BFvCVfWl+icmsDcXZZ1JiDxYvZKBUzsWbSqDQ0NgqOUcrxn3Ra7TXHGs44FHAv8WNTgZi19ipijrNBzOkbSqrNpzQfCmGDvui+B0yeQszCYtb6ptShzOBDzDOk3BHwrqE4XhJjrgViFhIz7WcrHagUjNtCigcbYl6gyzBRq/WpcIn9sLfIb4Fi1he7KsSsNfhE7Xszaxdzrvp5NHr3H08dY41uKHQ5bRvBJ2pfNqdZzLnrRnMsl+IcskJJoxsK9cLLv9wqnSChXtJ9hAkQKTTLJL+Ydc6luBDSa9aYg9WI+V/zXu2jXs2rMzQ2CsnG0SnN8SVCxvE15mA1QxlaK4Cg+/pTPuhoFDP1kjueXaO9ZpoIf1i546LGHKR4fCigfTuJWfPMda2TgBobxYSEmH83mAREDo4UuDXw/D/Q6RDSwUoFfUP+Vz7waBTPyLFMrrWY2li7TYHWeBXYWWuvEsaKSHNYZSq+GZ0z4k/1ISPmL6bdXvOapxStOVjgODP/j1oPaJ2S8pN88J24M7qHlggpMWvPcxv05Oi7V7NWMdOXc2E+4P9xZ16JByx1ZRRQAVb+p7gxPEdSzDS+qHXzriV2nk+OmnOxsOEM+w9oHs5Ye1RRLsZli3rjf14Xso+SrcQ5NO6an9zGQ36Lec9hKWF1P+ZRT+mrfCXMNIC2ZCEt5o3yPLfhcyamZjETJOdCfGD/AdoqUPvkCFXGrXxF/II2h9ce80ukxUzj+Jof02PFXruYp3gU0HNe/qEWem4kwl5YyL0Z30ZrcbxTWsxjnrfZax6H9Nxi1MqXF8WEcjLliycLyxWXL9DCt+RYGdfDSwcSUugaSnou9tJipi0xW+iEzMffbTijtfgcToJ+CMythyG/3g7XOgzcLC0+WL7onw1VSIw9a33ozbhcq2UpT3GXFnOL4nke/4+ID8skaPoCozH5R/PmRW+a2jKNT9PLed0wHHl1+p35J+BgMbdWIVMFpD7AdfwGbW/Ygou5tJSJzbFOWhxKIlyWLLbkgeWcvfk15GETsO33g8VMk4CtJew4CfDOexG+DZL99vRNKn1/JVGKmFuWj8u6/lbH4QXi7Z6wrT5uH4bDQW+GgzzX9qI78+o0ZNHWl5srJYl5e+w1S8dDim5hXX+rDkhBNDG3vLn4UzCvT2NHV0M8SNbfzPvhdc6/zDjIvzGvh17x7vSIg2R2i6u0kCf6hgW0tGcEeszxiCbmsWLaTFiQlpLETLSyEukSeqLbWnrNaP/xiCrmXcOPeSAdpYn5Y8MSstVFq19YaeIcUcz41gQpKE3MYyekzcd224GtO7T9iHGOLOYdxppBZEoU89/GNDtZy71wslF8gEb+GEcW89hrbrM3AdJQopiNaXcSkKuPj6bdgwXixziBmDcNbG4E8lGqmLXvSW6vk/mNfFr9sorNIYWYx14zKgjEoVQxt5znXI+u1XjEJpmYH0y7Y3AgLiWL+VBAfCSgtv1tptcMMceLbxIxE/8UcIOgfkoW861pd1x1rl46TP5HIamY8Q0KYlCymEcZtZnjNJ5MR5w9jwVtIi9dLg0kF/Mj5AwCKV3MLZ2/eMlh5sDWVp8g4sY1sZjHHgUeb8B6ShezabjzMXe6D+aWwskiZnyLghBqEHPLS0S7ixdO8B5DONnE/EfDvQoQRg1iJrpGxXxZPy0fXhuLbGImHszrZnsVYD21iLnlTby6Y9s+/5JCrzmErGIeK+wd5Ay8qEXMxz+a7SlevnDS8luRMcguZnybpuRG5XBRLWImWh1fJTF/eRELfbmYCxEx96bdtZ+poIYxnsCrTww1iZnOgGy313xeT5uGh3ZCERHzlMD4Ro3HdIoxxCxPq71mksnvL2KBNr42liJiJr6i4qLwfPPyg0Ip1Cbmz6bdtby7ixdOvmPCfxWiYibGzY4g57WQtB6exRM95jJotcMxt+ucxpxMjbiYiUfzttlEDoFi9tjAMqUaxdzq0VPE9qLXPK5rRq/ZhyLEPMkZPWe/inuc2acAYi6HVjsbc/X1gM6XF8WImfhkMKzhAj0ubphj5CHmcmj1/MsxP+dy8y16zo4UJWbiL9NuT8MFis2BkTLEXBbjyqM2RcQd2EovmEHOyxQnZuIj5DwLxeRywxiIuWxaXa9PT74fmJjs8PavQ/wKFPNTUuPbdYLktLX0lCHmMmn7CZCvN+pRY9iSp2gxE1t8uw4JfOcYL4i5PFoVEN13b81VrHHmY1e4mIlpwX5rvefxfv2kBDGXx0PTezXbn/K+Giylm6MKMU9shwRvo/dB98mtvLCh8XXg2sU81kub8uEmAS/BuPM5VYmZuDPjmJ1WQdN97RYeAW2gx1wmXaMb+pBs748dKpcYPTTU8VqiOjFPfDLjjLeWx6DDsGXn1fGefguKC/bKKJPjH81Kx7f+NLXrtVQr5on9KeFrnWA5DL3/qxd72a5F4/IsDWImWn1N+3Cxn4sLP820KktfPrvFrHIxT/xtxt5iLd+0h2FN8rthYjN2HP4174dXYDm+MGwW2B0fNX34fqSLwLcC8isGxz+GuDw0Bt2z66qiS6ahy1raNcRs4ftpw/jSHh0PpxdEaAlgX0CcAKiJzbC8Tu/65/3pBKLxRTLrU6J8ZYSyG3pdV6chg7wV+jzQdFDnzwLiAYAGtsNk6vWv9lXLio4nJ1wN8qXhrd3pSfbW/f7lKyAm9FhEJ3XvTt9IMVd3jJN3E1dRx40BAHZoPXQ37GB3dSbrnEMg4+dd/+KpLG+H5YCdMauHdC6QD3hq+lOwOvNq+PbqziqW/v/NRUVf//qZSfAk+z8KuBcAwDm3hrYUHt8ypJ4pzetsT73V/bMn6cthhO6iNz71cA+//ED/+27YUOzH8PPRpOuCfGABAACcIV4AAAAA54gXAAAAwDniBQAAAHCOeAEAAACcI14AAAAA54gXAAAAwDniBQAAAHCOeAEAAACcI14AAAAA54gXAAAAwDniBQAAAHCOeAEAAACcI14AAAAA54gXAAAAwDniBQAAAHCOeAEAAImgg3tpE3k6aJcOvM240TsIY/yP7bDz//UL6CQA2wU2w6GoL3+PThLwKUg3HMvi/tn7mZ+Px2+zn/mP+U+Cz3pnjcsXpl5s0GkM3a/zxq6PDfPd6tNXdqfrXPLocY3x9Ji5sr4OTuCOKd9uIW9fXsc/zq5smbbAtbmHgLjcDXX29lceXJ6TN53iQXHbeLbRl7kx3wYfPK5Bp73Pxyw8N/ZMfYTeN0H3+Hi8ziURT3ufEvPd7BlXdCO2C/zDno937XPw4OypuHvLZ6c8dJVLLErm2J91WIjvZjjWJs55hYcVCc/Fee8hvk9H5nPL/qW0xGYo3/x5bwtHw8/k33z+x6BjYtUxsd2tiMvtKT99TpeeJH2/Mv57pj3Y2u0l35jcWOoQLvHdvLG2hZBrj/myrj17MCVJXDH7JhjEzMknjpjPG6N7j4EX882xUb13ukYqMXM5+1SP7vdZs5g/Wa7llhPUi/QXCidmEp9rrzmVmG1+8MldPl/WtWcP7EkeImYKTu98oxDzHLHFPDWc7bFHEZrgB8fGk07M9hxYyt3z/KtTzJ8itYXDMPzlJxVOzD6xlxCzb4zn82Vde/ZgSpL4Yh4D7BYAiHmeFGKeGqLLRFCMnkcKMf8ccsZ+bL3PI3WNYr6L3A72nnK2iZmu5TJEkkLM95FzYz5f1rVnD6YkSSNmCoCLACDmeVKJeYzvsgCW4sxJ5zkpxGyTwnM5bJwbWn1idonBU57ZRfUUM/fJu6XPd5F8CjG7tFPKjb9XXn/Ml3Xt2YPpZtKI2bUB+ov5avh3Dq5yDpbfmeAqjLvm0vVs/FgpZu564/2NKxUOvz5jfRItiXk/DIvYx3LTiNlVNG4N/Id55Vhf/nX/yNxniJgpL2wxIBHTihxanUIdo+MvDRLcntrNkpzd6sAuQJdecwoxu06AhuSfCjG79Jp9xeySuLEDx4l5EzgelvI+xsSfb8DUcL4s/L7Lk8lSrzm2mH86lsslf32YE2FYPq0Xs00+LkNMFHuuF30YJoiXc9rtqcUen9hipuV3rl/aJNe1dadCzC6NEGJOdx90Da4RLq3QcBEgNQTbuubYYuafIubEeRNtbWkpYr5nyjK1GdeXSPbD8jr+Oi6/75IbO8s1Yot5z3hsLl4+sbpEjZgPC0GAmNPeB9fDWpKAa8/U1sOKLea5Mh1Oa3LnPydO/ZQiZu4+x2VqfuvUubyge/24GA+3MW5bO44v5jmP3LCxXvs5asS8lHAQc9r74KUVR8yHodc83/uOLea5Xt5hGE+df6kgdAb+KRZli3nNF9AdE0+33HAT88Ey0RZTzOO9zH1pX1vnatbloCIx2x4dIOa098E1Zqq/Nb/nk+QxxfzA1MHu9Nlcj+lrhLooQcx3TDnWyozge832e/NZFcJ5JKaYufZJ1+LmJejef18Vs0rFzI+BzScdxJz2PrjGt7TOnBMdV+dz47kxxXxgZcCLebzP8AZTgpi5dkq90n71ffHXtP/ey7qw5cbcPERMMc+PIz+9hcg/afjXYcVi5sbB5t8GhJjT3cfDsBRsfmKM27DpKdnn66VjH39fliummLnx5SmntpaJwdC6KEHMPyztam05Hi0xs80LzYnZtkRzroyxxHxrOIc81TvvOP/2W7GYX7NjV3O9tJrFPK0Z9sXl/kLvY2PesA3FbeZ9vl527Jpukv35NWKJ+fGYU0sNi3tkpXJ9DmwsJYiZz8H1nYOeuTfC9hIGJ+adZWXEp4trxBLzgf1yeboOt5SOyvzTM2bVinnHNJCpYfcvbrReMa/F5RGKv49pa89Lxhnop5dN+DWda9/8m+qPWx99GeNYYnad9OLHTMP2RyhBzHx9hr5izMWWX+XBibm31tV5OeOJ2W3VBV8uv61AqxazbaJic5F8ELPffYSy9JhqS+SpXraOveZYYp77Ipi7D34cNqzRlCBm7ndClwTyX2a8sDgx27xwua48hph7M7+yZK4DyPXm/edsKhazrcIvx5ohZr/7CIFi4Lolpk3MvbG/6DBdI4aYO+az5saOuX2aXb+M+FjIi5mPt9tugT71PJaFv65NzLa2v3v2MzHEvLFsP3r5s9w+zb65Ub2Yvxh+neTzBISY/e5jLXT/3z0asU3MY/n4lx2mDYTiiJlbJjffgHnRxN2fI7eY+SGHsFM51qxYWBKzbb/mqdccQ8zc53DX4Ffu+OwfX7mYuYS+bOAQs999+DJtbuTbY1wSc+9QvzHEzK3G4F5q4Seg1td/CWLmYh06lMHPB60byli+7vhzccQ8P9nL7ZLn4qMlVIh5a/he87SRSM1ipkez+Yk4O5fj7D734S7km6DlfEtiHuPC95ppJUSomL8yjcmWH4+WtwDXDmeUIGZ+jDl0YnP+utzOeOPvLIuZ35Fx3EArVMzfmHq21Ytt1UjvGC8VYuYq8fmN1CxmmXXMtKXim2EM8PF0+KbtDa6lrTl9GuxcvdjmEkLFbLsv6hVx8D2jtfswyIt57Vt6a2NsO7jURcy2+6S/DxUzd21bbvxtuV/XQ3zViNl2BM64yxXEHHofD9Zd5Ogw1jgvdMzVC79PxY1l/XGYmNeydivQEsTMt6H1L9BQz5W75poXTF7mBj/W3JlXQWJ2PQDAFdc4qhHz+Bn2zetdBOBKi2ImtpZ9dsdN2/0+36de+De+OEEui9m2yc76xrduf4QSxMzFMqytxNsrYy4ePRM7W264iPmz5bprca1PVWJ+sDZevzHE5WRrU8xcg3Gtz5fXchfzlh3vW7d7ma0BhGJbBsbHQl7M95YY+5wKvlTHLvfmKmZbTvJvB8fZqH8Njw5bp6oS83hD7sGEmNfdh+0LcEz6eMvlXH6ew0XMPtfzYc04cwli7plyrL2n341tfsB+PR8x28o9n6MuYk6TGy4rXNSJ+atHQCHm9ffBzTxPdXrr+Pm+Yu48VpEsiTn2KdCX9+Aag6dYyIt5LAd/9qTvihPbEtDNwhe4j5ht5Z5jScx/MfURKzeW4qZOzD4VBDGvvw9bT8gntmvG/l0n65bEbFuR4rdhFPeCk9+jfyli5nbQm8rTe+QWv8pjeRLMV8y9cZ8vWBKzbYmm30Zi8+W5XxjOUClm114zxBx2H9w+u1MCu0yArRHzzrHXvCTmWGt2Q3bXO79OGWLuF9pP5yDnbuEaLpsi+YrZ1oZ8xRzrzU7+OkudD4Vi5iq1VjHTInx6hAwhxX30xt5DcTsJed1qGZcvXptge8M/qvpO3HG57bs/QiliJnYL8R3Xrr/s9d2a6YRs29PU8nl/XBteisdSTrqImXth7bDipJq1G17xK42uYjnAXsBUYnbpNdci5lBsDTH0PmxjvpTI/11sfOvEbHvcdhHzNuIr1Z8NLwOfrUBLEjM1ZG7b1eeCnbaHHbeB5U8Yca2X83j4i5ng1jW7ipnbtGhNbnwz79ky2PaUib1aiOrl9vwzpiTJK+bxM+0VBDHHuQ/bSpilXnPI+vKlL16bAGLsZ+ByPZ/lgyWJmdhaDqNYLwifeKwT8/GPfulLxSZmfiOndXVhe2uV/x3FYv7LEpSQRkhAzE/Qukx+gf9N/8Ha+NaLeWmfD7uYuR3A1q3Vte3Z0DteozQxT+021uoEyoU/PMq/Vszc757X87yYuZOwiQeH9cc+ZbFNgKoW83iDtt4cxBzvMFbbSyd+gvTbhcs2STX/uQ/MK9xr39gj7g3fa3Z9/bdEMY/X4d/2dOWwYq/qEDEf/+htvWauTlKc6chtGcAdIDvmtXIxj5uax9+YBWI+Z2dsO/xd93+yjS9MzNxBn2Nuzd93inwwlvt3fTGjVDGPcX63as33tLxszY57IWK23T/hu5fy2mEMomfq1paj2cS8PT0SvWT5tcy533MVM7FjrhESbBLC3DV/BHyzdkw5Q7Ft0M3fh39suLoa4RLw2jsn5hrTfI7Mf+YPpoxLS5hcRHA4TYid47o/wvrf5eIyd02fDdufc2fG1RrTpN+SkMc9i9c9/o/xuJotv+vv92xM+a1q98zPh57g0jE5yjloG9kFdFbn7flnrL8ZAGqjZ0j9uz7XjHGftE6ZvvhILE9M+4C/DTpiy1b+1DFIFa/S+D/hEd3YFPsptAAAAABJRU5ErkJggg==</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
           <t>Healthcare &amp; Medicine</t>
@@ -1393,7 +1413,11 @@
           <t>WVIM</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEAYABgAAD/2wBDAA0JCgsKCA0LCwsPDg0QFCEVFBISFCgdHhghMCoyMS8qLi00O0tANDhHOS0uQllCR05QVFVUMz9dY1xSYktTVFH/2wBDAQ4PDxQRFCcVFSdRNi42UVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVH/wAARCAB5AkEDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD06iiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKZLEJVwWdfdGIp9FDVxp2KMmnyH7l/dJ9WyKqS6bqgz5Wps3s2R/jWzRWUqMX/wAOzWNece33I5iaDX4v+Wkrj1Rs1Qkv9UibbJPOh9GyK7amuiSLtdVYehGawlhW/hmzohjEvigjiP7V1D/n7k/Oj+1b/wD5+5PzrqLjRLCf/lj5Z9UOP06Vl3Phlxk284b/AGXGD+dcs8PXjs7/ADOuGJw8t1b5GX/at/8A8/cn50f2rf8A/P3J+dNudPu7XPnQMo/vdR+dVa5nKpF2bZ1xhTkrpIuf2rf/APP3J+dH9q3/APz9yfnVOil7Sfdleyh/Ki5/at//AM/cn50f2rf/APP3J+dU6KPaT7sPZQ/lRc/tW/8A+fuT86P7Vv8A/n7k/OqdFHtJ92Hsofyouf2rf/8AP3J+dH9q3/8Az9yfnVOij2k+7D2UP5UXP7Vv/wDn7k/Oj+1b/wD5+5PzqnRR7Sfdh7KH8qLn9q3/APz9yfnR/at//wA/cn51Tp0a75UT+8wH50e0n3YvZw7Itf2rf/8AP3J+dH9q3/8Az9yfnVWRdkjp/dJFNo9pPuw9nDsi5/at/wD8/cn50DVb/P8Ax9yfnVOgdaPaT7sfsofyo9Fooor6A+ZCiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKADqMGqF3o9ldZJiEbH+JOP/rVfoqZQjNWkrlRnKDvF2OUvPDlzFlrdhMvp0NY8kUkTlJEZGHUEYr0Oobi1guk2zxK49xyPxriqYKL1g7HfSx8lpNXOAoror7w2Rl7N8/7Df0NYM8EtvIUmjZGHYivPqUp0/iR6dKtCqvdZHRRRWZqFFFFABRRTkjkk+5Gzf7oJoAbVrSo/N1S2TGf3gJ/Dn+lLFpd/KRttJOe7DaP1roNE0ZrKQ3FwVMuMKq8hf/r10UaE5zWmhy18RCEHrqc9qkZi1O5TH/LQn8+f61Vrq9b0Zr2QXFuVEuMMrcBv/r1z8ul38RO60k47qN38qK1CcJvTQdDEQnBa6lSgdac8ckf342X/AHgRTR1rnOk9Fooor6M+WCiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKiubaC6j2Txq6+/UfSpaKTSasxptO6OY1Dw7JHmS0YyL/cPUf41hOrIxVlKkdQRXolU7/Tba+X96mH7OvUVw1sEnrT0PRo49rSpr5nDUVf1HSbiwYsRvi7OvT8fSqFeZKLg7SR6sJxmuaLugpyyOn3HZfocU2ikUWotTvoSCl1L9GbI/Wuj0TWGvmaCdQJlGQy9GFclV/Q5PL1i3PqSv5iumhWnGaV9DlxFCEqbdtTd1zWGsXEECgykZLHoo/wAa52XUr6YkvdS/QNgfpUmtyeZrFwfRtv5CqNKvWnKbV9Aw9CEKadtRzSO/33Zvqc00daKB1rnOo9Fooor6M+WCiub1Txrpek6hLY3UV0JYyM7YwQcjII596rw/EPQ5ZkjAul3sF3NGMDPrzQB1lFFFABRRRQAUUUUAFFFZWu+ILDQY4nvS/wC9JChFyeOtAGrRWfousW2t2Zu7RZREHKZkXGSPT860KACiiigAooooAKKKKACiiigBsjiONnPRQScVx/8AwsjRP+eF5/3wv/xVdbdf8ek3+438q+e6APc9A8QWfiCGaWzSVViYK3mKByR7E1rVwfwp/wCQbf8A/XVf5V3lABRRRQAVma9rlpoNpHc3aSsjvsAjAJzgnuR6Vp1xXxT/AOQBbf8AXyP/AEFqAH/8LI0T/nhef98L/wDFV18Eqz28cyZCyKGGeuCM188969/0v/kFWn/XFP8A0EUAWqKKKACisHX/ABXZ6BdRwXdvcN5i7leNQVPPI5PX/Gsr/hZWjf8APtef98r/APFUAdnRVbTb6DU9PhvbckxTLuGeo9j71ZoAKKKKACiua1rxrpejai9jNHPJKgBYxgEDPOOTUPjPX7iw8MwXNorwTXZCqWHzRgjJ/GgDq6K8Gs9c1Szu1uob6fzAcnc5Ib6g9a9w026+3aZa3m3b58SybfTIzQBZooooAKKKKACis3xFqD6VoN3fRqDJEnyg9Mk4H868WfWdUku/tTahcGbOd/mEYoA97orE8H6rNrHh6C6uOZgTG7D+Ijv/ACrboAKKKKACiiigAooooAKKKKACiiigAooooARlDKVYAg9Qe9YGqeHw2ZrIYPUx+v0roKKzqUo1FaRrSrTpO8WedujRuVdSrDgg0ldtqelQX6EkbJgOHH9a5C8s5rKYxzJg9j2P0rx62HlSfke3QxMay7PsQVZ0w7dTtT/01X+dVqltDtvID6SKf1rGOkkbzV4tEmpHdqVyf+mrfzqtUt0d13O3rIx/WoqJO8mEFaKQUDrRQOtIo9Fooor6M+WPOfinpmHtdURev7mQ/qv9a88r3bxJpo1bQbuzxl2TdH/vDkfrXhJBBIIwRQM9w8I6l/avhu0uGbMir5cn+8vH68H8a2a81+FmpbLq60x24kXzYx7jg/pj8q9KoEFeXa7491SLWbqLT5YltY3KJmMHOOCc+5zXdeKtT/snw9dXQbEu3ZH/ALx4H5dfwrw08mgD2/wlrDa3oMN1IQZwSkuBj5h/iMH8a2q8u+GGqfZ9Vm052wlyu5Af76/4jP5V6jQAV5B8QNRbU/E7W8WWS2xCgHdu/wCvH4V6lrN+ul6RdXz4/cxkgHu3YfnivKvAtg2reKo55sukBNxIT3OeP1I/KgD1LQdOXStFtbEAZjQbsd2PJP5k1oUhIVSzEADkk9q5DWfiDplhI0NmjXsq8EqdqA/73f8AAUAdhRXmsfj3xBeZay0iN0HXZG74/EGnW/xJvIZvL1DS044YIxRh+BzQB6RRWTofiLTdcjJs5v3oGWhfh1/Dv+Fa1ABRXN+MvEk/h2G1eG3jm85mB3kjGMen1rmbf4lXstxHG1hbKrMFLFzwCetAHpVFef658R1huHg0m3SVVOPPlztb6AdvesqD4lauj5mtrSRfQKyn880AeoXX/HpN/uN/KvnuvcNG1g654fe+Nq1uGV1Cls5wOoPpnP5V4fQM9N+FP/INv/8Arqv8q7yuD+FP/INv/wDrqv8AKu8oEFFc/r/i/S9DYwyMZ7kf8sYuo+p7fzrjrr4l6m7f6NZ20S9t+XP8xQB6jXFfFP8A5AFt/wBfI/8AQWrJt/iDrcKiW80uOSH+8qMn6nIqHxj4o0/xB4egW33x3CThnhccgbTyD0IoA4fvXv8Apf8AyCrT/rin/oIrwDvXv+l/8gq0/wCuKf8AoIoGWqKKKBHMfEDSf7T8PSSxrme0/erjqR/EPy5/CvHa+iCAylWAIPBBrw3xRpR0bXrm0AxFu3xe6Hkf4fhQM7H4W6tujuNJkblf30WfTow/kfxNehV4LoWpPpOs218mcRP8wHdTwR+Wa94ikSWJJY2DI6hlI7g9KBDqr6heRafYT3kxxHChc++O1WK4L4oat5VnBpUbfNMfMlx/dHQfif5UAct4bs5fEvi4SXI3KZDcT+mAc4/E4Feqa/o1vrumPZTkpyGRwOUYdDWB8NdJ+xaI19IuJbs5GeyDp+fJ/KpvGPiu48O3NtFDbRTCVCxLkjGD7UAYVp8MphdqbvUIzbg5IjU7mHpz0/WvRYYkhhSKJQsaKFVR2A6V51Z/Ee9ub2CA6fABLIqEhm4ycV6RQAUVheIPFem6D+7nYy3JGRDH1/H0rkX+I2qXEhFlpcWB2O5z+mKAPS6K80g+Jd9FJtvNMibHUIxQj8811nh7xbp+vymCBJorhV3FHXjH1HHegDYvbSG/sprS4XdFKpRh7GvPH+GNz9qIj1KL7PnqyHeB9On613HiLUpNI0O5v4o1keILhWOAcsB/WuD/AOFm33/QOt/++moA9C0nTYNI02GxtgfLiHU9WPUk/jVys7w/qL6toltfyRrG8wJKqeBgkf0rRoAKKwNe8X6VojGKRzPcj/ljFyR9T0H865RviLqt3MY9P0mMnsvzSN+mKAPSqK81PxC1qykC6hpMa5/hKvGT+ea6XQvG2laxIsDFrW4bgJKRhj7N/wDqoA6Wiiqmr3jafpN3eIgdoImkCnocDNAFuivMf+Fm33/QOt/++mrof+E70+30W2urrDXkybvs0ByRyRye340AdbRXmd18QdckUy2umRxQddzoz8fXgUyy+Jl+jgXljBKncxkof1zQB6fRWVoXiHT9egL2chEijLwvw6/h3HuK1aACiiigAqC7tIbyExTLkdj3B9qnopNJqzGm4u6OI1PTJtPlw3zRH7rjv/8AXqkjbXVvQ5r0GaGOeJopVDI3UGuQ1fSZLB96ZaBjw3p7GvJxGGdP3o7Hs4bFqr7k9/zM1zudm9TmkoorjO8KB1ooHWgD0Wiiivoz5YK8W8caZ/Znia5VVxFOfOT6N1/XNe01xPxP0z7Ro8OoIuXtXw3+43/18fnQB53oeoNpes2t8ucRSAtjuvQj8s17yjK6K6EFWGQR3FfO9exeCNYS58IpLO+DZKY5SeyqMg/984/KgZzXxS1Pzb220uNvlhHmyD/aPT8h/OuY1nQ59Js9OuJc4vIfM5H3Tnp+RX86s6fFJ4p8ZAyAlbiYySD+6g5x+QxXo3jvShqPhmby0/e2375AB2HUfln8qAPItPu5LDUILyI/PC4ce+D0r3y0uI7u0huYTmOVA6n2IzXz3Xq/w01T7XoT2UjZktGwMn+A8j9c0AU/inqfl2lrpaN80p82Qf7I4H65/Krvw00z7JoL3rriS7fI/wBwcD9c1w2uXEniTxg4gO4SzCGH2UHAP9a9hSOLTdMEca4itosAeyj/AOtQI89+IviWSS5fRbOQrDHxcMv8bf3foO/v9K5nwro/9ua7DaPkQjLykddo/wAeB+NZdxM9xcSTyHLyMXY+pJya734Twgz6jcHqqog/Ekn+QoGeiW1vDawJBbxLFEgwqKMACuf8a+H4dY0iWZIwL2BS8bgcsB1U+uf510lHWgR892tzPZ3MdxbStFLGcqynkGva/CuuJr2jpckBZ0OyZR2Yd/oeteManCLfVLuFRgRzOo/AkV1/wsu2j1i6tMnZLDvx7qR/iaBmj8WP+PXTf9+T+S15ug3Oq+pxXpHxY/49dN/35P5LXnEX+tT6igD2RPA/h8WItzZFjj/Wlzvz65/yK4nW/AV/ZX8KWWbm1mkCB8fNHk/xD09/5V6wv3R9KWgRTitIrDRhaQjEcMOxfwHWvAq+hLr/AI9Jv9xv5V890DPTfhT/AMg2/wD+uq/yrV8deIW0TS1jtmxeXOVQ/wBwd2/wrK+FP/INv/8Arqv8q534k3TT+KniLZWCNUA9Mjcf50Acq7M7l3YszHJJOSTXqHgPwpBbWUWqX0KyXMo3xK4yI17HHqetecaZbi71S1tj0llVD9CQK9+VQihVACgYAHagAZQylWAIPBBrzX4j+H9PsIItSs4hA8sux40GEPBOQO3SvS64r4p/8gC2/wCvkf8AoLUCPK+9e/6X/wAgq0/64p/6CK8A717/AKX/AMgq0/64p/6CKBlqiiigQVxHxO0n7TpcWpxrmS2O18d0P+B/ma7eorq3iu7WW2mXdHKhRh6gjFAHz3Xrnw41b7foH2SRszWZ2fVD93+o/CvLtVsZNM1O4spfvwuVz6jsfxHNa3gbVv7K8Rwl2xBcfuZPTnofwOP1oGezuyojO5CqoySewrxe4eXxb4ywhO24l2r/ALEY7/kM13/xD1b+zvDzW8bYmuz5Y9l/iP5cfjWN8LtJwlxq8q8n9zFn06sf5D86BHoEMUcEEcMShY41CqB2A4FebfFf/kIaf/1yb+demV5n8V/+Qhp//XJv50AcbpP/ACF7L/run/oQr3LWL3+ztIu70DJhiZwPU44/WvDdJ/5C9l/13T/0IV7jrVkdR0a8slOGmiZVJ9ccfrQM8Jlne7vGnupWd5H3SOeScnk17vpNvYW2nQppqxi2KgoyfxD1z3NeCzwyW87wzIUkQlWVhyCK0NI8Qapozf6FdMiZyY2+ZD+BoA9k1nQtO1qAx3lurNj5ZVGHX6Gs7wj4YXw6t2XlWaSV8K4GPkHQfXrmsTR/iTBKVi1W28knjzYeV/EdR+tdza3MF3bpcW0qSxOMq6HINAjE8ef8iff/AET/ANDWvFq9p8ef8iff/RP/AENa8WoGe1+Bv+RQ0/8A3W/9CNU/HniN9F09be1bF5cA7W/55r3b69h/9arngb/kUNP/AN1v/QjXm3j67a68WXYJ+WHbEvsAOf1JoEYUMct5dpEuXmmcKMnJLE17joGi2uh6dHa26LvwDJJjl27k15R4GgE/i6wUjIVi/wCSk17VQMp6pptrq1jJaXcQeNxwccqfUHsa8M1Oyk0zU7iylPzwuVz6+h/Gvf68i+JUIi8VM4GPNhRz7nkf0oEdP8PPEsmowtpd7IXuIV3Rux5dPQ+4/wA9K6LxR/yLGp/9ez/yrx/wtdtZeJdPmU4/fKh+jcH9DXsHij/kWNT/AOvZ/wCVAHhVekfDnw/p1xp39qXMInn8wook5VcY5A9a83r1z4af8iqP+u7/ANKBnWYGMYGOmK87+Inhm3gtv7YsYliwwE6KMA56NjtzwfrXotZHi1Q3hXUgRkeQx/LmgR4vpt/caZfxXlq5SWM5HoR3B9jXuumXseo6bb3sX3JkDgenqPwrwCvYPhxI0nhKFWOdkjqPpnP9aBnU0UUUCCiiigApskaSxtHIoZGGCD3p1FAbHHazpL2MnmR5aBjwf7vsay69DljSWNo5FDIwwQe9cbrGmPYTZXLQt91vT2NeTicNye9HY9rCYr2nuT3/ADM6gdaKB1riO89Fooor6M+WCq+oWkd/YXFnKPkmQofbI61YooA+e7q3ktLqW2lGJInKMPcHFXLDV7ix0y/sYvuXiqrHPTB/qMit/wCJWmfY9eW8RcR3abj/AL44P9D+NclFG80yRRqWd2CqB3JoGejfC3S9lvc6rIvMh8mMn0HLH88flXfsoZSrAEEYIPeqejWCaXpNtYpjEKAEjue5/PNXaBHhPiPTTpOu3VlghEfKe6nkfoabo2sXGkSXLwdZ4GhPPTPQ/UV23xT0vMdrqsa8r+5lI9Oqn+f6V5xQM7X4Y6Z9p1iXUHXKWqYU/wC23H8s16fdRefaTQj/AJaIy/mMVieBtM/szwzbqy4ln/fP+PT9MV0FAj54kRo5GRxhlJBHoa9B+E8o3alD/ERGw/8AHh/Wsz4heH5NO1R9RgjJtLptxIHCOeoP16/nVDwRrCaP4gjknbbbzAxSE9FB6H8CB+tAz2iikBDAEEEHkEd6yPFOsRaLok9wzgTOpSFc8sx/w60CPGdXkE2sXsqnIed2H4sa6n4W27Sa/cT4+WKAgn3JGP5GuMVWkcKoLMxwAOSTXsvgjQW0PRsTri6uCHlH930X8P5k0DML4sf8eum/78n8lrziL/Wp9RXo/wAWP+PXTf8Afk/ktecRf61PqKAPoZfuj6UtIv3R9KWgRFdf8ek3+438q+e6+hLr/j0m/wBxv5V890DPTfhT/wAg2/8A+uq/yrmPiHA0Pi65Y5xKqOPptA/oa6f4U/8AINv/APrqv8qs/EXQJNSsE1C1QvcWoIdQOWTr+nX8TQB5vocwg12wmb7qXCE59Nwr3uvnYcHNe1+ENfh1zSY8yD7XCoWZM85/vfQ0Ab1cV8U/+QBbf9fI/wDQWrta4D4o6haPY29gkytcrL5jIvO0YI59OtAjzXvXv+l/8gq0/wCuKf8AoIrwDvXv+l/8gq0/64p/6CKBlqiiigQUUUUAecfFHSdslvq8S8N+5lx6/wAJ/mPwFeejg5Fe961p0eraRc2MmMSoQpP8LdQfzxXg88MlvPJDKpWSNirA9iODQM1tV1W88S31jGykyrGkCLn7zdz+Jr2XSbCPS9Lt7GL7sKBc+p7n8TmvNvhnpP2vV5NRkXMVqMLnu5/wGf0r1SgQV5n8V/8AkIaf/wBcm/nXpleZ/Ff/AJCGn/8AXJv50AcbpP8AyF7L/run/oQr36vAdJ/5C9l/13T/ANCFe66lexadp1xezH5IULn39B+PSgZleIfCem69+9lUw3WMCaPqfqO9ef6v4B1nTw0luq3sQ7xfe/75/wAM13fhTxXba9AIpSkN8o+aLPDe6+v9K6OgR87urIxR1KsDggjBFdZ8O9ZmstdjsC5NtdHaUJ4DY4I/lWl8VLW0juLK4jVVupQwkx1ZRjBP6/5FYXgOzku/FdoVGVgJlc+gA/xxQM9H8ef8iff/AET/ANDWvFq9p8ef8iff/RP/AENa8WoA9r8Df8ihp/8Aut/6Ea8z8c27W/i2+DDh2Ei+4IBr0zwN/wAihp/+63/oRrG+I/h+S/tU1S1QtNbrtlUDlk65/Dn8DQI47wFKIvF9iT/EWX81Ne0V8+2N1JY30F3F9+GQOPwOa9402/t9TsIby2cNFKuR7HuD7igC1XknxNkD+KQo/wCWcCKf1P8AWvV7m4htLaS4nkEcUalmZugFeE67qJ1bWrq+IIEr5UHso4A/ICgB3h23a68Q6fCoyWnQn6A5P6CvZPFH/Isan/17P/KuP+Gnh+RXOtXKFQVK24I656t/QfjXYeKP+RY1P/r2f+VAHhVeufDT/kVR/wBd3/pXkdeufDT/AJFUf9d3/pQM62snxX/yK2p/9e7fyrWrJ8V/8itqf/Xu38qBHhleu/DX/kVF/wCuz/0ryKvXfhr/AMiov/XZ/wClAzrKKKKBBRRRQAUUUUAFR3EEdzA0Mq7kYVJRSaTVmNNp3RwupWElhcmN+VPKt6iqg613eo2Ud/atE/DdVb0NcTPBJbXDQyrh1ODXjYih7KV1sz3cLiPbRs90egUUUV7R4IUUUUAc/wCNNDk13RfJtwpuYnDx7jjPYjP0P6VzHhTwRqNjr0F5qMcYhhy6hXDZbt/j+Fej0UAFFFFAFDXNOXVdGurFsZlQhSezdQfzxXm+n/D7WPt8H2yOJbbeDIRICduea9XooAAAAABgDoBRRRQBHc28N1bvb3ESyxOMMjDIIrz/AFn4bZkaXSLlVU8+TNnj6N/j+deiUUAeY2lh4+0mIW1rvaFeFG+NwB7Z6VDJ4Q8V63cibU5VU9N00oOB7Bc4r1SigDmfDfgvT9Edbhz9qvB0kcYCf7o7fWumoooA5Lx9oWoa5BZJYRK5iZy+5wuMgY6/SuMTwF4iV1JtY+D/AM9l/wAa9gooAQcACloooAZOpe3kRerKQPyryH/hAfEX/PrH/wB/l/xr2GigDlPAWiX+iWV3FfxqjSSBl2uGyMe1dXRRQBxniTwDa6jI91pzra3DcshH7tj+HSuOPhTxRpV0Jbe1mEi/dlt3B/kc17JRQB5lBbfEDUF8l5p4IzwXkZU/Uc1Zufh48WiTGOT7ZqkhUhi21V55xnqcdzXolFAHj3/CA+Iv+fWP/v8AL/jXrVjG8NhbxSDDpEqsPcAVPRQAUUUUAFFFFABXnfjHwXf3+uPe6ZEjpMoaQFwuH6Hr68H869EooAx/Cukf2JoUFowHnH55SO7nr+XA/CtiiigArifH3hzU9bvLSSwiV1jjKsWcLg5967aigDyXT/A2vwahbTSW0YSOVWY+avQEH1r0jxBo8euaW9jJPJCrMG3J6jpkdxWlRQB5LfeAddsJfMsylyFOVeJ9rD8D/Q1NFf8Aj+1TyRDeuBxlrcOfzwa9UooA8iTwp4o129+0X6OjNgNLctjA9h1/DFeieGvDtp4eszFCfMnk5lmIwW9h6D2rZooAyPFdhcan4cu7O1UNNIF2gnHRgev4V5r/AMID4i/59Y/+/wAv+New0UAZPhaxuNN8O2lndKFmiUhgDnHzE9fxrWoooA43xD4AstRle50+QWc7HLJjMbH6dvw/KuetPDnjPQZG/s5sqx5EUqlW/wCAt/hXqdFAHl15onjfXcR3+REDna8iKo/Bf8K19C+HVtayLPqswunHIhQYT8T1P6V3VFACKqooVQFUDAAHAFUtctpbzQ721gAaWWFkQE4ySKvUUAePf8ID4i/59Y/+/wAv+Neg+CdLu9H0H7JeoEl81mwGDcHHpXQUUAFZ+v2s19oV7awKGlliZEBOMk1oUUAePf8ACA+Iv+fWP/v8v+NeheCtLu9I0EWl6gSUSM2Awbg49K36KACiiigAooooAKKKKACiiigArJ17TftcHnRL+/jHb+Iela1FROCnFxZdOo6clKIUUUVZB//Z</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr">
         <is>
           <t>Protection &amp; Social Work</t>
@@ -1485,7 +1509,11 @@
           <t>MTSTM</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAIEAAACOCAIAAACZlPzSAAAACXBIWXMAAA7EAAAOxAGVKw4bAABalUlEQVR4nOy9B1hUWdY13AIVbqxMEARMYAAzooLknEGyknMQkCQ5C6IkEUFABETEBCKIopjAhFnRNsc2gIggGSrc+m+BdvcbZnrab3p03n/OUw9QUFDcs87Ze60dzv2J/5/xvcdP3/sf+M/4DwY/wPgPBt9//AeD7z/+g8H3H//B4PuPHxAD3vf+B/7V40fDAOPz2QIYMD6GYRNPMcF3BV//nx0/Dga/Ln8uhvHGxzEubxzj4w8O9uuPsMmXcb/PP/iXjR8QA3ymOTwej8PtG2G/4vJHePxR3pdtgG8Rzvf6//668WNiwMMwzji3u7xRa5z3noeNfbVL3Ekz9X9s/JgYCOaai/XFZcuevW3Jwz5OLH/s6+z/XwPhx8QAN0W4+Rkr3quYtJV596kbxu/Fv/f1Bf/XzNEPiAF3cpYxjH3xcoyHD5RbTOseyMV4QxPk6P8aAPwfCYP/PnAf0Nt7OcSXVlkkVrmbOThYgfGHuLg7ECDB/UpWJyHBuRMX+2qkcB418fj1BT+67fpxMeALTFJ/XKy8qz2QvYny/MVyDu85jz/G4/+qG3i/cxK8r9/kTH79FZIfHQD+D44BPoO9vW32pmhiKOXl41Xdb0Mw7BNn0lj9CgQ2MeFfEOH99iPBVsD+LTT3D44BF+MO78jVdXOAcRiePVzY9zkDwwZxEYc/eBPyWTDTfLZAygmecSd+hH3FgPsfDP6fh2B1j9cd8Ldfg3jaQS2N4iODIcO92zFeD8Ybm7BLYxiu4Pif+PxBDrt7nNfN4eFosL/8rgCbf4PxY2OADw63rT7e0RBZqwPlhNN+uT73VovCp7dho/31/Z/y+3tKOSNXfnltOzZ4cKDnwGB/Ha6ruZMUS/Dh38Ah839wDAS2hce+UZfkqoo4LYDtl5OPZ4nlhsGdV+dz+2Ox8aTP7zU4nxOvN4s+aFHouqF1dLf0+Ej7F7Ik8AW8f4so7A+KgcC4Yzx8RbN52KsDhY4LAZdlYJIN2rJd9EObYucZ2Q/XZAaeKP1yYf6lPcyTRdTem5pnimn3Wgxe3bbncse++GPs32EX/DgY/BaGwCY/cblcnsDzcjnPD29xXgwEqkGJtkjXTbfWEoniSPDuYdaDOtbJwqk97Qq54WD3VdWbddN6buumBKLs0Q4eNjIhEsb/DXbBj4fBZLCIK+A7AnrDHe15GGUkmmrPWLeS6KNPulIudr1S9sQO2WfHp17cxdwVBz1uWnC9mlmdJn59n1z/XavKFPovV8x4vJe4u+ZjbB6f/X2v6x8ZPwoGgvE7WTXxmYfxhoqjDU0XEZuyxV4cm+NqTGgrEb1Yzmgukgi0IOxLpSZ7kmuyl6b7kY8XSm4PB9orxV43yp0vk+3/kM3FRrF/E7f842AwKXpxC8L+Eo/A+GP9P6e6MVbLC53YNfdECaXz6qp9KdSjubT9GZQwK3Jd5rTSGGpdFu1+nXJrGf3INmZlMvVcodTVGkbXY81PnTv5GEcgGH74HNyPg8EXxYvxx9nY2IQyGHv74OjmAPqto+q1BYz6AmaKP7hWXdhWRfjCTokjWxk7o5EjW+g5AXBjLv3JCbX7dRJ70kRzQ9HwdYSmXZS3d4wxfv/voq0/7vhxMMAmEwc4Crg7xm1Ib1f17XOhgTbkk7uYr87q26qLbPejp/lA5wsl9qfSr1dLbA0EblSIp7lCu6NhH2Ph2gxaVQramE1/d1L7Y6tG7zOH8ZFbOJDf+7r+ePw4GHwRt4LAAy50cV/AfrPBBb1aOztvI1y2ke6oSmzaLO5oQKhKoSc4Aw3ZjE0ucJg18Uqh2JFU2usmvbpUqp36FCdtYk0Cpbddsf+9M2fw+o/vDPg/EgacSVYksB4T0oqHfa7erliRwnDVJRxLl/AzouwOZWT5oOGW5P3xzC3+YIoTcCFHYm8AI0KP2BBOe18xe6DVeOSqw/gtq5E71gcSqG/PhXD5nB8/+fnjYMDjfalp4eCemSsAgtP7piXKgWK+jLDBEPQzIOX6UHf5M7c6o4W+tDg74Fjq1HUqwhmWcL41GqZO9FtO8lYmRRsQbuaxfjkyLc8H7moPwv36hNz7oWH4YTDAJqtWsIl6FjZnIuzJ54x33krZ5EPZ5IgG6gGRxoibCqnInXY0VrI+hmWnRPDXJMXoA4l6YIkDNduCFrQaOBEi0RgOf241sF8ldLfOks8dwP3LfzD4Bwfva1KGM4GBwDXz2ePDH87ErEUCdMhh+lCMPmq/jBCoRdxkC1YEiLsvI0frgcn64A4jylYjOFSVtMsb7qyedTmG1n141sgty/GXIbyhDv5/MPg749epmZDEX/NjglAPrpM5D45EDj05w+196qWCxJkgnqtJTopkfxWgxJOWtw7atk4iZCWUoIls1ocubmD01szn3HTDnmzgPfB9t0tquFl/sG5l3xnF0TcFGG/0v73djza+8z4QROa+UHgef9Ip8yazX5xkZ6lAQyTWkm43D/BdBpV5MB8WLLiTLX1so1iOM5y3jh62EkzQAONUyEXG8MNU5uea+dgtH+xJyIV0RrK2cJEuMNSsPfwoAcfg92D/gEh8Nwz++3QICkwFInnCKfB5nNGHR1LKPMXSbdANhpDFPEKqObzfl77TGy4JRILNCGVBc6KUwAR1HAMwSQUqXQPeiKMM1i/GHgZyr3ldChU94kQZbtEevpvIx7645V/H97rkvzW+ry3Czf74SHc7JlBS+OrHdwRuN9hcriALOfbhUawxcmAD40Aoy2kJOWQ1GKoCHPRkFbpSclyQ5qiFgQvJm9TgFHU4cSWcrApUWSOPNzFGTmqPtnlXr6OmaJD2BdMGbyXhagPjcfhs3oTsGMYN3eSbf8cL/2/j+2AwGQ7CsPHx7nvXKmbzxz7iMGDY6MeuMh733cTK5XOHu8L0ke0eSE3Q1Bp3STM5kc2GtOBVwIbV5FQz+IAHw2MeMUcdzVaDMtWheFUgQx2qsUNvhdGPOUL7TNEUTeLNrGmfO1LxPyvguwKdwOl8HskevjmxCbk/zp74LhgIUvETkQn2FtdFV0tlW3fr8nmDT1pqnA3A4f5yPj5r+M/HBuKNaAWuSEsy637JEqdlxHWLSL7LgU0qtI0aiN98MGwunKOC7jVCC/SgLVpQhhqUpQHts0Kue9Db/Gnde1d/PqY1cDeTz//M5Y9zMA7GHQxwBEc+5vMm8syTroj3AwSUviMGGG/ok5E8nOWBbPVGXp9f77dKdJW48LvLVp0d2/ncofGBS4k2lKuFak1JYvHmYLEjc70KGKYGmc4UiTFCneQA42kiLrNJ29TQ/faUAj0kTwXJ1oG2GIGVFmirM/1huFhHssTHK/GDH2vGeK95GPft2fR9sQzOp108TFArxuFwuNwfgrZ+LwwEH7rOVa4WI+jI/3SzSPR4PCvXhWYwQ7h588JUD3iTN+tO63xvK1LL1tmlIZS9IWIuS4lnI5VKHEU36oHRxpC1PHHtQrLvYjBqMRS9nJyuCpVqUUr0KAUGSIkpmmcC7dSlXo1Yyht6/u6OBXu0dvjp8bS1zFxXaOx9Lp/fh7//+Pg4m83+/+c++JJnx3jca/meGhTicomfuk6sqfCBj0SKZdkgJgpCh1KkziSKOeqL3D2rZKUu3F6t0Z431XGpSLAqEKJJTjCHfFXI9nMIJVbi4UrAzpWUraugmOXkkKXkoMVA6ALAbYXwu9sanP5WPvfzeP+9nBDKuYP6h6NF2zZJRBmTBp4kYbyPP1Tl0ffYBwIOipMg7qEIGzWUqMYS2WJNOxnNbE6l5TiClvMJ7TsVHxaKJjqASaHw6RoxF0ORF4dmN6UzGqJZT4pmVvnRcJ+cbAyX2EmnKkF71dAKdRR3y3HK0IYV4PqlQIABqfPl/M4XGk/O2oSbQhVBlDPF2k1hzIPrGUlm5M6zVvzx3h+q3OL7YMDjj+NE9JC/nRaNtJpK1JQWerxdcZsHVGhDSTaEjRSF3lUtKN9AcTYUaW2UeHhOOtkdqgyldZ9fd3679FYvRlvu7JaU2esUCXHLwd3aaIUGmqMOZ6yA8af4VnBSIO9IQbseztmbyTgVy9wTjJ7buijZAChypoTpEio2UPtfV+JuX1Be/2NQo++CgSBFw+aPn4h31mUSdWWFtljQ4i3QU8kSQWrkUlfqgUDWem3ig32KOQFwWgjSelz04/1V9irCVguEXVcSY4zAABWyrrSwyxxS8nJ4hwpcro3mrIazVqDJSnDYKiDXlG6kJHT7qkTn/aU7AsC9QWix97QEA6DEm3pt0wy9eUI/H9HlDlzE+CM87qRd5H6p5fhzVyH43a91+pNhX+63FdN8J402ERd6WVOgLD5loMWuOYHmqSLSFCFV7UNPM4WSTMAUI3iDAfTk0FI7TZHLTVOvtk5t2ydT6kYtWksLVIa8VMgl7mLxunDsMqBADdqhA2ZqgqmqUNRyMFyXWOAiZr+CeGyvWMelaa27pzbGi3oqEfJtKWXetAQj5HSSTGE4NPgyHOO+xKkZnzPZdvhtog2bKKcc/93Tb0HhO2AwEaHDFfIYb/DV5e2L+xoW1YVRCh0QF0VC+9bp+e7IkQBWhBoYvQIxkhdOMEWzwqlHDjPe/qwUbEw8sIGaYQOV+1J8VhFz1jIvpk6r82Zu0QXTtMF4TWC9KrEySD7JAsx1pCUGwwcrqO875jamzkzUgc+mzY/WRldO/en+TsUCb/DNqZXjn2v43H4+Z4z3ta8E+9NegjfZpojxfy2v/BY/88/E4A9t66T95U1uYx6HN9TRd0bjTjb1ZAy91AuNVoOs5wt37JCv3iCRYAwkaMNBKwCbuQSnleT8FNrVNon7jYv9dEhns+Vub5uVakE+Gy2+QZe4QZt4MHDaq8O+t/KWP9ytUeHDXK9FKPNgmmsI785jvLwzK9kdqIudGWUrpSclrCYr1BjNLHOhXs1hDj7ww9iv+NivOVT+n51B3KYK6BVXwG8nfp37bZV9/zQMJmXnP+Li2BiXM9FHM/qipOuA1MNM1qV0sZZU0VIXuv8S0Hi6cJWv2ONdC301RLKt0VB1wGqu8L5NYvlZ6C/35lwuEU+3ARJsoEtZEo0plFMp1B3O8OEAht1CIV8VQqAGcaMBubvBeK0SQV1hyp7tovX7xZ5dkL1x0DRUD7JbQIg0haMMydsdkfpI5N2ReezuJoElmQgg/flNwOdw+aPcTmzkNZ87OoElbzIP+2fHv9QWPXr0aFKaYvgS4g18vux0Yyu9xAOMtyamrwXPJ4jfz5Z3UyLaziCtnvrTJmPkfbXtNgeK0zyi+swp/mvBqgrW61szui8s76pdmecGJtiIFPoCXQ1a3Q2KRb5QsRf6+bz921rV5DWkk+HiKnOnlGazcrcgLy5PDzQku2gSDOdMeVkub6IwJd8GbYlh3M1jDN4Jx7BPk9P2DRjgRqx/8OiDmjkPU5Qxdo8g7zShfP7s3/nXYTBZtIJNHoKAjYw9r/l4VOlRvuizUpm7hZKVQVCAjnC6Lb0mgFFgyTCgEg0kRYzlhA3kpsQZwtFGyN4ESQ1VoR3ZtDv1My0WCp1IkHl/YNHNHNapFFqgvoi/nvB2b9BVTTjRmnwpU/LRPlMl6Sk5Ccy0ZPiXdrmKaLTvoqX5XJG+0y4+KsQ0Izh/HXg5jfa51Yg3dudrbfCfZKkCg8oZGTzS26ZVZkl935rCxcb4Aqb1Q2LwlXXg0kxQPMHmjWKDDwavON4tFjsUxzi3Vf5J8ayBk8ZPSxRrglEXZeFcM7oFjazJEmkKkarxZVS6idrNJ2jNFarOnmpuQCjJp1/dJxllAYTqEx8dNH9Xv+JIAnIqld6WxqoJQlsz5IvdJC3lRDRniOQliUWGgl235K9XMHpOKtgvE2rLYCWZwNvtkbuZYuezxB8cZvU/icSwwcmOwv9qzLE/nk0eb/Dj3v5W00Ij6KCfLDbWw8O4v/tF7B/6I38pBl/XloA5Y2x8B4wJ8vWcUT7v01BH7ECram/Twje1M17sE+06OOPtoekVPmhNIDXbFHVZQvYQh61EyWpThcr96GUByPVk6Qg90McYDHFFHRzJ1eWs60elCoJgZxWhXFfgyl6r/usezVmzzqTIOS8kRmiTa3zo6nOmlG2TjAyHPtybd7OMcatS6U75MmXxn4pd6E3rWTX+6JnsaQMd5iPP/Hm9ggTGmKC4j439thu+prf/3gWyu1/G9p833KJLrrCnj/5ygcvhTDZofX3BP9SZ+Jfugy8d95NtkjxsGMOfjnUOPUrqOjPvVT3rba1oax5aFQW83Cd1Pp15Olp0mwXVew5oIUXWYhDUGQRNGlFbRvhqqfLReLTGnxJpCmVGMNbZQN7eUF252PNmyTdHl7TtXJXgTIpfRyzwhdNtoGo/yr2iOe3bVusvFirbPjU+Bup+NK+zeWmmBzr4MEdfRmiDErjDDrmYxryawbxRSH1VJzbYEYRxcWuOKy42X4AE93crmPe31zJ+TSPd98M/1StlagO711A7itwxHhv7LTH+2+/9fbr0l2Lwa/HuREiAN4KNPRp44t13Rrnn5MpPTUs+Nul1VS4v95sWazXVeSlJX0pYFxUxhog6dKImQtRgEbVRkgadoCUr9ODwmnx/xvEElsUq4VAv1NUeiAyG9hczrzZKRDjTO09rvWsPu1DAOLeZ+rnVOsttmp68UGYkMzScsm0L5eOjOacyKNsDwfNFipp0YT0ywVRSZL0m6VQM6+3+xaM3zD/fVRkezOLxuybKy7i/X75/tBtGuh8GvS6RTdckV1jRjoTrYNwR/hdzxP2v2+DvOfy/1hZ9Yc34A7+8obfDz/36Lxns9WWYzRUyU5iS5w5eShJrCRfPsaKtkyWbMggWFKIZS8RvIaTCFFGjEQ1AqjaFqCdK1Jw95VVbwGZP4EKupLUqyccWiYqgJKai6UnIi4sLDmYx1BWEYx1Fr2yStlwgojFjSoIHmpLIsHMHL1+W7n2y6HgK/UbNouL1tKXkn/QJsBkZdpsBRGoAe/zgzZ7kwgjq6GPH0Q8JvNG7PIz9u6Zb3t9fwTysf+hN/M9ZEvG6xDwP8HDBfD72aXIX4XuKg418OeHkj0TDX4vBBPoThVvcoYGncc1xdCPpKQ2xjKELdj3HDY5F0MJ0CU6KBK2pwmsYZDMayYAudCVc/G2l0aKpUzRECWZMkgmLrMsk600jrJL56ZdT5jtCKHuDxAxWkmxMwJhwauF2pp6WkKMp6cHJ+T8fXdxWKP2gbl7aBlpBomhcOC14A9D1TP7T3fn5XuD7owsfbJuvDP9kzSKZ00g204hhK8j7/NGuo7Ljt2zGLhmXRQB990L52CBXEH6Y7PSfwID3v0/hRJiim92VezaDdrFEkt+dg73OHOup4PMGubzJdTf5uj+utfxLbRHnK/Mex3gf+h64HYkSGz+/rv+kQkMy5dIm0Ufb5xTbUv3nAXazRALmg07TyCELSW8PGr7bu8hMmWjAIFtLkaynkdcwIAcpwEmevFp6yqNG651BLC9jRG8x4GOJZMXTD1dIrLUCVq8QMdUhGagSTPVIG8JoUeupwQHg66dzGoppr87PrAmkZbuKvymYr0UT1mAKmYiLBM4Dt+ghVe7IoSDk7lbq+Hk99lXLF/WzuQP3BC6BwxHYTt4k4f9bEQhsjPNwfCie35vOfRB9L4N+xBf+Zd+q0WeFvLHXfP7Y15OueH/Iev9KDLCv21lwMb0frpmxb1uOXzIePKvesWPqZltSgC4hSAXwXEQKnA84zyTZSRMP2jMGj9u/LBaPc6HgnsBKkmw/h+Q2nRwgB/ktBsJXIAayQh01Bjt8KGbLCLrKZDNzIC+bWZLPLCkQTUmhe/vC7p7gelyvZVKunp5x+tS8tVbESzXiN7fOrvWiXoqSMKIQjECShRjRVRYIWQxmmcNHwiifahVGLqqN3dEavLn6w2Ojge7M4U8HOWOPMawfEyyjr33nv1vPExJn/NOzEOxjwuhli4a1SNwKss8SYq4JeL104aOzKtcubeBgQxj2xRZ8P1vE+0I1+AJp1jXS4cO+ptN/TuHlIekPp+R72xY/3C1Z4ISEKAMus0n4wkxYSX5VtmL0vNXFNMr+OFFNKtFMgrx2JuAzCwhWAGJXwhtVoajVkPVc4UtZ8zOcUIOFJI0VJH0dIDqOkppESYhA87LpeyrFTtZJth6VLc0V01slsm+bxOltzBx35oMs0SPBMqoMYV0aQZcp4jcbCl8ObjFBanyR+zm0gTPKb89Me31F+upp0bNHmXcuSb55vqjr7drR4VY+ZxSbTDQIivIn00+ciajjx7FPm7ivg35OY6UokQOXE4/HsQp8mDt90OZC1Y1BtK27Fkx0q7MnIpT/TAz+d5b2N0HgT8SQeENjrytHb1iMXtXoa1/45qzcg+Oyd2qnXdwlcSKVWeJAi9QGfZeS91khw80OYy12zSHQo2JpdTGCsTjJdhbJRxEIVQJj1aBkYyhWG9yiRbVVFDmTPmebG814AUlnGWikD/h5I7mbWU52gKEewcyArLaSoL6aaGlKvHBUIdEWqvREn24TH33aeOPQdh0awQQlWlBIDjNI/svIGRbguWz6s5MSF+slG2pYJTvp+ZvpicGwryMQ6AIX5Mh87MzHOSgHG//KdyZOYOCye3u3cYcSh85pHnNCfRRFru2zfnJKpaVwUVXs0pPpGoPd530Txa48Sca3C06f/r41+uZ98A8ocnwVTNQv8Nm/jN70G76odv0w9eFZVscF1p3zog/Oij8+K/Hw+LRUd2CDBuCykNjmSe2pXDR6xKjJE3pfKq8uJmLOJNlIk90VSUFK5FgVOEUXTtODcQNy2I9pN1+4Llhspz9TX4GouRDQXQE7WcPZaazCHaKJUVRfNzhyI/VkvcwaNWKUEdQWxTodIcYdfIPxxpvSggxYBEtRgqMMacMysCSA8rBl6qEq+r69onHxaFAgrKsskr+BeqfJuu9n+zutxr/cXcMdvoXx+/g49x/l8AQdu5/5WM/ISA7vXeT7XbMSDITfNHs82yOf6wmfKbQdfNLKG35z5rWNjgcxqkKezfvMn4yP/dMw+I01c3/zVP8rbZgwmRPVi+OjL/OHL+mfzkVvn2M27qVdqBU/mM/MS0SKM2mPLsrcbsI3xIJYTdKtKPGb8dSe8tVH7JBfNk8LUgL1pwlbMgBnKcBHkRy3Ek7TQpJ0wDQz4FQkvSNFykFRxEeL5KAiYq0AGMyDtJcBWsokCxNSWhwtNYLm5QKqLxGxWkba7Uo9Gka/mbsUZywj2CDGGd5pu8pMimAznRCoSXp8VLIsDy3IpwUFQqHrKbqLCTv8GQ2bGFd3MJ/vYwzdUuK8sWO/8x15Edj3MJzTd4XP6x7oy+l9484bSOf+7NlTKPm5zqTnkMIeT7jIT5E/NoobqkHOnYQjUt47RXfftHk70MHl/kE4+c9hMBl3m4xR//2qEPwFYzgb4o3xxz8PtDvtSYBbqhkXz4rv2EpXXS6ksVA41BEMtgcMVaZoLP2pMo12f9O0N/v1mwPhsWbXY/ZoWxC1a+sszs042wUiDjOJ7gtI65WABDU4XQverAftD0BvZ4lutYY7slZuWktVnTHlVKKszWJAZzGgugJYvpSgsxLQXgIazgUy1yHVXpRqf2pX+zZcJI6Mv+LyOfzxkQSVaWsWENoPTCvYSslMpcUGU4I8UFNVcqw+NdkMznQE68LQo+Ho5Qzap0bp0Zt6w3dV2K+sh54ZdN+07b2pcrpMEXsZwrvnzL1kz2l1ao+gbtKCu65sF1wvF3vxsbyPe9UliXHjVbqgjFPgDv6eR/gTGEws7fGfXx4aZ/diAjM32cz9v593Oem+8M+fn1deyJeszKSeOC5eWsww1ybmBlDfVkv21c4fOr1y5JrJx9Pq7lrEi/6MvgbTA85g726NQ1bo2bWMuKXE06G0sUvBASoEF0VC8FIgdhWUYgxucQSj7NEXB1c/r9b0VBOO1IA91MBQU2KsJuy7CjJYRNRUJBgrEQ0WEq9tk9vlgux1o+5yog2+PMWZzHkJwlZs3siTm3Wzk+ORyFj8QVtjBHgYoybLiNF6ULwBmOkA7Q+hHAik1AVR724Tq0+Gfzkm98up+a0F6O4gsO+Cz/2KxdwbDuw286EmjRe5oiUW+OJg8Pq7x7FRNtb78FPp1qYZNfcW7ruxBncdPOwP8mt/DgN80kfGuoJiFU5diu0duoHxB3nYGJfL+Z8FCpMvxtica4fNtidQ9uxkebmTt2WxrDSI59NFX1ZJduTQn+yS6DkmM3JVc/C4de0a+GmCWJ07eiVC4pATY68Jsk6G4DeH+DJT6njc/NjVUII2lGAAPSmd/6LF+2LJtHRHcqYVeMCHvtkQuVO4Ym/ynDw7JHw1kGWHpjmCXftN9OSEKyIlnlWp7HBGLsQqcriDvewPE5JljM17ef+h6fbtjIQYSkwE1coadLFGjSeOxAhXBmNVwXwbtNgBrXChVPmj5V7I2QTRLevAMh80304QVXxx1P5x0byRE4bdZbJPNjGLzZBYNbitwBl3FfgaPfnUNbqaZb0Rud1bUHXZTMBIJqXzPwsDwSkePF7v0P310fPdgli1Z216+lu/Nhv9j9CKgJyOtR00zs1lbAyj+LjDa4wBA2VCYxTzYjr96U7xjm20x7sluPfcrsVRz3pRPxXN7Sta3Jk+59p6ev0aJEcZsRATavNh3clets0S3WwOhesQc53gNFtgTwC1OVRsmx2ctQY66s4ynD7l6VHzAxlzMtdBKTbkDyfNQ/RJuVZIrgNaFSv54LDqq7aUUT57iDeEsUfZ4w877ursLmdGxyAhflCQB8VeD9VfCjgsAP0XQUFKQOgiMGoFmKgO5hgjxQ7U7bZooh64x4m+2QTxWEiK04Ju5S3faQ2d9ac3uFALDeBoVWh7wCwe5z2GjfaO3W96Zh2+kxaYxRzgPrv5PElATP4ogP1neRFvslJ2aOxVQZWeiT3sHsBsPOWLYSM8bJz3RY5gX10y/nL2qVNWoZEUGxswPJyhtoxgoUzatg4tc0YrfZHDG5Dumvl3S6ef9KdcdqVd96c2OcGHzZADhmiBMhw9CzJmCUUqkz7sVKj0Qn/eLB+vQ76VJplqDiatIZd6U9vjpqcZomazpux2pkTrk58d0NyxnnF+87SyYFaABunwegZuhbZawlWp09k9Bzn8QZxiDg4dvnhWrrSIERND8XaDwwIpRppkvcWg4yLEXg70UAS8FwG+CoDffMBdgei9iBS0CNy4AsJnOU0biVYFPRYQAxYCV2LmWM0SDlxIDl4CBCqCLVmB48M9PB4HJ6yD2LM9N3WC81mxuxVw38zm9PP5/4uR+H/CAJtwL5NzzcNGH76ot3WmWTqg+4458bCR3yWRvpo/Hvd4g6WPH2JrAwf40dWWkMyXAMlGcJIOtMkQTjUFDgZR3DV+2rMWuhJE/yVO7AquZh3pldpouCLoJEncpSt+P1Zhlx0jxQDOMoND1Ym1vqJ3igwPh4nFmCGbzcGT65k/Z4q+LRd7XznfQ0noQpR0pR+1NpIVrkV2WUJsDGU1BoknWQCpzuh4/8nOtwEnGqZvyaCGh6CuuDZ0pZtrQFrLAZ2V0NiHJ70Pz7VXx1d5yKfpM9atELFVnuKsOsVfU8RFSShoFSFRh5xpCoWokNbOI7T4S9vMJrjOBdbMItV4LuUL6laxicOIR88+c808Ku6RQu8cucHGzYMgQMCd7LD7O3vhT+uDr4n7yVnGPvdfNbSEDS2Qxy8KeDz2fzFFgigFr7HJMiCQameD2q5BdFaAlgpguBIYpgSsXwJ5LyNFaJEbNtBKLaBL62mfMube82DU6aIZK8mRy8lpK8FL9mJJK8G85YxaA7FSY3q0Lrh+FSl8NSlVFy6yp1R4IZdT6Z27xD8dkO7ZN/1RjrSl/JSttuC7PVNf7ZgaqUtyWEhoiGCciRKLtwO3b5KMDEPWB4DhgdQ1JsA6XGbrALoqkNlqdODDcT734ejn0rHerb2P7Ede+o93hfHeRgy2Gw6cVv/coPShQrarTLqzTOJGhmipI8VnOcl9AdlhHnmtAjz08h5H0Eg6NtHPO3Dk0ZodJ1RDC1ifOc8njp6ZPGSS8/cDRt+m0TD+ZNOSAJOx/KIFmlqAV8BUNvcN/7eCp4kqNC6n4ZiVvz/V2hwx0APMDBETBXD9AjAA3/LzgYAFIK6Sbm8Ry9AkXfGid8VIXLajHtVFT9pT3myUeOAuWmtKsZ4u7CUHeMuRAhWBgJWkUCUgVR3JMIJLHNGDvtRTEbQHW5k9VdK9+2U/HZZ5UcZ6s0f03R7Rm5sZjT6MeDXYbRVxtw/VTwd0XYs4u6P+/jSdVSQnA4qRMqS3lGStLfKiVYvTmffputbF3dTPl1c3bUIHO7TGXuoP3VDpOSbZd0ym56Bkd5VUZ7nYjSzqk3yxPHswRg1yUSB6KQJXS1Nw1jOOb3YuV3DeEjb6Zvx0WCHjSIfdKK/3d8f2/IGe/dP+4Hdf8CYPE+3tvamnDWtoAJcvRfCxYf5kvFYQcsT5wHjDUXM/P6qlCaylRTY1RQyUQOfFsN8iyHc+aD+NaC9NrIukxWqQ6m3Rdj/aNXfaGTvKqzjWw2D6JVt6nhqCo7VOnuQiT/SdB/gtAYKWgJEroHRDeJs1vNuJ0uRHb4ujP9su2rNftq9+TvdB6U91Mo+KWPXhtD1uaKUDzXcFqcyVHqwJ2moC+ktI1itB+xXkdcqkGGuw65TFz1Wyl3IZx1NpNVFIdSRaEYjc3y071mHSd3lGz2nJwTalwfOL+07M+FQn27lH/NkO5r0s1okwRr4e1WU20VMObMsPwbjjnMnIJA+nvGNvR0+l1Eisz5Hi4Fr6t+PRsX8aN/1vf05g/Sfi0uzxd+YGqLYG6OIqNs5+86uZmmzwqz9o7utKMTWENDRI+maQgQY8+LT5zf6MCj/jjUukHKRg0wVCLRFS8UrkKhPKPiNqgxntghvjmB0tcQloJSUSuBCstmelmMJeyoTAxYDfPCB0MRSlCiYaAoVr4d3uyJkwZpU3cjub0b1/xrlMZPyu1WC7yq710C5XtMAZqo+WPBxGKbNnbHGGdwQgR6MYJ6NEj0ax7tfIF26ceSyZdiJBojGW0Xd2VUf1mn3BlIGTyr0nZXrPS3EeObJvmo6cW86+bDbaptt1ULp9M/XqJkZjBC1FHXGWI/lMR16fqZvg4NzJBJzgfgH8ocefqxrv27/uPf472fQHeelvi1UIZvnL+aIYd3TwlaUxoqUK6aymfHh5ZqL+kvvlZhE89sFqIzdHxNwQ1jYEja0QAwOk73WrQLjg/yJ3fPzVk/tV0edj5SOUQZdZhHAFIHEBlLkaiVZH1ioSkzTQEGXAdo5wsglyMWNac6xspi3kvkIkSJmcqAXvdKCUuKBZNnB9JPXN4Rn9rRr5/sThmzrD17Rqw2jJ1uTL5WqH0udnOgHPi6Tb82UqA9FLaeKnE5hVocjgHedYG9KTcqmLmdSWRMqDUtkcJ6CvccmH/VMH2pZwXjt1Xlg4fHU59tSZ89Cq99Si9i3Uc7G01gTmmUTG+hVkF0Wikzw49PahoEpBkHqbUMICRznG4Q+P8ft2HNf78s3faiz+yRgIvpooFsIJwfjttngjPVhNhaypCr950vi15lGAEU6WqvaoOznBJoagiQlkaQFbGKGdrxp+q3eZkH09HXtPJM6u85EsMKKGroTslwD+RlTTuUSPBaTaYLGj8axTsbLrNQhlAUh5rOwvjUvO7VI7mCJTHABvdQDN5gld3My6Xkj/fFY924MwdFF15Jr2gzLx2vTl2e7g1W0y1wuk9/hTdvlScTq7249a6oMcTxDb7MKoC6PXxVIK/cHtLmC5H7Vrv/zLnayummndDbPeNIpzn9jyHruMXFb7eGzOlWz0ZAzlTByjaSPtaBjDewEpQA7YZDKbNzxBPb8ERbGvtwwQpH/Y7OGJQ7n/oVqjb/DJvzbSCKjqwHC7vT2amCzq5EL19ZMcH3/71RbxJmTC8I5CeWdn2NgQtLBAzI1hC3NKx4e6rzlursCf4VyXO9pc6BpiBgeZwMbKZGN1wGgxwU6RuEUfjdYhN8UwL2SynpbJHI1Db2+TS7UjXtu9cOt6+q7EhQcSFwdokW4Xiud6ET8cX14SQB44rzx8ReVDw/woc2Jzivj+IGp9hMRuL1qWHbzXl7rdHT6VJX1ym/qJqKmXtylfLJz/YL9kz2GD5gTGs1LWta20S7loX+tK3hP30Rvqn1vkXu2RuppOa4mj1YZSDoVQG8Po6eagtyKwfi78YH/GRF5k/HcK7Es1z59thP42DASugCcIS7+1XIMEbKBU7l1x5bLt2Ojrryfn876c+cHpigqX8PBATY1BS0vEUAc006N0Pjs64bHxlwpqNLGJ3CuOZmmWncYKku5yspMatGUNWuPOTDKCruQrfji99lgc5Xqe+K3toi/Kpw62O3WfWfbuksX7Y6t8lhNzLSlddQpbPcC39UtqwsGBc8sHLy7+dFoh1ZZcu0F0pz3VV5kUok6uCaG0xNJPbKKMPQqMtSedSWW0plLPZVE+tWknrCE934G7DaR1Czp0RWvslsHnltk4HbqWSbmWSb+cyDy0norvpHIftC6AnqAFec4DfBYi/ffOT87DxPrn/Nc8258b38CLvvjkMXans6eYlh7h0TNTjNeLccawL3UIEzM7sQoGB666u1I9nVBLc8jcHNbXAg3UoI8Pavk83q+1C4IIGu8jn/cR4z6pL5q1y5u+zQq9HCd2MZlZ609PMAKtlv60OxhpzxK9kSV+KYuZuFbkYr7EpVKxl3VybkuJW6yhzto5xcHo69qFhzfCg22qfafle8/PLvFFnJcQ1i4QSTWEg3QIW61w/4GM3g5es0QoUg3XieBWB/LzavlzqdNPR7JyHcDne6SGr2gPXVr1vgantrSrifT2TbQ7uYy6CHz2KeXeaJUvjgEjcBEQsBDKtJLhc0a/NJDw2RxsdGLlfYkL/dnenm/hpgKVxmfn7zQzMgHDI2k//2z0W13UV8I6sSW5L5+XeTmjXk5UKwtYTxcw0of1dND3PRcELfMTO4GDD2yUw+/tfOXz+uaaZ8cWXMxiNsdTygOhDFvyBj1CY7Lc/RKZs5FiyfqQjaKQwyLhTBv4VsrMmxmy5+IkrOUJx6Pp7+pmVm+kvjw4ryEeHmhd2d0o09Ms86pKbrsNNd4IPBHL6KxbeCFvao4bxXk5Yb8HI1aXHG1AvpwnH2NGDlxOStEHftkrM3xF6VPz9Bv51AvJ1BvJ9MubqG/KptaGo+X+aIUPpcwdORZCPerDdJlDDFkM7421EuSmJmdDUPw+/PBBGpf9GuN8S+v5t2g0/D3GuR9dvcR0dEmB/tSH9xy/rILfPk4GSfr37lng5YY4WaNWRrCOOqCrBenpUHpHX2CTx7PgPnt8nM8dGPt48UmjS7QFOcaa+L7du/PMvPbKpR9PLv3l6KJzGZQjEZRttrCzstClLXP3etCilCH3GWQbGYLBDCHLuSKvKmZezKK150u82DfrVAql/9yKxwckOxvEP583dlspst2REmdBOpFKG+3wsV9FSNCHq71oJ6IYu8Oh4fshVgrCQSvJl7Ilx25bDLauuLwFPZWAtqZQH+1gvS4TO7QBrfKh7PZBd3og+/zR9iRmhTMtaBkQvBR+UZc+Eb2fFMC4VxsdHDi1t0aFzx3619T8CkTy4MgjSzM67mMd18DXzmv+jxoQfIZH+weuhIbTQgIpTuao4WpQazWgpQ5ZWDB5WA8mOIe3j9N/Y/BJydU9hqlOULIDuS5BujlOFFe2lkrCNSnMwWsWL2rm7QtBoywIjTGMm4VzK7yRDFMw3ZrSuF48RQ1xUCC7KhO7Di/IciN+qJd7Ui7amkH9dGrOiwPSP1fSB9t1Q/WJhyJZN4vkm9PnOCoLlznTovUATxWRYH2R500mmV4zHBRF9kdNHe+w7TmhdCoVOZWI3tlGe18leS+feSAIrfRG9/hQSr2QKn/KsQjqzXRmqjkUvhoKVabwBvqwL6ttwg/zhj9+LNh7aEZfz+mvnvlPIPFnuSlvovWEPTr6ytyEbmGK6GmTD5Uu5QuOmOZgv94ABRvnYZ3V++SDAlCvtbCpPqSlDRppQppKpHC3acPvd37o8P2lWflWuVTrrhknS5c+OmL0oFZrVwjFz0B4uwtyZINo3jrUQ4UQZUCOMBf70GLaUS27dwMlxQRsipc+tFE8wZRU5cY0mCWywwP9dEQpxZrYd2pFxw46TvY/Ns3oOix3Kh0dvKpdG06LswD8NAhRukCxK7V+I+1UHP1sltjjJuu0dZK2ciLRJqSRm9avaqWuZFE6ttHf7ZN5Uy51Po1aHYSU+6JlXmiRO1zmgxxcT72QRr+xSXSDNjlaDU40n4PxOLzJRiiBR+ayR+/cubPCzR06czT1G2578Wf3wUSjA85l2P3rnCX09EBNdVJq7Eycg3KxMa7gbGN8dYxx2B3nmpcHB6MeToiZLqivBelow3qqoOYS4dPbZkdb00+kzejcvag9RfxR1bynNdKVYVCeD/lkhvir/TMvZbNw5h6gRXRdKZK/lpJiDPtrExKcRK9vmRaqSU4yZ16KnNGwQbrKd4buDOErmWKvSqSyHcm9Jxe1peE0hvHhiFRf09KD4XDf+SUPy6ZbKwpX+VIflq0IMyIcCKBXr6fcqJDPdGPYzCY4LRR517BysH3RwPllvccUug/Our+deTyGWh2IVAgAoJR6ojvd4doN1MPrKffyWecTmaGaQOwK5HishaCOXGCIRnlYX8+HPc31C328ENs1yJ1LOX9UyPJPwOBrBAQbj4pV1tYAbU1hN1fq8+5dHEFF1DgX637TmdTQPHu9P+rqihjrQ4ZqoLk2pK0Oaa4glsVQe08odB6Se1W97MFOxSelcsdikUgTkXRz4HiiTOdp/WMJlCxncrYn6cFemZdlswpcYC9Vwg5/+PbuudkOcMgKsukcIX9VoquyiLU8MXAF8KRQ/EAoUhtG+dS0sCWe0p5B/1A3tb9FpSIQelQh/r5+rstSkW2OaFMs9XWNXIIjlOEEPK63NJglFLoUaoib3nd2cW/zrNcHWTd30I4noEfCKdW4B/ZFK70ouz0pO92QCh/0RCSjNhh9WiR6Op4epQX6zoM+nqicqBpic7nvTpzVcHOHbc1BJzvEfS1zuP/+N9xK8k/7g6/Sm71r1zpdLdjCGNZWI27PEt+ZI9NWuyQrVdLNFbBzAE2NcAdAtjQC1zqgmpqAqhIhdh3wqXZ+f738QPOCwWaF4ZMrh06uGmhe9Llh/oeyObjxDdEmXdm8/MVhxw/H5PbEQ5u8Ra6XSY3eC7tbOfVoAiXeENSX/+n9UUEcYpMFRU9KZJ8H/dkOsSQb0tPiqV21cxsi0NvZzNf7mH2nlesjKHvDoO6WZckmoN9KYs1GtCYBOZUhvVEdsp0rkqpBcVMSeVEh1ZJCOZNAOxKFNEZQ9wWglX7obtwH+FHKPCkl7pRid7RuA/VoOPV8PO1VsWhDODVaA3SaBzwsCZ7wxuy3b5PjUmhebrCvA2OtPSU1finGGfmz8/ktGHwFgvviRYW2KqK2gmxuAuEwpKcwfTygddaglRHZzIjosRaO9afFR7BWaZBUlEUyPODPtUsGaud9PjK/98jc3vo5vbUzumvE3u1hdFWLvt8r+rZ6xj5f2vrlZHsFYdtFQvvDaD0Xl92pZJ1KoTan0LLWAfE2YFfjqqpwZIc9Zc1sotNi4t0MsVubWNEmxJ5GpSc7GQeC4evZjKfVkh+blc4k0bc5A5/OLDoWzvJVJZaH0940WxvNEApbDiZoQp5KxNv5ij8XS+4Lhg8FUw4EUPb5Usv90IpAAQa4E8Z3QKkHussTORpOOxSM3MpgvCoWK/dEk7Vgm8UkH2vmwPBdnFc3HzeMS6K7uqJOVvS1Vqyhj3exbzoG45tjFVweNhoVsxynOsZGOPcHDfUBZ1e4IF+irHRqzR6p3ExRWz2y1jKi8QqRlsxpn47M/lw/o79BbvDkot6jMu/3ib2sYDwpYd7OZNaHU5oSKadTGPXh9Dxr1FOJ5DiLZDqdkGCF+9ipTTGMg+GURzVzuy7YF/lBGWaI7xKyqTRhuxPyII91wJ+SbEPubV7Wvpm2xxe6mEl/WCnzfK9k+1bRTFvys70yVzJEbecQKtynGs+estOYGa0NeSsRmwJFM9cADTFSd/LFmmKotUFU3OjjOmC3P4IDUOqBlHgiO92RPX5ofRi1KgDG3+h5oViRIxqjCtupkkJ86AlpCuzR9/UHTd3dER0tQFsF6X1zXnDTEu4fhKn/GRj8jnHxcG6AjcTEKWurwbqqsIE2ZKQHmeiCxmpk3WUkzcUiJssIyU7oq8o5PXvkeg/Jf6yX6qqV/rR/Vk/dzP4zCz+fVXhbN/3xLubJBCp+zSlGQKg6KcUQzrOgp+vRXJeRrGYSTaQIBjLC0ea0jurVGW6kcD1ytAZsOZPgsYR0IYV5bTMz0xY4GI72nVp8fQtjlxuM25ZX++XPZFBfVUzLsQNrIhhPKuUDVMkui0nFNrRMA8RpGWH/hmkXkuh1G2hxBuQSZ+RDrdLZVGrVerjKj1LlQ6v0QnEMit2RQle4OpCC75KaQOT5drGHeaJZNnC4EmSvBSTFs/yDqFlpS2JiZ1qugQwNIc+10zHeEB/7+yWN/0QMfuWfgrA5rguHjzWG6amBWivJGkpErSUE6xXEXA/0+m759/XTOw/LduxgnU+mnIjEKTZ6IAgu94Xqw9DjcdS2zcx7JTN7jy3sOTLreZl0eyZzvz81xQRyVSBZyom4zwf9ZiEOM8iOcoCtFNlClhBtiKZZiNnOJtspEss8qG1JtMPBlARz4OnuqR+PzbiSwajEpWw80nt8+aGNSHf94lx7MHct0N24JMMCNp1BSFiN+iwipVrAz8tm3CuU7tgz70S8aIIuOcmI9KRoxvEEaqUPgtNQXA+XuaNFzkixK1rtL3DRdcGUl9vF7uWyMtdAAQtARy3IyRnJLhBPiKHb2EA4Bk5O1NwdqyZOHvgWAL4RA+yrSMd4oxycIYy9f7RLqSVT9nTGzHtFsz8ckP94SPZdueSzYlbHdvrtbfR72xn388XubpN6UTHj51LpExnMCBNCsAYxUo8Ub0oqcINaEugdeRKvd0+9lSt6OIS22RwOWQo5y5EsZhDWyBLXzCRaSZFMphHsppPNZAhxJuDVTaJnYhnpFuQ4U1LX8bkv9rGupjGrvdDDEfDgad0yP6izdmaxC7TZAnp3QH5vENVISthSguC7inAjf/aJGHTogtHrw9K38xhtSYxEfSBMjXQihn46jlHmKbBFRR7wTje0wgM3bmi5B9ocSXu8TaxjKyvLHHZSBCxXQVaW6FpXqKJUPG8rKymBZW9D2Vuo+aVV5F+zDybeZfKQDa7gMFjewPNDq8+l038uYt3aTr++jfp6L/NdDfPNHuaHKrGPB6R6Dkh9PDAV/6K3bubnpjlD51aM3zFnd9h3t1nXp4hbL55iJi/ku4QUqwGmmYH5TtCBIFqVH3W3G7XAhrLJFEk0RKK14Ch1JGA+bCNJClhJelQqdSiMss+PkmoElHkhXbWSd3fSz8fRD7lTD/ojw+eNd3iS7+QzzsTRE03JrZvFLmdIOsgTDWcJDVx2OJ9ByVkLvDiscrd89v1i5oMi0ZvZEsXr0MCVhP1u9KubRcu8kSI3GHcGu9zQXR5ouTvaFEU5m0q7lMZKNYaclch6c8hmqwVpQSs9yM+J6mCBWBih0cEKE6eocr60of21GHzp0mJ/TZPxeu+WHYqiN4RTbmxmPC0QfVLEeL6b0XNoWs9h0e4KZk+V+Ntd9F9K6B/KGR/20HsPSQwemzfUPH+oRWH0+mrshSe/K3r4YeT17WLqM34ynTvFeykpbBUYvhqK0YLiDaF4YyjBGA5Xh7yWkI0kRIKXgA+yJe8UsPaHUDKswXg98t18qXvF9Jt5tEof+IA7tdwdGmrVPxpBPRiEvCqbnmBMrg6EH++esVGXtG6J8OEY6tg9z7NZlENh6IFg9GXFzPYs1oM8yfZM1s1s0fUaImE6hAd58k+zZWsCKLg/KHZDypwoxzZScXlxPIKRboy4LgOC1MQ0FHHnB5tpIDaaqKkGbKyNpm1ZhivTL513fzUGXzvlJtOYAltUFTqzzBst80NPJzFa4mh3MpnPixi9NTID9csGmxYPHl881LxspGX1SIvm6FmdkVOqo6fVRltUh08qDTQpfD4+Y+Cs/PD1Rdgvvvyujby36SUhLHNFIbOZwmvlyG4LQPeFoPMc0HomSV9aOEwFrAujvdkntcsDLnKipBqDW83BD9Vyt7MZHVnMHBvgiC891wH43KL8slQmzZLUtX9hijG5xAXGlfPIOdO+Sg3X+YRMe2D0usOFTOoubyjXCbiRLbM/kNoaLXotXexNjWzHdpkcO9h41k+3s+VbEpg7vaFSV1yvUUvdkXIvNNkI9FQCMU6/f9Ri1dWQnjKotwLUU4VMdemdnU3YpDz+F9iiL/fEnYRCkC3o3+xAL7BGCt3RPHdwbzB6KoZ+O5fRc1i278iCj7ULuw7Kdh+a2Vc/p79pyeCJ5Tge/c2L+puX9DctGGhYMHAMB2nR0PEFgyfmDZydNXZLnftwHee+283ieUF6oKbUFJOpxDWS5DUyhKjVcKE78v7Q9EOhaKkDJd0YxjFoDKfdyWV25DAfZIummpJObGCmWwJvj8x7Vy0bqU94XChR6g7VhFHGrzsMH1PvypS5EyDmtZiQbIMOtVk0xqKNobStFlC+PXzQm57vCvSfX90Yj5MF+vkEyVAtksU8oZ1rqY3BrJZEZueReZ+aF/c2avquArChD+PYyKP7RzaYKxipo2Y6jLbWUEwQK/stP/vXYjDpCb70HAs+DiSZU9L1kUwrONMOLHBGCl3Qg+HUPSFwsQ9U5ALWb6CciqPiWvRkHOVkHNqWjt7fwXhSzHxYyHhWTP+0X3Lw2MKhpmWDDUo4JIMn5g61LB46u2Dspg77jltvi3XlxtkbDIk4icx1AJ/tnn45QzzbEs7SRzfrIxlm4PlExuVNtPsFjI5s1hZLclukGG58HpfP7twrs9FIuD4a/qVKgX3DbuS0enfJ7HZ/yikH6hZVyGchKduZ9alZ90gUuteLGrSaUO5AzV8HDl5Wr4tADoVTH+1bmOMC4E4iwxxyW05YpyyUYE2sCERwAeG7irTfbz67/2dBjJLD5Y72cDl9PN4Yh/Pr/Zy5f22sYsL8cCZbnHAqJsjDcIdTTFix+lCGJZJhDW+1RrZYoxnWSLoVnGYKpZhCaRZgph2U4wDhbG9/ALXaT2CIG6Mp13DnsUP0474ZHw/Mfl3Ger9H9NMBmb56ub5D8/qOzhpoWdQYS9kfC7EfWXMerR25Zvq8bsXLQ/N3rQcybcjx+qQEI1KBO1ARBN4tknh/Rv1No272OtLVZNE4I9KtrZIf98t8OKY9ckGffd5uvNV8qFbtfprM/Q30a67M7auhxGWQoaxQS8a8h7tn43I6bw0Stpy82w0euqJ1PJpS7gO/aVDOcSIXuUGnknD2PP1cxrz2rZJVfujZBIngVaRYFeRkgtzw2xYujz1ZQyWoPBfcPXWyB/VbNMLfwgD7kpnjTbb2CZ4IEvCTzwVvhL/xCB8b3WQoHaYKpuogqfpwsjEUZwxuNASi9MBYPTDVAN5igWZYwmkW0CZLMMcBLvdGG0JpbUnMK5uZrWm0kwmUK+k4K2U+2sG6m8+4vY12O5feUUC/U8SItyAeiaWN3TcfbJ03eH72eIfR2G2jsXtrPl8weZIlPdigN3begX3ZZ6TNjHN/Hf9VxGiH35kEarIhsNcXHW4z4933Z1+1Gji8rDt/6oe86fc3su76MC670IvU4UxlxFmOrCo15XKO/I1sqWIPuCmStUGL0Fu/5F6RIm6+3p9QLfAE9wegHSVij6rkzm2Ve7J/QUOy+MloerwukLYKKbBAbmbLfX51CMPYX1pfsfEJfzDR9CRo5MQx+a0e9A87M/8WBoKjF7HJIl/eAJ/Xz+f18dmdfF634IHh3xkVHIaGjTw9mu6/nBy4DEjUQGI1oY1aUKwBlG6CbDKGcWa5yQze7ogWu1IrvWl1IYxTG1mHQ6gVvmiJB1LgBB8Moh6Pop2KpzbFoFc2M86nUK9sol9IZ5S4IUkWQNfBmYMXtPpPKX1skHlzYFqpH3QokfLu8MzdDsDH/Kk9eVKdOVP79y7rOziTc8eB98jvRcX0dGMw0xbkdHiNXzR7Vyh2P5n2NIr1OIp5K5B23ZV+2ZGetwrcpIwYiBHU6SLqkkKXM6Y9LJIsdoPzbeBoI2J1MLM1mfX+zMorO8QL3aAr+fSupmUVAfDVolkX8qUqgig1PswsPbTQDlfR0MMdc9gfb2GcIQ6HM5ETxKeMO3Gw9iDGHZvcD9gkAoJPf+9WeX8DgwmrP4JxxoZe/1yh27Vft++IaV+jxaeD2q9L5t3JkXtZueTT1SiM3Ys76UrXWc4LyP7LwOhVcNQqOFoNTjdCt62h7LCl5tqim63gJFMw2RRMMgY3mYOJZkC6NYj7j1xbpNgFqfBBGiKojZHU+gj0bCr1XBL9oC91izV4OJx6KAwp8CBvdwOvZ0+9mCWaYkFOsiY/yJmaoUE8v47S6kg544SecILfbGIOn1AbvajX02Jc7IyuWyzy+bzN8HGt2xG0Nh/KLT/GnRDGdW/abVdGuzMjWxmKWADpihJ0pEgqNAIOw5FIRtf+JTudwKvJ4gUe8GYLIM+D3HdM+0761HI/+F6l3L6N8OlM6q0iyZ3eyNnNon7qxK3W8G53FMf7cf6MkqBpvQ8r+dwePvcDf/g1993pnjNujyv1MXY/nz3K/0phvrU/WZCsYwt6cbkjPRfyzmyaUepD2ROEHAmm5q0FW1KZF7aK3SxehHE/YeMDMSvFXeaD/gvBoGVgwDJgvZLgEbQcCFkBhK8GI9XBRF04UV/Q3LrJBEo3h7Ns4CxbuNiZkmcPFayD6oKppzdRz+VRruWwcuzAthxW6w7K+5rpjwrEt9qBKdZATRQ13pRc4Am1xovnqUP1OpRjumidLnzcFLnlSftUNGMEp7zta/YFUnyXkP1VRT5Vq79NEb/oRbvsQbvsSW/3pt/xZF5xZmxeAYYtAA1FiVYzwLXzQDMqSY0lsk5Z5Fmm7M9ZotucgbMJzGMhjJ0OSKgmIVaXnLsGOuhH2+WO1AXQmtezKt0pbstEYnWgKn/qfh/qzQyxhg3UhxlSb/cuf7dfrXO/xrsDcr2Nytdz5wgwmIhe/Hr6xTdiMKG/J86sZ/OxkQ9Ht8gfTmFW+KNHI+i7vNAENTBeCc7VknjfdvztmYNWsmQneZLbXJKXAtlvAeA1n+wxF/CaB/gqAoFLwcgVcKI6EqcJR2qBggOrDcAEQ3CzJYSz76NRtNMptFs7mbdKGYc2omczmB9OzP58YVnvqXmtW/E3gqoDqDtdKbh7v7hFTOBa1MFydWS/DnpIBzmqj7Y70C8HUcdOm3PueJ7bQo3SApxmEb2WEpqDmGf86e1O9Auu9Eue1Jue9FYn2pZVYORS0F6WbClNTNNAdxmxjKVEVESFVCSE8mwpz3bIXcsR3+WB1PnQCx2hq4liVZ7UbTa4XYUyrMCdLmi6EVBtQ3eYTyx1odzOEH1ZMRfnYy93SCcaEmN0SWnm5L3u0Ocjqz+3J/J57K9xnT++jfPfxAD7chgSF7dwAubF5XC67zdEsU5H4eIF2RtCzbdBg1aSPZaRnecD0ar0dfJkG1niWlmS8yzAdQ7gqQB4K4Cuc3EkyDgenvOAAHyXLAfwPZFgCCcZwP9fe9cBFdW5rVeEmdPbnGkMMICCig07CBZApEvvvQ9VQKSK9N6bCEgRFBWjaCzRaDT2GGNJLLFEEo3p0USNiYLMcM8MgyXvrXuvNybctx7fGliz4AwznP2Xb+9/728XOSIlbnCLBD1RRl9o4G1bSbZK0M86hD8fM7i6UW1/Dr6/gOjbOvl0sVqnhGgOwrcmEoezBX4G7FRjuNIUXW+JtS5FN1ig22yxLc7InSqt/pPO370zp8oTqrLDQwzA5RNVK62wo96ck8H0iRDybDh1NpyuW4ykzobln1Af9tBldTiRe/x4sTNgO3XWUk0VU81xhY7op2tnXF8n3pkibA5AG70wZuzvjCV7JESjP7IpijibKQ6czWaGxdcduiV+4I4k4ssmrVMZvAOp9J5VxPEc6tttsx7e2vKSXue/9hn+6TyQZwH1D5/iy0VlZP0XGo0+Lhc2hKBrbJACWzTHHl5lDsfMgUINoOApQMgkMFgX8hSDHlqA1wQwQB+UzICjZsORs8CImWCMIRhnDCSZg8mWYI4j3ByKfZDPu1Qv3L2aqg1EticRHVF4fTh8br344bF5N7u0s52BCl94bzq9PYVqCkePZfPaAijf6aDEAEqeD+cshOvM8JalzAPdsBTd7Y093DLr2XnJ9iS60Q9p9iY99dguIlbeIuiQP+dkKHU2gnMrUdC4GF09E/EUA356UJgYTNOEimdBG6zxdfOJmEmgmw6wTFN1oWCclea4TAt0Q5h4byTvTKrgcon658Ua5wt1W0I1zMRvpVnA16vFpV5gRxB2tUV3UwzREUa2hqFHMqifNk49mqs1+Pg7qUz6Z/fkEakL6UhgQk6QZM8Gf+07eqJE2BWJ1roQLW5k0gIg1RhJXogkzIHj58AJ85DY2UiYPmInZFvzASdttsdkIMkQLbDAK5zwLHuwVYIfK1Y/Vys+WsQ7kEkfSOeWeyB5TlCJO/xpg+jHA3O2r8bXRSDHSznXWrVao7B6xukLwJvD8aYY5HguVzINtOSzvbSh8GlQyjwkZy5asQhbZ4q1mWCbrdCPEuhHO0weH7DfGIG8LSHK7QhXDXbodKDTDj8eSp2P4PTF8dvMsbxZqJ2AFSuGC8bDpbpQyxR4lzH+zmJygw3e5EWUmWPRumCoGuROA1a06hKeygLhOBP1t5ZovuU0UTXfnHg7jPtBMq/IBtqzStBXq7srDd+XTTND5HgqfaNO/dPa8Vd7M+UV/bJ+RXcrpXDNG9PxkldBPfllT6KAcbU6Y8n2EIJxcBLMwKTFcKoJwmzF3lNAlwmAoxhwEgHOatAybVULLRVbLVbWQvxAMu9YEb03l96cTDaFoFlOYLoNmOcA1/rCm6LxtUHovmze41PL9pVwm8PQGj90UxzVHU91xZHNIXi5L3y6htcaQtqIVNzFkL0O23ESO2IKlDQVYUZAgRlWswhrNkU3OSB92cIHrdN/7py5Kw7vDiZXzoG99diVFujJIPpsEHU9ltdiC1fOxixolaQJSKYQzBcARVwwgwbSRKy1M6Dt1tROOyJfD86YDBbOQ3MWo8VWeJk1UetGbAijemI4jb54nj2cawdeyVc7k8djGGp3JF7nj+xMpM4V0n1NervyzGX9v8peM7/l9fzkQdmjT7rtz5SIMqzASGN2TyQnwwxcZQjHz0X8Z7I99QH/yQwRQspdiEZnzvZw/v5IDUsdFWaCu0xhHcwW7Ign272IpiCUmRAMKeqMwe/tW3CmkisPbEjgb3ZNuPeOcUcIkeUI1Pij7cFkbSBaGAJealc7X6hhq6MSpAcF6cEBkwBffcBVEwgej0QZwCkmSL4xUmIMNzB8yQO/nET/UKn1eKfN7kS83AELnArkzoeP+3JPB5PfV07d5oOXzsVdBYCfBjtPHSzjQJkYWKiGtE/HiieAGWIgRawao8ZucicrvNBSZ6TBB10fhnVF4m/HknsTaYaS9iZQl2sEbRLkfAXvWotoRzp3jS28I5Toqxu/Pm6i7OkvilTbvyzXUSZfj548fXR+R7Jgbxx39wpBSwh+eBW9zhuPMwTXeVGxpkC2I1zgCR4t5u3PolvCsc5E9HQZP9octBivYjZ+XFsgVeeGHqsU3N2pVhUCtsYgnzTRpyt57SFkZxjVKIHbJVi1G9oYhDYGo6Xe8PZk6na7VmcMx1Zb1V0biJuNRBtC+U542Cz5+ZqjFuikw47Wh1fPQXOM0YJFSNUSeL8n9Vkifb9V53ajoDuMDJ8JhE1hb3TBT0YwJJW6niRcb4NF68AOCCsdgwpgKBRgZerAnc74jQK1zwqEeyK57YH4sQxegwe6cxX1bbfON60G10pFZwu5fTVqd9eK765Tu9kovFjDP5TPaY9GqzyZdY88lydanzBxcOAnmbw67bU7gL1mvEhenvzg4saAC/nqyZZA7GKg1h/dFc9rcSWz7YAL5eJvNs/6dpvexRa1d7LInWlUmR+0K4M8mS0ssMeXa8l9otoAvDUavbt1wnt5dEsEeqqMdyiPU+KOZFvBxS5IRyjB+FnVAcimJGJ/Hq87nracOG6JuorPdLDQmgybz05dCnb5U5W2hLs+20MfdNVhu6izQ3ShVXPRnIVo7kK42hze54V/W8a9t2XpkXRemgXkPoGdbYJscsBP+NJ9CcJNjHtohIaK2YEkK5oFJ0BIEgeO1Qd6V3A+qqRP1fA+ruYzhPj7runnivnlnmCtB9IcgK0LxvLcwHIf6FAW50wx92az8HYr/1a18MtyrcNpgg+aLWX9D6XPlEpBf3HOr6Luo/+X680SvUNJaoyr1eRLxC5iZy4Hj2Xr5NvCfjNVUm2Byw2CHzaPP10mXC/BD2fx14fgmyJIhtV4zQQcDVT3pXOvNgvOFPPqfdBGX6wtmCx3R8qckRrGWUvl9Kwi3s3k9a4USIwgI+Fblhqq8YZIgSOatxxNNYca3dGdQVR3KO09g+U+HvDTYh7s5RqqLrpA5DQ4dR5StBBtNIPv5PK+a1u6K5UjD3bOBN20WIlTkFwjZLMrudmLbLfGG4zwfC0kDYOjcDBFC5ZMBCXz2T1R5IVS3oHVxA+b5/QmUiUe8LZE8mwF/0Qef1sM1REq3wI3RGK98URvIvlJofBIDv9oxbTvz5QNybvTPhsW7vsPgtevWyOuqBcYGvztztm2KO3jBWqlrtimYG6VDxUxGwyZAYbPhlz02eHzwLfj6S9atU5V85ok6NF8PrO8Vnti3VFcFz1WfQh+s0t4vpy3PhDrjMJ74zntEXilN7w/l3+zXXNtBB60AFiipmIjZPszq7klxnCwKju0zAQpnw+3LUH3uBN7vDgrdYF0GsniwlkiKEkEBqoBziKAYcZJBkiFIXI6murLm1zmD11t1s8xh8PmscIWsZfpjLNWV/XQYxeYYA0LiHVGVPFU0olmBWpCodMAhj2vNITW+2Lna4W1gXClB3y5RHimkLctWV6vuSWK2BPNOZHC/aRE41C+5u7VwuP1NveudUmf3pdJn0iH+hX9vv4ZAX1zNpA+UygEKsRIfv2mOWJqqSsn3RILmQ9EzoQTjbFIE2xDhKX05+/frQ3PsEUu1Yjez+MWusINvsTWeDrXEW5ype0mjjucyfuokHcij3sok2aW/pYQ9ErLhENZWl6z2CZCFVM1VdfJ7HRTtMASr7DBmu2IeiO0ehpcMwlq04fXTQLLxEANF06HoWwKLOaALRSax0eC1QEnMStsEtC8ED8Ty1nvSpR5wbsT6GwbqNyTuLlhEbNoJBhDzuPZDmKWvzbbS4/FeLyJi8B1PpTnRFU/XSBsOpRgCHeHUMUu0O1WzS3x8mBwlBFY5sm50RN0Y2PQnQNFt080PLzVK/39+6HBAcXRjXSkNlJR5fgfTYTXPcMZVHbNGN4env72+PaFi71lCcu43x5Ye+/K4YdfXhx61q/QpXz69Ufb4xahH2YLe+M4uQ5wezR5Mletwg2LMATdp7HaGArvB631x3Yncj/MFyXbIYs0x1nxGceC5TmVVemOtUdhbaHomqXsfAsgzxAsnw6V6IKFOkChGpgCgeGQarY6UjkRL+XDq2F2LKqawIUCRUD4dHb9EqQvWeykq9IRQFY4Yu8nCQsdMddpKvtj+D0xlGQ67CZmp8yHsy2hQ8m8z8pF12rVLlWpS4zYzOLmORFMXAC9s0IuaRK3hOWqzXKepLLaDjnX6DU08EhRfTYwnEIxsvE+k8leO9n9T9rgBYbfVV6iLq/H+k2eaimPUilVEOW7k/TJg88ORyyADiQJmJ0j1Q5a7QBVeKOtgbSDLqs+kOrNoPcn8ytdyWVaKtYito0aYKWummvKzHrupULhV3WiGyXCs5n0nRr1L8vFVQ7Qpwn8E6H8NANgpSbYNpPIngSk6wIV4+FKNSCPAnI5sJuAlTAL6l5G7fdSc52kUmmPRxqxLzfMTjSBcsyIhfy3tsfS0fPBBBPwWoXoWpVwVzzR4AWXuLH3r8G+3ih+J4X2naPqOokVOhe4XifuXcWp8yB2RPPKvbGUZcTjzz8eGl6JpcNtDt9YH9Q/a4MRMHf8FZGY4Ro56cDjB9f2+c8HO4O5WbZIhh1c5onlM9uvM8d5uuoirbfMRCqmPFV7ddBJE7TTZicuRtuC6Vw38GgBfbyQszUB+aiI+146N9RYpT0Ae28leSSW3mBPZsyCVs8DCpfAsbOBPV7cyiVQ+GTVtKlIjAEUOBmI0gHNBeNi58MJc6GQuar39iyMNAbWLCDNBOMOJaonmoJHc3gX6rgX6uieFPROk/rdWt2DKznb4rDbrRpfrdMsX45GzAAiZwPBc9jMjIwxgvMdiFgzqv/e18rdUHkooxz+f76z1JuxgUz2xydDw9FCeaekZxd6C0ONiBJ7PN4USLdEqr3wEg8s1xHznAo6a4GO6pDjeNBnCjvPFumUED1J+Mly+oMi6uMq+nIN9/10qjOcqHJDrtVo3mrgnc2h2j3R9Fngbl+6zhVduRhc74HfKBIeSeOlm8plMMKmgT7abFdtINgAjJkKJSwDrjSKmFnoOZ0lMYBbnbkMu/1us+7NFrqvhfd5veBsEa8zDN8QQDT4YkVecEc0sTOB0xNJbYogWoLwEhesYDle6KH98+V9I3WMz/4dydLXwpvRN301RC4dqY0dHB4ozNp0/9y+KBO8xo3MMEeSlyDJpkiqORpqADtpAg7arGBD9sFstVOFvCu1gmv1wo+reOcq+efLeJcqeVfX8o6WkidrOZdauKdriZst/GOr6SJHeHcKdb1O1BFG1gWgJwuoT8q42bZgxHyg0h2vdsMZA/hPBhOnIdsS+Lc7NTZKiCRrMMAATDOFDxaIftqp/eN24XdbRJ/U8XZnku0SvIGhXvZE8XK0xBlZ64M3+OAbJJwmxl9Lnv39keah3x/IiYhcnFEmG8kg+q+zwQhkQy/C5cMFmnIJb0XF/pNfLr8bZojW+5Dx5lDsDNR/AuQiBL1EcOhc9ldder25nKoArMAOTTKDVtlB2W5QuQ/Sm8g5XyO41SG62al9bT3/o1rOlXrevmSyyAlulWAflvGrfVHmDl5t5N9uF5wpEKy2gRif8Wq1xkpT0GcSK2wa0BGOfdEuPLiGV+qKRhlCreHE/QMTfn5P74sujdYoNN0KyliGZFojOTZYrhVeaEOWO3K3rph+sCa0b1/FwM/yjkXD0Tf5WjvcavUlHZA3hb9I51c6IpQxoMwBkOs6DD66csJtPpDvhMfMRJy1WXZaLBd91qEswa40KnoR6M0svrOhgJmgtyEYbY1GWSJRS+AVi+FUa7DOH92bpf5Vt+b1Dv4HRZxWP3x7LFXth+Qsh+oD0G0Z+LY1WG8qyZCuFCuoM5g8mSpMs4QzHKGueN7GJF5bBNXoQQbNA0p94Z/26L9fxF+xhL1iHtLppnOxJ/fuyea7JzoeXD0ycO/O4JOfFPr5/YrEEZnslcw5ZRD0jzpZfxp/iQ2GP6fiFGNQmQqjOJWTPRv85erJuKlkrjkVZ4h4T5BLYfkYqmZawcVOGLNjr3FCm6JEFw7nbNxhU9U6MSCC9PPDI13wOAss2RxdZQU2hWFXqtUvVKm/HU9sjSTagrGOSPSDYvpoPudgDtUajTLO4FovrMYTznSC17jDjd5EvT/e4E0UO2PhC4B3UwS9q3hxRtD2BPP7147KBn7v7x+UjrQ5k44E/BU0X954SyZf/uWiLC9OAv6v2OB/hZJCDEoHH93v8J2XZkbVutJdfrw2X87HuVoXKyZW+JIHS82kT75jxuBT6cAz2dNHT79+/PTO7R/2P/jxaP/DL7893lTsyS90JxnnvNYb7ZYQR9Loz2uEfU1qd9o1bzQLr9YKL5QIPy0XfdGh/WmjaFM0FTCHZT9lnN1klXQzLMEELncgVixGb+5IUpB96Rthln8ef3efQJmys+Sg7Ncf+3ZEb0zT25AyviZK/FmP5+CjW0PyxJxng8oudszzJ8/FbBUrw1N5Ts3gg/sX6veu1i9wp4pd8QpXTJ60YQ/Hm7PjLNhxCwHFCSvbcybLYaKqywTAa7w81l1hTQbNAhOMqV9O9DKU+XnD0lE3wNDfZoPn/6p0aLBfLo7QL5XHuZ7KV15FbfNwu71BxbQfabs3IBfJlQ6r1cp3lQGlEMGA4qiceeGvjC9+pcurJ8e0I9O4p8hsa97Syy3+t7uSvu5e0+iikW9FFthgqRZwizc3diGS4zJ5qP83udzoy1Pg/48NXoZSXWY4aVI2cnA9nKmpYCBDSgUCRfBFphRfUKTav1pnIf/9gFKaQVEoOaTUgJHXT//+5am1QRrF7li2HZZqTV/fXTz07HeZoqb1uaTJfwn+fhsMj+kXN3K4lGGE9r3owyR7hYe/xEn++Bj+kikvGJlI8unz+72fLvWc6sj/9eb5weH+eAqVnjdKLN8ARsEGsheZyTJFBFAqHclXHhx6lXqM2GE45/75TJFnnsmzPaTDYj2yl6+VXyWfHIPPlRtkyreQvpTp88Y4zZvAaKxFym/PJ4Ts1WEv+4MhlPd55GcyZS7n/0xxVgYwn18xpOhOqzzYGvkD/0LfbzQwSj2s5Xjt1ogvLvs3Lx7J0XndN/mbMYo2GIMSYzYYfYzZYPQxZoPRx5gNRh9jNhh9jNlg9DFmg9HHmA1GH2M2GH2M2WD0MWaD0ceYDUYfYzYYffwDW0UZwBNBaLIAAAAASUVORK5CYII=</t>
+        </is>
+      </c>
       <c r="N12" t="inlineStr">
         <is>
           <t>Administration &amp; Operations</t>
@@ -1661,7 +1689,11 @@
           <t>Mercy Corps</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEAkACQAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCACEAXYDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD3+s/WtXt9D0m41C6P7uJche7N2Ue5NaFeR+L9Ql8YeNLTw5ZufskMu2Rl7sPvt+AyB+NROXKvM7sBhfrFW0tIrVvyRY8J+IdTtvFEM2sufI19PMiBPCMGKoB6DAx+K16pXnXxR0tYfDmnXlovlnT5VRNvGxCMD9VWut8La0uv+HrW/BHmMu2UDs44P+P41MHZuLOjHxjWpRxdNWTvFrtbb8DYooorU8kKKZJLHCm+WREXpljgU5WDKGUgqeQQetAW6i0UUUAFFFFABRRVe7v7Swi828uobdP70rhR+tA0nJ2RYorj7/4meGrIlUuZLpx2gjJH5nApml+NdT12dBpnhuc2pPNzcS+WoHr0OfwzUc8b2udf9n4nl55QsvPT87HZ0UUVZxhRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFAGF4w1v+wPDV1eKQJiPLh/324H5cn8K4j4R6QZJL3W5gS2fIiY+p5Y/y/Wq/wAXtUMl/Y6UjfLEhmcf7TcD9Afzr0Hwjpg0jwrp9ptw4iDyf7zcn+dY/FU9D3WvquVr+aq/wX9fiO8V2P8AaXhTU7XGWaBmUf7S/MP1Arzf4Ta59m1SfR5W/d3I8yLPZ1HI/Efyr2BlDKVPIIwa+a3ebQPErtCdstldHb/wFv8A61TVfLJSNcnprE4athn5Nev9JH0rVbUb+DS9OuL65bbDAhdiOvHYe9Gn3sWpadb3sBzFPGsi/iKoeKtMl1jwxf2MHM0kfyD1YEED8cVu3pdHhU4L2qhU0V7Py11PC/E/ie98Tai09wzJbqSIYAfljH9T6mum+FeuXkWvDSTI8lpOjMEJyI2AzkemelcE9rPHcm2eGRZw20xlTuz6Y9a9p+HXg59CtG1G/j239wuAh6xJ6fU9646SlKdz7bNZYbD4F0rKzVor9flvc7qimySJDG0krqiKMszHAA9zXnXiT4q2lmXttFjF1MODO/Ean2HVv0FdcpqO58bhsHWxUuWlG/5Hoc9xDawtNcTJFEoyzyMFA/E1xGs/FTRtPLR2CSX8o7p8kf8A30ev4CvI9W17U9cn83UbySY9lJwq/RRwK0PDXg7VPE0oNvH5VoDh7mQfKPYep+lc7rSk7RR9HSyLD4eHtcZPb5L/ADf4GjqfxL8R6mxjgmSzRuAlsnzH/gRyc/TFS6T8PvEXiKUXWoyPbRPyZbolpGHsp5/PFeneHfBOkeHUV4YRNdgc3Eoy34f3fwro6tUm9Zs5a2c06PuYGmorvbX+vU5PRPh3oGj7ZGt/tlwP+Wlz8wB9l6D+fvW2dWtY9dj0YA/aGtzccdAoIGP1/StEnAyeleXeFtUOufFjUr1DuhW3dIz/ALClQPz6/jVu0LJHn041cYqlWtJvlV/n0PUaKKK0PNPn+Xx/4oWVwNWkwGIH7tP8KZ/wsDxT/wBBeT/v2n+Fc7N/r5P94/zpledzy7n6WsFhrfw4/cj6K8G6w+ueFrO8mffPgpMemWU4J/Hg/jW9Xlvwf1PKahpbN0InjH/jrf8AstejatfppmkXd8/SCJn+pA4H51205XgmfCZhhXSxkqUVu9PnseR+LvHmtQeKL6303UGhtYX8pVVFPIGCeR65rE/4WB4p/wCgvJ/37T/CudlkeaV5ZDl3Ysx9SaZXG6km73PuKWX4aFOMXBOy7I9w+Gmt6lrml3supXTXEkcwVSVAwNuewrD+I3irW9F8SR22n37wQm3VygRTyS3PI9qu/B7/AJAuo/8AXwP/AEEVzPxZ/wCRui/69E/9Cat5N+yTPAw9Ck83nTcVy9rabLoZP/CwPFP/AEF5P+/af4Uf8LA8U/8AQXk/79p/hXOIu+RUBxuIFejj4PX5AP8Aatt/37asY+0lseziFl+Gt7aMVf8Au/8AAOb/AOFgeKf+gvJ/37T/AAr2yS7nHg5r0SH7QNPMu/A+/wCXnP515x/wp3UP+grbf9+2r0bULc2ng26tmYMYdPeMkd8RkVvTU1fmPAzSrgqrprDW31srdvI8U/4WB4p/6C8n/ftP8KP+FgeKf+gvJ/37T/CuarrPB3gr/hLIbxxffZvs5UY8vduzn3HpWEXOTsmfR16OCoU3UqQikv7q/wAhkfxF8VRNn+1C3s0MZ/8AZa6vw78WHkuEttdgjVGOBcwgjb/vL6e4/KuZ8U/D/UPDNoL0zx3VpuCs6KVKE9Mj0965Gnzzg9TH6ll+Npc1OKt3Ss/69T6mR1kRXRgysMhgcgimzzxW0DzTyLHEg3M7HAA9TXG/C3VJL/wp5ErFmtJTECf7uAR/Mj8K5L4oeKZLzUW0O1kItrc/v8H78np9B/P6V1OolDmPk6OV1KmMeGvtu/IveI/iw4le30GJdo4+1TLnP+6v9T+VcJd+K9fvnLT6veHP8KylF/IYFY/U13mhfC3VdUtkub2ZLCNxlUZS0hHuOMVy806j0PrPYYDLqackl5vVv+vI5SLxBrMDhotWvkb1Fw3+NdTonxS1qwkVNQ239v33ALIB7MOv4g1o6h8ILyKBnsNSjnkAz5ckezP0OTXnlzY3VpfPZT28iXKNtMRX5s0PngODy/HxailL5Wf6M+gE1VPFXhuWfQNQMFwV+RsDdG/XawOf89K8hufHHi+zupba41OaOaJijqY0yCPwrpfh74U8SadqceoviytGGJIpvvSr6be31NXvih4T+0wHXrKP97EMXKqPvL2b6jv7fStZc8o82zPHwv1PDYt4Z8s4y2bSdn2bMXwl8R9Sj1qOLW7wz2c3yF2VR5R7NwBx617KCCAQcg9DXyvXr/w68axTaY+mapOEls4y8crn70QHI+oH6fSlRqfZkVneVJR9vQja26X5/wCZt/EDxS3hzRglrIFv7k7Yeh2AdWx+n1NeVf8ACwPFP/QXk/79p/hVPxTr0viPXp758iLOyFD/AAoOg/r9TVHTNOuNW1K3sbVd00zhV9vUn2HWonUcpaHo4DLKGHwy9tFN7ttJ2/4Y9P8AAl14n8Tfabm91m4js4hsRkjQFn6/3egH8xRXf6NpVvomk2+n2wxHCuM92Pcn6miuqMLLU+SxeMVStKVKKUeisv8AI8V1wnXvijLCfmV75bf/AICpCn+Rr3kAAYHSvBfBP+n/ABItZW53Tyzfoxr3qs6Gt2ehn3uSpUVtGP8AwP0Cvn74hWn2TxvqAAwsrLKP+BKCf1zX0DXjPxdtvL8R2lwB/rbYAn3Vj/iKdde6Tw9U5cXy90/8zpPhNq/2vQp9MkbMlm+U/wBxuf0OfzFehV4N8NNSOn+MreNmxHdq0DfU8r+oA/GveadGV4GWeYf2OMbW0tf8/wASI20BmExhjMo6OVG4fjVHXNf0/wAPWJur+YKOiRjlpD6AVU8VeKrPwvp3nTYkuJMiGAHlz6n0HvXgusa1fa7qD3t/MZJG6D+FB6AdhSqVVDRblZXlM8Y/aVNIL8fQ1vFPjbUvE0xR2MFiD8luh4+rHua5mgAkgAZJr1/wF8Pls1i1bWIg1ycNDbsOI/RmH9727fXpzRjKpI+qr18PltDRWXRLr/XVmT4M+Gsl6I9R1xGjtz80dt0aT3b0Ht1PtXrcEEVtCkMEaRxIMKiDAA9hUlFdkIKC0PiMbj62MnzVHp0XRBRRTZJEhieSRgqICzMTgADqas4jk/iH4hGh+G5I4nxd3mYosdQP4m/AfqRXJ/B213XmqXhH3I0iB+pJP8hXI+MvETeJNflulJFtH+7t1PZB3+p616d8KbE2vhNrlhhrqdnH+6PlH8jXMpc9X0Pqq+H+o5U4y+Kdr/5fJI7qiiiuk+VPlqb/AF8n+8f50+O2eW1mnUZWEru+hyP50yb/AF8n+8f511ngrTf7W0/xDaAZdrIMn+8rZH6ivOirux+nV6yo0vaPZW/NFTwFqf8AZfjGwkZsRzP5D/RuB+uD+Fek/FbU/sfhdLNWw95KFI/2V5P67fzrxRWaN1dSVZTkEdQa6zx94h/t6/09lPyR2cbMo7O4DN/QfhWkZ2g0edi8D7XH0q3RXv8ALb8Wctb273MpjQchGc/RVLH9BUVdb4N0zz9M8Q6iy/LbWEiKf9pgf6A/nXJVm1ZJnpU6ynUnBfZt+Op7D8Hv+QLqP/XwP/QRXM/Fn/kbov8Ar0T/ANCaum+D3/IF1H/r4H/oIrmfiz/yN0X/AF6J/wChNW8v4KPnsN/yOqnp+iOHiYJKjnorA17CPi/o4AH9n335J/8AFV42AScAZJrQ/sLV/wDoFX3/AIDv/hWUJyj8J7GNwWGxPL7fptrY9Xi+LmkSzJGLC+BdgoJCd/8AgVdjr3/Iu6n/ANekv/oBr59tND1db2AnS70ASKSTbv6/SvoLXv8AkXdT/wCvSX/0A10U5yknzHzGZ4PD4arS9h1eut+qPmevWfg3/wAeur/78X8mryarFve3doG+zXU8Ib73lSFc/XFc0Jcsrn1WPwrxWHlRTte353PcPiTqNpaeD7u2mkTz7nakUeeWO4EnHoMda8Hp8sskzl5ZHkc9WdiTXXeG/h3q2uGG4nUWlg4DeaxBZ1/2R/jVSbqS0Ry4SjRyrDtVJ7u9/wDJHYfC1G0/wfqOoyqQjSM491Rf8c15FcTyXNzLPK26SVy7se5Jya+jbvTIbLwldabZR7Iks5I41H+6f1zXzdVVlypRObJq0cRWr111a+7Wx2Hw20ePVvFkbToHhtEM5U9CwIC/qc/hXvFeN/CCdE1+9hYjdJbZX8GGf517JW1Be4eLxBOUsZyvZJWCq5sLM33202sJutuzzig349M1YorY8RNrYKRlV0KOoZWGCCMgilooEeBeO/CreG9YLQKf7PuSWhP9w90P07e1coCR0r6E8eJpz+EL06l/q1XMRH3hJ/Dj3z+ma+e64asFGWh9/k2MnisPee8dL9/66hXr/wAK/DP2WzbXLpMTXA224I+6ndvx/kPevPvCPh5/Emvw2mCLdf3k7jsg/qen419DxRRwQpFEgSNFCqo6ADoKuhC75mcHEGO5IfVoPV7+n/BH0UUV1nx54J8NTt8eWOePllH/AI41e918/aXINB+I8Yf5Vgv2ib2UsVz+Rr6BrChs0fQcRK9eFRbOP6v/ADCvK/jJF/yCJu/71f8A0E16pXmPxjx9j0njnzJP5LVVvgZyZK7Y6n8/yZ5bY3LWWoW10n3oZVkH1BzX0Xrmv2ehaK+pXDZTaPLQHmRj0Ar5src8ReJbnxA1okmUt7WBI4489woDMfckfliuanU5Ez6nMst+uVabeyvf000Ketazd69qct/ePukc8KOiL2Ue1Z9Fdr8PvCB8Qaj9tvIz/Z1s3zA9JX/u/T1/+vUJOTsd9arSwlFylpGP9WN/4b+CBiPXdTi/2rWFh/4+f6fn6V6pSABVCqAABgAdqWu+EFFWR+e43GVMXVdSfyXZBRRRVHIFeZ/FLxV9ng/sGzk/eSgNcsp+6vZfx6n2+tdf4s8SQeGdGe6fDXD/ACwRH+Nv8B1NfPV1dTXt3LdXEhkmlYu7HqSawrVLLlR9FkOXe1n9YqL3Vt5v/gfmNggkubiOCJS0kjBFUdyTgV9L6Pp6aTo9pYJjEESpkdzjk/nmvIvhZoJ1DXW1OVMwWQyuehkPT8hk/lXtVLDxsuYriLFKdWNCP2dX6v8A4H5hRRRXQfNny1N/r5P94/zr0X4Pc6xqX/XuP/Qq86m/18n+8f516L8Hv+QzqP8A17r/AOhVwUvjR+hZv/uNT0X5o4/xTpv9k+J9QswuESYsg/2TyP0IrHJJ6mvSPi9pnk6rZakq/LPGYnP+0vT9D+lee2ls95eQ20QzJM6oo9ycUpxtJo2wGIVbCwqvtr8tz1jw7pv2D4RajMy4ku4Jpj9MYH6DP415DX0Tr1qlj4Ev7SIYSGwaNfoExXztWlZWsjz8krOv7aq+sj2H4Pf8gXUf+vgf+giuZ+LP/I3Rf9eif+hNXTfB7/kC6j/18D/0EVzPxZ/5G6L/AK9E/wDQmqpfwUcuG/5HVT0/RHEQHFxET03j+dfSy6vpm0f8TG06f89l/wAa+ZaKzp1OQ9PMssjjuW8rct/xPpz+19M/6CNp/wB/1/xqLXGV/DepMpBU2cpBB4I2GvmivoqX/kQH/wCwWf8A0VXRCpz3Pm8flccDKm1K932PnWu28I+HF8R+FdbgRR9rheOS3b/aAbj8en5VxNes/Bv/AI9dX/34v5NXNSScrM+mzarKjhJVIbpr80eTujI7I6lWU4IPUGvT/hb4r8uT+wL2T5HJNqzHoe6fj1H41Q+KPhr+ztUXV7ZMW122JQBwsv8A9fr9c1wEcjwypLG5SRCGVlOCCOho1pzFKNLNMH6/gz6mIyMHpXzf4o0Z9B8RXliykRq5aI+sZ5X9OPqDXtfgrxOnibRFkdgL2DCXCD17N9D/AI1H418HxeKLANGVjv4AfJkPRh/db2/lXTUj7SN0fM5ZiXl2KlSraJ6P9H/Xc8R0LWJ9B1m21GDlom5XPDKeCPxFfQOh+JNL8QWqzWN0jORloWOHQ+hH9elfO+oadeaVePa31u8EyHlWH6j1HvVYEg5BwfaueFRw0Po8wyylj0pqVn3Wuh9P3t/aadbtcXtzFBEvVpGAH/1681uvi6sWtutvYibTF+UMSVkY92HbHsa8reR5Dl3Zj6sc0iqWYKoJYnAA71Uq8ntoc2F4foUk/bPmv8rH0Xofi7RvEKgWV2omxzBJ8sg/Dv8AhmtyvMPh94BltZ49Z1eLZIvzW9u3VT/eb0PoK6fx34lHh3QHaJwL24zHAO4PdvwH64rojN8vNI+cxODpPFqhhHzX/P18jzv4neJv7V1j+y7Z82lkxDEHh5e/5dPzrgwCTgDJNKSSSSSSeSTXcfDPwz/a+s/2jcpmzsiGAI4eTsPw6/lXJrUkfZ/usuwnlFfe/wDgs9F8A+Gh4e0BTMmL26xJOe6+i/gP1JrqqKK7opJWR+fV6069R1Z7sKKKKZkeFfE3Tm0/xlLOowl2izKR69D+oz+NeueFdXXXPDVle5zIyBZfZxwf8fxrnviloh1Lw6t9EmZrFi5wOTGeG/Lg/ga5T4WeI1sNSk0e5fEF2d0RJ4WT0/EfqBXOnyVLdz6arH69lcZx+Kn+S/4Fmey15d8ZG/c6Quf4pTj/AL5r1GvJfjHMDeaVDnkRyOR9SB/Q1db4GefkivjofP8AJnmNFFKqlmCqCSTgAd64T781/DXh+48SazFYwZVPvSyY4jTuf8K+htO0+20rT4bK0jEcEK7VA/mfc1g+BfDK+HNCQSoPttwBJOe49F/D+ea6iu6lT5Vd7nwecZg8VV5IP3I7efn/AJBRRRWp4wVT1XVLTRtOmvr2QRwxDJ9SewHqTUl9fW2m2Ut5dyrFBEu5mb/PWvBPGPi658U6hn5orGInyIc/+PN7n9KzqVFBeZ6eWZbPG1O0Vu/0XmU/E3iK68S6s95cZWMfLDFniNfT6+prNs7OfULyG0tozJPMwRFHcmoQCSABknoBXtPw78FnRbcapqEf+nzL8iMP9Sh/9mPf06etckIupI+xxmKpZdh/dXkl/X4nUeG9Dh8O6Hb6fFhmUbpXA++56n/PYCtaiiu5Kysj8+qVJVJucndsKKKKZBxzfDHwwzFjbT5Jyf37Vq6F4R0jw5PLNp0UiPKuxi0hbjOe9blZmreIdJ0NN2o30UJIyEJy5+ijmo5Yx1sdn1rF117LmlK/TVhrmgaf4htEtdRiZ40fzF2sVIOCOo+tZOn/AA98PaZfw3ttbSiaFt6FpWIB+lZVx8W9BiYrDbX03+0EVQfzbP6Utt8WtAmcLNBewf7TRhgPyJP6VLlTbuzrhhczp0+WKko9v+Adte2kN/ZT2lwCYZkKOAcEg8GuU/4Vf4X/AOfWf/v+1dFpeuaZrUXmadexXAHUKfmX6g8itCrajLU4YV8Rhm4Rk491qjK0Lw7p3hy3lg06N0SVt7BnLc4x3qprXgvRfEF8LzUIZHmCBAVlKjAyeg+tdBUF3eW1hbtcXdxHBCvV5GCgfnQ4xtboKOIr+19pGT5n16nKf8Kv8L/8+s//AH/aj/hV/hf/AJ9Z/wDv+1R3vxT8OWjlImubsjvDFx+bEVXh+LmgyPtktr+If3jGpH6NWd6Xkemo5u1zLn+9lz/hV/hf/n1n/wC/7V1JsYG0w6eVP2cw+RjPO3G3r9Kp6R4k0jXFzp19FMwGTHna4/4Cea1a0io9DzsRWxMpKNeTuu99PvON/wCFX+F/+fWf/v8AtW3oXhnTPDaTppsToJyC+5y2cZx1+prXrk3+JPhaN2Rr9wynB/cP1/KlaEddjVVcdiouCcprqtWdBqmmWmsafLY3sXmQS43DODwcgg9jXM/8Kv8AC/8Az6z/APf9qk/4WZ4V/wCf9/8AwHk/wqRPiP4UcgDVME/3oJB/7LSbpvexpSpZlRjy04zS8ky1ovg3R/D94brTkmjkZSjZmLBh7g10FUdO1nTdWQtYX0FwB1EbgkfUdRV6riklocVedWc71m+bz3KOp6Pp2sweTqFpFcJ23jlfoeorj7v4S6HM5a3uLu3z/CGDAfmM/rXR614t0bw/dR2+pXLRSyJvUCJmyMkdh7Vmf8LM8K/8/wC//gPJ/hUS9m37x24X+0acU6ClZ9k7f5GRF8INJV8y6jeOvoAq/wBDXUaN4O0PQmElnZL5w/5bSne/4E9PwrPHxK8KHrqTD628n/xNaFj4z8O6jII7bVrcueArkoT9N2KUVTT0sXiKmZzjatzW9Gkbtcj4k8BW3ifUheXeo3SbUCJGgXao9sjua66itHFSVmefQr1KE+ek7M85/wCFP6V/0Erz8l/wrtdD0a10DSYdPtAfLj6s3VyepPvVHXPGeieH3MV5d7rgf8sIhvf8ew/HFc0fjBo+/A0++K+pCZ/LNZ/u4M9KUczxtNcyco/d/keiUVyWmfEjw5qcixm6e0kbotyu0f8AfQyP1rrFZXUMpDKRkEHINaKSex5tbD1aLtVi16i0UUUzEbLGk0TxSKGR1Ksp6EHqK+ePFegzeGPEMlupYRZ822kHdc8c+o6fhX0TXOeM/C8fifRmhXat5Dl7eQ+v90+x/wAKyqw5lpuetlGP+qVrT+GWj/zKPgPxlH4isBa3TqupwLhwePNH94f1rzv4n6kt/wCMJIo2ylrGsOR/e6n9Tj8K5dHvdG1Pcpktry2fHoyMKrzSyTzPNK5eSRizMepJ6muaVVyjys+owuVU6GKeIpv3WtF2v+gyu8+GPhv+1dZOpXCZtbIgrkcNJ2H4dfyrhoYpJ5o4YlLySMFVR1JPAFfR/hrRY/D+g2unoAXRcysP4nP3j+f6U6MOaV+xGeY36vh+SPxS0+XU1qKKZLLHBE0ssixxqMsznAA9zXafCJXH1Q1fWbHQ7F7y/nWKNeg7sfQDua5DxF8UdM05Xg0oC+uem8cRKfr/ABfh+deS6vreoa7eG61C4aWT+EdFQegHYVjOso6I93AZHWrtTre7H8Wavi7xjeeKLvBzDYxn91AD+rep/lXNqrOwVQSxOAAOSas6fp15qt4lpY27zzv0VB+p9B717P4N+H1toGy9v9lzqOMg9Uh/3fU+/wCVc8YyqO59JicXhstoqCXol/X4md4C+H/9n+Xq2sRA3X3oYGH+q92/2vbt9enpFFFdkYqKsj4fF4upiqjqVH/wAoooqjmCiiqeragmlaRd38n3YImfHqQOB+Jo2KjFykordnG+PvHZ0MHTNNZTqDLl5OohB/8AZv5V4zPcTXU7z3Eryyucs7tkk/WnXl3NfXk13cOXmmcu7HuTW74M8MN4o1nyHZktIRvndeuOwHuf8a4ZSdSR+gYXDUMtw7lLotX/AF+COdAJOAM0hGDg19M6domm6TbrBY2UMKAYyqjJ+p6moNZ8NaTrts0N7aRsxGFlVQHT3BrT6u7bnmLiWnz2dN8ve+v3f8E+dLO9udPukubSd4ZkOVdDgivcPAvjVPEtq1tdbY9ShXLgcCRf7w/qK5iw+EEpv5Pt+oKLNXOzyR88i++eF/WvRNH8O6VoMPl6fZxxEjDSdXb6seadGE4vXYwznHYHEU+WHvS6NdP67FfxT4mtfDGlm5n+eZ8rDCDy7f4Dua8G1vX9R8QXhub+dnOfkjHCIPQCtDxxrr674muZQ5NvAxhgHbaD1/E5NY2m6fcarqVvYWq7pp3CKOw9z7Ac1nVqOTsj08qy+nhKKq1Piau328v8yrRX0L4d8FaR4ftkCW8c91j57iVQWJ9s9B9K1b/RtN1OAw3tlBMhGPmQZH0PUVSw7tucs+JKSnaMG497/p/wT5ohmlt5llhkeORDlXQ4IPsa9f8AAXxAbVJE0nV3H2s8Qz9PN9j/ALX864nxz4QPhfUUa3LPYXGTEzclCOqk/wAq5WOR4ZUljYo6EMrA4II6Gs4ylTkelXoYfM8OpLrs+q/rqj6lPQ18vXf/AB+T/wDXRv519E+F9Y/t7w1aX5x5jptlA7OOD+oz+NfO13/x+T/9dG/nWtd3SZ5PDtOVOpWhLdWX5kNFei/CFFfXNQDKG/0YdRn+IV3njPw5p2p+Hr6V7WJbmGFpY5lUBgVGevpxURpOUeZM78TnEMPivq8o6aa37+R4LZ3lzYXSXNpM8M0ZyrocEV794L8Sf8JNoK3MgC3UR8udR03eo9iP6189V6h8HJH+06tHzsKRsfrlqKEmpWIz7DQqYV1Wvej/AJ2sU/i//wAjHY/9eg/9DavO69E+L/8AyMdj/wBeg/8AQ2rgLbm6hB/vr/Opq/Gzryp2wNN+RFRX05LpOmzoUlsLV1PUNCp/pXhfj/RrTRPFUtvZLsgeNZVjB4TPUD24/WqqUnBXOfL85hjKjp8tna/c6b4Z+MLgXqaFfzNJFIMWzuclGH8OfQ9q67x/4lfw5oObZsXlyxjiP90fxN+H8yK8Q0id7bWbGeM4eOdGH4MK774xM/8AaWlqfuCFyPrkZ/pVRqP2bOPF5dSeZU3bSV215r/M82kkeWRpJHZ3Y5ZmOST6mtC18P6xfW/2i10y7mh7OkRIP09azlIDAkZGelfRXh7xLourWEC2F1AjBAv2YsFdOOm3/CopwU3qz0czx1XBwjKnDmvv2R88SwSwzGGWJ45QcFHUgg/SvojwhpL6L4XsrOVmMwTfJuOdrNyR+HSrWo6FpmrTW817aRySwOskb4wwIOcZ7j2rSrop0uRtnzOZ5v8AXaUYKNrav9AooorY8QKKKKAPHPi8tkmt2XlRKt28Jedx/EucLn34bn6V51XTfEC+N9421Fs5WFhCo9Nowf1zXM159R3kz9Iy2m6eEpxfb89S1puoTaVqMF9bhDNC25N67hn6V2q/FzXgmGtbAt67GH/s1buk/CzTb3w9Zy3kt1DeyRiSQxsMDPIGCOwIFRyfByEk+VrMgH+1AD/WtIwqJaHmV8wyuvP99q1pqn+hzlz8U/Es6kJJawe8UP8A8UTXM6jreqau27UL6e47hXf5R9B0Fejp8G0z8+tMR/s2/wD9lWlZ/CPRIWDXN1d3GOq7ggP5DP60OnVluKGZZVh9aSV/KOv4njCqzsFRSzHgADJNdt4d+GmrasyTX4NhaHn5x+8Yey9vxr13S/Dmj6MB9g0+CFh/Hty//fR5rUrSOHS+I4cXxHOS5cPG3m9/u/4cy9E8P6b4ftPs+n24TP35Dy7n1JrUoordJLRHzc5yqScpu7YUUUUyQooooAK5L4lyNH4GvdpxuaNT9N4rra5zx3Ytf+C9SiQZdIxKB/ukMf0BqZ/CzqwMlHE03LbmX5nz1Xsfwgt0TQL64AG+S52k+yqMf+hGvHK9R+EOrxo97pMjAPIRPED3wMMP5H8646LtM+0zyEpYKXL0t91z1eiiiu4+BCq2oytBpl3Mv3o4XYfUKTT4bu3uJJY4Z4pHibbIqOCUPoR2p08Qnt5IW+7IhU/QjFIpe7Jcx8tk5OT1rvvhJbJL4qnmcZaG1Yp7Esoz+RP51w93bSWV7PayjEkMjRsPcHFdN8OtYj0jxdCZ3CQ3KG3Zj0GSCD+YH51wU9Jq5+i5jGVTB1FT6o98ooor0D84OO+J9sk/gm4kYDdBJHIh9Du2/wAmNeEV7J8WdYit9Fh0lXBnuXDuvoi+v1OPyNeN1xV2uc+64fhKODvLq3b0PZvhFKz+GbyI5IS6JX8UWvH7v/j8n/66N/Ova/hbYtaeDvOcYN1M8oz/AHeFH/oJ/OvFLv8A4/J/+ujfzp1PgiLLZKWNxLj3X6nSeBfFFp4W1G6ubuGaVZYvLAiAJByD3Ird8TfFE6rpc1hp1k8CzqUkllYFtp6gAevrmuHsNKuNRtL6e3G42cQmdQOSmcE/hnP0zVCoU5KNjsngMLWxDrSV5K3/AANAr2/4Y+H5tH0KW7uozHPesGCMMFUH3c/XJP5VhfC/TfDuoQPLLaiTVbZssJW3Db2ZV6e31r1atqNP7R4Oe5k5XwsYtd79fTyPG/i//wAjHY/9eg/9DavPY38uVHxnawOK9C+L/wDyMdj/ANeg/wDQ2rzxVLMFUZJOAKxq/Gz3cp/3Gn6HpU3xivmQiHSbdG7F5Sw/LArgNV1S71nUZb+9k3zynkgYAHYAelav/CDeJ/8AoDXH6f41bs/hv4nu5ArWAt1PV5pFAH4Ak/pTftJaMigsuwl5U3FfP/gmZ4U019V8UafaopIMyu/sqnJ/QV7H4+8Kv4m0hPsuPttsS8QJwHB6rn3wPyqTwf4LtfC0DOX8++lGJJsYAH91R6fzrpJ54baB5p5UiiQZZ3OAB7muinStFqXU+bzHNXVxcamH+xt59/v2PmG6tLixuHt7qGSGZDhkdcEVDX01qGkabq8Wy/s4LlccF1BI+h6iuK1v4UaZcwPJpMklrcAErG7bo2PpzyPzrKVCS2PXw3EVCdlWTi/vX+Z53ovjXXdDkXyL15YB1gnJdCPQZ5H4Yr2zwv4ltvE+lC7gXy5FO2aInJRv6j0NfOkkbwyvFIu10Yqw9COteh/CC5dNevrYE+XJb7yPdWGP5mlRm1KxWdYCjPDyrxVpLW66nsdFFFdh8SFFFFAHzNrchm1/UZD1e6kY/wDfRqbw1pv9r+JLCxIykkw3/wC6OW/QGl8T2jWPinVLdxjbcuR/uk5B/Iiux+EekGfVbrVXX93bp5UZ/wBtuv5D+dcEY3nY/RcTiFRwLqr+XT5rQ9gAAAA6CloorvPzoKKKKACiiigAooooAKKKKACiiigApGVXUqwBVhgg9xS0UAfPXjTwzL4a1uSMITZzEvbv22/3fqOlYVrdT2V1Hc20rRTRtuR1OCDX0pq+j2WuWD2V/CJYm5Hqp9QexryPXfhZq1jI0mlkX1v1C5CyKPcHg/h+VcdSi07xPtctzmlWpqliHaW2uzL+mfF+4igWPUtNWdwMGWF9mfqpBqvrPxav7y3aDTLRbLcMGZn3uPpwAP1riLjRdVtXK3Gm3cZH96Fh/SnW2hateOFt9Mu5Cf7sLY/PFT7SpsdSy3LlL2vKvv0/OxBa6heWV39rtrqaK4znzEchifc969j+HnijW/EKTJqFvHJbwDH2sDaWb+7joT9MY/GuX8P/AAq1C7kSbWXFpAOTEhDSN7egr1uwsLXTLKOzs4VhgjGFRf8APJrWjCSd2eTnePwlSHs4JSl37fP+keV/FHwrJDeHXrSMtDLgXIUfcboG+h/n9a80r6mkjSaJopUV43BVlYZBHoa8u8TfCkvI91oEigHk2shxj/db+h/OlVou94l5RnMIwVDEO1tn/mZHh/4pajpVqlpf24vokG1HL7ZAPQnnP+ea1L74ws0BWw0rZKRw88mQv4Ac/nXAXvh3WdOcrd6ZdR47+WSv5jiq0OmX9w4SGyuZGPZImJ/lWftKi0PTlluX1Je15V9+n52DUNRu9Vvpby9maaeQ5Zm/kPQe1XvDXh+58SaxFZQAiPO6aXHEadz/AIVvaH8Mda1ORXvkFhbdzJy5Hsv+OK9e0LQLDw9YC0sItq9XduWc+pNVCk5O8jnzDOKGGp+zw7TlsrbL+uxdtbWGysorW3QJDCgRFHYAYFfMl3/x+T/9dG/nX1Cehr58ufBXiR7qVl0e5KlyQdo9a0rpu1jzuHa0ISqupJK9t36nQ/CFFk1rUUdQyta4IPQjcK5zxr4cbw34glgRT9kl/eW7f7J7fh0/Ku2+GHh/VtH1e9l1Cwmt0eAKrOOp3Diur8ceGx4j0CSKJQbyD95bn1Pdfx/wqVT5qfmbTzGNDNG1K8JJJ/5/I8N0LWbnQdXg1C1Pzxn5lzw691P1r6L0vUrbWNNgv7R90My7h6j1B9weK8C/4QjxN/0Brr/vkV3Pw6g8R6FevYX+l3S6fOd25hxE/r9D0P4UqLlF2a0NM7o0MRT9rTmuaPmtUZfxf/5GOx/69B/6G1cBbf8AH3D/AL6/zr1H4neHtW1fXLSbT7Ca4jS2CsyDgHcxx+tcZb+CvEi3MTNo9yAHBJ2j1qakXzvQ7csxNGOChGU0nbuj6FooortPggryb4q+J/MlXQLV/kQh7kg9T/Cv4dT+HpXrNcH4w+HEGuSyX+mutvfNy6t9yU+p9D71nVUnG0T08pq4eliVOvstvXzON8K/Eq90SBLLUI2vLNBhDuxJGPQE9R7H866m/wDi5pSWbGxtLmS5I+VZVCqD7nJ/SvNNR8Ka7pchW60u5AH8aIXU/iMiqEem30z7IrK4dv7qxMT/ACrmVScVY+qqZZl+In7bT5PRkMsrzzPLIcu7FmPqTya9Q+D+lyB7/VXUiMqIIye5zlv6VheH/hprGqzJJfxtYWmcsZB87D2X/GvaNN0610nT4bGzjEcES4Uf1PvV0abvzM4s7zOl7F4ek7t726ItUUUV1Hx4UUUUAea/FTQrJraHVwrJdl1hYqeHXtkeortPDek2mjaDbWtmhCbQ7FjksxGSTRRWMUvaM9nEzk8tpJvqzWooorY8YKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACjFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB//2Q==</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
           <t>Marketing &amp; Communications</t>
@@ -1741,7 +1773,11 @@
           <t>KKEC</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEA3ADcAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCAEMAmUDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD3+iiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKZIWEbFBlgOBnqaAH0VBa3Ud3CJYzx0IPVT3B9DU9JO4BWPqPiKx05zGzGWYdUj5x9T2rO8R+Ifsways3/fHiSQfwew9/5Vh6b4dvtSxKR5MLHPmSdT9B3rmqV5X5Kauzop0Vbmm7I0z42k3cWC495f/rVoWPi6yuWCXCtbOe7HK/nUK+CrTZh7qcv6gAD8sVm6h4RurZDJayC4UDlcYb/69Z3xEdXqaWoS0R3CsGUEEEHkEUtcP4a1qS0uRp9yzeSx2pu6o3p9KXXPE008r29i5jgU4Min5n+noK1+sx5eZmX1eXNyo7Ca9tbc4nuIoz6O4FNh1GzuH2Q3UMjeiuCa8uG6ViQGdu/c0EFGwQVYdM8Vh9cd9jb6orbnrVFcX4e8RyxzJZ3rl42+VJGPKnsD6iu0rspVY1FdHLUpuDsxaKKK0ICiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAoorP1fWLHQ7BrzULhYYV4BPVj6Adz7Ur2E3Yv1Dc3ltZQmW6uIoIx1eVwo/M14v4h+Kmq6hI8Wkj7BbZOHwDKw9z0H4fnXHxW+q67dN5Ud5qE/ViA0jfie1ZOquhjKuvsn0C3jXw0hwdbsj/ALsob+VPh8YeHJ2CprdhuPQGdRn8zXi9r8N/FN0A39m+Sp7zSqv6ZzV0/CjxMFzttD7Cb/61Lnn2F7SfY9zjkSVA8bq6sMhlOQadXgSeEPG+hSiW0tbuMr/FaTg5/AHJ+mK2NN+J2vaLcC08QWLTgH5jJH5MwH0wAfyH1qlU7opVf5lY9OvdKuBcveaZcfZ52++jDKSe5HY+9VZ4PEt0nlGa0gU8F485qfQfFekeI4t1hcgygZeB/lkT6j+oyK2qHTjLVM6Y1NO5g6d4WtLNxLOTcy5yC4+UH6f41vYAGBS0lVGEYKyFKblqxaTFLRVknC+MbVIdRimRcGZDux3I7/yqbwzoMdyn228TdGf9Uh6H3NXfFFm19qGl265BkZwSOw+XJ/KujiiSGJI4xhEUKo9BXHGinVcnsdUqrVJRQqRRxKFjRVA7KMU2a3huEKSxI6nsyg1JRXXZWOW7PPfEmlR6XfJ5GRDMCyqf4SOo/Wu40yVp9MtZZPvvErH64rlPEbHVfEEFhByU+Qn0J5P5CuyijWKJI04VFCj8K5aMUqkmtjprSbhG+5JRRRXWcwUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAU9S1C20rTp767fZBCm5j/AEHueleE311rnxH8RkW8LMi/6qLP7u3T1J9fU9+3YV1vxEvbrxD4jsfCWmsGYMHnx0DEZG72Vfm/Gu+8PeH7Lw5pcdjZp05klI+aRu5NZNObt0MZJ1HbocroHwp0nTwkuqMdQnwMofliU+w6n8fyru7e2gtIVht4Y4YlGFSNQoH4CpqKtRS2NIxUdgoooqihO1QXdla30Jhu7aKeI9UlQMPyNWKKAOB1b4XadLKLvRLibS7xPmTy2JTd+eR+B/Ciw8U6v4cmTT/GEGIidkWqRDMbHtuwOPyH0713tRT28N1A8M8SSxOMMjjIYehFRy9URyW1iOjkSaJZI3V0YAqynII9QafXLR6ReeFpGl0ZZLnSyd0mnFstF6tCT+ZQ9e1dDZ3kF/apcW0okibow7HuCOxHQg9KpMpO+5ZooopjK72yveRXB6xoyqPrj/CrFFFIBKytd1ddKstwIM8mRGv9T7CtauQlQ6p428qTBhtgDj2Az/6EazqyaVluzSlFN3eyL/hzR2s4mvbrJup+Tu6qD/U1v0UtVCKgrImUnJ3YUUUVZIUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAVHLIsMLyucIilmJ7AU+uf8cXTWngrVpVOCbcxg/wC98v8AWk9FcTdkc78NrJ76XU/FV0hE9/OyxZ7JnnH48f8AAK9CrI8LWP8AZvhbTLQjDR26bv8AeIy36k1sUoqyFBWiFFFFUUFJmud13xKNPc21qFe4/iY9E/8Ar1zcba3rLHy3uJh3w21R/IVzzxCi+Vas3hQclzPRHo2aK4mHw1rkY3pdLG3oJmz+gqWLWtX0aZYtViaSEnh+M/gRwfxoVdr4o2E6Kfwu52VFQW1zDd26zQOHjboRU1bppq6MWrC1QeyMN013a/K7/wCui/hl7Z9mAHX8D2xfopgNVgygjp706qd7qNpp6BrmdUz0HUn6AVhTeNbdSRDaSOPV2C5/nWcqsIbsuNKctkdTRXHjxu2fmsBj2l/+tV618X2E7bZlkgPqwyv5ioWIpvqU6FRdDoq5Sw/c+ObxG43oce/3TXTxyJNGskbq6MMhlOQa5rxLb3FnfW+sWq5MXyyf0z7ckUVtlJdApbuL6nU0VjWHiSwvUXdMsEp6pIcfkehrVEsTDKyIR6g1pGcZK6ZDhJOzJKKie5gjGXmjUepYCqM2v6XCcNexE/7B3fypucVuxKMnsjTorHXxPpDHH2rHuUYf0rTguIbmMSQypIh6MpyKUZxlsxuEluiWiiirJCiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigBK5H4mPt8C3q/33iX/AMiLXXVyPxMTd4Ev2HVGib/yIv8AjUy2ZM/hZ1kQ2xIPRRT6it3ElvG4OQygg/hUtUikJVXUrsWOnz3J6xoSB6nt+tW6x/E6s3h+52jONpP0DCoqO0W0VBXkkzhrC3fVNUjhdyWmcl2PXHUmvS7eCK2gSGFAkajAUdq8+8NOqa/bFjwSy8/7pr0brXNg0uVy6nTi2+ZLoFQ3NtDdwPDOgeNhgqRU9FdbSaszk2ONUXXhS/Od82mytyf7v/1/511VvdwXcYkgmSRT3U1JLEk0bRyIrowwVYZBrnL3wdbyuXtJmgJ52kbl/DvWPLOn8GqNuaM/i0ZvXF9a2qF57iOMD+8wrnNT8YIoaPT03n/nq44/Af41XXwTcbvmvIgPUITWrY+FLC1IeXdcOP8Anp938v8AHNZt1p6JWLSow1bucxaaVqWuTm4bcVbrNL0/D/61b8Hgy0VB9ouJZG77cKP610oUKAAAAB2paqGGgtXqyZYib0WiOfbwdppGA06n1D/4iud1nw9PpQ85G823Jxuxyv1r0Oop4Y7mB4ZV3I6lWHtTqYeElorBTrzi9WefaDrMml3aq7H7K5w6n+H/AGq9DIWRCCAysOR2NeVXELW1zLA3WNyp/A16XpMjS6TaOx+ZoVJ/KscJJu8GaYqK0mjG1DwfbTsXtJDbsf4cZX/61ZT+DL8E7Zbdh65I/pXd0lbyw8G72Mo15rS5w6+C73HzTwL9Mn+lD+DL0D5J4GPocj+ldzRU/VaY/rNQ8wvdIvtP5uIGCf315X/61Q2d7cWE4mtpCjd/RvYivUnRXQqygqRggjqK8+8R6Wum6gPKBEEoLIP7p7j+X51zVqDpe9FnTSrqo+WSOx0bVo9WsxIMLKvEiZ6H/CtOvPvClw8OtpGPuzKysPwz/SvQK68PU54XZyV6fJOyFooorcyCiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACimSSJCheR1RR1LHAFUl1vTXfaLyLPucD86VxXRoUUyORJVDRurKehU5FPpjCiiigBKwPG9sbvwVq8QGSLdnA/wB35v6V0FRzxLPBJC4yjqVYeoNJ6oTV0ZHhG7+3eEdKuCcs1sgY+4G0/qDW3XD/AAynlj0S80i4I87TbuSEr6KTn+e6u4pR2FF3igqOVEljaN1DIwIYHuKfXHeJtfl897C0coqcSup5J9B6VFWpGEbs1pwc5WRi6rZrpepbLa4VwrbkKtlkPofeul0rxZFOqw3kbrMB9+NSwb8ByKzvDvh6K/h+13Zbyd2EQHG7Hcn0rsbe0gtU2W8KRL6IuM1zUKc7860TOmtOFuV6tEiOJEDrnBGRkYp9FFdxxhRRRQAUxmCKWYgAckmn1h+K53h0RwhIMjhCR6d/5YqZy5YtlQjzSSKV94xhhkMdpD5wH8bNgfh61e03XZboqt1YzW2/7shU7D+OOK5jwtZR3mrgygFYl3hT3OeK9AwO/Suag6lT32zasoQ91IdSUVT1O/j02xkuJOwwq5+8ewrqk0ldmCV3ZHn+uFW1u8KdPMPT1r0Wxh+z2NvD/cjVfyFcHoFlJqesiWQZRG82UkcE5zj8TXodcmFjq59zpxLtaHYWiiiuw5QpKWqcup2MLFZbyBWHUGQZFJtLcEm9i3XI+NZFxZx/x/M2Pbir954t0+BT5Ba4k7BRgfma5uK21DxNqLTMNq9GfHyoPQetcleopR5I6tnTRpuMueWiRb8IWLS6i12VOyEEA+rH/wCt/Ou5qrY2UNhapbwLhF79yfU1arejT9nCxlVqc8rhRRRWpmFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAcx4wdxb2yA/u2clvqBx/WuTru/ElqbnSJCo+aI+YPoOv6E1wlZT3MZ7k1td3Fm++3meM99p4P1Heuj0/xZnEd+gH/TVB/MVy1FJNoSk0enxTRzxiSJ1dD0ZTkVJXm9hqV1p0u+B+D95G5Vv8+tdnpet2+pLtB8ucDmNj/L1rRSuaRmmatFFFUWcHCo0D4rSqSwttct9yeglTqPyBP/AAKu7rmfG+lzXmkR31kCdQ02UXdvjq237y++R29hW7p19DqWnW97btmGeNZEPsRmpWjsRHRtE8hKxswHQE15O8jSu0jnLOSxPqTXrR6GvNNasG07VJYtuI2JeP8A3TXHjE2kzvwjV2ju9EQJotkAODCp/MZ/rWhXP+FtViubBLRmCzwjbtJ+8vYj+VdDXVSknBWOaompO4lLSVBc3lvZxmS4mSNf9o9fpVtpashK+xPRXKXvjSNCVsoN/wDtyHA/Ks4eMdS3ZKW5HpsP+NYSxNNPc2WHqM7yqOr2A1LTZbfOGIyh9GHSs7SvFFvfyLDMvkTNwuTlWP1rfrRSjUjoQ4ypy1PMrO5uNE1QO0ZWSM7XRuMjvXd2mvaddxB1uo0PdZGCkfnU97plnqCbbmBX9G6MPx61jS+DLFiTHPOntkH+lYQp1KWkdUbSqU6mstGXb7xJp1mpxOJ3xwkR3Z/HpXKySaj4ovwETEanAH8EY9z610Fv4P0+IgyvLN7M2B+lX7u+sNDtVDBY1/gijXlvoKJRnPWo7IIyjDSmrsl0vTIdLtFghGT1dyOWPrV2uMn8a3BP+j2saD1kYt/LFRxeNL1WzNbwOvouVP8AM1SxFKOiE8PVlq0dxRWPpfiKz1MiMExT/wDPNz1+h71r1vGSkrxMJRcXZhVW8020v023MCvxgHuPoeoq1RTaT0Yk2tUcRqvhOW2VprFjNGOTGfvD6ev+etQ6D4hk09ltrklrXOM94/8A61d7Xmeu7P7cvPLHy+Yfz7/rmuGtD2LU4HbRm6qcJnpSsHUMpBU8gjvT6x/DErS6BblzkruUfQEgVsV2wlzRTOSS5XYKKKKokKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAayhlIIyDwQa861SybT9QlgP3QcofVT0r0esXxDpRv7TzYlzPDkrj+IdxUyV0RNXRw1FFFZGIUqsyMGVirA5BBwRQFLAkDp1pKAOq0jxNkrBfkA9Fm/x/wAa6cMGAIOQeleXVsaPr02nMIpcyW393PK/T/CrjLuaRn3O6PPFc/oyf2NqlzorDFtIWubHjgKT88Y/3WOfow9K2ra5hu4FmgcOjdCKpa3pz31mslsVS+tn861kboHHY+zAlT7Grfc0fdGnVHU9Lt9Vt/KnGCOUcdVNGk6lHqunpcxq0bZKyRP96JxwysPUGr9JpSVmOMmtUcBc+FtTtJS1uBMFOVaNtrD8DUsN34ogURrHcMBwN8W79a7mlrD6sk7xbR0fWG17yTORUeK7tdpYQA9ztX+XNPg8IPNIJdQvnlfuF5/8eP8AhXV0VXsI/a1I9tL7OhQtNHsLJAILaMH+8w3H8zSXmi2F8hWa2QH++o2sPxFaFFackbWsRzyve55nrGmNpOoGDeWQgMjdDiu50C9e/wBIhmk/1gyjH1I4z/WuW8YXCy6usS/8sowCfc8/4V03h2zey0aFJBh2y7D0z/8AWxXJQXLVko7HVWd6UXLc1qKKK7jjENeY6tePfanPM5JG8qo9FHSvTjXluqQG21O6iIwVkbH0PI/mK4sZflR14S3MzX0fww+oQi4uJGhhb7oUfMw9fataTwXZFMR3E6t6kg/0roYFVLeNUGFCgAD6VJWsMPTUUmjOVeblozhLzwjf2532zpOo5wPlb/P40+w8TXmnSC21CJ5EXj5hiRfz6/jXcVVvdPtdQj8u5hVx2PcfQ9ql4fld6bsP2/NpUVxllqtlqCg286sf7h4YfhV3NcVf+ELmB/MsJPNUchWO1h+PQ1QSXxDbAxr9vA9CrN+RxS9vOOk4j9jGWsJHY61q8Wl2jMWBnYYjT1Pr9K85Aknmx80ksjfUsTV0abqt7P8ANbXLyN1aQEfqa63QvDiaaRcXBElzjjHRPp7+9YyU68trI2i4UI73Zp6VZmw0yC2ONyL82PXqf1NXaKSvQSsrI4G7u7FooopgFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFAHJeItDKM99arlTzKg7e4rma9SIyMVy2teGyWa5sF56tCP6f4VnKPVGcodUcuCVIZSQR0I7VaRIr3gFYbj0PCP8A/En9PpVUgqxVgQw4II6GkqDIdLFJDIY5UZHXqrDBFNq/Bfo8a29/GZoRwrg/vI/oe/0NOm0p2iM9jILqDvsHzp9Vp2HbsRadqdxpk++Fsqfvxno1dzp2pW+pw74Www++h6qa86qW2uprOdZoHKOvp3+tOMrDjKx0mrM3hnVjrcak6bclU1FB/wAs26LMB+St7YPaunR1kRXRgysMhgcgisjTtVtdbtXtp0TzGQrJC3IcHrj1FYGkX0nhDW18N6g7HTZyTpdy56D/AJ5MfUdB9R6iqvY0vb0O5opM0tWWFFFFACVk65rUek2+Bhrlx8if1PtVvUr5NOsJblxnaOB6nsK4vRrZ9e1tprwl1X95J6H0X6f4Vz1qjTUI7s2pU01zy2Ra0DRZdQuv7RvgTGW3qG6yH1+ldrSKAqgAAAU6rpU1TViKlRzd2FFFJkbsZ561qQFcd4w0wrKmoRr8rfJLjsex/p+VdlUU8MdxA8Mqho3BDA9xWVWn7SNi6c+SVzM8Oait/pUYLfvYQEcfyP41sV57mfwxrxAJaMdv76H+v9RXewTR3EKTRMGRwGUjuKihUuuV7outCz5lsyWiiiugxCiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKAMvUtEtdSBZl8ubtIvX8fWuTv9BvrAljH5sQ/jj5x9R2r0CkxUuKZLimeW1JBPLbSiSGRkcd1Nd9d6LYXpLSwKHP8afKaxbnwgRza3Wf9mUf1H+FRytGbg0ZZ1G1vBjUbX95/wA94Plb8R0NNOki4+bT7qO54z5ZOyT8jTp/DupwniDzB6owP6VTksbuA5ktpk9CUI/WjXqLXqNdLiynXeskMq8rkYI+la92LTxloz6TqBEV396CYDo46Ee/qPSqMOr3kKiN3E0XeOdd4/XmpBcaVcEGW2ltH/v27ZGfoen4UIESeDPFVyLx/DHiAmPVrYlI5GP+vA9z1OOc9xzXd15t4q0CPxFp6Xmn3scusWY3QunySTKOdpH94dQf5Zq94C8dLr0Q03UmEeqxDGTx54HcD+96j8R7OMrOzKjKz5Wd5RRRWhqcp42lYQWkQOFZmY/hj/GofBJXzb0E/MQhH61qeKbBr3Sy8a5kgO8Adx3/AMfwrjdI1FtL1CO4ALJ911HdTXn1XyV1J7HbTXPQcUen0lQWt3BewLLbyK6HuDUryLGhZ2CqOpJwBXemmrnG01oOrKsdQW91q+iRgUgVEHucnd/QfhWZrXimFInt9PffKwwZR0X6eprH8K3a2+shHbCzKU5/vdR/X865p11zqKN40HyOTPQaKKK6jnOQ8bQjNpMOvzIf0P8AjU3g29MltNZu2TEdyf7p/wDr/wA6peMrxJLqC1RgTECz+xOMfy/WovB27+2JCOnknP5ivP5rYnQ7uW+H1O7oo7VS1TUE0rSrq/lR3jtomlZUxkgDPGa9A4S7RXnC/GHSGcKNOvsk46J/8VXowORmpUk9iYyUtgopaxfEniSy8Mab9tvNzbmCJEmNzn2z6DJptpDbtqzaorzy2+LOnXl1FbW+lahJNKwREUJkk/8AAq9CHNCknsJSUthaKKKZQUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUm4ZxkZ+tLQAUUlcn8QtW1HRPDQvdMn8mZZ0Vm2K2VORjBBHXFJuyuJuyudZS1454L8c+ItX8W2Nje34lt5S+9PJRc4Rj1Az1Ar2KlGSkromE1NXQtFFFUWFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFADSit1UH6im+RF/zyT/AL5FSUUAMEaDoqj6CvK/iR4Pktbg+JtHDI6NvuVi4KsOfNGP1/P1r1amsquhVlDKRggjgiplHmViZRUlY4jwH48j8QwrYX7LHqka9egnA7j39R+Xt3NeGeO/B83hbUk1TTN6WMkm5Ch5t364+nofw+vb+A/H0evxpp2ossepoPlbgCcDuPRuOR+XtEZ2fLIzhNp8stzvK5PWPCZkke408qC3LQngZ9j2rraKdSnGatI6YVJQd0eWvb3+nSHck8DeoyP1HWgR6hftjbc3B99zfzr1HAPajA9K5vqn946PrXkcXpXhKaV1l1DEcYOfKByzfUjpS+IPDzwSG9sEIQcvGnBQ+ortKStfq0OXlRn9YnzXZxNn4yuIYglzbrOQMbw20n68U278Y3c0ZW2hSDIxuJ3Ef0ro77w5p18xdojHI3JeM7Sf6VRTwZYKwLTXDj+6WAz+QrJ06+yZop0N2jjI0nvLjaivLNIc4HJJrvtA0YaVakyYNxJy5Hb2q9Z6daWCFbaBI89SByfqat1dHD8j5nuRVr865VsFZHihPM8KaunrZzf+gGtes7XV3eHtSX1tZR/46a6Xscz2Pmi0G68gX1kUfrX1OOgr5b04btTtB6zIP/HhX1BNNFbQPNNIscUalndjgKB1JrGj1OfD9SHUL+20uwmvbuURQQrudj/nrXz34o8R3fi3W/PKuIgfLtrcc7QT0wOrHjP5Vp+OPGE/ivU1srESHT4pMQxqOZn6biOv0Fd34B8AroiJqmqIG1FhlIzgiAH/ANm9+3QUSbqOy2CTdR2WxJ8P/Ao0CFdS1BA2pyrwp5ECnsP9r1P4DvnvKKWtYpRVkbxioqyEorL8Qa3B4e0abUriOSSOIqCkeNxJIA6/WvN7v4y3BYiz0eNR/emmLH8gB/OiU1HcUpxjueu0V4ofjDrueLLTwP8Acf8A+Kq5Y/GS7WUDUNLhePu1u5Uj8Gzn8xU+1iT7aB69RWToHiPTfEln9p0+bdtwJI2GHjPoR/kVr1adzRNPYKK5zxb4si8J2kFxLZy3AmcoNjABTjPP6/lWH4V+I58Sa5JZPYJaQrA0vmNNuPBHXgY4JP4UuZJ2Jc0nY76lrzvXvixpunyvBpcBv5V4Mu7bFn2PJP8AL3rmD8YdcLcWOn7fTa//AMVUupFCdWKPa6K8w0X4v21xMkOr2RtQxx58Lb0HuRjIH0zXpUM0VxCk0MiyRyKGV1OQwPQiqjJS2KjNS2JK5f4iTSQeBdSeN2R8RgMpwRmRRWxrWr2+haTPqV0sjQw43CMAtywUYyR615p4x+Ieja/4WutPs1ulnlKEeZGAMBwTzn2pTkkrE1JJJowfhiklz47tpHdm8qKR8sc/w7f/AGavea+e/APiCw8N69Lfah5vlNbNGvlruO4sp9fQGvRX+L3h5fu2+oP9Il/q1Z0pJR1M6M4qOrPQK4/4nIG8B3xP8LREf9/Frd0LWINf0eDU7aOWOGbdtWUAMMMV5wT6VjfEgZ8Bal/2zP8A5EWtJaxNZ6wZ5T8Nhnx7p3/bT/0W1fQVfP3wz/5H2w+kn/oDV9Amoo/CZ0PhCkrJ8Ra/aeG9Jkv7skqCFSNT80jHoBn/ADwa4tfjFp7sFXSbtmY4ADKSTWjkluaucU7M9LpKhtJnuLOGaSF4HkQM0T9UJHQ47is7xJr9v4a0h9RuYpJUVlQJHjJJOO5pt2Vx3srmxRXkF18ZbpmxaaRCi9jLKWP5ACqZ+MOu54stPA/3H/8Aiqz9rEz9tA9roryLT/jJcLIBqOlxtH3a3cgj8G6/nXpOia9p3iCxF3p04kTo6kYZD6MOxqozUtiozjLY1KKSvPdS+K1npmp3VjNpd0ZLeVo2O5ecHGR9apyS3HKSjueh0Vm6FrEWvaLbalAjIk4JCseRgkEH8RWjQNO+otJVDWtVi0XR7rUplLx26biqnluwA/GuItPi7ptzeQQNp9zEssioXZlwuTjJ9hmk5Jbic4p2Z6PRSClqihKK5fxb42tPCctrHPbS3D3CswEZA2gY65+v6UvhLxnB4ta7FvZTwLbhctIQQS2eBj6VPMr2J5lex1FFFFUUFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAV72yt9Qs5bS7iWWCVdrowyCK+fvF3ha78IawoRna1dt9rcA4PHYnsw/+vX0TWdrWjWevaXNYXse6KQcEdUbsw9CKznDmRnUhzI4rwH8Q01UR6Xq8ipfYCxTHgT+x9G/nXotfNPiLw9e+GdWeyugSPvRTAYEi9iP8O1eheBPiRv8AK0rXZvn4WG7c9fRX9/f8/UxCp9mRnTq292R6rRSAgjIpa3OgKKKKACiiigAooooAO9UdYGdFvx/07yf+gmr3eqWrnGjXx9LeT/0E0nsJ7HzJZzLb3tvO4JSORXYDqQCDx+VdZ4y8f3XiYfZLZHtdOGCYy3zSn/ax/Ln1rk7KJZ762hfOySVEbHXBIFei+LPhY2n2rX2hvLcRoMyW0nL49VI6/Tr9a5I8zTscUVKzsbvw08MaNBZLq8V1Df3x43qOID3UA8g89T/+v0avmbw/4gvvDeppe2T+gkiJ+WRfQ/419CaBrtn4i0qO/s2+VuHQ/ejbup963pSTVjoozTVjVooorU2MbxNoC+JNHbTpLh4I3dWZkXJIBziuctfhL4cg5ma8uT/ty7R/46BXedqr3V7a2UJmu7iKCIdXlcKPzNS4p6shxi9Wcw3wz8Jsm0aayn1FxJn/ANCrjPGPwyg0nSptT0iaZ0gG6WCXDEL3II9OvOeK7e5+I/hW2yDqgkYdoonbP4gYrn9a+KPh+80i+s4Yr13ngkiUmIBclSBnJ6c1nJQsZyVOxwfw/wBWk0rxjZbWPlXLi3kUHghuB+Rwa+hq+ZPDgJ8T6SP+n2H/ANDFfTlFF6BQehwnxZh83wXvx/qbmN/zyv8A7NXi+mWV5qWoRWFiCZ7g+WFDbQR1OT6cZ/Cvd/iTGJPAWpZ/hEbflIteR/D3/kfNK/33/wDRbVNRXmiKq/eI77R/hDp0Eavq11LdTfxRxHZGPx+8frxWpefCzwzcRbYbee1fs8UzE/8AjxIrtaWteSPY29nHsfNfinw3c+F9YaxncSIV3wygY3r9Oxr0/wCEWpy3egXVjK5YWco8v2RhnH5hvzrL+M8ShtGmx8585Sfb5DTvguD/AMTpu37kf+h1lFctSyMYrlq2R3virRZPEPh650yKdYGmKfvGXcBhg3TPtXj3iz4fy+FdJjvpNSS53zCLYsJXGQTnO4/3a96rz74wf8ipa/8AX6v/AKA9XUimrmlWCaueaeEPCreLNQntFuxbGKLzNxj355AxjI9a69vgxdD7utxH62x/+Kqt8HP+Rhv/APr1/wDZhXs9TThFxuyKVOMo3Zj+GNHfQPD1ppjyrK0AYF1GAcsT0/Gs74i/8iHqn+6n/oa11Fct8Rv+RD1P/dT/ANDWtZaRNpK0Wjyr4Zf8j5Yf7sv/AKAa9t1rWrLQdNkvr+URxJ0A+87dlA7k18++FNai8PeIYNTmieVYkf5EPJJUgdfrUuq65f8AjLXYTf3cVujvsiWRiIoAf8jJrCE+WNjnp1OWNuo7xD4g1LxnraHy3YFtlrax5baD/MnjJ/wr0zwN8PI9E8vUtVVJdRwCkfVYP8W9+3b1rZ8J+C9N8MW4khAuL11w90w5I9FHYf5Oa6etIU/tSNYU9eaW4Vh+KfDkfijTI7CW5eCNZhKxRQS2ARjn6/pW7SVo1fQ1avozhbX4TeHIP9d9ruD/ANNJsf8AoIFXH+GXhRkKjTmU/wB5biTI/wDHq6a8v7TT4TNeXMNvGP4pXCj9a5y4+JPhW33D+0/NI7RRO2fxxio5YIhxgtzgvGvw2i0LTH1TS55pIIiPNhlwSoJxkEDpyOPxrK+GerSad4xt4A7eReAwyLngnGVP1zx+JrrvEXxN0HUtBv8AT7eK8aSeB40ZogFBI4J5rzzwcCfGWj46/ak/nWMrKS5Tnlyqa5T6Trw/4saT9i8Tx36A+XfR5P8AvrgH9Nte3iuO+Jej/wBqeD7iVB+9sz9oXjsB8w/75JP4VtUV4nRVjzRMX4P6r52k3mlyPlreTzY1J/gbrj8Qf++q9Mr55+HurnSfGNmzMBFcn7PJn0bp/wCPBa+haVJ3iKjK8Tzb4v6v9n0e10qN8SXUnmSAf3F9f+BEflXkE9vNaOizIyM0ayrnurAEH8iK6zxPcy+MPiL9kgkDRmZbSEgcBQfmPvzuNdB8XNES3XTNSgULGqfZGAHTGSn/ALN+lZTvJuRhUTleXY9D8Kat/bfhiwvmIMjxASY/vjhv1BrZryn4O6vxf6O56f6TF+it/wCy/rXpep30WmaXdX0xxHBE0jfgM1vCV43OmErxueH/ABO1Mah4znjQ5SzjWAe56n9Wx+Fel/DTSDpfg+3kcYlvD9pb6H7v/joB/GvHNFsZ/FPiyCCZi0l3OZJ39vvOfyzX0iiLGiogCqowABwBWdNXk5GVJc0nIfRRRW50BRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQBieJvDVn4n0p7O5G2RctDMB80beo9vUd6+etY0i80LU5bC+j2Sxngjo47MPY19QVzfi/wAJWvirTPKciO8iyYJ8fdPof9k1lUhzaoxq0+ZXW5534G+Iz6X5emazI0llwsVweWh9j6r/AC/l7JFIk0ayxOrxsAyspyCOxBr5e1DT7rSr+WyvYWinibayn+Y9R3zXUeC/Hl14ZlW0ud1xpjHmPPzRe6/zxUQqNaSM6dVr3ZHvtFVLDULXVLKO7sp0mgkGVdD/AJwfarddB1BRRRQAUUUUAJVDWzt0HUT6W0h/8dNX6zPEbbPDGqt6Wcx/8cNJ7Cex826ccalZn0mT/wBCFfUvavlizOL23PpIp/WvqcVjR6nPh+p5H8S/BHkGTX9Mi/dsd13Eo+6f+egH8/z9a4/wf4pn8LauJ13PaS4W4hH8S+o9xmvop0WSNkdQyMMEEcEV4D4+8JN4Z1fzLdD/AGdcktCf7h7p+Hb2+hpVIuL5kFWHK+eJ7zZ3cF9aRXVtKssEqh0dehBqxXinwz8Y/wBl3a6LfSYs53/cux4ikPb6H+f1Ne1ZrWElJXNoTUlc5/xh4ni8L6K12VElxIfLgiJ+83v7Dr/+uvDR/bvjbXAhaS8u3yQCcLGvf2Va7P4yzSHUtLhP+qWF3H1JAP8AIVb+DS2/kas2R9p3xgjvswcY/HNZS96fKYzfPU5Rmn/Br5Q2o6rz3S3j/wDZj/hVjVvhVoun6LfXkd3ftLb28kqhnTBKqSM4XpxXp9ZPiaSOPwvqhlkVFNrKuWYAZKkCtHTikaOlBLY+fvCy7vFukD/p8i/9DFfTFfNPhNgvi/Rz/wBPkX/oQr6WqaOxGH2Zy/xEOPAeq/7if+hrXj/w9OPHmlf77/8AoDV618TH2eAdR/2jEP8AyIteR/D848d6T/10b/0Bqmp8aJq/xEfRVFFFdB1HlPxoPyaKvvMf/QKd8F/9TrP+9D/7PVf40Pm50ZPRJj+qVN8Fz+71r6w/+z1h/wAvTm/5fHq1ee/GD/kVLX/r9X/0B69CrhvivatceC2kX/l3uI5D9OV/9mrSfws2qL3Gch8HSP8AhIb8d/sv/swr2ivBfhdqcen+Mo45SAt3E0AJPAbhh/6Dj8a95zU0fhIoP3Ra5T4kHHgLUvpH/wCjFrq65L4lnHgLUfrH/wCjFq5/Cy5/CzyHwJp1pq3i21sr6ES28qSBlP8AuE8Yqbxp4MufCt6GQtNp8pPkzEcg/wB1vf370/4anHj3TvcSf+i2r3bUtNtdW0+axvIhJBMu1lP8x6EdQawhDmic9OmpwPIfh/8AEBtLeLSNWlLWJIWGZjzCfQ/7P8vp09oUhgCCCDzkV83eKvDV14Y1h7ObLwtloJscSL/iOhFdx8NPHBjaLQNUl+Q4W0mc9P8AYJ/l+XpVU5te7IqlUafLI9brmPG3iuPwrpAlRVkvJyUt426Z7sfYcfoK6btXi3xhmkbxNZwsT5SWgZR2yXbP/oIrSpLljc1qS5Y3Ry1tba5421vaGkvLpuWkkb5Y1z+SjnoPwrvbD4NIFDajqzFu6W8eMf8AAjnP5CrfwcS2Giag64+0m5Ak9dm0bf1LfrXpdZwppq7M6dNNXZ5Vr3wu0fSvD99fw3V88tvA0ih3XBIGefl6Vw3gZd/jjSB/03z+QJr2/wAZyRxeDdW8yRUDW0irubGSQcD614l4EYJ450gn/nsR+akVM4pSViakVGasfRlMkRZEZHUMrDBB6EelPorpOo+ZPEOlvoXiG908k/uJf3ZH908qfyIr2u58V4+Gn9vowWd7YBc9pT8n6Nn8q5P4w6PtuLHWI1G1x9nlI9Rkr+m78hXCNrkjeEY9EZmKpeG4Gey7cY/Msa5r8jaOS/s5NHWfCPSPtev3GqSpuSzj2ox/56Nx/wCg7vzr1DxXo/8Abvhm+sFAMrx7oiezryv6jH41m/DrRxpHg+13IVnuv9Jlz/tfd+ny44rrK1hH3bG9OFoWZ81eF9WOh+J7G+bISOULKP8AYPyt+hz+Feq/FnVjZ+GYrGMjdfSgN/uL8xx+O38688+Iei/2N4uuQigQXX+kR47bvvD/AL6z+lU9c1mfxG+jwAvJLBapbYP8Um4jPvn5axTcU4nMpOKcTvPg/omyG81uUcyH7PDkdhyx/PA/A16pWdoelx6Lolnp0ZyLeMKWx95u5/E5NaFdEFyqx1QjyxsLRRRVFhRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAcn428GQeKbHzItsWpQr+5mP8Q/ut7fy/PPgd3Z3Fhdy2l1E0VxE210cYINfU9cd458EQeJrT7TbBY9TiX92/QSD+639D2rGpTvqjCrS5tUeQ+F/FmoeFr3zLZvMtnP763Y/K/uPQ+9e86B4i0/xHp4u7CXdjiSNuGjPoR/nNfNtzbTWdzJbXMTRTRMVdGGCDVnSNYvtD1BL3T5zFMvB9GHoR3FZQqOOjMadVw0Z9P0VyvhHxvY+KIBEcW+oIuZLdj191Pcfyrq66k09UdiaaugooopjCsTxcxTwfrDDr9jlH/jprb70hGaT1Qmro+V4VYTxnaeHHb3r6nX7opdo9KKiEOUzp0+QKzNf0S28QaPPp9yPlkGVcDlGHRhWpRV7mjV9D5d1LTLrSdSuLC6jKzQPtbA4PoR7Hg17V8N/FEmvaQ1neMzX1mArO2f3ifwtn17H8+9dvgegowB2rONPld0ZQpcjumcZ8RPCk/iXSIpLMA3toS0aE48xT95frwMfT3rxO1vNT0DUS8Ek9jdx/KwwVYexB69Ohr6gqle6Tp2pY+3WNtc7enmxBsfmKJ0+Z3QTpczujw0/E7xV5e3+0E/3vITP8qW00rxd46l8y4muZbZfm864JWMf7q9Ce3A+te0weG9DtZBJBpFjG46MtuoI/StTAxS9m+rEqTfxM+YNGnFrrmn3DA4huY3PthgTX0+Ogpiwxp91FH0FSVUIcpdOHIcV8VGI8DTqAfmmiHH+9n+leVeAgw8daSdp/1p7f7DV9EkA9aNo9KJQvK4pU+aXMLRRRWhqeOfGNi2s6agB+W3Y/m3/1qufBjI/toEEf6nr/AMDr1bAowBWfJ73MZez9/mFqhrOmRazo91p0xwlxGU3D+E9j+Bwav0lXa5pa58x6xomo+H79ra/geJ1PyyY+Vx6q3etO38f+KLW38lNXlK4wDIiuR/wIgmvoSe3huYjFPCksZ6q6hgfwNUE8N6HHJ5iaPYK45DC3TP8AKsfZNbMw9i1szn/hnfahqXhqW71G4muJZLptryn+HavT2zmpficT/wAIJfADq0Q/8fWuuChRgAAD0pSBWvL7tjXl93lPnz4dBl8e6YSD96T/ANFtX0HRtHpS0oQ5VYVOHIrGH4p8OW3ibRpLOYBZRloJccxv2P07H2r51u7O5sL2a1njZJ4HKOB2YHsa+pqbgelKdNS1FUpKepxPw58Vya/pb2d4Sb+0ADOf+Widm+vY/n3qP4k+EbjxDYw3lgu+9tcjy+8iHqAfUY6fWu7wB2oquW8bMrkvHlZ8w2Opap4fvmktJ57O5X5XXGD9GU9fxrfPxO8VFNv9oID/AHvITP8AKvcr3RtM1Ihr3T7W5YDAMsSsR+YqG28O6LaSCS30myicdGSBQR+OKyVKS2ZkqMlszxKLRvFnjGOW9u3uZLeBGkEtySFOBnCL3Jx2GKyPCs3keK9Jlz8ou48n2LAV9L4pixRp91FX6DFP2WqY/Y7O48dKWiitjc5zxxpg1XwfqMATdIkRmjHfcnzDH5Y/GvBtB0xtX16x08hgs8yq5A6L/F+gNfTlN2gdqzlT5ncynSUmmCKEVVUYAGAKdRRWhqeefFvSDd+HodRjQGSzl+c99j8H/wAe21wvwz0k6j4ygkdf3dojXDZHUjhf1IP4V74RmjAHQVm6acuYylSTlzC0UUVoahRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQBxXjrwNF4ktjd2irHqkS/K3QTD+639DXhU8E1rPJBcRNFNGxV0YYKmvqmuK8deBYvEkBvLNVj1SNeD0EwH8Le/of8AIxqU76owq0r6o8Khmltp0ngleOWM7ldDgqfUEdK9j8FfEuHUfL07W3WG8Pyx3HRJfr/db9D7dK8duLea1uHguImiljba6OMFT7io/asIycWc8JuDPq0c0teKeDPiVPpIj0/WWeexHCTcs8I9/wC8P1H6V7JbXUF5bx3FtMksMgyjocgj611RmpbHZCansT0UUVZYUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQBxXjnwLD4ktzd2gWLVI1+VuglA/hb+hrwu5tp7O6ktrmJ4p422vGwwQfpX1TXO6x4f02813S9Ultx9rgnwHHG4bWI3euCAR6VjOmnqjCpSUtUeIweCvEtxD50ei3Wzr8yhSfwJzWnoeseJvAk5aewulsWb97BcRsqH3VscH3/ADr3wUjKrKQwBB4INCpJapgqNtUzJ0DxHpviSxFzp827H+sibh4z6EVr1hT+F9KF1/aFrAbG9QHE1ofLJ/3h91v+BA1rWUrT2UMr43OoJxWqv1NY36liiiimUFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB/9k=</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr">
         <is>
           <t>Human Resources</t>
@@ -1905,7 +1941,11 @@
           <t>WHH</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAYoAAADFCAIAAADFZSJKAAAACXBIWXMAAA7EAAAOxAGVKw4bAAAsi0lEQVR4nO2dh58TRf/4v3/FDxF4rA92D4Gj9yZVpCrSpCMdpImAhSZFHgFpKgqoIHC5zpVc4Xrvvffee0kuyW/uoutkZnaz2eTuNrnP+/V58eKys7Ozm913Znen/J8OAABAlvxffxcAAACADegJAACZAnoCAECmgJ4AAJApoCcAAGQK6AkAAJkCegIAQKaAngAAkCmgJwAAZAroCQAAmQJ6AgBApoCeAACQKaAnAABkCugJAACZAnoCAECmgJ4AAJApoCcAAGQK6AkAAJkCegIAQKaAngAAkCmgJwAAZAroCQAAmQJ6AgBApoCeAACQKaAnAABkCugJAACZAnoCAECmgJ4AAJApoCcAAGQK6AkAAJkCeuKlTd1a0JQbVx0RUOrlUahwKfjLOf+BW8FjZbFrWMWztLrEyrayLm1XfxcTAGwW0NPfaHXa3MZMp/w/z8V/sTFg8Uy3d95zeM7uyf8TiBFPBtkrhn3oNfFA2IZbqReDy30bO+v7ez8AwHYY6Hqq66hxyf/rcMTWaa5vCstITCCjfeQz80rSqfiaKLlVrJB/wysCfUvcsHDPa8oSWCW2OsIwffcqZa0lvJvQalG9kkhf0JSDp4mrjqTyFBPuFW1lxOZQ7RV9jid7VuqJ6rwCe1TbUU2sYmoElSnVGrWI4w1YgAGqJ3QSo9u07UErRymeN99KzJjtbncx4URGfTLyQn/vbjfZDWl0Iae4vNbZ1cFMn1wbh6qH9CpLvSfzbcKnxI1O/7HvLC4Bqp/asfIUE+v8FxCb+/TZIjrZD0mnBA7C7pA15n+zT3LvmXLgAekMOD0VNuddSDg+2WV4L1mJCHSFr/Gb61b4pFPDtkCf0aRqYOoGHRBmekXe78w9Gq0YwldDuZ7yHZ1+X+g6LkFiTbTkI7mE0uIy5RQ62bexBwUOAtNopsavGVdNPPaARAaQnrIb049EbBulGNI3YiLi/afvPcj+pb2rrR+PwLyno+iCBZZ5MxN/n/gV375kNaQxVzkYvolOfCP1PJcA9ASYxIDQU1lr8Ymo3SMdeus+TnzMfTrSJf+vLm3/PLzYG7qWLtLdzOvMxLtCVvPthbLYlbnKMuVUOrFviTuXAPQEmISN66mzq+OntMvjnV7qdzHhsdrv/aTa2L4/GtdTztOF+TpmHzPxIs+xfOVHh5RO36VRj3H8D524qDmfS2OOnpD7iC1K0NPGgMXmf32/Zf5o6pEHpGHLekIXw1Lvyf0uI2aMcnj+YsIJ4ddMFsenxJ0uyXrqkTOiVd1i7ziMr/DHIj+jVylszqNTTnYZrtKouDR8ekLW2BO6ViBQvc+94DGxRQl68it5ujd0HZ3/OKcX6azme9jTKQ+Fb8aFC/QqtqkntUZ1I+V8fz1mEh9LvCel1iX02WEpYhlkuuubdBuInMYMgWJ/4juHzjywTGnUfXx6SqtPkrA7EvTEB7OqeD7+SwlZARbEBvVU2VZmkTp83wSqpDzMudM3jQ802q4Jzq8QBRjxZFBtRzWR0pfVRICLSc6v0ka7l3mdTnkm7jCeBvQEmISt6QldALPd3+136ZgaJ6J2903Lg3X+C+itx1aHE8l+Tv9BoLQjHJ6raCslVvk6Zj+dkmgiBHoCTMKm9KQsdhnr+EK/u0ZabAhY3ND7fWJOxx6iN+2Q9zuR7MuoncKljawMIlb59NlCOhnyEZ4G9ASYhO3o6XHub+85DO53y5gTy7ynVFJdNyx9lO7S272UcJJIttpvLp5gqsvrRJPORzm/4unRzek019eJbEcrhjapGvBkoCfAJGxET79n3WI2iba6WOQ5rpy/U5v5JLAEsTP4EzyNWque4vIanuDz8E3INfgn38Ufw1epaa+ie1B/4Dme2DroCTAJW9DTw5w7tuGmv69qr/FVbeW9dKxaVE0jqTrmAs8x+LP5qvYKIsHt1EsLPcbgn2wPWolnG1cdTu/IwfBNxNZBT4BJWL2enhYqjI58YnWx0mcGcVtkKZCGPvAcR2xulGE3uqiqECKBZ5HjjuCP8U/mPh2JZ8vsoEe33gQ9ASZh3XqKrgobw9960Krjs6CVKk1nbxy0z1k94zIbUrkE9POp1LqE7+K/wD/pea7UyK1yKfEknWcA1ZuPT0/JdfFdWrVAMHcE9GTzWLGeSloKp1tikCbZRs/zHcu3h7qd9j29Le9iFy7BhYTj+CJUOW3sbHiQ/TOxSnp9MrfKrpBPiKXodru0pYjYNJ+eJji/MtlluEB8wWqnDnqyeaxVTx1d7Z/4zul3g/RqoCvcvZDsyWE+AaVe9LZupV7iEhD3cbPc3tFoNSHlfsQq6I6PW2WBhz2xdKrL63TTTcl97qa7vqWhcgM92TzWqid06vS7PvogJji9km842qT5lLUW0Rs6GrFNv1Sr0843dM16/4W6ni51xPuHm6kX9au0qpvtDd/rodgU8CG9adATYBJWqafQcn/bexzOF2v85qotOgBLl1Y9lWqj9JHPTP3SNnUrMfLMieg9up5ujETbgiMRW/WrZDWksq7tY/SmQU+ASVifnrRa7f+Svj0cvkVkHArfsi90/faglat8Z890e7u/miCMcfzPB17jNzxbvCvkk8/DN4kvP4q46gjLHkO6T+J4p5f092KZlGt+Sf9BvxYqP9No3sUu9P465f9Jbxf0BJiE9enJHNCdS5OqIboqFF1ymwKWjOrlAepmub37VfQ+t4LH+U3Z/TUEHZPv4o/RpS1rLdZ1u8aZ+JwbfI4YoG6i86v6d4u30y7RuTFHYhDU0yCB2BywhO41DXqyeQaWngjqOmr/yvl1pc90y1oJVZSOR+2OqQrTaDX9vYtsHPP/pIuNbpl1rPd6Gf+8oSPe6HW/m2vtfjd3NGI7sYq947BWdQu9XT49RVWF1HfW8UVDZx1dddKBngYAA1pPetDPclhFwHp/Ro9WUwPdIv2Q9G1Ne1V/75MRUNWGLvwfWT+hRUcjDVyDKphc+yakcmKVsIpn6HN0l0d8zjebCzTLBEwC9PQ3SFLexS5z3EdIExOqShyO2EoPMyJPWrrftZHNWU/HHkKLVvnOwj+c426n/acOGF4RQKzyIPtntUY1kRpDinsPSAB6AkzCavSE9HEscscq39ni42ryGTwHRd79hzl34qoj2lj3HXoaOxu+jNxp6uPz6a5v+pV48JZcqy1rLVYWu95KvYTPSVnVXmHS7qBAgrDIwUQs8Z5E7MWmgCXd49U5GbhmI9Y+oKS1kFjlTNyR0pYi+nDxTRYAegJMwmr0hLRiao2Ge/OtZ3vQCv3n6BZsZ/Aq14JHqBJBbwh5UJH3u/i+Mmv85vGNMZDdkPa/pG8Xe03gLuDIymBuaSmr/ZFwbHj2gaWO55GIbUTmM93eRrU/4sNvYvZzqyB52TsatC3YErgstMKfLmdIuR9zo6AnwCSsRk8HwjZYSk9cTHF57Vry2fqOWnpzUZXBk5z/a3QT+8M+baOmrkOCi6oK3hq4jG6cZaaekOaSLTTFy530K3T+qIpHfPJbxjV8LaLOhe6F/8i6RayC9ppv1CrQE2AS1qEnVD2RMNv4YWN64iT1KOdXugcGEoHwZMKoAqLGpiHRU9JSuDd0Ld/toZl6susZ9tcihzS43JfOHN0+E5/4lTzF1yJmyhvlMORwxBZiFXSryzd0OugJMAnr0BOzF6ul9KQPdJ9SQf3mx1aHj2XN3WbXM4QbPaKAS/5fE51fFdiK+Xoa5/RSoyXGWkE7SzuU1nF2Qzq+Fj11ML3KtsDlfBsFPQEmYQV6Qj/Fi6ghiiyuJ7uevq+JNTHE1t0Ln9CX8TLvKc3YcCK6np4i5+K+MPpM3UBPLVL0hMIxj9Eg21RQbXGG29vCG7JXDG1RNeFrPcm9Z7R4SGF8GwU9ASZhBXpKq0uUdhmbqie7nroJ/XbsTNxhPM14p5dyGzPwBCqN6vOwjWKKZBE9ESNVSmZr4HLhDc19OpK4TYusDDJaPDdqvkwO0BNgElagp2vJZ/tMTz2GepHo49be1YaPMPkw5w6+VKPVHInYKrJIFtGTvWJYQ2ed+QeWOYYcHuiGl1ilvLXEaPEy61P4tsinp0+fLdoVslo4vo7Z39FlMNcWU09TXF5b6TPdaKA70EZsXhzQkzyxAj2t9JnRl3pCMc31jeKWAnzdnlpD943bWv/5RAeLq8lnxBfJUE9kMyLx4VXsbP6BdS14JLwVfUNNHHRLyJzvG1enwIR9krsE6yOlLh7Pjakn8RFVFcJlBXqSJ3LXU21HteSxUyTrCcVqv/c7DZ987wtdj0qSYDhxW1CZ0qTi4XoqMUNPeHMkyaBqjvBW7mfepNda5j1VYJWVyukCWzRTT8m1cQYlAT3ZOnLXk4/gbNrCcThiC56VSXqy65meBF89qyF1b+g6/BN0d2DqjMSW0hO62TR/nN82des4R6GqUECZF73W/rBPBVb5MmqXwBZBT4BJyF5PxW7HIndIi4c5v+BZXU0+vVw5dYLTyyJP37GOLxC3eHUdNfif4kfsHOkwGIlsvf9CfMYBlJvkXTsRvbtNTTYHlcAK5TSBYuc1ZdGr/C/pW4FV7mfeENgc6AkwCbnryeKgW7acxgyH3PsHwjYIt1FCcZy/DSQyF92rFo8RTwYt9Z5yOemboHKfmvYqvpaK/cup2IN85Z/s/N92qkG8rmfmLoFdTqiJEtgc8p3k4QDRTXSB4bjGG56Rg+qJD1QMfCqHNYazIuuDG60Y6C8GnJ5wWtXNHkWOGwMW810zoxVD9EMa0TBHdPv7wnYZjn54UUVJnkrCQUcgsMzbv9SDDmbVSdfT8y6iMoi5SnxNpNEtogoUc12jQTdJq2qv8C/1lJYb8XK2sq2MSBBUpuzoapd8YAGLMKD19A9adM3sCP6YKanrKd/RK7SqWyazeuRNdh7+S/oPFmnVDQAA6OlvUE0nuNyXfgax0HOsVktWgugRb9Gtx9cx+2s7qvul8ABgk8haT6Hl/iuU0yTH5cRv8NzuZv54PeW8b4k7uing2yKqFp2KPURUo3IM24gjiK6zs93tBEZi6tKqU+sSHuX8ejbuKN6FraKtzJy9Q9U9qccVAKwDWevpQfYvkp99ojgUvhnPjWtY8J7D4FW+s5Gtatormdt9WuiAv3H/K+dXfKlGq5n7dCS3dGPAYubovag6Fl0VciJ6Dz5rE96woLilwJy9m+T8X3q8BACwJWStp5upF3tDT1zYK4Z9E3NAP0MJQUJN9FSXv7VyMnovvqi6vWLEP00xj0ZspxtJa7Ua72KX5ax39hbUE91fFwBsDFnriR6+w7J60scYx//cTL3QSY2OklGfMs31DbvuaXIX4J/HVIX9o6099ChRaK11/vP5imRBPaEg2mEBgI0haz2djTtiztV7UJye9LHSZwb9Kj2pNna800vzno7CP/QsdETpD4RtICbvRTd9dzOvj6am8+49PVnLzAsAIA1Z6+l07KE+05Ndz9McepBsZbHrVNfX8RZMj3Pvfuw7i5jHraOr/bCIcQsM9ZRvpp6Yt6VA34BOCVR3lu1UhraBrPV0Lv6LvtSTXXc7zKHe1GAAN1Iv4HpyK3hc2JyHJ0Cq2hK4TEyRLKsnviG9xZBalxBUpsSDOa8vDqpdEqvEVkcwm56iO1wiZZKxIdJVGlVYRQCxFrN62KZuRb8iREp9FDTn0On1NKkag8t9DYtEtvMUplPTgb6+6ynn94SuXaacOsv9XXTvP9Pt7UWe4zYFfPhtzOdPcu/lN2ULCKtF1USUQWTEVodrqWwTaqIF1/KJrAzKbEht6m6FJ/fmwXzIWk/fJ35tnp424bmJ7BKMDBVYpsRXJOYfJ+7pVJrOHcEfiywSrqci8/Q04skgyc+e0FVED7SAPiky1C4Oqh6OZ3VXpOublW3l9OzwPZ1IhMacu595k858uXIanVJgmCp0J97E0yaWHkYdFcmokfVUtJVdTvx6uutbYr6UZd5Tfs+6xZwk+euY/ZK/7sAybzwrpHuR3YNGKYYsV079MeVcSUuhmJ2VFbLW063US+ZcwNL0hGKi8ytZDWkiC2nSHaiBnprN0lP3mzvWRFhiQBUHZp7EgEo4jZ31zKFj3AsdiJS5jVnMzCMqgwSKxBw2a7b7u3TK41G7BQ6Le+ETZv7MnxD9LMcCqDWqO+lXkPVM/XaOs0ZuEB7sQThcCv7Cs2LOZGHshBmGzN7W1Sq8y7JC1nr6K+eOORewZD3Z9UzDjW4ijJbQo1BhUh9XC+ppsstwoh4nHhvW0/7Q9cz8JegJVU63BC6V9u0cYc2T3L960sdqv/et6IWvrPVkzmBPdubpya57SP+vhYtX3V7JtY0SGRbU0yLPsZIPrA3raazjC8wbK1P1VNtRvUwpNPCecJyJO0znKQc9oVjnv4BuRiNPZK2n5No4cy5gM/U0WjGU7s6C81X0XlOLZKinPHP2jh4IXDw2rCcU3sUu9Fom6alT04GuYXO+nWvJZ+lszdGTa8EjPCtz9ITidtolungyRNZ60mg1zaomyUEMV5TflO1f6nEn/erhiC1z3EeI+RYPhm/kK1tuYyb9AJgO5Li1/vMuJBx3zPsDuQn/Ybfs3pmEbevpcPgWei2T9CTcHhidPBcTTngVOSfURKXWJcRUhXkUOV5LPrP+2cL3HAbr09xjDcvH1NMUl+FbA5cLx4GwDZVt5XhWTD2hk+1K8ukfU86hQP85FrljistrzF2Y4PQyPhOEbJG1nnoPrU6LakY/p/9viddEgRNxpMNgYgg0DuG3MPaOw1DdDd2cNsuy34lt6wlde7S7xespvT5p5D+WIXN2fuVx7l21hveRX0Vb6ZWkU6jYzC7iTD0JzFoqAFNPaMeJu7YmVePO4FXMfXmU85uE7fYxA1RPHD0dd0N3BX8ywoH9hPsy6wlUY2cD39uc6a5v/pR2WeYjq9i2nlD4l3oSa4nXE18zkVlu7+Y0ptPpxdP3etL1fHH6vllE7A5Zbc6+9A0DXU8ciTXR6/0X0t/i+0/foxvaubGmYBrr+MKNlPOSX/b3JTavpy+jdhJridRTVkMa81XsGMdhAgdHJP2iJx1P57AZbm+ZuTt9gNz1VNNe6Zj3h7QIKDWYaKS+s1a4rQDSkEPu/YnOrxBfJN2e8FD4ZiLN5sClAm0adT0zxNV2VOH3BdXtFdJ3zbCRnqnYvJ6muLzWaThnp0g9XUw4wczwesp54UMqhv7Sk1vBYzrxCIfn5P9TKnc9NXTW8T0IMBofeI3Hs7qe8p29Yugy7ymnYg+iyj+fqgqb81b5zsbz+SPrNp4AiWYWNn/USIfnf0n/QUMNXdCDtrA5917mDXT/j36sRimeb1b/+yjKt8Rd2n7Z8by3Fo/N68mOas4uRk/oTv99bCQvLia7DOdrjG4S/aWniMpA1iEaVN5aYvY+9S5y1xNite/70q7hcY4v4oMxeRhOMYJ+YM/FHWX20kLmwutHxJ1CRVspV/9HVS10otA5qDQqzyIndLeIX9Lo1MfT3M34UbKekNrMOaS2pyd0D058QsxUKkZPOY0ZzDs7erZkafSXnrghgIiQfzcXK9DT7TTpXVtyGzO5fFBFhk4wWjHk6+h91dTwvqiKxPVWWes3D18UVRWi/3yqy+sphjOv6Xp+gf1LPZZ4T6K39XmYQTMFZD1pOzXW8YUmVaM5h9T29HQ+/hhhFlRdVWGjiYrRkyLvd2bJQyv8xRxVo/SXngLLvOnE6HDxjRYrH6xAT1kNqZL15Jz/kMtHo9XM9xjNTIZq7875D4jO9yi9vvXAXMNaz9NCB7vuetOr9MWMNLcvdD1fN5fHub9xKdG2FntNkLZTu0I+MfOQ2p6eXPL/or9cvBGsGD2h2jSdxl4x1FJNhPpLT8zu1qMVQ7ukdorqM6xAT4il3hLngyXm1L6QcFww8U6ivYxao0IuQPIixnsapRhC/6LGVofPcnuHL/ORDoPx8U/Qbb/kZ2p8vV7Fw6enbUHLD4VvYcZ+Hu3KRE9uBY8vJZAjGZyNO8KtJUZP24M+otMs6p4v3jL0l562skb7Waacau7+9D7WoadfM65Ku5JnuL6FvyxLr08S7sG73n8h8VPZpGr4yGcmrqcH2b/QU3V7FzsLTxq8I/gjPL1D7j1pezTR+RXzhxjn05OEkI+e4qsjiQ/nuI/gvn0xelrqPZlO85nhF4doVjXlN2ULB/24QMejJ1SLmeH2tkDM8xidUBNNZCVeTyHlfiNY1V7c3bLFOvRU3V4pPEiuQODtd5FlNgYYmfn6E985zYZPdrIb0nE95TRmEC2hvIqdjVaFiCfokrvCfxvzufnH0yb1pNF2zXa3Iz6Pq/574mIxeprhxhjRiRgapeftHvkYno7RiiE52HNPPZL73P2W8SORlRg9VbVV3M+6ydd+OLoqVODrkAnWoSfE0Yjt0r7awxFb8XzQRWJ0CJRtQSvEz9EUUxVmVJ2r/ebigitszpV2ZzfCYVBGfYr5B9Mm9aTrbn9IPjy6mHBCv5YYPTGvZKKWodKomM/g6AivDCRK3tt6susefO55faATTOA8X+U7hznMqdywGj2l1MabNLIS9oUNwdt3oG9lT+hao2sx+7LQVLaVzzA2iCI6m+OqI/C1hB+BCcRWSc8paGxVT9xLVS7me4zWz6ZjVE9arWas4wt0GvRl4VuXuZ7ExCiH5xOpu0V5YjV6QufPZ6wnl2LiXNwXeEalLUWTnP8rvAo6BSMFL6fuAmm1YobxJVrNoBtVCaMv6iMKexVlDraqpy6terrrm8Qi/etIMbWncazv5VzcUTyNtesJVcAf5twR+CJkhRXpSRdfEymtAoVuvogeJ+6FT4xmtdhrAtExgsCjSGF000u9J7cadh04E3dY2om1MWCxpY4kn55up33/tNCBGQ6595m9pmWlJ8Q3MQeIRT8kndKJ0xOtNhQnovbgafpeT+85DPYreUpkJU1P45xedMp/IPAtyA1r0hNif+h6adf2rpBPiJtt+j00HUR3FpyOrvZ5HqOEV5/q8hoxd15qXYKYUaLoQDK1YIXc9to9cXoKLfcjFqGfGY1WI0ZPzNF1dgWTrcyORmxb4GGPx2QXRmVcpJ42PFtU0VYqEDXtVfRBkKCnhR5jCptzBb4CGWJlespvyh7j+B8Jl7cdNd5gl7bri8jPhFdBlwfSELMkT4y1DJjg9HJcdTi+Sqem4yOfmdIKzxy7WjI2rCeVpnOy83B8ETJ7ZkOKGD1tDVpOp1niNcno8byRcp5eUaSeLNjuCX1BS7wnL/Wegurs9M0BunCsbt5WK9OTjuc8FhMTnV/NNxxbTq1Rn4zeI7wWd97joF/jZYItRae4DI+tDiPWkvxEfILzK5Y9sWxYTz0JdhFLb6SeF6On03GMSXfQVW20Z79M9IQ3LGA+qL2U+JWEbfUj1qenNnWr5O4gy5RTGjsNup4j0dxOvSTwmp85pLfwLGOoePS4Zej6kfbgDMXDbAs/y+xVPRWw+jbaGTZAo7mSdIpehehOpMeonp6VehJLlyunMi9XQk+Pc+8yS260iZAM9RRC3eTa9bTprbeeaVp01qgnXU9TI2lPcPS6oUd6RVcOX1u7UYrn6Yl3fkj6lpkYCehE9G66vy66DITblAvE5oClPKO1SKdX9VTZVs7M/Bk1giXO+fgv6VWWeDNurIzqCX2/EwwH7ULfyzxWd0tCTxn1KcySG21lIkM9od9dZr/0m6kXJWyuv7BKPSGuJZ+VdrXbdfcv+Zge7KlZ1fR94tfMB1vKYlci8ce+s+hky5RTmYPDog/HOb0orajoJrGstdjiR69X9YTswKyNKvJ+FyjSkYit9CrMl5VG9YQ4zMrNqJ7QzwCz1+Qcdzvhd7gy1JOu+/EoozI41fUN+Y9Cx2GtelJpVEa7pwjEev+FzMkIy1tLLiWenOxi8GyVmPAOfbv2jgZVobX+8zyLnLpYdRyPQgWRWHwgHfiVevTG0etVPaHf7TlU55Kew/iVQJFW+sygV2HOtStGT97FLhL0pOue8/kwM+WT3HsChZenntBvMHMexvtZNyVssV+wVj3pursUldN9rMTHfI/RfFdjR1e7b4n7yeg9CzzsRzgMQrUtfGlGfbJdz6BLG559cDvt+1yqa5UetUaF7gElP29CcTX5jOWPWg+9qiddd9f/lXTKVb6zdTwdKWo7akYrhtCr3M28TicWoyf0EyKmxkrrKaU2jvmVTXN9g5jKCUeeetJ1v3A4TSeb4z4CH6ZRzlixnhDocpJ832TXM+v8nfQrwt3rmlQNxFxSzarGouY8Zl2JI68xc63/fMkFQ3EgbIPwJsyht/V0iz2C4CC+/H/LuMYsT0JNFJ1YjJ504prIMW/G+Wrlq/3m8o0CKFs9obsBZodQ4Rtt+WDdekIElHlLfkyujxU+0yMrgyzVQxLJC9V6xki9odPH+mcLhWdtMJPe1lNafSL7UCun00O7pdYlTqCmn0Ax0+1tFeuXQ6Se3AufSNNTfHUEX513qfeU1LoEehXZ6knH05d+kee43vvxsyBWryeEa8Gj96QO7fZPDNoauDy8IsCcd2R1HTU/pV1mzilmUqz0mVHfWWvB40PT23rSajV8DVDnPR31IPtndJEXNOfGVodfSTrF1wPxe573ZSL1hApstAUv3yzBdM8YLkY6DN4dssYp/090rAqb83IaM0LL/ZFiJOtphutbB8M3C8eh8C1B5T54VuL1xNcIxqvIme+7lg+2oCeEY/6fkgefxONDrwlIMbnUiE4CtKpbAsq8jkZsY/Z3NzVWKKfVtvf6FJ69rSeEstjVnOOAnMXXElWknhC7eCbINaqnFnXzcuVUM79KC3YJtuserMKg/Z14PaHbgk9ZEzh+5DND/mOq2IiedD1DgEseso4I9GuzwMP+y6idf2TdDq3wLzDsqYTO3ZTaeM8ix6vJpzcHLJU8/AAda/zm1Xf0br1JTx/oCfl9Z/Ankg/FPWo8Ug7xekJ1HOGt8OkJUdpahCp65nybltXT5oAleFYmDebL91MRXMaYZEhW2I6eECEVfhOdX7WULLiY6vo6/jvjwDOfh5mxO2R1nzVI6QM96brvdqs/ZHWyNRpHIrYJ1F7F66mmo9pe8BdLQE+Istbij1jNHURGhGz0pNKomJOAbHj2gcDuywGb0hMisyFloecYy4qjt/WEKmsXE07gY6L3Nn2jJ13PeLLr/ReYdChOxx4WfpcqXk86nlkAuBDWk66n6dCFhOOjWI0ehGOi8yt0e9r+0hPibuZ15tGONey1LjdsTU8IdH+0K2S1BfXRq3pCp5T5M6+YSi5rvkn0CdFlGqe9q20s60lzoLHp1NFPN7pHnuXOO4cNFx/5zGTOaUrwXfwxet2AMi9mYofc+3yb6x6jpjbG6OYQ2Y3pX0buFPlscZrrG5cST+Kz8nCciBY1vzEz9oWuw7OKryHnfbDrftf5jppnbqiGzjrmqC+Xk74RcwT6CxvUk66nd8K9zBuSh17pMz2t8p1NDAjVZ0RVhXgUKvBAnwivklqXQKwSVKYU+Q6hs6sjoNT7XNzRdf7zZ7m/O87xxdGKoUjN6KZjW9CKH1POJdXGisyqSdXoVeQsshhdWnVAmTdRbH2gqpNJz4ZR/dGzyPF07CG0C7Pd7cY5vYjuHNG/M9zeWq6cui90/c3UC5GVwXz1F13PD6dnkROzMMKBtktM/YJKHlLuTyTLbiA7ouPkNmYS6dFhZPadkA+2qSc9OY3pq/3mylNP9ophN1MvqvhPZRtGq9V2abvQ7zz6V/4vj5igYnO7IP4lL2AqtqwnXU816mHOHaIPXb/raUvgMr6uMAAAcNi4nvTUd9Z+F39MctdcC+ppifckv5KnVlplAIA+ZkDoSU9pa9Hp2EMSGk9aRE9ITK4Fj+Q/qz0AyIcBpCc9VW3lt1IvznEf0Td6GukweFvQimelXlbRxQkAZMWA05OeTk1nYJnyUPjmCU4v94aeRjwZ9KHXxJupFwoNJ7ACAEA8A1RPHC3qZv9Sz1OxBxd6juWbv0y8nsY5vbQpYMmd9CtZDWlaeKEDAOYx0PXEgQRU3lriW+J+LfnsntC1i70moIqVvu0in55GKZ6f7vrmGr95J6P3/pF1O746sldHQQGAgQboiZfOro6a9ipUD0ownP+ysq08qTa2qDmvWdVk8UkK+oycxoyoymA80CfCq5S0FBKrpNYlMN9C1nZUR1WF4CnjayKZrwVQ7TW6KhRPGVMVRs9VIYbq9gqieCKDmJyyoClHSj5VIcz5MgFzAD0NRNAFOZIaw2+kw+DilgK+VTq62idR3a1R7TKMNT3Ux76z6Tvf37Nu0SmPRGyjU56JPSxhpyRPLzbW8QVuoIhaY72IBWKFcho0GbEsoKeBSK92CUaXKHNWrh+STtHZbmF12d0ftkHCTpnT+BZVDPWZoKqT5Exmur0DLcgtC+hpIAJ6Aj1ZBaCngQjoCfRkFYCeBiKgJyJKW4r0mZijp1lu74KeLAvoaSAycPSESrLOf4FwnIjazQ2Ax6enJd6TjObzc/r/JBQbEAD0NBAZOHq6lXbJpEz49BRa4S+hSICZgJ4GIqAnPkBPsgL0NBABPfEBepIVoKeBCOiJD9CTrLB6PSmLXfeGrt3TE3tD1wWWKYkEKk3nyei9e/5Ns9Yx7086n+8Tv+LSfB6+qbq9Uv/5jynnuM/3ha7PrE+h1w0p90Ob5pI9yvkNXxpeEYAvfZj9C50DuvgPR2zl0pyI2t3R1S7peIgC9MQH6ElWWL2ebqRewE+jA9SZnVafRJxqy5RTiTQtqmbDmUsGFbfk6xdNd30TX5cpl3PxX+BpPn22EF96MeEkvnSN3zw6B9oX9DREFgT0xAfoSVZYvZ58S9zx02iJ9yQigUeRgjjVJji93NHVgadBlyWeYIrLcO5NM+hJD+hJQpEAM7F6PRU15+Gn0TinF9sNb4tupJ6nz7ai5nw8jVvBY3zpev9//QJ60gN6klAkwEysXk8arWaC8yv4mVRgOJfk4fAt9NkWXO6Dp7mWfBZfejbuCLdoQOlpd8iaE9F7mHE0Yjs9c6f89XQz7SIqj3DgmQjqSSsYgOWxej0h1hlOk/2s1BNfutJnOn223c+8iac5ELYBX+qQe49bNKD0JCFkridUm57m+oZALFdOa+is4zLh09N017fmPh3FF/OejjoWuQNGU7E4tqCnM3GH8TPp14xr3KIubRc6Qemz7dvYz/EclnpPxpcm1cZyi0BPVq0nMZFcG8dlIrnP3VjHF3r1ZevAxBb09CT3Hn6inIzewy0qaSlk3pJsfLaYS6PWqu0V/06BZ68Y2qRq5JaCnkBPoKf+whb0lFgTjZ8oa/3nc4tCy/25z5dgVaRZ2NgXBc0GZ+QHXuPxzEFPoCfQU39hC3pqVbfgL5Wmub7BTSr3Z9ZP3OffxBzghqMd6TCYG781oMwLP88Ohm/GMwc9gZ5AT/2FLegJschzHHeiIFVVtVfoPz+NPZb6PevWSp8Z3J+JNTH6NHczfsTPs5/SLuM5E3q6lnw2pzGDiKOR28XraYVyGp2DZ5GjHPR0LeWsIu93ZvyRdXuEg/W9uTMa6Bersq2My0SynhZ7TYCZVi2OjejpYPgm/FyJrgrVf745cCn3YWCZEk/mkv9Qn+ar6L34uoFl3njOhJ7EhLCeRAa0ezIVpp4uJ31T3V4pEC3qZjwTPj055v+JFgkEkQ9gEWxET6jKg59MT/5pGTDL7V3uw/ym7KvJZ7g/rySd1qfB2yWMcHiutLUIzxn0pMdK9QTNMq0aG9ET8fzoQsJxXfcVVTdS8fd0SaMVQzq7OpzzH3Jp9oWu1/VcS1NcXuM+nOr6OjF1HehJD+hJQpEAM7ERPaGLGT+ZdgR/jD5MqY3jPlngOQZ9ElcdwX2yxKu7d15NeyV+1W0K+JDIGfSkB/QkoUiAmdiInlCVB68EzfcYjS4SvCedXlg17VVcMyj9q5aY6nD8LDyf8CWRs8UfjS9nPxon+y2DnkwF9GR72IieEBsDFnMn02jF0GZV07WUf3vSfRd/DKVRa9S4xdC56JB3Hz8LnfIfENkOqIYFoCfQk6ywHT0hAeHnU0Z98udhG7k/H2T/rE+2yuff+bUDSr0Id6TWJRLZgp70gJ4kFAkwE9vRk1P+n/j55FnktMx7CvdnSIWfPtmRiK3ch79l/LgzeBX3p71iWJu6lcgW9KQH9CShSICZ2I6eUg2HlLuSdGq800vcn0XNefpk11O+4z78KnrffA977s+l3pPpbEFPekBPEooEmInt6AlVfEYrhnLn0yrf2dxTcPS5WqPWJ8Ofly9XTsNXORqxnc4W9KQH9CShSICZ2I6edIbjouADFeC9fBNrYphp7LpHYrlK5wl60tOXeprm+sbmgCVGY1/o+tr2Ki6rXtUTKuexyB3CcT7hS/rhAGAONqWnIxHbmOfW7pDVXJq6jhrmZYYipNyPzhP0pKcv9SQ+lMWuXFa9qieRAZUsy2JTerqTfpV50lxIOMGl6dJ2oR9nOs2IJ8/hXUM5QE965Kkn72IXLis56Cm43NekzQHC2JSeQsp9mSfNo5xf8WRr/ObSaZCGmIOxgp70gJ5AT32PTekJVX+YY2OGVwTgyY5F7qDTbAtawcwT9KQH9AR66ntsSk/oxm2W2zv0SVPaYnCp3079nk5zOekbZp4zDTMkZgDWcz7hOJ5mY8BifOn3id/gS9f5L6RzICbaQ1HRVir5OBgluyGd6fG8piy+VdrVrfaOw+hV/A0nntD16OlD74l0SmIgLT17Q9dZSgdMJ97PuklvVAC+XziREVsdbtLmAGFsSk+IxNoY5/wHeDwr9SLS1HfUuhT8hadxyX9Y11HDzDCmKpQbks0p/0Gjqp5OU95a4pj3B5csoz4ZX4pEgy9Noxqm63rE+rRQwaXxLXHv7Wk/0IVNDDhn9Jc/viaSWEVZ7Mocgy23MRPfZRRuBY9a1S10SnRwnPL/5BsDTzjQ1rkRmRGZDanERt0Ln7R3tZl6ZCIqg6SVx7/kKUzWYllsTU8AANgMoCcAAGQK6AkAAJkCegIAQKaAngAAkCmgJwAAZAroCQAAmQJ6AgBApoCeAACQKaAnAABkCugJAACZAnoCAECmgJ4AAJApoCcAAGQK6AkAAJkCegIAQKaAngAAkCmgJwAAZAroCQAAmQJ6AgBApoCeAACQKaAnAABkCugJAACZAnoCAECmgJ4AAJApoCcAAGQK6AkAAJkCegIAQKaAngAAkCmgJwAAZAroCQAAmfL/AfLkmNlZcvJNAAAAAElFTkSuQmCC</t>
+        </is>
+      </c>
       <c r="N17" t="inlineStr">
         <is>
           <t>Healthcare &amp; Medicine</t>
@@ -1989,7 +2029,11 @@
           <t>ADRA Myanmar</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAZ4AAABuCAIAAACY++L1AAAACXBIWXMAAA7EAAAOxAGVKw4bAAAYS0lEQVR4nO1dW2/cthLW/+lj/4AfDgoURYv2YXGaNIm5TmGgBYLaib0rabeAfvqhpPV6Tc2Nw6EkH/MDURjNijeRn4bDuVTVa8fuY9Vuq2Zbta5q3PDf674cbuDS//j69OODGx7c9n8UFBQULINv76v2+kRkGHOlF1/5SJGPbukBFxQU/F9iv6kOA5e1ObmMLrWnuZueUrtfl56OgoKC14vNZiCU5biMkelcT3OecwsKCgp47D8tKZopy3VVf1p64goKClaIGtf3v6LSDtcRBQUFbx13vw4XlEtTUo5SLh8KCt4idp96GSc7xQwWHp49m6cDY7fpLwT6f8rfeq+MKwfVgoK3gC757EmYqj1zyrYnNQmaG55hW5fKg76GLuu0FhQULAglLww2H56DRvgzLP1jz32xaDizkvr90xBGe2DVRYfvWGc1lQUFBWtArTJJ81zw99WLejyvEfX4VjZaa4yu6s+PBGM+/PDi9/cbpWGKl+AKCgpePRoXfVHgeeRvhKGIw2N7Az8ShfoTxbMgPMfFsvZoE1dQUPAq0b6Pc4Tyu/3LH2SFuFS1s9PWP3ykekigl+NijPL85NTOrNsFBQXZ4a5ipJhtdfyTr/NAnEOdcf/3G/SuQ6LIO3yOIDhPl866/wUFBfZo5WKak9bZ4JLU8T3/uAIUk4olxCiCKygoWCl6rZPQMiNyJ2MckfVAd8DHch9zWeEFQNHBfNtfkhQUFKwL7Qd+9/YmaS66ZsymrM3v0oTdWiiErMO16DqlLSa+BQXrgURYO6puMA/YlaUzHgIGjN32qiPkccsTXF28UAsKFsftrUBYSzDLAI+iM18sYsdhNSTiW1fCJRUULIUdS2qu+vKjvv4jpqKaV+m+Q5hI4fZwxl8/8R5jj3luSAoKCijwzu3JByvQAmOR8xp27ZtaLXe9UJeb04KCOcEeqfYfUpvA9HcpYqAa2Lk73WijY53zLbwsCgoKeDDymouzjcAAVn5cTsV+zCO4VUOodNoY0H9IVg56Sdx+P3d/6s/Vvzdh6b/HW7wMv5nzw9m+48492tIOnnz9FdynXu9hsh/VoCP9rOjL3eJeliOv2bSSjUfU6LDIJUZsy3ww1n1tOiaywEr6tU8mCmDLZVgHc+SjNphErpeJAt2RvklrMVanNd8pavUAcP1OVdXg11kPYZGa4SvRh6L8XVPVHhq+oXkdzW4rdzil4qC41MqXojbgdQ/5G03kID21OaD0gblkkRDb4Zdzyqd0f5Y3BqB5zTDvyeN7uIlY7DkrWQVXgvXobNxA7G7IqE0r+cRBoJdv8y6p8vbmlCkxjgK2Tw+OZftces/li3JwT2EBxQQx2p/XCTplL860T0QTNS4WDz/IMltuq8dZaIXphpujDygIZwM/g9/SFm7YlsX4hcHUYs1TYMYxdSHwk0k4ZqXfz+QAall9sYussN9K/ZQT4ReGJJP3+PlUBwo84/BZGiknCuxc5Q4gSITSOW2fZT/Y2AT59xrEaEwEdhd5K146t9+L1sdl8bMvB1hDFz9SAl5EJw6ndOinRSAJBGDc4gf+mt64RcdoDDwx7ZIbvSe1lupx0XPld/ftz6k9xyAKErGUCSf6Ll0cKUgAX1PE8Hosr42LMqJ+aJWYf/o8QWPLcYX5ACWTnOPjTG+bHPCnSFDl+rwStv3nORE0E+nA5vfokrsNtytYG8tcJmCKAP8KH/8b/th/cwKh2r+kqA8CvCvEm1mdn0XOF7tf4NmQw5909i/76ZlxKot9w9XMK7oy9xMiUxXlsLWmtVRZQbNPoo6CPuDr+8zpDcyxZzUVs7wsAJgxF9gb4lQv3Pmb75KG7TlUx2uxkwsKC0IQ3/zmpp+BSzzgK2M9VwpEbLsZlu+Cu+WOjHaTKIlkGhd9GWguPclvSGYI5PMC6Kdp8lHifYYEXQd1GfIx0ycFvogbAtW9kjMp+9n05f7l3GJh4wxNbRIR9IoanbNvvcalp3lA5NPwH3ssyweLTNRG1+zL0fROLNjItPnufECjlU06IckNehAEIwOXqdxuQMlo54actCFQ18tS8D9iO6bAfJ/QCSyO6YmD0LXn0BISa282EPTa72ddOK9sFEBfWRq6vgRE1lxzXiv/MWuaQoePP9CdydVbrFyT8iIbwdUSW+QAdxSNCOF8IpFhG/ivpaODBINyV9Xud2poj9bCJrH85sSePLVoYpdmo7YKOXaci5VxeHCSG0G1O8+nmlCcXYL2sJkW4rsNHtbkN48HznxGxCniyQW/P494b7/8GNeTwN79+Ccyn+L5yQRwbdhucqYD66C2ShALJwpW9YCoueVngssKz7Q1Q7sU9uJ1yYc2CopDGwW10Y0g2dWpJ4mKtnGAcnUbeHbGH69JWQboyWSiMCPknbX9jRzBJJxjjtJCgS3WQ20VN/Co71DuCaRNea+uUusPxdgztZHq5uwJyNFdNJlW3gw96Dr+YkCy+Ci2B1ZkpwdKlIFbzLITqiOfi5OOcUEH46A/3dP17vek1bQulDyGVVFbxa3DvVhJT1RiAsbzIfky4QCdRkcQlwl5HaUPyBkTlGgMuSPxLcqTBOq6B7QIbSrM4UZuIXGabWjsaCULJYu57ENwY0tQue2XeW3UVhmdudJrYOqn1W3J38sXFb6sjWb/dJc1FNii5AcgKQ6upwPvHJEfg6gRp/qoEgVwU2HuGdEnd6Qz2Md2fgT6muC0VSPKwbF0DqxSgxVSGyuhS2C1SjEwrp1pGv1glQZSEe1MlpJKhUHUUGO3K6aNAq2WY2/NYzsTlFhbCpBlsM+dxDdQ8oIxirxzcZ1PR7CBga7OonFbIbVV3BliJ4ipNcfUEZ10STU3+Gn09IMMnmQMsJ0T+3usYMYKIE10V3Gdj+rJtMRSG+j8gEmasTekxJybdD4R4XCg1um1YYV1UhtznyA47s0xddmojd0RTGiDHCZN4CvZ49vmW+QxEEOK69IZiY5WikN+1BijbhII8+Y1hCAOaAsUxh25fK2iM62T2iruQ8vG+FNsIsMepuhDJR3uOiVRWHbrwDljy7cr8bGasrhucmO19anNxbyVllQ/yV8tJhHsZgx2FDSNZT+gLhOMxMzVUhsttOrM123HRa3AhLcTGKj6LxyIWaO2EAuxuelv9OEukk7CzwUZ4QigRe3kathN2xb4eojo0kILFWLsRA2znUmb3160SxiR0+cOk8jRq6U28GZMuE6qpaktxaJIuCazhk4JwUamxaRowkNYyFOGk7uJZDc/arWBIlwn+VZY7SR2FK2vGQ3ObAZugcsk7RpMddhil66W2irOjJy24M1NbV/+oJq406oLAiqghVOKamy/07Rf/pmkwI8tlumqj9FODs8/iF01pphrCT1bUySdxuGO6yTLKI5pQl+LeRA06q6oH9PfS4POrJnauE8sgdxvOZNxWeCEsCfrmc9rRbJ5xnJ08OBb9xRLfnvKHUVAlJli+LZ/VRHQjksUojvz+gM4EenhXPrf0MO/Oc3V6QVj5jUxd9DH/ILb18BkyTG/p7+X6VGa10xtDz9wiwQXjnLv+Uy08mJtcPuLPu2ZxVvdxduU9lFK4gXX7p3WKcopo181A8ucaU43ZX0SEFW3+9QhYk/YM/yeVzTHho1KR+BfLPEcova2S+3Pmqmt4sSFXaRzjuG4cnBKE5gBC0QHil6szqQp7uV+E3p5gfgC+zPs47WRm2eGHFoE6vfSPEOSbu8+UJlBOtcb0yS9iPz7OWhRkhk+65l05dTGZIpx6IP5ZqzKdnMdVHUUiOTMRZPTd+aiDYvIGTMXL6TUkdn2JPBE7GecTZi0wpI74tVjYM4mO/9iEZlOL9EldWnl1MbeaGHXxMQj6aCEDO0SCnLRCSmSsW02Wc/CxJ3rLOfkuGqx5bA9JZ20Ei2XKlkRSJQR0fSId5eYQ2Dd1IYlnzwXzAQk3yumcpi4hGqDFyGuit7XBgCXCB07dOXFz3VzQVhevqufkoS3gyGFwmV9PSUqioEVgrbkms8jOdUpcvfaqY3LiosJJsQjKWjIKPbqTA7VRBKUhxGk18a/6ew2lVbG40Z3tfw2LuWy+M0wqjXBf82H6X2WHHR0gCT9zrqpreJuEjAdAvGIGrRb5L8Jd1B/T96vHDTDGERwA7fQGXtBsu5S5igX6w/U4+RDICd+jdwJxKDeMrVh/Yz9PQvaYqlJu1sPNBWxOt+8TldApdNw4dve48p8u4Kk2R8e8xGESdmiyyWLwm6y+GamtuCVxYK++VU71qyf2lhLeBCxv6exJ3htaxD9MbgNIJKEgKDD66cmAAEqRfS7e2ezdUdGq7gtelgZx41qO2rehs731stGci4m1MxJbUGKeJ3unx6mDuunNl06GKuJ8q1j3NpsbQJ23/1qMPPEoTD13h8cOdsbDcdNXK+EW7Qevu0m6V1iiz+LHa/hbxG7+Jotn0AInCXs0yJv2hAzXLno8AqoTeVulThRNbc3DXOhqcPtyEtSGprpREg0IHtx8FiCKBXSR+/cO7hzWdnTTkvPode861LU4uvPBbIOS/J1qte9ArnX7kGrMH6D1LaHyrgdjuLtcGU3wBnWRlKqIHCJsJBTGwFQIohF+ylJsmhHj6h4X67YwQq5eFXUNo9CQHnIfXvUZlKsckexfrJWRQ/QZJeFDbXZ6Yzmn7vYql4jtc1m3qjAK6A2a10bWxqZ8blJPo3ZjEPv1VHFF5TadE3DVc27r7AWCVhRG2gplsnRap61exB7br3o2yunNkznRTzSbeByP/7RnWpgLVJNsibOZhOmWBsnwBzPbRUbaoNuBnRImTsFgnizY6FFfStqAyO16F8/jil3NJ+SCrV8nUH3EpeQOZh3ndNklxWpEp00byavL3Ft0LZldFxiFDsoLyG7VfIdSGtBQrMporgsfSfAS4dcLlbUBja9d5pRMA0F1pjJ2Ybo8Fmx9b92asPGa7VQ6dYTnTSDO7F0b/Y96XKrT1EK1DULtYVhnhKWZhSXpTcHWqLUpPecFbXBPqSfNaOgkYMvDDM8rJzaWB/SDnnQaqHuSGvYvjj96AJqMwFt3aWtNF6db0Jt4OvXfU9i6Sxx1kBLDvpUZUVt82xmSVI+TbXkJEhiwJ2xcmpT57UyXKjsfYIuF9pdnrVBhyCSXK8BgA+GjnrEhNoqlcAorEdeNM1BC5cOim1CbeCbypHRqrFwQpjiTrvhp1g7tZGve4930nahMiHLnKbO0HnLaG08IGc4xdp4BvyFIevKSG2qMehIzXbF0DChNng/Z6C2fGRhFXp35dRG7VLyfdkuVEzncy51PDE1GU6jYM02rzW2Litqm7Lqq6A2RT021AY+4jRDIBC8FFvLEvqq9Iv4iLRmaqMVbXQ+OvO9zeYPiorW7V7WZntiYC52Y/r5DFB5RAiBVtQGWsecLXQi+v8GqA27IDdH8FKO1jlliOHLt8qaqY02ZaBhu1BP/aH1ADGCW2CwZa4MIfqp9KMA790IAcrsQApNuiLWSiydpawYTO5gnkqmNvD3Zul/ntBN3og5aMFNiDVTGzE69lBiuFAldQp79VyVs+kShiz3pPCYkeqsqG0HjUSR6EDYGZP5gieKO0klUhv2eHcb3X8awaEgR2p6evlK8iFVK6a225+TFpv9xh7A3NjKheWLpxR6Or6f5NrQXibETKgVtVXQu1RIuVFclrhiYKNZTtLMQm05nBCCJmZ34RLaZ66W2ggSkXyzDRfqJbqOWXiSTRec7dRhRGlQa0O3GlG2gqrLSm2KtxjFZYltgR8WFinUhiXISIz+PMVfkyD6mZCeq22d1LbB94VQ4jBcqAF2H1L3QrDynWxEsWDM8XTshlU6TQ9sSG0gU9z+J67nciJLXzG6SlKoDTY8zCBPBaE+zBV5ZxxIdRt9h3iqYZXURkTlu/lFVkM2aqsERryEbWYQl8EwpGWAHbk2lPekR+SgOxWkDantCLYY6TkUS2fqFQOvXYkwr6U2dLdkOA7MSROJKT9WSG2Eb1MrTmFntVAxsBE7sEu84Gf5qG3als087GXsZkht36AMibHygrAz6TMFaiQ7wYM6asOkmxzy1O6PsJUoz6dY0GGHWY3bCqkNU4HHWVdkprYvPzIrEDs4B4q2TuWkJQSWbFe4NmDcf0ZrvNSUG1JbZaFukxNZYkPTSRdeeiiorcO/sTnUHGGK+Ax3FJeg7VpZI6a1URsmhMZOo9VCpbrKCW7TQ1/gBZUpPuBzc3T6Wr0VCPaSLvOTmlIb6HzTvIvp8yzUhiUMlkBBbdi3a57AkzlcUwOkGDGtitqwl6uJQ5ef2iouOemUPoIB6slFDKs9GwLbVOdzkLHUBh27oqxm5ESWMk3gdsoktWE/yKTan3Yv62l0BK1uo68U10NtVvLaiCz7Gew2x24Pl1m9X/5TbCIR++45bb1Ttcvz1hqm2JbaquQzqbAzia2k5KmJorYWvyTKpL4NmCKrkvhFu/hU0CS+EmrDchir7XJMFmp6W6dR/Lf/WcAG86yNm1/Mtm0IIpuRl6fMqQ08k+qMpGOLHLHb7xJyaiMOC1bpiAJMVcsm4fMlYLYWThAEtdHRpQxheA49g5iN+oNZz0dIslKN+d5e/M/8mooRdMd0web4qrGLVDVxgKtELtILO5PSQ5Dr5VwjpDaC1/LRzTRJRe47hOemuX2leDCfOd4ZxB3IMYGA/iFNunJoPw8TI21+ic715aC7kfqWNVniVcSBjaS70j9r20PwslKO9JzQmYQRMDtvJvFwCnZaWkRwox7JzMvYgca3m+jSSyuYMr0UMDsKURpr4RED35OUFy0/eCYSR4XcXaS7p5j0ED7+xOhTEqktk4KDCAyZyY3mEve03fk4cOjjzGYe+JacpAaEX43sDZsaHW539bwd8rA2pjGEyywHUjo8zLkk+bHSPjEmxDHiHpGNRZ3M3EPwwV2MGJVCbZl4jYkGITNFVsPL42yUxNPwJ/uZPUz4HxhG6Ow21Fz57nXJN4a3PzOmMM9DcwbNTeGni7UIyb0gz+iqXqEv3SApdJ+SKToK6vgW6u5JegjmS40VhtXUluND7T+80hS5eaI7CLfx5V56fB/97D6NBf5511MkMVFe5sXOy1GgHTOwCWkzHAzBpQ4vSydVFsVCrse/XKX36qRuQvlwWtJbEcWBUPVN2ENs28QNTUVtVlcHt7d9+JD+E6VYN8Me9hJW+1mv7/MP9qeeLXXznrFsTyRFGGT5Hh4/DNmCb3j2bKGYEXL419GMpJkgNIzFf2J7U6GPZqrYqC75FdUOy+PrNi4Q+Rl+HjyXHYeqFBQfvOV+NhSrVLcrYoHNoOIpkx6CEqtCIFdQm+GNWOL+CcpdzPBtm1629Iq2ZCG6hZymzYrFmrndJHBujPSU9WXFQcFuscA+mPnmSFGzQmccS22251DbRfPWqK2/PdhG57fHsH5qG9F8FGstLssrpbZqUDfmbQBTEsenekrvIahY1QlTcmrz9ZvHL223luU2RoFl2/Q8pRkMpzPZxz38lrPneTI30qE4zmU8D8qR9SVqsL/NS21gBLcD6bmWg9owEt+reEdObfVPmvoLCrJis6keN6E6rL3pdbj3m95USJGIbo1gDYtSqK1C7GOJiBc5qA37UilHJKA2/5v7/I7HBQUFDCRH8VbsUXCJGrFxw+4TzKmtxWKpq+6hRLaByNAKCgoWgFTR6KKD5KA1O+DHttSGpVmJ1dF6GV5oBjmbY1NBQYEUXiiTKpIi7bYxU+Hd7+EvDakNizfpi7zzG9J+/bJkMi4vKCiwARFibLqZv8rEnwPuuBvcxFtRmxctsaOo0P3gTpAS7VShmy92UEFBgR69qCK+B+zviQVkQVTY/Pb8MxNq8+In5i4u4aDeMltu9zdX0KuCggIbHH6P9NXYMvuciE5xlt3Sqe3Rodo9moLbD3EOIr1niTOY54KCggVwEJv5nct+i/q4UnEX3Km5FGpr8JMvZvt356KjBvgJUeYZKygoWBVaXBQiSu3CVNt3v1In0zot7BJhmeEbffjhRU/uN2GKdUlhJdOCgoLXh9gINs9ijntmhPSgmIry7Slh4Eisck3iZTm6hea9oKBgBqgJ7iT4zM5rjTyoGV4KCgreBPbXBnyx8tKWi4KCgreJ0QVVd75bc/GC3myZ4goKCtaLGs+j8YrKeHQtKCgoCHH/vrdfS89oN1sZY2p36ojsBQUFbw3NGFRvnSq5oWOxrv4FBQUFL3Bwp2wOS3HZaJI2Wzb1goKCN4er0U9zPLTmkenqwbO1Hur/8uPSAy4oKHiz2HxXHbentN7n8PCnvyfy1/kHh7MJ7kCRBQUF/1/4HxADTQoqcV4QAAAAAElFTkSuQmCC</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
           <t>Research &amp; Data</t>
@@ -2087,7 +2131,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>https://tdh.rokka.io/open_graph/7605d2480a50935a58f361b205f135e7f42dfac8/choix1-un-enfant-badini-sourit-95847.jpg?h=4f6e2068&amp;itok=U2nq7Pnp</t>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAoEAAABvCAYAAACTghpjAAAACXBIWXMAAA7EAAAOxAGVKw4bAABzY0lEQVR4nO3dB5gsRbk38EVyDpJRgoLkJKAEQQQRSZIk5yQChyRKkGQCiWJAkKuYRTAhKoiCGTNJRUFJKipGvF696vV6v/7m13PqbE1t90zP7uzOnnPqfZ732d3Zng5V1VX/+r9pZGRkpJjOuswySxfzzjtvsdhiixXLL798h66++upZs/alxs3iiy8+9HGdNWvWrFmzTgMd+g1U6jbbbFPsvffexUEHHVQcfvjhxcc+9rHii1/8YvGjH/2o+MUvflH89a9/Lf7xj39kzdpYH3vsseL2228vttpqq2KPPfYoFl100aGP86xZs2bNmnWIOvQb6FCs3/rrr1+CwFe96lXFNddcU7zpTW8q7r333uKBBx4o/vKXvxQ///nPi3/+859Fliz9ivF08MEHF2uttdbQx3rWrFmzZs06ZB36DczSJZZYojjqqKOK4447rtT3v//9xRVXXFH87Gc/K/74xz8OGz9kmQPk//2//1cCwd13371YeOGFhz7ms2bNmjVr1iHq0G+gVAvy05/+9GLDDTcsDjjggOLss88uPve5zxV33HFHZv2yDFRuvPHG4m1ve1ux6aabDn3cZ82aNWvWrEPUod9Asc466xTPfOYzi80226zYdttti7POOqu4++67ixtuuKH429/+VvpzZckyKOFacM455xTLLrvs0Md+1qxZs2bNOkQd+g0USy21VLH22msXl1xySXHGGWeUZuBvfvObxb///e9h44Usc6BwLbjsssuK5z//+UMf+1mzZs2aNesQdbg3EFJ37LvvvsWRRx5ZfPzjHy8B4IMPPpj9ALNMmnz4wx8uTj311GKjjTYa9guYNWvWrFmzDkuHewPPfvazixe96EWlD+CMGTOKT3ziE2UqGMEgWbJMljz00EPFBRdcUOyzzz7FuuuuO+yXMGvWrFmzZh2GDu/iAkEAwB133LE4+eSTSwbwrrvuKp566qlhY4Qsc7j88Ic/LK6//voyGp1P6jR4EbNmzTrN9GlPe1qx4QYblGnL/B4+X3GFFYrNN9+8dGUa9j1mzTpBHc6Ft9tuu2KD1su19dZbF6997WuLE044ofjGN75RRgRL45Ely2TLVVddVbog7LfffuWGZBq8jJOiK664YnHbrbcWP33ooeJrX/ta8ZGPfKS44orLi5NOOqnMmbjbrrsWz3/e88r38TnPeU6x5pprztL11luv/PwlO+1Uumwcc8wxxbnnnltcd927iltuuaX4wQ9+UObvPProo4f+nFknrptsskk5Rr773e8Wb33rW8tUXa95zWuKm266qfjxj39cvP71rx/6PU6lXn755cX//d//lWvSH/7wh+K+e+8tfvHzn5f+6j77wAc+MPR7zJp1gjqcCyvdpSKISODjjz++nHBMMBaVLFmmQh5//PHiHe94R5kzEBCcBi/jpOjFF1/cuE0sbv/6179madMNmSTuSy655NCfNevElDWmmwD8w77HqVLj+c9//nPX9kBaDPs+s2adoE79ReeZZ54SBB544IGlYgI56mMCs2SZKnn00UdLVowrAgZsGryMk6KecbIFYHzWs5419GfNOjH905/+1LWfsYHDvsep0qWXXrr4z//8z67tkUFg1jlAp/6iq666avHc5z632H777UvT0le/+tXik5/8ZPHwww8Pcl3KkqWrPPLII8V9991X/Md//Ec5HqfByzgp+q53vWvS2/J//ud/ylyfw37WrBNTidS7ifytw77HqVSlS5988smyVGkVILzpphuHfo9Zs05Qp/6i/K845B977LHlAswE8eUvf3my1qcsWSoFcLnnnnuKj33sY2WUsEj1afBCDly5WaSC8cFiXHvttcV73vOekuGpk//+7/8uPvOZzxRXX3118cEPfrB02eAnFYuk7ossssjQnzXrxHSxxRYr9txzz+JlL3tZ8epXv3pMrta5DQRS43rBBRcsttpyy+J///d/O9rjhhs+MvT7y5p1gjp1F1t55ZVLP4tddtmlOO2000oWUEoYkZoWkSxZplqMu9tvv7146Utf2pE8WlBEHA1ocVxggQWG/bKOS0879dSOZ2YGx8bHxyjb+KUvfWlM+1j0vK/xsfPOO2/x2nPO6Tjut7/97dCfM+tgdd7W+H/ssUc7+vn73//+0O9rWOod+dWvftXRHhkEZp0DdOouJhXHC17wguKQQw4pKzZcc801xc0331z85Cc/GdCSniVL/4INfNOb3lQcccQRJcCxUeEPtNxyy3WM39k1glgEdCwXXnhh5XEHHnDAmLb50Y9+VHmsthAMEuSnP/3p0J8z6+BVyq5YRIQP+56GqSljjkkf9j1lzTpBnbqLyamkQsMOO+xQ+ikxwwkGyZVBsgxTnnjiibJcoSClZZZZplhooYXK3JVzip/gzjvv3PG8M2acVHmcXGipmVcJx6pjMaN8pYLcMxeaCecG5QYQy9wOAtUdjwWRMex7ypp1gjo1F1prrbWK1VZbrXje855XpuP41Kc+VQaE5MogWYYtQKDJnc/bC1/4wmK++eYr1lhjjWLTTTctI9mnwUs6Id1pp506nrcOBK680kpllG8sb3nLlZXHpiDwO9/+9tCfM+vgVdaGWLjvDPuehqnf+c63O9rDnDHse8qadYI6dReTGHqrrbYq3vve9xZvf/vbS2o9g8As00GMRSZhbJixKt2JaNfgB7hSCyBJazQNXti+lZN/LFjPquM4v//jH//oOPaNb3xD5bFLLLFE8fvf/37WcT+4//6hP2fWwWsKAqUbGvY9DVO/+tWvdLQHv/aq42ySVBXJwVJZZwOd/IuIuuRfteuuuxaHHnpoWalBhKFkvVmyDFv+/ve/l6li+KbKWQn8cVswZrGBxrBJXbDINHhh+1ZVPmI577zzao/VFrFoj6rjUp9A6Xa63QMAvcceexSXXHJJ8aEPfajUSy55czknLLroorXfE5zz4hfvWFoPsLPzzz9/abLfZpttipe//OUla+s4YN1xF7WAvAhm4IXfMVM4837VefknH3DAAcXaa69dAmC+oIKDfOZvxzn/tq3j3vjGN5bnbVdbuaIE1uNZ4LnE7LPP3uU5tIFzSub94he/uAw8mMpxwe9Vu77trW8tPtJqL9UvXve6C8vNemhXG/ZY+gGBnkdZUOd0btdwLdd07fHcs/7fpnV/xvD73ve+8n7e+c53luvKsssuWx5jPH32s58tfve735XtW9X/49U6EMhiYDxxn/jFL35R/POf/yxZdZsqloabbryxHOt8jifSX7IYGNfGjjGOTPHsgi67fVd99KuuekurL15XjjVrsmA449pYDOXv9LvP9Zf58JFHHi79gmXxkNItDpaL5wJzjPtxrO/Q73/ve8V7r7++fJ/Mn3X35l2WtP/MM88sx56crQpJeE7+y+FdNJ7EE0gnp/a7a/Dnhic23XSTynOvssoqxemnn17GHjz44E9m3Rtf12uueWf5rMbUePvEZjjc6+i8dknxkpe8ZNwbAOPXvHXRRRfNmsvecuWV5ZwT5kpWVZH6AvLOP//8iVqsBj+5xLrxxhuXg0Q5IoMB2+KhfvOb34xhHbJkGZbwS8VKK5EF7Fk4tthiiw6AwpVhdqyK4ZliefOb31x7bFMQiBm10MXtV3WcdpQJwEJYJSqSPProI2X5uqoF5pRTTpnlp+h6v/71r8sqDr7nc/OL2q7M0VXVTXx2//33l30Xn/fwww+fle7DYm0+kjbH8ZTf8lqtcXDnnXeM8ZMMYiFiam86sZ9//nkdJvT0Pi26JvrJdkHQJ+ecc04JkqpEWpg777yzjCBPc0w2AYGAhMVasFBdxRntcMarXtV4AdYmKvvYrNX1B2baWNtrr7062tVCP6i2S0GgileAANCUpo9JxX3fdtttxQorrNDXNZ0fWIuZ91T+67/+q3jPe97dOvfyY75vg5Tm4E1T//CHBpjuuKN+vHu+69/znmLRmeBGn/ied6eXPPjggyXYq5pH4s1kem/6j2+29xzgqxNY4oILLpg1hwDbQGWvZN/Of9c3vtF3onuAVN+bj+rO+9OfPlTs19qoVs1rde/NK48/vszeUPfe2Gwr3wn4BRlAjtbJm2w0lAXVYmr3IS+gnYicgFhAAzdLlukiXr4TTzyxfMmMX4liY9BnIccOYqIm870ZtAJ9sbz3vdfXHtsUBD7jGc/omKx9L20X7IQ6tE3EwmNHn06Y0kd1EzkQ68BMLH/961+L7bd/4azzVqXDiQU7VzfBx2Lxedkee3RtfwymXXsT0aZvetMbGy8c/arxyxe7iXgfPve5z3Z81gsEYnxuuOGGxuUGBZ50Y4kosIFpSYFLnaT9Nsi61ikIBDx6ldpLhf8xYNfkehg7m5imIoUNl6v4HKwaveTiiy4qHnvssUbXAHiNT7XHm/YJAcg222yzjns7oCIjQSrauFf5viBnn312eW/K0PYjQHIvNjWe+771rW81Oq/2wbT2ep+NBwxnEzFXpsB7gkGMg59oggJ/zGlQqh0zapd5AaKPWYQsWaaDKBDPvGKzYuFG88cTKgp+In6Bw0ox8+EPfajjObsVvW8KArFEsaRl41ZcccWuCajr5PLLL++YMNMUJan0swj98pe/nGUy/PSnP9312KYghmBB07yL8SLOPNiPuLad/qDHAXPid7/73b7uJZVuIBDD+JWv9J/0n6mujhE0Fi699NIJ3fP+++8/sDZMQaBE6uORJlHF5pumwCwWYGvLLbecdR6m3pRtS6Wf94i84x1vH5clT57J4GpAAdRe106D1boJVuytrc1kP+9vEBbKXn0Cy2Dj+hH3wk2ljuE39m+99da+7zeWCZY9nbzFB7LmByT/msUE0pUWBjvQa1BmyTLVYjGXsoh/ChAI8PERYyYxngEIrIVI9/G8D1iYbv5vk6UfSkBgXdoX2g8IjCdaE7U28z8+PF/84hfHtG9IzH3llVcW7373u0vzezpZMzntteees65jMcO02Dj2ApWPtxZMVS740/A7+8IXvjDm/MEfcsMNN2wBlq+UrAz/5G6Lhl2370mazVwrs0F6vEUxbSN9XQW6sJJ81rTD9ddfXy70Ve0gUn1QYwCYSoM8gvzh978v24H51iLaTepAoPNXlSd0PvP92972ttJ3z3VSc6Nn57dVdV7kQWpmRSAgE/QFZmm33XYr3nn11ZWWpWBOHFQ7piAwva8PfvAD5X1tsMEGJQly3HHHVbLZwGM3H2PAoIptApiMqbe85S0tcHxJWfUnfWeJMnfxppNvpkhmrBQgVifaS3/xM7QBZko3H/Yibbh78I9k8fPOYvjcWzqu9T1/ufhZHWtsYHsff7we9Hp2mze+wK6hss1HP/rRWvN1EH6KJ8+YUfo0MkmrVvbtb397zHHmsDDXV6lNTpVlw/t82223znqfH22BxKr32bxUdd7TTz9tzPGAvM2P8W8c7bffy4uP3XRT5fvp+uP1sZ2pg11wNBSHSD4+pb9Oa7JlOzdodRgg2KvTsmQZhgCBwIaXGYjA4qQvrh3XeH227IAFIQz6neulGPhYmFfqju0nMCT2t7GpCwD35JNPHtO2TJDps/NV4vOXTmz8h4IzeKxMJnWsGp/AwPLF7f2RBPgw+6TndR8PPPBA5Xkt4KmZiL/Ru669tuM4DtppYAfXl1Q+//nPzwLLQRdpfc8Cms6L3/ve9wZWpYY/Xcq46GsuD7Fpku82v7A6qQOBu7TAQnp+/bjlls/vOE7bYeZSX62nnnqqcgFOgZCNBKBRdQ9YpbSih+NXWnHFgb1LdSCQPyk/0qrveC/0eyp171bdO+QawEAaXOK50/yFBLCqOrd1uY59YwmpYmUlnK9bt/UzE2n6HfcJQKbis7rn5mNYJUDSqaeeWmlWFWdQJ9w+qkzv3lUgNZXjjz++9t5S3+pw/tSf0Ln5I6ZtzJ81ndeQCqmvpzkuZKlIFamWVlfT/jG7Og4dzMsRVIMbRKuvvno5ODnqYiLs/E2oHGN7OWtmyTIssWs0qXiJTd4xE0iBH2aa8b4fWItBv3O9dO0WcA0siZ/dmMymIJB6p4OEfGnLL7/8mEnNQt4t8pUfZrwT9jsmoupY80cqJsU6c4jFKX4mE7O5KT0OO5oKZqCORTIO4iT3zmtxrbsuYfKpi1S1sTj33Nd2HK8d0pJ941HntgDFAnjvUePL6B7rgGAVCARUU6d9TNSKXcAXNigF/0xm8TECflIWsI4xDIrxir+DxZ3gAtmhVSBQ3+8ZsddVyoz4l790rntcHaqO5YecglljSfRx3flZGYCBWJhrq9hGJE2VKVcfdgvUqfOD6xYctVhrDuWGEQsmss5HDoNaBTZvvPHG2s03IJW2V7fnD2qTnzKconGrjhXMk+KWL33pzq7zmg1WOq/tu+8+HcccdNBBHef07HWbnKCnJBsEQHSC43owLwc1GRjAgCAGEADEAH79618vB1iYNPux8WfJMpXCNAfc8E2zkwWYAgj0t0kSAIgnsX58/bwXg3znmqoJjxmllym7HxBoV7vbrruWi0BgrF7z6ld3fP+/WwBtvfXW63pNbZo614tOrTqWNSEVgQh159ZPKcsnDUV6nHkqFUxBN9Y39VfEHof/CSyJBYvTK4JPO6QlNAeRnNmikoqUE92ebY01Vq80AVaBQCxjvNgBRb0icl3bghsLsBADtle84hUd/8c294qsdd7YBG9DMshcfVUgEMvXJJAndcswJqoYb+5TqWCVe52f+0AKoJhYq45NAy30n/mh2/nPOuvMMfcleKhX2pvUTcC16xhu81S6OQDqMdTdrvG+JJURubXH+/u0p80zxrwL6FYdyx0kFmOxV8ow73PK0N7W2gh2tk2nRQEJMf/83TctxvOfn3pq1nfqNhN96GBeDguhxdKEzyfCDhZ9q7YiEJhzAmaZHYSvznve857St8PkhtGxAzeZWKCAuDj3HFNAP0yDQKnUbDmdtB8QmKo2MonF8v73va/Rdw879NCO79koVoHrqqi/usWrzCm3zTZjWIIqX7s0gpoIEKo6rwWfn87DSaJ7JjP/NzZSh36+WE3awcY5FhvniaYlSllOjEZVKpFUb7rppjFtUgUC06hGfrVNQBGfs1Q233zzWf+/orURi6Vpfeq3v/1ts74DyFYxv+PVKhC4Xw/wNGuMH3ZYx/eAnarUJCnbzVQe8vj1Upk3YgHSqoBmGlHf5BpVm4mPfKR3MMVRRx055nt111p11WeOYSnr6pfHKlI5FZHCvb7HrzIWOCVtL/P7Tx96qOO4puUCmZdjYYmJnz1l3PkKNxuHoxH+v3riiYnmGB3My2Fhg9axAvwB5WqSzJMjuJ3ZUxFyzZJlugp/DCyUydSYtusKkXZ2r4JFjPPYbNIPE2hx7Dcn1VTqREDgOuusM8YPpmlwA7+79Lu77jrWFJqCQAxGlT8Sa0RV6g7Hx5GTQS+88IIxx25Uwdou3AJ4t1f4dxFznmO4EKTX3GijZgwwX6A0T1oVc9lUjd8UBL+vITDff7/9xjxjCgKZ4tIgvxNe+cpG5weWUzDy6qiaTcruMDE3Sbb8hje8oeN7kjQP6v1IQSAg1xSgmTdiCXku42M4+Kcs3XXXvavx/cnPGIuxFBLex5qOCUFSvc7NDSZ9R5vMDzbRqdT5RleBwGsbAC7McyqyO/T6nrEai01XmrKIW0IauNH0ncRsxpZP51GXPvw/ZSLhpSbnZSGI+3iVhultanRiL4VFke+HaEEMCT8TZhHZrjGA4SGb5PLKkmXYYtfJJAcI2rkb45y0g1nBjguzEPs78X1tanJyHtn7J5KlfjJ1IiDwlcmE+p+txazpAlkFCM6p2MmnjJ1Ju8rPTsBJlTAtSVCbHp+CQMdVmaxscOvOq18do81ikXqoaTBRGnBDRJiOtz8Bj3QBU3WiyXeN89QknIJAEZep31NohyZqjYgljlxnso4F4OplFqSiP2MJDO0gNAWB/Nyb5nRkKUtNnRjl+BiAKe2vfvyIbabStDVVwQ5p8ui6IJJY+fuKRI2lydg0HlJJ8wUGtfFOr9EtWCNo1cararOXapxYnGi7dM5K5xLvZ9OALSx+7DtMnC/83zoTiwCzJnOmbASxDC1PoAmL8jPyckLeEnMyA4sIFt2WOqtmyTLdBRixM8YgGN8WurCIczwH+EwCYfK3Q+4HBGJ7BhX1OWidCAhkRo/FQtMU7DoudRkJwSaxqpwQi7QxVexQlXmX3P3971dePwWBfMmqgFsK8OJnDfeRmkf5JDZtQwtAajV585svHnd/poAIWH3mM8cyp1U6b2t8p4xRCgJT8zUWR5BC0/tLF8GvfPnLs/6XbirK/rv77p4R9v4fwBYWJq0WMxFNQeCnP31z4+9qlzSNTQoCU/MhUNI0iXHQdM1V8i09JgWBr7vwwp7nXWbppceMzbBR7qZpTlFSBwLNt2kbvfzl+/a8RpoQG8vqs17fE9Edi/kvBWGp72r8rvdSJFm6ueV/HP6vb1KRBqeX7yvwGjYL+mSCOWjH/0KgrikQCO1zXmWukavruuuuK/1i+k2UmiXLsAUY8WKpAWlzwwE4AAJRqHyZsEnBD6NfnyNRx/2wJVOpEwGBgHMsWKSzzjyzOOjAA3uq5MhpJKh6q+k1UhDI5Ft1LxiKVLpFHaeRuXIYVoHAvRPmIIiNbzjmgQc6/SK16YyTTmrUDgJKUpNb1SLeVC9P/OosSP18/+67O3PKpSAwBf7aWH6zJs+qzf6cgAogL5ybf3lVEKH2FCCE0axiTfQb9o/J7IgjDh/o+5GCQL7DTb+L5UpN5ykI5Dsay89bc1G/9YY/+clPdJyjKsgqBYGnReO3TgGaNPK/V1Q0NU+m0g8I7BUtS4GmWIDAJum4sIXp2ErHFDIrFvOayN8mY1ymiXQMCxAK5z5g//3HtA2x/tgEe/YqgsGm+eyzzyrzLr84Mi+PU8f3RYuYnY2dpsZm52aX93LKA8TBkSNvliyzm5hARHV9/OMfL8GE4IIQVcs0g/kLZqngC9uP8z5/taZm0qnW8YJAk9Jjjz460H5oAgIlhK5beGJTI3BiY1oXxAOQxMIloAoEWpDT/GI3tua8wOxWmbUnKoDWePszTRAtMXY/31fWLZYUBFal7JmIpEEA6fVTwTzqZ36A1qAJJs3tqSkIbBogQJuAQO0bS120ajeVmDuWhx56cMwxKQhsYjIfFghkfel1jfGCQCxxLCkIXKA1r/FFHaTE75AglEe7zJvmLeZn8xxyjdl7kNHuM7X5wW5Yw3L2RqOKnmPaMoGihdm6oVfZuPnB9FuKJkuW6SL8UoxnKmVDSITsp81OSEDqp+S3/S4+w0oV00vHCwKBnz/8ob7A/XgEuEqv0xQEUpOlvpHewY66WxR3UxAY5kGuL85rEYxN3vymBl0THXgdb39+OamRLJ1JP99P05qkILBpDdWmgnWJzy+Iqh9rkrQrGEB5CPtl0JroZIPAtJwhkN3vPaqnHctvf/vkmGMyCGxrLxC4dOt3Y2qQkpbt9HxpAug68VxcNMwJ/ADHW7gg0eYHW+hE4omekdSRGUzJl8MPP7y0c/OFEbosMSnTUAaBWWZXYRIW1CRXmZct+Jf4KVDEYh/eC6kI+vU7AgKHUUKul44XBHqW8dZRrZPLLx+b46wfENiP9gMCuyk3gaYTelM579xzx/1czKuxYNb6+X6a4y0GgdonPf9EpQr0WMzrKrrUCQYF4O1WBmw8OtkgUHRoLP2Ym4Oec845HedAyKTHZBDY1l4gsKrPJirmsPQ+EAsSm/cjzMzGxwTTw9BmB+ocEZFYQKkg+GvwyaDMFfynZPUGBJmChblnEJhldhURXUCgl8wkZKPjPTD2mYgBwwDilDqqm9TqVOmwOR0Emog5qfPb61fVHl6/Isn07AgCzYPMnONpB6BoInnu0mS1/YLA1HE9BoGYtqp6znzBx/OsiIM6/y/s6wknnFASDP2sK1ySBCYM6v2YahDYrc53nWYQOLkg0LmN+/GMcf1bl2Tadd/4xjdU1hLvJtapxSa2lnQ/QEMyd8h2H5JBe1EhV4DQgsgHAfCT+FAOqlAmJg2NzpJldhKUu/HMD8MY9z4Ab8Z/nGaEz2C3kk5VavIfZDmrQel4QaCJ/s9/7nTytyEc9DNOdxBoo5yCQAv5ZJgmm+h3vvOdjnuRs7Wf76c+hak5mOtPLHwOB8BMzFK+lnEkvbWIFQob/6EPfrC4//77S8Kh26KpSsOAzGaTDgJvvvnmjv83zRsXa1pL98knszm4TnuBwKqUTciuQb7PNjjxPKm9BKzIsCLw46GHHhqTNicV2RAmcA+9X0ILnJvk/6fzgD8+FxgQ1UEMOhP+pz71qTLPTQZ/WeYEwSJwb5Aqhs+rl3W77bYrNz6AYXhH5MZMQWCvRceEOh0rh4wXBGqbXyfpROJUCIPS6Q4CBQilPkRNSn5Nln6x1T6xiHru5/tpRYMUBH4p8TkcVH9QlWC8gxznRVrWHWfR9v6JhK4y3QEEKdgar042CEx9MIH4fu/xnVdf3XEObHx6TAaBbe0FAlk4gOhY5EAexFgyv3Al4nok32TdGHWc55OHWQWmqnKOooknsJ6M/ZDfH9UhfKAAPuyHz5gmAD8AUHUQAFAIOvONCeZnSSmlLFlmV2F6Eu1+xhlnFPvuu2+ZHsYLCdwo/B2SFAOE6aTGBNUriaxs8oOYTAap4wWB2kVh+FjUYO7n2jacp59+eplmauuttqo8ZrqDQJpG+1111VV9fV9Ay5lnnlmOsy222Hxc9xCUO0MsWI2myY1pWss4BYFYkViUjOvn/tyLwKu3v/3tYyo8BIsSAQab5JxkrUpTehDr1CDGyWSDQG5VsWiDfhPL33rrrR3nsDanx2QQ2NZeIJACaLHwk+2nPzz/a17zmnIe2Cqa1/iVx8nDEWlNzqcCTJq/k/Sq/dxFx34I/QoCscgF1s8FgD7VQERMigxmKjjmmGNKU5mGygAwy5widlYWuCuvvLIMDvE+KPEEGEgTI2VMMAlYeLwbIY1MeMH7WWyng7rfFAT2w2KxBMTSbyRq7MvE/PGMCqf+yQKBaZ7AiYDAtH5rnBesiV522WWzvivdzEQSwb7+9a/ruBe5GJuWLRT5npYwS0Fg2h9MV/P1YSqzrliwCV+/wKhr+ziHoFQwISK/l3q+FEg0rcnaSycbBB59dGdyb88tJVXTa3iH01RNVaAlg8C2ppVGqkBgCqqbgrXRd3A0Wtu6EqpNcbGL5Wc/a1Ybm1pvUt/YCVgcOj+w67Aj98JBnAYgEweTl0XQbs2AwQR6AUwCJm95mrIZOMucJJz5LeDSjJjAQxb3XXbZpSNCmJ9snEswTGaDWHSmUldoPU+a2PSyyy5t/H0Jn2Ox0DStjOK4Rx55pOP7zB/pcSnoqGI5xqNpxZCJgEA7/ljuvfeext+10KZRgtJxjfe5zNepNKmpSjfffPNZAC1ICgLT+sL8IZuapbSv/otFEt7w/zQiuJ80TGl+wbvuumsg42QiIND8kfqLmjd6tXk/DA8AnJoLj29tYtPjUhD4qtNPbzQ2UxDIItLre/BDKoMGgZ47lqYg0LljqQKBzL+xCAppusEHgH+eVELafffdZ7VL/KzYvab9jIBISbcJJJXv/IC5V+SjUlmSQUsBgzIV0aJupmhgRapN+MAgp2c733vuuafUqgzvgxQ5o5gc7Ows0hhIneInlM3cYaCi0Qed5DHL3CXG0i233FJOdCaZUDmEfyAgGKJ7+QxiyDmsx5PZIBadqdSVWjvU9P298sorGn/f7jR20Mc6NZmIqZQ5qVRN/qpRxFJXMaRfHSQI3D+pAqBNm44HgC+txdukXm6dcuFJ69U2zTuYgnpyY5LAe43WepFWetm19W40Ob/FNo0onzFjxqz/c4qPpZ/6qGnlDRGUgxgnd931jY7z9gMCWQxSgKYCTXyMOSVNNv7RinyZdZqW2sMWbVoxfkSgxnJuA7ePqiCJkDWhm5o3U4Evqo4VcJeOiT322L3nNYyNWLw3TTI2pGXjvKvLLLNMxzFAW9qmTUv5wU7p+7z11luX/xNnEbtbYH37KSeaWhyu7WMsJtr5AX+UbbfdtqQsUfNu2ATNJCwimCnMQONDw3eH6ULEmVQEmMCJmIR1Pt8PYPKJJ54ofTuuvfba8kXj9GtSUptY5+p0dnY+SxYL94UlYL5Dv/KtuOCCC0rHWkAVYNTg6PiUsRx0frMsUyP6zaTaK3JqvGKiRP2feOKJ5YIVfACZh43DwATaOFn4J7JYTwfFZKYmhn4SFWMKUvOhd7bJd73LsdjJB7NJrOacWMZTUaFKU7Op+We8INB9p2b1k1pjqMl3U9bBojuRDQXG4O7EV1NS714VayxQVRWfbIrSY1PGLmUL65R1KZWwQNK05F0/JQzN+bGo/jOIcZKm3PngBz/Q+LsAebrJ2neffcYcl/pZmud8t9f5jVdrcSzW4wUqfApToNkEBFbVPubP2et7VSCwjt1bddVnlmAolr333qvnNWCCWIAtrGqv76kyk0rKZHtX0jVG9Y4mfS6hfCzmhXheS5nw3Vs4pul44rMeixKd4xzXnS++DhOerEAxs4HFja2ZHyDneLU35WtiDuO4LLrFSy9VAIBlkPQDqiw62D1UKEdyL7ogFBQ4M5trWpywLO4lBK34TNBKeDk44gOvWJrw0/f9BAaZaDgfu1cvCjrc7lAnuHfsISYxm7Snh2AXjCdjyUQmQkskorxp+k+/6T9MkCo1/uaPFE8gxlTYmKRsRbhGlfiOseA6xoydoMU0gAKgz6QTL87YwLgKCNNVlckgNhlPN/VMaaqNfv1fbrjhho7vM21aPLp9B/uRBiDYCFaBsDR60nvcr+N8laYmXLnVxuvT6b7Tcmrus5dPGxAdB0OQQfg8CjJJxeLU7TusPFVSxahdeOGFHcdY6DaemVy9Tr1Pt97aWX5Pm8dMSHrf5gB+VL2e13h6PDHBndnaZEy0HY2HlOS4+eZPNf6+9SgVvvXpcXtV1Ke2Geu1KRGwmb6/dZGsqW9ik8CZKiYTDuj1vU022XjM89gAVB1rfkyBMmtkr2ukZl0inqHX9w495JAx35MFJT5Gu5sHY2FlTBnDqnGYmt2VOIyPYdGMxZrTJMUSnBZvNPU7S8w4x/boALeImVCZugBBVCbFCKJvRZqZPAA/4MrAkeATbQ9cWTifSgqCV4ldtslOjiffda53vvOdpbkZvaxxd5x4UeQx6pzoX6BQFCKGR2SzUj3yW1n8f/3rX5cd7N4A2nRHn2XwwpyvvY0lkZXGGYZZniSTzLnnnluOjVjTz8Lfxx9/fLlQEQyyxdgmIyRhDQDPT9GsVaDfLtl4UCPWJMr/1e5NpZwwlvwd13A0qdl8hL/rQOB0VmbvVLA8/ZxDCp2UTfR+VbERQS+PAiGCsDZUHet9jQXzOIi8dDfddFPHeT3DRJJ5c5hP5b3vfW9tfjFjxUKfysENfK56aVUpO8yGvqo6/rmbblq7GfZ+psfLnZn6ut1zz90d70uq+jf1fUujqC9LTP/Ehj3O0Vml/NPTvpTkfaLtWBXYYd5q+p4jNFJhsUqPY3GQ1iV9BiRI3bmB418k7k820PomPbaKkWxi1k7Ztrr7TzU1uZLTTjut8lg+kimQjV0E6vSQCjB35JG9Wco0KwBh8UyPYwlNx+tHWxveujyogGNaw5mkoD9NDk7MRd3qA8NoaXnB3/zm113ftx7aOfigZ2gc+EP1apCjjjqqBIb8LCQlFAiCBZQ6A3iTS+qkk04qd+/YGJMdIGXXYHKwmzVZy7lmEmeyxfQxqzHdOp/BOlWLputQjclZlwnCIPKMBrWdGACAlWRW8DtgACBm6V+0nUWFKcXgZeaxswLYjBuThH7QH1TfeInGMx58z0KLUeB4y1fPOUWxA4TGKpOi8YfSt8u0aLgvL61JXpSrcW/ysUnBTMf3EtK/xDvzMKbC33UAYrc+6P7J1jLxdWtjtNZaa5aLiHGeCn8yARoWDhtDk3Qwi9e9W19IctORW1vnXnfddTuOtahafNLJVYBImNC0sfvkW7jl85/fAvBj63gGn00LvWs0BW/60XeY8ave7Ve2xmc4LxbHeOpnHKYpcyxun2qN+7QCCIZF4uN08QMwurV1P5rWkyXmZnOvvreYeQdZebpZQ7DnFkTpkqwTYcxbB1KxHoi+jN8LbOgF558/BoQwe6ftkgLzIEgETGXKrLp/VoF0E1Jlwm6qntG88NYWQE1Zm9CnNq0sBtaONHjF+y4615xXVfqOBcq66j3Q9qGtzE/peGDlEDiTAgRpR6y7qThvOEY6KqTHIYccXLnZeLT1znmP3ENcYcW7pK1ZAKv6AzNq8w3Ux35y5lybZ9gBQZTKt775zXIusdYe1To/gLzVVlsWH2y9B6nADYceekhxbGsOj9vX5sYacvDBB5UWoVT4zFnXjznm6I5319xiPUA+BcIgFmuEe9dewc/b+4zFS8WcmUbb861WRS3tP9aOeG6yTtWVQ0RCmHflX43PbR78TGs8p1JViq4PHenocEycHeLFF19cgiA+PVA7poVZGEPjJxbQIFMM2QC2WHpwk4GHtZB6QBnQ7d40loHiRXJuzIkHTB9yWGqyDQl8NTRqHTgBADxfYD1N7NjBEH2WOl1nKWYBf8AK2MO8elmrdqVTrSZ1/QzwY7iZcQFRAMekAOzYCLlf4AA7bvzH/n6+n5p1mYZj8zAAWbVLtCgAKsNmCT138HOxsHdjvOP/h5qs3RyYtVnKPBHnMBeowuIcVVYD1/LuhXNZYLxjgGJduTD/AyrCpGvR6OVgDeS7H99pet77WpuYfnbbNpdV7er9+FrrHrWDBacqwbHrbttnFZpu6r6Byipxj8z2TX1rQ1/QM2f6IVmQMe5Vz8F3iRnffFBVH1X7xlHBQYHIbmJziUnRjhb81B+VGGPrrbfuuNpsnnlGyqjifsT6F74P1Pbjr6wdAgtlfkhNkEFEmwJLrgWYVK1B1uAAks1DKbPYTaxxgbEGbptKXI1GtPFkSPA3BcqqWLQ6+cAH3j/r3tJSiN2EC0Lw/eZjWFUXHOMqWNU4DIRXKv/beg9Sc63+SQNtYvGe6WubGDhL+1bNJzYA/WxQK3RkVqMKtrAwQslAn4fC9kHrIpQMOg2ItrcwerGxehCzQek7/EPcsJ2PYwFG/lqOA/yoh58doicBVLsuO3X3DCgAyBhMjKY2wRTmwJL2ZM8PhzM5Bpk5TIohEyFQPaiyTYNW/WuXbDdtTAr4CDWx7YyZC/R/vMsFAqvGb/yZTUMVENEOzjfsknG3VOwm+5FNN+0eBHPYoYeOYfiaCFY2Bshf+cqXe38pEdfdqIdP2ic+8Ym+z0uq0tZ0U77U/baD409vkLKjX+Xr1E+ReiAvTZSbCtY2jGVzY9Ui2UusHen74D3hIxhLGszQS4CjCSTQLQMCqjYz3QSACt9Po0qbiA1z+D5CohcQrhLtFvsnY/b6EX0YTO6PJmmbekkATGnk6qCEG5nzr7DC8n0BbGBuwdZ8vFBrTa9KtNxNYuuNalH9vs/APcY9XQP1b8wWwhH9jjdMctzX49TRl86CjQ62+2bSxfoBfhY0OzX+WX73QExqGoSZAcPH1GbQA5CAH6BoIWWOs1vkzzCeQugW0l4+IFOtcifqQKwpACyZJId4wJApZU5PTeP5KMYFEDZx2bUaDxi2QdYOHZYyO2AuMX5Vm5b0b5NfHHFp7NexUU0clidbRd2PVyyuscmoTgHqphM11xGWh3Si/EIfu/0gwEtqek41DTBpIibsJjnLYvU8M2acVFnqqUosBCe25uDJ6vcNWkCwynSYij5mykujsVP5yU9+3OHnuOMOO5SlQ5uIxdQ4rArs0W4xU2yTySRfZZKrEmBhAo7ysxTD04+84x3vmPVd610Vy9utPTD08fWtM2mQUTfBAKagAAvcT8CjrAhhDr/jji/2/sJMAT6DZa/K5DwIAS6d3+Y9zSvaTWQJMU5tMJuOIeI9iDeUxqV1rmmsABN+3YbO+hKDwEcffaRkG5tmWLnn7ruLdQfg6zoSfrHYYfzYwKVrwOQx73pJ+f8BevwB7dT5PnDap0AQ05fjmdPCMVhBDJDFMfhnpSYwA4aDPSZG4AkQyQRrAbWDA0j5lGCW+KGEcnV2nHbk/FJClCamRqNanKaKZXT/ggGwmwAhsyKK2u6Nj5GJiCnEQtjPZDAdxSJm4GP6pOUA+viKGC/aAOs32e3NVIutdk0vCzDFV0XuOBsWLgeq2BiPGGkTEXOG/2O0meeMSWOFWtCNJb8Hc66X3ASI7QvF6/VzL1M2v7EYBNpIWbSqFjfjfdjm4DVb9xBSgFh8jE8mI/1qA+c9xuQzh2GPgsnJTy4iTZndTTbeuHQBqQNBzifqW99UndP7Lb0TQPDIww+X7xf3DC4lElmbn0LOULtiC5H/9Wpf4+De1nvqvIIdvvSlO0vfrYsvvqic31yDKwvfnODTakM8XgaXj/UXvnB7rfuI9jF+ezGsg1AbnKuuekul2cpY4LsbElRzi9BG5rSrr35HadFh2cGsaLcqJ3pzsNQpdRsAIN35rDfd+okJL4j+BRa9i+7ph61+SdtSGwoyO7u1LvWK3GyqK6+0UvHG1nrGJxARAqTpI8SEOYjFw1pnnkF2pBtg49r7ZH087thjix1ac451C0DkE2f+EnwGPCJMqt4Bzy2gADioY6EAb+epMwtya9Jv3jXXOu20U8t11ppqfTV/MmUCnHGaHvfJ1Qsjb/xjtmUN8T2bhEsvvaQct74bb5CAV5ZERAE/TSmS9Lf2YknTHtwDmDilgqPIFFjjxJnHuoZj+WR+dWYAalxqEzbgVmKjaDzDKM5PjRHtzt3i0633OM7h6t03z7ln41nb+o5rWsNtfG677dZyA2Bdr+oT65C26jav3X7757vWrLa23N0CckEQSeH9RKQhWtIMFlhagBbZNkCyZbTTNKrJysRqItXpBgwka6DrBKyPAc/nj2O9AQSwmUAtDjpQFK4F0cBLL6hBTewWVYMJgND4Ohuo8LvrBsd8i7TF3IBjmrM4UaCQM6kX0+++7wX1YnIQ1vgWcr5cnilO8TFZ6uXBlGoL5iY7Dk7MBovf+UhWTbzTUYKflJ0Kdf/YEy+XtmYan8y2DAEewBU1xmw6bAyMRRsN46RJNHo34ZNhQWIetcs0GRhnXkILjvcCwLVBMfG7JxOj/8XjKfUJ9F6kIDD4EdoYrVJREm2q1fvhHrVvtzQu/GW9r8yJTUuOpSqlgQn14tZCBVxadDCFrt3rvQS8llxyiZ7Htf16m/vstc+7ZMPzLj6QMe15zWWeXzsAnMaK9pnq/jcODzzggNY9vLk1Z11bWnhe2JpvYwbbPVcBC23Sy+/S5ioEXl133btmLfAW0CZg2hpySWuu5wcWAxMKPK6xxuoleWD+5z/JQlMXfT0nqDYHHLliAUY2Kthz5speeR+zDl69GwD90SUYvrR8ny9tvc/e76apwIxZeOF9733vmDlAfzuP4D1j3Jq78uRYRdu/MHkBTIAVpscCK2+fqBOoGdrHEGJagBovM4AI9ED1zMJ2AlUJGp2bWkige+DRQA67KJOD86BZgUvnBaJEXbkX9yDZJ/87ADDcE99DuwyAFQA1sXo5AEjMDyAIiGIbTTwW9LBYi4hrknNqPKozmb9N7pgL9DpWENMiwgoDk+YDm04CANqlYT/sHo0DOzbtbYAD7koIDrLNwhihNgKuIR2R3bU+dT+YGQwEvwk/J1OAS8ySnaJnBnwFTgW3BlFnqUk0BoGOq5uYmTJCCbqsWbNmzZp1iNpegC1o6GE+XpgQkWSoStF8mD9gRiZzQAzAwtIBhRbqQN/a5QaKEqWJZQAKmW6ZTDF/FtUQLepcfgf+UNkBdKJjXQ+oc3wAoUw9KFKMpEUa9U9RyYApkIDFdCzGyLmwR67NR8huUuALcIZhZOu3y8WCuO9BpWMIaqdtlxbAoOexe/vTn/5Umtg8T4h8nE6C+eOszXcInQ6U24n0U9KmiWpzwAkrhm3TJ8aDsaTfOfBqo7qkzlMhzIHGF5MjUwHTjIARmxljOzBjNhTB189zYT/STYaNiA0JtiLUj8yaNWvWrFmHqO1f2MyBuVALGNB6eKYPDru7qCfsHBs/mzRmzucAo2AAJlfnAf6wHPy3nA+w813ALgSVYHYAP2wjYCT1CnMcBopvQ/A/AwAApLSMTJVwqKaAA58W/hOYLEAm+IxhlQBRwBUwxVzyw8DsMIV7jh3LvGmDreqA+XE9gBWg4gcSql1oX8CW31FdqoqpkHDt0G7YSuBbgFC/zvDdNORcM960OROh/uF/gRHWHtpiPFFxkyHGlHdCSiB+GMyCgKpxbGMRQKDNRJzgnOk0zXQfxpWfs0N0fNasWbNmneO1/QtWg2MloEaZYTGBWBB+bVg2PzEj/Nr8j1mXA7EFDcsmMARrKHiDrx7AKEAC4MPQcRRl/mVeY95j7uVcHCKXJtNfDrgBMPm2ATdAp+tjDTE4WBqmY2yov7E4WJtB+loAgkznfCy1CX8g5tYAuIcZPBLaHsAHvplcjQf3OZGgjxChx5/BGAm5Jm0gsGvAHtN4nGYnLfk0bMHcGvc2NRyTAXmMLlAYwJxxwj+J03F4dv0atwUmdQJZ3bNmzZo1a9ZBa/sXQRkAECYmsEEAIB9AvlGYIp/76X/Cs5m8OEMyD/PNs0iKyPE3BtC5MCjMexZOwIuZDwOGaeo379OgxHUBWuH0oXwYQIuV0g5AKn9CzCD/QkxhiGLDcI43wMT3sGCAsnbQRphL7cT5mel1WMmnQ+1kCV+BZP3GpA4EYk+bpAQJyh8OWPKsQBKwZKxggEPEqc0BsAf8zg71mgWQcGHgOuGd0F+CVYx54M5zSqEU2D+MeFq03iajKilu1qxZs2bNOiRtO7TzXQN+LFzAX2CogBRsjQWbWRYrIsrV/5mHhTVb2PmQCR4AZLCGQBWzMjMwsMM3j1nN8QIl+MQFEySfL0AAAAHQmIAtuvwSQ+oH1/VTyhUmSj6A2EWLsXvxGTDl3piXQ9g5sArsYbg8A3UdzBOTs+sBt8yR7s15LO6AD+d//nyYQYBGwEdIQcOk1yREOzBFjmcuZDYHFIAHoEjks/YRdAEcaUMAdar94PgBhkAQfajvpTlxn8Bw0yAaIJnJVyAFv9HgUyiy2PNhhzGy0kdUVRiYrmKMcH0AboFAY1z/YUmDryQ3Ayy434FAx8SRlcZASF6bzcFZs2bNmnUaaHvBsnAz1Qr+YKoDwpgFgZJYgDGgRRSvRdyxssoDhBgki77gEt/HDgosARJDgAeQBgRKrMwUjAnCDDIvCzRxPT59ocYwJgqLBHyNN3CDyVpkMF9FJl4R0BZrbBcTNZAI/MhTJNKYvx5zNR9CYEbyTQu8gABMjoWf+VhwQForsk6DH5jn8dP5qDZnIvb8QAUTqTbRRlMpQCezrP4EmJn2sbpAIAAo7xawk4LB+PmxZNpGO3uGkP4Cw6h9feY5mVa5G8xOYjNhfBoLGFKbHgy35w3pLjyrtCehPUSyx3mtjBcpHabBS581a9asWbPStpmyzOHVAkBy1vAPYyIFkoCDtL4dRg6jY0HHvnHoBx6AtpAPDwOI/WMaZh7EJlr8nR+4xDQBYH6GesSiLyVulO8PcMPGTXYDAGcAD1Of52eyttgDge5NShcMofYRyAC08W0LZdFEHsvdBFymhb2pyFfPIuUJplUaHkEFAKb24ScITADKrgNQTzVDBsBjWD03AOh3QBioAeqBuZCUWyQ1/z7Pzr9NniTpeSRn1n+eC1Om3zG/2DBt6BoArjHAFGx89TIDCxDSHsaOxOVAaTe1OQE0MY1NqxY0Fe+A8S2gBTNqs4TR9byhKDgWWaqk0PeOC2WUqICgNN9Z1qxZs2bNOkRtMziAGp9AJtjgH1aXugS7B8gxu2L3sHbMyBZ+rJrFkG8dYMdsy9QJVFg4LZIWdos60OU72BGgwn1glnolEp2sUnKhVjCTHaaT3yLg4l4BJEAGC2ThxwoCQBhBQTUUwAtVJgAmP50P+wdsYsgCEBQc4tkBYCDa+TGowBQQNtl58GJh6gTcmcplUddPoqYFCGEC3TOgF54RAMYcM5MD7QCyNpPmR7CN7zvGeYFbQRRMwUBacB2wwSB8II0lZnnHMLmHih4AFNCpX0I5ol79h7EETqk253+p/zDMNiCuM16/SyBdG4hqt/nh42ejgGV2fcwfoBfux3iO7xtLaLMxDV76rFmzZs2albYXK4t6MHMBI3zm6kCgxR1g4Efmd+Za4AEbaCHHykjNYtHFejEzMr+effbZJUMI/GHBsEu9yvtgKX2XPxYGCrMmy/YgMvj3UrnctAUm6oorrihL5ngmEa8AMyAH7AoIAJYwZ8A0k6GAEgARkAEcfCZZtvQiAJVzYBC1HcaIT2YImnA9vpjA+FSJ58TQAfgCOQB7z8ocjgkEVoE7AB7DB9jbBBgHwJ3P9DUgaBPAH9RzGk/Ak/GA+fNsIo9DMA4wPd4s/1g16Wtok2AdoNyYA3CBbu3NJaGpuG/ML19RmyX97Z0JJnGbHgCx7vrYYu0zDV76rFmzZs2albZ/wVAwb1moLewW+G7CRwqocyzgYFG3qDITY36YejF8FlyAwIKJlcGUAAXyqHUDcpgk7A1WLOQXHIYzveTSwApGkM8gwBPqRPLhAwgknWbWBQwBP+yY/HGCQAJIEVjCF1F7ABJAIIDlb8AAOAa8ACigizk6BLJMtgDyfPYE0mB2ATXP6T6YdrFdgnD4ePofoOpe1aEE+IHVkEjccfpNexkLGD9MnPGBbfSZtmMeH2+fhKovorYlmAbotBs3BvcKfOoz/VF3DkyjzYRjmKwFKQGEAdjWSfAP1Q4ALBY0VP/wrDEIZCaO/Vi5E+jzafDSZ82aNWvWrLT9CzBi4ecDxhSpUHGVCAyxAFroJT8WnWvBBwRFujKjAgQSADMNqtoB5PC7A+SwTEx8aeFwfwNLwKPkyUyxwKJoU4tp8LsajwKgmK40CbR7ZdbD8HU7v3sARDn2YzGZtD2f58L8MZcCE3z7gEAsIJAnzQyQyBwMmAAsQKVAEDn4RN86LzbJOYAZbReqswBlTJcYusmSkA5IdLQ2B7r5dbpf7cPMD8QxWfsdSMTu8Z3U7+Fz9w8U8/8T0Y25dYxz+L4xI0oY+6nqxiAGL2aP6wDTryhcpQiBQGOUX6UoawCViR2LXBXN7RzYWqZdQB7DCQRW+Sv6TC5Amxxt5BmNAePDuYBAPqPh3FjrGIga444ddDLyrFmzZs2adZza/oWvF5+mXkEJTMTUQimKl88fEAC4YMiC7xXWCADEFmK+AB2RkinYsjD6HDDCOmGJsIBYnvEWq0+V6ZkZ06IcPvOsAg8IBglwYSqsOwe2Z6uttiqBGwAoSAB7ivULCaaBQGyPwBYLvcTBmCLsp88BQ6wh0y8TN1MyVolvIGAJEGoDgJVizgBiwRSTKYCglD3AptQt+lC/+SlyGzAM7J4+x1piATGj+tl9Az9MxpJvA4PaN2wK/A4A9wLyzMJAXWza9bfz2HBg3tIi27GGMnRYZowbUMZNwbNh+fSxVDXAotrHoYRb+L7vYvoAd0CPSZ7ZF6gUzQwk26gYo8AvcO+5w7hyPW0QzsfVIfUBDOmFcoqYrFmzZs06DbT9i4XPgtVLLKZMexZl7A52hL8ckACsYBOZCPm6MYeGmsRVwR7YG4sq8NRPMmIKIFrs4zxs/Sj/rVClQuQnsNAk3QvAKojFs2Et3TtQB7h6Tgs8hkighN+BQ9dSe1e0M0DMLAxIMFn6H5AkaADgwlphV5kl3Zf2FfE6FeJ6osH574VrA3oAv37Xxz5zn5hCeQCxfVgxAAtLCjwBwcAfVhBg5nPapE9EFwPrwFn4DICPBTvcb19rUy4JsRi7TO5cFmK/VCCT7yZWEPML5PH3xI7rB5sZpmfPx9fTOLeB8l3t4u9wLgEj/GTjewnHZhCYNWvWrFmngbajKi28ghYwOb2EmY1vF8UCAgjYLOZePlEWSYsoNo+5LTV/YdVCmboAnJrcrEUVmwaMMJNiaoCq8T481g0DqeRXSPjbRPl5YfIABMwghoo5EZADEvi7MRMzC2OJtAXmCTOonQBuQSUAoOcHngAVAAKTFKqqNEmjMmjR/5hBbQwYA4TSxmDEmIKxfO6PGZT/nz4XNc3Uy/yPGdYmgK1NRVXanCplInZt4FNKnfC5zUYQLHVcn7cfxfjZOACRUhuJSNa2EqDLyYiRFXEOENqw2BAAg/rIc/N3DSlgAH7Al/len3E3AOpCcEy4pufXjvF9YBq5Rtg49PsMD+w3Ujz12qxZs2bNmnXi+sezZ4JAKijEwtY0WtIiylzJlAogMJVhfYAZDJlACOa/4P9lEQaImFSBIAtoqCvbRC2yghFSYY4dBnrGbmH0+ABiirBGFni+ZxZ/TKCoX2wfP0CAEQAEjrBozMTAochifmhMlEywTJ986DCBQCAByoYhmFIpf0K5QCbRBx98cFawCNDD9A8s2gy4fyZuY4CfZa9UP3VAP/6bryFm1NhqwtSKcrcxYBruBuxtQPRN8AE0noFDANY4DWZi4J25m28hMAzoSg0EDOp/ycOxwcYnwOhvfo++a3MA1MYBUNhg78B4/AJ/cshI8Z/nZ82aNWvWrIPRWSAwlLTCQImW7CXMY5g4TAjQwgzMR0qACUAZFj7mU6ZTjJcFlZ8gFqRXihfm0/hvQAprkwoWarIBH0YToIs/A26BXKwVIAgIYAM9v+fEOvH/A+78lM4EOPQTUML+ARyYQ+ABy+T/fNaADmZWPnraeJgC5Iefxob7w1ZiPTF3/ECZ//kJGgfMwXHVDKpdMGQ2BpPdVyGg6S9/+Ut5f0z33Y7nTqC/gHPtbkMjUlq/AYreC2Cdy0MY494TGxmATz+HBNDaBzBmDve35wWk+UOG67lO1fie20HgH88dKX72qlH9/WuHf09Zs2bNOqfrLBDIv46JDxMYFv5eImBAuhAMCd8nUaMAAoYPy2LxxI5hTbAr2BLgKXX+D6okmWOwOXL0MTcGfzLHAxKpYFosyJMFKpgzPSNfOYt+/D/3BAAyD/of4AAQYP0AiHXXXbcECT7HcGHKmIm1NTDBp45vIPDHjA5MAbWYL2ZL7Uum2iQciwAQCZb9xP6JWOZfp2+wv/ra/7CbWEym0TjYAoMnsEL7TWbJNGMKuxrqUQcBCplfe31fxLq+Atiwj+6Vq4ANDL9E4N7zAfuCTjC+ooodG6KD/V+7AP3+ttGRJD34rWImjQ9BQs4bvje3g8CvHTdSHLxxa2M176iuu9xIccthI8Wfp8H9Zc2aNeucqrNAIOAlihX71BR0YOaYC/lMYYCwRIAk0MMkxsme6ctiWQX6MCV8sORsAyZCqhQ/3QvQJKWM4BHHiyQGsNJqGiJpmegGDSws4hi7+HmZdNPjsJT8/wAhIA/z5f61AcDHjw24YDL2GYARaiIDkEyEroMl0pZYtQAC+0lmPEgR6AH8MQX7XSCEIBHgVj8DfoA/9kykLCaTaTuwfcqrAUWijYP43mSBQDn/AK4qMaaBvKrvhRx/flKsoJ/6SV9j/wB0Y9qzAm/eFcc5BuDTvzYLACCfycAEUibmwP5RLDim1Hn6TZUzJ4LAGw4YKRaev/18T5unBZTnHX1eYPDCHUeKp84b/n1mzZo165yos0AggAXIAB51OQKrRI1W4IC/HuDiHIIeMGOCJwAcEZFMaAARdjCkgAH8gCN/S0zMDO0coeYwYIldtPg6JtwrkCh1ShBgBVgcNLBwT3//+987npeZMS4NRrFC/AJFtwIMcslh94BD942pxAB5Xr9jxwTh+B/Qx6QKGDBDhhq7wLWAhclOD1MngJM2Zo6WGJxpFdBjzmca5UsHILk/zCD2Mvi5CYDhF5hWnLG5wIJNBggEsKvkX//6Vwmw6yqKYJ/1k/EoQt2zAWg2J0y2gHoIetFfgF9I8cLFwfdEgPNBBIqN38AEUlHITPvhb2OHz6Jr9vuMcxoIvPekkWLJhdrPtstzRoo7jx4pfnDySPHxg0aKrVcdBYb/sffw7zVr1umknz50pPjIAZkpzzpxHYkXGSAN6yP6tx9RPi785GAv8TBGUBABgBAAW0gfAyBhR5iOAR4mRoEQIjCBCtGnfgeqBJAAmf6PjQEw3Ct/OgAqSMgjNwhAgaEBZOtqzAJIcdQrs57FncmQGRsgxPhgMkUKhwASQFAgC1AMYDCVM59i17SFXIvAlAAMJcqYW/0clgQWD8AHcELtXwqwM5NLEo4t1F6hPfRDnfiO5M6DBIBcBoy5VIBOJt2q78T3ANQx3TN3C2jRBxhdpl8+hcarwBCbAn2I7QQCMYbcHvShCPswbmMQCCwb4+Fv9+O8xsjcDgIP2Kj9XOsuP1L8LvEB/O05I8Uay7T/v+bTh3+vWbNOF/3GK1qb1yVb605LX7Nt9p/NOjHtAIGYDuwTNqNJqpg6wb5IHxMDGIs/X0PmMUma/R4YxzT6lV+XVCMAZVDgNFSDUE0D82LhleA5lPly3YmW5cIAWex7ifsJ3xH8gvW0wGP4+PkJ/gAMgUEmbqZSrCdTMYYTY+o6jmFC9H/nBLZE2gKA2iUktB6GuLZ7AEqBbPcJeDMNY0hD/+lrfVEu6C0w1Qu4YkIHCQDTsWozgsGsqkvtPrU/8MqkrR/C50zYgpoANCljPK+xhnnmV6jvMJlAIObcs4aSgHwSBYVgdeMNAtO+fIkxQMYccweYm0EgkLfKku3nesHqI8WfzmsHhPz4tJHi8de0j9lujfb/52npz18z/HvOmnU66MOvar8zKy/R1kM2ye9H1vFrBwi0eGHiAJBhiyoPhB9eYJ8kYWaSlJJEJKoFVcAFMx5/PMl8gUSACjDrd5FV5g34bCIAZzB/AhuAAhDA5Mt8yBwKMGADgUCgUHCMKGPmbiCAmRsIdO8hzyIg2atu81QLlo0vJkbMvQGFsWB1AwjEpPUSALJJsEYv5ecHkAoOikUfyvkXH8vvFONskxP7KYreNbaws0Cg/JVSJUlzpDoKVtzx/sbUYv2AP4wvFwSMId9HZmXRwczlwfTsp7YDJMNnvs+H0NjgKzu3gsBfnjlSLLto+7nme9pI8ZxlR4qF5hsp5m39vsRCI8X2zxr1D8wgMGvWTn34jJFij3VHgeAOz25toE4d/n1lnf20AwRiVSxYzLeBXZsugnXCnAF5gQ1kZmNuA7KACv6HghQwiUyYTMlNkkDz68J+PvXUU13vQYQrVsc1mHljgIE5AkgAAffFvOv6QBHfMUCBmTCUi3PPQB9fQEDCcczdfM+AcEzVsAULiNXj1wb8AUV85OJ7A5I8f2gLDC2QQ7VHnQD5XAbGCwCBNaA77jN5K103rhEsYIQpPvVPTEVSbBVEsLjyM2Ks69hwTKL+B+CZh5nJgUAg0T0Zh64tQIR/IZ/E+B3zHQFTko7PrSBQShjAr8lzL7lw9n3KmjVVbPoJzx8FgpusNFJ8/RXDv6+ss5d2gECsGqD1y1/+sk+4MPWiegSGBkjBtjClCtqwmIf7x9YBCZgroJGZD5vIjwuzJXUNwNXN5ArkAG58+DBFdQsVZghIYs5l+ma6BhalLcHyiShVlQUgkYoECMQKYp0ARs8gytnfAHjKbg1LtCXfOiBce9IgzK7M33VBFxhaAFv7palbCJ9L0c9M5v2U/8P0uqdwTrn9gL/4HAJFtGc/0dVAPpbSmIqfMxUmXmZf9yHoQ/JsJmEMcFwrmN8qQMi3NXxmU4I5BgTjVDpzGwikr3pBs+fec73h32vWrNNRuVG84cWtuXapNhBcq7Wx+vjBedOUtbl2gEDMBPYCC4Jtm12kaTQz9qkq4XQsn/nMZ0rQArTRqtQzzIFpyhElxrCEfB2Z1LFKADWGj+kX4GMKBHhESgOjUsVIK+J3PzFKIZgGoIxLpg1TAGXsmICYWICm0A5845jgUzNsUG3puTGumNI4Cbb+Y27VPoJlqr7L3M5Hj0lXNDjxE5sIXFNAHKvKFK8te7F/45VQIzioqG4bBEm/Afpw30rGAcGxa4LxZCxoi37rB89pIPCh00eKpy/S/ZmZhL9w1PDvNWvW6aoA33v3bQdSAYKrLz1SvPNlw7+vrLOHjqSTLr84vnWYtblRAEX55ropdvCHP/xhGSTBDC0oABjCihEAGqMHjPBh5DuGDaQBAPIL5BMoqpYfIJMrU6KoWwAJq+nnsCuGEGwqU2sKAjGsxgxm1e9AMLOxUnLM41hQPpGeWURs7AMnkpr/HEYtBuZV7Y+NjM2+2h9QZpbFrArYENE7VQKg63uAVv8BnPw9Rb5LEeT5lLizIcD4xtVxsMDSJHERmNtBIP3EwSPFogtUP688gZe8dPj3mDXr7KCfP3KkWG/5NhDccMXh30/W2UPHgEB+a1dffXVpnsT0ZKkX5lCAj7kPEwWMyJsIIIqYBYiAITkTmQqDf6BAECBQQIJoZtGyzMhM2QCGvHzTTQL7FotKMSKeAUR+gkzY8hsS5lrmWIEXxhIGD3CSB5ECf56dbxygzHzez71QScOdG4CeStE/ngFox04C8fwi/R1S0gB7gDywG4NAZmNsqXyD/QYvzYkgkKoYsts6I8Xyi7XzBq7SWsT2WX+kuOPobNbKmrUf/d6JI8WxW4wUX8zsedaGOgYEUilKSAaBvQXQw1SFqhIhshcwAQIwWUyGWD9AULAI8zCzs6AWOQSZfZkUBRD4Hfs3rEoh/QifTJG4AJ9niUVQCb860bgAojx73fzsZicBApm0mbH1n75UHQew5wLgHRIQAqQyB/NPDO+W9DAiqQWILLXUUtMaBAJgqnVMBIjxWRIE0uTYX5/dTn+R5gzs657Pm9oKI57tTw2fbxg6qw8btInn0PYTeZ5wvYl8/0999KH2b3psP2NxkO0vj9/vzmlfv0kf9HOPnv13fZy/H/3Due17bzJ2HOsextv3rtFPO2UdnFaCQFGPAAwgMjv5Bg5bMGEh56HgAmwXpoq/H19LrJBcjCExtNQqctUxJwKSWEAVUuRFnN1FGh/mY8wgkyimM05C3rQ+9XQUz8FsDwRiMSX75k/LJxC76x2ScgZTLJG4COUQPBOAn59TnSKGD97HDhop3rNP22eIA/lvzu48xgLkc2zCVquNFJuuMlJss/pIcdoLRopvHt9wQj+/bZo6dNORYuOVR4p1Vxgpdlyz7cD+o1Pqv3PaNiPFhiu1r/3h/dugsMn13PNHD2hdb5N2hOT6revtvNZIcdFLRoqfnt77+6Isr95jpPhBcm8fPXCkuHKX6vQ0T7bu7dXbjhSbP6PdTsrb1SXt9WzX7tl+vj9EC7zqKIJjvtWwXfvRe04aKV6zXTvVjj50jyJJv3zM2GO/1Prs6M3bbS/AwM/DnztS3FlxbN3z8ds8/nkjxfOf2TZFqgBzyc4jxWOvbn6/572onepkk9aY2azVrgdv0h6LVcACWDhqs5FineVb11x1Zju+svrcgNWbWmNhy1Xb59VvdX3l87e3xsL79u38/Dutc5/7orFpWDz3Ma3xeu1eY8fU23cfKV669kix1nJtfz1j5dRt2v0+5h7Pa7s+aD/HGSuesa69Hn91+3601QqLt1l0puAZW7XZwPGOG32pGsl+G7aTuK+5bLtPrtptpPhF8h5o188dPlIctHG7H1ZdeqTYonXv52zf7L0r36PWM17Weu6tVm2bsVeY+RyvfF57TAz6vcg6VitBoMAIZs1QO7afMnITFdfi0J+Wa5sdRFuFusvhOaSqYS4V9MB/TFoYvoLyHIoeZlLFpgHc2DSgmz9mXBZvdhaBLqKARdDyNdVGop+nelwNUrwX+ggbCLQD8Uy7Uv+E6GA+gqKXRQHzieS7ODIzqIhJWFWaqfIJtIDJKSb/3kLzd+ozlmovine9og0GTPgLzz/2OLrYgq0FrwUWnjiz+6R+3Bbt4xeYb6wu3rqHk1sL1RNndX7PArPogp3HSiZtQe7GDHz3hNbCvko7l2BVmzEvX7FrPZvxwKlt4OhYgCkcp6bxPPO0P1+t1UbfOaHze69/cXvhjdVCmZ4fqACG3Z/zfSNK4RFK48mX+O0aANOvAg6v3q6dVqeqDxdZYKTYtgXqL9ix/QwvWavtk1l3rHvvlqNRgu+dn9Mu71fV/p7t3V3K/tmEAC5VY5MuvEAbSD2e3MMth4091tgCnp5MwNO79mrfR6wAanovnnPLmX3yzKVGP7fJWG5mTksg+aGZAAdgkrTZtQGxsKHSl8akZ6rSFVvHvnX3TnBrY5be4/k7VLfZbUe0AVPdPLFg6925YIf+GbVfndUG3t5zfZ/q0xdtvyPAt4h9AHHRmmNXat3fB17e3YqgnQDNuudYpNWuF78kM4OTrZUgEHvBp42TPjDWK6J2kOJafONCtYoAqjCT/MtmF8Hw8Q1kFhYlCuBhBDFiodQa828os6edPfN0CAQZr0jV4rn8rPqfKOMAAIFebBoRTT079S3QLppZKiABMQJEmIMxgaEcnHrChFmYhqhnaZj4hvYD/iYCAkUNWsDCQrn0wu0FSiqJePEPk3e8+K62dJtpsGjFi+0L1hi7KFOT9cEbj4K4BedvswOYDaAkBngWz8cjlshCe+KWI8Xqy3QCSOewsFctJt8/sQ2+QvuIJJZ70D0DsuFz4OtNO439PrCgLWb5Q6/UXpjp1qt1tr3FH+AJ3912jbEg8GXrjr0GgD1PdI643U7devT8GJSJmMHL9j+3zcrEfaXd11uhHTFqwa4CWnF/b716ewGP/4edeuSMsddjuo8XcYm+yzGzUmewjwCfKiAINO26due1gJ/nta639nKd4/GFz+oEd3ef1PYj1Q8rJONz3w06mb79NxoLsIC92Oyq7QCbcM+brjz6PxuDlz5n9H/u+U8z3SS0TQCB2L97Z7THYAB83jMVPQ6cyZYtOfPzpRbuDHo6YOOx94i9TU3z2NklFuxs88Cg+T0es+e8sLkrh+TtNgRhHjBWnrVMu51sxhatAHpBgW9Mpz7zXOFzz/mOPaqvhw195pKj9+r83jkWA/NN+NzmAuM5bKA0J2slCJRsV/RlWPD4QE1Wuo06ARRiUzRwWFfLdzoJUyGgAwQCriFSWIoV/mJYozvuuKP0FRQoAfQBSMBuALzh5+wiwC4QZ8x4fuwf8ItNFhCiL5mF5XYMDCdTMTaNz6Bce7OTAPHuWb/xAQX+RAOLdsb8BRDIvL/DDjuU/qChugyzsKAQTKCI8n78AvsFgUw1Sy08CvKOe17rHKeNLnqfOaw9caeAYIMVR4qbDhpdSH991khxzZ5tdiReaGMmw+9nbNtmIYC35RZrA9Bwjp+2AMPZ27cXjADwjnju2Hu2MN96RJuRjEEjE1V8HLNqDNR2X6eTrcPWvPL5owsjViE1k1mEw/ctpMHcjR2c72lj2/8VW4x+97mrjAWBO63VuegyTwYwukyrH756bOf1sXZ7rT96/okudtiluB/1dzC/h3Zlnk/72wL+wf2i/m6Bs3e8rBMM7rJ2JyDR33tFoAmY5gIQxgRz4JGbjTKENh8/Pq3zfplGw/mBqMt2GTUfA1k3HtgJ8C6uYO8ocG4DEUCjNucKEP5vrKYAyxiPQbdrBeZ33dY7cf+Mzmu4L24R4XmDuRjAc03t6tkBxAAAD9u0Da7COYBYbLFn8n9jJjDAe1fcI9N17D7gPfS+hnsA0m45bNTXEZP/4jU7wfeXj61us1h9/2XrjYI3tbq5V/xhZvsA69e3nvdZTx8LAAHHrx7Xvr6xDwQftfkoQygF1Jcq3ApiUA34PXBq53Oeud3o2PEu5jRRk6eVIJDjuihHYvGeapYmlPXiJxf8yAIwAii6+czFJcGGJcyFfOKwXcCOQBs+gAAgnzHpTFTTED0LKAHZTKOOnx2DcQR9ALbMvdhjJlLsJnOpTUSowIFdBgJjwKuP77vvviE/QX8C5GJ0BfN4DoE/wJx0OOuvv36bVdpoo3LjJCjEsXId+pwJ2P9stCjwOBkg0MRuoQsLqMWnihUAlrA54TgL0wM15afuPakNGBxn5x5PzABWAGwrLtFeGKrOAZgGVtA56q5lQeVbFFhBZqgYdN586Gi7HLBRvcnoLbu1FxMg8LYjRz+3uAYWy/++Ft3vh/brXGhXmMk2LrXQKJPHvy4FgRck5jtms7CIfaqm77BHG6wwc/M9/yhI71ct1M9++iir94YK5pMCM5tEQFBffPeE6mN/eErbvzIcK51P+J/2CkAZAPz1WWO/b7zx8wPEtfFXIkByXwssLL1I+7zYw7tr/NiAswDunrNcvZ+ca139slFXBv0R3BbevPNYgHXSlp3ffdGz2s+CqavzqcOGBpZqjaXbbX76TCC7w5rtah2B6XvRszsBXKyfPqx9D44DmHyGqU7v0SYm/t7bdo+Y6SWr/Wu9BzZX4bj9Nug9dvi3Pmcm84q5v7fGF+/B09qscgCAfD9/W9Ef2vOKXTqBYvx/fqkB4GFcq85B+dkGYL7js5sFqGTtXytBoEoGFq8Q4Ql0TSU7FeoGA59MhUSgBQ3CfApA+UwUJmFO9V2+WHGalRCsMdUSTKBAAjDNDxAIxIABRpgxjBmTYty+sxsTqM0lx+b7COwBt9ivW2+9tYyalgJHBC2zqed1TACDcZ/OLgLcYnKlifE8M2bMKMGcqO8AAlWYAeglh9YOITAECJTQ2vGBNZwMEHjX8W0wYIHCNnUzC1ncw+Jph97tvBiQAAqYOsPnJnLmNIsJxqnbOXwvAMYP7Fd/HOZp+5mMID+l2BxrgQzt8v0ujvCAo/tJjwFCAog5ZOPO/10aMYRMavzHwt8fmwmEAAJpbDCIz2gtyAdt0sn6aO8AGPaoMBPH+pEDRk3Gl44zL+LnjhjtF0Ex3fyoPnv4KLDa4pndIzo/dejoeY+NmFCsZWiTGBxWtT9wdF/CrF2+y+h5r9ur/vuegyk4gNsYrKeqzZnkw3k/tH/7c75uL9+g3Vf6BPP002gsMWsvPtPEyvWgWzvP2HL0uW2C+DMGczUmFbv5kue0GbFu5+FrCQQC7sY5H1nBGNhXTOF2a7RBV/wdwDJc++jN2iCwChjxrw1jb8XF60FWrOYLfZr6vqYqYCuAu+O2qD9OvzFnO4414uGoveNKQR/ev/4c2jNs1Bact10veTzvRtbuWgkCqQL3AEzwyxPpOAxxXfdg0QX2MEtAKdYJyGKClKTYvWINARG/u2c/SWzKdr4APoCX8Fx+xjpecQ/AK5MhUOonsOc+P/ShD5VACCMm+TEQ4ZkoP8ggwwKtExF1dqnnUP8Y4JU8W0JnEdFYMuAJ4AXsAUXsYajiMh0Y3KaC5fWMnhXYlQwcew4EhprSL3jBC0qGVP5IeTfXXnvt8nOMoOOllvG/yQKBooDDYghkdDuW+e8ZM029FppuxwI64bwHbtT5PwtSHfsR6+1HjoLAt9f4DAV980tHj43NSkyvgbmJF7mQouTJHukqMJKhXVO/pRgEAkzY0vA3M1U4zvlFMP6wYjF+9NWjLEadg39Q7BxA4NjDNx3fRI7xDP3SLRCD6qOnz2ThmLW7tZNgiWUXax+76zqjn+8dmYLjwJHQ/r3SvBy7xej9xoCsSi+LAGOvShjX7zN6bNpXInvvP3lsCpbbjxp9lg922ZTQ/9h79Fj3EoPAfvrrXXuOmo1/ceboPRpLAHPVexT7v5bAaL6224SxnI4/vrmBXU7B5ERUX3vngLujN+9+LEAcAOOdR49+vvNMU/BC840G2dSpDWN43s8fOfH7zzpWa0GgCMbApln0+LlNZYBIkOAXCFypyMCHDrgDrkSc8rOjABbfuyuuuKK8V75agjGAL+ZGPnpASuxn6HeMlP/JzwesMeVONC0OX8AggACQJ4hAiTOmQYAHWA3X4esYKrTMjgAwiLbkB3fdddeVfoL6CzASLIENVV1F2hw+dGo3M48zjQNUIa9i0OkuIrwBXGPsgAMOKJk9dYKZhVWQAQ69N+onA7yBCRQgwhy8yCKLzDIRTwYI/HTE4Nx8aPdjAbuVZ/p/CY7odixwE857ag/WpE75xjUFgZdGIPC2iGHcMfJ94n92y2Ftn73SBD5f+3MLLEYFyEuDLhwfvp/eA3+o8L/Xbt820Ya/sRjhOCbQLx7dNnOm53/w9FEQKDCGj6Wgje1WH9Wd1myzYJjGYB476fn9tyeNgdLHD+p+LNC8zCKj/p/d8gLy41t8ZuTuoRFA3WOd0TbBtGHFXtUaD5uvMgpo/XzhGu1n/EPSPs4V7vcXXaLNKfNhOPZ1L+5+rA1POPbkrTuf2XmAkTT10Kcj14K9128ziPwdpS3BqnI30HdAX2xqZarGSI8HBDLtpiAQ88WHz5j6VYV5nV9l1bxgnPE/jL/DNaEJU96vGvOihAG7Kp/eWGdsPTPIZIHODdxWMyOwfd4t8pwyCYfn+GQXxjnr+LUWBKp4wIwVgApwMgwQGCT4JfoJ5AEK2EDJlwEIwIPvHbMjfzugShUKvnhMlXL4YRCBE//3ObMk4Bhq9ZLwjBMxyYakyMyBGEdgGkACity/v/3UthRTyYQ9JwjQC6R7XrkAAXBAT2k5YOitb31rCQIFTEibAzjJl8g8rs8AZQxbqBGsr0kAx+kY9HcMnAH9yQbSfAKNG/ctwlmeQClgbEBECS+55JLluyN4RE1hIDeAQJH36kwDgnILThYItHgHk19stq1S+fCCO</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2181,7 +2225,11 @@
           <t>MRCS</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAS8AAAAkCAYAAADYbryvAAAACXBIWXMAAA7EAAAOxAGVKw4bAAAAm0lEQVR4nO3OsQ2AABADsd9/aZiBNCckF+59d/cA/FAeAFjkAYBFHgBY5AGARR4AWOQBgEUeAFjkAYBFHgBY5AGARR4AWOQBgEUeAFjkAYBFHgBY5AGARR4AWOQBgEUeAFjkAYBFHgBY5AGARR4AWOQBgEUeAFjkAYBFHgBY5AGARR4AWOQBgEUeAFjkAYBFHgBY5AGARR4A+OwFHuZz20lnCYsAAAAASUVORK5CYII=</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>Healthcare &amp; Medicine</t>
@@ -2265,7 +2313,11 @@
           <t>MRCS</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAARIAAAAsCAYAAACpMDdKAAAACXBIWXMAAA7EAAAOxAGVKw4bAAAAtklEQVR4nO3OoQ3AQBAEseu/6aSIB6uRDMx9d/cBPJoHgL55AOibB4C+eQDomweAvnkA6JsHgL55AOibB4C+eQDomweAvnkA6JsHgL55AOibB4C+eQDomweAvnkA6JsHgL55AOibB4C+eQDomweAvnkA6JsHgL55AOibB4C+eQDomweAvnkA6JsHgL55AOibB4C+eQDomweAvnkA6JsHgL55AOibB4C+eQDomweAvnkA6JsHgLgfaOrrm6Z/fdkAAAAASUVORK5CYII=</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr">
         <is>
           <t>Healthcare &amp; Medicine</t>
@@ -2351,7 +2403,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>https://www.rescue.org/sites/default/files/2022-09/og-image-default.jpeg</t>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEA3ADcAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCADkAKIDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD0iiiivzM+iCiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKYEq/dH0ooX7o+lFbGRFRRRWJqY974q0HTrt7S91a0guExujkkAZcjI/QioP+E48L/wDQesP+/wAK8K+Kn/JR9V/7Zf8AopK42vqaORUZ04zcnqkebPGyjJqx9Tf8Jx4X/wCg9Yf9/hR/wnHhf/oPWH/f4V8s0Vp/YFD+Z/gT9el2Pqb/AITjwv8A9B6w/wC/wo/4Tjwv/wBB6w/7/Cvlmij+wKH8z/APr0+x9Tf8Jx4X/wCg9Yf9/hR/wnHhf/oPWH/f4V8s0Uf2BQ/mf4B9el2Pqb/hOPC//QesP+/wo/4Tjwv/ANB6w/7/AAr5Zoo/sCh/M/wD69LsfU3/AAnHhf8A6D1h/wB/hR/wnHhf/oPWH/f4V8s0Uf2BQ/mf4B9el2Pqb/hOPC//AEHrD/v8KP8AhOPC/wD0HrD/AL/Cvlmij+wKH8z/AAD69LsfU3/CceF/+g9Yf9/hR/wnHhf/AKD1h/3+FfLNFH9gUP5mH16XY+w4ZUnhSaJw8cihlZejA9CKfWZ4d/5FnSv+vOH/ANAFadfK1I8k3FdD0ou6uSr90fSihfuj6UVZBFRRRWPU1Pmr4qf8lI1X/tl/6KSuOrsfip/yUjVf+2X/AKKSuOr9Ewv8CHovyPBq/GwooorczCiiigAooooAKKKKACiiigAooooAKO9FHegD608O/wDIs6V/15w/+gCtKs3w7/yLOlf9ecP/AKAK0q/Oa/8AFl6n0EPhRKv3R9KKF+6PpRTIIqKKKx6mp81fFT/kpGq/9sv/AEUlcdXY/FT/AJKRqv8A2y/9FJXHV+iYX+BD0X5Hg1fjYUUUVuZhRRRQAUUUUAFFFFABRRRQAUUUUAFHeijvQB9aeHf+RZ0r/rzh/wDQBWlWb4d/5FnSv+vOH/0AVpV+c1/4svU+gh8KJV+6PpRQv3R9KKZBFRRRWPU1Pmr4qf8AJSNV/wC2X/opK46ux+Kn/JSNV/7Zf+ikrjq/RML/AAIei/I8Gr8bCiiitzMKKKKACiiigAooooAVQWOFBJ9BT/s83/PJ/wDvk0ttczWdzHc28jRTRsGR0OCpHcV9B/D34hQeKLZbG+ZItWjXkdBOB/Evv6j8R7ceNxNTDw54w5l1NqNONR2bsfPf2eb/AJ5Sf98mj7PN/wA8pP8Avk19g4+lLivG/wBYf+nf4/8AAOv6h/ePj37PN/zyk/75NHkTf88n/wC+TX2FijAo/wBYf+nf4/8AAH9Q/vGb4eyPDWlAjn7HFn/vgVpUUV83Ulzycu53pWViVfuj6UUL90fSitDMiooorHqanzV8VP8AkpGq/wDbL/0UlcdXY/FT/kpGq/8AbL/0UlcdX6Jhf4EPRfkeDV+NhRRRW5mFFFFABRRRQAUUUUAFS21zNZ3MdxbyvFNGwZHQ4Kkd6ioo0aswTPoj4e/EKHxRbLYXzLFq0a8joJwP4l9/Ufj9O9r4/trmazuY7i2leKaNgySIcFSO4NfQnw9+IUPii2WxvisWrRLyOgnH95ff1H+R8nmuVezbrUV7vVdj1MNieb3Zbne0UmaWvnzuCiiimBKv3R9KKF+6PpRWxkRUUUVj1NT5q+Kn/JSNV/7Zf+ikrjq7H4qf8lI1X/tl/wCikrjq/RML/Ah6L8jwavxsKKKK3MwooooAKK6e28F3t/4LPiKxzMsMrx3EIHzKoAO4eo5Of845iojUjNtRexTi1uFFFFWSFFFFABUttczWlxHcW8jxTRsGR0OCp9RUVFGj3DY+ifh78QofFFstjfMkWrRryOgnH95R6+o/H6d7Xx9bXM1pcx3FvI0c0bBkdDgqR3FfQfw9+IUPii2WxvmSLVoxyOgnH95ff1H4j2+TzXKvZt1qK06rsephsTze7Lc76iiivAO4lX7o+lFC/dH0orYyIqKKKx6mp81fFT/kpGq/9sv/AEUlcdXY/FT/AJKRqv8A2y/9FJXHV+iYX+BD0X5Hg1fjYUUUVuZhRRRQB9BfBkZ8Ct/1+SfyWuZ+JXw1+zedruhw4gAL3Nsg+56so9PUdv5dP8Gf+RFb/r8k/wDQVr0IjIxXxtfGVMLjpzh31R68KUalFJnx1RXrnxK+Gv2Yza5ocJ8n71zaoPuerL7eo7fTp5HX1WGxVPE01UgeZUpypyswoooroMwooooAKltrmazuY7i3kaKaJgyOpwVI6GoqKGroa0PrjRriS70OwuZm3SzW0cjtjGSVBNXqzfDv/Is6V/15w/8AoArSr84rJKpJLue/H4USr90fSihfuj6UVRBFRRRWPU1Pmr4qf8lI1X/tl/6KSuOrsfip/wAlI1X/ALY/+ikrjq/RML/Ah6L8jwavxsKKKK3MwooooA+g/gx/yIrf9fkn8lr0OvPPgx/yIrf9fkn8lr0Ovgsz/wB7n6nt4f8AhoQgHgjivFviV8NTb+drmhwExffubZB9z1ZR6eo7fTp7VSEAjBqMHjKmFqc8Pmu5VWlGorM+OqK9c+JXw1+zGXXNDgzCctc2yD7nqyj09R2+nTyOvuMLiaeIpqpBnjVKcqcrMKKKK6DMKO9FHegD608O/wDIs6V/15w/+gCtKs3w7/yLOlf9ecP/AKAK0q/Oa/8AFl6n0EPhRKv3R9KKF+6PpRTIIqDRSVianinjz4eeJNc8aX+pWFnHJbTeXsYzIucRqp4J9Qa5z/hUvjD/AKB0f/gTH/jX0cGHIBo3D174/Gvap53iIRUEloccsHTk73PnH/hUvjD/AKB0f/gTH/jR/wAKl8Yf9A6P/wACY/8AGvo4sB1IH1o3DGcjHrV/27if5UL6lT7nzj/wqXxh/wBA6P8A8CY/8aP+FS+MP+gdH/4Ex/419HBgehB+lJuBOARn0o/t3E/yoPqVPuch8NdB1Dw54Wax1KERXH2h5NocNwQvcfQ12NISBwT9KAR2NePXqyrVHUluzqhFQjyoWik3A5waTeucbh+dZWZVxSAQQeleP+OfhNPdX/2/w3DH++bM1qXCBT/eXPGPbt29vYNwzjPNIXVTgsBnoCa68Ji6uGnzU/uM6lKNRWkfOX/CpfGH/QOj/wDAmP8Axo/4VL4w/wCgdH/4Ex/419HFgOp4oyCcDrXo/wBvYn+VHP8AUqZ84/8ACpfGH/QOj/8AAmP/ABo/4VN4w/6B0f8A4ER/419HbhnGRmgkZAJ5NH9vYn+VB9Sp9yno9vJaaJYW0y7ZYbaONxnOCFAP8qu0CivEnJyk5PqdiVlYlX7o+lFC/dH0orUzIqSlpKxNTA0QMPEfiUkHabqHB9f3EdcO0OqW+p3MirJNp914jQMmP9Q6zIQ3+6y5B91HrW34i+KmmeHNdudKubG7kmg27nj27TuUN3PvWYvxv0IsA+m6gF7kBD/7NXvUKWLT9oqV00vwRxznT2ctjpPHul2t/osMk1qk0sd1AqMRkqrTIH/Mdab42soLP4fXlpaQpFDH5QWMKSqjzVzwO3WtTw74o0vxTYtdaZMWCHbJG42vGfcf16Vxkvxr0SKV4m06/wAoxU4Cdv8AgVc9CnipONOMG+R3sXOVNLmb3Og8DrYLb3a2cmnO25S5sbZ4QODjIcnJ61ylnYzr4qjuntYoIn8QTj7eu4ynBOImHGEbkZ5qx/wu7Q+2m6h+Sf8AxVegPq9pBog1e5kEFp5Kzsz/AMKkZ59+e1a1JYjDzlKcPj0JjyTSSexzfjO1vrvXvDw02UxXcZuJImP3SyoCFb/ZbGD9ateFb/yvCM+o3cMsAE93O8Tr86DzXbGPWuSvvjhp0NwyWek3FxGDgO8ojz74wa2PDvxY0PXbxLOeOWwuJGwglIKMfTcOh+tOeGxUcMoSp6LXz6/5iVSm53UiPwRNqFprBTULO5t/7Wtzd75mUh5g5LbcE4+R04OPudK0YNA02L4jzTpYRKRYpcBwv/LUyvlvrjFbmv8AiHTfDWnG91Kby0zhVAy7n0Ud685k+OlqJiI9CmaLPDtcANj6bT/OphHE4lyqUoWTVtxt06doyZ3O1v8AhY27B2f2TjPbPm1zOvjSR4g1tfEUM0k0scY0rCMxI2YIhx/HvP6iuj8K+N9I8WxN9ido7mNQZLeXhwPUeo9xWFf/ABc0jT9auNLksL1poJzAWUJtJBxnrSoQxEajj7N3St2HKUHG99y94jgvX+FZgv8Aeb429us+Dlt+5N3Tv1o8J/2inirWINSV2ntra3g88jicBpMOPqCM++a2vE/iO28LaOdSu4ZZYhIqbYsZyfr9Ky/DXxA0/wAUW2pT2tpcxLYRiRxKFywIbpg/7NRF1pYebUPdb37XaG+RTWuphz399/wnba8LS7axhvF03zgVEYhxtbIzk/vWBzjGB1rc8VXsGneKPDN5dOY7aN7nzHCkgZjwOnua57/hd2h5/wCQbqH5J/8AFU5PjZockioNNv8ALHAyE/8Aiq6pYbEtxl7K1lbfpYzVSmtOY9KhlSeFJozujkUMpx1B6VJSClr597nYtiVfuj6UUL90fSitjMiooorE1Pmr4qf8lI1X/tj/AOikre8V6x4CuvBot9LtYP7W2xhHhtTEVYY3EtgZGM+tYXxU/wCSkar/ANsf/RSVd+IPgiDQLLTNV02Jls7iJVmXJbZJjOck9+fyr7mPI40VKTTtpbrotzxnzXm0jb+B1tdDUdUutrC18lYyxHBfORj6DP515tDPb23iJJ7uD7RbR3W+WH/nooblfxHFe6/CfxHb6v4ZXT9kcV3YgI6IoXevZ8AfgfcZPWvDrO6trHxTDd3kHn20N2JJYtobeobJGDweO1Rhpynia3MrbDqJKnCzO2Txj4Dd1UeCQCSBneK9B+J+l3V14Akt9NiYrbvG7RR9417Y744P4Vy4+JHgIcjwqf8AwCg/xrpfE3xCl0vwnZaxp2lzTLfLlHl+5D6b8Hr7frXn14VfbU5Qg1Z9Xc6IOPJJN/ceL+Ftf0/Qbid9R0G11VJQABOeY8emQRz9O1egeC9R+H994pjuINNksL9wFghnbdFv9VP94+/pxzWRF448I6tYqPEnhcSXw+/PZqqeYf7xwVPPpzXIadZHWfF8NvocM0EctyDbqWLNEu7OSR/dHOfavUq0/bRlzpwdt76f18jmjLkatZnSfF7VZr7xtJYsSILGNI0XPBLKGLY9fmx+Ar0vw38O/Di+E7SK606G5muIEkmnkHz7mGeD1XGccfjXB/GPw3Pa68uuRRs1rdqqyuOiSKMY9sgD9au6D8ZI9N8Nw2V5p0s15bRiKN0YBHAGF3dx+tcNWFWrg6awj23sbRlGNWXtTq/CfwssfDeq/wBpveTXFxGzeSoOxUU8DOPvHH4c9K8a8Tf8lB1T/sIyf+jDXo/w68c+KfEGvPZ3EMd1ZEtJLMV2/ZxzgAjrzwAcmuE+IOm3OjePL+SVDsmnNzExHDqx3cfQ8fhWmC9tHEzhiJXk0TW5XTTgtLnrPxi/5EJ/+vmP+tcb8IP+QT4r/wCvVP8A0GSqvjn4m2virw5DpttYTQytIskzSMCFIHRcdeT1OOlbnwr0a4svBuu6nOpRL2IrEGGMqit830JbH4VkqcsPgHCro2/1RXMp1rx7HlmgXlhp+uQXWp2P26zTd5lvnG7KkD8jg/hXoGneKfA17qdrax+DAjzTJGrFx8pJAzXDeFtSsNI8S2t9qlp9rs49/mQ7FfdlSBw3B5INemJ8S/AkUiyR+F2R1IKstnACD65BruxsZN6Qb06O36mNFrq0j18dKWq9jdJfWFvdxqypPEsqhuoDDPP51Yr4eSak0z2E9CVfuj6UUL90fSitTMioNFIaxNTk9Zg8EPrhTV4dObUpiu4zLljwAuT27Yziuhu9Msb+w+xXdrFNa4A8p1yuB0rk2s9R02/1u1/sH+1I9TuhPFO7J5ZUgApLk5AXBxgHPtXbKCFAIA9hXdiW4KDjNv5+m3Yxgk73Ry0I8F+HNaWCAWFjqDAJhBtOG6Bj0GeOtWj4I8LuxZtCsSSckmIc1g3+m6rFb+IdHj0d7z+1rh5YLvegiQOAPnycgpjIwDnArubaIw2sMTNvKIFLHuQOtaYicqaU4VG299RQSk7NHJyaF4CimvYZNO0xZLFBJcqYxmNSMgn8K6OyttNm0aGC0hhfTZIh5cYXKMh5HB7VweveFdVvfEmp3MFrm2v5EgmYsBuhCRNkc/3oiv8AwOu38OWs1l4Z0u1uIzHNDaxRyIf4WCgEVWLSVKM1UcnppfbT/MVP4muWxzV34I8BXGtGzl0+BL9ozP5McrplM4zgEDHXpW14X0vw5aaet14dtbdbebIE8YyXAOD8zcnkVz3jDQNZv9bnvdKt/wB6baK3SUsBhW85JBnrwJFb/gIro/CGnTaV4bgs5ofJeOWYiPjhTK5Xp7EVWIk/qyl7Vtu2lxQXv25TRvZLGWSPTrwRSG6VtsEi7hIF5bg+mRXL3vw58EwLLfXOlpFEgLyETSBQB14B/lWxqVlczeLNEvI4i1vbx3IlfP3SwXb+eDW2feuSNadBR9nNq+9n5mjip35kYXhu+8NywNZ+HnthHEMslum0Dtk8cmn+Jo/D503d4ijt2tN21WnTO0kdiOR07UeGLKex02eO5jMbteXEgBOcq0rMp/EEVY8Q2st54a1S1gj8yaa0ljjQfxMUIA/OqbisVpJ2vvfX1uCT9nqjnNE8FeBLtF1DS9NguIwxAZnkdc/Rjg/lXQ6tq+j6PDHBqVxDbxTqyIjA4YDGQAB7j86m0aCS20OwglTZLHbRo6nsQoBFc/4usL651nRrq1g1CSO3S4ErWEkayLuCbeXIGODVxl9YxHLUm7a7v9SbckLxRYtPCHg++tY7q20WwkhkG5HEXUfjVDUtL+H2kXS21/YaZBOyCQI0PJXJGeB7Guq0xpG0238yO4jcIAVuSpk44yxUkEnGeK5XXtP1A+MDfw2+rtbtYxxb9OkiU7hI5IbeRxgjpWmHqTnVlCdRpLz/AFFOKUU0vwOwtVhS0hW3AECoojC9AuOMVNTIXMkKOY2jLKCUbGV9jin15kt2brYlX7o+lFC/dH0orUzIqKKKwNQxRiiigBMUuKKKADFGKKKADFFFFABRiiigAooooAKSlopgFFFFIAooopgSr90fSihfuj6UVsZB5S+po8pfU0UUrIoPKX1NHlL6miinZAHlL6mjyl9TRRRZAHlL6mjyl9TRRRZAHlL6mjyl9TRRRZAHlL6mjyl9TRRRZAHlL6mjyl9TRRRZAHlL6mjyl9TRRRZAHlL6mjyl9TRRRZAHlL6mjyl9TRRRZASCIYHJooorWyMz/9k=</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2446,7 +2498,11 @@
           <t>MPG</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAHgAAACfCAYAAAAyJR3oAAAACXBIWXMAAA7EAAAOxAGVKw4bAAARbklEQVR4nO2dB5AUxRrHuTuPjBJFpAARMRBECYqZZCIooIcoAmIiCBYoWAgqpQ8lCAeCWghiQBBJWlpKFBTkAaKgiAQjCChIzhn69a/f9tbc3s7FvZ3Zve+r+tfuzvb09MxvOnzdPT0FChQooERxLc8TIBLAIgEsEsD5VJ4nQCSARQJYJIDzqTxPgEgAiwSwKPeAzzvvPJWSkqI6deqkOnToIMoDdenSRTVp0sQbwLVq1VIHDhxQYnlrCxcu9AZw7dq1BXAU7Msvv/QuB+/du9fr8497mz9/vgCOZ/MV4LNnz6pXX31Vde3aVfXq1ctT9ejRQw0YMEBt27bN9eL9888/qmfPnkZep7dbt27q3XffNdfQt4AxtkcwQblSiRIl1A8//OAK+KeffvI8jU61adPG/4AbNGjg+YWyKl++vFqzZo0r4J9//tnzNDrVvn17/wO+5pprPL9QVhdccEFMAb7//vsFsAAWwAJYAAtgASyABTBKSkpSffv2VVdffbUAjjfAiYmJ6o033jBxbdiwQVWtWlUA51YltNomJKjSHgNO0GkYO3Zsmvi+//57Va1aNQGcExXW6qAv6rKERHVM55zV+nsfrVIeAU5NTQ0bJ71jHFcAZ0O3aM3TMAF7Umu/1qnE/4Neq7f306oRJcAUyyNGjHCNE1uxYoWqVKlS/gScGFBWjlFHa5KGt1df1NMBsHsCstvOaB3Wah4lwIMHDw7uf/z4cXXs2DHzHTD8trZ69WpVrly5/AO4rFZHDat/YoJqpovZ5uYzQTXUqquV7Ixba7TetkOD01lGHXRABfKJANylOkxPHbaMSxrzAvAvv/xi9t25c6cZASIOa+PHj1fDhg0L/r722mvzB+CqWss10K0aSmMNJUUDTk1MUlP078Vaq7RG6W3t9X8DtTYHwB4KQN0dyKUnA8XyHB2mvY6zeCZpzAvAf/zxh8m1t912m5mXxm9r1MuE+eCDD8zv66+/Pn8A7l6smNKVkppQsKD5XUSrutYQDWoRwJIS1UqtXQGIRxw59kAA9g4ddrJWI71f0SymMdKAk5OT1apVq1THjh3N78qVK6s///wzGB8uE9sLFSqkJk6cqJo2bRr/gJO0ZlSooFTNWmp4csF08YwokKDWB3LrgQDUfYEcS9G8SUPlRqiXgxPKC8DOYveiiy4KCxgVLlxYnX/++fEPOEErtWhRpUqWVNOSkkx9WTGhgC6mE9RcDXCL1lEH2KOBenaj1nQdZqL+HKRV0weAQ5UR4JwoJgEjimNy4lZdDPfWsPrpzzEa9hJdD1Pf7tPfj+rv1K/rtObr/8fpz1la/9XftwWK7wnZzMkCOEqAEQ2taRrQfzSozlrDtKZqcEv053KtBfq/VjpMJS382rWBxtWOpP/Xx/sDdfF2rZH6/yoC2F+ArWhgVdP1bgvdam6nQbXUqhAmXGu9fSXukM7dhx2t6SOBTo5NgRZ3RQHsL8DZUTmtARri7oDfu8/R0XE4kKM3aBGmsgCOPcBW9bVmaohnHQ0yZ28WoMnNAjhGASPcrRTd+salOhuokymuj5tOkgRT9AvgGAZsRX09NJCb6RnrkkFYARyDgK1aaNXNJExeA7744ovVnj17gvHxZIIAjqLyGjDxA3X27Nlqzpw56oknnhDA8QQ40hLAAlgAC2ABLIAFsAAWwALYewngPAB85ZVXen6hrJgzFUtP+Ldt29b/gO+77z512WWXqZo1a3qqK664Qt18883BWZDh7LffflM1atQw8jq9l19+uerXr5//Af/777/qr7/+Ulu3bvVUW7ZsMYusnDx50hUw/3mdTiuumbPb07eAxSJrAjjOTQDHuQngODcBHOcmgOPcfAUYH+7gwYOmub9v3z5PRRpY7vjMmTOuF+/06dPmHLxOq03vkSNH/A34xIkT6qGHHjLP79xwww2eqmHDhuree+81/rCb0QnCE4DID+llIVdfA+YBaHpkIpigXImHvzZu3OgKmDU1vE6jU4888oj/AUdiOaFIiVmPv/76qytgnsL3Oo1Ode/eXQALYAEsgAWwABbAAlgAC+Bs6umnn1bvv/++evvtt9WkSZPUVVddJYDjCfDSpUvTxMcUFgEcR4B5y5fT7r77bgEsgAWwAM4F4JtuuslMr42EPvvsM3XuuecKYD8BbtWqlev+2TUm1pUqVSr/Ap47d26a+FgP0mvArVu3jgxdbTt27FClS5eOX8BlypRRt956q2rcuHE63XLLLWYdSKfx7kGKyNCwxFGvXr2oAGbO9OjRo41GjRqVY7H/s88+q4oWLRq/gAFz9OhRdejQoXRiogAD8E4jLIP2oWHZvnjx4qgAjqZiHnDz5s1dL3Z2jUdSBLDPALdo0SJigLPy4JgAjjJgpsb8+OOP5sKG6rvvvjPFtNNYbPvbb79NF5Y4WHQ7GoB5QpGpP5HQ7bffrgoWTL+kctwA5uSYRlO2bNl0wn2gXnXagw8+aJ4QDA1LHCVLlowKYFy1SBnPSsV1KzozcTJOo87OzQlFAnAkqxXSktGNGfeA/djRceedd5rWfSS0bt26/J2D/QgYv5UV7SIh3qXEuw4FsI8AR1NxD3jhwoUCOJ4Bf/PNN2nikwH/OAPcp08f876hcePGqXfeeUem7MQb4EhLAAtgz9MogAWwABbAAlgAC2DvFROAc+vaRFJVqlQRwJEGLE/451wPP/ywvwGzRsczzzxjZiKyKKmXohesZ8+eZgzWzXjnUUpKipHX6W3Tpo3p4PE1YLHImwCOc/MlYIo+Roa+/vprI75n1Nhx2qlTp9SyZcuC+zOEuGHDhixfEKbUMmjx1VdfBY8fKqYGMQeMZXzzwn7//XdT3L7wwgvq+eefN+L71KlT1e7du7MVl+8Az5o1S1144YWqSJEiqlixYkYMmleoUEG99dZbGZ4McNq1a2ee32Efuy/zsLhAmRnAmObjPLabihcvbmZX4EoxmR7ooYtxZ8eYMPjee++Zxb2ZlnPOOeeYOWj2ePxOTk42DT9miYRO8nczXwE+duyYuuSSS8xFY1GvkSNHqhEjRpiZ/eXKlTMuVEYX0bZqO3bsaPZh39dee82s3A5oZlhmZDw9wP7PPfdccP9wGjZsmMlVXbt2NceqWLGi2Y9Jfixonl0j3fZdFfXr11dPPvmkAfP3338HJ/Vv3rxZTZkyxayFxbWw6cxowXLMV4B37txpZkc+/vjj6RI6aNAgc0dT/LoZ+5UoUSJdcc7QIcfk6f+MbPjw4SaXZNe4+KSPY+AB4O5l1T799FOTZqB9+OGH6vDhw5nuw6sE8Hk5Xjjf12m+Akz9wol27tzZ/GadSLtW5LZt28x+vILVzcj9zB8O3ff11183+1KHZWTkTgCTa2wc2bE333wzmLOyUlxTzFKdZNZj5mYvvviiOd7gwYNdw8QMYHIFF4LJ3+EW3Zw3b56pO4cOHZpu35wCBhIzGRcsWGAaXVaLFi1SK1euDFsc0wZISEgI+/4Ep+3atcvckJUrVzYT9O3xMK4LNzJ1rX1g7oEHHjANvNAbx85a4dHScBYTgO1JUSe7nQxvHOE/6i3nvlhOAWNdunRxncmYmJioevToYcLbNH7++eemQZRZdTBkyBATB6+Vxez+/KYhxX+1a9dWN954o2lD0MhkG6CdD9lRfxcqVEg99dRTYY/je8CcuD15+0Rg6MXjArNCLXJaJAAzcY800YKfMGFCGtEYIl6gWqN04ZU85Cw3I114Ck2aNDElkz0/SorChQubAZeZM2cal88aN/XAgQPN8ULrXRqfrDYbrsHle8Ak2oLav3+/OflQkPZBMgueOxyXyV643ABu2bKlcV3CGQ2iatWqmTDOopP0Ac/NcIfI/Sz3ZI3iHveIXEtj0814iTRVAA07a3gc5OIVK1akC+9rwBh1FY6/NVwRLoQtirGXX37ZxEm9aONx5qrcAGYJBnJkOCOH1alTx7g4zgYZgJs2bep6nF69eplnprgJrY0fPz5daRDOOEfC8XA7HgW5mYff8TBCl5HCfA+Y3MnJWPviiy/M/s67v3r16uquu+4Kuif0Yjn/zw1g4iWXkqtYWZ00I4rMjz76yMRL/NaATi4kV4czShcGJ3iFn9MoYrkxsuJiMbCAX1+1alXzljjqaJ6WdBbp1nwPmPcDUg/aljMnQS9S7969ze/169ebesvZU0UuHzt2bPB3bgDj17IvQMitfALQNnpYbZ3i1RbRtLC5+HSwhDO6YelZs+nHgE4pwcslnYa/S+ORsFZMDcaT4Nj0cNFqZ2kHt04c3wPmgvCMrfOxFHqPbBGHD0h8PPOLUS82aNBAjRkzJhg+N4DxaUmrfUchIBizBjydFORqzAKmNcuxnFWI06gn+Z8i2RpuEtAfe+yx4DbOzb6oky5RzteK64GLRQ7mRuOGYv0SW0XFFGDemUB4OhGs0dpkG3UQxR0nao2iigYMvVe5BZzdjg58ZI7dqVMn132XL1+eLi0MXFAK4XJZo3uScORgSi9n9WBfBML6I9wIdJi4nZ/vATMAwEWnj9ZeeO547mBW0KFzw/kyiv79+5v4aalaiwZgbjq6WWkPsNyRm1nA3IjWmDVCw9HZRUsaaDjRBZqZMSmBOKdPn57uv5gAbJcOcr4BhQ4IGxfOPkbvERc4GoDJVQwrUhU8+uijJn6OvWTJkgyPQVVCR8grr7wS3EYuvPTSS03VY400ECfdkW5m00eDL6YB06hin9TU1OB2YLCNFiRFFWZdiEgBxgDRqFEjs65W3bp1zSei9WrXy6AUofFDf3lmRtzXXXeduuOOO9JsJ258ZwuNkTWuETm7WbNmZlE3lpHik0bW5MmTg/V+zAO2yxZwotbYl5ztdKEYvos0YJZgYN977rknzYIotHiBSjsgKyNATiPH01ByGudBBwb1sTVyO+PT+Nm4UNaVIj10eFiLecDkYPpnKQLxizFcC+7mjz/+OBiWeprcRKuTpwyt5VVPVk6Nlj/HoVFmDW+BbdzEzuNjzr5ncjZ1PTeztZgGTL1LZz9+Li6CdS+YgYnLYftfcVk4cYpP/MNIAaYnC7cos4H17Bg3LcU77QjMFrXTpk0LVjs02jhHa4Shfrdtj5deein4X8wDpujCTeJCM5riPHFrffv2NYCBRPhIuElYXgDGOEduxLVr16bZDiR8YtJLicSgBcK3ZxvuFF2z27dvD94YtNpjGjDhme1gp9TYyW62QYJPSCMFGLb70O+AcfWoSqhf7QJuFhg9Y7TOOSeuE+I76QvXgUK9ba9RqMUM4E8++UStWbPGfGdhbOcFIRewnZMhXCwAxhgSJF0M7Gd3tqQ1Jjqw+g7zwmxvntN8BZgOfbrcaGVaIwzhcQsomrnYzHBwGt2JDJdRF82YMSMdTAYe2ObsXAhndJgA2NmooXikcReuWoiEkVNJG2O64boa3YwpPnRtsi/dp26zLH0FmM4D+lbxOzkBci8D64S3bg+PaeAe0bmxadMmU9ThctglA2fPnm3C89gJRTmih4ht3O0ZGZPuCEdjhpuFgQwGFmhFhy5VHEmjRLKDF9xQ+PuhLWmMKonXBXE+NDgJT993RtODfAUY49kk+nOZjEZuJiytStuJwJQWANMK5X97orZIxo2gf5pt/G/j6NChQ6ZDcXQjUtxRGrAfjSDSwjTZvDZuKLpZy5cvb9KLW8h8LTpUyKHMR7PTc+kXYBSJpxszM98BZjgQWDj+TFFhEl1ow4I7nv+Ym8xQGfOFnUZxyrxm4kAUg+HGSsMZxaR9ooB9M6u3I23U9bhLTAfiZdncmIh2Sbdu3cwTD3YEKyvmO8BikTUBHOcmgOPcPAOMWyCW92ZnkEQdMC1BJo/ZJ+RFeSNcTk8Ai2JSnidAJIBFAlgkgPOpPE+ASACLBLBIAOdTeZ4AkQAWCWCRAM6n8jwBIgEsEsAiAZxP5XkCRAJYJIBFAjifyvMEiASwSACLBHA+lecJEOWh/gc4l35O2us3BwAAAABJRU5ErkJggg==</t>
+        </is>
+      </c>
       <c r="N23" t="inlineStr">
         <is>
           <t>Human Resources</t>
@@ -2530,7 +2586,11 @@
           <t>HELVETAS Myanmar</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAaYAAABvCAIAAAAog/OcAAAACXBIWXMAAA7EAAAOxAGVKw4bAAAMcElEQVR4nO2dW5LbOhJEew3exvzMhmY/s5O7TN5wtENWk0Ah6w2KmaGPbhKoKiSAY1CS7a9jJ/363/8Nr+6qKYq6jb66C/gjG+wIQYqiVGpD3jeYcIQRghRF+VWKPAOnZj+QehRFGVSEPP8ZLeToVzNYiqK2VTrytEQ7Rie7YRwwOMFHUdRLicjTPrTiP8t9Tz8Mr1MU9UxlIW9JNy3mZoc7JOa1quVFiqI+UsHIwx8th0Ac/mxAnvAkS+pR1JMVhjwcc2DH0933X6+hhL6zXLMyogyhKGpDBSBPppvqKVU4vgm/yrdm1coj8ttCUdSGCkPe9Qfkdfw8i82OeEsCyi2HBQtc43GPoj5VKac8hHHg6Qwh4OnutaV5UHZTKIraUnbkqdCGBFn+eqxIhLfEB+iJQFHUbjIiL+lYpyLgDIhEFUVRM1mQN+Ta8LqAvyGVPARcBqcoiopB3pVB2tPfe+TZr9cuIPLIQYqivqVG3gxwx9t3O67kArsjz7zDemSo8fRHUdS3dMhbPsnK7Ye3DIdEuRI5l2q8FEV9mFDkvYPmAPB0zE9tw1+RmKpop+KjkEdoUtStBSEPP2GBp7b3jtdEp7Dyr0vkxZ7veFqkqFtrjTwZPQeAvFkbAWF4VQJAbZHB1CGhKIoqlgJ5ArBOLd9/Hd6Vz4PXBq8IhhGGI+8g9SjqtlogT+adjJLlLRx5wqlQVTlgCCQij6JuKh3yhhevj7HHnFmnu7MsOPJAqlIURR0I8o7VoUwGlu2oReRRFJUh6JR3TB4kEeRdmx36B0Mij6Kof/7z39PLEERCnvAoempwvYs85Mr8kmmF4KwGeddp8EyMMxrS3fly1h9rhW3RG8LWG1uQEXcvby5C8qoKmCJPflA9NECRATd87DUc67oUuxSc0do3SbEVhm1mC1tvbEFG3L2kuXCms1UyRh7yxDrDn8ymZcxrs1mbTRS7FJzR2jdJ7K7I2Ga2YdYbW5ARdC82WmA6Wz0D5A2hNry+xOKpo/zrLNHwyj6KXQrOaO2bJHZXZOw0W8B6YwsygtaFBwxJZK5nirxDRJXAuCUBES0huI9i14EzWvsmid0S4dvMHLDe2IKMoHXhAf1ZPMM8I+9Kq/cfTs2uXQ4AeUN4LXG2J+8OIk9ZAG5FiCE2f8wdA40tyIhYFx4wJItnpD+Qp3qcnD3/Hj//ZhgSU4bghph7V+w6cEZr3yThW2ITe+uNLciIWJcRs8XeV2F/kTc70w25M8PWdTC29+l2fpI9KXYROKO1b5Lw/RC4zTyh6o0tyIj4lhGzZaT/zJAnvN6rlNvgZ8PhldnFPRW7CJzR2jdJ+H7we6I1x9M30NiCjP7ZDJni4pGiyDtVKTBrSSvkGZbIs0Xbf5PgVkR5EhKn3tiCjP7Z9M+yM6yh4w/kvX5YsmaGvAOjFcIyVRmNWKxfAWXFGJSRPWqbeYK0G1tfkgpGqQt+GVDVd/FVZKRoLfJmDbT82uQkWL8CyooxKCl79q5YBmk3tr4k0DFn6uxQ12Z/kDekjxBd++g66+t5kiXysosxKCm7f1x3N7a+JJxu4ZzyjGLZcYy8pYRjmqovkRcbrX1nJmX3j+vuxhaXZGCcLXXGKOReMchT0ScKedcyWhQ7Z3ffmb2b0NN3c2OLS0Iih2SvN7YBecM415gqNVIvds7uvjMbN6EQ3G9Lu7HFJSGRQ7Ijo4j19gfycOKEn9E8wOo964FzFvhyFtPrRl5kIbjflnZjK0sCw4Zkj13/iH4j74Qe8yHLc1Q008pfvFM2bHlejcX43ci2OqmqXldj3fBHDiyg3sOvKzIMx7TD9GhJ5IXPbmNqsIBsq6N6GYLkuRroRkhkQ0vPKGL9tCMvnFa2ICGVeJS6GbQz2pgaLCDb6qhehiB5rga64Q8bXkOxsQPkgdYE0srcPTyOQambQbuGGlODBRS4nVFSr6tRVoSEDa8h1dtrAV9mWOzwBZGTWurJnjDVGmpMDRZQ4LanvSdvnqshViTF3N/eUw1fZnJ53gTMUFcl2bOlWkONqcECCtz2tPfkzXM1xIqkmLdw+L0GO/JeqmHNMguRV1CM340CwzPq6XXVXFJ4zNQyUk1+ldGGvPBvtBB5BcX43agxPLyeXlf9PqQGDCwj1efvSnqQl9GFyCsoxu9GjeHaliFJ81x1+pAdsKUSs9Vfv6zfqnvJ+WnvrNepAd7FNgqzYufbGS1vg0XVX5lln3nJUD1oyirRBsdfRwjyvpX6lLrPhyRXxc63M1r7zqzJDg5zn3nJ0L0Wnnu4ulKFl/1LKh4ZkFdcIa57rbzsnVmT3bno6+clQ1sNsNcf1aR/tTBF9VS7+UGPK09VQFmi2ErajU0tyW/mDv6AZfQg7yWBYob38loUO9nOaO0rryx78Q5sNza1JL+ZGZ4bhNTQiTwVxfzISyJm7Ew7o7Uvu7Lsxduv3djUkkJwtoNFSA0bIU+ugchDorUvu8rslXuv3di8kgKJ5q/HaSZSQ8/HF9+qPOXlPRfHbgZntPadWZk9de8ZcgUOrbIkP8iinHdaChbQibyj8N8mIPJqdmZl9qSNZ84VOLTKkjw2BjpfM4rD8y+p3E6zz0OuDVRhYzeDM9rOCzc8lzkdPh37GGsraZ9xLUvK63gK0vyJ7UzZp7/roc+ccat1vP/CDcxlTodPxz7G2kraZ1xyVZWp//7fF7jX2Sr4Fp6MPFXGrdZx46rNKyB8vPh07GOsraRNBiVXVZz3HsgLJyBPebGrNrUAv2O2udjKWFtJIYPKMKrRWCJv8P9SqkJttY7rF1BBAX7HbHOxlbG2krIjmI1qNPZLO6QaRT11LlP442y1jusXUEEBIaYZ5mIrY20l+UeU5FWxt+/pNkXeSdlv7Xl0x3Ucu4ayCwgxTTsRuxlrK8k/ojyvyuw9lfcHeRui5CQV75Z8DBzvHddx3s6szGVIik/EbsbaSsrr7vfK3NFp5m2Qh0s+EoafFm+3jlN3ZmWuvFnY0NjYIYcXU1+bOf4ZeR/APhx5fC8vfD1V5sqbhQ2NjR1yeDGBtakqNNQ8Rt6tqVeMPIqishXI5b8fX9waebNvnAgtbzdGiqL8GnxiezscLA9up+u3GyBFUVH6cOQht2qLpSiqUw9FHh9vKeqZujHyru/c4R9WEHkU9UxNkbczC5DPZK8tZxGKiqYoagON/8LZ5ixAzm7L+jcfI0VRGXoK8uRTYUXRFEVtoHv8swIneT6f5Tt6FPVk3RJ5M4GfYyDtKYr6SN0GeUuWDa8LzVRv/FEU9Rm6B/K0b95pP88tGAJFUTvoWciTGxcMhKKoXt0DeYfyzTicj/5n21NYIc615a/RP3OvimCr5MAGLkebDcdQeWxj/hlGCboN8o7JV2eWu9Fw0VDVcrMJ27IdebOWBuThY8drMyOPBKSuuhPyXjKwb9gmZD/4kTe8i0QwlAFGG7ZRjSi2NqE9jjxSjzruiLzhCl6CYHbFvxN2Rp6KFMs2qhEZLIoaCKlHCfoE5M3WtHwxox4z8oYN5O7a+P6yzRmJPGoffRrybC2FRKp6cGAhzcBbeHxt2YcJeeDYtYXNuhicmaWmnqD7Ie8YwQjZRQeMPAMZM5D3a0RqLX1AUmyCPP9AkJjDONRDdEvkqWRY6KougcgbtrxexGuwwWXWzB+hBXlgG+oh+nDkGRa6ub2wRT3I03YZXrGVfXQjDxkLkUep9BTkBbacdZztahW//O2Fi4YsNuQhY08aCDLSaxvqOfpw5IHy7IePRN4wjqHOXuThqanniMj7Lc9mOO2lJTWQ7efh4/D6suOsC4487diRkpCxyOQl76iTiLzf8myGJTgqkSdEWHYcdilDnlBwIPKGblOPEpHn1RIcBuQN4yDNwFuzuypeIND0ANQ2EPKOkkXkeaUCx/UuEhbknRNYSPFyhEDk4WMh7yiViDyvcOQN7yJhQ5AnkwKJiVSIj71+IDOrqUeJyPPqw5C3rF+OsDPySD3qIPL86kKeFhOfhDwBbXLYmdvUc9SAvA9bfNojRiPyQFLI9csR8KRdA5kZTj1E6ch7rTNkF713ucsCBbfx7BYSFkGeNo4BqbbIWuTFDoTIo04qQt5pzeF/1A8bzK60qAV5+E7+VOQNl4FtINSjVP1gO2MfuHlkMrYs63shDyeFtgbt2LUDmWUk8iiV2t7LuyJPaDmD2gx/let7lqsSeWB5WuQJo5Mj4NcLkKfNQn22mj+xXQLLtme4simKGmqLL6kgh4jZ69qyYwQURd1D/wIUFnF2T1BjVwAAAABJRU5ErkJggg==</t>
+        </is>
+      </c>
       <c r="N24" t="inlineStr">
         <is>
           <t>Administration &amp; Operations</t>
@@ -2618,7 +2678,11 @@
           <t>MYS</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEAYABgAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCACtAS0DASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD3+iiigAooooAKKKKACiiigAooooAKKKKAEpaYzqgyzAD3OKzLrxHo1jxc6paRsP4TMufyzQk3sgNaiuRufiP4Ztzt+3mRh2jjY/0rKm+L2hoD5VtfS477FUfq1aKjUfQdj0OivLZPjHAP9VpEp93mA/pVZ/jHN/BpCD/elP8AhVrDVewWPWuaOa8dPxi1A/d022H/AANqF+MWo/xaZbH/AIG1P6pVCx7HRXkafGO4/j0hD9JT/hVqP4xwH/W6PKPdZgf6Uvq1XsFj1KivO4fi9okn+stL6P32KR+jVqW3xK8M3A5v2j/66RsP6VLoVF0Cx2FFZFp4m0W9wLfVbN2P8ImUH8s1prKjjKOD9DmsnFrdCJKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooASlqrd31tYW7T3dxHDGB992wK4DW/i1Y2paLSYDdv0Er/In4d2/SrhSlP4UB6MWAGScCsTVPF+h6QGW61GESD/lmh3v+QrydtR8a+M5Ctv9pNu38MX7uP8AE9/zra0v4QzSYk1bUFT+9FAuT+LH/Cuj2EIfxJfcPQual8YLWPcum6dJM3Z5n2j8hk/yrnpPHfjPW3KadFJGp7WtvuP/AH0c16TpvgHw5pm0pp6TSD/lpP8AP/PiuhWOG3i2xokcY7KMAVPtaMfgjf1A8VXwf441r5rySZVbqbm4P8q07T4O3Tc3mqxJ7RRFv54r0q51vTrXSrrUjdRy2tqjNM8JD7QOvSvOLz486FHcwxWGm6hepMNscoTYrSdkGevOKTxM+mgXNa2+EejRKPPu7qU+zKtakPwz8LwgFrFpSO7zN/Q1jeCfiJqfiafXNO1DS4tO1XTkLrE8hCdP4iRxg15ve/ETxZpt3Z6p/wAJK2owi98q5itrQCzC5+6spHzEgdunrWbrVH1Ee4R+C/DUI+XRrXj+8uf51YHhrRIkJi0eyzjgCFea8n8Y2d/r3xttPDrazfWml31mJHjgmKg7VY/KOxJUfrXtkEKwQpEudsahRn2qeefcDy6w+IHhiRPEEeo6BFp13oylpLeVEJlwcfLx/ewPxFdB4P1HTvFPhqPW7rw7a6bBMx8pZdrbl6bs7R1NeZ/G/wAO2J8b+HrkKY21WQW91sON6h1Gfrhv0rb+M0CWNv4T01zJb+GhdeVeiLIUIuwAHH+zvo5pdwPTI9C8OXsfmR6dp8yH+JY1YVXbwb4YuBn+ybQg90GP/Qa8n8AyQWvizxrbeHJpZvDMVizw4YsglwMBSf8AgVcRH4jRfhPpelW+qONTfWmkkiSVg6x7cc98ZIp88+4HuOs+EvAmnS28F6q2lxeSCKBFnffI2QAFGT/KszUvh/4Tt9Vt9LOtSWuoXQ3QQSOpaTHoMDPeuX+JmjXWpfGHwxY22rXFtNcQK0UmNwtipPzKuep2/wAqPG7azN8bNNh0V4JdQ03S94e5+7na5Zj785pqtUXUDeu/g7eLzaarFJ7SxFf5ZrLfwb410Y7rNpmVen2af+ldv8KfF2oeM/Ckl/qUca3EN01uWj4VwFU5x/wKoviv40v/AAX4cgudNiQ3FxP5ImkGViGMkkdz2rVYqot9R3ONTxx400R9t+srAfw3cGP/AB7iug034wwsVXUtOeP1eBt3/jp/xp3gzxhrmq642ia/Z2d9byRedb6pYqWt5eM7c4xnB/DHNbF34d8Fa5q1xpkaWg1KFN0sdq+141yBlgOB17in7WlL4o2C5saX4z0HVyq22oxrK3/LKU7G/I9fwreDBhlSCD3FeTar8IZk3PpWoK47Qzrg/gw/wrAF7408GSYlN1HCp5Ev7yIj69Pyp+wpz/hy+8ND3uivMdE+LdrOVi1i2Nux/wCW0R3L+I6j8M16DY6lZ6lAs1ncxzRsMhkbNc86U4boLF2iiioEFFFFABRRRQAUUUUAFFFZOua/Y+H7Frq+l2r0RR95z6AUJNuyA0pJUijLyOEVRkknAFedeJfina2bNa6Mq3U4+UzN9wfT+9XHav4k17x3qIsLKNxbt923jJxj1c9/5V2/hb4Z2OmKl1qwW7uvvCM/6tD9P4q61ShSXNU+4ZxFpofirx1cC6uZJDAek1w2EX/dUdfwr0PQvhroukhZbqM31wP4ph8n/fPT867RUVFCqoUDoAK5bx54rk8JeE7zV7a2+1zQlYwm7hGbjLe1ZyxEpaR0QXOpjjSJAkaKijoFGBUE19bW9zBBNPGk052xIW5c8k4H4V534O8bat468CXosJ4LXxNbAxusifLu/hbHYH36EHNefW3iu+1X4jeC7fXoWg1/TLyS0vAy7RIrY2MPzP8A+qsBHZeKvi/e6W+oPo+jR3Fnp8whuLy6m8tXfOCsa9WxzyPyrE+J2u3OraZ4O1201K8s9H1MiK8igmIADY3Zx3C7h+FaviPwJ4r1zx/qExWxm0e6t/s8U9w277GjABzHHn/Wfe5P96up0b4aaTZ+EbTw5qkj6tbWtwbiLzxt2tzwAO3J6+tAHBeB9HXQ/HXjHwKjSmwu7Rnt95JGGXH54b/x2s/S/h54o1L4aaPYf2cbTUtO1ZriP7Sdn7thkn8wK+gI7eGIkpEikgAkLyQOnNTYHpQBwNj8Png8f6z4hlu0Nrqtn9mmtlQg5IUMd3/AT+dZlp8ENDj07+z7zVNVvLFJfNgtnm2pE3qABycV6jiloAwm8KaQ2vWetyWpfUbOLyYZ2c5VcEfQ/eNbtJ3zS0AZWsW+jeSL/WLazeOz/eLPcxK3k+4JHB6dKeBpniHS1Zo7a/sLhcrvQOkg+h9683+MutfuLLw9ExDXDfaLgA/8s1zgfi3/AKDUnwb1nfZ32gSv81q4mgB/55v1H4N/OtPZvk5x2PSbDSdO0u1Ntp9hbWkBOTHBCqKfwArDb4eeEWBz4fsFLSiYlItp3+vH8q6mk4rMRy3ibwDoPiy+tb3UoZPtVrxFLDIUIGc4OOtQTeArKXxXqXiRLq4W/vrM2pBwyRgqF3KPoPWuwxS4oA5TwF4QXwR4aXSBdC6/evKZvL2bi3tk+1cx8U5Nbgu9Pk/s1tW8LyLs1KzSFXYEHO4fxA4PUeleo0YoA8G+D9vdWuveI57KLULPwsIiYhdcMrdsA/xAbufzpvwN0bUZL/VPFKXx/s95JIHjm+aSbGCrF/bP6V7vLCksDQugaNl2suOCPSuAn+F2n2XhXXdH8P3NzZnVBnEkpKRtnPHGQD0oAZafFMRamlpr+gX2kQT3H2e3u5SHikbPHzL0/Ue9ehSRxyoUkVXUjlWGc186x/DDWYfFHhXTrzRIYLSGQPdXlrO8qzFOSzbsBSdvT3rZfVvF/jL4qaxL4R1FLW00mMW+ZyTC55ByvQknd9NtAHfa78NNF1VXktENjcH+KEfIfqvT8q86vvD3ifwRdNd20kqwg5+0W7ZQj/aX/GvUn8c6DpusW/h7VNYt11oxr5i7GVCxHr0GfTPeumYLIhDAMp7HkVvDESjpLVDueZ+G/itFOyW2uIIX7XMY+Q/Udvr0r0qC5iuYllgkWSNxlWU5BFcH4o+GVjqQe70nbaXf3in/ACzc/T+GuC0vXte8Cam9pPFIIlP7y1lztb3B7fUcVq6VOquanv2Dc9/orE8PeJrDxJYi4s5PnHEkTH5kPvW5XG04uzEFFFFABSUdqqahfwaZYz3l1IEhhUsxNCTbsgM7xL4ktPDWmtdXB3SHiKIHl27fhXjdtb638RPEBd3+X+N+dkCegpl1can8QfFipHkByVjU9IY++f8APNe3aFoVnoGmR2VomFUfM56ufU12aYeP95j2IvD/AIbsPDtkLezj+Y8ySt99z6mtrAo4pa45ScndiKt5FLcWU8MNw0EsiFUmUAlDjhgDXyrBD4l0W98UaPNJJdzFHXUrORixuIyP9chPVl+Vv/rZx9aVxXiHwHDrPi/RvElvdvZXlg+2VkXJuI+oX07kfQn0oA8v+F2k6reX2h+KNCMSptaw1mORioOzGG92KlfxFdp4j8H6t4j+KmkamtjbWum6WyyPe7/3lzyCFx7Yx+P4V6PZ2Fpp9uILO2it4QS2yNAoyepwKtUAFFFFABRRRQAVS1TUI9K0q6v5kkeO3jMjJGuWIA6CrtNKgjBAIPBzQB5YPjhpkke+HRNRf6tGBn67jTG+NkP8Hh27b/enQVr+J/hbpWsl7vTMaZqDcl4xmNz/ALSdPxFeQ6zouqeHNQWy1a2Eby5MUsZyko747110IUp6PcasJrOrT+IPEF7q9yhje4YLHEXDeXGOFXj86f4f1p/DfiWy1dEd44iyTxRjLNGw5/WqFFen7CPJydCj15vjXo+35NH1dj7xxj/2eoJfjfpsabv7E1ADqd7xr/7NXl1hY3+rX4sdLtJLq6OCVQfKgPdm/hFet+EvhVZaaY77XGS/vh8yxgfuYvoP4j7mvMr06VPRO7JdjudC1ZNd0S01OKGWFLiMOI5Rhl+taVNChQAAAB0Ap1cggooooAKTFLRQAmBzx1rL07QdN0Y3baZZw2jXT+bKY0wGbHXFatJQB8w+I5LxfFSx67Yt/bWoTrYahaxxHy7u3+UJNE38LDGOO+OOor6Q0qyGm6VaWImkm+zwrF5khy7bRjJ96tmGNnVzGpZTlSRyKfQAYHpWL4h8N2HiOy+z3ifOOY5VHzIfUVt0lCk4u6A+er+w1rwB4hWRHKlTujnUZSRPQ/4V7D4T8V23ibThKn7u5TiaInlT6j2NX9e0Oz1/TXsrtAQeUfujeorwsHVPAfivA4mhbBz92eM/0P6V3XjiI6/Eh7n0TS1naPq1vrWlwX9q2Y5Vz7qe4NaNcLunZiCvJPizr7NJBocDEKAJZ8f+Or/M/lXrDMFUsTwBmvnyMP4r+IWHGUubzn2jB/8AiRXThYpycn0Gj0v4a+G10jQ1vpo8Xd6A5z1VP4V/r+Nd1imJGqIqqAABgAdqkrCpNzk5MQUUUVIBSYFFLQAUUmaM0ALRRRQAUUUUAFFJmjNABgda+ffiRqw1fx3cIjZg09BbJ6F/vOfzIFe+XDypayvDH5kioSiZ+8ccCvB/D3w18Sa/cyXGr+ZpkMsrSTSSAGaRmOW2jt9TW1CUYz5pdBo5OJJrq6S0tLeW6upPuxQrls/SkkEtvcvbXUMltdJ96GddrD8DX0h4f8LaT4ZtPJ021SNmH7yU8vIfVm6/hS6/4V0jxLbeTqdmkhH3JQMSJ/ut1FdP1+XN5Bc8h+FOsDS/GMmnysFg1KLCg/8APVeR+Yz+le8V4fqfws8Q6Lq9neaBOl/HDcLJGZWEckOD37MP19q9uQtsG/72Oa5a8oynzR6gx9FJmlrIQUUUUAFFFFABRSfjRQAtFFFABRRRQAlcL8SvDi6voRvoE/0uzBcYH30/iH9fwruqa6B0KsAQRzmqhNwkpIDxv4Ua+1rqkmjTufJuQXiB7OOo/H+lez184ajC3hfxnKkWV+x3QeP3XIYfzr6Jt5luLeOZT8siBgfYiujFxSamuo2VdZlNvol9Mv3kgdh/3ya8Y+F0Qm8aozDJSCRxn8B/Wvbb6EXWn3EH/PSNl/MV4h8NpfsfjuOJ/lLJJDz69f5inQ/hTsCPeaKKK5BBSUtFAHFat4yvND8RLY3emSPZyDMdxEc/hium0/VLTVLcTWc6yL3A6r7EdjSajpdrqto1vdRh0PTHVT6g9q4PU9GvtBn+0mS5kjHCX9qP30Y9JV6OtXo0c/vwbvqjoPGevXGlWsFtYsBd3LbVY/wL3NcKda8QabKZodXmuSp+aO4+ZW+npTtW1O+1C6026mSO6jhLJ9stT8rbum5TypqlqM0cG5ncAA9KynNpqMNzaFJSi51PkeqeF/EEfiHSlulXZIDtkT+6a3a4j4caRcafos1zco0b3cvmiM9VWu3q3uKF7ahTHkWNGdjhVBJJ9BT6guYBcW0sJON6Fc/WkWtzzTWfiBeXl09vo7rBCjbfNZcu59hVrw/40vEvY7fVphLBIdon2bSjf7XbmuPvdJl0XVZrWRSrKTtz0ceoq3boAMOnzsPmx0rz6mIqRqa7H1Ucvws8OnBatbntQIZQQcg+lOxXD+GvE8cGkGHULhXkhcxoEO93H0FWbvxPeFN0SR2cJbAknO52/wB1R3/Gu3njbQ+dnhqkZOLWx1Us0UKGSWRY0A5ZjgUkNxFcRCSGVJEPRkbIrizoF34ijP2xp1hf70lyQXI/2EHC/jVSbw/eeHVH2aOd7ePhbiybbIg/206MK1ilIXso2tzanohIHamPIkcbO7BVUZJPYVxNj4m1VAGU2+q2w6vH+7mX/eXp/Kq3ifxba32mLp9vK8FzcSeXIki7So/iFPkd7BDDznJRSINb8aajePKujyrBbRnb5pTcz/QVBonxIubWdLXWtsqE7TOo2svuy9/wqiYVht9qLhVGOe4rEh0abW9Vjs7WLdJJy7Hjy17k1vFQas0fQLA4aOHfP06+Z7tFKk0ayRkMjAMpHcGparWlstpaRW6fciQIPwqzXK/I+Ze4lYfijxDF4b0h72RTJIWEcMQ/jc9BW52rhfibpV5f6Lb3FnGZTZzebJGOpXHJ96ukk5pPYlq+hzMWr+IdXm8+fWZ7MscrHbbQkf8AvZ613Hg/XbjVrOe2viv26zk8qUqMBx1VvxFef6PPFcbHjkBV/wBD9Km0zUtUsdU1fULeKK0trgqourvOwbf7qjlmrrnBSTS+R04ihGEYuHzPU9R1Wy0m1M99cpCnbceW+gHX8K57QvGU3iDxBJaWmmTR2ESHfdS8ZbsAvaszTPDlxrEv226e5WJx81zc4+0Sj/YXpEv05ruLKwtdOtlt7WFYo16BR1965nyQT6s5dWXKKKKyKCiiigDwf4pQrF41ldePMhjY4+mP6V6/4WczeFNKdicm1j6/7orxv4m3AuPG9wq8+UkcYx64yf1Ne06Hbmz8P6dbsMNHbxqfqFArsxGlGA2adeDeJ7eTwr8Q/tcYxGZluouMZUnLL+h/Ovea4n4j+G21vRDc26ZvLPLqB1dMcr/X8Kyw01GdnswR19pdR3lpFcwsGjlQMpHfNWK8x+FvidZrZtCunxNCN0Ge6f3fqP616dWdWDhJoQUUUVACYFBAI5GaWigDzTxfYWema9ZTWUXlTXRbzgnRh6kVy1wn2PUUvrMKl2W2rmPeH/4D3/Cup8Uz/bPGJQcrawAfj1/rWbow3+NNJVuhldz9djVEtaitukOCSjJPZmvonxOtpCINajFrJnAnjyYz9c8qfrXfW9zDdxLNBKskbDIZDkGsPW/BWia8WlubUJcMP9dCdrfjjr+NcO3gzxb4TuftHhy/F5bA828h2nH0PB/CtdGZJOOm56yTgVnalrenaQm6+vIouPuluT+HWuFuF+IWtqI2ij09COdjhf15ptl8MLiRhJqepFnP3vLGT/30f8KycpXskelTw1FLmq1F6LVi+IPE+m69GIbfT2kdf9XcTfuyvuP4v0rFtYJWh8m5fzS3UgYrqtf8IWFh4ameBpd9uA4ZpD2PT0rHsBsVSK8/Eqad31PbwVSkqL9j3LHh7QJr6N208w2cCOUaXGZDj0H+Ndtpvh6x01vOCmW5I+aeU7m/+t+FZHgWYLb3tofvxzlwPY111d1KCjFHg4utUlUkm+ouKMUtFanIYmpeHNP1CTzijQXIHyzwHa34+v41xut6Jf6dEGvUg1Cy3BfNI2yLk9x3/CvSu3vXJ+PJv+JZbWacvPcLx/srya0hJ3sdOGrThUST3Zx+pRTPbrDbP5TKOoGcVe0HxJYeF7fyLuxKs5zJcxNvLn1YHBouCkdu3lIScZJqx4e8I2Wt+HEu7p50lmdzlJOBhiBweKtNW12PdxMqXskq21+h2WmeINM1hd1jeRSnuobkfh1rUBBrzG/+FtwCsmnakqOn3N6bW/76H+FJbx/ETQvkVU1CIdAXDf4Gl7OL+Fnj1MNRa5qU16Pc9LnuYraJpZpVjjX7zMwAFcDrfxSsLd2g0hReSfd85zthB+vVj9KxT4M8YeMLgT+I74Wdtn5bdeSP+Ajj8zXa6H4D0HQikkNr59wvSe4+dvw7CrUaVP4ndnCnqecWCQ6tqB1W4ET3DHGY4/LVf+A/1611/hG2s7/xFqsl1Cs1zZyIIWkOfLVh2B75HWsWfaPGmtqnCCcHj+9tFanh6Q2Pj5kziO+tePd17flmtJu8dOx11Heimu56PijFLRXEcgUUUUAFV7u5itLWW4mcJFGpZmPYCrFeYfFPxMILT+wrWTMs2DcEfwr/AHfx/pV0oOckgOJ0aCXxb48R5EJWe4M8o/uoDn+gFfQSrhQPSvP/AIYeGW0zTG1O5TbcXY+QEcrH/iTXoVa4qalLljshsWkIB6ilornEeO+O/CtzoOpr4g0YMkIk3uIxkwv6/Q13Hg7xfb+J9PAJWO/jX99Dn/x4exrpZYo5omilVXRwQysMgj0NeR+J/BmoeGNQ/t3w68ghVt7RpyYvw7rXVGUa0eSe/RjPYaK4rwj4+tPECJa3RW21FeDGx4f/AHf8OtdpmuacJQdpCCmtwuSadVLVGnTS7praMyT+S3loOrNjiktxPY80DfaLzU7/ALzXDqp/2QeKq2UwtfEelXLnCrcAE+gIx/Wuh03wXqcuiwreXospwMmGJA4B/wBonqfpXK6/p99pT/Zr1AshO6GaP7smOmPQ+1ZyUubmXf8AA0pyXJy7aHtdGKyPDmrrreh2t8p+Z0+cejVr1oZp3DFGM0tFAzF8UEL4bv8A3iIrh7KPNug/ixXYeMJhHohi7zyLGPxPNcxAmycbvugVxYq0mkz2sufLRb7staLKdN8SxlziO8TYf94dK76uB1Oza6tVe1f/AEiE+ZHj29667R9QXU9MhuRwxGHX+63cV0UpXgrnn4uP7zm7mjRRRWpyiVwutS/2l4r8ocw2UWCP9pq63U7+PTdPlupSNqDgf3j2Fclp9lNDAbi4+e5uH82UYxjPargranRhl7930Ksse1WTHBU5zW74DYt4UtieoZx/4+ayLkb5CxGB061qeBD5eiS2xILQ3Dg/QncP503sehjNaF/M6vFFFFZnjiU1mwCScAd6dXPeM9WGjeFr25DbZWTZF/vHgU4xbkkhN2VzzyyuBe61q16nKT3jlPdQeK0tRf7Fc6Vq2Cv2S4G8j+63BrE8N2l9cpHYaZCsk6jM87nEcPrn1b2rrNZ8H61/YksNpfpeu65eCaMIGP8AssPu/jXbPljKzZ1TqxVDk62O/UhlDKcg9DTu1Zmhfahodkt7GYrlYVEqk5w2K1K4WrM5U7oKSjNcX4u8f2fh+Nra2ZLnUDwqA/Knu3+HWnCMpu0Rlrxj4vg8M2DbWEl9Iv7qLPT/AGj7CvPPBfhW68Vau+tavue1Em5mkGPOb0+lS+G/B+peMNSOs67JKtq7byWHzTegX+6tew29tDaW8dvbxrFFGu1EUYA/CuqU40Y8sPi6sZMqhVAAAA6AU6iiuQQUUUUAGKQgEYIzS0UAed+KfhtBfu1/ozC0vQd2wcIx9ePun6cVkaR4+1bw3c/2Z4otZmVTjziPnUev+0K9arP1TRdP1q2+z39qkydiw5X6HtW0aya5Zq6HcdpurWGr2ouLC7jnjIzlT0+o7fjV6vK7/wCHeraHcm/8LahLlTnyWfax9s9D+OKfp/xNv9MuBZeJ9OkjkHBlRNp+pXv9RxTdHm1pu6/ED1DArP1jSLbWtOks7pAUccHup9R6GotK8Q6XrUe6xvI5T3TOGH1BrV6jisbOL1QmjzjwD9t8P6zqHhrUeoPnWz4+WRe+PevR/eq8tlbzXEM8kSNNET5b45X8as05O7uZwi4ppi0UUVJocF44vgL61tskrCvmkLyWY8AVZ0Tw29zai41hSS/3LfcQEX/a9TUlnoNzeeML3VdSjxDEQtqh74/irrcelQ6acrs6niWqSpw+Zz0+hNYAT6Rw68m2dyUcegz0rM0TUorDWJIixS3vJCDE4wYZu6n6121c34l8NDWLZ5bSQQ3qj5X7N6BqtJXMVO6akdJnjIpM8c9q5zwzq11NG2narE8OpW4+cN0kH95T3FR+MNbudOs47PTonm1G8ykIUfd9zVKLbsZ3V9zN1zVra+1URySb7KzfPlpyZ5uyj6Vfs9CudU/0nWSY0b/V2cTlVUf7XqaZ4V8Jf2TCl1qDCe/wct2jz1x7+9dbgYxVyklpE0crK0Tj9Z8OS2kf2vSFyF/1loWyJP8Ad9DVHwXqCDW7q3Vj5dyglVW4KuvDD/PpXelQT9RXE3/he7tPGFlrWlBWid9t1FnGAerClGSaszWFe9Jwn8juaKQUtZnMJXl3xD+2+IvEGneGNNGWBE879oh0yfoO1eoVWjsbaK7mu0hRZ5QBJIF+ZgOmTV058kubqTK7tYpeH9BtfD+lx2VqMgcvIert/eNa2MUe9ZWq+ItK0VC9/fRREfwZyx/4COal80nfdlGrxVHUtWsdJtTcX12kEYGcs3J+g7/hXnWp/FC81Cc2fhvT5HkY4EkiFm/75HT8agsPh7rev3X23xNfSIGO7y925/p6LW0aFtajsvxHYbrfxC1XX7k6Z4Yt5lDnHmqP3jD1/wBkVp+FvhnFayLfa8RcXJO4QZ3ID/tH+Ku20fQNN0K38nT7VIh3bqzfU1qdqJVklywVkFxqqqKFUAKBgADpT6KKwEFFFFABRRRQAUUUUAFFFFABVLUNMsdTt/IvbWKeM9pFBx9Ku0lF2tgPOdU+FFjI5n0e7mspRyqk7lH9azw/xE8L8Mo1S2X/ALa/4NXq34UVqq8tpajueb2XxZtA4h1bTrm0k7lBuA+o4P6V1Vh4x0DUv+PfVLcOf4JG2N+TYrQvtK0/UYyl5ZwTg/30Brl7/wCF3h27yYYpbVv+mUhI/I070pdLBodmsqOMqwP0OafmvMG+GWr6eSdH8QyRgfdR9yfqpP8AKkFv8TdL4S4ivUHYlH/mAaPZRfwyA9QxRXmA8aeNrHi+8NtIB1McL/zBIp6/FmSHi90C4jPfa/8AiopPDz9fmFj02kwK88j+L2jH/W2N+n/AVb/2arS/Ffw6fvfa0+sP/wBel7Gp2Cx3GxSc4GfWkMaFgxRSw6EjmuNHxS8Nf895x/2xNB+KXhof8t5/+/Jo9lU7C5TtMClrhW+K/hxfu/a2+kX/ANeqsnxf0Zf9XZXz/wDAVH/s1Co1Ow7HofFGBXmT/Ft5eLPQLiQ9sv8A4KajPjbxtfcWPhtoweheFz+pIFUsPPrp8wseo0xpEQZdgo9zivMDD8TtU4eaOyQ9gUT+WTSD4Z61qJ3az4hZwfvIm5//AEIgUexivikB2t/4x0DTeLjVICw/gjbefyGa5PUPi3aBjHpenz3T9mcbQfoOtaNj8K/D1oM3Cz3bf9NJCB+S11Nho2m6YoWysoIfdEGfzp/uY7K4aHmpuPiH4p4jj/s21foceUPz+8fwrQ0z4TWoYTazfS3ch6pGdoP1Y8n9K9K/CjFJ15bRVguUNM0fT9IgENhaRQL32Lyfqa0KKKxbb1YgooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooATA9Ka0Ubj5kVvqKfRRcClJpOnS/6ywtn/3olNVW8M6G/LaRZn/tiK16KfNLuBhnwh4dbrotl/35FH/CIeHR00Wy/wC/Ircop+0l3AyF8MaEn3dIsx/2xFWY9H02L/V6far/ALsSj+lXqKOaXcCNIY0HyRov0XFSYFFFSAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAf/9k=</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
           <t>Finance &amp; Accounting</t>
@@ -2706,7 +2770,11 @@
           <t>MHAA</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEAYABgAAD/4QA6RXhpZgAATU0AKgAAAAgAA1EQAAEAAAABAQAAAFERAAQAAAABAAAOxFESAAQAAAABAAAOxAAAAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCADnANMDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD5/ooooAKKKKACiiigAooq/pOmtqF2qkMIVIMjD09B70m7K5dOnKpJQirtnbeGvhtB4kvJLOC9EVwqb1WWbb5g74+Q9K6v/hni+/5/Yv8AwI/+11z9pdz2N3DdW0hjmhcOjjsRX0H4P8UQeJtGW4Xal1H8txCD91vUex7VjRq86s9z081y14SfND4H+HkeO/8ADO99/wA/sX/gR/8Aa65jxN8Lf+EXuIIbydm85CytHMCODgjlBX1YThTXm3xftTNo9neqmTbzmNz6KwP9VH51pUbUW0cOEjTnXhCps3Y+f/8AhFrL/nrP/wB9j/4mj/hFrL/nrP8A99j/AOJrdorh+sVO59h/YWC7P72SeGPhO3ik3H2OZkWDbuaWYDOc+iH0rov+GeL7/n9i/wDAj/7XXo3wjsjB4Xnuz/y83LbT/sqAv8w1ehHmu+Dbimz47FRhGtKNPZN2Pnf/AIZ4vv8An9i/8CP/ALXXK+JfhrB4bvY7Oe9Ek7JvYRTbtg7Z+Qda+j/F/ieDwxorXB2yXMmUt4ifvN6n2HU189Xd3Pe3kt3cSGSeVy7uepNZV6vIrLc78qy54ufNP4F+PkeX0Voavp0lheP8v7l2JjYdMelZ9bJ3PMqU5U5OElZoKKKKZAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB1GgaRZ3Fgt1PF5jliOW4HOOldBHHHDH5ccaxqP4VFdT8KvBVn4o+Hl3IW8i+ju3WKcDI+6vDDuP1rM1zw/qPh69+zahAUJzsccpIPVT3+nWuHEQne+6PrMkxWF5VTsoz79/n+hl1seG/EN14a1mO/twXUfLLFuwJE7j6+hrHp0aNI4VASx6AVzwclJcu57mKp0qlGUavw9fLz+R9MWOqW2p6ZDf284a3lTcGPGPXPoRXIeOvEWmal4evNJtpDcXMgXa0a5RWDAjLHjt2zXA6dDdWumNaPdTfZpG8x7cNhN2PTv/KrR2sMfdr6zDZVKpHmraX6H4xj88hQquGE96z+Lp8kc/HoUxi3SSIjegBb/AAofQZRHuSVGb0II/wAa6S3tpLy6hgX70rhR7Zpbm1ezvJ7cnPlOVzjriuj+ycDfk5dfVk/63Z5/G9rpftG3psdj4L8RaPpug2WkzyG1mhTDGVcIzEkkhhx1J64rrb/VbXT9Mmv7iYLbxJvLAZyO2PUntXjm9NuCM1U1OO9udNSziupPssb7xblvkz7en8qwxWVyhFyo626Dy/O4Vqqhi/du/i6fNGX4l8Q3PiXWZL+4yqfdhiJyI07D69z7/hWPSspVipGCOCKSvkptuTctz9pwtKlSoxjS+H8/MHjSWPbKgZfQisHXdMtI9KaaKJI3hI27FAyCQOe5/Guy0TQdR8QXwtbC3LkYLueEjHqx7fzpPjD4Rt/CmiaGiyNNdzyS+fKeAcBcADsOfrXRh4TvfZHhZ1isLyunZSn+Xz/Q8ioooruPkwooooAKKKKACiiigAooooAKKKKACiiigD6c/Z3/AOREu/8Ar/b/ANBWvTdU0ix1eya0v7aOeFuqsOh9Qex968h+Aet6ZYeEriyu72GC4kvGdElfbuGFHGfcV7arq6hlIKnoQaB6o8F8V/Dy+0INdWQe80/PLAZki/3gOo9x+NZOiWa7GuXwd33fpXvmu332DQ726QDckR25/vHgfqa8YgjWOFI1GI0GBXoZVgoSrOs1t+ZwcQZ9iVglgub4t31sunzYuMtxWpp+h6jqkRks7YSoDgkSKMH6E1l5w3y1e0vVLnSbxbm2l2kcMhHDj0NfQ1vacr9na/mfDUPZe0Xtr8vludV4V8M31lrQur+ARpGhKfOrZY8dj6Zpni/w/d3GtfarK1eZZUBfYOjDj+WK7XS7wanp9vd7Gj81A2xu1N1W9Gl6bPeFGk8tc7V/z0r5tY2v9Y57e9tY+veWYb6n7O75fiv1/LseTXWk3tjFvu7VoUJwC7AZ+lUAdrcVf1HUptWvGubqTJ6Kg6IPQVQ6txX0tHn5f3m/kfH1vZc7VK/L5mRrtkFQXSkDPDf41s+Efh3fa/tu70PZ6eTwxGHlH+yD0Hufwpk0e+N8fdI9K9n0a8GoaJZ3Zx+9iUnAxz3/AFr5zNsFCNdVkvi/M+74fz7EvBPB83w9etn0+RLpekWWkWi2lhbJBCv8KjqfUnqT9a8a/aV/48fDv/XSf+SV7lJIkMZeR1RByWY4Ar58/aD1rTtUt9EhsbyK4eB5TJ5TbguQuORx2NcB3as8MooooEFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAdr4c/5AkYPQu2fzrp9M8Qavo4VdP1C4gjU5EavlP8Avk8fpXL+HCP7Fj5H32/nWtkeo/OvNquUajsfc4KlQq4OmqqT06ncf8J/rGuWn9l3wt2R2DGVFKtgc4I6H9KT/V7TXL6Lg6rDhh1P4/Ka6b7w+lfX5E3LDNve7/Q/JuNaVOjmfs6XwqK/G4nU1Pa2xub6G2A/1jhfzqDo1PRnWRZI2ZHXkMpwRXsTu07HyUGlJOWx6HrfiaHSYBp+nlWmjUJu6rEAMfiaXRvEcOtW76bf7VmlQoD/AAyAj9D7V5wX4yzfUk0Kw4dH5ByCDXmf2ZS9ny/a79bns/21X9t7R/Bty9Lf5+Y+VGt7mWF/vRuVP4Gm0hZnYsxLMTkk9TS16avbU8SVr6CY4pF+IGt6RZLpNkbeKOAsBLs3OdxLd+Bjdjoaf9zbXJ6kR/a93yP9YO/+yteLnzccPFx3v+jPsuCKVOtmMqdVXjyt/c0SalrOpav/AMhG+nuRnO2VyVH/AAHp+lcl4r/48rb/AK6H+Vb+R6j865/xVj7Hb8j/AFh/lXydFydRNn6nmdOhSwNSNJJbbeqOVooor0T4kKKKKACiiigAooooAKKKKACiiigAr03VPh0ll8LbfVlQ/wBpoBdT/wDXNv4fwBB/OsLwL4Zs/EyatFcSNHPbwLLA+flBBJOfbAr127i1TUNGtra7KQ2WrqLaSE8m1Vh8pBxyxAIOehYenPj47GShWhCnK1neXmrXt91/mvQ6KVO8W2t9iX4A6bZXfge6kubSCZxeuA0kYYgbV9RXrH9h6T/0DLP/AL8L/hXEfCPTrbSdI1qxs1b7PBqbpGWOSwCIM16P2r04SUoKceupg1Z2PNPiFaWWnafpctvZRRubsqTDEqk5jfjtxmuW+xajs/5Bl1/3yv8AjXa/EqIHT9LRuQbtsg9/3T1yEXia706ELcwrdQghRIZNjJk4+Yngj3rqqYjMsNhfa4GMZJN3T32Wq1R4mJoYCvi/ZYtuLaVmtt3psV/smp48v+y7z/vlf8aZJBeW8XmT2FzFGCAXdRgZOBnmujk1fVP7TW2FrZWryJviknuGcSeoACjkcHGe9OjM+oJfaRq/kmXYGDwKVVkboQCTyGB/SvEhxfmEbSqwhy6N2ve19ba2O6XDGBaag5X/AF+4f4D06yvdQvLi8SOWeBVEKNztU9Wx65GM9vxqLxxYWVhrFrLZrHFJcRsZokGAcEYbHY8ke+PasLTxdaZ4k06GV2juVuYlLISBIjOFJHqD3FJLHPqviC7jR2e4klfzJSc+WgYgE/QDgV9S8RQVX677ReztzX8trHkeyqvBfU/Z+/flt573+4iit725iWSCxuZIm+66qMH6c082Wp7Nn9m3Z99o/wAa6SeW5tpbTS9HMCvHF5kjXCllWMcDoRyT/I1DBrGrG/mtzaWdz5ChpZobkqqE/wAJyp5xz16V8rLi7MZXlThC26ve9r6X1sevHhjApJScr/r9xhmx1ER5OmXf/fK/411fw4s7HUdF1G4msoZXN+wBmiUtgRx+tcvL4ivNYtNsUAtbVwQSH3O49iOADXZ/DOMHRNSVDhRqDAD/ALZx17sK+Y4jCqpj4xjdqyW+z1erOPCUMDRxcqeEbk0ndvbdabHXf2HpP/QMs/8Avwv+FeIftE2NpZ2Ogm2tYYS0s27y4wueF9K99615f8VdEsvEOseHtOv1YxS/aQGU4KsFUg/pXJOrGEHUlslc9qMXJ2R5Brfw5TT/AIaWeuRhxfRqJbtSc5VyMcdsZH6mvNq+hr5tWvPCNzJI8L2lyhsvKXhY4z+7E2cZ65JHoR6V5B490O08OeJP7Ls9xSGCPczdWYjJJ/OvOy3FTqOUKsk5XbVui0uvk3Y1rU1GzjscxRRRXrGAUUUUAFFFFABRRRQAUUUUAegfDLiDxE6OBKLLCpnlxyWAHfgV7Nq1zbS2dnDDLGzNcQMAGHyqCHLH0G1Sa8f+GCW0um+Ixc5zFDHLCynDI4LYKnsSdo9+hr0d/C1npv8AYc8oLsZRBeY484vyM/7IcAbemOOgr5bMlSli7zbTT00391P+vU9ChzKnp/Wp1nwsnhuNP1ySCQSRnVJMOOh+Va9B715x8JJjcafr05GPM1iYj6YGP0xXo/evpKStTin2Rwy+JnBfE0/6HpQ9bpv/AEW9eflQ6srAFTwQa7/4mn/RdIHHNy3/AKLauCH3Gr6nKf8Ad36/5Hxef6Ytei/NkGoM/wC5t5r25k0oPiaFNrFVxjK5BIwcHj8K1reCC1niMWsSSzIP+JddTz7o3U4zC+O/HfnoRyDVD7vDLUUVjJqFw8VnpwufJxJcbVBManoQP4m44ArxM1yGjVftKc1TXVWVn5+vR90ehlOeV4pUJQdR9HfU3L7WbK7vdNtLmMW+qRahbsIXwSR5i5KMOGH+SKj0jWLO3imsrCJLjUpLmZ5I1woX942Gkbtx+PoKzWtbfTvFn9n7FeW0urfMnlFM5ZT3pljYRarqgtAipNMJpQ3kGQnbzjj1z3NeW+HKP1T2Htfd+K9nbta172v5/M9dZzU9r/C96/La67XvfYu3Fpa3Us3m61Miuc6lcxTbUc4IESfTPbsPU1lwCSe2ltRdXK6czHyoH2p8nbdtA6+/4046fLZXCW95p62s7J5sQ2j5kP8AFjsexB6Gpz12EfPXrZTkVGg/aVJe0XTRWXn69PJaHj5vnleX7mEXTfXXX/hhVUBNqgBQMADtXf8Awu/5Aup/9hFv/Rcdef8A8FegfC7/AJAup/8AYRb/ANFx162b/wAGPr+hxcPf7xP0/VHc1578QJoIfFHhVp5ViUvcAMxwM7VxXoXavOPiJt/4SrwjHIivFNLcxOjLkMCg4I/KvlMWr4Wp/hf5H2dL416mXDcWsfgWW3lZBJHZvG8efmBGV6f71eL/ABSwfGRbzUkY2sO/ac7WC4IPvkV6f/wjcMvhq51W3aQXZna5jdvmZY1+UJk9flGQT0bB7V5p8VoLW18UWsFnGqQpYRYx3yWOSe5OeteJlKoxxMuRtt81/La/9dTsxHN7NX8jhqKKK+lOAKKKKACiiigAooooAKKKKAPQfhvHKtnrDbMLOsaQuWwGlRvM8sf7RA4r1W98TWWp3NjbWyzN5c0d0fkx5igEqEz94luP+At6V5x8Nwtx4U1eweMSC8vILdQwyFL5y31Cgn8K9Wu7GKz8Q6LPbxouFks8BRwmwsMfQp+tfKZlOksRJzWqvb5RX/Dep6NBS9mu3/BND4RxPDo2rpIgjcalJlA27b8q8Z716N2rzX4MytP4Z1CZzlnvmZj77VzXpNfUQTUUmee9zgfiX/qtH4/5eHP/AJDNcCv8Vd58S/u6OM/8t5P/AEA1wg719NlP8B+v+R8XxD/vS/wr82OB8tq4bWtb1bwv4oe+0y9ltvtMCxvsP3lHUc9+4Pau2PI3Vn61oVtrNjsnBV15R16qa6MbQdelyx33ObK8XHC4hTns9GSabeWt1HaXNowffcRO7E5YtvBO49c/Wq1zqltZ6RHeTuYpUG+J0bDh+209c1wGnrLovim3s4b0yoLmMSmNSFOGGQR7VFa2Uuva59iub0xYJEfmKeg6AD6V5X1yTnyqGtuW3Tc9/wDs2EYc7qPlT5r63tY6Xw1rWreJPEk+p6reSXMiQeWGfoo3DAA6Dua7U8S5qnpmkW+l2Cx264A5Zz1c+pq5/wAs8162DoOhRUJbnz+Z4uOKxDqR22E/5Z16D8Lv+QJqf/YRf/0XHXn3/LOvQfhb/wAgXU/+wi//AKLjrkzf+FH1/Q7uHv8AeJ+n6o7gV5z8Rt6+JPCkqQNMYpZ3KKQGICr0z1PfFejCvOfiTKyeJ/B+08tdyL+BCg18tX/3ef8Ahf5H2NP416nO23iWxstDm0keZJcRK0ceEO1y7ERjPYnPQ9Np9K8l+JmZNetZ0XdbC0S3jnA+WUx/KxU9wDxn2r2i10a01XSdaM0SFtTuJd529Nh2L+WzP1NeS/FG6S7i8PSRxiNfsZG1RgKQQCB9CDXg5VKksTJU073d/W1/zTO3EKXs9TzyiiivpjgCiiigAooooAKKKKACiiigD034fXD2HhLULt42jijvEmjuQpZfMjAPlsByMhuD05r0NNU1bU9bjE1gtvc2cTTW6MxZFWReJJCO4GV2juT25rjvhqC3gG4hLYjuNahhf/dPl5H49Pxr0jVoyviPSXiOGnSe2kA/iXZuH5FR+dfK5lWgsRJSir+9r6RX5q6f6Ho0IvkWvYX4EtJJ4LupJSC73rOSBxyqmvU68u+BoMfgu6ibhorxo2+qooP8q9Q3CvqVtoeceffEw/Pow/6ayH/xyuEHQ13PxLYGbRgP+ekv/oNcP619LlP8B+v+R8bxD/vS/wAK/NiCmzBmjcDPKkDHrilor03qjw07O5554Ra3gtNUinG26UhssOSoPI/A9ab4sMb3ujJbYa6CDfsHzdRtz79aXxmlnb63DJaOVu3OZ1Ucc9z7mrHgWK1uLy6uLh2e/RvkWQdF6ZHv29q+bUW6n1XTtf53+8+2lOKpfXte9vVKP3dTvx0paKK+kPhSMfdr0H4X/wDIE1P/ALCLf+i468+H3a9B+F//ACBNT/7CLf8AouOvJzf+FH1/Q+h4e/3iXp+qO8ryj4uvPFrng17Z40m+3MqmQZXkoOfzr1bIryz4sRGfxB4LhX7zX5P4KUY/oK+ZnZQnfaz/ACPs4fEjEfX9S0q41KFLAyRQ7rq5BbBgL/3eMMpOXyOcE8ZFea/EtVWz0FIonFvFC8cc7jb9oPylmCnkDJ74617NpVutzbatNN8z3N1Msmeyr8gX6YX9a8k+Kkz3GieEZnOS1pJ+P3Ofxr5vL6kHi0oxs72fryv/AIPy89Turxfs7t/1c8zooor6k88KKKKACiiigAooooAKKKKAPSPh1eXLeGteskQSwxbboqrYkjYDIkXPBwUHGc16DHc67cappNxeGGJ9Rtyts4X5bQlQzj/acgDGeOteW/DPedQ1xEBJfSJxgfVa9v1bbJodlLDhtk9q8RH++oyPwJ/OvmM1tTxEVyr3nv2ukvz+9K3c76GtO99v8zlfhIuo38mo6W2qXtlbJNNc5ttgeZ94VtzFT0+Xpjqa6fwraR+JNt3qVw8lpM8iRwy6hN5wZQDzhtr/ACnJwBisnw1aeGkuvEsWrytHHY6kzpJHPJGcTYJT5CCwynT2qvBqt3b+INUfwtpFrC8blbWJ7dvMlAQsdqscjeACWwO3XmvpITU4RmuqRxSVm0WNSlBsLO2SUywWup3sMD7948sYKgN3ADY/CqH/ACyat3WtK1e20eJr4ySW9tcRPG8iRqymVGEi4TjAcr+vWsIf6tq+mylr2DXn/kfGcQRaxSfkvzY6mMTgkDJA4HvT6ZXqHgI848PiCeTWJb/P28I+0ScEcHdgetTeIzDbeJdNmsCBeEgSrGc88AZ9yM5q34psYb3Wxb2qpFdJH500mcZUdsdzT/CthbWOrX1lcBJb6H5lnyTlT7Hoea+fVOXP7DTf4vx+8+0lVh7P63rt8Pk0l93U7YdKWiivoD4kUfw11fgPVodL0W4WRJJJbvWDbwxxjJZjEhP0ACsT9K5E/dWu78NaJptz4BVtUg3wyySXjYJVlIJ2sCpyDtA6V5GcNezivM+k4di/bTl5fqUr+5Ou3t7qukeJL6ztRLDYLIsO6Hzd4zj6HCk4xk9TVf4qxTyeJPBMcE7QzG7mCyqASvyrzg8UaNYudVs9OltrjSdF1B/t1pZK6OHdNrbWONyZwHK85556in+OriK5+JXh2yJHmWlrcXSjPVmG0D9DXy2MnyYepLsn+R9lTV5pHLT6jrltpusalAsa2hm8iZUXdukyEeaP26fKe+ea85+J+ozz61aaZLCIV0+3VFiDbtu4A8noTjb0r19wkXw1YMAu+x6ersP5ljXi3xP3f8LB1EN1Cw/+ikNeJldVVMS4qKXLzfhypfmdWITUN97fqchRRRX0hwhRRRQAUUUUAFFFFABRRRQB1Xw6vLm08ZWqWs8UL3CtDmYEo2RkK2OxIFeswabrdzZ6isUz2s2m3G23so5PMiwFDcEgHPzZXP3eB2rwOyuXs763uozh4ZVkXPqDmvqLTrmO2v8AVvtEiRq7JdBmOBsMaqT+BU18/nM5UZKcEm2u3Zr9H/kdeFSk7MyvBt1ZWPxIjtbMBbHUdOjaHd1ZhuIJzzu4fOec10Hjy/XS9e0Sa4maxsZS8U99CAkiE42jfg4HcjjP6HgdQnmmnOsaM8Mh0K4kusod29GkJ2jHbCMT7NXsUmoT614Yt9R0QW80kyxzRpP911yCy57HGRnsa9LA1FOik946Pv5X9UZVo2nfuVEkt/GPgaT7HMXW4hKI7kFg6ngtjgHIBx2ry+FmNuPMRo5FJV0Ycqw4IPuDxXQTeModDu9UdRa2mo3twkLQRgzRWhXarSTFMDPzjp6AZzWbfwXNxaL4gIhaKeRluGiUopYMVE6qeQj4B56H619BlmJVKpyy2Z89neCdeiqkFrH8irRSA5pa+lPiDmPFlosnlXFuWXUASkQX/lop+8G9gO/vT/DNqFN1czO51GR9tyHGCh9APStO5tTJei5xlkgeNf8AeJB/kKW1sng1O+uCOZ1jwfcZB/pXAqP7/wBpb+rb+vQ9t4r/AGT2N+n6rT06+pdoooJGCSQMckk13njEiw3E8kOnWylp7pxFHjsT1P0AyT9K9R1xLnSvC8dppTMsitDbo6gFlQuqsyjuQuT+FYHgHQ3Zv7evVK7l22kbLghT1c/XoPb61keJNUj1zVpjcaVLNYzW7WenTMNyLP5vllz2TLEKCeeM4xXy+PxKrVfd2R93k+DeHoXmvelq/wBDo/DunxyeJ9RuhfXepR2KiC2uLmQv5TnPmqvQE8Lk/h2rgtY1BdT8ceKLlVd3s44LSyaL7wn3NtA/4FnPtnNei3upT+C/h0tzfyCW9tbRY89fMmIwB78/nXm2hsPD01jZavcQRTvMb2Z5GC/6yNgM56kMpB+or5/MKvLQajq309NX/l8z3MPG87sszaXrFnqOlWKypeq6NcSJcSFYYZEIIZVAyQN3C+2a8O8UXs2oeKNRuJ5vOkM7KZNu3cF+UcZOOAK+g/E9+1ub+4hkAex0yZ2bspbG0fX5Sfyr5lrkyVyqQ9rNK9l+Lb/KxeKSjLlQUUUV7hyhRRRQAUUUUAFFFFABRRRQAV6j4K1C48R6FLo76pIL6xXzbWF41O9F52h/vYOMEe9eXVZ06/uNL1G3vrSQxzwOHRh2IrGvS9pG3Var1KjLldz6bNpb6hZxa1o6xRXUsYkRsbVmUj7kgHUdvUGqOheKLXwgn2SKOW4tdQiN1ptr/HHIWAeHP90E59sN14rBj+IGmWWitq2mXNvtlzK2mXJKOj9/LYA5BOeMY9xQdHu5rO4/4SRVg3usmn6hZndHa8lhk8Ect1Iwa+dwPtcHJzq3Ub2s92u1uvLo9PO252VeWqrR3/r8zp7rwnf6LrEWrzyWM/2m4UC1CEK08rNkFjyIwzBu5yo6cVcsrJbW/wBf1PxIkAm0+bzpJbVWcTQNF/q8MOV/2fUfjVrw/rsfiGzk8LeKYkXVkQZG7C3SDlZYyO/GeOQRUeo+HVbWJ7Gf+1RL5SJpF6rySpAdpyXIPXd13dRgV9NCcZxUou6ZxNNOzMu98KyPbR6x4dR7nT7hBKtowxLGp/u56geh59M1gGaPzWiCGOVTho3BVh+B5r0G38atbR2lxqdiLXSbo+Va3qybjI4B6xgZUNg4wT2q1rl34d1Pw62qSWkGpwqypGFAD+YXCBQTgqdxAPTFeph8yqUlyy1R4mNyahXlzwfK/wAPuPNwA3RP1pCcdVrurLwTpmpWgle11DTJQxV4DMGwQex5yPQ96vxfDnQYx++F3P6iS4YA/guK7Xm9O2kWeWuHa99Zq3zPNkfdMsMKtLM33Yo1LMfwFdd4b8DTXMkd9rkQjjHzpZZBJPbzCOP+Aj8fSumiuPC3hm5i0uGXT7C4kXckAKq7+/qehrnta8baiNLtrqxsZrS3nkWSK5nAbz4QCzAKCSrFRlc9QDyDXBicxqVlyrRHrYLJqGHfNL3pf10H+O/FQ09f7JtWH72NkuTE+yWJSMDZngHng9MgA4yDSeDdAS6t4bq5mSextZS9gsUhCyH/AJ6Sp3kB9ehz7GsKGz12Oz0/WtUihvPDmnQbljZ8TSQMjKzOjL94K2SNxzjiqs6NpF/eWHhnWH8u5iEk8pbEdjCyj5n/AL0u0YXocdema8ypKFODnN2SPZScnZGp4n1eHX9XkFvMlxa6RcpDDAD8kt43AZj3VM9u+fSmanp0WnaNdySBLnVrtPIW4kQFnkf5VA9FBPQdAK5u4ju9GtodS0GyRNF0+Lzp/tjFGumXdh14Jydx5OM8VS1fx/Yx6Wupvf282ohT9js7UFlgdhjexIG5gM8HH9a+axMa+JrqrT1jfbqu0Xbbu/XXVJHdDkpws9/61OV+IepNplvD4YtdXe6jjAa7URqo38YDMOWP1PpXndOkkeWRpHYs7EliepNNr6OhS9nBRbu+r7vucUpczuFFFFakhRRRQAUUUUAFFFFABRRRQAUUUUAdh4I8YjQbj7BqEEdxpNy2JldASmeMj29q9y0XUbcWq6XfSoSkf7iWQjZcwH7rKTwTjgjr+dfLtdr4Y8aTRWSaDq12i6WQVjmkthM1vn0z2/PFeRmWXLELmhv1/wA15+XX1SN6NZw0O+ubez1S9t40vp7ZbRJv7N1NkdEU7kKLvPDY+devQV2+gfEK4sZY9J8YxraXRwsV+p/cTg9DnoD/AJ4rF8Kva6HaRaO12LvTZhvsbtgNsm7loz2Bzkgdwfao/E1rDZJNo8Fu91DfW0ksNmsRfy5EwQV7BSSAR249TXDQx0qdf2MVePS/VdX5Puu/Y6KlFSjzdT0TUNMtLSzXVrFYX/s+FpLaKSQ/Z0HJZwFB+baWAPNeWa4LxLHX726gNxa3k8S3ctsGCW28LLjb1YcRK3TnPTNSwq+nI1tpOoXWm210DG2lavCxt3DDBVW/hz7Gk0/WtR07wze6Ff6BfOUvVluriCUTOw3q+cHBKlV2g89Oa9qjjKNRfFZ9np/w/wAjllRnE0ZvFmsaFpOi2mnTm1hWGXIubeSQtEG2rKNw3BQoZgp5wBknvsx63D4m1DUp5dSv20GxgSfNvG8Th2GNuU5bgBgB/e56Cr1p8UfDd9IiNZagLgqQEazLNjuOM/lVdvij4Z0xGt7DSdQY7yDDb2YT5vpkc11cytczsULDw54ruIkJaIQ6hMtzNczkCdAoVUV1KnOFXOBjlvY51rvwFp+lWV7eWmpXEEyR5tjdTjyoGUhlycAkAqByTgEgVmXXxC8Q3d1Ba6Z4aFp5sZlM2oTACJBxuZV6ewzmuX1QS6/b3E2pXuo+ILgowigsoGjtI2xgHsGx65NctXGUYfau/LX73svmzSNGbN6+8f6j4o086foVvFa7k232pTsGghB4IQnhzWBokenWupSafLNcNYS3/mG5ljYpdv5aBQZCMH595xnqK6HR7ey1CWV3BFrpri3htHiKLGVUHewI5Y5+gHvWL4slsNfh8y51D+z9Hsm3i52BlnmHZQfvKoz26n2rxJ5hPEVnSkmo+XRvbpdvtbbp3OqNFU48y3NbxBq9nOrQPKh022YTahPkFAq8rED0LMcZHYdeteE+L/Flx4p1Hf5SW9lEcW9uigBR6n1NWfFnjK51yNNOt5FTS4TlI44REHI6EgE1ydejl2XRw0U2tenl5+r/AAWnc5q1Z1GFFFFeqYhRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB0Phrxhf+GvOhijhurKf/AF1pcLuRvceh969D8P6z4d1PUrXULfVv7N1aJdkFrKzmH/dZnJLA8Zxj9K8borlrYSFS7T5W97dfVbP8/MqM3HY+qW1eGS0aHU9NukYriSPyDKh45wyggj8q5Pw/q1tqMt1cyatqKXETPFFHDDgvAGOwgFSW47nnrXjdh4n1m0WOD+178WS4VoFuGK7M8gKTitpvH7zXRW501JNOYbGtRMykr0BLDG5seuR6AV5MMn9jGUY637f5Pv6/M6niuZps9Lv7m/u1KLFdXmmxkPcvcrEJ0RSCTHsO7OM9ga6PTdMu7qxhmF2dOgkUNFa2UaAIp6ZYg5OOuK8U1vxdozaUtn4f026tJM4M08uSi+i4PX3JrS034j6bDokdpe6dfGWNAmy2vGSJ8e2fl/Cs6+XVpUUqcba7WX32vYca0FLVncaxfWemeIbO1bU7y9hu5hHfq0fmrhVOyPKjgliPl785rq59ZcwGLTrGbeBgSTxGKGIerE46eg/SvEl+KN+8H9ntZ29tpTZBhto13KD3BYHJzg/h+NczqfibXNWgS3v9UubiFRwjPwfrjr+NN5POryKpZcvnv52SWvS19rai+tct+U7/AFPxF4Z0Oe6mt7yTX7q4m8yZJN0aM3c5U4xnHykHj6VwPiLxNqHia8S4viirEuyGGJdqRr6AVjUV7dLDQpvmesu7/RbL5HLKbluFFFFdBIUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFAH//Z</t>
+        </is>
+      </c>
       <c r="N26" t="inlineStr">
         <is>
           <t>Healthcare &amp; Medicine</t>
@@ -2782,7 +2850,11 @@
           <t>MHAA</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEAYABgAAD/4QA6RXhpZgAATU0AKgAAAAgAA1EQAAEAAAABAQAAAFERAAQAAAABAAAOxFESAAQAAAABAAAOxAAAAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCADnANMDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD5/ooooAKKKKACiiigAooq/pOnPqF2oIIhQgyNjoP8aTdi6dOVSShFXbO28NfDaDxJeSWcF6IrhU3qss23zB3x8h6V1f8Awzxff8/sX/gR/wDa65+0u57G7huraQxzQuHRx2Ir6D8H+KIPE2jrcLtS6j+W4hB+63qPY9qxo1edWe56ea5a8JPmh8D/AA8jx3/hni+/5/Yv/Aj/AO11zPib4W/8IvcQQ3k7N5yFlaOYEcHBHKCvqsnCGvNvjBambRrO8VMmCcxufRWB/qo/OtKjai2jiwkac68IVNm7Hz//AMItZf8APWf/AL7H/wATR/wi1l/z1n/77H/xNbtFcP1ip3Pr/wCwsF2f3sk8MfCdvFJuPsczIsG3c0swGc59EPpXRf8ADPF9/wA/sX/gR/8Aa69G+EdkYPC892f+Xm5baf8AZUBf5hq9C613wbcU2fHYqMI1pRp7Jux87/8ADPF9/wA/sX/gR/8Aa65XxL8NYPDd7HZz3oknZN7CKbdsHbPyDrX0d4v8TweGNGNwdslzJlLeIn7zep9h1NfPd3dz3t5Ld3Ehknlcu7nqTWVeryKy3O/KsueLnzT+Bfj5Hl9FaGr6dJYXjjb+5diY2HTHpWfWyd1dHmVKcqcnCSs0FFFFMgKKKKACiiigAooooAKKKKACiiigAooooA6fQdJs57BbqePzJCxADNx1x0roUijhTZEioo/hVa6n4VeCrPxT8PLqQt5F9HeOsU4GR91eGHcfrWZrnh/UfD179m1CAoTnY45SQeqnv9OtcOIhO990fWZJisKoqnZRn37/AD/Qy62PDXiG68N6zHf24LqPlli3YEidx9fQ1j06NGkcKgJY9AK54OSkuXc9zFU6VSjKNX4evl5/I+mLHVLbUtMhv7eYNbypuDHj659CK5Dx34i0zUvD15pNtIbi5kC7GjXKKwYEZY8du2a4HTorq101rV7qb7NI3mPbhsJux6d/5VZ3KV6ba+sw2VSqR5q2l+h+M4/PIUKrhhPes/i6fJGBHoUxi3SSIjegBb/Ch9BlEe5JUZvQgj/Gukt7aW8uoYF+9K4Ue2aLq1ks7yeAnJicrnHXFdH9k4G/Jy6+rI/1uzz+N7XS/aNvTY7LwX4j0jTdAsdJnkNrNCmGMq4RmJJJDDjqT1xXW3+q2unaZNfzzBbeJN5Yc5HbHqT2rxzcirgjdVPVI72501LSG6k+yxvvFuW+TPt6fyrDFZXKEXKjrboPL88hWqqGL927+Lp80ZniXxDc+JdZkv7jKp92GInIjTsPr3Pv+FY9KylWKkYI4IpK+Sm25Ny3P2nC0qVKjGNL4fz8xHRZI9kqqy+jCsLXdMtE0ppookjeEjbsUDIJA57n8a7LRNB1HxBfC1sLcuRgu54SMerHt/Om/GDwjb+FNE0JFkaa7nkl8+U8A4C4AHYc/WujDwne+yPCzvFYXldOylP8vn+h5HRRRXcfJhRRRQAUUUUAFFFFABRRRQAUUUUAFFFFAH05+zt/yIt5/wBf7f8AoK16bqmkWOr2TWl/bRzwt1Vh0PqD2PvXkHwD1vTLDwpcWV3ewwXEl4zokr7dwwo4z7ivbldXUMpBU9CDQPVHg3iv4e32hBrqyD3mn55YDMkX+8B1HuPxrJ0OzXY1w+Du+79K9612++waFe3aAbkiO3P948D9TXjMEaxwpGoxHGMCvQyrBQlWdZrb8zg4gz7ErBLBc3xbvrZdPmx2MtxWlp+h6jqkZls7USoDgkSKMH6E1m5w3FXdL1S50m8W5tptpHDIRw49DX0Nf2nK/Z2v5nw1D2XtF7a/L5bnVeFfDN9Y60Lq/gEaRoSnzq2WPHY+maZ4u8P3dzrX2qytXmWVAX2Dow4/liu10u8Gpadb3exo/NQNsbtTdVvhpemT3hRpPLXO1e//ANavm1ja/wBY57e9tY+veW4X6n7O75fiv1/LseTXelXtjFvu7VoUJwC7AZ+lUA21uKvahqU2rXjXN1Jk9FQdEHoKo9T8tfS0ufl/e7+R8dW9lztUr8vmZOt2QVFuVIGeG/xrY8I/Du+1/bd3oe008nhiMPKP9kHoPc/hTJo98b4+6R6V7Po14NQ0Szuzj97EpOBjnv8ArXzmbYKEa6rJfF+Z95w/n2JeCeD5vh69bPp8iXS9IsdItFtbC2SCFf4VHU+pPUn614z+0p/x5eHf+uk/8kr3OSRIYy8jqiDksxwBXz7+0JrWm6pBokNjeRXDwPL5vlNuC5C45HHY1wHdqzwuiiigQUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB2nhz/kCID0Ltn866jTPEGr6OFXT9QuII1ORGr5T/vk8fpXL+HCP7FTkffb+da2R6j8682o5RqOx9zgqVCrg6aqpPTqdx/wn+sa5af2XfC3ZHYMZUUq2Bzgjof0pv+r2muY0XB1SHDDqfx+U10vUV9fkTcsM297v9D8m40pU6OZ+zpfCor8bh1NT2tsbm+htgP8AWOF/OoOjU9GdZFkjZkdeQynBFexO7TsfJQaUk5bHoeueJodJgGn6eytNGoTd1WIAY/E0ujeI4datm06/2pNKhTP8MgI/Q+1ecFu7N9STQrDh0fkHIINeZ/ZlL2fL9rv1uez/AG1X9t7R/Bty9Lf5+Y+RGt7iWF/vRuVP4GimEs7FmJZicknqafXqK9tTxJWvoMxxSL8QNa0iyXSbI28UcBYCXZuc7iW78DG7HQ0/7gWuT1Ij+17vkf6wd/8AZWvEz5uOHi473/Rn2XBFKnWzGVOqrx5W/uaJNS1nUtX/AOQjfT3IznbK5Kj/AID0/SuS8Wf8edv/ANdD/Kt/I9R+dc/4qI+x2/I/1h/lXylFydRNn6nmdOhSwNSNJJbbeqOVooor0D4kKKKKACiiigAooooAKKKKACiiigAr03VPh0ll8LbbVljP9pqBdT/9cz/D+AIP4GsLwL4Ys/EyatFcO0c9vAssEgPCnJzn24r1u8j1TUNGtoLsrDZauotpIeptVYfKQccsQCDnoWHpz4+OxkoVoQpytZ3l5q17fdf5r0OinSvFtrfYsfADTbK78D3UlzaQTOL1wGkjDEDavqK9X/sPSf8AoGWf/fhf8K4j4R6fbaTpGs2FmrC3g1N40LnJOEQZr0bPFepTlGUVJddTBqzsea/EK0stO0/S5YLKKNzdlSYYlUnMb8duM1y32LUdn/IMuv8Avlf8a7T4lRA6fpaNyDdtkHv+6euSi8TXenQBbmFbqEEKJDJsZMnHzE8Ee9dNTEZlhsL7XAxjJJu6e+y1WqPExNDAV8X7LFtxbSs1tu9Nit9k1Tbs/sy8/wC+V/xpkkF5bxeZPYXMUYIBd1GBk4Gea6OTV9U/tRbUWtlavIm+KSe4ZxJ6gAKORwcZ706Mz6gl9pGr+SZdgYPApVWRuhAJPIYH9K8OHF2YRtKrCHLo3a97X1trY7pcMYFpqDlf9fuH+A9Osr3ULy4vEjlngVRCjc7VPVseuRjPb8ai8cWFnYaxay2axxSXEbGaJBgHBGGx2PJHvj2rCsBdaX4l06GV2juVuYlLISBIjOFJHqD3FJKk+reILuNHZ7iSV/MlJz5aBiAT9AOBX1LxFBVfrvtF7O3Nfy2seR7Kq8F9T9n79+W3nvf7iKK3vbmJZILG5kib7rqowfpzT2stU27P7Nuz77R/jXSTy3NtLaaXpBgV44vMka4UsqxjgdCOSf5GoYNY1U381ubOzufIUNLNDclVQn+E5U84569K+WlxdmMrypwhbdXve19L62PXjwxgUkpOV/1+4wzZaiI8nTLr/vlf8a6v4cWdjqOi6jcTWUMrm/YAzRKWwI4/WuXl8RXmsWm2KAWtq4IJD7ncexHABrs/hnGDompKvCjUGAH/AGzjr3YV8yr4VVMfGMbtWS32er1Zx4ShgaOLlTwjcmk7t7brTY67+w9J/wCgZZ/9+F/wrw/9oixtLOx0E21rDCWlm3eXGFzwvpXvteYfFXRLLxDq3h3Tr9XMUn2kBlOCrBVIP6VyTqxhB1JbJXPajFydkeQa78OY9O+GdlrcYcX0arLdAn7yuRgY7bcj9TXm1fQ982rXvhG4kkeF7S5Q2XlLwscZ/dibOM9ckj0I9K8f8eaHaeHPEn9l2ZYpDBHuZurMRkk/nXnZbip1HKnVleV21botNPk3Y1rU1GzjscxRRRXrGAUUUUAFFFFABRRRQAUUUUAegfDL5YPETo4EossKmeXHJYAd+BXs2r3NtLZ2cMMsbM1zAwAYfKoIcsfQbVJrx/4YJay6b4jFyDuihilhdThkcFgNp7EkqPfpXo7+FrPTf7DnlBdjKILzHHnF+Rn/AGQ4A29McdBXy2ZKlLF3m2mnppv7qf8AXqehQ5lT0/rU6z4WTw3Gn65JBIJIzqkmHHQ/Kteg/wAVec/CWY3Gm69ORjzNXmI+mBj9MV6N3r6WkrU4p9kcMviZwXxMP+h6UPW7b/0W9eflQ6srAFTwQa7/AOJp/wBF0gcc3Lf+i2rgh/q2r6jKf93fr/kfFZ/pi16L82Q3rNiGCe9uZNKD4mhTaxVcYyuQSMHB4/CtS3ggtZ4jFrEksyD/AIl11PPujdTjML478d+ehHINUT8vDDNQxWEmo3DxWenC58nElxtUExqehA/ibjgCvFzbIaNV+0pzVNdVZWfn69H3R6OU55XilRlB1H0d9TdvtYsru9020uYxb6pFqFuwhfBJHmLkow4Yf5IqPSNZs7eKaysIkuNSkuZnkjXChf3jYaRu3H4+grNe2t9P8Wf2fsV5bS6t8yeUUzllPemWOnxarqgtBGqTTCaUN5BkJ28449c9zXlvhyj9U9h7X3fivZ27Wte9r+fzPXWcVPa/wvevy2uu1732Ltxa2t1LN5utTIrnOpXMU21HOCBEn0z27D1NZcAkntpbUXVyunMx8qB9qfJ23bQOvv8AjTjp81lcJb3enrazsnmxDaPmQ/xY7HsQehqc9dhHz16uU5FRoP2lSXtF00Vl5+vTyWh4+b55Xl+5hF03111/4YFChNqgBQMADtXf/C7/AJAup/8AYRb/ANFx1wH8Nd/8Lv8AkC6n/wBhFv8A0XHXrZv/AAY+v6HHw/8A7xP0/VHdV578QJoIfFHhVp5ViUvcAMxwM7VxXoXavOPiJt/4SrwjHIivFNLcxOjLkMCg4I/KvlMWr4Wp/hf5H2VL416mXDcWsfgWW3lZBJHaPG8efmBGV6f71eLfFHB8YlvNSRjaw7ypzhguCD75Feof8I3DL4audVt2kF2Z2uY3b5mWNflCZPX5RkE9Gwe1ea/FaC1tvFNrDZxqkK2EWMd8ljknuTnrXiZSqMcTLkbbfNfy2v8A11OzEc3s1fyOFooor6U4AooooAKKKKACiiigAooooA9B+G8cq2erttws6xpE5OA0qN5nl9PvEDivVb3xNZanc2NtbLM3lzR3R+THmKASoTP3iW4/4C3pXnHw3AuPCmr2DxiQXl5BbqGGQpfOW+oUE/hXq13YxWfiHRZ7eNFwslmQFHCbCwx9Cn618pmU6SxEnNaq9vlFf8N6no0FL2a7f8E0PhHE8OjaukiCNxqUmUDbtvyrxnvXotebfBmVp/DOoTOcs98zMffaua9Jr6mCaikzz3ucD8S/9Vo4x/y8Of8AyGa4Id67v4l/d0cZ/wCW8n/oBrhB3r6XKf4D9f8AI+L4h/3pf4V+bFB2NXD61rWr+GPFLX2m3stt9pgWN9h+8o6jnv3B7V255G6s7W9DtdZstk4KsOUdeqmujG0HXpcsd9zmyrFxwuIUp7PRj9NvbW6S1ubRg++4id2JyxbeCdx65+tVrnVLaz0iK8nkMUiDfG6Nhw/baeua4GwWbRfFVvZwXplRbmMSlAQpwwyCPaobWyl13XPsVxeGHBIj8xT0HQAfSvK+uSc+VQ1ty26bn0H9mwjDndR8qfNfW9rHT+Gdb1bxJ4kuNS1W8kuZEt9gZ+ijcMADoO5rtDxLmqemaRBpdgsVuuAOWc9XPqau/wAGa9bB0HQoqEtz57M8XHFYh1I7bCf8s69A+Fv/ACBNT/7CL/8AouOvP/8AlnXoHwt/5Amp/wDYRf8A9Fx1yZv/AAo+v6Hbw7/Hn6fqjuBXnHxH3jxJ4UlSBpjFLO5RSAxAVemep74r0cV5z8SJWTxP4O2nlruRfwIUGvlq/wDu8/8AC/yPsqfxr1OdtvEtjZaHNpI8yS4iVo48Idrl2IjGexOeh6bT6V5J8S8ya7azIu62FolvFOPuymP5WKnuAeM+1e022i2mq6TrRmiQtqdxLvO3psOxfy2Z+pryX4o3SXcPh2SOMRr9jI2qMBSCAQPoQa8HKp0liJRpp3u7+tr/AJpnbiFL2ep55RRRX0xwBRRRQAUUUUAFFFFABRRRQB6Z8Prg2PhPULuSNo44rxJ4rkKWXzIwD5bAcjIbg9Oa9ETVNW1LW4xNp629zZxNNbozFkVZF4kkI7gZXaO5PbmuN+GwLeAbiEtiO41qGF/90+Xkfj0/GvStWjK+I9JeI4adJ7aQD+Jdm4fkVH518pmdaCryUoq/va+kV+aun+h30IvlWvYPgS0kngu6klILves5IHHKqa9Try34GAx+C7qJuGivGjb6qig/yr1HcK+qW2hwHn3xLPOjD/prIf8AxyuFHeu4+JbDzdGA/wCekv8A6DXDjvX0mU/wH6/5HxnEP+9L/CvzYgpswLRuFzypAx64paK9R6o8ROzueeeEnt4LTVIpxtu1Ktlh8xUHkfgetN8VlXvdGS1Aa8CLv2D5u23Pv1pfGSWltrkMloxW7c5mVRxz3PuaseBYrSe7u7i4dnvkb5FkHRemR79vavm1Fup9V07X+d/vPtpTiqX1/Xvb1Sj93U78dKWiivpD4UZ/BXoHwu/5Amp/9hFv/Rcdef8A8FegfC7/AJAmp/8AYRb/ANFx15Ob/wAKPr+h9Fw9/vEvT9Ud5XlHxde4j1zwa9s8aTfbmVTIMryUHP516tkV5Z8WIjceIPBcK/ea/J/BSjH9BXzM7KEubaz/ACPsofEjEfX9S0q41KFLEyRQ7rq5BbBgL/3eMMpOXyOcE8ZFea/EtVWz0FIopBbxQvHHPINv2g/KWYKeQMnvjrXs2lW63Ntq003zPc3UyyZ7KvyBfphf1ryT4qTPcaJ4Rmc5LWkn4/c5/Gvm8vqQeLSjGzvZ+vK/+D8vPU7q8X7O7f8AVzzOiiivqTzwooooAKKKKACiiigAooooA9I+HV3ct4a16zjQSxRbLoqrASRsORIueDgoOM5r0CO51241TSbi8MMT6jblbZwvy2hKhnH+05AGM8da8u+GYdtQ1xEBJbSJuB/vJXt2q7ZNDsZYQG2T2rxEf76jI/An86+YzVqniEuVe89+14pfn96Vu530Nad77f5nL/CVdRv21HS21S9srZJprnNtsDzPvCtuYqeny9MdTXTeFbSPxJtu9SuHktJnkSOGXUJvODKAecNtf5Tk4AxWT4atPDKXXiWLV5WjjsdSZ0kjnkjOJsEp8hBYZTp7VXg1W7t/EGqP4W0i1heNytrE9u3mSgIWO1WORvABLYHbrzX0lOanBTXVI4pKzaLGpSg2FnbJKZYLXU72GB9+8eWMFQG7gBsfhVD+Bq3da0nV7bSImvjJJb21xE8byJGrKZUYSLhOMByv69awh91q+mylr2DXn/kfF5/FrFJ+S/NiGgkgMQMkDge9Bor1DwkeceHxbzvrEuoZ+37G2rJwRwd2B61N4jMFt4m06awI+2EjzVQ554Az7kZzVzxTYQ3ut/Z7UJFdJH500mcZUdsdzTvClhbWOq31lchJb6HDLPknKn2PQ818+qcuf2Gm/wAX4/efZyrQ9n9b12+HyaS+7qdsOlLRRX0B8SKP4a6vwHq0OlaLcLIkkkt3rBt4Y4xksxiQn6ABWJ+lcifurXd+G9E0258AK+qQb4ZZJLxsEqykE7WBU5B2gdK8jOGvZxXmfScOxftpy8v1KWoXJ128vdV0jxLfWdqJYbBZFh3Q+bvGcfQ4UnGMnqarfFWKeTxJ4JjguHhmN3MFlUAlflXnB4p2jWLnVbPTpba40nRdQf7daWSujh3Ta21jjcmcByvOeeeop3jq4iufiV4dsiR5lpa3F0oz1ZhtA/Q18ti58mHqS7J/kfZU1eaRy0+o65babrGpQLGtoZvImVF3bpMhHmj9unynvnmvOfifqU1xrdppssIhXT7ZY1jDbtoYBhk9CcbelewSBIvhowYBd9j09XYfzLGvFPidu/4WDqQbqFhH/kJK8TK6kamJa5UuXm/DlS/BnViE1Dfe36nI0UUV9IcIUUUUAFFFFABRRRQAUUUUAdV8O7y5tPGVqlrcRQvcK0OZlJRsjIVgOxIFeswabrlzZ6isUz202nXG23so5PMiwFDcEgHPzZXP3eB2rwKzuHtL2C5jOHhkWRT7g5r6j0+5jtr/AFY3EiRq7JdBmOBsMaqT+BU18/nM5UZKcEm2u3Zr9H/kdeFSk7MyvBt1Y2PxHjtbMBbHUdOjaHd1ZhuIJzzu4fOec10Hjy/XS9e0Wa4maxsZS8U99CAkiE42jfg4HcjjP6HgdQuJprj+2NFeGQ6FcSXWUO7ejSE7RjthGJ9mr2KTUJ9Z8MW+o6ILeaSZY5o45vuuuQWXPY4yM9jXpYGop0UnvHR9/K/qjKtG079ypHJb+MPA0n2OZnW4hKI7kFg6ngtjgHIBx2ry+FmMH7xGjkUlXRhyrDgg+4PFdBN4yh0O81R1Fraaje3CQtBGDNFaFdqtJMUwM/OOnoBnNZt/Bc3FouvkQtFPIy3DRKUUsGKidVPIR8A89D9a+gyzEqlU5ZbM+ezvBOvRVSC1j+RVopAc0tfSnxBzHiy0WQRXFuSuoqSkQX+NT94N7Ad/en+GbVVN1czOx1CR9txvGCh9APStO5tTJei5xlkgeNf94kH+QpbWzeDU764I5nWPB9xkH+lcCo/v/aW/q2/r0PbeK/2T2N+n6rT06+pdoooJGCSQMckk13njEiw3E8kOn2ylp7pxEmOxPU/QDJP0r1HXUudK8Lx2mlMyyK0NujqAWVC6qzKO5C5P4VgeAdDdm/t69UruXbaRsuCFPVz9eg9vrWR4k1SPXNWmNxpUs1jNbtZ6dMw3Is/m+WXPZMsQoJ54zjFfL4/EqtV93ZH3eT4N4ehea96Wr/Q6Pw7p8cnifUboX13qUdiogtri5kL+U5z5qr0BPC5P4dq4LV79dT8c+KLlVd3s44LSyaL7wn3NtA/4FnPtnNei3upT+C/h0tzfyCW9tbRY89fMmIwB78/nXm2hsPD09jZavcQRTvMb6Z5GC/6yNgM56kMpB+or5/MKvLQajq309NX/AJfM9zDxvO7LM2l6xZ6jpVisqXqujXEiXEhWGGRCCGVQMkDdwvtmvDvFF7LqPifUbmebzpDOymTbt3BflBxk44Ar6D8T37W51C5hkAksdMmdm7KWxtH1+Un8q+Za5MlcqkPazSvZfi2/ysXikoy5UFFFFe4coUUUUAFFFFABRRRQAUUUUAFeoeC7+48SaDLpD6nIL+xXzbaJo1O+Nedof72OMEe9eX1Z06/uNL1G3vrWQxzwOHRh2IrGvRVWNuq1XqVGXK7n02bS31Czi1rR1iiupYxIjY2rMpH3JAOo7eoNUdC8UWvhBPskUctxa6hEbrTbX+OOQsA8Of7oJz7YbrxWCnj/AE2x0VtV0y5tytxmZ9MuSUdHz82xgDkE54xj3FB0e7ms7j/hJVWDe6yafqFmd0dryWGTwRy3UjBr53A+1wc3OrdRvaz3a7W68uj087bnZV5aqtHf+vzOnuvCd/ousRavPJYz/abhQLUIQrTys2QWPIjDMG7nKjpxVyysltb/AF/U/EiQCbT5vOkltVZxNA0X+rww5X/Z9R+NWvD+ux+IbOTwt4piRdWRBkbsLdIOVljI78Z45BFR6j4dVtYnsZ/7VEvlImkXqvJKkB2nJcg9d3Xd1GBX00JxnFSi7pnE007My77wpI9rHrHh5HudPuEEq2rDEsan+7nqB6Hn0zWAZY/NaIKYpVOGjcFWH4HmvQbfxq1tHaXGp2ItdJuj5VrerJuMjgHrGBlQ2DjBParOuXfh3U/DrapJaQanCrKkYUAP5hcIFBOCp3EA9MV6mHzGpSXLLVHiY3JqFeXPB8r/AA+483AD/wAH60E7eq13Vl4J0zUrQSva6hpkoYq8BmDYIPY85Hoe9X4vhzoMY/fC7n9RJcMAfwXFdrzenbSLPLXDte+s1b5nmqSbplhhVppm+7FGpZj+ArrvDfgaa5kjvtcjEcY+dLLIJJ7eYRx/wEfj6V08Vx4W8M3MWmQy6fYXEi7kgBVXf39T0Nc7rnjbURpVtdWNjNaW88iyRXM4DefCAWYBQSVYqMrnqAeQa4MTmNSsuVaI9bBZPQwz5pe9L+uhJ478VDT1/sm1YfvY2S5MT7JYlIwNmeAeeD0yADjINJ4N0BLq3hurmZJ7G1lL2CxSELIf+ekqd5AfXoc+xrCis9djs7DWtUihvPDunQbljZ8TSQMjKzOjL94K2SNxzjiqtwraTf3lh4Z1h/LuYhJPKWxHYwso+Z/70u0YXocdema8yc4U4Oc3ZI9lJydkanifWIdf1aT7PMlxa6RcpDDAD8kt43AZj3VM9u+fSo9T06LTtGu5JAlzqt0nkLcSICzyP8qgeignoOgFc5cR3WjW0OpaDYomi6fF50/2xijXTLuw68E5O48nGeKpav4/sE0oam+oW8+oBT9jsrXLLA7DG9iQNzAZ4OP6183iY18TXVWnrG+3Vdou23d+uuqSO6HJThZ7/wBanK/EPUTpkEPhm01d7tIwDdhY1Vd4xgMw5ZvqfSvO6dI7SyNI7FnYksT1JptfRUKXs4KLd31fd9zilJyd2FFFFakhRRRQAUUUUAFFFFABRRRQAUUUUAdh4H8YjQLj7Bfwx3Gk3LYmV0BKZ4yPb2r3HRdRtxarpd9Kh2x/uJXI2XMB+6yk8E44I6/nXy9Xa+F/GcsNmuhatdIulkFY5pLYTNb59M9vzxXkZllqxC5o79f815+XX1SOijWcGd9c29nql7bxpfT2y2iTf2bqbI6Ip3IUXeeGx869egrt9A+IVxYyx6T4xjW0ujhYr9T+4nB6HPQH/PFY3hV7XRLSLR2uxd6bMN9jdsBtk3ctGewOckDuD7VF4ltYbJJtHgt3uob62klhs1iL+XImCCvYKSQCO3Hqa4aGOlTr+xirx6X6rq/J9137G9SipR5up6HqGmWlpZrq1isL/wBnwtJbRSSH7Og5LOAoPzbSwB5ry3XBeJY6/e3UBuLW8niW7ltgwS23hZcberDiJW6c56ZqWFH05GttJ1C6022ugY20rV4WNu4YYKq38OfY0mn6zqOneGbzQr/w/fOUvVluriCUTOw3q+cHBKlV2g89Oa9qjjKNVfFZ9np/w/yOV0ZxNGbxZrGhaTotpp05tYVhlyLm3kkLRBtqyjcNwUKGYKecAZJ77Metw+J9Q1KaXUr9tBsYEnzbxvE4dhjblOW4AYAf3uegq9afFHw3fSIjWWoC4KkBGsyzY7jjP5VXb4o+GdMRrew0nUGO8gw29mE+b6ZHNdXMrXM7Gfp/hzxXcxKS0Qh1CZbma5nIE6BQqorqVOcKucDHLexzr3fgLT9Ksr28tNSuIJkjzbG6nHlQMpDLk4BIBUDknAJArMuviD4iu7qC20zw0LTzYzKZtQmAESDjcyr09hnNcvqgl1+C4m1K91HxBcFGEUFlAyWkbYwD2DY9cmuapjKNP7V35a/e9l82aRozZvXvxA1HxRp50/QoIrXcm2+1Kdg0EIPBCE8Oa5/Ro9OtdSk0+Wa4awlvvMNzLGxS7fy0CgyEYPz7zjPUV0WjW9lqMszvkWunOLeG0eIosZVQd7Ajljn6Ae9YviyWw16Hfc6j/Z+j2TbxclAyzzDsoP3lUZ7dT7V4k8wniazpSTUfLo3t0u32tt07nUqKpx5lua2v6vZTBoJJUOm2riXUJ8goFXlYgehZjjI7Dr1rwnxf4tuPFOo+Z5SW9lESLe3RQAg9T6mrHi3xlc67FHp1vIqaXAcxxxwiIMfUgE1ylehl2XRw0U2tenl5+r/Bad781as6jCiiivVMQooooAKKKKACiiigAooooAKKKKACiiigAooooA6Hw14vv/DXmwxxw3VjP/rrScZRvceh969C8P614e1LUbW+t9W/s3VY1KQWshYw8/wsz5LA8Zxj9K8corlrYSFS7T5W97dfVbP8/MqM3HY+qG1aGW0aHU9NukYriSPyDKh45wyggj8q5Tw9q1tqMt1cPq2oR3ETPFFHDDgvAGOwgFSW47nnrXjdh4m1m0WOAavfrZL8rQLOxXZnkBScVsnx+812VudNSTTWGxrQTMuV6ZLDG5seuR6AV5UMn9jGUY637f5Pv6/M6ninJps9Lv7m/u1KLFdXmmxkPcvcrEJ0RSCTHsO7OM9ga6TTdMu7qxhmF2dOgkUNFa2UaAIp6ZYg5OOuK8U1vxfo7aUtn4f066tJM4M08uSi+i4PX3JrS034kadFokdpfaffNLGgTZb3ZSJ8e2fl/Csq+XVpUUqcba7WX32vYqNeClqzuNYvbPTPENnatqd5fQ3Uwjv1aPzVwqnZHlRwSxHy9+c11c+suYDFp1jNvAwJJ4jFDEPVicdPQfpXiQ+KWoPD9gNnb2+ltkPDbRruAPcFgec8/h+NczqvibXNWgW2v9Vubi3XlUd+D9QOv49KbyedXkVSy5fPfzsktelr7W1J+tct+U7/AFTxF4Z0Oe6ltr6TXrmebzJ4pCyozdzuU7SM44IPH0rgPEXiXUPE16txfGNVjXbFDEu1I19AKx6K9ulhYU3zby7v9Oi+Ryym5bhRRRXQSFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB/9k=</t>
+        </is>
+      </c>
       <c r="N27" t="inlineStr">
         <is>
           <t>Administration &amp; Operations</t>
@@ -2858,7 +2930,11 @@
           <t>MHAA</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEAYABgAAD/4QA6RXhpZgAATU0AKgAAAAgAA1EQAAEAAAABAQAAAFERAAQAAAABAAAOxFESAAQAAAABAAAOxAAAAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCADnANMDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD5/ooooAKKKKACiiigAooq/pOnPqF2oIIhQgyNjoP8aTdi6dOVSShFXbO28NfDaDxJeSWcF6IrhU3qss23zB3x8h6V1f8Awzxff8/sX/gR/wDa65+0u57G7huraQxzQuHRx2Ir6D8H+KIPE2jrcLtS6j+W4hB+63qPY9qxo1edWe56ea5a8JPmh8D/AA8jx3/hni+/5/Yv/Aj/AO11zPib4W/8IvcQQ3k7N5yFlaOYEcHBHKCvqsnCGvNvjBambRrO8VMmCcxufRWB/qo/OtKjai2jiwkac68IVNm7Hz//AMItZf8APWf/AL7H/wATR/wi1l/z1n/77H/xNbtFcP1ip3Pr/wCwsF2f3sk8MfCdvFJuPsczIsG3c0swGc59EPpXRf8ADPF9/wA/sX/gR/8Aa69G+EdkYPC892f+Xm5baf8AZUBf5hq9C613wbcU2fHYqMI1pRp7Jux87/8ADPF9/wA/sX/gR/8Aa65XxL8NYPDd7HZz3oknZN7CKbdsHbPyDrX0d4v8TweGNGNwdslzJlLeIn7zep9h1NfPd3dz3t5Ld3Ehknlcu7nqTWVeryKy3O/KsueLnzT+Bfj5Hl9FaGr6dJYXjjb+5diY2HTHpWfWyd1dHmVKcqcnCSs0FFFFMgKKKKACiiigAooooAKKKKACiiigAooooA6fQdJs57BbqePzJCxADNx1x0roUijhTZEioo/hVa6n4VeCrPxT8PLqQt5F9HeOsU4GR91eGHcfrWZrnh/UfD179m1CAoTnY45SQeqnv9OtcOIhO990fWZJisKoqnZRn37/AD/Qy62PDXiG68N6zHf24LqPlli3YEidx9fQ1j06NGkcKgJY9AK54OSkuXc9zFU6VSjKNX4evl5/I+mLHVLbUtMhv7eYNbypuDHj659CK5Dx34i0zUvD15pNtIbi5kC7GjXKKwYEZY8du2a4HTorq101rV7qb7NI3mPbhsJux6d/5VZ3KV6ba+sw2VSqR5q2l+h+M4/PIUKrhhPes/i6fJGBHoUxi3SSIjegBb/Ch9BlEe5JUZvQgj/Gukt7aW8uoYF+9K4Ue2aLq1ks7yeAnJicrnHXFdH9k4G/Jy6+rI/1uzz+N7XS/aNvTY7LwX4j0jTdAsdJnkNrNCmGMq4RmJJJDDjqT1xXW3+q2unaZNfzzBbeJN5Yc5HbHqT2rxzcirgjdVPVI72501LSG6k+yxvvFuW+TPt6fyrDFZXKEXKjrboPL88hWqqGL927+Lp80ZniXxDc+JdZkv7jKp92GInIjTsPr3Pv+FY9KylWKkYI4IpK+Sm25Ny3P2nC0qVKjGNL4fz8xHRZI9kqqy+jCsLXdMtE0ppookjeEjbsUDIJA57n8a7LRNB1HxBfC1sLcuRgu54SMerHt/Om/GDwjb+FNE0JFkaa7nkl8+U8A4C4AHYc/WujDwne+yPCzvFYXldOylP8vn+h5HRRRXcfJhRRRQAUUUUAFFFFABRRRQAUUUUAFFFFAH05+zt/yIt5/wBf7f8AoK16bqmkWOr2TWl/bRzwt1Vh0PqD2PvXkHwD1vTLDwpcWV3ewwXEl4zokr7dwwo4z7ivbldXUMpBU9CDQPVHg3iv4e32hBrqyD3mn55YDMkX+8B1HuPxrJ0OzXY1w+Du+79K9612++waFe3aAbkiO3P948D9TXjMEaxwpGoxHGMCvQyrBQlWdZrb8zg4gz7ErBLBc3xbvrZdPmx2MtxWlp+h6jqkZls7USoDgkSKMH6E1m5w3FXdL1S50m8W5tptpHDIRw49DX0Nf2nK/Z2v5nw1D2XtF7a/L5bnVeFfDN9Y60Lq/gEaRoSnzq2WPHY+maZ4u8P3dzrX2qytXmWVAX2Dow4/liu10u8Gpadb3exo/NQNsbtTdVvhpemT3hRpPLXO1e//ANavm1ja/wBY57e9tY+veW4X6n7O75fiv1/LseTXelXtjFvu7VoUJwC7AZ+lUA21uKvahqU2rXjXN1Jk9FQdEHoKo9T8tfS0ufl/e7+R8dW9lztUr8vmZOt2QVFuVIGeG/xrY8I/Du+1/bd3oe008nhiMPKP9kHoPc/hTJo98b4+6R6V7Po14NQ0Szuzj97EpOBjnv8ArXzmbYKEa6rJfF+Z95w/n2JeCeD5vh69bPp8iXS9IsdItFtbC2SCFf4VHU+pPUn614z+0p/x5eHf+uk/8kr3OSRIYy8jqiDksxwBXz7+0JrWm6pBokNjeRXDwPL5vlNuC5C45HHY1wHdqzwuiiigQUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB2nhz/kCID0Ltn866jTPEGr6OFXT9QuII1ORGr5T/vk8fpXL+HCP7FTkffb+da2R6j8682o5RqOx9zgqVCrg6aqpPTqdx/wn+sa5af2XfC3ZHYMZUUq2Bzgjof0pv+r2muY0XB1SHDDqfx+U10vUV9fkTcsM297v9D8m40pU6OZ+zpfCor8bh1NT2tsbm+htgP8AWOF/OoOjU9GdZFkjZkdeQynBFexO7TsfJQaUk5bHoeueJodJgGn6eytNGoTd1WIAY/E0ujeI4datm06/2pNKhTP8MgI/Q+1ecFu7N9STQrDh0fkHIINeZ/ZlL2fL9rv1uez/AG1X9t7R/Bty9Lf5+Y+RGt7iWF/vRuVP4GimEs7FmJZicknqafXqK9tTxJWvoMxxSL8QNa0iyXSbI28UcBYCXZuc7iW78DG7HQ0/7gWuT1Ij+17vkf6wd/8AZWvEz5uOHi473/Rn2XBFKnWzGVOqrx5W/uaJNS1nUtX/AOQjfT3IznbK5Kj/AID0/SuS8Wf8edv/ANdD/Kt/I9R+dc/4qI+x2/I/1h/lXylFydRNn6nmdOhSwNSNJJbbeqOVooor0D4kKKKKACiiigAooooAKKKKACiiigAr03VPh0ll8LbbVljP9pqBdT/9cz/D+AIP4GsLwL4Ys/EyatFcO0c9vAssEgPCnJzn24r1u8j1TUNGtoLsrDZauotpIeptVYfKQccsQCDnoWHpz4+OxkoVoQpytZ3l5q17fdf5r0OinSvFtrfYsfADTbK78D3UlzaQTOL1wGkjDEDavqK9X/sPSf8AoGWf/fhf8K4j4R6fbaTpGs2FmrC3g1N40LnJOEQZr0bPFepTlGUVJddTBqzsea/EK0stO0/S5YLKKNzdlSYYlUnMb8duM1y32LUdn/IMuv8Avlf8a7T4lRA6fpaNyDdtkHv+6euSi8TXenQBbmFbqEEKJDJsZMnHzE8Ee9dNTEZlhsL7XAxjJJu6e+y1WqPExNDAV8X7LFtxbSs1tu9Nit9k1Tbs/sy8/wC+V/xpkkF5bxeZPYXMUYIBd1GBk4Gea6OTV9U/tRbUWtlavIm+KSe4ZxJ6gAKORwcZ706Mz6gl9pGr+SZdgYPApVWRuhAJPIYH9K8OHF2YRtKrCHLo3a97X1trY7pcMYFpqDlf9fuH+A9Osr3ULy4vEjlngVRCjc7VPVseuRjPb8ai8cWFnYaxay2axxSXEbGaJBgHBGGx2PJHvj2rCsBdaX4l06GV2juVuYlLISBIjOFJHqD3FJKk+reILuNHZ7iSV/MlJz5aBiAT9AOBX1LxFBVfrvtF7O3Nfy2seR7Kq8F9T9n79+W3nvf7iKK3vbmJZILG5kib7rqowfpzT2stU27P7Nuz77R/jXSTy3NtLaaXpBgV44vMka4UsqxjgdCOSf5GoYNY1U381ubOzufIUNLNDclVQn+E5U84569K+WlxdmMrypwhbdXve19L62PXjwxgUkpOV/1+4wzZaiI8nTLr/vlf8a6v4cWdjqOi6jcTWUMrm/YAzRKWwI4/WuXl8RXmsWm2KAWtq4IJD7ncexHABrs/hnGDompKvCjUGAH/AGzjr3YV8yr4VVMfGMbtWS32er1Zx4ShgaOLlTwjcmk7t7brTY67+w9J/wCgZZ/9+F/wrw/9oixtLOx0E21rDCWlm3eXGFzwvpXvteYfFXRLLxDq3h3Tr9XMUn2kBlOCrBVIP6VyTqxhB1JbJXPajFydkeQa78OY9O+GdlrcYcX0arLdAn7yuRgY7bcj9TXm1fQ982rXvhG4kkeF7S5Q2XlLwscZ/dibOM9ckj0I9K8f8eaHaeHPEn9l2ZYpDBHuZurMRkk/nXnZbip1HKnVleV21botNPk3Y1rU1GzjscxRRRXrGAUUUUAFFFFABRRRQAUUUUAegfDL5YPETo4EossKmeXHJYAd+BXs2r3NtLZ2cMMsbM1zAwAYfKoIcsfQbVJrx/4YJay6b4jFyDuihilhdThkcFgNp7EkqPfpXo7+FrPTf7DnlBdjKILzHHnF+Rn/AGQ4A29McdBXy2ZKlLF3m2mnppv7qf8AXqehQ5lT0/rU6z4WTw3Gn65JBIJIzqkmHHQ/Kteg/wAVec/CWY3Gm69ORjzNXmI+mBj9MV6N3r6WkrU4p9kcMviZwXxMP+h6UPW7b/0W9eflQ6srAFTwQa7/AOJp/wBF0gcc3Lf+i2rgh/q2r6jKf93fr/kfFZ/pi16L82Q3rNiGCe9uZNKD4mhTaxVcYyuQSMHB4/CtS3ggtZ4jFrEksyD/AIl11PPujdTjML478d+ehHINUT8vDDNQxWEmo3DxWenC58nElxtUExqehA/ibjgCvFzbIaNV+0pzVNdVZWfn69H3R6OU55XilRlB1H0d9TdvtYsru9020uYxb6pFqFuwhfBJHmLkow4Yf5IqPSNZs7eKaysIkuNSkuZnkjXChf3jYaRu3H4+grNe2t9P8Wf2fsV5bS6t8yeUUzllPemWOnxarqgtBGqTTCaUN5BkJ28449c9zXlvhyj9U9h7X3fivZ27Wte9r+fzPXWcVPa/wvevy2uu1732Ltxa2t1LN5utTIrnOpXMU21HOCBEn0z27D1NZcAkntpbUXVyunMx8qB9qfJ23bQOvv8AjTjp81lcJb3enrazsnmxDaPmQ/xY7HsQehqc9dhHz16uU5FRoP2lSXtF00Vl5+vTyWh4+b55Xl+5hF03111/4YFChNqgBQMADtXf/C7/AJAup/8AYRb/ANFx1wH8Nd/8Lv8AkC6n/wBhFv8A0XHXrZv/AAY+v6HHw/8A7xP0/VHdV578QJoIfFHhVp5ViUvcAMxwM7VxXoXavOPiJt/4SrwjHIivFNLcxOjLkMCg4I/KvlMWr4Wp/hf5H2VL416mXDcWsfgWW3lZBJHaPG8efmBGV6f71eLfFHB8YlvNSRjaw7ypzhguCD75Feof8I3DL4audVt2kF2Z2uY3b5mWNflCZPX5RkE9Gwe1ea/FaC1tvFNrDZxqkK2EWMd8ljknuTnrXiZSqMcTLkbbfNfy2v8A11OzEc3s1fyOFooor6U4AooooAKKKKACiiigAooooA9B+G8cq2erttws6xpE5OA0qN5nl9PvEDivVb3xNZanc2NtbLM3lzR3R+THmKASoTP3iW4/4C3pXnHw3AuPCmr2DxiQXl5BbqGGQpfOW+oUE/hXq13YxWfiHRZ7eNFwslmQFHCbCwx9Cn618pmU6SxEnNaq9vlFf8N6no0FL2a7f8E0PhHE8OjaukiCNxqUmUDbtvyrxnvXotebfBmVp/DOoTOcs98zMffaua9Jr6mCaikzz3ucD8S/9Vo4x/y8Of8AyGa4Id67v4l/d0cZ/wCW8n/oBrhB3r6XKf4D9f8AI+L4h/3pf4V+bFB2NXD61rWr+GPFLX2m3stt9pgWN9h+8o6jnv3B7V255G6s7W9DtdZstk4KsOUdeqmujG0HXpcsd9zmyrFxwuIUp7PRj9NvbW6S1ubRg++4id2JyxbeCdx65+tVrnVLaz0iK8nkMUiDfG6Nhw/baeua4GwWbRfFVvZwXplRbmMSlAQpwwyCPaobWyl13XPsVxeGHBIj8xT0HQAfSvK+uSc+VQ1ty26bn0H9mwjDndR8qfNfW9rHT+Gdb1bxJ4kuNS1W8kuZEt9gZ+ijcMADoO5rtDxLmqemaRBpdgsVuuAOWc9XPqau/wAGa9bB0HQoqEtz57M8XHFYh1I7bCf8s69A+Fv/ACBNT/7CL/8AouOvP/8AlnXoHwt/5Amp/wDYRf8A9Fx1yZv/AAo+v6Hbw7/Hn6fqjuBXnHxH3jxJ4UlSBpjFLO5RSAxAVemep74r0cV5z8SJWTxP4O2nlruRfwIUGvlq/wDu8/8AC/yPsqfxr1OdtvEtjZaHNpI8yS4iVo48Idrl2IjGexOeh6bT6V5J8S8ya7azIu62FolvFOPuymP5WKnuAeM+1e022i2mq6TrRmiQtqdxLvO3psOxfy2Z+pryX4o3SXcPh2SOMRr9jI2qMBSCAQPoQa8HKp0liJRpp3u7+tr/AJpnbiFL2ep55RRRX0xwBRRRQAUUUUAFFFFABRRRQB6Z8Prg2PhPULuSNo44rxJ4rkKWXzIwD5bAcjIbg9Oa9ETVNW1LW4xNp629zZxNNbozFkVZF4kkI7gZXaO5PbmuN+GwLeAbiEtiO41qGF/90+Xkfj0/GvStWjK+I9JeI4adJ7aQD+Jdm4fkVH518pmdaCryUoq/va+kV+aun+h30IvlWvYPgS0kngu6klILves5IHHKqa9Try34GAx+C7qJuGivGjb6qig/yr1HcK+qW2hwHn3xLPOjD/prIf8AxyuFHeu4+JbDzdGA/wCekv8A6DXDjvX0mU/wH6/5HxnEP+9L/CvzYgpswLRuFzypAx64paK9R6o8ROzueeeEnt4LTVIpxtu1Ktlh8xUHkfgetN8VlXvdGS1Aa8CLv2D5u23Pv1pfGSWltrkMloxW7c5mVRxz3PuaseBYrSe7u7i4dnvkb5FkHRemR79vavm1Fup9V07X+d/vPtpTiqX1/Xvb1Sj93U78dKWiivpD4UZ/BXoHwu/5Amp/9hFv/Rcdef8A8FegfC7/AJAmp/8AYRb/ANFx15Ob/wAKPr+h9Fw9/vEvT9Ud5XlHxde4j1zwa9s8aTfbmVTIMryUHP516tkV5Z8WIjceIPBcK/ea/J/BSjH9BXzM7KEubaz/ACPsofEjEfX9S0q41KFLEyRQ7rq5BbBgL/3eMMpOXyOcE8ZFea/EtVWz0FIopBbxQvHHPINv2g/KWYKeQMnvjrXs2lW63Ntq003zPc3UyyZ7KvyBfphf1ryT4qTPcaJ4Rmc5LWkn4/c5/Gvm8vqQeLSjGzvZ+vK/+D8vPU7q8X7O7f8AVzzOiiivqTzwooooAKKKKACiiigAooooA9I+HV3ct4a16zjQSxRbLoqrASRsORIueDgoOM5r0CO51241TSbi8MMT6jblbZwvy2hKhnH+05AGM8da8u+GYdtQ1xEBJbSJuB/vJXt2q7ZNDsZYQG2T2rxEf76jI/An86+YzVqniEuVe89+14pfn96Vu530Nad77f5nL/CVdRv21HS21S9srZJprnNtsDzPvCtuYqeny9MdTXTeFbSPxJtu9SuHktJnkSOGXUJvODKAecNtf5Tk4AxWT4atPDKXXiWLV5WjjsdSZ0kjnkjOJsEp8hBYZTp7VXg1W7t/EGqP4W0i1heNytrE9u3mSgIWO1WORvABLYHbrzX0lOanBTXVI4pKzaLGpSg2FnbJKZYLXU72GB9+8eWMFQG7gBsfhVD+Bq3da0nV7bSImvjJJb21xE8byJGrKZUYSLhOMByv69awh91q+mylr2DXn/kfF5/FrFJ+S/NiGgkgMQMkDge9Bor1DwkeceHxbzvrEuoZ+37G2rJwRwd2B61N4jMFt4m06awI+2EjzVQ554Az7kZzVzxTYQ3ut/Z7UJFdJH500mcZUdsdzTvClhbWOq31lchJb6HDLPknKn2PQ818+qcuf2Gm/wAX4/efZyrQ9n9b12+HyaS+7qdsOlLRRX0B8SKP4a6vwHq0OlaLcLIkkkt3rBt4Y4xksxiQn6ABWJ+lcifurXd+G9E0258AK+qQb4ZZJLxsEqykE7WBU5B2gdK8jOGvZxXmfScOxftpy8v1KWoXJ128vdV0jxLfWdqJYbBZFh3Q+bvGcfQ4UnGMnqarfFWKeTxJ4JjguHhmN3MFlUAlflXnB4p2jWLnVbPTpba40nRdQf7daWSujh3Ta21jjcmcByvOeeeop3jq4iufiV4dsiR5lpa3F0oz1ZhtA/Q18ti58mHqS7J/kfZU1eaRy0+o65babrGpQLGtoZvImVF3bpMhHmj9unynvnmvOfifqU1xrdppssIhXT7ZY1jDbtoYBhk9CcbelewSBIvhowYBd9j09XYfzLGvFPidu/4WDqQbqFhH/kJK8TK6kamJa5UuXm/DlS/BnViE1Dfe36nI0UUV9IcIUUUUAFFFFABRRRQAUUUUAdV8O7y5tPGVqlrcRQvcK0OZlJRsjIVgOxIFeswabrlzZ6isUz202nXG23so5PMiwFDcEgHPzZXP3eB2rwKzuHtL2C5jOHhkWRT7g5r6j0+5jtr/AFY3EiRq7JdBmOBsMaqT+BU18/nM5UZKcEm2u3Zr9H/kdeFSk7MyvBt1Y2PxHjtbMBbHUdOjaHd1ZhuIJzzu4fOec10Hjy/XS9e0Wa4maxsZS8U99CAkiE42jfg4HcjjP6HgdQuJprj+2NFeGQ6FcSXWUO7ejSE7RjthGJ9mr2KTUJ9Z8MW+o6ILeaSZY5o45vuuuQWXPY4yM9jXpYGop0UnvHR9/K/qjKtG079ypHJb+MPA0n2OZnW4hKI7kFg6ngtjgHIBx2ry+FmMH7xGjkUlXRhyrDgg+4PFdBN4yh0O81R1Fraaje3CQtBGDNFaFdqtJMUwM/OOnoBnNZt/Bc3FouvkQtFPIy3DRKUUsGKidVPIR8A89D9a+gyzEqlU5ZbM+ezvBOvRVSC1j+RVopAc0tfSnxBzHiy0WQRXFuSuoqSkQX+NT94N7Ad/en+GbVVN1czOx1CR9txvGCh9APStO5tTJei5xlkgeNf94kH+QpbWzeDU764I5nWPB9xkH+lcCo/v/aW/q2/r0PbeK/2T2N+n6rT06+pdoooJGCSQMckk13njEiw3E8kOn2ylp7pxEmOxPU/QDJP0r1HXUudK8Lx2mlMyyK0NujqAWVC6qzKO5C5P4VgeAdDdm/t69UruXbaRsuCFPVz9eg9vrWR4k1SPXNWmNxpUs1jNbtZ6dMw3Is/m+WXPZMsQoJ54zjFfL4/EqtV93ZH3eT4N4ehea96Wr/Q6Pw7p8cnifUboX13qUdiogtri5kL+U5z5qr0BPC5P4dq4LV79dT8c+KLlVd3s44LSyaL7wn3NtA/4FnPtnNei3upT+C/h0tzfyCW9tbRY89fMmIwB78/nXm2hsPD09jZavcQRTvMb6Z5GC/6yNgM56kMpB+or5/MKvLQajq309NX/AJfM9zDxvO7LM2l6xZ6jpVisqXqujXEiXEhWGGRCCGVQMkDdwvtmvDvFF7LqPifUbmebzpDOymTbt3BflBxk44Ar6D8T37W51C5hkAksdMmdm7KWxtH1+Un8q+Za5MlcqkPazSvZfi2/ysXikoy5UFFFFe4coUUUUAFFFFABRRRQAUUUUAFeoeC7+48SaDLpD6nIL+xXzbaJo1O+Nedof72OMEe9eX1Z06/uNL1G3vrWQxzwOHRh2IrGvRVWNuq1XqVGXK7n02bS31Czi1rR1iiupYxIjY2rMpH3JAOo7eoNUdC8UWvhBPskUctxa6hEbrTbX+OOQsA8Of7oJz7YbrxWCnj/AE2x0VtV0y5tytxmZ9MuSUdHz82xgDkE54xj3FB0e7ms7j/hJVWDe6yafqFmd0dryWGTwRy3UjBr53A+1wc3OrdRvaz3a7W68uj087bnZV5aqtHf+vzOnuvCd/ousRavPJYz/abhQLUIQrTys2QWPIjDMG7nKjpxVyysltb/AF/U/EiQCbT5vOkltVZxNA0X+rww5X/Z9R+NWvD+ux+IbOTwt4piRdWRBkbsLdIOVljI78Z45BFR6j4dVtYnsZ/7VEvlImkXqvJKkB2nJcg9d3Xd1GBX00JxnFSi7pnE007My77wpI9rHrHh5HudPuEEq2rDEsan+7nqB6Hn0zWAZY/NaIKYpVOGjcFWH4HmvQbfxq1tHaXGp2ItdJuj5VrerJuMjgHrGBlQ2DjBParOuXfh3U/DrapJaQanCrKkYUAP5hcIFBOCp3EA9MV6mHzGpSXLLVHiY3JqFeXPB8r/AA+483AD/wAH60E7eq13Vl4J0zUrQSva6hpkoYq8BmDYIPY85Hoe9X4vhzoMY/fC7n9RJcMAfwXFdrzenbSLPLXDte+s1b5nmqSbplhhVppm+7FGpZj+ArrvDfgaa5kjvtcjEcY+dLLIJJ7eYRx/wEfj6V08Vx4W8M3MWmQy6fYXEi7kgBVXf39T0Nc7rnjbURpVtdWNjNaW88iyRXM4DefCAWYBQSVYqMrnqAeQa4MTmNSsuVaI9bBZPQwz5pe9L+uhJ478VDT1/sm1YfvY2S5MT7JYlIwNmeAeeD0yADjINJ4N0BLq3hurmZJ7G1lL2CxSELIf+ekqd5AfXoc+xrCis9djs7DWtUihvPDunQbljZ8TSQMjKzOjL94K2SNxzjiqtwraTf3lh4Z1h/LuYhJPKWxHYwso+Z/70u0YXocdema8yc4U4Oc3ZI9lJydkanifWIdf1aT7PMlxa6RcpDDAD8kt43AZj3VM9u+fSo9T06LTtGu5JAlzqt0nkLcSICzyP8qgeignoOgFc5cR3WjW0OpaDYomi6fF50/2xijXTLuw68E5O48nGeKpav4/sE0oam+oW8+oBT9jsrXLLA7DG9iQNzAZ4OP6183iY18TXVWnrG+3Vdou23d+uuqSO6HJThZ7/wBanK/EPUTpkEPhm01d7tIwDdhY1Vd4xgMw5ZvqfSvO6dI7SyNI7FnYksT1JptfRUKXs4KLd31fd9zilJyd2FFFFakhRRRQAUUUUAFFFFABRRRQAUUUUAdh4H8YjQLj7Bfwx3Gk3LYmV0BKZ4yPb2r3HRdRtxarpd9Kh2x/uJXI2XMB+6yk8E44I6/nXy9Xa+F/GcsNmuhatdIulkFY5pLYTNb59M9vzxXkZllqxC5o79f815+XX1SOijWcGd9c29nql7bxpfT2y2iTf2bqbI6Ip3IUXeeGx869egrt9A+IVxYyx6T4xjW0ujhYr9T+4nB6HPQH/PFY3hV7XRLSLR2uxd6bMN9jdsBtk3ctGewOckDuD7VF4ltYbJJtHgt3uob62klhs1iL+XImCCvYKSQCO3Hqa4aGOlTr+xirx6X6rq/J9137G9SipR5up6HqGmWlpZrq1isL/wBnwtJbRSSH7Og5LOAoPzbSwB5ry3XBeJY6/e3UBuLW8niW7ltgwS23hZcberDiJW6c56ZqWFH05GttJ1C6022ugY20rV4WNu4YYKq38OfY0mn6zqOneGbzQr/w/fOUvVluriCUTOw3q+cHBKlV2g89Oa9qjjKNVfFZ9np/w/yOV0ZxNGbxZrGhaTotpp05tYVhlyLm3kkLRBtqyjcNwUKGYKecAZJ77Metw+J9Q1KaXUr9tBsYEnzbxvE4dhjblOW4AYAf3uegq9afFHw3fSIjWWoC4KkBGsyzY7jjP5VXb4o+GdMRrew0nUGO8gw29mE+b6ZHNdXMrXM7Gfp/hzxXcxKS0Qh1CZbma5nIE6BQqorqVOcKucDHLexzr3fgLT9Ksr28tNSuIJkjzbG6nHlQMpDLk4BIBUDknAJArMuviD4iu7qC20zw0LTzYzKZtQmAESDjcyr09hnNcvqgl1+C4m1K91HxBcFGEUFlAyWkbYwD2DY9cmuapjKNP7V35a/e9l82aRozZvXvxA1HxRp50/QoIrXcm2+1Kdg0EIPBCE8Oa5/Ro9OtdSk0+Wa4awlvvMNzLGxS7fy0CgyEYPz7zjPUV0WjW9lqMszvkWunOLeG0eIosZVQd7Ajljn6Ae9YviyWw16Hfc6j/Z+j2TbxclAyzzDsoP3lUZ7dT7V4k8wniazpSTUfLo3t0u32tt07nUqKpx5lua2v6vZTBoJJUOm2riXUJ8goFXlYgehZjjI7Dr1rwnxf4tuPFOo+Z5SW9lESLe3RQAg9T6mrHi3xlc67FHp1vIqaXAcxxxwiIMfUgE1ylehl2XRw0U2tenl5+r/Bad781as6jCiiivVMQooooAKKKKACiiigAooooAKKKKACiiigAooooA6Hw14vv/DXmwxxw3VjP/rrScZRvceh969C8P614e1LUbW+t9W/s3VY1KQWshYw8/wsz5LA8Zxj9K8corlrYSFS7T5W97dfVbP8/MqM3HY+qG1aGW0aHU9NukYriSPyDKh45wyggj8q5Tw9q1tqMt1cPq2oR3ETPFFHDDgvAGOwgFSW47nnrXjdh4m1m0WOAavfrZL8rQLOxXZnkBScVsnx+812VudNSTTWGxrQTMuV6ZLDG5seuR6AV5UMn9jGUY637f5Pv6/M6ninJps9Lv7m/u1KLFdXmmxkPcvcrEJ0RSCTHsO7OM9ga6TTdMu7qxhmF2dOgkUNFa2UaAIp6ZYg5OOuK8U1vxfo7aUtn4f066tJM4M08uSi+i4PX3JrS034kadFokdpfaffNLGgTZb3ZSJ8e2fl/Csq+XVpUUqcba7WX32vYqNeClqzuNYvbPTPENnatqd5fQ3Uwjv1aPzVwqnZHlRwSxHy9+c11c+suYDFp1jNvAwJJ4jFDEPVicdPQfpXiQ+KWoPD9gNnb2+ltkPDbRruAPcFgec8/h+NczqvibXNWgW2v9Vubi3XlUd+D9QOv49KbyedXkVSy5fPfzsktelr7W1J+tct+U7/AFTxF4Z0Oe6ltr6TXrmebzJ4pCyozdzuU7SM44IPH0rgPEXiXUPE16txfGNVjXbFDEu1I19AKx6K9ulhYU3zby7v9Oi+Ryym5bhRRRXQSFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB/9k=</t>
+        </is>
+      </c>
       <c r="N28" t="inlineStr">
         <is>
           <t>Healthcare &amp; Medicine</t>
@@ -2934,7 +3010,11 @@
           <t>MHAA</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEAYABgAAD/4QA6RXhpZgAATU0AKgAAAAgAA1EQAAEAAAABAQAAAFERAAQAAAABAAAOxFESAAQAAAABAAAOxAAAAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCADnANMDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD5/ooooAKKKKACiiigAooq/pOnPqF2oIIhQgyNjoP8aTdi6dOVSShFXbO28NfDaDxJeSWcF6IrhU3qss23zB3x8h6V1f8Awzxff8/sX/gR/wDa65+0u57G7huraQxzQuHRx2Ir6D8H+KIPE2jrcLtS6j+W4hB+63qPY9qxo1edWe56ea5a8JPmh8D/AA8jx3/hni+/5/Yv/Aj/AO11zPib4W/8IvcQQ3k7N5yFlaOYEcHBHKCvqsnCGvNvjBambRrO8VMmCcxufRWB/qo/OtKjai2jiwkac68IVNm7Hz//AMItZf8APWf/AL7H/wATR/wi1l/z1n/77H/xNbtFcP1ip3Pr/wCwsF2f3sk8MfCdvFJuPsczIsG3c0swGc59EPpXRf8ADPF9/wA/sX/gR/8Aa69G+EdkYPC892f+Xm5baf8AZUBf5hq9C613wbcU2fHYqMI1pRp7Jux87/8ADPF9/wA/sX/gR/8Aa65XxL8NYPDd7HZz3oknZN7CKbdsHbPyDrX0d4v8TweGNGNwdslzJlLeIn7zep9h1NfPd3dz3t5Ld3Ehknlcu7nqTWVeryKy3O/KsueLnzT+Bfj5Hl9FaGr6dJYXjjb+5diY2HTHpWfWyd1dHmVKcqcnCSs0FFFFMgKKKKACiiigAooooAKKKKACiiigAooooA6fQdJs57BbqePzJCxADNx1x0roUijhTZEioo/hVa6n4VeCrPxT8PLqQt5F9HeOsU4GR91eGHcfrWZrnh/UfD179m1CAoTnY45SQeqnv9OtcOIhO990fWZJisKoqnZRn37/AD/Qy62PDXiG68N6zHf24LqPlli3YEidx9fQ1j06NGkcKgJY9AK54OSkuXc9zFU6VSjKNX4evl5/I+mLHVLbUtMhv7eYNbypuDHj659CK5Dx34i0zUvD15pNtIbi5kC7GjXKKwYEZY8du2a4HTorq101rV7qb7NI3mPbhsJux6d/5VZ3KV6ba+sw2VSqR5q2l+h+M4/PIUKrhhPes/i6fJGBHoUxi3SSIjegBb/Ch9BlEe5JUZvQgj/Gukt7aW8uoYF+9K4Ue2aLq1ks7yeAnJicrnHXFdH9k4G/Jy6+rI/1uzz+N7XS/aNvTY7LwX4j0jTdAsdJnkNrNCmGMq4RmJJJDDjqT1xXW3+q2unaZNfzzBbeJN5Yc5HbHqT2rxzcirgjdVPVI72501LSG6k+yxvvFuW+TPt6fyrDFZXKEXKjrboPL88hWqqGL927+Lp80ZniXxDc+JdZkv7jKp92GInIjTsPr3Pv+FY9KylWKkYI4IpK+Sm25Ny3P2nC0qVKjGNL4fz8xHRZI9kqqy+jCsLXdMtE0ppookjeEjbsUDIJA57n8a7LRNB1HxBfC1sLcuRgu54SMerHt/Om/GDwjb+FNE0JFkaa7nkl8+U8A4C4AHYc/WujDwne+yPCzvFYXldOylP8vn+h5HRRRXcfJhRRRQAUUUUAFFFFABRRRQAUUUUAFFFFAH05+zt/yIt5/wBf7f8AoK16bqmkWOr2TWl/bRzwt1Vh0PqD2PvXkHwD1vTLDwpcWV3ewwXEl4zokr7dwwo4z7ivbldXUMpBU9CDQPVHg3iv4e32hBrqyD3mn55YDMkX+8B1HuPxrJ0OzXY1w+Du+79K9612++waFe3aAbkiO3P948D9TXjMEaxwpGoxHGMCvQyrBQlWdZrb8zg4gz7ErBLBc3xbvrZdPmx2MtxWlp+h6jqkZls7USoDgkSKMH6E1m5w3FXdL1S50m8W5tptpHDIRw49DX0Nf2nK/Z2v5nw1D2XtF7a/L5bnVeFfDN9Y60Lq/gEaRoSnzq2WPHY+maZ4u8P3dzrX2qytXmWVAX2Dow4/liu10u8Gpadb3exo/NQNsbtTdVvhpemT3hRpPLXO1e//ANavm1ja/wBY57e9tY+veW4X6n7O75fiv1/LseTXelXtjFvu7VoUJwC7AZ+lUA21uKvahqU2rXjXN1Jk9FQdEHoKo9T8tfS0ufl/e7+R8dW9lztUr8vmZOt2QVFuVIGeG/xrY8I/Du+1/bd3oe008nhiMPKP9kHoPc/hTJo98b4+6R6V7Po14NQ0Szuzj97EpOBjnv8ArXzmbYKEa6rJfF+Z95w/n2JeCeD5vh69bPp8iXS9IsdItFtbC2SCFf4VHU+pPUn614z+0p/x5eHf+uk/8kr3OSRIYy8jqiDksxwBXz7+0JrWm6pBokNjeRXDwPL5vlNuC5C45HHY1wHdqzwuiiigQUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB2nhz/kCID0Ltn866jTPEGr6OFXT9QuII1ORGr5T/vk8fpXL+HCP7FTkffb+da2R6j8682o5RqOx9zgqVCrg6aqpPTqdx/wn+sa5af2XfC3ZHYMZUUq2Bzgjof0pv+r2muY0XB1SHDDqfx+U10vUV9fkTcsM297v9D8m40pU6OZ+zpfCor8bh1NT2tsbm+htgP8AWOF/OoOjU9GdZFkjZkdeQynBFexO7TsfJQaUk5bHoeueJodJgGn6eytNGoTd1WIAY/E0ujeI4datm06/2pNKhTP8MgI/Q+1ecFu7N9STQrDh0fkHIINeZ/ZlL2fL9rv1uez/AG1X9t7R/Bty9Lf5+Y+RGt7iWF/vRuVP4GimEs7FmJZicknqafXqK9tTxJWvoMxxSL8QNa0iyXSbI28UcBYCXZuc7iW78DG7HQ0/7gWuT1Ij+17vkf6wd/8AZWvEz5uOHi473/Rn2XBFKnWzGVOqrx5W/uaJNS1nUtX/AOQjfT3IznbK5Kj/AID0/SuS8Wf8edv/ANdD/Kt/I9R+dc/4qI+x2/I/1h/lXylFydRNn6nmdOhSwNSNJJbbeqOVooor0D4kKKKKACiiigAooooAKKKKACiiigAr03VPh0ll8LbbVljP9pqBdT/9cz/D+AIP4GsLwL4Ys/EyatFcO0c9vAssEgPCnJzn24r1u8j1TUNGtoLsrDZauotpIeptVYfKQccsQCDnoWHpz4+OxkoVoQpytZ3l5q17fdf5r0OinSvFtrfYsfADTbK78D3UlzaQTOL1wGkjDEDavqK9X/sPSf8AoGWf/fhf8K4j4R6fbaTpGs2FmrC3g1N40LnJOEQZr0bPFepTlGUVJddTBqzsea/EK0stO0/S5YLKKNzdlSYYlUnMb8duM1y32LUdn/IMuv8Avlf8a7T4lRA6fpaNyDdtkHv+6euSi8TXenQBbmFbqEEKJDJsZMnHzE8Ee9dNTEZlhsL7XAxjJJu6e+y1WqPExNDAV8X7LFtxbSs1tu9Nit9k1Tbs/sy8/wC+V/xpkkF5bxeZPYXMUYIBd1GBk4Gea6OTV9U/tRbUWtlavIm+KSe4ZxJ6gAKORwcZ706Mz6gl9pGr+SZdgYPApVWRuhAJPIYH9K8OHF2YRtKrCHLo3a97X1trY7pcMYFpqDlf9fuH+A9Osr3ULy4vEjlngVRCjc7VPVseuRjPb8ai8cWFnYaxay2axxSXEbGaJBgHBGGx2PJHvj2rCsBdaX4l06GV2juVuYlLISBIjOFJHqD3FJKk+reILuNHZ7iSV/MlJz5aBiAT9AOBX1LxFBVfrvtF7O3Nfy2seR7Kq8F9T9n79+W3nvf7iKK3vbmJZILG5kib7rqowfpzT2stU27P7Nuz77R/jXSTy3NtLaaXpBgV44vMka4UsqxjgdCOSf5GoYNY1U381ubOzufIUNLNDclVQn+E5U84569K+WlxdmMrypwhbdXve19L62PXjwxgUkpOV/1+4wzZaiI8nTLr/vlf8a6v4cWdjqOi6jcTWUMrm/YAzRKWwI4/WuXl8RXmsWm2KAWtq4IJD7ncexHABrs/hnGDompKvCjUGAH/AGzjr3YV8yr4VVMfGMbtWS32er1Zx4ShgaOLlTwjcmk7t7brTY67+w9J/wCgZZ/9+F/wrw/9oixtLOx0E21rDCWlm3eXGFzwvpXvteYfFXRLLxDq3h3Tr9XMUn2kBlOCrBVIP6VyTqxhB1JbJXPajFydkeQa78OY9O+GdlrcYcX0arLdAn7yuRgY7bcj9TXm1fQ982rXvhG4kkeF7S5Q2XlLwscZ/dibOM9ckj0I9K8f8eaHaeHPEn9l2ZYpDBHuZurMRkk/nXnZbip1HKnVleV21botNPk3Y1rU1GzjscxRRRXrGAUUUUAFFFFABRRRQAUUUUAegfDL5YPETo4EossKmeXHJYAd+BXs2r3NtLZ2cMMsbM1zAwAYfKoIcsfQbVJrx/4YJay6b4jFyDuihilhdThkcFgNp7EkqPfpXo7+FrPTf7DnlBdjKILzHHnF+Rn/AGQ4A29McdBXy2ZKlLF3m2mnppv7qf8AXqehQ5lT0/rU6z4WTw3Gn65JBIJIzqkmHHQ/Kteg/wAVec/CWY3Gm69ORjzNXmI+mBj9MV6N3r6WkrU4p9kcMviZwXxMP+h6UPW7b/0W9eflQ6srAFTwQa7/AOJp/wBF0gcc3Lf+i2rgh/q2r6jKf93fr/kfFZ/pi16L82Q3rNiGCe9uZNKD4mhTaxVcYyuQSMHB4/CtS3ggtZ4jFrEksyD/AIl11PPujdTjML478d+ehHINUT8vDDNQxWEmo3DxWenC58nElxtUExqehA/ibjgCvFzbIaNV+0pzVNdVZWfn69H3R6OU55XilRlB1H0d9TdvtYsru9020uYxb6pFqFuwhfBJHmLkow4Yf5IqPSNZs7eKaysIkuNSkuZnkjXChf3jYaRu3H4+grNe2t9P8Wf2fsV5bS6t8yeUUzllPemWOnxarqgtBGqTTCaUN5BkJ28449c9zXlvhyj9U9h7X3fivZ27Wte9r+fzPXWcVPa/wvevy2uu1732Ltxa2t1LN5utTIrnOpXMU21HOCBEn0z27D1NZcAkntpbUXVyunMx8qB9qfJ23bQOvv8AjTjp81lcJb3enrazsnmxDaPmQ/xY7HsQehqc9dhHz16uU5FRoP2lSXtF00Vl5+vTyWh4+b55Xl+5hF03111/4YFChNqgBQMADtXf/C7/AJAup/8AYRb/ANFx1wH8Nd/8Lv8AkC6n/wBhFv8A0XHXrZv/AAY+v6HHw/8A7xP0/VHdV578QJoIfFHhVp5ViUvcAMxwM7VxXoXavOPiJt/4SrwjHIivFNLcxOjLkMCg4I/KvlMWr4Wp/hf5H2VL416mXDcWsfgWW3lZBJHaPG8efmBGV6f71eLfFHB8YlvNSRjaw7ypzhguCD75Feof8I3DL4audVt2kF2Z2uY3b5mWNflCZPX5RkE9Gwe1ea/FaC1tvFNrDZxqkK2EWMd8ljknuTnrXiZSqMcTLkbbfNfy2v8A11OzEc3s1fyOFooor6U4AooooAKKKKACiiigAooooA9B+G8cq2erttws6xpE5OA0qN5nl9PvEDivVb3xNZanc2NtbLM3lzR3R+THmKASoTP3iW4/4C3pXnHw3AuPCmr2DxiQXl5BbqGGQpfOW+oUE/hXq13YxWfiHRZ7eNFwslmQFHCbCwx9Cn618pmU6SxEnNaq9vlFf8N6no0FL2a7f8E0PhHE8OjaukiCNxqUmUDbtvyrxnvXotebfBmVp/DOoTOcs98zMffaua9Jr6mCaikzz3ucD8S/9Vo4x/y8Of8AyGa4Id67v4l/d0cZ/wCW8n/oBrhB3r6XKf4D9f8AI+L4h/3pf4V+bFB2NXD61rWr+GPFLX2m3stt9pgWN9h+8o6jnv3B7V255G6s7W9DtdZstk4KsOUdeqmujG0HXpcsd9zmyrFxwuIUp7PRj9NvbW6S1ubRg++4id2JyxbeCdx65+tVrnVLaz0iK8nkMUiDfG6Nhw/baeua4GwWbRfFVvZwXplRbmMSlAQpwwyCPaobWyl13XPsVxeGHBIj8xT0HQAfSvK+uSc+VQ1ty26bn0H9mwjDndR8qfNfW9rHT+Gdb1bxJ4kuNS1W8kuZEt9gZ+ijcMADoO5rtDxLmqemaRBpdgsVuuAOWc9XPqau/wAGa9bB0HQoqEtz57M8XHFYh1I7bCf8s69A+Fv/ACBNT/7CL/8AouOvP/8AlnXoHwt/5Amp/wDYRf8A9Fx1yZv/AAo+v6Hbw7/Hn6fqjuBXnHxH3jxJ4UlSBpjFLO5RSAxAVemep74r0cV5z8SJWTxP4O2nlruRfwIUGvlq/wDu8/8AC/yPsqfxr1OdtvEtjZaHNpI8yS4iVo48Idrl2IjGexOeh6bT6V5J8S8ya7azIu62FolvFOPuymP5WKnuAeM+1e022i2mq6TrRmiQtqdxLvO3psOxfy2Z+pryX4o3SXcPh2SOMRr9jI2qMBSCAQPoQa8HKp0liJRpp3u7+tr/AJpnbiFL2ep55RRRX0xwBRRRQAUUUUAFFFFABRRRQB6Z8Prg2PhPULuSNo44rxJ4rkKWXzIwD5bAcjIbg9Oa9ETVNW1LW4xNp629zZxNNbozFkVZF4kkI7gZXaO5PbmuN+GwLeAbiEtiO41qGF/90+Xkfj0/GvStWjK+I9JeI4adJ7aQD+Jdm4fkVH518pmdaCryUoq/va+kV+aun+h30IvlWvYPgS0kngu6klILves5IHHKqa9Try34GAx+C7qJuGivGjb6qig/yr1HcK+qW2hwHn3xLPOjD/prIf8AxyuFHeu4+JbDzdGA/wCekv8A6DXDjvX0mU/wH6/5HxnEP+9L/CvzYgpswLRuFzypAx64paK9R6o8ROzueeeEnt4LTVIpxtu1Ktlh8xUHkfgetN8VlXvdGS1Aa8CLv2D5u23Pv1pfGSWltrkMloxW7c5mVRxz3PuaseBYrSe7u7i4dnvkb5FkHRemR79vavm1Fup9V07X+d/vPtpTiqX1/Xvb1Sj93U78dKWiivpD4UZ/BXoHwu/5Amp/9hFv/Rcdef8A8FegfC7/AJAmp/8AYRb/ANFx15Ob/wAKPr+h9Fw9/vEvT9Ud5XlHxde4j1zwa9s8aTfbmVTIMryUHP516tkV5Z8WIjceIPBcK/ea/J/BSjH9BXzM7KEubaz/ACPsofEjEfX9S0q41KFLEyRQ7rq5BbBgL/3eMMpOXyOcE8ZFea/EtVWz0FIopBbxQvHHPINv2g/KWYKeQMnvjrXs2lW63Ntq003zPc3UyyZ7KvyBfphf1ryT4qTPcaJ4Rmc5LWkn4/c5/Gvm8vqQeLSjGzvZ+vK/+D8vPU7q8X7O7f8AVzzOiiivqTzwooooAKKKKACiiigAooooA9I+HV3ct4a16zjQSxRbLoqrASRsORIueDgoOM5r0CO51241TSbi8MMT6jblbZwvy2hKhnH+05AGM8da8u+GYdtQ1xEBJbSJuB/vJXt2q7ZNDsZYQG2T2rxEf76jI/An86+YzVqniEuVe89+14pfn96Vu530Nad77f5nL/CVdRv21HS21S9srZJprnNtsDzPvCtuYqeny9MdTXTeFbSPxJtu9SuHktJnkSOGXUJvODKAecNtf5Tk4AxWT4atPDKXXiWLV5WjjsdSZ0kjnkjOJsEp8hBYZTp7VXg1W7t/EGqP4W0i1heNytrE9u3mSgIWO1WORvABLYHbrzX0lOanBTXVI4pKzaLGpSg2FnbJKZYLXU72GB9+8eWMFQG7gBsfhVD+Bq3da0nV7bSImvjJJb21xE8byJGrKZUYSLhOMByv69awh91q+mylr2DXn/kfF5/FrFJ+S/NiGgkgMQMkDge9Bor1DwkeceHxbzvrEuoZ+37G2rJwRwd2B61N4jMFt4m06awI+2EjzVQ554Az7kZzVzxTYQ3ut/Z7UJFdJH500mcZUdsdzTvClhbWOq31lchJb6HDLPknKn2PQ818+qcuf2Gm/wAX4/efZyrQ9n9b12+HyaS+7qdsOlLRRX0B8SKP4a6vwHq0OlaLcLIkkkt3rBt4Y4xksxiQn6ABWJ+lcifurXd+G9E0258AK+qQb4ZZJLxsEqykE7WBU5B2gdK8jOGvZxXmfScOxftpy8v1KWoXJ128vdV0jxLfWdqJYbBZFh3Q+bvGcfQ4UnGMnqarfFWKeTxJ4JjguHhmN3MFlUAlflXnB4p2jWLnVbPTpba40nRdQf7daWSujh3Ta21jjcmcByvOeeeop3jq4iufiV4dsiR5lpa3F0oz1ZhtA/Q18ti58mHqS7J/kfZU1eaRy0+o65babrGpQLGtoZvImVF3bpMhHmj9unynvnmvOfifqU1xrdppssIhXT7ZY1jDbtoYBhk9CcbelewSBIvhowYBd9j09XYfzLGvFPidu/4WDqQbqFhH/kJK8TK6kamJa5UuXm/DlS/BnViE1Dfe36nI0UUV9IcIUUUUAFFFFABRRRQAUUUUAdV8O7y5tPGVqlrcRQvcK0OZlJRsjIVgOxIFeswabrlzZ6isUz202nXG23so5PMiwFDcEgHPzZXP3eB2rwKzuHtL2C5jOHhkWRT7g5r6j0+5jtr/AFY3EiRq7JdBmOBsMaqT+BU18/nM5UZKcEm2u3Zr9H/kdeFSk7MyvBt1Y2PxHjtbMBbHUdOjaHd1ZhuIJzzu4fOec10Hjy/XS9e0Wa4maxsZS8U99CAkiE42jfg4HcjjP6HgdQuJprj+2NFeGQ6FcSXWUO7ejSE7RjthGJ9mr2KTUJ9Z8MW+o6ILeaSZY5o45vuuuQWXPY4yM9jXpYGop0UnvHR9/K/qjKtG079ypHJb+MPA0n2OZnW4hKI7kFg6ngtjgHIBx2ry+FmMH7xGjkUlXRhyrDgg+4PFdBN4yh0O81R1Fraaje3CQtBGDNFaFdqtJMUwM/OOnoBnNZt/Bc3FouvkQtFPIy3DRKUUsGKidVPIR8A89D9a+gyzEqlU5ZbM+ezvBOvRVSC1j+RVopAc0tfSnxBzHiy0WQRXFuSuoqSkQX+NT94N7Ad/en+GbVVN1czOx1CR9txvGCh9APStO5tTJei5xlkgeNf94kH+QpbWzeDU764I5nWPB9xkH+lcCo/v/aW/q2/r0PbeK/2T2N+n6rT06+pdoooJGCSQMckk13njEiw3E8kOn2ylp7pxEmOxPU/QDJP0r1HXUudK8Lx2mlMyyK0NujqAWVC6qzKO5C5P4VgeAdDdm/t69UruXbaRsuCFPVz9eg9vrWR4k1SPXNWmNxpUs1jNbtZ6dMw3Is/m+WXPZMsQoJ54zjFfL4/EqtV93ZH3eT4N4ehea96Wr/Q6Pw7p8cnifUboX13qUdiogtri5kL+U5z5qr0BPC5P4dq4LV79dT8c+KLlVd3s44LSyaL7wn3NtA/4FnPtnNei3upT+C/h0tzfyCW9tbRY89fMmIwB78/nXm2hsPD09jZavcQRTvMb6Z5GC/6yNgM56kMpB+or5/MKvLQajq309NX/AJfM9zDxvO7LM2l6xZ6jpVisqXqujXEiXEhWGGRCCGVQMkDdwvtmvDvFF7LqPifUbmebzpDOymTbt3BflBxk44Ar6D8T37W51C5hkAksdMmdm7KWxtH1+Un8q+Za5MlcqkPazSvZfi2/ysXikoy5UFFFFe4coUUUUAFFFFABRRRQAUUUUAFeoeC7+48SaDLpD6nIL+xXzbaJo1O+Nedof72OMEe9eX1Z06/uNL1G3vrWQxzwOHRh2IrGvRVWNuq1XqVGXK7n02bS31Czi1rR1iiupYxIjY2rMpH3JAOo7eoNUdC8UWvhBPskUctxa6hEbrTbX+OOQsA8Of7oJz7YbrxWCnj/AE2x0VtV0y5tytxmZ9MuSUdHz82xgDkE54xj3FB0e7ms7j/hJVWDe6yafqFmd0dryWGTwRy3UjBr53A+1wc3OrdRvaz3a7W68uj087bnZV5aqtHf+vzOnuvCd/ousRavPJYz/abhQLUIQrTys2QWPIjDMG7nKjpxVyysltb/AF/U/EiQCbT5vOkltVZxNA0X+rww5X/Z9R+NWvD+ux+IbOTwt4piRdWRBkbsLdIOVljI78Z45BFR6j4dVtYnsZ/7VEvlImkXqvJKkB2nJcg9d3Xd1GBX00JxnFSi7pnE007My77wpI9rHrHh5HudPuEEq2rDEsan+7nqB6Hn0zWAZY/NaIKYpVOGjcFWH4HmvQbfxq1tHaXGp2ItdJuj5VrerJuMjgHrGBlQ2DjBParOuXfh3U/DrapJaQanCrKkYUAP5hcIFBOCp3EA9MV6mHzGpSXLLVHiY3JqFeXPB8r/AA+483AD/wAH60E7eq13Vl4J0zUrQSva6hpkoYq8BmDYIPY85Hoe9X4vhzoMY/fC7n9RJcMAfwXFdrzenbSLPLXDte+s1b5nmqSbplhhVppm+7FGpZj+ArrvDfgaa5kjvtcjEcY+dLLIJJ7eYRx/wEfj6V08Vx4W8M3MWmQy6fYXEi7kgBVXf39T0Nc7rnjbURpVtdWNjNaW88iyRXM4DefCAWYBQSVYqMrnqAeQa4MTmNSsuVaI9bBZPQwz5pe9L+uhJ478VDT1/sm1YfvY2S5MT7JYlIwNmeAeeD0yADjINJ4N0BLq3hurmZJ7G1lL2CxSELIf+ekqd5AfXoc+xrCis9djs7DWtUihvPDunQbljZ8TSQMjKzOjL94K2SNxzjiqtwraTf3lh4Z1h/LuYhJPKWxHYwso+Z/70u0YXocdema8yc4U4Oc3ZI9lJydkanifWIdf1aT7PMlxa6RcpDDAD8kt43AZj3VM9u+fSo9T06LTtGu5JAlzqt0nkLcSICzyP8qgeignoOgFc5cR3WjW0OpaDYomi6fF50/2xijXTLuw68E5O48nGeKpav4/sE0oam+oW8+oBT9jsrXLLA7DG9iQNzAZ4OP6183iY18TXVWnrG+3Vdou23d+uuqSO6HJThZ7/wBanK/EPUTpkEPhm01d7tIwDdhY1Vd4xgMw5ZvqfSvO6dI7SyNI7FnYksT1JptfRUKXs4KLd31fd9zilJyd2FFFFakhRRRQAUUUUAFFFFABRRRQAUUUUAdh4H8YjQLj7Bfwx3Gk3LYmV0BKZ4yPb2r3HRdRtxarpd9Kh2x/uJXI2XMB+6yk8E44I6/nXy9Xa+F/GcsNmuhatdIulkFY5pLYTNb59M9vzxXkZllqxC5o79f815+XX1SOijWcGd9c29nql7bxpfT2y2iTf2bqbI6Ip3IUXeeGx869egrt9A+IVxYyx6T4xjW0ujhYr9T+4nB6HPQH/PFY3hV7XRLSLR2uxd6bMN9jdsBtk3ctGewOckDuD7VF4ltYbJJtHgt3uob62klhs1iL+XImCCvYKSQCO3Hqa4aGOlTr+xirx6X6rq/J9137G9SipR5up6HqGmWlpZrq1isL/wBnwtJbRSSH7Og5LOAoPzbSwB5ry3XBeJY6/e3UBuLW8niW7ltgwS23hZcberDiJW6c56ZqWFH05GttJ1C6022ugY20rV4WNu4YYKq38OfY0mn6zqOneGbzQr/w/fOUvVluriCUTOw3q+cHBKlV2g89Oa9qjjKNVfFZ9np/w/yOV0ZxNGbxZrGhaTotpp05tYVhlyLm3kkLRBtqyjcNwUKGYKecAZJ77Metw+J9Q1KaXUr9tBsYEnzbxvE4dhjblOW4AYAf3uegq9afFHw3fSIjWWoC4KkBGsyzY7jjP5VXb4o+GdMRrew0nUGO8gw29mE+b6ZHNdXMrXM7Gfp/hzxXcxKS0Qh1CZbma5nIE6BQqorqVOcKucDHLexzr3fgLT9Ksr28tNSuIJkjzbG6nHlQMpDLk4BIBUDknAJArMuviD4iu7qC20zw0LTzYzKZtQmAESDjcyr09hnNcvqgl1+C4m1K91HxBcFGEUFlAyWkbYwD2DY9cmuapjKNP7V35a/e9l82aRozZvXvxA1HxRp50/QoIrXcm2+1Kdg0EIPBCE8Oa5/Ro9OtdSk0+Wa4awlvvMNzLGxS7fy0CgyEYPz7zjPUV0WjW9lqMszvkWunOLeG0eIosZVQd7Ajljn6Ae9YviyWw16Hfc6j/Z+j2TbxclAyzzDsoP3lUZ7dT7V4k8wniazpSTUfLo3t0u32tt07nUqKpx5lua2v6vZTBoJJUOm2riXUJ8goFXlYgehZjjI7Dr1rwnxf4tuPFOo+Z5SW9lESLe3RQAg9T6mrHi3xlc67FHp1vIqaXAcxxxwiIMfUgE1ylehl2XRw0U2tenl5+r/Bad781as6jCiiivVMQooooAKKKKACiiigAooooAKKKKACiiigAooooA6Hw14vv/DXmwxxw3VjP/rrScZRvceh969C8P614e1LUbW+t9W/s3VY1KQWshYw8/wsz5LA8Zxj9K8corlrYSFS7T5W97dfVbP8/MqM3HY+qG1aGW0aHU9NukYriSPyDKh45wyggj8q5Tw9q1tqMt1cPq2oR3ETPFFHDDgvAGOwgFSW47nnrXjdh4m1m0WOAavfrZL8rQLOxXZnkBScVsnx+812VudNSTTWGxrQTMuV6ZLDG5seuR6AV5UMn9jGUY637f5Pv6/M6ninJps9Lv7m/u1KLFdXmmxkPcvcrEJ0RSCTHsO7OM9ga6TTdMu7qxhmF2dOgkUNFa2UaAIp6ZYg5OOuK8U1vxfo7aUtn4f066tJM4M08uSi+i4PX3JrS034kadFokdpfaffNLGgTZb3ZSJ8e2fl/Csq+XVpUUqcba7WX32vYqNeClqzuNYvbPTPENnatqd5fQ3Uwjv1aPzVwqnZHlRwSxHy9+c11c+suYDFp1jNvAwJJ4jFDEPVicdPQfpXiQ+KWoPD9gNnb2+ltkPDbRruAPcFgec8/h+NczqvibXNWgW2v9Vubi3XlUd+D9QOv49KbyedXkVSy5fPfzsktelr7W1J+tct+U7/AFTxF4Z0Oe6ltr6TXrmebzJ4pCyozdzuU7SM44IPH0rgPEXiXUPE16txfGNVjXbFDEu1I19AKx6K9ulhYU3zby7v9Oi+Ryym5bhRRRXQSFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB/9k=</t>
+        </is>
+      </c>
       <c r="N29" t="inlineStr">
         <is>
           <t>Administration &amp; Operations</t>
@@ -3014,7 +3094,11 @@
           <t>MHAA</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEAYABgAAD/4QA6RXhpZgAATU0AKgAAAAgAA1EQAAEAAAABAQAAAFERAAQAAAABAAAOxFESAAQAAAABAAAOxAAAAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCADnANMDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD5/ooooAKKKKACiiigAooq/pOmtqF2qkMIVIMjD09B70m7K5dOnKpJQirtnbeGvhtB4kvJLOC9EVwqb1WWbb5g74+Q9K6v/hni+/5/Yv8AwI/+11z9pdz2N3DdW0hjmhcOjjsRX0H4P8UQeJtGW4Xal1H8txCD91vUex7VjRq86s9z081y14SfND4H+HkeO/8ADO99/wA/sX/gR/8Aa65jxN8Lf+EXuIIbydm85CytHMCODgjlBX1YThTXm3xftTNo9neqmTbzmNz6KwP9VH51pUbUW0cOEjTnXhCps3Y+f/8AhFrL/nrP/wB9j/4mj/hFrL/nrP8A99j/AOJrdorh+sVO59h/YWC7P72SeGPhO3ik3H2OZkWDbuaWYDOc+iH0rov+GeL7/n9i/wDAj/7XXo3wjsjB4Xnuz/y83LbT/sqAv8w1ehHmu+Dbimz47FRhGtKNPZN2Pnf/AIZ4vv8An9i/8CP/ALXXK+JfhrB4bvY7Oe9Ek7JvYRTbtg7Z+Qda+j/F/ieDwxorXB2yXMmUt4ifvN6n2HU189Xd3Pe3kt3cSGSeVy7uepNZV6vIrLc78qy54ufNP4F+PkeX0Voavp0lheP8v7l2JjYdMelZ9bJ3PMqU5U5OElZoKKKKZAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB1GgaRZ3Fgt1PF5jliOW4HOOldBHHHDH5ccaxqP4VFdT8KvBVn4o+Hl3IW8i+ju3WKcDI+6vDDuP1rM1zw/qPh69+zahAUJzsccpIPVT3+nWuHEQne+6PrMkxWF5VTsoz79/n+hl1seG/EN14a1mO/twXUfLLFuwJE7j6+hrHp0aNI4VASx6AVzwclJcu57mKp0qlGUavw9fLz+R9MWOqW2p6ZDf284a3lTcGPGPXPoRXIeOvEWmal4evNJtpDcXMgXa0a5RWDAjLHjt2zXA6dDdWumNaPdTfZpG8x7cNhN2PTv/KrR2sMfdr6zDZVKpHmraX6H4xj88hQquGE96z+Lp8kc/HoUxi3SSIjegBb/AAofQZRHuSVGb0II/wAa6S3tpLy6hgX70rhR7Zpbm1ezvJ7cnPlOVzjriuj+ycDfk5dfVk/63Z5/G9rpftG3psdj4L8RaPpug2WkzyG1mhTDGVcIzEkkhhx1J64rrb/VbXT9Mmv7iYLbxJvLAZyO2PUntXjm9NuCM1U1OO9udNSziupPssb7xblvkz7en8qwxWVyhFyo626Dy/O4Vqqhi/du/i6fNGX4l8Q3PiXWZL+4yqfdhiJyI07D69z7/hWPSspVipGCOCKSvkptuTctz9pwtKlSoxjS+H8/MHjSWPbKgZfQisHXdMtI9KaaKJI3hI27FAyCQOe5/Guy0TQdR8QXwtbC3LkYLueEjHqx7fzpPjD4Rt/CmiaGiyNNdzyS+fKeAcBcADsOfrXRh4TvfZHhZ1isLyunZSn+Xz/Q8ioooruPkwooooAKKKKACiiigAooooAKKKKACiiigD6c/Z3/AOREu/8Ar/b/ANBWvTdU0ix1eya0v7aOeFuqsOh9Qex968h+Aet6ZYeEriyu72GC4kvGdElfbuGFHGfcV7arq6hlIKnoQaB6o8F8V/Dy+0INdWQe80/PLAZki/3gOo9x+NZOiWa7GuXwd33fpXvmu332DQ726QDckR25/vHgfqa8YgjWOFI1GI0GBXoZVgoSrOs1t+ZwcQZ9iVglgub4t31sunzYuMtxWpp+h6jqkRks7YSoDgkSKMH6E1l5w3y1e0vVLnSbxbm2l2kcMhHDj0NfQ1vacr9na/mfDUPZe0Xtr8vludV4V8M31lrQur+ARpGhKfOrZY8dj6Zpni/w/d3GtfarK1eZZUBfYOjDj+WK7XS7wanp9vd7Gj81A2xu1N1W9Gl6bPeFGk8tc7V/z0r5tY2v9Y57e9tY+veWYb6n7O75fiv1/LseTXWk3tjFvu7VoUJwC7AZ+lUAdrcVf1HUptWvGubqTJ6Kg6IPQVQ6txX0tHn5f3m/kfH1vZc7VK/L5mRrtkFQXSkDPDf41s+Efh3fa/tu70PZ6eTwxGHlH+yD0Hufwpk0e+N8fdI9K9n0a8GoaJZ3Zx+9iUnAxz3/AFr5zNsFCNdVkvi/M+74fz7EvBPB83w9etn0+RLpekWWkWi2lhbJBCv8KjqfUnqT9a8a/aV/48fDv/XSf+SV7lJIkMZeR1RByWY4Ar58/aD1rTtUt9EhsbyK4eB5TJ5TbguQuORx2NcB3as8MooooEFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAdr4c/5AkYPQu2fzrp9M8Qavo4VdP1C4gjU5EavlP8Avk8fpXL+HCP7Fj5H32/nWtkeo/OvNquUajsfc4KlQq4OmqqT06ncf8J/rGuWn9l3wt2R2DGVFKtgc4I6H9KT/V7TXL6Lg6rDhh1P4/Ka6b7w+lfX5E3LDNve7/Q/JuNaVOjmfs6XwqK/G4nU1Pa2xub6G2A/1jhfzqDo1PRnWRZI2ZHXkMpwRXsTu07HyUGlJOWx6HrfiaHSYBp+nlWmjUJu6rEAMfiaXRvEcOtW76bf7VmlQoD/AAyAj9D7V5wX4yzfUk0Kw4dH5ByCDXmf2ZS9ny/a79bns/21X9t7R/Bty9Lf5+Y+VGt7mWF/vRuVP4Gm0hZnYsxLMTkk9TS16avbU8SVr6CY4pF+IGt6RZLpNkbeKOAsBLs3OdxLd+Bjdjoaf9zbXJ6kR/a93yP9YO/+yteLnzccPFx3v+jPsuCKVOtmMqdVXjyt/c0SalrOpav/AMhG+nuRnO2VyVH/AAHp+lcl4r/48rb/AK6H+Vb+R6j865/xVj7Hb8j/AFh/lXydFydRNn6nmdOhSwNSNJJbbeqOVooor0T4kKKKKACiiigAooooAKKKKACiiigAr03VPh0ll8LbfVlQ/wBpoBdT/wDXNv4fwBB/OsLwL4Zs/EyatFcSNHPbwLLA+flBBJOfbAr127i1TUNGtra7KQ2WrqLaSE8m1Vh8pBxyxAIOehYenPj47GShWhCnK1neXmrXt91/mvQ6KVO8W2t9iX4A6bZXfge6kubSCZxeuA0kYYgbV9RXrH9h6T/0DLP/AL8L/hXEfCPTrbSdI1qxs1b7PBqbpGWOSwCIM16P2r04SUoKceupg1Z2PNPiFaWWnafpctvZRRubsqTDEqk5jfjtxmuW+xajs/5Bl1/3yv8AjXa/EqIHT9LRuQbtsg9/3T1yEXia706ELcwrdQghRIZNjJk4+Yngj3rqqYjMsNhfa4GMZJN3T32Wq1R4mJoYCvi/ZYtuLaVmtt3psV/smp48v+y7z/vlf8aZJBeW8XmT2FzFGCAXdRgZOBnmujk1fVP7TW2FrZWryJviknuGcSeoACjkcHGe9OjM+oJfaRq/kmXYGDwKVVkboQCTyGB/SvEhxfmEbSqwhy6N2ve19ba2O6XDGBaag5X/AF+4f4D06yvdQvLi8SOWeBVEKNztU9Wx65GM9vxqLxxYWVhrFrLZrHFJcRsZokGAcEYbHY8ke+PasLTxdaZ4k06GV2juVuYlLISBIjOFJHqD3FJLHPqviC7jR2e4klfzJSc+WgYgE/QDgV9S8RQVX677ReztzX8trHkeyqvBfU/Z+/flt573+4iit725iWSCxuZIm+66qMH6c082Wp7Nn9m3Z99o/wAa6SeW5tpbTS9HMCvHF5kjXCllWMcDoRyT/I1DBrGrG/mtzaWdz5ChpZobkqqE/wAJyp5xz16V8rLi7MZXlThC26ve9r6X1sevHhjApJScr/r9xhmx1ER5OmXf/fK/411fw4s7HUdF1G4msoZXN+wBmiUtgRx+tcvL4ivNYtNsUAtbVwQSH3O49iOADXZ/DOMHRNSVDhRqDAD/ALZx17sK+Y4jCqpj4xjdqyW+z1erOPCUMDRxcqeEbk0ndvbdabHXf2HpP/QMs/8Avwv+FeIftE2NpZ2Ogm2tYYS0s27y4wueF9K99615f8VdEsvEOseHtOv1YxS/aQGU4KsFUg/pXJOrGEHUlslc9qMXJ2R5Brfw5TT/AIaWeuRhxfRqJbtSc5VyMcdsZH6mvNq+hr5tWvPCNzJI8L2lyhsvKXhY4z+7E2cZ65JHoR6V5B490O08OeJP7Ls9xSGCPczdWYjJJ/OvOy3FTqOUKsk5XbVui0uvk3Y1rU1GzjscxRRRXrGAUUUUAFFFFABRRRQAUUUUAegfDLiDxE6OBKLLCpnlxyWAHfgV7Nq1zbS2dnDDLGzNcQMAGHyqCHLH0G1Sa8f+GCW0um+Ixc5zFDHLCynDI4LYKnsSdo9+hr0d/C1npv8AYc8oLsZRBeY484vyM/7IcAbemOOgr5bMlSli7zbTT00391P+vU9ChzKnp/Wp1nwsnhuNP1ySCQSRnVJMOOh+Va9B715x8JJjcafr05GPM1iYj6YGP0xXo/evpKStTin2Rwy+JnBfE0/6HpQ9bpv/AEW9eflQ6srAFTwQa7/4mn/RdIHHNy3/AKLauCH3Gr6nKf8Ad36/5Hxef6Ytei/NkGoM/wC5t5r25k0oPiaFNrFVxjK5BIwcHj8K1reCC1niMWsSSzIP+JddTz7o3U4zC+O/HfnoRyDVD7vDLUUVjJqFw8VnpwufJxJcbVBManoQP4m44ArxM1yGjVftKc1TXVWVn5+vR90ehlOeV4pUJQdR9HfU3L7WbK7vdNtLmMW+qRahbsIXwSR5i5KMOGH+SKj0jWLO3imsrCJLjUpLmZ5I1woX942Gkbtx+PoKzWtbfTvFn9n7FeW0urfMnlFM5ZT3pljYRarqgtAipNMJpQ3kGQnbzjj1z3NeW+HKP1T2Htfd+K9nbta172v5/M9dZzU9r/C96/La67XvfYu3Fpa3Us3m61Miuc6lcxTbUc4IESfTPbsPU1lwCSe2ltRdXK6czHyoH2p8nbdtA6+/4046fLZXCW95p62s7J5sQ2j5kP8AFjsexB6Gpz12EfPXrZTkVGg/aVJe0XTRWXn69PJaHj5vnleX7mEXTfXXX/hhVUBNqgBQMADtXf8Awu/5Aup/9hFv/Rcdef8A8FegfC7/AJAup/8AYRb/ANFx162b/wAGPr+hxcPf7xP0/VHc1578QJoIfFHhVp5ViUvcAMxwM7VxXoXavOPiJt/4SrwjHIivFNLcxOjLkMCg4I/KvlMWr4Wp/hf5H2dL416mXDcWsfgWW3lZBJHZvG8efmBGV6f71eL/ABSwfGRbzUkY2sO/ac7WC4IPvkV6f/wjcMvhq51W3aQXZna5jdvmZY1+UJk9flGQT0bB7V5p8VoLW18UWsFnGqQpYRYx3yWOSe5OeteJlKoxxMuRtt81/La/9dTsxHN7NX8jhqKKK+lOAKKKKACiiigAooooAKKKKAPQfhvHKtnrDbMLOsaQuWwGlRvM8sf7RA4r1W98TWWp3NjbWyzN5c0d0fkx5igEqEz94luP+At6V5x8Nwtx4U1eweMSC8vILdQwyFL5y31Cgn8K9Wu7GKz8Q6LPbxouFks8BRwmwsMfQp+tfKZlOksRJzWqvb5RX/Dep6NBS9mu3/BND4RxPDo2rpIgjcalJlA27b8q8Z716N2rzX4MytP4Z1CZzlnvmZj77VzXpNfUQTUUmee9zgfiX/qtH4/5eHP/AJDNcCv8Vd58S/u6OM/8t5P/AEA1wg719NlP8B+v+R8XxD/vS/wr82OB8tq4bWtb1bwv4oe+0y9ltvtMCxvsP3lHUc9+4Pau2PI3Vn61oVtrNjsnBV15R16qa6MbQdelyx33ObK8XHC4hTns9GSabeWt1HaXNowffcRO7E5YtvBO49c/Wq1zqltZ6RHeTuYpUG+J0bDh+209c1wGnrLovim3s4b0yoLmMSmNSFOGGQR7VFa2Uuva59iub0xYJEfmKeg6AD6V5X1yTnyqGtuW3Tc9/wDs2EYc7qPlT5r63tY6Xw1rWreJPEk+p6reSXMiQeWGfoo3DAA6Dua7U8S5qnpmkW+l2Cx264A5Zz1c+pq5/wAs8162DoOhRUJbnz+Z4uOKxDqR22E/5Z16D8Lv+QJqf/YRf/0XHXn3/LOvQfhb/wAgXU/+wi//AKLjrkzf+FH1/Q7uHv8AeJ+n6o7gV5z8Rt6+JPCkqQNMYpZ3KKQGICr0z1PfFejCvOfiTKyeJ/B+08tdyL+BCg18tX/3ef8Ahf5H2NP416nO23iWxstDm0keZJcRK0ceEO1y7ERjPYnPQ9Np9K8l+JmZNetZ0XdbC0S3jnA+WUx/KxU9wDxn2r2i10a01XSdaM0SFtTuJd529Nh2L+WzP1NeS/FG6S7i8PSRxiNfsZG1RgKQQCB9CDXg5VKksTJU073d/W1/zTO3EKXs9TzyiiivpjgCiiigAooooAKKKKACiiigD034fXD2HhLULt42jijvEmjuQpZfMjAPlsByMhuD05r0NNU1bU9bjE1gtvc2cTTW6MxZFWReJJCO4GV2juT25rjvhqC3gG4hLYjuNahhf/dPl5H49Pxr0jVoyviPSXiOGnSe2kA/iXZuH5FR+dfK5lWgsRJSir+9r6RX5q6f6Ho0IvkWvYX4EtJJ4LupJSC73rOSBxyqmvU68u+BoMfgu6ibhorxo2+qooP8q9Q3CvqVtoeceffEw/Pow/6ayH/xyuEHQ13PxLYGbRgP+ekv/oNcP619LlP8B+v+R8bxD/vS/wAK/NiCmzBmjcDPKkDHrilor03qjw07O5554Ra3gtNUinG26UhssOSoPI/A9ab4sMb3ujJbYa6CDfsHzdRtz79aXxmlnb63DJaOVu3OZ1Ucc9z7mrHgWK1uLy6uLh2e/RvkWQdF6ZHv29q+bUW6n1XTtf53+8+2lOKpfXte9vVKP3dTvx0paKK+kPhSMfdr0H4X/wDIE1P/ALCLf+i468+H3a9B+F//ACBNT/7CLf8AouOvJzf+FH1/Q+h4e/3iXp+qO8ryj4uvPFrng17Z40m+3MqmQZXkoOfzr1bIryz4sRGfxB4LhX7zX5P4KUY/oK+ZnZQnfaz/ACPs4fEjEfX9S0q41KFLAyRQ7rq5BbBgL/3eMMpOXyOcE8ZFea/EtVWz0FIonFvFC8cc7jb9oPylmCnkDJ74617NpVutzbatNN8z3N1Msmeyr8gX6YX9a8k+Kkz3GieEZnOS1pJ+P3Ofxr5vL6kHi0oxs72fryv/AIPy89Turxfs7t/1c8zooor6k88KKKKACiiigAooooAKKKKAPSPh1eXLeGteskQSwxbboqrYkjYDIkXPBwUHGc16DHc67cappNxeGGJ9Rtyts4X5bQlQzj/acgDGeOteW/DPedQ1xEBJfSJxgfVa9v1bbJodlLDhtk9q8RH++oyPwJ/OvmM1tTxEVyr3nv2ukvz+9K3c76GtO99v8zlfhIuo38mo6W2qXtlbJNNc5ttgeZ94VtzFT0+Xpjqa6fwraR+JNt3qVw8lpM8iRwy6hN5wZQDzhtr/ACnJwBisnw1aeGkuvEsWrytHHY6kzpJHPJGcTYJT5CCwynT2qvBqt3b+INUfwtpFrC8blbWJ7dvMlAQsdqscjeACWwO3XmvpITU4RmuqRxSVm0WNSlBsLO2SUywWup3sMD7948sYKgN3ADY/CqH/ACyat3WtK1e20eJr4ySW9tcRPG8iRqymVGEi4TjAcr+vWsIf6tq+mylr2DXn/kfGcQRaxSfkvzY6mMTgkDJA4HvT6ZXqHgI848PiCeTWJb/P28I+0ScEcHdgetTeIzDbeJdNmsCBeEgSrGc88AZ9yM5q34psYb3Wxb2qpFdJH500mcZUdsdzT/CthbWOrX1lcBJb6H5lnyTlT7Hoea+fVOXP7DTf4vx+8+0lVh7P63rt8Pk0l93U7YdKWiivoD4kUfw11fgPVodL0W4WRJJJbvWDbwxxjJZjEhP0ACsT9K5E/dWu78NaJptz4BVtUg3wyySXjYJVlIJ2sCpyDtA6V5GcNezivM+k4di/bTl5fqUr+5Ou3t7qukeJL6ztRLDYLIsO6Hzd4zj6HCk4xk9TVf4qxTyeJPBMcE7QzG7mCyqASvyrzg8UaNYudVs9OltrjSdF1B/t1pZK6OHdNrbWONyZwHK85556in+OriK5+JXh2yJHmWlrcXSjPVmG0D9DXy2MnyYepLsn+R9lTV5pHLT6jrltpusalAsa2hm8iZUXdukyEeaP26fKe+ea85+J+ozz61aaZLCIV0+3VFiDbtu4A8noTjb0r19wkXw1YMAu+x6ersP5ljXi3xP3f8LB1EN1Cw/+ikNeJldVVMS4qKXLzfhypfmdWITUN97fqchRRRX0hwhRRRQAUUUUAFFFFABRRRQB1Xw6vLm08ZWqWs8UL3CtDmYEo2RkK2OxIFeswabrdzZ6isUz2s2m3G23so5PMiwFDcEgHPzZXP3eB2rwOyuXs763uozh4ZVkXPqDmvqLTrmO2v8AVvtEiRq7JdBmOBsMaqT+BU18/nM5UZKcEm2u3Zr9H/kdeFSk7MyvBt1ZWPxIjtbMBbHUdOjaHd1ZhuIJzzu4fOec10Hjy/XS9e0Sa4maxsZS8U99CAkiE42jfg4HcjjP6HgdQnmmnOsaM8Mh0K4kusod29GkJ2jHbCMT7NXsUmoT614Yt9R0QW80kyxzRpP911yCy57HGRnsa9LA1FOik946Pv5X9UZVo2nfuVEkt/GPgaT7HMXW4hKI7kFg6ngtjgHIBx2ry+FmNuPMRo5FJV0Ycqw4IPuDxXQTeModDu9UdRa2mo3twkLQRgzRWhXarSTFMDPzjp6AZzWbfwXNxaL4gIhaKeRluGiUopYMVE6qeQj4B56H619BlmJVKpyy2Z89neCdeiqkFrH8irRSA5pa+lPiDmPFlosnlXFuWXUASkQX/lop+8G9gO/vT/DNqFN1czO51GR9tyHGCh9APStO5tTJei5xlkgeNf8AeJB/kKW1sng1O+uCOZ1jwfcZB/pXAqP7/wBpb+rb+vQ9t4r/AGT2N+n6rT06+pdoooJGCSQMckk13njEiw3E8kOnWylp7pxFHjsT1P0AyT9K9R1xLnSvC8dppTMsitDbo6gFlQuqsyjuQuT+FYHgHQ3Zv7evVK7l22kbLghT1c/XoPb61keJNUj1zVpjcaVLNYzW7WenTMNyLP5vllz2TLEKCeeM4xXy+PxKrVfd2R93k+DeHoXmvelq/wBDo/DunxyeJ9RuhfXepR2KiC2uLmQv5TnPmqvQE8Lk/h2rgtY1BdT8ceKLlVd3s44LSyaL7wn3NtA/4FnPtnNei3upT+C/h0tzfyCW9tbRY89fMmIwB78/nXm2hsPD01jZavcQRTvMb2Z5GC/6yNgM56kMpB+or5/MKvLQajq309NX/l8z3MPG87sszaXrFnqOlWKypeq6NcSJcSFYYZEIIZVAyQN3C+2a8O8UXs2oeKNRuJ5vOkM7KZNu3cF+UcZOOAK+g/E9+1ub+4hkAex0yZ2bspbG0fX5Sfyr5lrkyVyqQ9rNK9l+Lb/KxeKSjLlQUUUV7hyhRRRQAUUUUAFFFFABRRRQAV6j4K1C48R6FLo76pIL6xXzbWF41O9F52h/vYOMEe9eXVZ06/uNL1G3vrSQxzwOHRh2IrGvS9pG3Var1KjLldz6bNpb6hZxa1o6xRXUsYkRsbVmUj7kgHUdvUGqOheKLXwgn2SKOW4tdQiN1ptr/HHIWAeHP90E59sN14rBj+IGmWWitq2mXNvtlzK2mXJKOj9/LYA5BOeMY9xQdHu5rO4/4SRVg3usmn6hZndHa8lhk8Ect1Iwa+dwPtcHJzq3Ub2s92u1uvLo9PO252VeWqrR3/r8zp7rwnf6LrEWrzyWM/2m4UC1CEK08rNkFjyIwzBu5yo6cVcsrJbW/wBf1PxIkAm0+bzpJbVWcTQNF/q8MOV/2fUfjVrw/rsfiGzk8LeKYkXVkQZG7C3SDlZYyO/GeOQRUeo+HVbWJ7Gf+1RL5SJpF6rySpAdpyXIPXd13dRgV9NCcZxUou6ZxNNOzMu98KyPbR6x4dR7nT7hBKtowxLGp/u56geh59M1gGaPzWiCGOVTho3BVh+B5r0G38atbR2lxqdiLXSbo+Va3qybjI4B6xgZUNg4wT2q1rl34d1Pw62qSWkGpwqypGFAD+YXCBQTgqdxAPTFeph8yqUlyy1R4mNyahXlzwfK/wAPuPNwA3RP1pCcdVrurLwTpmpWgle11DTJQxV4DMGwQex5yPQ96vxfDnQYx++F3P6iS4YA/guK7Xm9O2kWeWuHa99Zq3zPNkfdMsMKtLM33Yo1LMfwFdd4b8DTXMkd9rkQjjHzpZZBJPbzCOP+Aj8fSumiuPC3hm5i0uGXT7C4kXckAKq7+/qehrnta8baiNLtrqxsZrS3nkWSK5nAbz4QCzAKCSrFRlc9QDyDXBicxqVlyrRHrYLJqGHfNL3pf10H+O/FQ09f7JtWH72NkuTE+yWJSMDZngHng9MgA4yDSeDdAS6t4bq5mSextZS9gsUhCyH/AJ6Sp3kB9ehz7GsKGz12Oz0/WtUihvPDmnQbljZ8TSQMjKzOjL94K2SNxzjiqs6NpF/eWHhnWH8u5iEk8pbEdjCyj5n/AL0u0YXocdema8ypKFODnN2SPZScnZGp4n1eHX9XkFvMlxa6RcpDDAD8kt43AZj3VM9u+fSmanp0WnaNdySBLnVrtPIW4kQFnkf5VA9FBPQdAK5u4ju9GtodS0GyRNF0+Lzp/tjFGumXdh14Jydx5OM8VS1fx/Yx6Wupvf282ohT9js7UFlgdhjexIG5gM8HH9a+axMa+JrqrT1jfbqu0Xbbu/XXVJHdDkpws9/61OV+IepNplvD4YtdXe6jjAa7URqo38YDMOWP1PpXndOkkeWRpHYs7EliepNNr6OhS9nBRbu+r7vucUpczuFFFFakhRRRQAUUUUAFFFFABRRRQAUUUUAdh4I8YjQbj7BqEEdxpNy2JldASmeMj29q9y0XUbcWq6XfSoSkf7iWQjZcwH7rKTwTjgjr+dfLtdr4Y8aTRWSaDq12i6WQVjmkthM1vn0z2/PFeRmWXLELmhv1/wA15+XX1SN6NZw0O+ubez1S9t40vp7ZbRJv7N1NkdEU7kKLvPDY+devQV2+gfEK4sZY9J8YxraXRwsV+p/cTg9DnoD/AJ4rF8Kva6HaRaO12LvTZhvsbtgNsm7loz2Bzkgdwfao/E1rDZJNo8Fu91DfW0ksNmsRfy5EwQV7BSSAR249TXDQx0qdf2MVePS/VdX5Puu/Y6KlFSjzdT0TUNMtLSzXVrFYX/s+FpLaKSQ/Z0HJZwFB+baWAPNeWa4LxLHX726gNxa3k8S3ctsGCW28LLjb1YcRK3TnPTNSwq+nI1tpOoXWm210DG2lavCxt3DDBVW/hz7Gk0/WtR07wze6Ff6BfOUvVluriCUTOw3q+cHBKlV2g89Oa9qjjKNRfFZ9np/w/wAjllRnE0ZvFmsaFpOi2mnTm1hWGXIubeSQtEG2rKNw3BQoZgp5wBknvsx63D4m1DUp5dSv20GxgSfNvG8Th2GNuU5bgBgB/e56Cr1p8UfDd9IiNZagLgqQEazLNjuOM/lVdvij4Z0xGt7DSdQY7yDDb2YT5vpkc11cytczsULDw54ruIkJaIQ6hMtzNczkCdAoVUV1KnOFXOBjlvY51rvwFp+lWV7eWmpXEEyR5tjdTjyoGUhlycAkAqByTgEgVmXXxC8Q3d1Ba6Z4aFp5sZlM2oTACJBxuZV6ewzmuX1QS6/b3E2pXuo+ILgowigsoGjtI2xgHsGx65NctXGUYfau/LX73svmzSNGbN6+8f6j4o086foVvFa7k232pTsGghB4IQnhzWBokenWupSafLNcNYS3/mG5ljYpdv5aBQZCMH595xnqK6HR7ey1CWV3BFrpri3htHiKLGVUHewI5Y5+gHvWL4slsNfh8y51D+z9Hsm3i52BlnmHZQfvKoz26n2rxJ5hPEVnSkmo+XRvbpdvtbbp3OqNFU48y3NbxBq9nOrQPKh022YTahPkFAq8rED0LMcZHYdeteE+L/Flx4p1Hf5SW9lEcW9uigBR6n1NWfFnjK51yNNOt5FTS4TlI44REHI6EgE1ydejl2XRw0U2tenl5+r/AAWnc5q1Z1GFFFFeqYhRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB0Phrxhf+GvOhijhurKf/AF1pcLuRvceh969D8P6z4d1PUrXULfVv7N1aJdkFrKzmH/dZnJLA8Zxj9K8borlrYSFS7T5W97dfVbP8/MqM3HY+qW1eGS0aHU9NukYriSPyDKh45wyggj8q5Pw/q1tqMt1cyatqKXETPFFHDDgvAGOwgFSW47nnrXjdh4n1m0WOD+178WS4VoFuGK7M8gKTitpvH7zXRW501JNOYbGtRMykr0BLDG5seuR6AV5MMn9jGUY637f5Pv6/M6niuZps9Lv7m/u1KLFdXmmxkPcvcrEJ0RSCTHsO7OM9ga6PTdMu7qxhmF2dOgkUNFa2UaAIp6ZYg5OOuK8U1vxdozaUtn4f026tJM4M08uSi+i4PX3JrS034j6bDokdpe6dfGWNAmy2vGSJ8e2fl/Cs6+XVpUUqcba7WX32vYca0FLVncaxfWemeIbO1bU7y9hu5hHfq0fmrhVOyPKjgliPl785rq59ZcwGLTrGbeBgSTxGKGIerE46eg/SvEl+KN+8H9ntZ29tpTZBhto13KD3BYHJzg/h+NczqfibXNWgS3v9UubiFRwjPwfrjr+NN5POryKpZcvnv52SWvS19rai+tct+U7/AFPxF4Z0Oe6mt7yTX7q4m8yZJN0aM3c5U4xnHykHj6VwPiLxNqHia8S4viirEuyGGJdqRr6AVjUV7dLDQpvmesu7/RbL5HLKbluFFFFdBIUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFAH//Z</t>
+        </is>
+      </c>
       <c r="N30" t="inlineStr">
         <is>
           <t>Research &amp; Data</t>
@@ -3102,7 +3186,11 @@
           <t>BRAC</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEAYABgAAD/2wBDAA0JCgsKCA0LCwsPDg0QFCEVFBISFCgdHhghMCoyMS8qLi00O0tANDhHOS0uQllCR05QVFVUMz9dY1xSYktTVFH/2wBDAQ4PDxQRFCcVFSdRNi42UVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVFRUVH/wAARCACWAbEDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD0puFJxzjNeb3HiDVYb2cJeEBZGGCq8c16Q3+rb6V5Jff8f9zx/wAtW/ma2opPc9fKqcakpKSudBZ+NLyNv9JhSZP9n5SP8f0rp9L1+x1L5YpNsmOY34NeY9KVSyuHRirA5BHUVtKkmejXyulNXhoz2MY44pfwrkPC/iJrhhY3jZl/gf8AvV1341yyi4ux85Woyoy5ZDqKKKkyEpvWlZgoySBWNf8AiPTbAsjzb5B/AnJz/Smk3sVCnKbtFG1RXEXPjeQki2tMDszt/Ss+TxfqzdHiT6J/9etFSkzuhlteXQ9HzRmvMW8T6yScXm3PQBF/wpP+En1n/n+P/fC/4VXsGaf2TXPT80ZrzD/hJtZ/5/j/AN8L/hR/wk2s/wDP8f8Avhf8KPYMf9k1/I9OzS5rzD/hJtZP/L8f++F/wp8XiPW3lSNb45ZgB+7X1+lL2LJlldaKuz02imISVBPXFPrFnmNDeOKKyPEt5PY6PLcWzBZFK4OM8ZANc3YeM7mJtt5Cskf95OCPzq1ByV0dNLCVKsOeB3fTpRxVWxvIb2BZ4HDIwyMGrXQ5qWrbnO007MdRRRSEFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAMf7jfSvIr7/j/uf+urfzNeuv9xvpXkV9/wAf9z/11b+Zroont5P8UiCiiiuk+iHo7xSK6MVdTuBHY16pot6NQ0uC47svI9D3ryj3rvPAcpfTZYichJDj6cf1zWFZXVzxc2pJ01PqdSaqX99Bp9s09w4VR+dSXdzFZ273EzBUQZNeZ6xqs2q3ZkkJEanCJ2UVjThzM8rB4R4iXkWtY8R3mosY4iYIOgVThj9TWGRRyaK61FI+oo0IUVaCCiiiqNwooooAKKKKAF7Z9a0dAtjda1axc4Dhz/wHn/P1rO7V2XgbTiqyahIMbvkj+nc/59KznK0Thx9ZUqL8zs1GABS0UVxHyBgeM/8AkXp/qv8A6EK84r0fxn/yL031X/0IV5x3rro/CfTZR/CfqdF4Mv2ttU+ysSY5xwOwYDr+X8hXoWOa8q0Mka3aHp+8xXqi/drKsrM83NKahWuuo+iiisTywooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigBj/cb6V5Fff8f9z/ANdW/ma9df7jfSvIr7/j/uf+urfzNdFE9vJ/ikQUUUV0n0SFrt/AH/HldH/pp/QVw9dh4NnFtpF9M5wqMWJ9toNZVVdWPNzNXo2RF411NpbkafERsj+aT69q5U8VJcTNc3EkzkFpGLE062tri6k8u3haRs4O3nH+FVG0ImuGhDD0UnoQ0VuReE9WkUExRofRn/wok8J6sg4hjb/dejniV9dobcxhgUYq1cWMtq+y4YQsegdWGfp8vNT2+kSXTBYby0Zj/D5uD/LNO+l0W8VTXUzaK3x4Q1Q9Gt/++z/hTv8AhDtW/vQf99H/AApc6M/r1BfaOfzzSfWuli8Gaix/eSwoPUEt/hWxp/g20gO+7kadvQ8L+QqXVSMamZ0Iq6dzmtC0SfVpwSpW1X7zkdfpXpFvDHbwLFGoVEAAApYoY4UCxqFUdgKkGc9eK5pT5j5/FYqWIld7DqKKKg5DA8Z/8i9N9V/9CFeb969I8Z/8i9N9V/8AQhXnFddH4T6bKP4T9S9omP7as/TzBXqoIC+1eU6MwTWLVjjaHBOTWzr3iaa6draxcxwLwZAeW+hpVIuUjHH4adeulE6q+13TrH5ZrlQ46qMsR+VZTeNrAMQILhh6hRj+dcITzk8k9TQTmhUUtzSnlNK3vPU9Bg8ZaZJ/rPMi/wB9c/yzWzaaha3qFredJB/skZFeS59KfDLLbyeZDI0b/wB5TyKHRT2Iq5RFr929T2HPTmgGuR8P+KDcOtpqBAlbhJBwGPofeutB9xXPKLi9Tw61GdGXLNEVxPFbRNLNKsSLjLMQAPxqr/bml/8AP/b/APf1ap+Mf+RcuPqn/oQrzfGMVpTp8yO3B4FYmLlex6rDqmn3EwihvIZJG6Irgk1ez1yRXmPhf5fEdp7M3/oLVteJfEbrI1lYybSpIkkHXPoKHT1shVMvkq3soanRX+u6fp/yzXC+Z/cXk1knxvYAn/R7g++0f41whLEksSSTkkmjrWqopLU9OnlNNL3ndnq2lajHqdkt1CrKpJGG68VernvBWf7Cj7Dc38zVPxH4nNtI1nYkGVfvuein0rDkvKyPF+rSnWdOmjprq8t7WMvPMkajqWOKx5vF2lREhZmkI7Ih/wD1V59PPLcSeZNI0j+rHmouO4rZUV1PWp5RG3vs7w+N7AHH2a4Pvhf8aki8aabIcOk0f+8uf5ZrgOKOKfsYm/8AZNDuepWet6denFvcozH+E8N+RrRBzzkYrxwYBrf0XxNdWMix3LtPbk4JY5Zff6VEqNlocOIyqVNc1N3PRqKht5kuIlljYMrAMCO+amrnaseM007MT8KY8ioCWYAe9Zus6vBpNv5kpLSH7iDq1cDqes3upuTNIUj7RKeBWkabkduFwVTEarY7q58S6Vbna10GPogLfyqg/jawBIEFww9Qq/41wXApeK3VGJ68cppJas76LxrprnDxzRj1Zcj9M1p2eu6be4EN2hY/wn5SfwPNeXdPejr2pOiugTyim17rPY9wIBGCKU15tpHiS805gkjme37qxyy/j/n8K7+yvIb23SaBwyMM8VhKDieLicJUw797Yt0UtFQcgxvun6V5JqS7NTu1xjEzf+hGvXPavMvFMBg1+44AWTDj8gP6VtRep7GUytVaMeiiius+mFxnmta0ufI8MXiA4aWZUH6Z/TNZOeK1NJtTqHkWIztedmcjsoUZ/n+tTLbU5MZyqF2WvD3h99UYTz5S2B/F/b/P/wCrvbOygtIRHBGqIOgVcVJBBHbwrFGoVFGAB2qUdetckptny+JxU60tXoOFBoorM5SneWVveQmKeNXU9iM1wPiLQH0qTzYcvbN36lPb6f5+vpBHPWobm3juYWilUMjDBBrSE3FnVhsTKjJdjy2z1S+siBb3Lqg42k5FdRpnjKNwIdRi2Hp5icg/h1/nXLapYnT9RmtiSQhyp9u1VOorpcYzR9HLC0MTDmtuevwTxTxLJE4ZCOCDxU2a8s0bWrrSZQUJeE/ejPT6ivRtPvodRtVuIGyrD15Fc04OJ8/isHPDvXYvUUUVmcQUUUUAYHjP/kXp/qv/AKEK83716R4z/wCRen+q/wDoQrzeuuj8J9NlH8J+ouSOhIPrU1paz3k6wW8ZeQ9uw+tQdK9H8LaWthpqyOuJ5fmckcj2/X+dVUlynRjcUsPC63ZmWPgpAoe9mLN1Kp0rQbwjpOwjypAcdQ5/xrou1BFczqSZ83LGV5O/McDqvhGe2jM1lIZkAyY24b8+/wClcwcg4Ix65r2M88HGK4XxnpK20wv4VwknEgA4B7H/AD7VpTqX0Z6mAzCUpezqHLd+K9C8J6u2oWRgmbM8JwSf4h2P+f61550rW8OXn2HWoHJwsh2N754H64rWpHmR3Zhh1VpOXVHZ+Mv+RcuPqn/oQrzavSfGJz4cnI7lP/QhXm3epo/Cc+T/AMN+pYs7mS0uRPGSHVW2n6gioCSSSST3JNJ9a6fwpoS3zm9ulzAhwikffPr9P89ubk1HU7sRUp4eLqPcybDRdQ1ABoYCEP8AG/ArR/4Q3VAM7oD/AMDP/wATXoKIqDAAFO+lc7rNvQ8GeaVnK8dDkWa58O+FWilKidmKpt6fMf8AP5VxPJJYkknqTXd+MrG/1BbaO0hMqKSzcgYPbqfrXMf8I5q+cGyb/vtf8a1ptWuzvwFWkouc37zMxVLuFQEliAABkk11WmeDZJY1kvpTHkZ8tMZ/rR4a8P3sOqC4vLby441O0lgTu49D6ZruAMVE6ltjDHZhK/JSehgL4P0kLhonY+pc5/nVW68F2bqWt5ZImxxzuH/1/wA66riisvaSPMji6yd+Y8m1HT59NufIuB1+6w6N/n0qoRg12vj1E+zWzYHmB8Z74/ziuJ6gmuuD5on0+CrOtR5pbnb+Bb1pLaWzfkRHcp9j2/T9a6a8uI7O1lnkOERSxNcV4Dz/AGlcc/8ALIVd8d3rJDDZqSA53Nj27f59KwlG87Hh18Op4zkj1OW1K+m1K8kuZieeFXPCj0qn2pfatTw9pn9p6okTDMSfM+e/t/n3rf4UfQycMNSutkT6N4cutU2ysfIgP8RHLV0sHg3TEXEgklPqWI/lXQxqEQKoAAHan4rmlVk3ofMVsfWqSunZHL3fgyxkUm3kkhbHHORXJarpN1pc/lzjKsflkHRq9UI98Vm65p41LTpICAXwShPZu1OFV31NcLmFSnNKbujy3vW94U1RrDUhA5Jgn4x/dbsf8+1YPQ4NKGIYMpII6Edq6JWkj3q8adem4tnsHnrRXE/8JQvr+horH2aPA+oSO7rjPHVkSIL5QODsc/y/X+ddnVLUbSO/s5LZxw4646elZQlys5MNVdKqpnk1Gc1PdW0lndSW0y4eM4Pp9agrtTurn2cJqUVJdQrsfAcSubiUj5lO0ewOP8BXHV2fgCQFLuPuGU/n/wDqqKvwnBmd/YM7SiiiuI+UCiiigAooooA4Tx7AEurWcDllZSfyI/rXKd67Hx+eLRc92P48VxtdtJ+6fW5a28OrgOtbHh7V30q+G5v3Epw4Pb0NY9HJqmro6q9KNWDgz2NGDIrDoRTvSud8G35u9M8l2y8B2c9cdq6OuKSs7HxlWm6c3Bi0UUVJmYHjP/kXp/qv/oQrzevSPGf/ACL0/wBV/wDQhXm9ddH4T6bKP4T9S3pkH2nVLaEgENIMg9x1NesxgKgHtXmHhn/kYbXP94/+gmvUBWdfc4M2k3VSHUUUVgeQM6fhWfr1r9s0e4hwCSmQPcdK0jio5cGJgfSqT1Kpy5ZJnjtODFWVlOCCCCKbRXb0Pt/ip69j0TxO4k8JO46EIf8Ax4V55/FXc6oxbwDGxOT5UXP4rXCnrUUjzcqVoy9RwUu4RRlmOAK9Y0u1Wz06C3Xoi4/+vXl+mjOqWnGf3yD/AMeFetLwo+lZ1n0OPN5vmUR9Haiiuc8Qb1HNJgelRXM8VrC00rqiKMkk4ritW8XzTM0Vgvlx/wDPRuSfpVxg5HRQw1Wu7QR3JZQOWA/Gq02p2NvxNdxJ/vPj+deW3F9d3RPn3MkgPUFuPyqv0rVUe56kMoe8pHpcvijSIjg3YY/7Clv5Vn3XjWzQEW8Msp7E8D9a4SpYLea4JEMMkmP7i5NUqUVubrLcPDWTLWqapcapciWchQuQiKeFFUOnWrd9p9zYCM3MXlmTopOfSqp962SVtD1KCgoWp7HT+BP+QnP/ANc/6iqfjCbzfEEy/wDPNVX9M/1q34F/5CVx/wBc/wCtZfiM7tfvD1+YfyFZJe+eZTinjpNmZ2rt/AUAFtcXBHLvtz7AZ/qa4ivRPBIA0FSP77Z/Oiq7RNM1lahodHRRRXIfLhRiiigCt9jt858lP++aPsVt/wA8U/75FWKKfMyueXcrfYrf/nin/fIoq1RRzMOeXcKKKKRJzfibQhqUP2i3AFynT/a9q8/kjaORkdSjKSGUjkV7F261h654fttUXzAPKuBwJF7/AONb06ltGergswdH3J7Hm/HrW34TvhZa0gkYiOYbDz37f1/OqmpaPfaaSLiE7B/y0Xlf/rVngkcg4I6Gt3aS0Pdm4Yqk4p3PZAc8joaXvXMeGNfW+jW1uWAuUHBzjePWumyPWuOUXFnyVWlKlJxkOoooqTISkJxkn0o6d65bxTr62aNaWrg3DDBIP3B6/WqjG7NaVKVWXLFGD4qvPtt/K6H91E4iXnuAd388fhWCOhq/NCY9DglP/LWZjn8Mf0qj/DXbFWPrcGlGmoroJRRRVHWdF4LufJ1kwk4WZMY9x/k16HXlOiS+Trdo/rIF/Pj+terL90VyVlqfLZrDlrXXUdRRRWJ5ZgeM/wDkXpvqv/oQrzfvXpHjP/kXpvqv/oQrzeuuj8J9NlH8J+pe0Wf7PrNpL6SYz6Z4/rXqyY2jHpXjmSOQcH1r07w5qS6lpccmR5i/K4/2qisupzZvRd1URsUUUVznhDcjNVdRnFrYTzngIhb9KtcZrlfG2oiKzWxRhvlOWAPO3/Iq4q7NsPTdSooo4UHFJjjNLjjNXNKtjd6pbQAZDOCQfTvXa9EfY1H7Ok2+iOz8QQ+R4NaPptWNeP8AeFcB1Fej+Lxt8Mzr7p/6EK84rOlqjzcpd4SfmWtL/wCQtZ/9d0/nXrS/dH0ryTS/+QtZ/wDXdP8A0IV62v3R9Kyr7nFm/wDEXoOpKWkPQ1geOcD411Jpr0WSMRHFy4HdvT+X51zGMCrutStLrN4zdfOZfwBwP5VSPXFd0FaJ9jg6cadFWNHR9In1acrEdkSffcjP5V2dp4S0y3UGSNpn9Xb/ACKTwbFGmgRSADLsxbH+8RXQD3rnnN30PAxmNqyqOKdkilDpNhAcxWsKH1CAVcWNFHCj8qfQSBWV2zz3OUt2cP4/AFxZ49H/AKVyPeun8cXKzajDApBMSEtg+pHH6VzFdtL4T6zLk1h1c6jwJ/yE7j/rn/Ws3xPG0ev3QYYDFWHuNoH9DWj4E/5Cc/8A1z/rUvju0KXcF2oOHUoT2BBz/j+VRe0zjU+THtPqcpyR9K7zwJNv0qSI/wAEhwP1/rXBg9fet7whqH2PVfKdsRz4XJ/vdv8AP0qqivE6sxpOpQdj0iikByMilriPkxKQkAEn0pM5rK8Q3w0/SpZt2HI2oD/eNNK7sVCLnJRQHxLpAJH21KT/AISbSP8An8T9a8xqSGJp50hXG52Ciuj2Kse88qpxjzOR6X/wk2j/APP6lFUv7Ft/+edFL2ce5wexw/dnR56UetBPGc9q5LxD4nNs7WdgVaUffc8hfb61jGLk9Djo0Z1pcsEdNcXdvaoXmlRF9WOKzZfFGjodpu8+6qWH5gV5xPNNcSGSeRpH9WP+eKiroVHue1TyhW99noreKtEcYeUn6xt/hWNeyeFLs5DNC5H3o0Zf6YrlM470ZJqlTS2OqGWxp6xkzTnt9MSTfaaq+QcrvhYEH6jFaumeKp7RfLupY7pBxuG4P/6Dj+Vcv096Tr2qnBPc2ngoVFabuehR+MdMYfN5qH3U/wBKWXxjpaJlTI59FQ5/WvPKKj2MTn/smjc6TVPFt5dgx2q/Z4+mc/Mf8P1rnW3OxJJZmOSTySTSY71s+FrA32sxswzHB87f+y/4/hVWUVobunSwlNyii54ltDZaNpsOMEZzj171zJ612vj/AIitAOxb+VcX2opu6uTlz56NxKKKK0PRLOnf8hO1/wCuyf8AoQr1uP7i/SvJNO/5Cdr/ANdk/wDQhXrcf3F+lc1c+czf+Ih9FFFc54pgeM/+Rfm+q/8AoQrzevR/Gf8AyL831X/0IV5xXXR+E+lyj+Exee9XtK1S40u58+E8Hh0zw3/16k0C1W+1MW0n3XRh/hUWqabc6ZdGG4U4z8rjowq209Gdk6lOcnRkd1YeJ9Ou1+eUQt3WQ4xWkdQs0Te1zEE9d2K8l4o+lZuimefPKIN3i7HoOqeLLG2iKWrfaJT02/d/OuFurma8uGuJ3LyMfwHoKg470cdquMFA7sNgqeHV0Lkjiux8D6awL6jIMA5SP+v6/wAqx9B0KfVZw7qUtV+8xHLfSvRoII4IUijUKijAArOrNWsjz8zxi5fZQZkeMv8AkXLj6p/6EK82r0nxl/yLtx9U/wDQhXm1VR+E1yf+Ey1pf/IWs/8Arun869bX7o+leSaX/wAhaz/67p/OvW1+6PpWdfc483/iIdSHkUtFYHjnlviS2Nrrt0mOHbzFPrnr+uay69C8VaKdSgW4t1H2mLoDxuHpXnzo0bskilHU4KtwRXbCSaPrMBiY1aSj1R0HhzxCNMBt7gM9uTkMOSv4eldhba1plyAYryPcw4BOD+VeXZowRSlSUtTPEZbTrS5k7M9Xl1SxhXMt3FH9WArA1TxfbxKY7EGaTH32BC1ww+maOpwKlUktTKllVKD5pskmleeV5ZWLyMeWpnbitN9EvY9Me+liKKuMIRz7k1me2K1TXQ9OlUpyXLDodL4Efbq8q/3oj/Out1zT11PTZbbID9Ub0btXn2gXv9n6tDOxxHnY/wBD/kV6ipDAMpyCK56t1K58/mKlSxCmjx+SN45WikUq6HawPY03JHOcEV33iXw99vJurQBbleoPSQen1964WeKSCVo5kZHXqpHNbQmpI9jC4uGIhZvU6zRPFaJELfUSVYDAlHOfrXUQanYzpuiuo2HqGrybBPSjGOoqXRuzmrZVTnLmi7Hp174h02zjO65R3HGxDuOfSuE1nWJtWnDP8sScIg7VmZo4FVGmom2Gy+nQfNuxRmul8G6a098b51/dQ8Lx1as7RtFudWnG0GOAfek7fhXo1jaRWNqlvCoVEGAPWoqzVrI5syxsVD2UHqWdgop2aK5rs+d5jn/FWqnTrDy4j+/myqnuo7n/AD6150STyTk9zWz4pvTd63IAQUiARQPzP8/0FYtdlKNkfV5dQVKlzW1YUUUVoekFFFFABRRRQAEY70ZoxmpYIZrmYRQIXduwH+ePek9NyJTUVdsSKKSeVIolLu5wqivSvD+lLpWniM4MrfM5HrVPw74fXTQLifD3JHUdFFdHXLUnfRHzOYY32z5IbHI+P0/0a1f0kx+hriDwa9I8X2n2rQ5CoBeIiQfh1/TNecdVrWi/dsenlM1Kjy9hKKKK2PWLOm/8hO1/67J/6EK9bT7g+leSab/yE7X/AK7J/wChCvW0+4PpXNXPm84/iIfRRRXOeMUdRsIdRtWtpy2xuu04PXP9Kx/+EM03+9L/AN910o+tIeapSa0RrCvUpq0HYxNP8NWWn3a3MBkLjj5mzWjeWdveRGK4iV0/2hmreKQ+lK7vcmVWcpczepyd54Jtny1rcPFns3zAVnSeCr0Z8q4if/eGK76irVSSOqGPrw2kcDF4Kvif3tzEn+6N3862dP8AB9jbEPcs1w47NgL+X+Oa6XHFJQ6kmKpjq9TRsbHGsa7VUADsKkoorM4223dlLUbCHUrRrafPltjODg8HNY3/AAhmm5+9L/33XS/jSHmqUmtjWFepT0g7HOweEtNguI5lMpZGDAFu4ORXQqMDAHTpSge1L3pNt7kzqTqO8ncWiiikQNIyKytS0Gw1IZmiw/Z1OCK1qafwpptbFRnKDvFnFT+B5AT9nvQR2Dpz+dVR4L1DcQZoMeuT/hXoOKQ/WtFVkdqzHEJWucXb+BzkGe8+XuETB/Ot7T/D2nafh44d8g/jfk//AFvwrWX60VLnJ9TGpi61X4pEUsSSxmNlBVhgg1yN74M3SlrOcIpOdjjIH412lH0pRk1sRRxFSi7wZwMfgm+Y4luIVHqozXU6Np0+nWohlu2nA4GV4FatAzinKbluXWxVWtpNiDpzVC/0mz1BcXECsfXHNXxS1KbWxzxk4O8Wcdc+CIyc2126ezqGqhJ4L1Efcmhb/eyP8a9AxRWiqyO2OY4iKtc4OPwTdsf3l1Gn0Xd/Wtew8H2FuQ1wWuH9G+7+X+Oa6Xt1pKTqSZM8dXmrORHFEkSBUUKoGAAKmpKKzbONtvVi0UUUAeNzyebPJJ/ebdz+NNr1T+w9K/6B9v8A9+1pf7D0r/oH2/8A37Wur2yPejm8YqyieU0V6t/Ymlf9A+3/AO/a/wCFH9iaV/0D7f8A79r/AIUe3RX9sL+U8por1b+xNK/6B9v/AN+loGi6WCCLC3B7ERij26F/bC/lPKQat2+nX10QIbWRs99uB+Zr1KOytovuQIv0FThQBwAKl1jOeby+zE4TT/Bl3Kwa9kEKf3UOW/Pt+tdbp2kWemxbbeIA92PU1oAUHpWUqkpHm1sXVrfExaKKKg5iN1DoUI4IrzXxBo8mlXhKqTbSHKN6f7NemfjUN1aw3cDQzoHRhggjrVwlys68JipYed1seQDil611GreELiFmksWEsfXY3DD/ABrnLiCe3fZPC8bHs4xn6etdcZJn1FHGUqqumSad/wAhO1/67J/6EK9bj+4v0ryTTf8AkJ2n/XZP/QhXrSfcH0rGseLm7TqKw+iiiuc8YKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKAE7VDJFFKCrorDuCKKKaGm1sUU0bTTKsq2cQdWyCEAwRWn0H0oook2Nyct2OooopEhRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFAH/2Q==</t>
+        </is>
+      </c>
       <c r="N31" t="inlineStr">
         <is>
           <t>Administration &amp; Operations</t>
@@ -3194,7 +3282,11 @@
           <t>DRC</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEAYABgAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCACwAXUDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD3W6uoLK2e4uZFjhjXczscACvGfFnxSvL6V7TRGNvag4M5HzyfT+6P1qn8SPFs2r6rJpds5Wxtn2sAf9a46k+w6CuErmqVXeyPosuy2KiqlVXb2Rak1K/mffLe3Lse7Ssf6062vLo3UI+0zffH/LQ+tNtdNv74MbSyubgL94wxM+PrgVdt/D2ti6iJ0fUAA45Ns/r9KzSbZ6lSpSjFxukfTMH+oj/3RXB/FxmTwpGVYqftC8g47Gu8hBECA9QoriPipZ3N74WjjtLeW4lE6nZEhY4wecCuqfws+TwzSxCb7nhXnzf89ZP++jVqy1jUtOlWS0vbiJgc/LIcfiOhqb/hG9b/AOgNqP8A4Cv/AIVQuLW4tJjDdQSwSjkpKhVh+Brk1Wp9dz0avu3TPYvBfxNj1GSPTtZKQ3THbHMBhHPofQ/pXpeRtPFfJte1fC/xdNqsEmk38hkurdN8ch6vH059xx+db0ql9GeDmWXKmva09uqPTa47xexF7b4JH7s9D712HauO8Yf8f1v/ANcz/Ot0eKc7vf8AvN+dG9/7x/Oruj2UeoagtvKWCsCSVPNdR/wiVh/z0n/76H+FMRyFvfXVo4eCd0I5xu4P4V2+i6umpwfNhZ0++vr7j2rldb0ldLnjEblopQSu7qMYz/OmaHM0OtWpU/ebYR6g8UDPRKjd1jRnY4VRkn0FSVjeI7r7LpEgB+eU7B+PX9KQHE3V1JdXcs5ZgXYtjPSr2gXjW+sQlnO2T922T69P1xWVSglWDDgg5FUI9Voqnp9wLuwgnBB3oCfr3/WrlSM851pmGs3YDH/WHvU2gai1nqaB3PlS/I2T09DUGuf8hm7/AOuhqhTEeqiuE8TMw1yUBiPlXofaun0K++36ZGzHMkfyP9R3rlvFH/Icl/3V/lQhlvwizHUZskn913PuK0vFpI0mMgkfvh0+jVmeD/8AkIzf9cv6itPxd/yCI/8AruP5NS6gcdG7+avzN1HevUq8rj/1qf7wr0fVJDFpd1IpIZYmwR24psDndd8Qyea1rZOVVTh5B1J9BXMszMxZmLMepJyTSV1WleGra4sI57l3LSDcAhwAKBHK1o6brN1psi7XLw/xRsePw9K6Y+EtOwQGnB7HeP8ACuRvrSSxvJLaTkoeCO47GgD0S0uYru2SeFso4yP8K5bxc7JqEAV2XMXY+5qfwhK5FzET8gwwHoar+MP+QjB/1y/qaXUZV8OSSNrsAZ2Iw3BPsa72uA8Nf8h6D6N/I139Ngcv4uZkhtSrFcu3Q+wrntPlkOq2YMjEGdO5/vCug8Y/6i1/32/kK5zTP+QtZ/8AXdP/AEIUIR6ZRRRSGFFFFABRRRQAUUUUAfJTu0js7klmJJJ7miNd8iqe7AU2rulafd6nqMNvY27zTFgdqDoPU+grhjqz7utJRptvQ+k9G0e00bTorSzhWOFBwoHJPcn1Nam0Y6Ukf3FHtT67j4aUm5XYUYB60tFBJHgZ6CuB+KOjWdz4Wm1CSIC6tdpjkA5ALAEH1HNegd65L4kf8iFqP0T/ANDWpmvdZ0YWTjWi13R8712HwwZl8dWYBwGSQH3G01x9df8ADL/kfbH/AHZP/QDXJD4kfW43/d5ejPoiuN8Yf8f1v/1zP867KuN8Yf8AH9b/APXM/wA67UfFFTwz/wAhyL/db+Vd7XBeGf8AkORf7rfyrvabA5Lxl96z+j/+y1iaR/yGLP8A66r/ADrb8Zfes/o//stYmkf8hiz/AOuq/wA6BHpFcV4tujJfR2yn5Ylyfqf/AK2K7F2CKWY4VRkn0rzS9uDd3s1wf+Wjkgeg7UIZa0SzF7qscUiho1BZx7D/ACKp3UDWt1LA3WNitdD4We1to5557iKN2IRQ7gHAql4j8htT8+3ljkWVQW2MDgjigRseErvfZy2pPMTblHsf/r10tefeHbv7LrEWT8sv7s/j0/XFeg0mM841z/kMXf8A10NUKv65/wAhi7/66GrWk2H9oabqCqMypsdPqN3H40wDw3f/AGPUhG7Yin+Vsnoex/z60eJ/+Q5L/ur/ACrH5U8ZBFWb+8N9cLOw+Yoqt7kDFAjY8H/8hGb/AK5f1Fafi7/kER/9dx/JqzPB/wDyEZv+uX9RWn4u/wCQRH/13H8mpdRnGR/61P8AeFekajG02nXMSjLNGwA9TivN4/8AWp/vCvUzTYHlXfBrasfEl3ZwpEyJLEg2gEYIH1rY1PwxHczNPayiJ2OWQj5Sf6Vg3Hh7UrfJNuZFHeP5v060AdFbeLLGbAmSSFvcbh+YpLjStN1qc3KXe5mAAEbjj8K4tkZG2upU+hGKEdkYMjFWHQg80AegaZo0GltI0Ujt5gAO7FYPjD/kIwf9cv6mtbw3qT39o0c53TRYBY/xDsayfGH/ACEYP+uX9TS6gZej3kdjqMVxKG2KDnaOeRXU/wDCWaf/AHZv++K4gAscKCT6AU7yZf8Anm//AHyaYjb8QavbanFAsAcFGJO4YrL0z/kK2f8A13T/ANCFV2R0+8rD6irGmf8AIVs/+u6f+hCmB6ZRRRUjCiiigAooooAKKKKAPn7Qfhtq+p6jJHdK1paQyMjTMOXwcHaO/wBeley6F4b07w7aC3sIVTj5nPLOfUmtR5FihZ3bCqCScdq8g8XfFOWcyWWgExx/da6PDH/dHb6msrRpq56Tq4nHT5Vt+B3uu+N9D8PSrDeTs8558uFd7KPU+lZH/C3fDv8Adu/+/X/168LkkeWRpJHZ3Y5ZmOST7mm1m6z6HpwyWko++22e7f8AC3fDn928/wC/Q/xo/wCFveHP7t5/36H+NeE0UvbSL/sWh3Z7qfi54czwl3/36H+NcZ47+IMev2a6dpiOlqwDSySDDNjkDHYV57RSdWTVjWjlVClNTV20Fdt8K7SS48aRSoPkt4Xdz9RtH8/0rj7SzuL+7jtbWJpZpGwqjqTX0F4G8Ix+F9L2uVkvJjumkA/JR7CilFuVyM0xUKdJ0+rOu7Vx3jD/AI/rf/rmf512Vcb4w/4/rf8A65n+ddaPlSp4Y/5DkX+638q7yvL4Lma3lEsLlJB0YVd/t/U/+fx/yH+FOwjX8ZEb7Id8P/7LWJpH/IYs/wDrqv8AOq1xcTXMplnkZ2Pdq2PDOnSXF8t2y4hiOQT/ABNQB0XiK7+y6PLg4eUiNfx6/pmuAro/F115l5FaqeI13N9T/wDW/nWVpFmL3VIYGGUJ3P8AQUDKNFeh/wBgaX/z5p+Z/wAabJ4f01kKi0RSRgEE8UXA8/VirqynDA5Br0uxuRd2cNwCMSID+PevNpomgmeJ/vIxU/hXYeErrzLB7YnmFsj6H/6+aGBzeuf8hm7/AOuhrc8Gfdvf+Af+zVh65/yGbv8A66Gtzwb929/4B/7NR0EZfiGw+w6izIMRTZdfY9xWRXfa/Yfb9NcKMyx/On9R+VcDQgOi8H/8hGb/AK5f1Fafi7/kER/9dx/JqzPB/wDyEZv+uX9RWn4u/wCQRH/13H8mpdRnGR/61P8AeFeha27x6RcyRuyOq8MpwRyK89j/ANan+8K9JvbYXlnNbscCRSM+h7U2B58NTvs/8ftx/wB/T/jXo0B3W8bZzlQc+vFeaXFvLaztDKpDIcEVctda1CzhEMM/yjoCAcUCO9mtLe5XbNBHIP8AbUGuA1q3itdVmhgULGuMKDnHFWD4l1QjHnj/AL4FZLu0js7sWZjkknkmgDpPBv8Ax+XX/XMfzpvjD/kIwf8AXL+pq94WsXgt5LqUbTMAEH+z61R8Yf8AIRg/65f1NHUZT8Nc67B9G/ka77aPQflXA+Gv+Q9B9G/ka7+hgct4xAFva4H8bfyFc5pn/IWs/wDrun/oQro/GP8AqLX/AH2/kK5zTP8AkLWf/XdP/QhQhHplFFFIYUUUUAFFFFABRRRQAlef+KPhpp2uXLXdq5srt+WKKCrn1K+vuK9AzWPqviHStGQNf3kUOegZvmP4damSTWprRnUhO9Pc8t/4U1qX/QSt/wDvhqP+FNap/wBBK2/74au2/wCFoeFM/wDH8/8A34f/AAoHxQ8KE4+3P+MD/wCFZ8tM9L61j+z+44j/AIU1qn/QSt/++Gpf+FM6n/0E7f8A74Nep6X4h0rWULaffQz4HIVvmH1HWtMruqlTgzGWZYqLtJ2+R4z/AMKa1T/oJW//AHw1Pj+DN95i+bqkQTPzFYyTXs1Qzzx28bSyyJGijLMxwB+NHs4k/wBo4l6cxz3hnwXpnhiH/RkMtwww9xIAXPsPQe1dK2favN/EXxW06xDQaUv224HHmZxGv49T+H51U+HHiXVvEPiG/a/uC6rCCsSjCJ83YU1KKfKiJ4bESg61T8T1X+HpWHrGhvqk0cizrHsXGCM5rc7Vga34t0fQZ44NQufKkkXco2k5H4Vd7HJGEpO0VdlD/hDpv+fqP/vk0f8ACHTf8/Uf/fJpv/CzPCv/AEED/wB+2/wo/wCFl+Ff+gif+/Tf4Uuddzb6tW/lf3Fi28IIsgNxcF1H8KDGfxrpIYY7eFYokCIowFFczZePvDl9MsUepwq7HADkpn8TXUKysoIOQe4oTTM505wdpKxzN74anvbya4a6QeYxIG08DsKuaPoY0uaSV5VkZl2jAxgd62CyoCTwBXJn4m+Fgcf2gcj/AKYv/hQ5JbhCnOfwps7Ck59a4/8A4Wd4W/6CH/kJ/wDCj/hZ3hb/AJ//APyE/wDhS5o9y/qtb+VlzUPDTXt9JcRzJGJMEqV796m0jQJdLuzKbhHVlIZQvWs2P4l+GJJFQX+WY4H7p+v5V1jyqkLSMcKqlifYU1JPYmdOcXaSsc7feGJbu9muBcqokYsAVPFaGiaO+lefvlWTzduMDGMZ/wAaxf8AhZvhX/n/AG/78v8A4Un/AAszwr/z/n/v03+FLmj3L+q1v5X9x2WK5a78KGa6kkhuEjjdtwUr0qv/AMLO8L/8/wD/AOQn/wAKfD8SPDNxPHDHf5kkYIo8puSTgdqOddxPDVlvFmjo2hPpl1JK0yyBk24C471a1nTjqVokCyCMrIHyRnsR/Wmazr2n6BZLc6hL5UTOEDBSfmIJ7fQ1jR/EnwzNMkSX+Xdgqjy26n8KbkluTGjUmrpNocvhCZWDfa4+Dn7prruKaDlc+tUtT1G20qwlvLuTy4Ihl2wTjt2ptkJNuyItT0m31NBvykq/dkUc/j6isE+D7jPF1ER7g0g+J3hb/oIN/wB+X/wrq4LiK5gjmibcjqGU4xkHpSUk9ip0pw+JNHK/8Ifdf8/UX5Grll4WiglWW6lE205CAYX8a6CWVIIy7sqoBkknAArkbn4meGbadoWv95U4JRGYfmBTcktxwpTn8CudkAMcVh61ob6ncRyrOsYRNuCM96xf+Fq+Fv8An6k/78v/AIVoaV488P6xcC2tr4CY8KkilS30z1qVOPRlSw1aKu4uxJpfhyXT7+O5a4RwgPyhSOoxXSUnBHFZ2rataaJYPeX0pjgQgMwUnGTgcCqbMkm3ZEWs6S+qRwokqx+WxJyM5zWZa+FZre7gnNyhEciuQFPODmq//CzfCv8Az/t/35f/AAo/4WZ4V/5/z/36f/Cp5o9zb6tW/lf3HYdVpOlcf/ws7wv/ANBAn/ti/wDhV/SfGuha5eizsbsyzlSwUxsOB16impJkSw9WKvKLSOipcisrWdbsNCsxd6hMY4dwTcFJ5P0+lYJ+Jvhc/wDMQP8A36f/AAocktxQo1Jq8ItnZYowa4//AIWd4X/6CH/kJ/8ACj/hZ3hb/oIf+Qn/AMKXNHuafVa38rOx/GiuO/4Wd4W/5/8A/wAhP/hRRzRD6rW/lZR8feOl8NxfYbLD6jKuRkZESn+I+/oK8Pubq4vLmS4upXmmkOXdzkk1Z1rUpNW1u8v5SS00pYZ7DsPyxVDBJwBkmuWc3Jn1OCwcMPTTa957hRXZ2fww8SXltHMIIYt4yElkww+o7VFqfw48Q6XaSXEkEcqxjLCF9zY9cUckuxqsbh2+XmVzmLO8ubC5jurSZ4Z4zlXQ4Ir3HwX4+ttesGj1CSOC9gTdJuYBWX+8P6ivB6KUJuJGLwNPER7Pue2eIvitpthvg0pDfXA48zpEPx6n8PzryzW/FGr+IZS2oXbOmcrCnyov4f41jUUSqSkLDZfQoa2u+4V6T8Gv+Q9qH/XEf+hVx2i+F9X16VRY2jtGTgzONsY/4F/hXsngjwL/AMIq0tzLdedczIFYIuFUZzx3NXSi+a5zZniqXsnTT1Z3JrxT4y/8h/T/APr3P/oVe114p8Zf+Q9Yf9e5/wDQq2q/CePln+8xPNaK6v4cW0N34wt4p40kQo+Vdcg8V7t/wj2j4/5Btt0/55L/AIVjCnzK57WLzKOHqcjjc+Xq9T+F3jCb7Smg3zGRWB+zO3VcDOz6YHFV/i5pVjp76XLa28cTyrIr7FwGA244/E1x/g4keMdIIOP9KQcfWhXhOwqrp4zCOo13/A+lZv8AUSf7pr5Rf/WN9TX1dN/qJP8AdNfKL/6xvqaut0OPJd5fIbRXt3ww06xufCEUlxaQyuJHGXjBPX3rtf7C0rOf7Otf+/S/4VMaN1e5tWzhU6jhy7HzFZ/8f1v/ANdF/nX1Fdj/AIlcwP8AzxP8jTBomlhgRp9qCOn7pf8ACpr/AP48Lj/rm38jWsYcqPLxWM+szi7WsfKlFFe6fDXTLG58H20s9pDLIWfJeME9feueMeZ2PosTilhqUZWueF1d0f8A5Dmn/wDXzH/6EK+l/wCwtK6f2dbf9+l/woTRdMRgy2FsGByCIlyD+VbKj5nlzzhSi1ynFfF//kUrX/r6T/0F68a0z/kLWf8A13T/ANCFezfGP/kVbb/r8T/0F68Z03/kK2f/AF3T/wBCFRU+M6MtV8LJ+p9UR/cT6VzHxF/5EfUv9wf+hCunj/1afSuY+Iv/ACI+pf7g/wDQhXRLZngUf4y9T50r6j0P/kAWP/Xun/oIr5cr6i0T/kXbL/r3T/0EVjR3Z7OcrSB5H8SvGUt/fTaLZsUtYGKTsD/rHHUfQV5zVrUmLareMxyTM5J/4Ea9P+EmjWNzpt5fT2ySTify1ZxnC7QeAfrUWdSR2KUMFhVJI8n2n0P5UAkEEEgg5GK+pv7KsP8Anyg/79ivJ/iV4OmOrW91o+myv5yHzhBGSoIIwcDoSP5U5UmldGNDN4VZ8k42Rv8Awz8XNrVk2l30ha+tlyrk8yJ0yfcf4Vp/E7jwHdj/AG4//QhXA/DrQNZ0/wAZ2s9zp91bwhJA7OhC8qcZ/HFd98Uf+RHu/wDfT/0IVom3DU82rCnHGr2ezaZ8/UUV9LaRo2mNpFmzWFsWMKEkxLnO0e1YwhzHuY7HfVVHS9z5pruPhR/yO0f/AF7yf0r2z+xNKP8AzDrX/vyv+FSW+mWNrJ5lvaQxuRjcsYB/MVrGlZ3ueRiM19tTcOW1zjfi7/yJi/8AXyn8jXhNe7fF3/kTV/6+U/ka8Lj/ANan1FRV+I7spfLh2/MbRX1BBomlGJP9Atj8o/5ZL/hUn9haV/0Drb/v0v8AhT9j5mMs6SduQ+W6K+pf7D0r/oH23/fpf8KKfsfMX9t/3D5ap8P+vj/3h/Ovp/8A4R3R/wDoGWn/AH6X/CgeH9HByNNtMj/piv8AhS9g+4TzrmVuU0Iv9Wv0qK9H+iTf7h/lVntVe7/49J/9w/yroPCi/ePlST/Xv/vGmU+X/Xv/ALxqfTQDqtoCMgzJkH/eFcP2j7lS5aNzW0PwbrXiBla1tWS3PWeb5U/D1/CvU/D/AMKtK05Vm1H/AE+4BzhxiMH/AHe/413kCbIwAAABgADpUp5rqjSjE+UxOY1quidl5EcMEUEaxxoqIowFUYAqakxS1oefdvcSvE/jL/yH7H/r3P8A6FXtvevE/jL/AMh+w/69z/6FWdX4T0Mr/wB5icX4c1t/D2sx6jHAsrIrLsLYByMV3X/C573GP7Kh/wC/x/wrznT9Ou9VvFtLGEzTsCQgIGcfWptV0LU9EaJdRtHtzKCU3EEHHXkE+orCMpJaH0NfD4WrUtU1kanizxfdeK7iB54FhjgUhEU55OMkn8BR4DsJr/xnpqxKdsMnnO2OFC88/oPxrn7eIT3EcRkWMOwXe3Rc9z7V9DeDfCVn4X07Mb+bdSgGWYjr7D0FOCc5XZzY6rTwtD2UFvsdPN/qJPpXyg/+sb6mvq6X/USfQ18ov/rG+pqq3Q5Ml+KXyOm0Px5rPh3TVsrEW/lKxYb48nJ6960v+Fs+JM5zaZ/65/8A16ytE8Ca14hsFvbBYDCxKjfJtOR14rS/4VR4m3Y2Wuf+u3/1qle0tod9VYDnfPa/U2/DHxI17VvEtjYXH2byp5NrbY8HGCfWvWb7/kH3Gf8Anm38jXknhb4ceINJ8S2N/dJbCGCTcxWXJxgjpj3r1u+/5B8+f+ebfyNbQ5re8eFjPZe2XsrW8j5UrqNF8f61oGmpYWRt/JQkjfHk8/jXL11GjeAta17T0vbFLcwuSBvkwePauaPNf3T6WqqHsl7a1vM0v+Fs+JM5/wBE/wC/f/163PB3xE13XPFFnp939n8iYtu2R4PCk+vqKwf+FUeJs42Wuf8Arsf8K3PB/wAPde0TxXZahdJbiCEvvKS5PKEDjHqa1j7S+p5ldYH2cuS17aG58Y/+RVtv+vxP/QXrxnTf+QrZ/wDXdP8A0IV7N8Y/+RVtv+vxP/QXrxnTP+QrZ/8AXdP/AEIUqnxo0yz/AHSXzPqlPuL9K5f4i/8AIj6l/uD/ANCFdOv3F+lcx8Rf+RH1L/cH/oQreWzPAofxo+p86V9Q6H/yLtn/ANe6f+givl6vqHQ/+Rds/wDr3T/0EVjR6nt5ztA+Z9R/5Cd1/wBdn/ma9h+DP/IuX/8A19n/ANAWvHtR/wCQndf9dn/ma9h+DX/It3//AF9n/wBAWpp/Ga5j/ui+Rl6z8VNU03XL2zjsbR0t5mjVmLZIBxzzVE/GLVzj/iX2f/j/APjVTxB4A8S33iHULq30/fDPO7o3moMgnjvXJavouoaFdra6jb+TM6eYF3BvlyRng+xqpSqIWGw2DqRS0crdz1Pwj8SNQ8QeJbfTri0t445VYl492RhSe59q3vih/wAiPdn/AG4//QhXlvwx/wCR8sT/ALEn/oBr1L4o8+Bbs/7cf/oQqoybg2zhxNGFHGRjBWWh8/V29v8AFLxFbW0UEf2XZGgRcxdgMetcRXaQfC/xHcW8U8aWvlyKGXM3OCM+lYx5vsnu4pYdpe2t5XJx8WfEvraf9+//AK9dp8OvGWq+Jr28h1DydsMasuxMck1xH/CqPEx5Edp/3+/+tXa/Dnwfqvhq+vJdQWEJLGqrsfdyDWsPac2p5GMWD9i/ZW5iz8Xf+RNX/r5T+RrwoEqwI6g5r3X4u/8AImr/ANfKfyNeFAFmAHU8VNb4jqyi31d37nbr8V/EaIFBtMAYH7v/AOvT/wDhbXiX1tP+/f8A9eoV+FfiZ1DCO1wRkfvv/rU//hU/if8AuWv/AH+/+tR+8G1l99bHe+APF2o+ILO9kvxFuhkVU2LgYINFN+H/AIS1PQLO9jv0h3SyKU2OTwAaK2jex41b2HO+XY4D/hafin/n6h/78rR/wtLxT/z9Qf8Afla4uiub2ku59L9Qw38qO0/4Wn4p/wCfqH/vytMf4n+KJI2VrqDawwf3K1x1FHtJdxrA4b+VCklmLHqTmnRStDMkqHDowZfqKZRWZ02hblOz/wCFpeKAMfaof+/K0v8AwtLxT/z9Qf8Afla4uitPaS7nL9Rw38qO0/4Wl4o6faof+/K12nw48Yax4j1S7t9RljeOOIMoWMLznHavF69J+Dmf7c1DH/PAZ/76q6c5OSTZxZhhaEKDlGKTPba8T+Mn/If0/wD64n/0KvbK8S+Mv/IfsP8Argf/AEKtanwnkZZ/vMTI+F3/ACPVr/1zf+VeseO/Dg8Q+Hpoo1BuIh5kJ77h2/HpXlHwu/5Hm1/65v8Ayr6B6mppK8LHTmlWUMUpx3SR8mMpVirAhgcEHtXuvww8SDV/D4sLh83dlhDnqyfwn+n4VwXxO8O/2P4hN9AuLW9Jfjosn8Q/Hr+dc/4W1yTw94gt79SfKB2zL/eQ9f8AH8Kzi3Cdmd2IjHGYVTjutT6Yl/1Mn0NfKD/fb6mvqhZ47mx8+Jw8cke5GHQgjINfK8n+sb6mrrdDmyVe9K/ke2fDDULK28JRRz3cETmR/ldwp6+hrtv7b0rP/IRtv+/q/wCNfLdFJVrK1jWtlCqVHLn3PqQa1phbAv7Yk9B5q/41Pfn/AECf/rm38jXy1Z/8f1v/ANdF/nX1Fef8gufP/PE/yNaRnzo8vFYNYapFXvc+V6+gPhb/AMiVbf77/wDoRr5/r3/4W/8AIk23++//AKFWdL4j1c1/3eJ29FApa6D5s84+MX/Iq25/6ek/9BevFbOVbe+t5nztjkVzj0BzX0t4j0SDxDo0+nTkhZB8rDqrDkGvnHWNIvND1GWyvYysqHg9mHYg+lc9VO9z6DKasJU3Se59IWmv6Ze20U0N7C0brlW3Afoa5b4ka5p0fhO4tDdRvNcALGqMCTggk8dBXheSOhNIST1OaTrNq1i6eTxjUU+bRBX1HooI8P2anqLdB/46K8K8DeEJvEmqJPMjLp8DgyMeN5/uD+tfQccapGEUAKBgAelXSi0rnNm9eEpRhHofLGpKV1S7VhhhM4I/4Ea9Q+EesWFtpt5ZT3Mccxn8xVkbblSoHGfpWX8SfBkthfzazYqz2s7F51A5jc9T9DXnPQ1nrCV2eko08dhVFOx9Tf2rYdftsGP+ug/xrw34n6pa6p4rVrSVZRDAInK9NwZiQD36iuM3N6n86FVnYKoLMxwABkk051eZWM8LlccNU9o5XOv+GIL+OrPAPCSE+3yGvUPil/yIt3/vx/8AoQrO+G3g19BgbUr4f6dcJtEY/wCWScHB9zgVo/E/5vAV0f8Abj/9CFXGLUNTzcTXjWxqcdk0j5/r6W0rWNMXR7NGv7cMIUBBlXPQe9fNNFZQlyHs4zArFKPvWsfUv9taV/0ELb/v6v8AjT4NRsrqTZb3cEj4ztWQE/kDXyvXcfCfnxsvP/Lu/wDStY1bu1jycRlXsabnzXsd98Xf+RNX/r5T+RrwuPiVP94V7p8XP+RNT/r5T+Rrwmoq/EduUq+Ha8z6gg1rSxEgN/bD5R/y0X/Gpf7c0r/oI23/AH9X/Gvlqiq9t5GMslTd+c+pf7b0r/oI23/f1f8AGivlqij2/kL+xV/OfRv/AAr/AMMd9Ih/X/Gl/wCFf+F+2kwfkf8AGumzxzXK+JfHGleG8R3TtLORxBCQW/HnAH1rVqK3PIhVxFSVoybfqSf8K/8AC/8A0CYP1/xo/wCFf+F/+gTB+R/xrjT8aUz8ujtj3nH+FN/4XSP+gQf+/wCP8KjnpnWsLjn3+87P/hX/AIX/AOgVB+R/xo/4V/4X/wCgVB+R/wAa4v8A4XSP+gQ3/f8AH+FH/C6R/wBAhv8Av+P8KOemP6rjvP7ztf8AhX/hf/oEwfr/AI0f8IB4X/6BMH6/41xf/C6f+oQf+/8A/wDWqSH4z2/mKLjSJlj/AImjlDEfgQM/nRzUxPDY1Lr951//AAr/AMMn/mEQfr/jV/SvDWkaJK8thZRwO42sUB5FGh+IdM1+0+0adcB1HDKeGQ+hHatntVpR3Rw1KlXWM2/mLXO634T0fxBPHNqNsZJI12KdxGB17Guh6DrUTtsUsWAAGSSeKbVyISlF3i7M57SvA2haLere2VmY7hQQG8xj1+pro29hXmOv/Fy2tLprbSrYXO04aZnwh/3ccn61j/8AC5dR/wCgZbn/ALaGo9pCOh2/UcXWXO1f1PVdY0Ow120+y6jAJotwYDJBBHfIrB/4Vj4W/wCfD/yK3+Ncnp3xlZrpV1HTlSAnBeFyWX3wetepWF/balZx3VrKskLqGV1PBFNOMjOpTxGGVpXSGafpttpmnx2NsrLBENqKWJwPTJrnW+GfhbJP9nnn/ps3+NdjwRXF+LfH+neGSLcIbm+YZEKHAUf7R7fSnKyWpnQdaUrUm7vsP/4Vj4V/6B5/7/P/AI0f8Kx8K/8AQPP/AH+f/GuI/wCFzal/0DLf/v4aP+Fzal/0Dbb/AL+Gs+ameh9Vx/d/edwnw18LRyK/9ntuU5B81v8AGusaFHiMbDKsMEe1cJ4U+Jdjr1ytleQm0u2+5lspIfQHsfau+yCuRz6VpHlaujz68a0JWq3v5nH/APCsfC3/AD4H/v6/+Nb+laTZ6LYJZ2MRjgUkhdxPX61wHib4n3eh+ILvTI9OjkW3ZQGaQgnKg/1rU8DeO5/Fd9c2s1lHAIYw4ZHJzzjvSUo3sjWpRxLpc8tY+p3vak+lFee+NfiFceFtYisYLKOdXhEpZ3IIJZhj9KptJXZz0qUqsuWCuz0LjFZGseH9N1yEx6hapMo+6SMEfQjkVxnhT4k3XiPxBDpsthHCsisxZXJIwM11HjHxDL4a0FtRihEzK4XYWIHNLmTVzR0atKoobSZlD4V+Fv8An0m/7/t/jTo/hd4WhkVzZO2052vMxB+vNch/wue+z/yCoP8Av6a9Q0TVYdb0a11GDGydA2M/dPQj8DkVMeSWx0V1jKKXO2k/MuWlnb2MCQW0SRRIMKiDAFWep6VjeJ9YbQdAutRjiWV4VBCE4ByQP615j/wua+H/ADC4D/21NNyUdGc9LDVa6coq57HJEkyFHUFSMEEZBFcjd/DTwxdTtMbBlYnJEUrKPyBrpdNvDfaZb3LKFMsSyFR2yM1X1nWrDQ7CS9v5Qkadu5PoB3NU0nuRTnVhLlg2n5HOf8Kr8LdrWb/v+3+NX9K8BeHtGuhdW1jmcfdeRy+36Z6Vwt18Zrnz2+y6Wnkg/KZZCGI98cVD/wALl1L/AKBtv/38NZc1NHoPC46cbNu3qe0ADGPSqGq6Taa1YPZ30fmQOQWXcR0OR0rifDHxRs9Yu0s9QgFncSHEbbsxsfTJ6GvRgQRkVompLQ8+pSqUZWmrM40fDLwqf+Yef+/r/wCNL/wrLwqP+Ye3/f1v8ag8deN7jwnPaRw2iTCdWJLsRjGPSsXw38UbvWtftNNk06KNZ2Kl1kJI4J/pUtxTsdUVi5U/aJu3qdD/AMKy8Kn/AJh7f9/m/wAauaV4L0HRL0XlhaGKcKVDGRjwevU1pa3qB0rRry/RBI1vA8oUnAJUE4ryz/hc191/sqD/AL+mhuMXqTThia8XZtr1PU9Y0Sw16x+yajCZYdwfaGI5H0rA/wCFY+F/+gf/AORX/wAa39F1D+1dGsr9kEb3ECSlAchdwBxWn9auyZzxq1KXuxbRx3/CsPC3/Pgf+/jf40f8Kw8L/wDPif8Av63+NdhzRzS5V2K+s1v5mcf/AMKw8Lf8+B/7+N/jRXYc0Ucq7B9ZrfzM8/8AiB46Hh2H+z7AhtQlXO4jIiU9z7+grw6aaW4meaaRpJXO5nY5JNafiW8lv/E2pXEpyxuHH4A4H6CsmuWpNyZ9TgcJChTTe73CivSPDXwrk1TT1u9SuJLfzAGjiRRuA9Wz/Kt3/hTWm/8AQSu//Hf8KFSkyZ5rh4ScWzxqivZ/+FMaX/0E7z/vlf8ACl/4Uxpn/QUvPyX/AAp+xkL+2MN3f3Hi9Fey/wDCmtO76ld/+O/4VxXjTwJceF9lxDK1xYucb2XDIfQ/40nSkldmlHM8PVnyJ6s5/R9ZvdDv1vbGUpIvVf4XHoR3FfRHhjxFbeJdIjvYPlOdsiHqjjqK+Z69I+D1/LF4hurHd+5mgMmP9pSAP0JqqU2nY5c2wkZU3VW6Pbeory34teIbiztYNHtWKG5UtMw7p02/j3r1PtXiPxk48QWP/Xuf/Qq2qO0TxsupxniIqR53FDLNOkMMbSSyMFRFGSxPQAV0w+HXicgEWA59ZV/xqf4Xor+N7fcoOIpCMjocV9BcDsMfSsqdJSV2erjsxqYer7OCPlvVtG1DRLkW9/bvDIRuXJ4Yex711vwx8TzaXrkelyuWs7ttqhj9yTsR9eldX8ZFU6Fp7gDcLkgHHP3TXmPhT/kbtKH/AE9R/wA6Lck7I1jUWLwjlU31/A998W6wdB8MXuoooaSNQEB6bmIUfqa+bri4murmS4uJGkmkYs7sckk1738UP+RBvP8Aei/9DWvn+iq3exjlEIxpSqdbnQab4K1/VrRLu0sGaF/uFmC7h6jPaprnwB4ktbZ5pNNYqikttcMSPoK+hrWJYrWNFUKAgAA6DipnGUIx2q/Yxsc7zmtz6JWPk5WZHDKSrKcgjqDX0B8OvEM3iDw6GuWD3Vu/lytj73cH64rw7XlVPEGoqoAUXDgAdvmNeq/Bk/8AEk1I/wDTyP8A0EVnSdp2OzNYxqYdVGtdDgviJ/yP2rf7yf8Aota6T4Nf8hzUP+uA/wDQq5v4if8AI/ar/vJ/6LWuk+DX/Ic1D/rgP/Qqcf4o63/Iv+SPajXhfxh/5G63/wCvNf8A0N69yFeG/GH/AJG63/681/8AQ3rWr8J5GVf7yjP+F/8AyPVp/wBc5P8A0E16R8WP+RKk/wCu0f8AOvN/hf8A8j1af9c5P/QTXpHxY/5EqT/rtH/Ooh8DO7Gf79H5Hgtep/CLX/LuLjRZ3+V8zQZ9f4h/X8DXllWtNvptN1K3vrc4lgkDr747fj0rGEuWVz18bh1XotdT6A+In/Iian/ur/6GK+da978XajDqnwxur23OY5oUce3zL/KvBK1rbo87KU40Zp9z6g8PHHh7Tz6W0f8A6CK8J8feIJ9a8S3UTMRbWsjQxIDxwcFvqSK910H/AJFmx/69o/8A0EV83a1/yHdQ/wCvmT/0I1VV+6jmyunGWIlJ9B2k6LqOuXLW+nW7zOo3NjgKPc1tN8OfE6qT/Z2cdhIv+NegfBtB/wAI7evtHN2RnHP3Er0jv04qY0k1dmmKzWrTrShFKyPlCSOSCVo5UZJEO1lYYKkdjXuXwy8Sy63o8lpdMXu7MgFz1dD0J9+MV5x8S0VPHeoKoAyIzwO+wV0fwXONQ1TP/PKP+bUU7xnY1xzjXwiqNa6MX40f8f2l/wDXN/5iuS+H/wDyPelf9dD/AOgmut+NH/H9pf8AuP8AzFcl8Pv+R70r/rof/QTSl/EHh/8AcH6M9z8Yf8ibrP8A15y/+gGvmevpjxh/yJus/wDXnL/6Aa+Z6K26Msl/hzPpjwf/AMibo/8A16Rf+git3vWF4Q/5E3Rv+vOL/wBBFbveuiOx4dX+JL1Y6iiimZhRRRQB806p4Z12TVbx00e/ZGncqwgYgjceelVl8La/uX/iTah1/wCfZv8ACvpnzFI52/nS71/2fzrL2SPY/taty8vKiCwQpZQKwwwjUEenFWxUfmJ/eX86POT+8PzrU8lpt3JKKj85P7w/Ojzk/vD86BcrHVw/xX/5Eib/AK6x/wDoQrtfMTH3h+dcR8VHVvBUwBB/ex9/9oVMvhZ0YSL9vH1PBa7z4Sf8jof+vV/5rXB13nwk/wCR0P8A16v/ADWuWn8SPq8f/u0vQ96rxH4x/wDIwWP/AFwP/oVe3V4j8Y/+Rgsf+uB/9Crer8B83lf+8ozPhV/yPEH/AFxk/lX0B3r5/wDhV/yPEH/XGT+VfQA60UfhNM3/AN4+SKOoaXYanGsd9Zw3KIdyrMgYA+vNUYPC2hW8yTw6TYxyxkMrpAoKn1BxXPfE3XdR0PSbSXTrgwvJPsZgAcjaT3rgfDvjrxHd+I9Ptp9RZoZbhEddijIJ5HSnKcVKzMaWFrToupF6Ho3xS/5EK9/34v8A0YtfP9fQHxR/5EK8/wB6L/0Na+f6yq/EevlX+7S9T6vtv9Qn+6Kkk/1Z+lR23+oX/dFSSf6s/SulHzsvjPl7xB/yMOpf9fMn/oRr1T4Mf8gbUv8Ar4H/AKCK8r8Qf8jDqX/XzJ/6Ea9U+DP/ACBtS/6+B/6CK5ofxD6PH/7mvkcB8RP+R81b/fT/ANFrXSfBr/kOX/8A1wH/AKFXN/ET/kfNW/30/wDRa10nwa/5Dl//ANcB/wChUR/iDr/7h8kezjqa8P8AjF/yN1t/15r/AOhvXuQrw34xf8jdbf8AXmv/AKG9a1fhPJyn/eUZ3wu/5Hq0/wCucn/oJr0n4s/8iW//AF2j/nXm3wu/5Hq0/wCucn/oJr0n4s/8iW//AF2j/nUQ/hs68Z/v0fkeDoNzqvqQKva5pUui6xcWMgP7tsqx/iU8g/lVKL/Xp/vCvXfiz4eEunW2swJ+8gAjnwOqHofwP86yjG8Wz1a+J9lWhB7O5yGjeIC3gPWdDmb7qCaDJ7bl3D8+fxNcdSgkdCRnrSUnK9jaFCNNSceup9QaD/yLNh/17J/6CK+bda/5Dmof9fMn/oRr6S0H/kWbD/r2T/0EV8261/yHNQ/6+ZP/AEI1tW+FHjZR/GmewfBn/kWb3/r8b/0BK9Grzj4Nf8izef8AX43/AKAlejVrD4UeXjf94l6mReeHdF1Cdri80u0nnbG6SSFWY44HJFTafoum6Vvexsba2ZwA5hiCbseuK8p8d+M9d0vxZd2dlfNDbxqm1AinGVBPUetbfww8Satrt5qCajdtOsMaFAVAwSTnoPakpx5rGksLWVD2rfu9jL+NH/H9pf8AuP8AzFcj8P8A/ketK/66H/0E113xo/4/tM/3H/mK5H4f/wDI9aV/10P/AKCaxl/EPYw3/Ivfoz3Pxh/yJusf9eUv/oBr5nr6Y8Yf8ibrH/XlL/6Aa+Z6K26Msm+CZ9MeEP8AkTdG/wCvOL/0EVu/xVheD/8AkTdH/wCvOL/0EVvd66I7HhVf4kvVi0UUUzMKKKKAPljVp5v7avv3r/8AHxJ/Ef7xqn9om/56yf8AfRq3q0Uh1m+Plt/x8Sdv9o1T8qT/AJ5v/wB8muFt3PuadGnyLQX7RP8A89pP++jR583/AD1k/wC+jSeVJ/zzf/vk0eVJ/wA83/75NK7NPY0uwv2if/ntJ/30aPtE/wDz2k/76NJ5Un/PN/8Avk0eVJ/zzf8A75NF2L2NLsL9om/57Sf99GkaWRxhpGYehajypP8Anm//AHyaPKk/55v/AN8mi7GqVNa2GV3nwl/5HM/9er/zWuG8qT/nm/8A3ya7v4So6+MyWRgPsr9R7rVU/iRzY9/7NL0Pds8V4v8AGSCRdZ0+cqfLaFgG9weR+or2jjFYnibw7a+JdKksrjgnmNx1RuxrqnHmjY+UwdZUaym9j5/8L64fDuvQ6j5XmImVdc87T1x7161/wt7w9t/1d5n/AK5D/GvJNd8Nan4eunivbdhGDhJlGUcdsH+lY9cynKGh9LVwVDGNVW/uO58feN4PFCW9raROlvC3mF5RhicYxjPSsbwPZy3vjHTI4lLbJhK59FXkn9Ky9P0u91W5W3sbZ5pGOMIOB9T2Fe8eCPBsPhfT98pEl9OAZnHQf7K+386uKc5XZz4upRweHdGG7G/EuCS48C6gY1LbAjkD0Dgn9K+fa+r5Y0mjaOQBlcYKkZBFeF+Nfh9eaJdSXWnRNPYOd21BlovYj096qtBvVHLlOKhFOlPS+x1elfFzSv7PhF/bzpchcSCNAy5Hcc1YuPi9oa28hhgvHlCnarRgAntk5rxGis/bSO55RQbvqT3l097ez3UgAeaQuQOgJOa9j+D0EkXh+7mdcRzT5Q+uAAf1rgPCfgfUPEd3G8sUkFgCDJKwxuHouep9+le/2Fhb6bYxWdrGsUMS7UUdqujF35mcea4qnyKjD/hjwX4mWctr45vZJB8twEkQ+o2gfzBqt4I8UJ4X1h55ome3lTy5Nv3lGcgj1r2Pxn4StvFWm7MiO8iBMEvofQ+xrwPVNIv9Fu2t7+1eJwSASPlb3B6EUqicZcyOnA1qWKoexnulax7N/wALe8PbcCO9z/1yH+NeWeM/Ea+J9dN5HEUhjjEMYb7xAJOT78muerQ0jQ9R1y6W3sLV5STgtj5V+p6CodSUtDalgaGEftb/AHnU/Cm1kn8apKgOyCF2c/UYH869B+LHHgiQf9No/wCdafg7wpb+FtOMKnzLiT5ppSPvH0HsKzfisGfwVIFBJ86PgD3rdRcYWPGniI1sapra6PB4v9en+8K+pryyiv8ATpbWdQ0U0ZRwfQjFfLsUE3nJ+6f7w/hNfVkf+rX6VNFaM6s5dpQa8/0PlzWtLm0TWbrTpwd0DkAn+JeoP4jFZ9ev/Fzw6ZobfW7eMmSL91MFHVT90/gePxryTyJv+eT/APfJrKUeWVj1MHiVWw1+vU+m9AGfDdgPW2j/APQRXzn4igktvEupwSqQy3UnX03HB/Kvo7w+CPD9hntbx/8AoIrjviD4EGuRnUtOULqCLhlzgSqOx9x2repFyjoeFgMVGhiJc2zOK8AeObbwxbXFlfQyNBLJ5yyRDLBsAEEZ6YArtv8Ahbug4/1d3j/rkP8AGvFbm1uLOdoLmB4ZVOCkikGoKyVWUVY9epllCvJ1O5q+I9abxBrt1qTRCPziNqg5woGB+OBXofwZspR/aV8y4hfZGh9SMk/zFcX4Y8G6h4ku0CxNDZg5kndcAD29TX0BpWl22j6dDZWkYSKJcKO59Sfc1VKLcuZnFmWIp06X1en/AMMeXfGj/j+0v/cf+Yrkfh//AMj3pX/XQ/8AoJrsPjMjtfaZtRmxG/QZ7iuS8ARSL450otG4AkPJX/ZNKX8Q3wz/ANgfoz3Hxf8A8ibrH/XnL/6Aa+Zq+mfFwJ8HawAMk2UuB/wA181eRN/zyf8A75NFbdGeS/BM9a0H4oaJpmhWVlNBdmWCBImKouCQoBxzWkPi/oOT/o16P+AL/wDFV4n5E3/PJ/8Avk0eRN/zyf8A75NT7WSOmWU4eTbd9T3vQ/iPpeu6vDp1rFdLJNu2GRABwCfX2rtOtfPnw3jkXx3pxaNgAH5K/wDTNq+hK6KcnJXZ4OPw8KFXkhtYfRRRVnEf/9k=</t>
+        </is>
+      </c>
       <c r="N32" t="inlineStr">
         <is>
           <t>Finance &amp; Accounting</t>
@@ -3282,7 +3374,11 @@
           <t>BRAC</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEAYABgAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCACWAbEDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD3l8iNiAMgZrwm88beIrXVbtYtTYKk7qFaNCAAx45Fe7OP3L8/w181ar/yGL7j/l4k/wDQjXVhYqTd0fR8OUKdac1USei3VztNN+K2pwSAX1tFcxeqZRh/MH8hXf6D400jXwI4J9k+MmGUYb/A/hXgP3TSozxyLJG7I6nKspwQfauieGjLbQ9vGcPYeor01yy8tj6hGOMClwPSvNPAfjh7110rU3BuAP3Mp/jA7H39+/16+l9eAa4JwcHZnxOKwtTDVHTmtfzH0UUVBzjT70w8+lK7qi5YhfrXL6v470PR2eOW6Esy9YoRuYH0OOAfqRVKLlsaU6NSrLlhFt+R1QpPwrya9+LkzErZacFHZ5pP/ZR/jWNL8TvEbn5ZLeL2WL/Emtlh5s9WlkGMmr8tvVnuWfpS5+leAv8AEDxOzEjU9gPQCFMD8xTf+FgeJ/8AoLN/35j/APiar6pLujf/AFaxnl959AZFGa+f/wDhYHij/oLt/wB+Y/8A4mj/AIWB4o/6C7f9+Y//AImj6pLug/1axndfee/5+lGRXgH/AAn/AIoP/MWb/vzH/wDE1LB478VS3EcKasd0jhR+5j6k4/u0nhZLqiZ8O4uEeZ2+898oqOJi0ak9SKkrmeh4LVnYZkcGjOa5rxvqd3o/hi4vLFxHMjIAxUHALAHg+1cLpHxVvrZ9mp2yTwn+OEYYfgTg/pWsaUpxujuw+W18RSdWmrpO1up7B06Cjis7S9UtdWs47q0lV43GQQf84+laPQ5rNq2jOKUXFuMlZofRRRSEFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUARSf6p/8AdNfNGq/8he+/6+JP/QjX0tJ/qpPoa+adV/5C99/18Sf+hGuzCbs+q4X/AIk/RFOiiiu8+1JYpJYJ0licpLGwdWHVSOQa+ifDOrLrXh+0vRgNJGNwHZhwR+YNfOXvXsPwluWl0K5gY5EU52+wIB/nmuTFRvG/Y+X4kw0XRVXqn+DPQzxWZq+r2miWL3d7II41H4k9gB3NT6jfwaXZSXly4SGIFmNeB+JPElz4i1Fp5iVhQkQw54Qf1J7muWjSc35HzuVZZLGVNdIrd/oaPiPx3qeuOYYGa1s+gRDh2HuR/IcfWuSIo5NJXpRhGKsj7/DYOjho8tONgoooqzrCiiigAooooAU9M+tbnhHTzqPinTrfB2rKJW+ifNz+WPxrD/hr1P4U6EyJPrUy43jyoP8AdB+Y/iQB+BrCtPlg2eVnOKWHwsu7Vl6s9SQYUD0p1FFeWfmpxnxN/wCRLu/96P8A9DFeF+te6fE3/kS7r/ej/wDQxXhfc16OF+D5n3fDP+7S9TuPhnrMlj4g/s92Jguwdq9g6jIP4gEfgK9rwCa+dfCrFfFemkHB84D86+iUOUH0rDFRSlc8PiKjGnik49VqS0UUVyngBRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFAEMn+qk+hr5p1X/kL33/XxJ/6Ea+l5P8AVP8AQ180ar/yGL7/AK+JP/QjXZhN2fVcL/xJ+iKdFFFd59qha9b+EH/IL1An/nuP/QRXkden/DW8Ww8N6vcynCRuZGPoAgNc+IV42PD4gi5YVpd1+ZX+KHiBri+XRrdh5UOHmx3YjgfgOfx9q85PBqe7upL6+nuZWBkmkZyfcnNPsrC91CfybO1eeTOCEBOPr6fjVU0qcLG+BpUsFhYpu3d+ZVorroPhr4jnjDGCGI/3ZJOf/Hc0TfDbxHEMrbQyf7kg/rin7aHc0/tbB3tzr7zkQKMVpXmjz6fL5V6620h6CSOQZ+mEOfwq1aeGZtQcJbalpskh6J9oKsfwK5quZNXRo8woJXT079DCpciuyHwx19uj2X/f1v8A4mpP+FXeIv71n/38b/4mp9rFdTH+2MGvto4nPPTFH1rvLf4Va07fv7i1iX1UlyPwwP5102j/AAs020bzdRme7kH8JG1PyHJ/OoliIpbnNXz/AAlNXi7vsjg/CnhK78SXiko0enof3kpGN3svqfft+le62dpDZWkdvAipHEoVVXoAOgp0FtDaxLHAioijAVRgAfSphnOc8Vw1Krmz43McxqY2peWiWyJKKKKyPOOM+Jv/ACJd1/vR/wDoYrwvvXunxN/5Eu6/3o//AEMV4XXo4X4Pmfd8Mf7tL1Njwtj/AISrTCennr/OvooEBM9BivnTw0yxeJ9PkJGxZgSSenNdP4t+IFzqEr2WlStDaJlWmU4Z/oew/U1Nem5zSRy5xgKuLxkY0+2r6I9G1Xxjomjny7m+QSjrGuXYfUDOPxrnX+Lejq5UWl64H8SouD+bV48Sd2TyT1NISCaccLFbm9HhrDqP7yTbPa7X4p6DOB5xnt8/89I8/wDoJNdRp2tafq0TPZXkcwHXYwJH1Hb8a+bM+lTW1zcWU4ntp3hlHR42IIolhYv4WZ4jhmm1+5k0/PY+nc9OaUGvNPB3xDa+lXTdZKi4f5Yp1GFkPoR0Dfofbv6SD3yOa4pwlB2Z8nisJVw1TkqKz/MrXl5b2Ns9xdTpBEmN0kjBQMnAyTx1rP8A+Eu8P/8AQYsv/AhP8azPiVn/AIQi9I9Yv/Ri14TjGK2o0FUV2z1crydY6m5uVrOx9GW/iLRr65W3tdTtZpnyFjSVWY8ZOADnoDWtu65I4rwDwH8njjTT6O//AKLeuq8b+OpEmk0rSZthQlZ516g91B7H1P5USoNS5UTXyWccUsPSd7q7fY7fVvGOjaKNl1ep5w/5Zp8zfiB0/HFc4fi3pAJAs70gdwi8/wDj1ePszsxZyWZjkknJJpOtdEcLFLU92jw1QjH95Jt/cfRuga5B4g0pb+2R0RmK4kAByOvQmteuJ+GG7/hEIR0XzH/9CNZfjT4gHT5pNM0kq1wnEsx5VD6Adz+g9+3G6Tc3FHy7y+dTFSoUVs38l5ne3+p2WnwmW8uo4Ix1Z2AH61zV18TPD1sSEuXnI6iOMn9TgV4pdXdzezma6nkmlP8AE7EmoOO4rqjhV1Z9DQ4Zgl+9k2/LY9hPxc0cHH2K+PvtT/4qp4PivocxxJFdQ/78YP8A6CTXi/FHFX9Vgdf+reEa3f3n0PpvizRdVIWzv4WkPSMna/8A3ycGtwEtzuBX2r5dGAeldn4Y+IF/o86Q30r3VkTglzl09we49j+FY1MK0rpnlY3hydGLnRlfye57jmlqpaXcV7bRzwurxyKGVl6EHoat1xtWPmGmnZjfwqKWZIlJkcKBzyawvEvie08N2XnXLF5m4iiX7zn+g9T/APqrxrXfFOqeIJWa5nMcGflgQ4UfX1Pua2p0JT16HqZflNbGarSPf/I9evvHvh6yO19QWRumIgW/VeKxpPi1pAJVbS9cD+JUTB/Nq8d4FHFdawsFufSQ4aw8V70m2ezQfFjQ5WxJDdQj1dAR/wCOk1vab4w0PVsLa6jEZG6Ix2sfwOCfwr57HHvQRntilLCxewVeGaDX7uTT+8+ot6sARgg0pxjArwjw7481PRJFjnka7s+hjkbLoPZj/I8fSvZ9L1S11ayiurSVXikGQR/L2I9K5KlGUHqfLY/La2Dl7+qezRpfhRS0VkefqRv9xvpXzZraeXr+ooRjFzJx/wADNfSp5yteA+PrQ2fjK84ASbEq++VAP6g11YV+80fS8NVFHEuPdfkcxRRRXon3YuM810un3/2TwDqcQYh7m5WIY+gJ/QGub3fLXQ+H9ObWvsmkqDtlvHkkYfwoqLk/k2B7ms6lrXZ5uZuCpKUtk038tS/4O8Ey+IXW7ut0Vgp+hlx2HoPU/gPb2TTdKtNMtRBawpHGvRUTFTWlnBZWsdvDGqRooVVXoAOlWB16151SrKTt0PgsdmFXFVG27R6IeKDS0VieeZmp6TZ6ratBdwpJG3VWXP4j0PvXjPjLwZL4dm+0Wu6Wwc4yeTET0B9vQ/h9fdiPm61VvrGDULV7edA8bqVKnoQa1pVZReux6GAx88NUTvePVHz1p3iHVtJZRZ38qRrx5bNuX8jxXoOhfFKGQLba1b+U3Tz4slSfcdR+Ga8817SG0XW7qwYlljbMbHup5H6VmdRXfKnCor2PtqmXYTH0VUUbX1TW59N2l5BeW6T28qyRMMqynII9c1az79K+efDPivUPDdyDEzS2rH95ATwfcehr3LRtYtdc0+O8tH3RuO55B7gjsRXDVoyg/I+NzHK6uDld6xez/wAzWooorE8sKKKKAOM+Jv8AyJd3/vR/+hivC+9e6fE3/kS7v/ej/wDQxXhdejhfg+Z93wx/u0vUcCVPBIPqKsafp91ql2tpZwNLM3QdgPUnsPeqnSvdPAXh1NF0NJ5ExeXIEkjMOVB5C/hn881pWqciv1OzNsxWCpcyV5PRIwNL+E8QVZNUumd+pji4X6ZIyf0raf4ZeHPLI8iYHHUTNn9Tiu27daUgGvPdabd7nw880xc5czm16HjWv/DK7sIWudLma5jUZMLgB8exHB+nH41wBypKsCMcEGvqE8nBwVIryH4m+Go7G6XV7WPbHMcTKo4Ddm/Hv7getdFCu2+Vn0GTZ3UlUVGu732f6M8778V7b8PfEz61pJtLp915akKzHq69m+vY/TPevEuldF4K1Q6R4qs5C2I5m8mT3DcD/wAe2n8K3rQU4+aPVzrBLEYeU7e9HVf5HqnxL/5Ee9/3ov8A0YteE9692+JJz4GvCO5i/wDRi14T3qMN8HzOThhfuJev6F3Tb6bTL5buEkSIjhCOoJVlB/DOfwqkSWJJJJPJJo69a7/4feD49XkOq38e6zjbbHGRxKw6k+qj9T9OdZyjBczPVxtejg4Sry3282c3pPhTWdaCta2hWE9JZRtU/TPJ/AGtv/hVniADO+zPt5rf/EV7VHEka7VAAHHFSYI6VxvFSb0PkK3EOKlO8bJHmbvf+B/h68FwYxePIUj2HIy56j6DJ/CvKeWJdmJYnJJPWvX/AIlaRrGtJYw6dameKMs8gDKMHgL1I/2q8/8A+EF8SbsHSpM/9dE/+KrejKNuZtXZ6+TYnDxhKrVklOTu+hgorSSLHGpZnIVVUZJJ6AV6JofwsmuYVn1a4aHcMiGHG4fUnI/AD8aPBHgrVbXxAt5qdkYYYUYoWdWJc4A6E9s/pXrYUAcis61dp2izlzjOp83s8PJW6tHGJ8MPDqx4aCVz/eaZs/oRWfqHwo0yVGayuZ7eTHy871/EdT+dei8Z4FH+etc6rTXU8CGZYqLupv7z5v1nRbvQb42l4o55jkX7rj1H+FZhGGr1f4uRxGwsX2jzhLgHvtI5/ULXk/UE16NKTnBNn3uU4qWKwynNanrPwo1aSaxudMlJKwMJIyfRs5H4EZ/Gu+1G+h0zTri8nbbHEhdj7CvKfhIT/bt4M8fZxx+NavxZ1Z4ra10yNiBMxkfHovQH6k5/4DXHOnzVeVHymMwSq5m6UdE7N/qeea3q9zrupzX1yTljiNM8IvYD/PrWZ2o9q6HwboB8Qa/HA4zbxDzJs9wOg/E4/DNdjtCPkj7OcqeBw7a0SRc8NeBb/wAQ7bhybWzPR2XLP9B6e5/Wu8tfhZoMSATCadu7NIRn/vnFdtFGsUSoqgADAAGBipcGuCeIm3o7HweKznFVptqVl2R57qHwq0iZCbOaa1fHHzbh+IPP615v4g8NX/h28EN2oMbk+XMv3XH9D7V9EMOPvYrB8U6Iuu6JPZlVMhUmIkfdfHB/P9CauliJJ+87o3y7O69Gqo1JXi977o+e+9dh8P8AxE+j66tpKxNpdkKQTwj9Afx6H6j0rjuhwacHYOroSrKcgjsa7J2nFpn2GLhRxVBwb3Ppv7WtFeU/8LCT1P5H/CiuX2ET47+xqnl95693ry34r6SSLTVkUfKTFKcdjyv4Zz+dep1la1pkOs6XPYSj5ZVIJx0PY/UHB/CuelPkkmedgMS8PiI1Oi39D5upc5q3f2M2majPY3KbZYW2t6H0I9iOfxqnXqxfMro/T6VVVIKcXdMK9Q+EtskjXs5H7yM7V9g2Cf8A0EV5fXqfwgmUxalBxuV0b8CCP6VliPgZ5GftrByt5HqtFFFeWfngUUUUAFFFFAHkHxbs1i1HT7tV5eN42P0II/ma83716h8X2401Aehcke/GP615dXqYd+4j9FyGTeCjfzFHWum8G+JpPDurDe5+xzkLKp6L6MPp39q5ijkmtJRUlZno4vDQxFJ05K9z6hicSRo68hhnipPSuI+GmstqWgC1lbMto3lnPUrj5T+XH4V3FeVOLjJpn5fiaLoVZU5bpjqKKKgxOM+Jv/Il3f8AvR/+hivC690+Jv8AyJd3/vR/+hivC69HC/B8z7vhj/dpeppaHaG+8QafasAyvOu4Huucn9M19IRKEjVfQV8/eBufGmnZ/vt/6A1fQQwRWOLeqR5HEs28RGPRIkooorkPmyLGPwrF8Waf/anhm9ttoZmjJUf7Q5H6gVunAqGfBgkB6FTxVRdmmXQm4TUlunc+X6kDtG6SIcMpBBHYimY4NJXrfZP1X46OvVHt/jqUT/DeWUHhliYf99qa8R/jr17XnaT4OQuxyxt7ck+p3JXkJ61jh1o15nh8Orlp1F2kx6xtLKIkXc7kKo9Sa+j9B09NL0S0s0AxFGBkDqccn8Tk/jXz5ogDeIdNyM5uogfoXFfSacIo9qyxb2R53E9VucafTclpO1LRXEfKEfVecUYUc4qtfXlvp1q9zcSLHFGMszHAAryjxB8T7q6d4NIj8iEcee4DM3uB0H45/CtKdKU3oduEwGIxbtSWnV9EevGRVGWdR+NZ9zr+k2XFzqNvFj+/IAf1NfPd5q2o6iWN3ezzA9VaQlR9B0FUuldKwvdnv0uGJNXqT+496n+IXhu2OG1FXP8A0zjZ/wBQMVi33xZ0yEFbO2nuGxwxAUfrz+lePVZtbK6vWK2trPOQcYijLH9KtYemtzqjkOCp61JX9XZF/XvEN54hv1ubsqqpkRRIflQHr9Se5rI6da0tV0S/0dYGvoPIaYEhCwJAGOoHTrWafeumKjb3dj38JGiqSVG1ltbY9A+E3/Ifuz/0w/qKzPiPc/afGlyvaGNIx+W7+bGtH4Uf8h28/wCuH/swrn/GrFvGOpnqfMA/JQKwiv3r9DwqMFLOJt9EYPavWfhJZhbC9vCMNJIFBx1AGf5sa8lr2/4XqB4QjIHWR8+/JoxLtTNuJJuOEsurSO5ooorzT4EKTFLRQBQ/suzJz9mi/wC+B/hR/ZVj/wA+sP8A3wP8KvUU+dl+0n3KH9k2X/PrD/3wP8KKv0U+Zj9rPuLSYpaKkzOE8c+Dhr1t9ts1AvohlewcehP8jXi80MkE0kUqNHJGxV0YYII7GvqDtyetcj4q8E2PiJDMF8i8UYWZB19iO4rqoV+X3ZbH0OU508NalV1j0fY8J4z1rrfh7rC6T4pjEzkQXS+UxJ4DZyp/PI/4FWZrfhfVdBYi8tj5IPE0fKH8e344rGBYcg4I6Gux8s42XU+srOjj8PKEXe63R9RK24ZHQ07vXn/gXxmmrQx2F9IFvo1wCTjzQO49/Ufj9O/BHXNeZODg7M/OcTh50KjhNWaH0UUVBgNprHGSR2pcgDk155498ZppkT6bp8gN9IMMyn/VKe/19B26+mbhBydkb4bDzxFRQgtzj/H2p/2trFxJG2beCRbeMg8FlDFz+bY/CuOHQ1sXFsYfCVnO3We5dgfYAL/MGsf+CvUppJWXQ/RssioUFTjsrr7hKKKK0PSO3+GOoG18Um1LYS5iI2+rLyP03fnXtw6V85+Frn7L4q02X1nWP/vo7f619Fp9xT7V52KVpXPz/iKko4rmXVElFFFcp4BxnxN/5Eu6/wB6P/0MV4X3r3T4m/8AIl3X+9H/AOhivC69HC/B8z7vhj/dpepreGbz7F4p064PQThSfQN8p/Q19GR42DHcV8ugkcg4I6GvoDwVrq69oEMxIMyDZKO4cdfz6/jWeKjszh4mw0uaNZbbP9Dp6KKK4j5IYSMis7WbtdP0e8u2OFihZ/yBNaPGfwrzr4o64ttpaaTE4825ILgHkIDn9SMfnWlOPNJI6cFQlXrxgur/AAPIAcUY4zRj5c1qeH9POp+IbG0C7g8qlgf7o5b9Aa9Ru0bs/Ta0lRw7ctkj1PxhbfZPhe8GMBI4UwOMYdRXjB5Fe6fEcbfAV2noYv8A0Na8LrHDu8W/M8PhuXNSm31bNDQf+Rj0v/r7h/8AQhX0on3B9K+a9B/5GPS/+vuL/wBDFfSifcX6VhjPiR5fE38ePoPpKWmt90/SuQ+ZPGvihr0l1qo0qJyIIAGkAPVyMgH6Aj864DGB9a1fE1w9x4o1SRuv2l0/BSVH6Cso8sBXrUoqMFY/TcqoQo4WPL1S+9m54b8MXfiS7aO3YRW8WPNmYZAz0AHc16lp3w10GyRTPC91KP4pnOPyGBSfDS3hj8HW8wUBpZJGcj1DkfyArtBxnP4VxVq0nJpPQ+PzXNcROvKnGTSTa002Mq38N6RaNmDT7aM+qwqD+eK00gijGFjUD2FSZpSQOtYOUnueK6s57u55J8XgBe6Xj+7L/Na81713/wAVL+O51u1tUYFreMs+D0LEYH5AH8a4CvTw/wACP0TI01go38z0D4T/APIevP8Arh/7MKw/HcLw+MdQDDCyMjqfUFFB/UGtv4Tf8h+7/wCuH/swqf4s6a0Oo2eoop2yRmJj2BByPzBP5VkpWrNdzzY1lTziSfVWPOeSPpXsXwnu/N8PTwE/6qdgB7HB/mTXjoPX3rsfhxrX9leIRbyvthuwEyTxvH3f5kfiK0rx5oOx6Ge4d1sI+Xda/ce7UU0HIyKdXln50N7UhIAJPYc03OT+Fc74y1gaJ4duLoPiUqY4we7twPy6/QGnFXdi6VOVWahHduwjePvDQJH9qRcex/wpP+E/8N5/5CUX5H/CvARjuamtrZru7htYwPMlkVFHuTiu36tG259fLhyhCnzymz3n/hP/AA1/0FIvyP8AhRWX/wAInZ/88aKn2EO54/1XA/zM7nPSgHk8UhYYzntmvNvGPxCawlfTdIKNcLkSTNyqewHdv0H8uaFOU3ZHm4XC1MTPkpq7/I7691Oz0+Iy3VzFEg6s7BR+tYU/xC8NQtsbUgT6xxs4/MAivC7u6ur2cz3c8k8h6s7En/8AVUFdkcKurPqKHDEbfvZO/ke4SfEbwrICslwxB45hfB/SuW1Of4eakSyvJbSMPvwQun6bdv6V5xnHejLGtI0FHVNnoUsgp0XenOSfkzoLqx0KGYS6d4hl3Kcp5ts6kEdPmAH8q6LQ/iNeaagg1C4gv4gcB13rIB75QA/p9a896e9HXtVypKSs9TpqZTSqxtVbfra/3o9rh+KWguvzm4iPoyE/yJpbj4paBFHujM8p/upGQf1xXiVLWX1amcX+rWFve7+87nXfiXqepK0Onp9jgPBbdmQj69F/DJ964ht8rliWd3OSTySTTccZFdV4C0VtX8TwPIuYLUiWT0J/gH4kZ+gNW1GnFtI65UMNl1CU4xtZfeafjfTTpXhjQrXADLkNj1IBP6k1wR616r8Xvlt9MA7M/wDIV5X/AA0UHeN2TkcnUwvM922/xG0UUVue0aGi/wDIe07/AK+ov/QxX0pF/qk+lfNei/8AIe07/r6i/wDQxX0pF/qk+lcGM3R8RxP/ABo+hJRRRXGfLnGfE3/kTLr/AHo//QxXhfevc/ib/wAiZdf70f8A6GK8Mr0cL8HzPuuGP93l6hznmtfQPEN54evhdWx+U8SRE/K49/f0Pap/CGnR6vry2E4zHLC4PqOOCPcdar69oN94f1BrW8Q4yfLlA+WRfUf4dq1lKMnys9OtWw9WpLC1NW1ez6nr2kfEHRNTjBluVtpP4knIXB+vQ/nW82t6bFF5j31uI+u7eAPzzXzZxR34rB4WLejPGq8M05S5oyaXbc9p1/4k6TY25j0+T7ZcHhRGflHuW6EfTNeRX9/c6peSXt3KZJpDk56AdgB2Aqpx3o47VtCjGnserl+VUMEm1q31YEleK9Q+FeguDLrU64UgxQDHUZ+Y/mMfga5jwn4Ou/EV2skqNHp6H55CMGT2X/HtXudpaQ2dtHbwIqxooVVXoAOlY4isrcqPGz/NI8jw9J3b38l2OZ+Jf/IkXv8AvRf+jFrwk17t8S/+RIvf96L/ANGLXhJqsL8HzN+F/wDd5ev6GhoP/Ix6X/19xf8AoQr6UT7i/SvmvQf+Rj0v/r7i/wDQhX0on3F+lZYzdHm8Tfx4+g+kPIpaK4z5o+efG1g2neLtRj24WWTzkPqG5P65H4Vz31r2zx/4UbXbSO8skH26DOAeN691z+o/H1rxaWOSCV4pkaORDhkcYIPoRXqUailFd0fomS46FfDxhfVKzX6nZ+C/G48Pq1neq8lkzZV15KE9eO4/+vXp9j4s0G/Ctb6lAWcZCswDfkcGvnrOKMEUp4eM3fYyx2Q0cTN1Itpve2x9H3HiDSbaPdcajbQj/akA/rXGa98TrKCMwaQpuZyMea4KoPz5P8vevIx9M0dTgVEcNGLu9Tnw/DeHpPnqyv5bIluLiW7uZbi4kaSaRiWc9STUX8OBW/J4R1SDQJNWuLdoo0wViZfmIJwSR2xnv6VgdRjFdEZRex7uGrUZpwpNNLTQ734TyhfEtxH3e3J/Jh/jXpPinRE1/QriyJAlI3RPjo46H+h9ia8V8I6sNF8SWt3I22EkxSn0VuM/gcH8K+hEYOqyIcqRmuHEXjU5kfHZ7GpQxqqx0uk0/NHzHNDLBcSW80bRyxMUdT1UjqKZkjkHBHQ17L438EDWSdQ05VS+QYZSMLMB2J7N6H8Pp5BdW89ncNBdRPFKhwyMuCK6qVVTXmfSZdmVLGUrN2l1R6T4W+JEUdutnrZZHUBVuVyQ31A5z7/yr0G18QaTeR77e/gkX1Dg/wBa+bsE9KMY6iolhVJ3Whw4rhyjVm50243+4991TxvoelwsXvopJRx5UTB2J9MDp+OK8g8TeJ7rxLeB5T5dtHkQwg5x6knuTWDmjgVcKEYO/U6sBktDCS9o/efd9PQBn8a734aaC95q51aVD9ntsrHkfecj+g/UisPwz4UvvEl2BGrQ2in95ORx9F9T/LvXuWlabb6Rp8VlaoEjiXaB6+pPqT1rPEVklyrc4c9zWEaboUndvfyRf8pfSin5orgvI+L5zivH/iNtD0fybY4vLkFI2HVB3b8M4Hua8QJJ+YnJPU11Pj3VW1LxXOAwMVuoiQA+nJ/HJP5CuU5PavTw8FGPqfoWR4NUMOpW96Wr/QKKKK3PcCiiigAooooAUjHejNGM1Pa2tzfXS29pE0srnAVRk/8A6vepem5nUqxprmk7Ibb2893PHbwRtLLKwVEUckmvefCHh2Pw5oywthrh/nlYd2PYew6CszwX4JTQQLy72y37LgsPuxg9QPf1P+T3GBnrXn163N7q2Pg86zX61L2VN+6uvdnmnxfj/wBA06XssxXp6qf8K8nPBr3T4j6b/aHhOdkUNLbETKPp1/8AHSa8L6rXRhXeFj3uG6qnheRbpsSiiiuo+iNDRf8AkP6d/wBfUX/oYr6Tj/1S/SvmzRf+Q/p3/X1F/wChivpOP/VL9K4MZuj4fij+NH0JaKKK4z5gyNa0a21zTnsbsv5T4zsbB4ORz+Fcx/wqnQ+73P8A38/+tXdj60NzVxqSirJnRRxdeirU5NLyOS0jwDpWiakl9amczKCBvfIwRg8Yrd1LS7PVLc297BHLEezrn/8AV9a0MAUh9MUnKTd2yJ4irOaqSk2116nnGo/CaxlLPp97Lb56K48xR9OQfzJrDm+E2qrn7PeW0npvBX+Wa9kPNL2rVV5rqd9LOcZTVlO/rqeNW/wn1Zj/AKRe28Q7+Wpf+eK6jR/hfpNiyy3zveyjtIAEz/ujr+JNd5jij2pSrzl1JrZvi6y5ZSsvLQjihSBAkaqqgYAAwAKmoorK55rbbuzK1rRrXXdNksbrd5MhXO04PBDDn6gVy/8AwqnQs8vc/wDfz/61d2OnWkPPpVRnKKsmb0sXWoq1OTS8jibX4Z6HaXkNzG1y0kUiyKGkyMqcjPHqK7RBgYA6DinAc9Kd3pSlKW7IrV6ldp1JN27jqKKKkzGEZXFc7rfgzSNdG66t9swGBJGcMPx7/jXR0w/hTUmnoXTq1KUuaDafkeU3fwhnBJstUUr2WWLkfiD/AErPHwp1reQ11abexDMT+WK9p200g+tbLETXU9SOe42KtzX+R5ZZ/CI7gbvU/k7rFFg/mT/Suv0fwTouilZIbUSTj/ltKdzfh2H4AV0i/XNLUyrTluzmr5niq6tUm7divcW8VxA0EiKY3UqQRkEHqK8z1T4Vb7hn0y8ESMc+VKpYD6Ec4+o/GvVcCk7cVMKko7Mzw2NrYaTdOVrnjkPwm1Z2xPe2yLnqgLHH0IFeheGtDvNDsFtbjUXu1XhQyABR6DqcfU10POKBnHNVOtKS1NMVmOIxStVaa9BB0+bGaxtX8N6ZrUe28tUc44YjDD6EcitoZHpQfaoUmndHHCpKnLmg7PyPML74SQsS1jqMkXfbLGH/AFGP61jy/CjWh/qrm0fn+MsvH5GvZ8UGtViKi6nqU87xsFbmv6nj8Xwk1Jz++1CCMeqxlz+pFdLpPwv0eyYSXhkvJBzhzhP++R/Umu7xx1o6ClKvOXUzrZvjKq5ZTsvLQhgt4raJUijVEUYCqMAD0xViiisWzzW23di0UlFAHy7dTCe8mnHIeQuc+5J/rTM19E/8Ij4f/wCgNY/9+E/wo/4RHw9/0BrH/vwn+Fd6xaXQ+vhxLCC5VB/efOlFfRn/AAiPh/8A6A1j/wB+E/wo/wCER8P/APQGsf8Avwn+FH1uPYv/AFoj/J+J850V9F/8Il4f/wCgNY/+A6f4U5fCmgKwZdIsgw6EQLx+lH1tdhf60R/kf3nzkDWlaaFq2oEC20+eTP8AEEIX/vo8V9Cw6TYW/wDqrSKP/dUCrioqjCqF+gqXi30RhV4nnb93D72eP6P8KtRuJFfVJ1to+6RHc5/HoP1r0jRfDOmaDAI7O3VSR8zkZZvqa2gKD0rnnWnPdniYrMsRif4ktOy2H0UUVkcBBLGs0RjYcEY5rwbxj4Xn8O6ozJGzWEzExv1wf7h9x29R+Ne+c561V1DT7bUrR7a7iWWJxhlYcGtaVRwZ6OW5hPB1eZap7o+ZhxR1r0LxD8ML21d59JcXEJ58pzh19geh/Q/WuGvLO7sZfKu7aaCQ9pFKk/TPWvQhUjLZn32FzTDYiN4y+XUm0X/kPad/19Rf+hivpSL/AFS/SvmvRf8AkP6cP+nqL/0MV9Jx/wCqX6VzYvdHy3E0lKtG3YlooorjPmQooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAKKKKACiiigAooooAaelVZre3uFZJIlcdwygg0UVUWOMmnoZMXhXQzcJcJptssqPuVhEBhh0PFb33VwO1FFE5NjdSU7czuSUUUVJIUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQAUUUUAFFFFABRRRQB/9k=</t>
+        </is>
+      </c>
       <c r="N33" t="inlineStr">
         <is>
           <t>Finance &amp; Accounting</t>
@@ -3374,7 +3470,11 @@
           <t>MHDO</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAJQAAACjCAYAAABsQzfBAAAACXBIWXMAAA7EAAAOxAGVKw4bAABUW0lEQVR4nO19d1xUV7f2/e+7942x9957770XFAuiFFGaIEU6qHRReu9VOgjoKFVEEQ3GboIxscSU15iuIirW1Pc+3177cMYBBhhgEJOb8/stheHMzD57P3v1tfZ//dd//Rf+oX9IidTuA/jLkkQiQVJBEv+/vcfyDlG7D+AvS6FRAdi92xahoQEoLS1t9/G8I9TuA/hL0smT+bC2MYeBgQ7MzAxhbm6KYF9PlJeXt/vY2pnafQB/ScrOzoa+ni4yUhORlpYEU1NTaG3RgoenGwoKCtp9fO1I7T6AvyTFx8dgGwPUrVs38euvv+LLr79AaFgQ1Deuh5OTQ7uPrx2p3Qfwl6OQkBBY7DSDjZUFvvvuO4jXl19+iV27HeDq6gwPD492H2c7UbsP4C9FAQEB2Ki2Hjo6Wig+fgwvXv0qBdSTp08QFBwENzdnRERYtftY24nafQB/GUpISGDK9w6YMiX80uXzePn6D8heL14856LQycnpHw71DzVNzs7OjDNp42TpKfzv//4v6l6kS+XmHYWjoz22bdvW7uNtJ2r3AbzTRJf4s7e3B5wdHXD58kW5gKLXLl86zwBlByurf0TeP1RDdJGfKSE5AampcSgpyeOvpaamwsrCDJGRoXj58mU9QNFFVp+Dgy0Tj1Ht/hztRO0+gHeKKiqKGCfaD+MdurB3sIDDbkuYmZkwncid+562G+ozMsTXX38tF1Dff/8d9u93ZUq5X7s/SztRuw/gnSFPT0+YWxjD0tICKamJOFVWitNnTkEiyUFoaDC8vPZhl4M1QkID8PP9SrmAIj3q8OFDMDY2+r8a42v3AbwTFBDgDe2tW2BlbYXi4mN4Wv2cg4Po1atX+OKrOygozGdKdx5u3/lKrg4lXh99fBV6uluQnp7U7s/1D6DaBUw+WKu2FpZWO/FxxUd4/fpVPZD88ccfePHiJV68fIXf//izQTDR9bDyIXz99sPe3vb/Ymyv3QfQrhQWFoZZc+fA0FAXtz6/if/85z+NgkWRi7jX2bOnsUl9I+NS6e3+jP8A6i0QXZ6ebli+cjlMTIxx58vbrQaS7PXgYRVMTY257+r/mC7V7gNoFwoKCsIGxkF27DDCjZu3lAomun777Tem2CfB1tYWmZkJ7f68/wCqjcnOwQrqm9TxQfkH+PPPxnWill4XLpznCXgUTG7v5/0/CaiCC3eYeECbf8+JEwVYunQhYuOi8PLFizYBE11f3Pkcrm57eEC5vef2/wygEioqkCApg4NLMYzMJQiI/qBNv49CIjt26EFHTxdffnmnzcBE15dfUTqLDfz9PZUydtLFdu0pgrlVHly9Chnneyd1s/b78qziG7B2KcLKtTEYPtYfoycGwsaxbbMdyUWgsmoFjhUfY+Z/w76k1l7kv5IckXAdKjo6WmmAWr8pGQOGe2P+0jhYORfCy6ukvQHU/oCiKyvrBtS1MzBxRii69NyLzj3csHB5LDw8ctvse8vKJNhhagQLC3M8rJTv6VbWdfvOLegZ6sPJ1YnHAJU1b4bmWeg/1AudurtjzOQQzJoXCVePYkREvDPAevtfWnDmM6xTT0OPvvvQq78n+gz0Rt/BnjA2bVsW7u/pBkMDPRzJlTTq6W7N9fuf/4tPPruOPY57oKmliZycHKU+Q0jcacxYEIWO3dzQb7AP24jumD4/Cq7+p0CY+1sCiq49noWw23MMiRmXpa+Twh12oBwzF0RyrjR6QjAmTg/D+11dsXBFHCTFV9vsQemiLAB7B0t8++29NgFTdXU1Sk+dhLW1Fc8tLyw80ibPoWV0EP2GePGNOH5KKHr224/BI32xZ98JeKS+8cxf/PTfcHIrhqVNIVRUIv66gAqKLMW8pTEYNsYfNk4F0omwZ6x55sJIdOjigsEjfPlkDBzG/p8aiuDwtg1RREREwMXNBX5+PnhU9UTpYHrBrMWk5HgY6G/lWZ1Hj2a12bMkZH6INWpJfFOOZWJvwrQw9B7giUEjfGDuUMA27pu5XLI2AUNG+UJNJ52P8y8HqIqKJ9ikd5Dtmn0MKCEwthBYvnfIMSxeGc8fnIBGIOoz0AtjJgXDzrUIJSVftemDki9o7z43RESG4X7lU6UDqri4COpq6+BgbY2gt5D+m5ByCbMXR2PAUF8GqFA+n8SpRo0PgIdvKVsHATwbNFLwXmcXTJsXjqiUs389QPkHnkH/YT78IWbNj8TOnRJunRhbHcHQ0b4YNSEIk2aEcTB1670PWwxS3opC6eBA1ShOiI6JxMNH1UoF07ff3YO+3jZs2aLJgFX8NhaNz2lkwnlu1JA+RfNKnGoAm3vVzUlISDjB77O0z+avka5qbK58EdymgErOPMfAEsJ1oq69PLBidSKz2k5i9+4CqKgmoe8gby73CWzdeu/FkpVxbWrVyRIVDTg57UFyciJevZKfbdmS6+WrV4iMjsDSpYtxpA10pqbI0f044/KBTI1w5puUFPVxU4OxXieN/93WuYiLwg5dXJl08IKLe0lbxxaVtGDMNF69IZmZs24YMtIfvQd6YuW6RLZTKphiWILeg/ZzmU9AI5G3RT8LidmCwl7B+HNrvx9E7HOq2WS9yM2tRyVMh3J0dOBJc5SKoozr999/R/HJU1AzNIWdR6AwDgZcGsdzOeP4OZlZJUpaTLro/xD2edaOBYw7hXA1g7g+WX7L1ydCQ0PCdNgijGaA6zfYm2/0ybPCEJt04d0H1B63Qia/A9G9z74a/Wg/lq9N5A+uujGZs+Who/2xRCUaFjZ5HETl5bfgH1yGlOwzLf7e+6WlDESFeBocjGobezzR0sFjdQ2BVq0RiP381cZNsLM3w6df3YayPAZf3P0BprZ7sNV6N1s8DbxITMRTKxs82ci+e+NmPF67EY+nz8ZjFVVhPJs0UW1ugWovXzxPzwHKylr83ClHL8OX6UrZBde4vuTrexLqjCuNnx6CHn092Kb2hYd/CXS2H8TU2RHMKvTG0FH+6NbLHdsMctqSS7X+Q9iehIHZYaYgemH0xGAOqMEjfWBkKoiAtVqpWK4ah90e+fCp0Zc8Mq9gjVYGZsyLRJrko+bv0IQEPA8OYwu1GY/GTEDViDF40K0nHnbvhYf0P1GX7gKxnzN69oLNrl24V6k8Cy85Ox96i1eiTH8Hnm7VR+WwUbjftQfu13znQ/bzw45dpGMQ/tYDjwYPw+NR4/DUYDueeXpzbtbc55ccr4AKkwhjJ4XAzFZQG1JTy7Hd+hC0tudwN8yBzAtwdi7kuiwp7KKLZjqbc7IU3zlA0UX/BwQwHWlDHBdn46aEcD1pODNV/f2FHVhQ9ilOX77B/VDbtyfB2asUS1cmsPv3YpFKnGLfRcQ+oNrPD093O+LJ8pV42LMPHvzrfYE6dK5HlT164/GQEfjh/c5YMW0kkg7m4tWvysksOPfJ19DX1MHBPgwgfQfgwXsd5Y+BjbGye+/ar9O9NWMmcFXNmYenNnZ47uODchKZUMy89w04zTi/Kw9bmdocRFTCJSnnyTtzk/8cwTbu0tUHeCSCrEHSY+l+EyYlZNdR0e9sE0CFhZVjv+8JhCee5r87+RVj3pJYpvz58V1Au2Em2xVJjB2L7yFwbTXOxmKmiPfou5/vlOHjAmBgfqjJ7/ueTcwTR0c8XrcBlVOn437NgtDur2Q7n+gx4w7y6Gv2t8AuHaFvZoG7D5Rn3R09fhbqo0fg3H+/h4eduzU6hrr0qE9/YdyMY4kb4lHvfng4YQoTj2vx2MoKVZmZCq3F6nVJbGO6M93JA1PnRmDL9iwYWuZKHZykWuiaHGY6lBdGjg/C2MnB6D/Ei712iANuEQOwi3cp3DxP4L+U42lv/psc3Y4yXSgB+sbCQ3v4lmAcGyiJuxHjArlCvs0omw84r+wqAiLysGRVHDNfSTF04XrWoGG+2LwlA1ZNuAyq0phy6+mJx1NncpEmTj4tStWAIY0uHP09u3dPaCxdiDOXP8Kf/1FeuOXjT2/DiOlKed26oqr/IIXBVIuGjuTPIRI92/1OXfFo7gI8s9/Nlfum1kLfNAezF0VxhZzmlUJYE2eGQUfvINev+PoEnmZgCmDcyQfjmQQhBV19SzLPViDpoqmbiXWbU2BlpRiIlQ6oVWoHMGpCAEx2CjqSs1cJBxMReb7JzxSRchEXLtyBPbMyps0O524CUsr7D/FhlqArVqgmIrvwcqPfU5mZyxXZB6QXMbFVyf6vGjRMocWqGjwc5T17YNvsaYhOzsazF782jZJmXGThxWcXwW3sGNzp0ImDo0Wgkh0ze7ZHvftzjkeb54nediA/v9E5IjXCkOmqxH3IZTCyxjDqz5Rwta2ZyDv+KXc2L1uTwNdmAtNv6T5VtWRmkAqAWrwqEiOYGNy1v+jtAyoy9SJ3ko1k4srcWlAGHdyPc6BwGso4j14m4jMuQZtxqUHDfXlkfNjoAC4OuzLWPI0phSm5je++aic/PNbQwn2uf3Tiim1TC/KAca57HToiq0MHRHfpDL0FsxAcEYfKJ8rzO4nXf5ipePzCTWipLMO57t0EQDF9rZLRfdLb2Ji/ZxznRwaMR80EG+ld9Mw/M9FOVuojn2CuQzY0V+dvfMfVCdKnCDQELtJnSV9avjYBIZElcHA8xtdABBT5CPX1U5kqUsF9hOTS0WfKvBKafCh+s7f3MSxff4A7ycZODJICaif7f/BIf4byQA6a1RtToLIumT2cD9enJs8M568Tqx3J7vH3P93o9zyxc0TVrDl4QFYS262KLMKPTDHO6tUL9jOnY6/RRrg47kFSxiH8+OCp0twEstetuw/g5eyOyMEDcLffQDzqNwjX3nsfh7p1QWCPLggfOgjhY8YgaNhwnOrHdKYWcDDSse4zPfHRhEl4bGTa6JzlllzBwlXxHBjkHqA5JwARt5qzMBrautmYNidSCqglqxKgoZHIAUXciu4bxiRIUMTZtwcojW0HOWcipXoiE2tbTCRSQNEgSeSJ4CGvLSnpsxdFS8FEFqC2Xnaj3/E4KByP5y0UlG7GlUh0KbKjI4YPgsEOPURlSHD5zi18X/kML1++ghLVJulFiXkxh4qwbOxwJHXtjA8Z6FP79YL73Klw3LYZrk6miIlOQGpOLnyCorBnxlR8QxZnC3QsEvM0F1UTp6C6ibDOAckVzGCgIQkyhIFqLjOUyLLjv7MNT6qICKg5S2OwlnEvAtS6jamcmxGp62RAUnKu7QGVVVSBRStiuVijAY1nA12nnSEXUETkiyIgEdeiXUOWhallHlMELzX4HY+ys1E1bTbflQ+ZckoiRJGJJ/GgsXAy0opP4umL10pVvuVdr3/9Dw4ePgyNBVNhO2kIdqkuhY2FPWKPpuHK9bv48dEjprP9gpevf8PHX96GydY1uNOxU4sV98puDFRsTh6rrgWaKBy1ZBbe9NkRfM4JVOTUpLUgonWpCygLizwsYwYWvUY0Y14UbPcUtj2gPDyO11gIpCv5ckCt1xFSNCxsjtYDFIFp6KgAroCTWWtpX8gXo6HPvxQSgifr1QRLrkMzJp9NeM7/vAetldNx5uZH+OPPtgWTeP30cyXyC44gJekArn5cgR9/esA54m+/vykU/Q8D9vmLV2C7ciG+6tS5VQo7ceufGad6rKndZPjG2/sEA04I06lcmA4ruHJk14XWau7SWA4oE5MsLFt1gL9GwWXSwTZsaVWqS9M30aWqmcZN0sFMjBHKxzDwbDU6zK0MOxdJLUDR/8Rm+w72wgomn5vSmYiqHJxROWaCwjqTSF936QHfju9Db/sO/Pu+crMImrqev/4TD578xkSg/Grj17/+ifRMCcJGDMFPCojuJjkxuUxGj0OVrS3//EbFX85V6O08zNeiN1M/SFKQV332ophaSnldQHHuxdSUBEmL46tN35SRUcrMzgOc05BMJkBRctzWGqvAybMUQ5kCSHJ6wFAfruDNXhCN3cz6i8q8yhTGzxoHLKMn6ps5d2rKtyRLdG9M725YumwRJEUn8OvvrS8jV+b14pffEZ+SgdDhg5UCqEe9+uF+py6onLcI1bGxjc5pWcVdpOZeh3foGWjoUR66jxCYZ+tEoCGHKPmd5AFqIltjB6cWF4soIO4SirhVQIo2sUwRULrGOTy47sAARX+jAPAIprTrGx9CbOoHSD9Uge0WEtg7N65MvmK6U+WMWTxEoag/h3w2nzLRaDR+NPYfOoPH1fUbXLT39QsDeKbkGCxmTca9Ya33U9HccGNl/CQ82rq90TlNyDgJVfVkBujLOJj/CSwdCjGPiTlaI6Llq+O5H4oyEkh5FwFFivmQ0b48SbLNAGVun48FS+ME9MoCyiSbA8rdr4TpS37MiguCV8QHOP3xXRwp/oyzVfKN+AU3XmtXHZ/Ize5HvfoqvlsHDkVu7x6wYeb03R+Vn9KrjItsgw/OX8XqxfMR+d57+IFcAK10gFb1H4wHPfrgiZ5Bo3NKDk1KrKOohbPXCRSdvoWCUzewectBnoK9Yk0Eb0K7XjsJsxfHSAFFcVjKV9fWz+bP0CaACoz8ANPnhksj1iKgjCyEbEy7EAniU4sQmpALV6986Jkc5gAkFjttTjhOXrrVsLijON3GzYJ+0AxA3Rs4BPuGDkBM/AGmCCsnv6ktridPHyM6OhIaKothMm8SDvfr1yrxV8U2EsUwq1asoh6Nja6bg9MxrqYMGOqNteoJsHbI5+GWyAMXkZh2meu/wbFXMGfJG0CREk8hMnIRRZS0KJO26Ztc/E5gukwKRF1AifdZ2OZiyoxQtiv286zM4WP8YW6X1+hnVxcWomrSVGGSmqE//ZvpW/vHTUDaoSNMKX53AUXX4yePUfrhx4g6fARG6zYgs2cPPFDQJSKPKnv2ReWI0XhR2Lh5T/lmi5bH8oS77n09MGZSEFauT2Rr9sZ1sz/kFBaujJcCitwLlPe/XiOl1n1vFVBE1i75PL5Hqag9+3ny2N1qtSR4SBr3mzyLjMXDTt0UCq3I0tf/0wGeEyYj/XDeOw8ousgS/OlRNfTNLeHcpSN+UDAm2RCgaPO9jG5cMSfS1D+IkRMCeSYnTwMetB8qG1OQLPmE/903/CzjUNHtD6hRE4OgY5TD2aZ3aBlHP3nQRTlMOtVO68a5E9ELZ1epV7xZgGLv8R4/HhmHJX8JQNF1+uKXcJw/F9fYZlAkAtAooJgu9Twsssn5zco6j2UqUTw1e0JNpVGvAfuhbZDN07PrWnlvBVD7g09h2tyIeoBS086EhX0eZiyM4vk4VCNG4RVKnKNsguLiG01+9jNrO8UANXQEn0TRe/5V3wGwHzMaMYkH32kdSryqnr7Abhd3hPTqhjt9+rdKMSdA0Zw9c3JRaJF1zA9h0EhfLjkm1lhy/ZleZWp9FB4+BbUARdUzfQd5YaNWKs8AVQqg0nOuIjX/zYd5BpzBnIUxvGqCAEU0aUY41mumYdXaJD4YchdQjR1xKXJuuvo3nS9NSmW1rr5CgPqRsfjz//0e7nXtwSc0r1NHqM2ficycHKUVHbTVReM7d/ka9BdMw5n3O3PFWhmAqjbZifsZGU3OcxgDBuWvkX9w1PggzoUIVORT1NJLw8Ll8Rg5Tixv8+ap3Np6B6W1fSSFDhZfQ17Z580HVEXFTzAwl8BeJp5DeclLViRI3QYEGIoREUciZybpU/QaJcIPGe0Hm10FCiXBU5J+tb6BQoDynzsJOxfNhce4odg5pAdMZo5DUmIy7t77kaeSvMsXdRSOOHAQ1iP74V4zMjubAtTTrXoKJeERhSec5YW3JD0ovYXAREWixJEoC0EMzXBADfeuVWkcFHSGJ0y6+SlUVFH7hVOXbzOxFYops8JRfF4QWWRqLl0dVQtQRENrcpzEcAsFJJdvULyVMgHqiQKAyvzvf8Fo62ZEZBxlDxeItSrLEZ6YjeqXv7czVBS7nrz4HSmZEmyYNACu/XuigulQ92tSfx+2AGAioJ7o6CoMKCJKwyYdikSauIYDh/lJf+ZMgYu+UJjZvknsW6wSj0EjfLFVX6Hy+rqA+pKLthHj/GGwI6eG5V3C+s2p6NV/f60AsEjEKin3adQEf7j7NM93QZUfigDK2cUN3z94icpHVbj51V08efqsvXHSrOu7739EoL8nTCkzYfk8RI0dg9gxY2A3YQxO9W1evpSUQxk27i2XRyobk5jo88DwMQFcbam7lkLoJQz+oUJpm4ZdCBauiuVuoBYB6lDxdR4AJofYajWhUJPEl4HJEd6XiGRv3UGQgkeA2ril+SeEK2LlEaD2uznifmVVe+OiVRdthmuf3cGZDy8i71gZjhSegtm+cOycMg1f9erTLEBRSouiSrks7XErxoTpIZxpDB8bWH8th/hgzpJYSEoEt4KTbwkvzG0xoNLzKhgXCuIfQK6AqHQh2crF4xjGTAzkCJYdAKWoEAtdsymFiSPhZPATFQopb5yqAwIU41BmOrjx5XdtnuvU1hepe+STevXrf/Ds1R/IY2qF2cYNuNmM9BbRD/UiIFjheS65Qs1IeGCCKdyZGF2Tgy67lhQ4FtNXxF6n6rqZPPZHUQ9NHYXie/IBRR9AHlZn12P89czcCsxfGlNrEDQAKodavi4RuR8KstzKrhA2u4/hxnfVCj0o+VIo6NkUoMzUl+OjT794a/lOb+MicH10+2vYaKpLAUUxTbG0qilAPZc07ecTyc/vNKx3FaLw9A1Iym9B2/gQr9Xr3NNdRp/yZQp6BLxrLPSkoxU8B46YC1mIWjot4VD5Fcxa8+Hd5UjJXrAyXtoclHoXEEskX9MwJoOFdAg/JB25ChMmGjcwLtW5uxu0DbN5xYtCgCooQNWocTxDU9bZd5/9XNSzNyK7dIbB2AHYbbYNP/z4Q3tjQKkXAereDw+x29IM7t274GKXLoju1hUJQwbjwMLl2DFvIvJ69JALqEfTZ6E675jCgLJhYKJA/ayFUbD3OM7L29ZqpKFrb3cev6M1JauPWgQlST7iLoMtBlk1jU08OCPR2tYCQJWcu4EJU4N5GQ65Achlv9PhMP+b8/6TXGGj13r028fvc/Q4AiurEmhuyWQWhCcHmXszynGoN8Fj1XX1gsPHGNfaZaQPFwcj7DLZihMlx/HLL7+1NwaUfv3++x8oPf0BDHR1YaW+Ef4OlohOToeOqwfjDtOR3r92wJw23cPO3VG1cDGqmhG8jYz7gHdhIVBREa6JSS4KTl3DopUJPLuA1pT0Y9Oa2KuL90lmxftxzkRqDQHKyLzxegC5gKJK03nLYjigyAFGIo3SfVNzLvPos76xhL82dnIgrO2F0Iu1QxYvNKTXiWUmHmped4/qPS48eUwEFIk/i8lj4ZuYiq9+/hF37/2AV69ft/fat9n16pdf8Mnn93D5ky8Zx7qP/HPXoLvdCL7duuObgbUD5jx9hcThJo1mzfHJD29itXoKdzx37umGpbzqRcIbwa3dlMws+H084hGVfhUlbJ0pz5xE4rjJIbx4l8rhrB0UMrjqv7iWfbEYSiERR2CxshUy+CTHrvO6u+AE4ZTL4tJbGDtF8EERiheuiEfxB02HXGTpRXIWnygph2LcKaB3HzgFeeDh87+2ZafoRZohicAffmYi0NwYYV06yc2donkikfdkm2Gz5vjSre+Zgp3B14i4znudnWFpfVRYU8lVbDM9BK9gwZkdl5qPUeN9ubgj3Wr42ABeQLpnv0Iitv6LhsaHuQ5F4ZTpcyN5ocGcxVFITDwpoL0mv8nDIx8LVeK4FTB8TCCvslDdnIqyqz8262Gp2uXRjNm8ZEjM2Py0e3eYzpgGB29nVNy+x89O+Ttf1D341etfEScpxJZZE3Gjm3wjhVcWjxyDJ+bmzZpjInunAu7IpHWifH/K+/euscwv1JxiQRdZ7JQTRcyEHNfE1WYzMWlq10IOtd08h/seBjI2R507iPuMGOPHxZ14DyWxazGTshOTycQOyeFJ6Dc2b34bZTDW+3jDJl6gIOZEka5wuXdvOPfrja2aWjhZ9gFev/6tTers2vOi5yEgXbl2G+k5uTDV0ERyr97yk/DIGn6/Mx7NmY/Hrl7Nnue0Ix/ykBm5eajIhBjBzIXR8PIqld5DyZLLVidwCUXqC/mq6Od1TGrFxp5vGaBMHCW82pSUNOolRCyvO+NY1JFO9E9s2ZGFSTPDpZXBBCj6cqe9jdfiywUUux4bGOABA5Nskh3ljX/VsQu8Or6PbdraKD53mYmEyjbrMf62L3qMh0+eo7D0LOwMtbFjDlPC+/ZrMFeKdMtKUgtU17eoE17ph19gcU2QmKw63geBravO9myUld3l9/hHn8GUWQJXWrA8jmNg4FBvmFgeUfQcnvov0pEZa5no6tlfSFeh6l+y3jaop8KOsT1yI6hppTLW6cfjPiKgZjGTMzihZe2hH9nsRuXEybx3Ur1dyci/ew+obdZGTPIhfMcU17/D9fT5r0g7lo+VqxcghG2a76khSCMhGO4AptQX0534KqL5fcfp0tp2kEuSMTUhNHIVkILu4yOUuu0LKuNNTQaP9OPxXG6UTQmFt3fTpXANAoosPRO7o8yc9ORydu7iGA6ueUuisX59EszMMrB4eTx3hPH8qJrym2VMPFIlaksA9TAwEA+nzeQNIuSld/ybTXZ8966wmTGBfb81Kj7/Ca9//eMv5zknx+yrX37HD1WP4ZEQBO358xDTtTO+pcrgRrzjxK05oBjgnri6tmiOicwsj/K2AKMnBAmVxNOE6m5qt0QXJUVSxgHPbZscwtsvLVoRh4ILClvu8v9AJ0RNmBbMrQHiPuTInDwzFB6Bpdimn8VNSRHl9DMhfQ0Dm0NQ0/k5cnePhweqdJnYq+lKV29CmU5BHemudegEm96dsWPHDmSePI1PvrqHHx4+fac96H+ysT19+Qe+f/AUl65/hZTDx+G83w72Y8fiSJ+e+Kp77ybL7ilNmiqHn2zTa7LHQWNk75rPIyGkI4uVxJSCtHTVAUSnnYf6lgwuEknXIt2JRKLL/tLmfIf8P1B5lDlDKyGU9CRC8qSZYdAyzMKKNQf4IMTUFd7KeFIIdI1ad3rA4/BwVDILprGwQ9XAIfi870C49ukBE/XlcLHWh5uDLfLLL+HlL21zkGJrrifPX6P49CXEJibDf58L9hjpwmPyZPj17IrbDXDjhgBV2W8gnrfyZCuqxVuqEiuVLhxUbG2nMwVc0yCL61jkOR81IZinDc+nI1OaqAtQCFBEFPehBhm8gLMmMk3IHcw7edSOUC9mLDP64MVWPSz5+5/obKsJFtcPOcjSz5TB2eF9JHfoALMxg7B2+RLknrmE17+9O6D65bf/ICv/LNRWLML2icOQ8n5HJL/XAVf/1QH3CUgKVr5I8580tPG8ZaVNUqKQiobuQS5VqEeFbHCY1nbKrAi+tkILxQBEpze7BXXjN/gGnOHl5X2YqUl5T/XzZ7x5kJg4F98BTCT6R7X8EMUXbAdWjRrbrO4r5G6wGzkIBoZGuPP1t23SD0qRi/S53/5gOhLT7R5UvUDRh59h44YNCO3ehRd5PuzYlYNDkWeqBageTA1g8/EiWrEGt/IoJ68CnsGneZ64tUMuJtW0XBKNKiKSOqIKQzlT2rotqh6WwymAWibi2s0p3Fs+pA5nIiK2uHAltTC+wjMCJ88Ow8yFUS1uZk9f/FhLh+/I5kz+rR69oDN2BGLS0/HiLcf8SH97+fI1vrz7LT64+AkOF55klnA4LDaoIah3b3zTjHpDeboj75O1aEmzsjPrkrn1UYydEgRLxwKeMEnRENKVSPTJricBjOJ6U2eHYn9QTQtwpv+I+eUtAlRMykXs9yvjye30u4PzMUycKshU0qXEL6eEd8ohd9gnfPFGjVSe8kKDzCz4pMUP/4qB4sGwkc0C1ANmBaUxvcTKbDvu/vj2wjUEpltf/4CYxAy4WRrDYd1K+M+ciqCB/RHfrWurwMRdJtRvs2sPPNmq3+L5TC0vhypbG2rvM356KHJLP0VixiUeJKaIiCygqEkcBflXbzrAkyvpCgovg3fgcXgo5vuq/6Ll7gKG0HBoGTCWBwGZ6zTSeFRaNh+KvngZr0SVII6hfjJT2jswJZ78FwnpLT8lgK7q9eu5T6o51cQVvfvCYeZkFJy7/lbARIlyFz++CVv7XTCeOgaJTKdL+td7+JjpSNRfszXVwSKgOKeeMg0P7exaPJ/55dcxZ3EM14W799mLgADBp+TucULoWz7mTeZmRx5mi0ZcmlCTR+fsLWASaOnKeBgr1iW4/osGJkIsjzrwW+wWgsIHcq9gKgMKpT9Qr2shu88Hzj6lfHK37zzCz2UTA4qenqdaPAFEj1U3oLLPAMHiUzDf+mbvfnAf0Av+KWFvxY1w69vvsd1mB3aMGgzJ+514T8xWAaiuuGOKO3GnqhWqCpVLNUQJORcwb0kMlx6UULdqQxJPsqMKJzK6qKEGrSk11x0xNgDmNU3xiUMZWaTziuM5CyPZWitkENR/0WpPPvsCIQ14yYp4ePge56+TN5XMS3q9K0P60lXxMDFJQFBQBuNgqbzilOJ+ZHbqmxxuFaBekF9q7gKhaWlvxQojiZtl9ukJvY0bcOebqjZ1etKJDF5h7PnHDMeNXr2U0la6nhhnHPohcTk3t1bNZXh4KcZPEZgARTwoC1NcU1vHLAwZITCCgSO8oWMi5DxFMQmjpZ+FAcO8eFsBFbUURd0H9V/csycXcxdFcxbZucde3ghUdM3vtMnHZMappjDl28ZRiNtZMBQvVxGqT0mvIifnWs3UVh2qSNcTa0dUDh/dqF+qLn3FdvTO8YORlHUMz563Xc+oK1/eh+7KFcjv0aNVZeUNETWipajBEw0t7vRtDaAcHYt44xLh5E8vfpyskfkRrqqQSKMe5qMmBmKbaTa18ERSwQXMXRrDVRoCGnVvMazTGKVZgPKJkPD2L4KC5s2VcTonWDyOLCrpLHzCT/OJpd/3B57gPgwCk5ibrLophXdRa81E8FY/mzS5h7gpv5R0Ibr1RCbTY2zsbPDv735sM0AdKT4Lo2kjcYFSbpQMJiKeEr1gMR0V2qo5JDK3OorBw4V0FPKS9xnkCR3DLOnxHSTaAqI/4BkkBBr9HYeYlPGRHjBOIRg/P4VdQfVfTODng+SwL97Po9JUYj5wmDe2bs+S2xjd2bNYepKCaCmobk5Bxd3WAYromaSAnzbVHL9UEQOg4dqF+PjGF2gLoUei9GjpVejMnNYmgKIQE4n6Z86tE3V1AcXLz6eG8gJdTd0UuWEyUyaBZs6N4tERAhI1J5vILMMkxZ3W8v+wx0PoSsd7kk8TnGAkew1M67M96rFJ8rktAEX0ZKclHlDqRg/FatcoZ2jnrAkoLjmJ178pt+8m5YDf/PZb7GJc3GjsSNzs3oL+440Qj1lSVcvyVU0ey9FSQJFqsnZDCg/DyN7nmXKZH45N/iniZH0He3MjbPO2g81RX+T/ISDpAhauiuP9nkZPCOauAKocHj85FFEptYsQ7J3ftJWmEI2yAXU/I5cfAcabkikQ+yJA+Q/qh9jIUDx6+kJpYPrzzz/x2Wefwt51F7YsmYvUHt1a3fiiFtX4naiZ2FO7XUqZu4YAtUo1kelWb1w7pJ5oGuZwBzaJRgrBUB+EYWP94BOqcOpKw4Aict13XHp6FH0BxfBIUV+jnowiGa+tvVOOFFCkPykbUETVDk6oHDpcoZOfaJfHd+4Cd8dd+O7nSqUBqrLqKfwDfKE9dSxud+qMn5WtjDOR/oCyVpcsR3VW6wLtTQGK+p9aOL1JNbLfXYye/fdJ+1dQ+IXWmowr0rGUAig6NJFO3KQPJpFGije5BMiMNDY/Kg3P0EkKFGgUdK22AdRPCQmonDWHn5WnyIlUn3fshL1b1PHNN98oDVCPnz6H3W4nqI0eiH83w/JUlHhQnHG8qm0GSpu3hgC1jFnlaUcuc8e1b9Q5rs6Q8UVrTIAi3xRVPiXnNTvi0fgNPv4nuYecHJ1UsDB7YTTve0D5xg7uguiztM/H4BH+PA5EgCIiv5QyDqcWiUznR/r6eNCrn0JuBAKUw8Z1+OyW8hRz6vN05uxFbNPSwr5eXXCn30ClgYkqhu936IQni5e1Kt9JHu1yLuRuA1lALVgRBzW1KKzfnoQV6xP5GdEkgajFNK0f9eTctl2hOrzmAYpIQzcTfYd48sLPmfOjuJ5EJuXKdQewc6cEu9yKaos8xsUMzZR/5Dx5i6uWLudcqqmOwV/2GwBr1RW4/PF1pRY2/PLLL8i/fAdrVq1AVN+eDAitB9WjvgP5cSRUDfzQzknp8xYUfow7NnmrnhpAqawVGt/v3JXLGYZ4uBBVxJDzc+aCaHgFNSuxTnFAkc+JHF3kBSen5eQZ4RxUBB5nzxNw2X+cN7F6AyhfWNi1uBN/o/SEib6q+Qu4F7kxUH01fCSsVRbh7LnLSveYf1P5G/TN7bFvaF+FLc/GiBr+P2Qc6kVQUJvMGYVeyAUgC6g1G5Nx5Pg13t6HIhxiahL5nQYN84albYstTMVutLQt5KXJ5DkVM/3Ik2qwQwL/8CKOaPGkqkHD/aUNF+gI2Kyjnyj1WPfqQ7l4NGR4rTq+uvT94GEImT4VZWcvKD2ud+PLuzAzNUHBf/+r1YCio2FJ1FUbN7/OrjHy8EhFXslN/jMdezZ/eSxnBrzaZVwQ06vyYG1fyAsQqFqJAEXrR70OdE0lrVFXFLuRErM09A/ydnmCTyqUt9MjmUtxnqVrDkjPEaEBB0UKx7hHJV/E4uVx8A5tXbC4HqfaqssDp/zkczmgIg5lsWpBmwDqwrXbMN60stWA4ucMU6XL5Ol47uysPI4kKeOpRBY1fQpKSj7hXehIyR7I1JEZTG3ZvCWTH7dCYKKQDCVRUr+K5WtjOQBb8f2K30y1W8YWEq7giaAiTkXijs5ZI0BRYvtCBiBJTT6UX+Bp7suaMjMUCVnKU9LvOzqicsYc7lGW50EnQFmtXoLzl67yY8aUeV2+/S10Nqu1GlC8bU/fAajW3trqeJ1IdG03y2KWtjfWaQonLUQwKbFeK42DhgAlVruIKStUd0lJdStVExGb1WqDoAkQVdxFXtmntTjVDmaGUsCQBiJm+Yn9oghoajoZKDn3BlBCgNELmgbpSgMU+wePd5jh4YDB3OFZd7HudO2G3RtVcOv2rVaBh07vfFRVjVev3gSaf3r4GLZOnrAd0K3FgKIsTL4ZVDfgkkbzGl80RlZWuZg5L4JvYlXNN0d3mDARN4As8BpASQsUpguijro8y5bA0ZGzx062KEmy8RtSc68xNpgIA342nqAH+fmdx6o1iejWay/3PYmDE0UeyWZxt1gx5ZzMVcrFoVo+6iisNC7FrL5qYxOeb10XVJ917ARHA3V88VPL/VBUoXz99tfY4+6N8PykWg3280s+xOoJE1H6P++hsl/TztZaVFNSXjV6nNLCKyKZ2hzhVhvlMFGW5unLgi/QN6BMOMdlqG+tdF8KrUydFQlzB+H8aFo1x5AzWKediV1OLVqrxm/IO3OTh12II2lvzZSCysurGGs3pnD/BaVEkPgbVnNmXkikEMUuv34PRhZHagC1FyPGB/AmVsqcwKrMXDyeNU+o+WcmPHnJyZse37kT3Hfb4ocHLU8Hvvf9T9jn6gKdEQOht2g6MnNL8KomX506+3qFxGHT8CE41as3qhQ9lq2mv9NDJuqehDZ9EkJziJLmFiyLY9a4Ow/uLlE5gMJyobGJJP8qZi+M4lEPatNEsTpyWE+dFYFdrsU8IYDu8ww/hVmLovlpC+Z2SipSqEtbDbM5IEh3MjI7ItN95QSPWlPTVhJ1RAtWxCOnWGCVRRVfQEPvYI3l58crZKgRgzInkehRcLBQxk5Ny/oO5ODaO3oYDubk4MXrlhUs0Gmc4fGJsBg/Cqc6vA+/Hl2hqa6GD6/ckCr5X35fiZ0u7tAeMRinuymQXsN0PRJ1D9gYn2htU/o8RCac4/FW2tQCoBKQXyYcfnn+/Hf8hCna3EJraW+m14Zhp80bf6Gvbxk/nJwiIdPY33a5ttFpVG6+p3gCFtW5U07yFuMc3lKP/kYWha5BNudgxGZXqiXh5Edf879RXd9mfQFQQhc0b04pR5SnnIv0bKc1Hg4dwcFU/N/vYcuGtbh6/fMWl1RdufktTFeuQGnPXjwcco/R3n594e4VgKqnz/k9pOxf//oHGDi6YuOI3jjVxPG2VYOH8ayJqqUrcM8jTKnPX3j5BtaoJfOALqkgdQFFtM/nFJcmFFZZyja2l5/QOpqS6sLDz2HsBIFrUYCYsg6C2sqxScnpC5cJnTgIHNRIQXt7NjJLBPOSyqfWrEviIRnZWq66gCITlT6Dsj6VDSgkJODJDlP8xMSe7cj+2OPkgq9/eNQiMJFR6BIZD8cRffCodz8pIOI6dYTd5s28nFwWqNe/eYhVFnpwHt4fPzXgxuCBX4rVjRyNp8xCVfbzJx76mG9WaglOpW4EirqACgg6zYP9oycEwLamVoAuT89SLFoexx3X4gGMWygBz6ONDmCMiMiEyroEjn4ChBgo3sY4ldjHPDHxMtapJ0l9H0Rk6enuOCQF1OgJQiL8Cl4p07IuLY3R07AwpI4dCZVR/ZB77GSLUoDp3OLyz36A1o5NiBtcO5f9C6b8u4wZiwOHDtc6DoSKO4sqzmHjhvUI7N8HP5DlJwMqXmzQoRMeUJ6T1pYWdU5pjGj+qcmFCChy45ARRIAqPnVTel9STil7LQ7GdrnSk6YIWMtWxfNeYCQqKf+NChVsXdrwzGG66OSiATWN74mlEkCIU1HfRlGniooqgOTYmyOxSCm32VUkBZTgXffiO8DN86TSAXWlpASWWuow0tHE9z/fb3bI5RemNx2/fBubzHdj/6A+uMUUZ1lA/ThgMMJ7d2MLYop7P9fOs6K+CtnHz8BAZTUOduokFBfUvI/SknkpuYqq0gO/RHSE2Yx5EXxtqIGJLKDOXLwtvY+yP6IOHJd6wc3pwMyaNaEsTgqnUe0elU1FZLa45F2xG9PTr2IRU7ipkafovyAFkMQc5Y/nltT3rtJlaV9QC1CknFPIZoNmOkrkvKc15BGTCMs97sgrzGP6jWKZmi9e/4GP//0Apy99iuCkTJhpaGJ/7978PD555v65nr2hOX4MkssK6n3W81e/IamgHJsXzMOhjp0Ebzj1HafA7/xFeGBtrXQwEdk6FfMWhhRWER3NBCg6xLr86r1690tOXoKj23GpxKB0I1pPckqPmxqM/SHNSqhrGaCIqHhz8AhfbpaKJenUs5FAtkErHREJ9RsrkGNTFlBitxbyX8VlXVbqxG7fvh22dpb46X5VkykrZKl9drcSkWlHYWm2E6YbFkN/ymAE9uqGu40Ul1JAOpBxL01HLzx8+mu9z3364g8ERKfBaNJIrsw/+FdHPJo1B89jYtoETJmZV6Cz/SBvEiauiQCovVinVf9MYl5rZyXhITQysmRPxKB1sbRvtZ+weW+gg5F7D9hfqx0McR3BqoiGh0/tIHBwaBnPs6EMBNmmDCMZe91u/uZeKpdu7eSamGyHkZEuTp06hR9+uo9nz57h5cuXePHLH4wT/Yknz3/Dg8fP8M0PD5nB8BGMTXbAeMJoSDq8jxJmGV5iVtqjJpyU5JY4/q8O2LxyIU5+/Lnc1JhPv/weuuqrkfv//oWHvfrh6SZtbjQoC0SkM5WWCtELF28JVq6N54cBifM7subYjR07c2u9L1lyDltNspi+JDQ/EdeP7qeUlaVrmM51teEDx9sEUFTWrKqeJICKgYSi1ETENkkETpsdDN/AMly69D2/P+3QGcaKg/nfxAemB6Gq47UaqTzOlM2swe1s15jZtC7lJSQkBE5ODjDdYYiQ0CAcluSgqIjpdfnHcSj3OJLTshEWGgr3PXYwX7UcgX264UyvXviJeqQrWExKdIMBz3DSYIQmZsrtSfXw6W9MSbaD5D1m1c1dAIQpz0XgwQwkW+cjCIwSdBwtoxxMnhXGHZV1AbXL5Y2B5ONTwlNWyL0jtAwPfrMWbB3HTgqCg7tS9Lvmv4ncBPMWC0rgIJnYEP1MspsOHdpmdphbEuSBXaoqWIgk5sTj0ChlmFclB5Uip6SChwFmz49gpmpuqx7I39+fmcEe2OvqBF9fL/j5eMBFYyVs5kxBwqBBiOvXFxHdu+Ja5864R36jFvQfIOdkbMf34ey+Dz9X/VIPUF9/cxcmOupIWK+C6la0L5RH24yS0X+YF+c0/HfiOCN8eAPWNxLAj1N4ouBn8vQ8wYt1u/bey9dH1LVE6TJ2Ugi26mUrK8WoZW+k/CjKKujEBjhApiUMBR/JwTlkpA9MLQQv7HbTI9KqYvE+egjyfbh4n+Dl7HOXxfCdo6WToZQHKy9PxZkzJ3A6Q4JMBwsc/u9/SQ/lqdcYttmA6oHM//c/sLKxxzc/P64FJor/lZQcg77aSiZ6lWfR0RWbUcG7CJInm5qX0Osm1rmc28sCitSLSTNDMZFxLSraXaoSxXWqukfTUVxv6Ch/OO4tUaaB1LI3ks7j4FLCMwC7MiBQbhRxKUpjoVgRyeTZCyJhZHoIDo7HOHeSBRQ11Z86KxR6JjlYtMgDazakcCWRrBUjiwxpKyGlLMb583isrllT29eA47GZRCdkWTF97c73tWOFP/98H55eXtjt7KC08dMGc/c/wcFEmRvU52mTngAoza2ZfLNSk1Ux4Es6qsr6JLi5FUDLIAt9BntyH5WgnggdmynDgKxtPbY+5298p7SxthhQIlnY5GPG3CiuU/EcKQYmGjg1eSU/1bTZkTyRix5UzJ8SAUWNQ40sJNBgE0bxQrHZBrXjU9NOQ0TyOaU96CMqcpgzH/epi5wSqn35kWuaa/Dp59/WUsyvf1IBO1trpjb5KQ1MVk6FmDBDOGaM5mfKjFBpX4nlaw/w/H4RUCJRQt28RdG8pJxqAcQUI+JIJAkGj/LDFuMsFBYq19JuNaCIzK2P8C53BCqKBdGgeeLWGMEUFVvtyRIBirgRtQuiy8jyKLvPlwOR19QP8uSuCGVxKvYPnlnY4NGkqTxLUtFeCY1yqDULcO7Wp9Jg8e+//47CggLY2dli27bWB3/5vDC1gTrhkBVNUoDE1qxFUXyznfvkK0yfF8E3YN12lXQwNempwhnCwt+oAIFcPuQE1dyWgYCANsn7V84HlVy5Aif3EsatInk9PNeZJgTVA5KsDkX3bKtJZ7FkgJowNUT6HgIV5bBb7i7kE6uscT4PD8f9rj25s7E1gCI9bOeSuSg+95EUUI8fP4a7uyusLXfK7QHRXNLQCOFhEeJMZMURaOjUKDoShQyewlOf8fkaMMynwXkWOw2SDkUSRGt7FhKPXGsLICkXUCL5+p7CqvWJGDxcOMSRgEEVFyQK5QFKXVNo2OAdchoLlsZwsSfeT7ty5rxIBEYrN+5XvXcvHlClCVXptrD6lwBlP20SMo+c4P0TXrx4jqzsHBgYGMDNw63VgKLMWMpHotgaWWziJiMfkpjAGJ/+EbfYqMq3Loho/iizgN5PLpupc8Kxg23avBLlZ3q0KaCIDmR8yBPp5iykGj4qMPTh4KCdRGKQ/CR1AeWRmgrVTUno3s9D2nZRlPcU+c4t/VRp46NDH6vWrMWDvv2Fo2lb4DogQEX2HYCopBzuHT9y9DC2bt2CPXscENHK4C8XdUyNIA5NXIVAQ2ESOoRg1sJohMed5ff5BZyuBSgqDqH5pXkmpZtOW53MuNpqtSTefU7Bs1rePUARUfmUo38ZHFyLsVYthcnxEO5dF1NgyOqgOBJVy4jvcfE/yS0Zel1MpO8/VDivT2dHi6pYG6QqtuhVmzTwoE9/oVVQMwFF3fLCu3dDgK8v7t1/Doddu5iI2ozc3Ja3LhSJDJ3xU4WTy0XOThuSOI3NrnxpcNeOWc8EnF6Mq1M0guaVH/Yz3Jd3YrZyKsJOu0Lu1JQoUW14a4C6wczP8mtf13udJuBA+kU4ORczcZjEH7xnP6E72vS5EbhwTTBb6eRuDWbt8ZyrEW8UeaE0KxBefi1K+GqQfk5OxmNu+XVhHKd5OhVxqOiOHeFraYH7lU+Ql5+LdWtWICkpqVVjosDt0tXx/NRNWRFGnJo2X96pN/qPpV0Bn0MiEofkEqDzniOjz+HU2dv1dM+SCzdx4vL1vw6gKI3FelcBVNWSsd38kLQtsfj38vLrSMv7GJ4+ZVi1MZl36l+98QBvHireE5d2rKasx6NWqQ95eekQSN+olncXlkePg8J5qglPflNAp+I54Yyj0Zk01zZsgI29La5+dgevXr3G3n2u0FRfD1evlnvH1zHLljzfxHl4VGF6GHe/kDPTwbm2o3SXSzFTuAN5h1/jnUcRm3wchXVUA/Lx7XErhtbWTBgYS5BV1KYKuXIBReThIzTXGDralzd1Nd2Zx3OVy8trBx3piLSoqLOITazPdegkLFLOh4x6w6Uocaz/UC9o65HoUy77fubkhMqxE2uOBOneIKjEJvSUE169fQeOxydhp+1uZGZl895RN2/ehNF2A2zT0WLir/mlUREHyjF3SbTUn8ctNGbFkQowe2Ekcks+q3V//smP4Bv0AT+2V9YIIF1JUlYBC/t8qKgnc685iUt1nSS+qf9SgKKGn1r6mbz7Hfk8+g725I0a9EwlcNpbgvQjH6Hs6ueNfgYVlK5cF8N3qTixZPlRMeKM+ZFIlFxS6piJqv38UMXE34MuPfhBPXJDLsSZGJgerVbF9yEhgtPRygLurntQ9aiSd2c5cfwYtDXVERkZ2uwxmFgc5fqiqGSTCCO9c/zkYOgaNl0tdPRkBYIiimBoLuGOzQFDvNF7qCt6DrXhTU78/JSf3NfmgCKiidY1zeaOS1HGk4VC54eQVaKuSzVfxYg7cB7ll+sngBGZmUkwe0E015+keT7jgngPI2Nz5Xd2IXrqFcQ41QS57YJIZyJXw5MNGzmYxPfY77FmYzXA5asXuXh//vwlgoNDoamp2Sz/mZ9fGT+6VTYrox/bUOPYhqJeA/IsNNI9c8/chAeTAKQ7LVMVvOY01+QLpHknR/O02eGc+70FMLUNoIhIEd/OTN9xk0MZp3LjQBBJVLopL30RE4ubtDKZaKQQw1EeLPaPOAMP7zKsZgq8bJd/IqrYICdfcKzywjKy9MTZHY9nzRdOcRg0TKoz3Wf0ZLMWKjNrZ0OEh4fDxMQQufkSvPpVyBK9/fkN6G7VYtbVXoWaTuSe+BDzlwknHcg+K4l5io3a7SmCX+gHcGNz47C3mCnj+dDQyeQul5kLorh7heaURKPsPA8Z7Q8988O8+8pbAlPbAYpIUl4O211FvChhHDODKVWCHG1UbChaerzKgqy48UE81kd+FpW1yVi1NonpEzH1HHYU2KT3q6qnMtGofCcdUlPx0tcXD0eO5dXIVJTJz1pZtAzP5eQ1xcUlw8JiB44cPSQF1K+//oojRw5DW1sDyclNnyBl7kAtJT3rnbtCRKJqBZsLmhNSvqk15bgpQmM3mjeaP+JK5FageaGfKfOAYqjrtNIgKb76NsHUtoASKSTtEix250J9SyrvgkdVFYIvSiB+ZEQdEjrRBtcqm6bfSexRegzlBOm2kegj+fLMwQGV4ydyMD1eshyPg4Pl3hvEwGex0xSnTp+sVRRRWfkQpmaGcHNzbJRLuXrlM5EutG+WLRMXOTNtMjJQ5M2R7BwOY9xo2twIqLDNa0z6qntRm8zNOwEovkgAdyMkZV+Fy97jvPErtVcUDvsTcszJoy5L9Dop5iKJk0d/o1SXKey9xeeVmnrxZryMqu12odpoBx7Z2DR4n7u7M8zNzXHpyoVaaSyUyZlxMIX9bQdiUuTnk5NlZmBxmPeA5323poXVelbZn2XnhXdaHi7U39EGXclAZGByBJEpl1Fw6g53FSgz/vlOAqouuMqvfIUsZu46up2A7e5CbNqWgdUbUzBvaQxTxqM4TWJcacSYAE7T5oRjIlNQhb9F8mJFOvMtNqN1p4g2Ok7ShJvQgQJCA2BkpI/Cwtx6lTaffPIJbG2tmS4lP65H2ay79x3nGa3Ud0B8bvKSi889lm008fXZi6L4HG3YkgZzm3zY7jmG4LBylH74hVIbuv3lACVL5J+igtDi4htIO3IVCSkn4OVXmyxtCmv9HpNQhITMEzh49JpSG8O2hNLT06Gvr4/dux3wsLJ2pfJPP/0I971OjIs5NcgxJJIKHJCUIyrpuJznzqv1e1RSAZ8j6ghIpecVd5+0N3jePUD9HcjT0xPLly3F6dOlvJ+UeFVXP0UI42CennvfJQ7S1tTuA/jL06JFi2DOLD1bWxv88NMPUkBRk7LMrDTs93RHUJDyUoLfcWr3AfwtKLfoENatXYP8glzuNqDrl19e4+jRHPh47VVKwt1fhNp9AH8Losvc3BQOu+xw795dqT8qN/8IXN13w8rKqt3H+Jao3QfwtyEXl13Q26rFFPUUnl9OAePy8g9gb28BIyX20XzHqd0H8LeirVs1oKmpjtu3hGaxd764AwdmAcYnRrf72N4StfsA/laUXZgNbQ01+Pp6ovrFL3ha/QzJqUlMaTfmxaftPb63QO0+gL8dhYaGwtBwKy5dvohffv0NVz/6CNu26iA/v21dB9RAg4o2swsvc6I+FAUFbzUwTNT6D8mUXEFgRCmik4rrkX/QafgGnGo04k35UW4eJ+Dkepz3TahLVvYFCA7+AFlF8p2Y5BSl+2gMoVmXEJNcUn8c7O/BYScQmlC/dwI1l41NOYas/BtNUlK2kPFYePIaUvOvo/jMbZz48HP++9FTnyD/5E3+moGZBftOX9x/8DO++fZb7HZ0wF5PN8allJtGQtex09cREnEWu5yPQ9MgCyvWJmL+0ljeHEPPTILdTsVISr+IUxfaPFuz9YAqvngbC1dSSz1/3mWFjj2TJeF0I3csWR3PvcLyPmO/dyn6DfJC7/77pcejyRLV6lP7aqqSlff+hIyT6NTDFT377sO4aSH1xkA0YIgP72JsYn+0Xu/IgOAynthPFSNTZ4c3SJQRQT3b6T2b2cLRc1GtHI1rxbpETqqbUrFJNxPjV9rD2NgQ//7ma95WKDEpHnNWrMce12O4euuh0mJte4PKsFglgY+d5omaklDgmNJXOvd052McREl6U0KhppMOW8dCns35zgLqyInrbFJD8X5XN56PQw8hS5TjQ83VKXIek/NRg4CiSaDP4JH0Op9Br9Npk0tWxaGkpH6rPiqxooYdnbq7yv0MGgNlj06fE8lTlOu+P03yMc89er+bC89kkPd++lxKbaZALL2HCgRosejZ6n4n3U/B3i26uvj67tf8SLTiIgkGT1uJyTPSoK1bCjuXY0jIvMTbGTV3zsnrHpHwIbboZ/MDpkXw0Djou6n3E2VljBofzHPx6XVxjING+GKjdhr2+5UhI0O5RR9KARSRqcVRXmdHO1i2JJqyMyklY9qsCOxh7Lih9+eVfQ7Nbdm8DJ0i6bUKQicL1cSq6gfg4dvwZ3iwnbpkdQJP2q9bsUwJeavWxcPTv+ECB/f9J/jppdQHYNyU2kWp9Fx0pJum/kG2mG/yiyyt8zBrQTTvOCP7nfQzZUNo627DV19/KQVU79Hz0K3/Lmn+17LViTBhn+HJVAJFHZ8EJipPm7k4kn8Oze8YNvdja44vo/GsZ4Cx3lXERGAx1m1O4ad1cpCx76RyKzqcmp7V0OoI8vKUni/V+g+hSdZmk01VrbIVwlRwSAlgfmHliJDDWWSJ2imKKb/i+2miaMIMdxxCSFzjCi0lBgTHnuVdRyjZTAQ0dSzeoJGOhISmq2UcmDiaOiu8Vi8GSquho9v8Q87UC0TT4u72OM7vkR03L3saaiwFFHXRy85KQ+8x89F7iBPPVhVr6GiO5i6OhlfomabnmolJF+8SzFwYgY6MG1N+GAFJnCcV1SR4M501u+AaCi7c4ScrkJqxY+dRtiGEjjgkGul9VAhBbRENLQ+z51LeUb5KARRdm3TTGfp9a03s0JqzX0ihbuozSFmesyi81vuJbdPvkYmKWSpk1azdnMo7lIjZnfT+rQY5Cr0/OCafgbr2GKhggI5wO8kUd3nvCU86xrhzoDR9l3K8aIG7j9GElfVOfPvdPU4e+5yha7YLW41ymF7pyzcalYnR51OJFOWP+wY0DipS+ueviOW9xsUWiMRNqSkG9YlPyKiQW9BpZRWBvb5HmHgM4eVpYsIiicqeA/ZBz+KwMq3B1n8I7VRTuzxeT1Zvp9Z0ls050XD5Dl12zgX8LJjRdUQHyf3dzscUKqMmU3m9Rn1ACaVXbQOo/b5lGFdTVk/3z1kUw8fdY+wmRIUHo7r6OT6uuAI9PV0Ul+ZzEbPdUiLtTCOeQE7KdH8miqxs8+U2nKcDFXW3H+I63uCaXgfi+EZPDISlY0GTir5/8Gl+xBkVQ4jvp7mawEBpaH5IWYZC6wHlISnHBs00PtC6TTF472u2o7bqN9xyj8qilq8+wLMTxT5GIlGeNZUESU423Uy0IUCt11TMoUinbM2eHykXUNTpRBFA0eGGpLyPmLkcJ08U4fnzZ0hKPgBLS1PpgpGI0TI4yMc5UKaZLf1OPbMMd9ZPbfYJOsMUaqHZquz8kNhUWUfHaDQtMsuu/gg17XSuQ4lFtPQ/ib+lbI49PFrcm1zJgAoqleo/stW+IvH88AkBCAiXf6qnveMx3qaGdLC676XeBqQHhUZ/2GJAKSrySM+aPV8+h2oKUKSfSBd5lC3mLFuDGzdv4rMbN2FqZso7ssi+L45tIsoB70alZTXNwqjcntwfc5nY3L37Te+mdMbVVqgm8rzzuo3FqLhhu9lhha1FJ7diQe+a+KbfKemMlCXqxAyTdwJQuzxOcO4ysqbloWxfAtFSI7N/o1aK9EgIkVJyP+ImO9XsiW2OZYleI/1EQy+zzQEVcSCXbYywFgGKRJF0E0w0wXq1TTxj82B2JnbuNIWdnV2991rvyeYcZtSEN8UY1LpnDNPJHD2Ovblvdz7v8ST7HUTko6ONGhZ3TKHnI7JhQF26KkEKKOk8sfWztM1T+HPaFFBkhVG/Rhoc1dqRM5MS6MUCTeHUBU9+nBadLCm+j4oW1mxK5j4SUuBptxC46nEp9rAqG5IgKWy8sWhdQJH1RdbPSrVk7k13CMpgOz9JLpHYdvYo5JxWtvpEBFRD1c51RR49Q79x5tDYaoSPP7oCd2dH7HHeI1c/CY46h+nzIqWnlYtjpt8NjA/xe+ikqG2mh/iGHCjTHFfgTj5c52xOzydnn0KsWZ8s1d/E7yQOq7E1Uxl5W60DE4VD5i6N4foTiTsy29dvTsJoNkhipaJfimrFCHSGpoek77VzL+FijkSaqJySDjZ/eVw9QE2dFQYPv8Zb+NUFlEhULKnKxrVSNZb9nyyftmTyrsYkhmrpgDWAKr3YOKBEVwVxYzosWlvbAF6ebszCMkNMjPwSLN+Qcvad8XIBtWZDMre8iOjoEypRr8v16T46l6U5zeo92CZevzmt1sEF3MXDVAvy4xWV32hfQIXFnJW6B4h1Wu4qgHdALmYtiOSec7EnNoGN+hjNYAuWe/FTfjjNAraAYtsaChuMmhCILUZZMLE+yp2c5CwVAUVWkc72xkVXQ4CiyaPXiBPS/w0ROSOHjvKXCyhFRB5x5/nL4jB6hjOmTZmCRYsXITDUr0HrydGxDKvXJdcCFM3T4Bo/WMm5G/z0gxW8BVLtltBiwzbVjcnNAhT1LNUyzOJrVhdQtB5FJ+Q/51sDFFkrZPKS7Kdu/PuDT3Gzl9oi9uj3pmM/EXEiAof9nmNw8j3JuFggb91DXIx6QFLMLTzxNA4ereDNtkQLiCw/+nnJmnjpUabNAdTsRdG8enkD+9vSdQfkkqbOQfb3NMxkCnFLAUU1cnREa98R69GhU0emO+1stDiBFG8SM7S4E2SsYzpXkDh1OpsHbgGvOVBPFRDPd24uoOhYOfE7ZQFFasrCFfHtC6jojMv8WAhaQOJOS1cdgElNh39q4TN2YiBv/lBr4Gz30e/kqxGVeHLy8Y7A9kImwLHTt3jvKNo1svoCia5oScOhAnlKOZHtLsW63abml2PT1oxa/RSa5zYIxZhxmujc5X0sXqHSpF+HAKW19SAHhzxApRz9BPn517FcNYFbg7KAor5R9J0qaknNB9S2jHqAojEsZsp6cflbPutFlgxMJdKTtgkcazemSn0ZZM3pGGZzQMkquURCcwdvzrZJF6DTrFQYl6DubfTeExWf87Y9fWUOuOFxKgYoJ6eGLZHWAkpy6RJ7f3qzATWlpvp5/CwH9OvfF+917Qt9k6Z9X1ZWmVIFWR6gMvOFukM1rTTG7WvrUDQuIXYXhZJyxblKbNZ5tmnSuCUuzq0oZlczXe38jXbSoYgVk2wnLkIPRqKLmqvK+kOiD1zATAYM8paPljGNRRojo8wmptW24FauS+RiT/S7EBcjc9rYTNLgzm8toChBjRx/zQXUgmWxPPwxYpERBo2Zih5Dt9UyPhoiv9jz/AxCWUARkGiTkoO0qOwT/qxqW9K4+jC8TuBcaHUUioxc+Vkc8oj6ba5VO1DLyiOVgkTqRu1M3h68XQBltUc464W4Dx/cNHIJHK212Dx46kxOSy+pW0GWKDBKHVjcfI7WC7xq1TlygoBBbFnXuGGPe3sBaiJbEN6iaIwnRk3ch35DPPn5Nk19n2/IGa5jyrPylqoekAZtzW3y+Hl4YptEWUANHO7NQyqKrpuaXhqzomOl6oa4sWlDmFkebS2YWggoBpplq+O5Z5cGQocwLlsdi4iE+uKIuv0vWikckDyq1kMEc2V+kUq83O8wsc3j94snWFEQlLeh1slo8HDlVos8pl+oaaa1SIcSlXKy9GicTQKKzaGZdW49xyY9LwHHyOTNpolNL2FzEVDPsSlYwF4wt85XOA63P+AUH2M9xyZTQezdGk4PalNA0cSvU0/hu4YGQ2fl0UKLOlBdct5bzCdJNteJApxDRvnB1F6+TuTgWijD1gVAUcxpnVoKVKzk9wFvLaCoFeMqJmpl01cIUNz6Od24H4oWm6xUsZtMU4BKSLnEPj+Mi3yRC5OYIy48amIQ7GQWVyI5B9XNKTz0Ins0GRHpmes2pSp0Lk5RUQW38Ag8sp9D3GoM45S7ldMCqPlv2mqSiXlLYznKSeRRLMpyV8O7xCv4JKbNDpOeIknUve8+zGOs19ROvvhyYA83syZQS4skHhQ4n3GLhAZSifPKrmLd5lYq5Vr1Rd6ilQkov3xH7ntCIk+y538TFiGuSk3VDE0adhd4+JzG6g3JPMYpG5uj5mKUXTF1TjC8AmvH5ix3H+JZoH3rBIfJwJk0PRR73I41yqUoP2qvZynngINkXBATubXojVkLI6UW+lsHlINLAUZPCpICivpnJ0saVuaoX5GmXib6D/XmnErovuYJG/v8BtNSKCtx/uLY2j022WLRe6mVjVxAlHyCdXI4lCL6DBFxKErwH1yHQ9GkZxXLt37oVChquUMGhAgoMiDWM12s6OQNvsj55fdw+vJd3nbbK/gMVqom8iyKus7KLkwF6D3IEys3JtbTE+kkzwWr4rjzlTi71ME5WUiuW7gsDjn58jdabm4FDCwkfL3qe8h90XeoV03O/1tOX6Frkb4HNLYclCZ40YAoSd8vlHxIDQ8oJiWfWW7xPLebcrfVtzV84gBdPgEfYJmqsLgioIQdGcD1DlOrvFpVMB5h+XBiO3De4hiu00n9Ney95AF2cT/Bgd3Qd5okJMBidx7mLKnt2OTimZnYqpqpCE46J11omnx3n1NYsSaR53XXfQ/5dEjBNzbPhalFLtdzVBn3HFVzvq8ocvhRcEzMUQCc3CdrNVIYAOVXxmTlXeN9sqgpq+yBi+Kh1YtWxiMq/TzSC64hNec6knI/xQG20XVNDnEDSDboTfNC+i995zLVBBzIbIcDGAPDyrGCWR+Umcl1onGC55sCvzPnRTDR0vDJUXQZWh5iom4v3/W5jZwgSSnDVFBAFiCBh1oo0ncREcehXUrAXLAqlvqBIaO0FKvYwvYeuJ8vFgVMxftpfEIvTy9obcmQm+YRlX6V62bk3iDuRmJEfD8RjYHEzYRpQTCyTufP4uRVjBHj/fnrtFiy99MYiWO96YD8higcRRyMNiSFl+i+nv33YxSbk60mh1FwquFSJ/69+09h4gzB3ULfRcAifx65GsRTq5apCJ5/2pATpofyZ6L7ecrwpBA+P5Q7TyJ3qUoCYhKV2m5a8Zt1jA7xgRFR9QQRWXo0sOFj/bF9p6TRaHUGU+bpUECqFWvoHkrj3aSdwUFDOhf5XsTvIqLfB7P/SQebNjecGwLZxZ/yRacOwTTBxAWk42O/U1iIjABSeg/k1gdyUuaH/P008bLfVZfouWctjBKsQabc8jEyoNa9j3xygxv5nOE1h1MSl6Lz7qiAYrvZIf7sTa0BZWhYMJ1wKnt2cUz8fMGBbwBM3I42FpH4Gt1HG4bWikBMBzNSl+XGCjfaHFDeIadgaHwIOyzS+Tl2IhmZ0+8S+EScblQxZNY+wmMvQlLWcFI8iRRnDwm26mXBxC6/1vfIEqXM2LoWcwAXnrkOfaNsmFjnMOvoWK37+O+Ows97PEpQJichnxrG6xsegq5RFiwcsmBqKeH/E5lbH8JO22z+sz7bUHRgT0bpp/AMOwMdvQz+nQ2NsSna5VYMJ78T8PAvaVZDMrrXza+EfwaFbuYvj+Gik7iTPBIzPkiHmsM2tCqz0Hfa5MHVq35J2VsF1D/07hGFuI6f/QzZhZ8gNfc60plifuzkdSnRa7JUev4OSi8q76g4OdT+k/IP/a2o3QfwD/29qN0H8A/9vajdB/AP/b2o3QfwD/29qN0H8A/9vajdB/AP/Y3o/wNqXDkFBvHIfgAAAABJRU5ErkJggg==</t>
+        </is>
+      </c>
       <c r="N34" t="inlineStr">
         <is>
           <t>Healthcare &amp; Medicine</t>
@@ -3530,7 +3630,11 @@
           <t>AHRN</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAGEAAABfCAYAAAD4dql+AAAACXBIWXMAAA7EAAAOxAGVKw4bAAAcvElEQVR4nO3dDayd9V0H8JpInEGXTEPMEjGyEQ1OMSxshIUgwb3ANpUlKCHZ3CRI2GQohDERRHQ4xyRkIOJGkDAhiNMh4rYwsiFDNkphpZS3AgVqoQxo6WpXCr19+Xs+//Z7/ffpOfece+85t9Xsl/xzznme5zwvv+/v/f/yLFq0aFH5Ydvrba/fwA9b2UfptVXPl5f/8Wvlxb+9qX4Pbdu4qTz1u+eXB970zrLmr67Z7T87tm6rx3/v0i+Wl//p62XTAysW+rZHpn0OhO2vvFq2bfhB2fHalult//3Ne8v9rz+y3LXogPL0aX8+vf0Hi5eXby86sNz3k0eUqefX7naeHdu3l+cu+ru6/+G3n1we/IXfKE+ceHbZuvb70/unXny57NixY2EebAbaJ0DYsWWqbPj6d6o0P3bsqWXZm99XGbfxW9+dPmb1Jy4r9yz6xXLf695WNj/6dN3m+Pv2f3t54Gd/vWxZ8+Ie5117/Vfq/h98e1l5pacJAInGAPqhw36nPP6Bj1eNeXXFMwvyrP1onwABAx/61ROrpGPIhq/9Z1ny44eVR4/+vbJ9l0a8cMWNZdmb3lvbMx+9uG4j2SveeVoFYfOjT+1x3v86+6+rBjFbU99bV0FY/cefm97/xAf+qNz7Y4fW6wCeaXPsQtOCg7B982tl88Mrd9vGNJDUJfsdVk0Ievx9Z1RJZZ7Qi1/4l/L4b55Zmfjdnz6qagnmrbvhK2XpzxxT1t9yxx7XWnnSJ8riH/2lKv00y/lee+rZuo8mAPrpUy6sv5/9k8vLAz/3nmkzxZdMrXlpkqyYpgUHAbPu+6m314dsiUl65B0fKst/+QPVB2As6Z/+383frPtJvH1s/JO/fU4FFCjr//n23c4HPIzXmLh7f+RXyivLn5jez1TRjOcvubZsee7Fsubiq8v3//1bdR+AaBeHb/+ObdsmyJG9AIIoZ/GiQ8p3Fr15j4jmuT+7qtp9pglQmB6Hi4EYitb8xRfKnYtePx0tAWHVH/zltOlCJN52QGIyX5LrccbVFL3u0HqNe3/isKoJIdeyb8XxHy0r3n16efSYU8rWlzdMjCcTBWHH1NbqcFvmbPyP+8ryQ06oUkwSW42gAQBiYjYvW1GZw4TwEZjEfPjEYA7VJ0mlGRiV8JVJwTxAs/O0gubQCMQHAcg+98jPRAsQP+Nazi/UdQ/8z6RoYiB4gBXHnV4Z7kFDrzz4eJV0Ev7Yu3+/AsHehzCU7d/60voa33Ocjl/1h5dUAByLyTERJJTt9pltJH3Tkoer1gF5e+/6zM13D/y1ynjnB1BMGMGInyI09nHqCV9pKNACcjeEni9NDAQhpYfGRA8WwlxMXf3Jz1XHyvZyyJjrOM6R/cZ0tLlnGsYVsWxZ/ULVKqbLPTBv1SH37oFpQ8wTUyiaCslNhLqJwL73uRuqtjBz46CxgkBC2WsMxTgMXHbI+8qyn39PZUA9pqfenC8NwRDxOSaIYkQqa//+X8vmh54cyvhtPanfvHlzbVu27JTK/N66deuM/0WSNkECbcVQmkP6aUGrmfEt7jkazZ8Ip1ufNR8aGwhTL6yrjsxDrP3irdPbxfRumAkQASEagOEYQcV9b7WlS8BFK1euLLfeemu55pprymWXXVbOO++8cuaZZ5arr766Mv7Tn/50+djHPlYuuuii8tnPfrZcf/315bbbbitr1qwZev+uj9ECA+AwN5JC9+qZ4jMIGRNKO5jLV5Y+VjbevXQ+rBsfCCSdCYnUUF3M5dTccM1Wew8gTyBBJD8moB9t2rSp3H333ZWJaNWqVZXhH/zgB8uHP/zh+qmdeOKJlflTU1PlrLPOKscdd1w5/vjjy7ve9a5y9NFHlyOPPLIet3r16nqeO++8szzzzDN9yxW0TzTlnpkqGup51l73b3X/un/YGdbShAQb/JHjBAjb5+gnxu4TSEctL/RsqJsFDodZQ8KerQeQRIz0tA4bvfZaD6BHHik33HBDOffcc6tEP//88+Wll14q559/fjn11FPLaaedVtspp5xSwTjppJPKJZdcUkE455xzyvvf//5ywgkn1E8NIEcddVT5yEc+UtavX1+WLVtWt59xxhkVYNu6JJpiKmlEQlNmk69gRml9iIbwaaIvZnQuNBHHTCO6UQ8tEPb1k342ndRfeeWVlfkkmqkhsWz8Zz7zmcp4pmYuINAKGuG8TNsdd9xR3vrWt5ZDDjmkatJ1111XNW8mSu2K+Qltuv+RWjyk8S0ws6U5g8CWt7a/pWSrtEGmS0JITFuQQ+z48uXLK/NJOsZrmLlkyZJ6DPuP6SR3PiAce+yx5Ygjjqi+JOc99NBDy1ve8pYKhuNuvPHGsnHjxr7PxLcJMEKYzgzxGa1Gz6UqOycQOFhRhSy0re+3RH0VzyRfqQe1xMx86UtfqiYn7cILL6yMtB194xvfqMznC8YBwjHHHFMOP/zw6twRzQACrfB50EEHlZNPPrncc889e9yv/MbzCG8lk/yGyK/mDD1+CFsf/62P19zHMa8+vmpUds4NBKVhdl1oV4tpvWSnS2wp+8n8CEtDQktSfumll5ZPfepT1an6BAItuPzyy6vJ4BswSRsXCBqzBAznX7duXXXkAKAVGiBohuiKKWxp0+LlVcMxX8YPAD7PNuZX5s0Uy97lO/o7JgZCS2wls9O19Zxxt8bP7t58883Vxqe1IGjCSc7SNswfNwgiJtpA4gUCtC0AaAA4+OCDyxvf+MZ6DL/UpURBhEUpRAhL2xNKIxGh7L9fP0eXZgVCajUiIHG13zJgqlizXEW0XaXnLolw2FyMZ5dJWgsCLeCckegI4zF1EiCIljD84ot39ku4PsYHhABxwAEH1OPvuuuuvs+k1EEAUw4P8ResQGpVYwNBGi/Vp3YYztb7LmJI6aEmZT272CUxugiECQJAFwS+gKOMqcLMtEmBwEnTCMBzxswSxrcgRCN80pguiY6YY0K5G696uYOyDJMszJ0pEZ0VCGyfRAbqGO9TrC/qUSRjjlKyaIk6y2jZ+iuuuKIvCMwQoDZs2FB/C1O1SYLAN3DIjmGWvvrVr04D0ILAR9AInxx6G/1I7uQHioL96NkL/qaWxPXazVSGmZNPwGgSAO2ZiOO79tprd9MAze+AQAswAN10002VkUzTQoBAGzDc/5HzH3jggZX5PmkBAN7whjfU3/7Dobek/M4kqTtlEEGIpoiSBDBtf8VYQEAiJGZIvcgNCNu6JLoQiqr5CPtkqPyCvAAIpJ6GMAcrVqyYzhHOPvvsyvgw//TTT59mvqw5APQrW2B4GB/mt0yPGUrjB2zDXFoLOOd1L+5TuOzes79fhs0isP+bm567EOsh0xbODwpbh4JAjQY524ShooC2ox3z3fjSpUunox2Rkcw46uy7fanpOJZGKLrxD5///OenzRZJxeh+GgIYzAICs+Z3qz1a/uMT6I6ndYSCDyIACUdTiaXF7u/JJ5+s93bLLbfUe1H+EDV1i4JtZISUPRK6qpXpFNLnPWsQAKDmU0/S+xR2iYRcQJKmUbW2Vwpxdph41VVXVT/gO8dMqjyMh3eMh0dA0rpxuYxa47B9YkyaaCuNLwGu7b47Fijatk7/sGu4loIgAJQwAAJwzOYfolG0h2lijvbff//6qe23337VDHazY1Kv84i/FLYy2bUTatvOgWi2sSCzAkEmyOkkEZG2yxpFR6Ih3Y/tYCxEZfkBLRINDBLoQSPVpNZD0wjHJHFLI3X5v+Y7ADW5xpe//OXaMFAISRKB61ptFk57mC5mS2OqREJJ3GKS2HwS7jz+wxfY1rb4CA0QNKolJRpBixqZModRGyhlHGa7Hw01R0rP7L4M0ckwnfQnSWsHTTE5GNMFQXPDiY44ZPtIKiAuuOCCyjCf/UwOh8kvdP0BpnHC8QmOJcHsOka3fkGW3DrlACBCStmCkxaK0hTbRERaPxBohm2to1YZUEnoRku1O3ZXX4pRHt2BZiM5ZgkZJKXjaibpj4V8S9Qb85memUDAND6DOtve1o5SyFuo6ChApGThnIhmJjTtB0K0gXa1pFj5Sh8HXcdWLX2s+s92ANpAEDCHP2htnm48yZqaiNDLaIiW2GORD8c6DATf2WYVVMxP2WI+IPAD8wUhRTzaScJpxiBzFD+hMZF7MH1XvUzYqlNIYY+p0pj1dghNXxBIPpPTVZuptetrcsIXpCM+xC4DYBgIbH3yAsfOBQQAaAHE+SO9QCGdzFHbyzYKCBpH7JqIuWt9QxeEOGnnExCEam7QM+EcNOeM8TRArrD5wSeqA2/7pvuCoCrKGTM9vH3r0e3TkdH2IolQRD5qPjOBwDkDQe4gNCXB6jejgoDhvjue/0iIyl/4D5/hu+1yDftaAEYBgfT77Zn4t5k0IdqAeYKFUPWjPSHGfGUc3aIzUV8Q2Kxq/3vmR1glGuITlCeAotM+xGSx75g/zBwxRY4RNnKA3VL2IBAS6wPNJ2aS2DCgbSQTkzCURiR3AAbmjwIChrtnJrM1SYNAcE1a15pvo0Z0+LTCi3ddoR4IQhK0OojqgRXV9AAEGHU0Re8CoZSnhYrDQKAFqZQKJROODgNBNGUbhnng2cx8wTCRlPPyFZg/Cgj+w5kygTFJg0AIEOkNrNrQ4x+7r9JMoFkWRU+hPQ3JyMC+IPijZEwK3i8LZNtaXyGjBMAoIGjMkGwT87v9CS0IyXD5EXa+n9TPpmGuc3LmmD8TCLSMk3avco/UjmYCwTWYwZb0OwAA0/kD/NPFK6rkWzMEdA8QqIvKn3jX2BvdevoJ/AFATtION2RW+INhIGCmbf5z++23DwXBJ9Awaj7MbxtmYRQgMH8QCBqGeyZA2I/xw0AAHF8SMm4JL/sN22eSVCJYnT1AUJ549k+vnJ4zwLszQVTJn1pSeBOejQICp5y+XccMA8Hx4wSgBYKJE/lg7iAQSD5Hz385FsOHmSOfbb+DvKCOxd2VqLWU4f86gPqCICtmy+IHDBEUDYlv2/yAKQLAqCDIC2SjJLxf9yYQUr0UWo4bgBYIpomzTsbcBSE9bYRRBDcMhGiD5wjpg2F2dOrEacsbmCWVVSPHjdTYA4TMH+g6YZ3aUG3H3XBEmD8KCCIjACjaiXK63ZspW9iOQbN1wLNtkjI+ZyYQNIJD2wEwCgiAlb2HdAdzxkLVlSd/svKwTnbsgZCBAHuAEFUREaVbTuXUn/UfZEi4wlv8wTAQSHbGi4qOUqDr19EPLAyaJABpzIwwttvRHxCYJM8hkEgP20wgJDxu+xz4zzpEhlXpJbkqDnj76mP/27fQF4QuOQkU265L/kDmOyoIEh/A+Q/m9wPBNjH9QgCgYTJHPUgTSD5tQbaNAoLzKntMgzDDYDACzWQNBYFN5MFFSCqAIWinnDwMBP5ARCT5sR+zuyDwB4718AsFgqb8wYT0AwGzaQtyzKgg4EWILxVpsiq19fyBT2OYlC+UvPuCgPGb7n9056iy3gn4CCMp2LeQ0A3zRwVBVg0Ev/uB4JNPiG31QDJj5iI3KFqSaNlOSjEtI69Jc7LhbIu0O14UlPM6Rmkbsx0nDxmkCYqAElKREqaPAoLnCrH7ujY5aNGlvEFXqG18rhrTbiCIiHQ8SLeFpnHQ0HJwO8BL582omsDOc3B6rdLp3x1tAShdh7kZDAhFO8TgnB4VZ7b0ivEztJIJsI/J01wrWifMZD4xHKMIA0HjcP1mkjIKr+sTAKbW5R5HBUH9aloTHl5ZyzyZjmvoUHre1OaAtBsI1MOsSBmeeVqSMyfY1Gc4H6b28wdhPkfclisc7+ExPb1rbVTkOPWX3Ezq+giT2m3O5YFpBgIOhqW71HGOQQp5KZUIJPyPdAPGp/PKG9ohLulDSA3KQAWCk1ygZXq/KC4mrFqVnsAkuZXoLjv4+Nrzpj6XIGe3/5uDRdppAm+uvkEjJG0KUO1oAX20TIzmITXlbM1EDA+sSfs10qTcq84kaWu7KQHpe0yIZntCPQDbBiS0ePHiaVMT04gZYTzGARkBuU2g2Hamiabket2BZu0oD7WjjBZRT+JDaGw7UQXTmTRNfYpwtSQXkACLjvQrpNNHoqavoa9PUIoVpoqI6qTqXhPXth36zECr+t2WUQtp1cE388y6DSMxz41Qc78xX3iICSQPA6uK944Hmv0Bwf6AgDEmgwCdOSEUmX9AWJzHOexzPVLOXGXAQbd5Vs+k4yrb2kEH3QEIbYiqb4ZQ86n4yM9ivEhTsMNXDI2O2LCMnWlBwBgP10/qhaGkXcMsjSZo+hwwr9v34JNzdSOcMaYABdOodBwvylSqMD0gYHxLtMD5JJWupbeMMNA8zAoINKAr1e6BVPtk5jwfB5+BAm3/dXd4JU0JGZEiuOGUtSzvoAGAeRopT6gPvuThMtVMGeUIB+UIXZ+gceSY1foE5YDWJ3gYN8JJB+iYJCbCfnT//fdX8wOkribQzAxXZBrZdce7Hh+A7HPemCPn7ucTBAc+UxkY1SfkOiG1I2VrFqZtShgszsggdIl0zCZPIIUkmJPuFx0Bwc17KMz34OxxZtbQsJgj9rmNoIDgdzSDRKprIZJMa1wvviZEaodFRzTQs3oWjB8lOuI3ZkNzBoFjnkuI2g8Ejsx3zGCmECa6KecJZbQek8JkZEaP87aDdYEebWLWSL1PgGBg+oMzb40ZmilE5ZdmE6J2+xUmBkKmO40KAsnGLBLfDghuM2b7MiDYg3iojAtVPmC27McQEQ6Jsy9doJnzRqOYlHYenP8mYWPr3Rsmst+OH1Q7Yv85WvczKggRgImD4MbaEHOYOeLYRCT29cuYk7BNsoTdbRgHPL5hUMZM4xDgRi1bpN9k4iBgKDs9agEPYDQh06VmqqJ6uIUAgY+Rebdz1rq1o5iWUQt4WszmxEFglzm8UUHwe1gpm8kAgjBx0gBgIDOVutMgc+T+aX1AGdaf4L+DpuGOHQQkTB21U4epER2JkgZ16vALgHAs6ZwUAKSVBjA1wzp1+DKmNGWMYSDIpGc7l3leIFC7UXxCG6bKKod1b/puO5s8CRA44vQjDOpjTvemvIPQjNq9mdGACwZCQsNRQcjwR/tn6ugXCWVCoQceJwCiHefPqOyZOvpTMBShjdLR77fEcEFBQGz8KOOOgGCb+tEoQ14SijJbqSnN1wTxNc47bPBXnDAtn82QF30UWXtpQUFwk7Md/PXCCy8MBaFdaISzjjTOBYAM/OIHADAMhEylVWqZzeCvTEBccBDSbwyAUYZBZmK22tKowyDZb3Wm1H9G6QLFGIyW0DmXOD9FtlGGQcbBuvYowyBtk8DuFRCQksSoA4LtS6gaBzwKCOpIPhNB2YfBkruUHzA5TldnTqqjsx2VLdvOii+jDAjGPFo2VxoLCBkUPGxovKGQTJC6k1IyUAAwm/kJWXjKd812g4tT3yHBmUbVnUo7Kgi2eyb3n0rqTCD4bEdY7BUQkJsYdZJICm9Zamc+M3UU5QAreXQ8xs91pk6mTLHtIj//HwYCxhGM7uDpvQKCMoYuSwAMmy6l0QQ2dFRztBBz1mhBBvXyXe18tUHTpWxL3/ZeBwEpP2fm5rCJg1lgkDZg/r4AAqa7NnJuDB40cTBa0I49nSuNFYQMlcf8mUBIn4KaTIaT7G0QaIDfOpQEDVnjYhAI8g55Qb9lFvYqCMhNiSwAMAiErPqVWY+SotT9+zE/a1uwve1Ihzhg4Ws7j7nrkLvzlwf5AsKBnHcmENKv0G+ZtrnQ2EFAzFL6mLO0QpjvMz1fgGF/1ZPSQZTBAx7QedjbtKyR0W3tuhSSQUGCpuNfAS4z/0Vv6U6lVZw6bQEUjYpf6xbruo0v6M7mnw9NBATk4WkC5krmMDaLeQgndTF2U3y/M2yEmVLwaxtgjLrT2hEeGJ7SuqZ+41qafYCR/bpuhti05JrZ5nhg0QpaSfsARXNSx6KV7fD3+dLEQFAjiuRKzjDJJwYDwgAuDOQ70kFPYtuQtWuW+IF2WEpyAcdiCuluQ1TffWb4iua/WuZCOz9QkU/AKasgQpEFSXLfWXZhnDQxEEIcnUSOVmSRkax1lCEvHKsHI60cc3f5tTjlUR1z65SzmEjXIccZ20ZTCELWs0hfgn0AzNzp+SRkM9HEQUg2HV8waA08SR4Snys5TDo6ChAqujQUs7tr4AGEM+YDHNsdXDYumjgIiErzC+0SbN1xR+pBiTYAspCrQRKOfqtBpkvTNWbbbzwbWhAQEB9ByjPcZVBHv4fN+tiTWheVVDuH6/RbFzVFPFpAK8ftA7q0YCCEsjY2KeyCkL6DhJoZfzTuFYLtFylptnVHWwhRffJjC0ELDgISEorbs7hIWzvCyDw8RxjHPA4QMosnowFFWhjf1o6yAtiknHA/2isgIObJg7LH/AEAUrbAzKyawlykZD0fEDBfy1wFWobpWX6N+QFSFhZZSNprIIR0nMgXsihtShdsceJ3+cN835+AwSmh80vtsmtMFNOYQcQLTXsdhBDnR0qznE5MUFZOYb7ahaZGBSFakBBYmT0aYD9AJhn5jEL7DAghMTvGYxbz1AKBkZjfLkg4EwhJ1DKjh6+hGUCmXbMdKTcp2udAaIkDlyDxD0oJ/EiAaKuonLoSQ7saZExR5hTTNCGyrtV9jfZpEFpK96E+i6wmrOKp9gQkmmAgGqkn5Rje2vh94eXXg+j/DAj/n2kiIJhqa9nO6VexT22ti1fVJXsefaquiOW3FWOsHGC7ZqajOb8mYPttv6V9nMt3+03Ey+/uAuA7VyLYuc85sixmtpv46Lxtp7wJ9PZpJna37wiiPXWd03qfj0wvp+a3acVzfa9alyYCQn2d136H1bWTMMIkOcuP5XVY1srIcpVmMNY3Ub3ubTsnsPcYbV2lOrPxTe+t//FuNstDe5WvqafO7XeWeTDfur67x7t43vGhOlm7XtsrZZ57sU6Idw5TWf3PascRECuaeT9o9nsHs9XPkPO5T+czrxsA7tGL+tzzuF4PPBEQ8qJqc3fzYmtSY7meTMPNO8rM5cUQD+elD1Y9yTp7mGz5AevxYbSV153Hfkypbznv7bMCQVZetHhHfQF2T1oJAFCyqn1eTeycmEvSnQOozo+pPu13f8gkeufLenUA3Pk6+qfHxa7JgEBivD3DHF2z2GM2MM6UURSg8nIHM949GC0JUADEYCbC8VnwKisNkHTHABujaZHX+/qOnAdDu29Bt+IWxlpIC9HCLLzufHV1911LSfgEUiaAA4ApHSdNzCcwJ16GlxdWU20TqFsQ7KMdJltjRPclEGa/A6F9NwOyGpnVs2gL7fCCbIxzbgukhKF54VL31QKAd3xAZaJoEgCYwPZFRXWVlv13vu4RGEztuGliILDrJIZk1tfr9mw20zANQs/hkWa222qJAOq+OC8gdJeLjgnKimScJECtRuMalpCr/+9pQH2r7K6XX4esvGV73rmcl7Za1Ze957xDWSrHf2iQlQ2yYPu4aDLmqMdMEoU5yBoZpA2j8urHvOeYL0C2c7ztyomAq8zqvHzawhzMHdPARjNLraOP+QM4jWnfW8APMJMca6IkTPYqAtfmmO0LeQYa4A1S/BXNIjjjpImAQLKpcNZS5XgxzfpJAYFJ8UAiF86SgybVHCUCUpyk/dmOMJIZ4guyUKIl4vxm+lqyAKDrANRapEwVP5X7oFXuiznKG7QAVyO13n1HEPyPvwJofa1xL4Ia9MrL2dLYQcAgN0763XjsOam0zAzmOsZ6P5hMgh1HovPeY2SZMvs1UVM3HMQspiehJoZYUSvRWMiaEoSBdDvedeQmIdd0r64DbM6a6SHtchRMz316Fvtzv/1edzkXakH4HxGmkBGJSx44AAAAAElFTkSuQmCC</t>
+        </is>
+      </c>
       <c r="N36" t="inlineStr">
         <is>
           <t>Healthcare &amp; Medicine</t>
@@ -3618,7 +3722,11 @@
           <t>TM</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/7gAOQWRvYmUAZAAAAAAB/9sAxQAMCAgICAgMCAgMEAsLCwwPDg0NDhQSDg4TExIXFBIUFBobFxQUGx4eJxsUJCcnJyckMjU1NTI7Ozs7Ozs7Ozs7AQ0KCgwKDA4MDA4RDg4MDREUFA8PERQQERgREBQUExQVFRQTFBUVFRUVFRUaGhoaGhoeHh4eHiMjIyMnJycsLCwCDQoKDAoMDgwMDhEODgwNERQUDw8RFBARGBEQFBQTFBUVFBMUFRUVFRUVFRoaGhoaGh4eHh4eIyMjIycnJywsLP/dAAQAFP/AABEIAIkBNgMAIgABEQECEQL/xAGiAAACAgICAwEAAAAAAAAAAAAABwUGAgMBBAgJCgsBAQABBAEFAAAAAAAAAAAAAAAFAQIDBgQHCAkKCxAAAQIDAgIFCQmBAAAAAAAAAQIDAAQFERIGIRQiMUFhEzZRcXJ0gbGyByQyNDViobPBCAkKFRYXGBkaIyUmJygpKjM3ODk6QkNERUZHSElKUlNUVVZXWFlaY2RlZmdoaWpzdXZ3eHl6goOEhYaHiImKkZKTlJWWl5iZmqKjpKWmp6ipqrS1tre4ubrCw8TFxsfIycrR0tPU1dbX2Nna4eLj5OXm5+jp6vDx8vP09fb3+Pn6EQABAQMCAwMGjwAAAAAAAAABAgADERIxBCFRBRNxBkFhgZHBBwgJChQVFhcYGRoiIyQlJicoKSoyMzQ1Njc4OTpCQ0RFRkdISUpSU1RVVldYWVpiY2RlZmdoaWpyc3R1dnd4eXqCg4SFhoeIiYqSk5SVlpeYmZqhoqOkpaanqKmqsbKztLW2t7i5usLDxMXGx8jJytHS09TV1tfY2drh4uPk5ebn6Onq8PHy8/T19vf4+fr/2gAMAwAAARECEQA/AGrBBBBjEEEEGMQQQQYxBBBBjEEEEGMQQQQYxBBBBjEEEEGMRg681LtqdfWlttItUtZCUjYmM4o22gOLydLNXjcDBVdzrxURb3oRkcOq+WERhGNOwbBRdEXRnKnsmUQQIRhTNJuzV8O0pKmKS3eItGl3Nw6tKQcerJ2EVuUr1Vk5wzrb61uLNrgcKlIXqAoWjYaiI+CJNFDu3aSkJBiKcaZLa++o1++WFqWQUmKQmkBYMw6NhlI1FQYmwJR8jNUoaSUdBRssOgYsMJuGJgO445QwFqKrj7iU247EgJIG8xw6KoZLoS0GAjCTY1C0pWdWg8ohVcvQCQkmWKU1UTNYIIII4jSbEEEEGMQQQQYxBBBBjEEEEGMQQQQYxBBBBjEEEEGMQQQQYwD/0GrBBBBjEEEEGMQQQQYxBBBBjEEEEGMQQQQYxBBBBjEEEEGMRRNtA3UpbXb19UXpSkoSVLISkC0k4gBFWwhpSMJSmco8y0+7LpLa2wsWEWk4iLbDjz8UZ6FUEPQpVJIBEbNTmi3DrSQp7Q6naKayQQmNMgGnAWdqLBG6alJqSdLE20plwcmrFmxGpGiI0xKAgiIpgtrpBSSCCCLMaRYhhYCboh15c2SYpdNo1Rqy7skyVJtsU4cq0nVqOLYDHF8oLMlQ5dFHdm2lzalKcUi8AbVWCwA2HOz8ccWjVJKJAMVRBgKZgKtRpGsl2tL6vVCSiSQFGkCTCAEZ7U01BBBEc06xBBBBjEEEEGMQQQQYxBBBBjEEEEGMQQQQYxBBBBjEEEEGMP/RasEEEGMQQQQYxBBBBjEEEEGMQQQQYxBBBBjEEEEGMRFVjCSnUbh2+ouPkWhlsWq0CTmARKws8LtOGb1be0JjPQrpL5clUYBMaViPBbiVoUSuhXIWgCUpYTE04RBMeGbisYTVKrKUgrLEucxhBxWbuIAKtjEfKTs3IOh+TdUysZ6TZboEZhGgY0QRJJdoSmSEgJqQ+kW19b548XXilqK44SjTFhUtTW6XwmpFYZTKYRy4CwLBMAWi3U5WxSNhaIzGCdGphNSqU3pWRxFtFhBVbjAJSSTsM2KdFqr+mnSO0NoVGBbuu1JS7UpCXioECYUo0ozNzXNEB+h4t+7Q8W4QFJURAmmBBUIShTs7a6lhhYzkKgtZCYTivgJSsjQABCdXbbFcU66t0vLWpThN4rJJXbqbc22MIIzodIdiCRPOZybEtw31EPX5itUYTAUkiwApBrLRsNZySsZqV6bZxALtGlUjY7i2Ji606pyVVY0vJOaUSDYoWFKknUEGFLFx2zzcU9qmfX44tF0O7CFPEiSRCkJjEwmaQrNo58p6hwsy0qjAqwkIAmezzWdrnBBBHAaaYggggxiCCCDGIIIIMYggggxiCCCDGIIIIMYggggxgP/SasEEEGMQQQQYxBBBBjEEEEGMQQQQYxBBBBjEEEEGMQs8LtOGb1be0Ji+1OtU6koKpt0BdlqWhlnFajELTscyK7N0yjYVqVPUya0lPKSC4yvHaUgDGk2EZlloxRyaENdKLxQIQUwlQMIxHDNH1ppFEIDl2pJepWFSJQCoAEUrTTmamQR2p+mT1Mc0lPMqaJ3CTjQrVKFoMddKVLUEIBUpRsCQLSTqAIkgQREEEVRM0EpKkmSoEKFmIgbY2MWvCDTTpHaG0KjXRsCZqbseqhVKtYiGxZpVQ3m7sRbFpn8HpCfpzVNXfbblwNIqScskgXRm227GOI/oh2Fu4GMhUSRTE0GkaEoF+XL4lMmvXYCQqkSYgzWaazsr4ImaxgvUqSpSwgzEsMYeQMwbuSCSNlENHKQtKxKSQRaGj3jpblRQ8SUqFmNuqhiLjtnm4p7VM+vxBUjB2pVdaS02W5cnG+sWIs0LSL2wizSc1g5gmTLImFTD7ykiYWnL3btuMhNoFluZjMYKKWFoU6TFSzCkkRhAg06jcys90p29RRDyDt0mN7lmTGIIpRnna1QRplZyVnmg/KOpebPJyDbsDqDoGN0RhBFI0iGnwQoAggg2cUwxBBBBqsQQQQYxBBBBjEEEEGMQQQQYxBBBBjEEEEGM/9NqwQQQYxBBBBjEEEEGMQQQQYxBBBBjEEEEGMRSa1hxMFxyVpSQ0lKikvrF5ZsxG6CLBsbYu0KCZ3MO9bV7MxyqCdIeKUVCMmEAZqcWjq1qIeuEOw7VJllUSJ6UJjZp2wccW64p11RWtZJUo4ySc+BC1trS42opWkgpUMRBGfGMESLQUTGMadVrRT8L1TCBTq80mal3bEKcAsWLcVpAxHYWGLXTKBS6StTkm1Y4u21ayVqAPJotzBCva46o1tOzEOGOBRiQ6gERSFxikGlShZmmqynhoiUX0FqcyZK1AFQCoxpz2ZiCCCOG0oxEDU6Jg/Jl2tzUuTpIX1ISVXFKJABu5ltp1UT0RGFem9Oawja0xkcky0gEgKUAYGFIlsNEpSXS1KSlRdoUoSgCAQCRO1Pq+F1RqaFS7IErLKFmk0Y1Eagqs2VkQUEESqEJdiCQAG1p6+eP1Sniio2m3CYCwbsyFQnKa+JiScLa7LDmEEagg2gxecG8K+Bw7kKaaDcwEFQUi0oWBm4jmd7hexP4EbryOtLuyEYqKdIW7Uoi9yUkg2ek3JrPoh67fO3aVGQtYBSaYp80bBmLBBBEW2xMQQQQYxBBBBjEEEEGMQQQQYxBBBBjEEEEGMD/1GrBBBBjEEEEGMQQQQYxBBBBjEEEEGMQQQQYxCfmNzDvW1ezMOCIasYLU6rJUtKRLzJxh5AzTu4AgK2ccihH6XKjKjBUKYs0G4NaVCLopCa7IlO5RkmlGMJjVpMtIIkqvQahRnLJlF9o7heQCWzoE2Cw6Bjik0KoVhy7KoutjcTywQ0NC2w2nQiRrxEmXKEmrZmg64e15XUhUuOEYU/paW6LXHVGtp2YhwxC0bBWnUpKXHEiZmRj0ssYgd2pJIGrzYmojqLfpfFMmMExpmzxh4DTlZtBroVCy8Ii8k3tFOEIzmrTYgggjjtzmIiMK9N6c1hG1piXjFaEOJKHEhSVCwpUAQRqCDFyFSVJVPJUDbC1j1FeO1ojCWhQjYiDJ2CL3WcCJaaJfpRTLOYyWjbpJR0M27sBZFLnJKakHjLzbSmlg5igQDog54iVdP0Phe008smdtbomg31Cm96YpsyxTSfAtbaIn8Cd15HWl3ZCCjYIT9TAfmNujFuatJ0oobtSbMWiTF4ptHp9KbuSTKUKIsU4cs4rVqNp2EYaJolASp2DKUoEUphYluVWfQD5TxD5QkIQoG905hUFvLd2CCCI5p1iCCCDGIIIIMYggggxiCCCDGIIIIMYggggxv/VasEakzUqu2482qwkGxSTYRiOfHJmJdItU6gDRUBvsGNsgjFC0OIC21BaVC0KSQQdURGUGMQQQQYxBBBBjEEEEGMQQQQYxBBBBjcKSlaShYCkqFhBFoI1BjhCENpCG0hKUiwJSAABqABGUEGQs7EEEEGMQQQQYxBHAUkkgEEpNhAzRn445gxiMHGmnbpdQldxV5N4BVh1ItzDGV5N67aLwFtmfZqd4jmDIRnYggggxiCCCDGIIIIMYggggxiCCCDGIIIIMYggggxiCCCDGP/Wu7+CtBlaa8Eyja1oYcOlVi84pV0kqJ1JOOI7A2gUWdwZk5iak2nXXEOX1qGWOXWNlFnqG5CZ13d2kxD4B6akhrDm9i4rZmN2jO0zBxmTpS9KpSQhiWAQty+oWAJBSDj1cSExNIlpdU06ldxCbyglJUoCy0mwWnFEDhYeIlg+OnqnZRN1LdOmtd3dpMUY3ErUGJ2TE9LBa2VpvINxSVLScYIBsMdFvCqkOy65trS65dpSkuOpl31IQU7iCiG8VmfG/BzFQKdrkxtCYqmD9alqVg7PmcYdW2qfm03wi8youEJCVKtsGPNtsisGNd5aZYnGG5qVcS6y6kKQtJtSQY0TVWkpV8SqlKdmCm/pBlCnnQnMvEJBujRNgjr4M05dJoUpIurS4tDZUpSDeRasldiTnjLYojsCXBONVCpP5aceqDyHlHcSUt2BtvQSBmCKMaUar1OXNIkXVLlphzjm3MNrYK9YKgEq2BjvPOhltTpSpQSLSEAqVsAMZivYfMNLwedmzlZiTcadl3RiWld9KcRzcYMTjCnVyDa3xY6phJWMzLFIKt5gxtVMq0nWGDMyBWtm0pDikKbSSMRAvAE2QJq0quoKpYDmSUIDikltQSEE3Qu9ZdstGpiJwA02met0xvYqOyzp4TPXKY3tcirGkZyoycgEZJcuqdVdabSFOOrObYlCQpStgI6rmEVOl1IE8HpNLiglLkw0400ScwFZTdB1ZERtOdE5hrU8lY1yMuy3KIVmIQsXnFp0SSLTqMUTFalJaepU1LTaQppTDhN7OsBIVoEEWwY3aW4Etl0ArAFoCBeJGhqY6lMrMjWELckCtbbayhS1IW2kKFlqcsAbRbHRwKemX8GZFyaJUu4pKVKxkoSpSUHvQEdbAEcQeY0alNbUIMaZfqksw+ZVIcffSgLW2yhThQk22FVgsFtmIE2nOjOWn2JuSE9Lha21XrE3FJctSooULpANoIOKK/WGq/RKu9XaS2J2TmUNZMls10aSF28jMO4dRbqonaROyVRp7U7TxdYevLCbLpCio3wRqb1tsUY3VZwnpczLKnJYTDzLZUFrRLvqAKNxDcGdEohYcQlacxQBFuI2HHFLwQerLdFmBISrMw3k2a46OFKyb2MXbhB73F1AsFgipY1PYrLsjhxOMvi7JT7jcslw7hD7TSCkW6khdmxEXAkAWnEBmmKe/SVVyj1dTA29IrEy/KLGJQWzdQmw6IRZG5GEDlboEpLSq7lRqC8iOgCxTRQBklyzOsRaRokQY2OD1WeqWFtScWLGHJNsyu7mW1qSlY0FFRMWiZmZeTYXMzTiWWmxapayEpA2MVoMM03DmSl5dIbZdo6mEJGZw6USBsAmNmErodr9DpkzuTfeddcSdwOONgFpJ1IvG2yDGk3K/JtN6XcamksAWl7Iz9wDnIi5eA0bI7srNy09LpmpN1L7LgtStBCkmNpAUClQtBFhBxiKvgg2ZWqV2ny+KSl51JZRyYhSwStKd4xRRjTUtW5KbnnaczpTJLFheQptabgONJJIAx51hjOdqsrT3WWZkOXplYbZuIUsKWbTdtSDYbBnxEUcDgsK6rP0nJDxyOzhDjmqNqeBq3vW7bFWNIztQlKdLZLnV6RZvISVqBsSVkJTbZbYLTjMdgKSpIWk3kkWgjGCM0WRD4VsNTVLRLPpvNPT0k24m0i1KnmwRaNAxFyU5OYIzgpdYWpykOruyE6rLaStzGnVYrBZmGzeMxBjWKSqctPreRLhy2XcLTt9CkBKxYSm0gWmwjMjpOYV0llkTL+SG2VKCUuql3w2ok2C6rSdhtsxWZsZUCwmpkYwaq+bRn5VuI7D9KUUBpCAEpTPSoAGIABWICDGmZWrys3NZDQh9t3SanbHmXWAUpISSCtKbcahG2o1GUpUouenl6TZbsvKzdxEJAAGM4zHYupvX7BeAICrMdhxkW7CK5XnJKp1DgTzpWZRiXU4+G23HOHzgusg3EqxpSSrHn2GKMaxpUlaQtBCkqAIIxgg4wY6NQrUjTHmWJvSiVzKw2zdbW4FrOYgFIOPVxG4E1ByapJkZlRM1TXDLOXgUqKU8c1WGw406kZ0a8L9z2D/AF2Wd9isKbGn5ibZlJRydmCUNNNlxZIJISkWnELTbGUvMMTbCJmWWl1p1IUhaTakg58dDCXTeqOuT20mIJOS8CplLidKPYPP2Facbq5Ras8Z9wk6Pe82jGl6hhdQqXMqk6g8tl5IBKS06rEcwgpQoWQVDC6hUuZVJ1B5bLyQCUlp1WI5hBShQsij4bqYnK4ZllYcbcl2VIWggpUki0EQYbqYnK4ZllYcbcl2VIWggpUki0ERWDUiwP/XZVTanZiTcl5EtpcdQpBU9eugKBBIu5+OOng1S56i09FMmVtOtMBQaW3eCzeUVZYEWZ+dEvBBjR1bo7dYl206UUxMSzyX5Z9FhKHE5hsIII1IjqKksJp5lUlUX5RqXdSUPOyqXRMKScRCb9qUkjNOOzOicggxtIZMtKJl5FKE6SbShlK7bgCQAkGy02WCISi4NPSlNm6RVSzMys2446q5fCrzlhUMeoItBzYsMEGNDUWnVqlESLsw1NU5q0MLXfE2lHJqCQLpAjU5QZ6nzz1QwdebZM2u/MysyFKllK5zTdyyVamw2RPQQixqrW6ZhVPssuu5DmUyz6XVSDelENvXcYtUogkg4wDYNTbEhTMK6TUnTJrUqUnE4nJWYFxYOeAcaTsDE1FF20ncLOsmKimxpZmm1OgqVL0WZlTJPulbbE7fvtrcNpSgozUk5xiUptNdlnnqhOuB6dmUoS4pIutIQi262gZoSLScZtJinYB7nkdajvkMGBY0NU6C49PprVJeyJUUI0mpSheYeRzi4nNOgRj3iMVyFfqTSpOrPy7Es4m69kHSgdWDmovOW3Qc+wW6MTcEUY2hLGRZMS1PQhsNNhDKFWhsAYgDZabIi8GKNP0OXelZpxp5tx5b4U3fCgpdl4WHFZixRNwQY0S8xhE3MzGQnpVUu8sLbyQHS41alKVAXcRGK0RvkKbwKaWiQp5CltJUUqdxJUtRKlKVdGeScQEd+CDGq9KomE1FklyUlMSSw4647fdS8VJU5jNlhAItzLYsNyabkw20pLkwhpKQt226pQABUqzHjjfBBjRGD1MqFKZel51xp5Lj7j4W2FBV51V5QIOKy04owpmDMrTazO1VrMmbC03nNleN4gWWC8QImoIMaBq1Fqc3XJOsSTrDeQW1JSly+Su/iUFWDELMyyO3WKIzWpZlMwpTEzLqDrEwybFtuCzGm0YxaMwxJwQY0K01hfdDLz8jZuEzCUO6Ws5yunKXt4jvUuly1Jl1My95anHFOvPOG8664rGpajYMcdyCDGhZ2jTrVTXWaI621MvtpbmWpgKVLupRuFWVywUNSI2S9NqM1OMz1acaUqUKlS7EsFBkKUCkuKK8spVhsGcIloIMaMrkhP1BthqTU0gNTDT6i7fxlpQWlOVziRjjtTkhLVOTVJ1FpLrbiQFozRbqQcRFhzDmx2YIMaLweoyqHKOyZdL6VTLjra1EldxQSEhRsFpF2NOE9Gnq5KokpZxpptLqHlKcvFd5BJSAALLNTE1BBjaW8l5G4ehvJN07hvaSvZ2aLbI6VEp87IpmV1BbbsxNTKn1uNXgDaAkJy2ckAAaEScEGNBtUaoSuEcxWJVxlMtNobQ+wb95RQLNKYhZezoK/R6lVZqRelXGW0SEwmZQHL5Upac42DEInIIRY0dWJOdqNKdkGFNNuTLRacUq8UpChYopsFp0LY7Lcup6SEtUUNuFTdx1CQVNKGZmKx2R2IIMakTm2evZIWadMITLE2ttvla1NjnAGw5UHMgnNs9eyQs06YQmWJtbbfK1qbHOANhyoOZF3gisSyDA/9k=</t>
+        </is>
+      </c>
       <c r="N37" t="inlineStr">
         <is>
           <t>Administration &amp; Operations</t>
@@ -4418,7 +4526,11 @@
           <t>SCI</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAiQAAABzCAYAAACo5xkWAAAACXBIWXMAAA7EAAAOxAGVKw4bAAARrUlEQVR4nO3dy3LbRhaAYa5HSRxLpnjTSBZJkJpUeaVn8fP4UWbvB0hVVtxkPEmVHMkiCZD2eJEn6cFp6EYSAHFpoAHwX3y0LJK4kVU4On36dKvVaqk6+/3kRLlOT62u+mo9HajVtK++/uvM/3egPP93nv//1aSn3NGp+liB4wUAAKGsH0Amd50jP9AY+EFIEIAkIa/1pl31qQLHDwAANlg/gFT8Bz+oCDIiSQORbTp7Mu3obdk+HwAAoFk/gMRurls6K7K6GmQORp6yJVcylNNX6vra+nkBAAD7B5DIjU/XiBgIRp4yJf62pL5EVeD8AAA4cNYPYC8pRvVS1Iqky5QMHmpLesodd9Xs4pX18wUA4ABZP4C9PKdvNDOyN2vyEKBIAeyf/R/JoAAAUDzrBxBq1m6p5eRUD6nkKWA1UWsilv5xfP7nCcEJAADFsH4AT2RoZu20dXZiXVJGJF32JOh14o57alaB6wUAQINYPwD1b5837uqbfZq+IvYCk8HD1OG++v3E/vUDAKAB7O181gqKVSXzUFaNiNnhnIEezvGcrvp0Zv2DBACgzsrfqXov/UQ6OhtSx0AkPGPSZwoxAADZlbcz/0HNR2093LE3+5DgNVUkGR/38o3tDxUAgLopZ0d/dX/QnVFXMTUiq8eeIOOe+mpxZk1eMpTjTros5gcAQHLF7sB/CKbuRmQ8JAiRrIL0GpmPXj+9b205IAnqWnqxAdTebch5XXRsf8AAANRBcRu/vXjlBxuD0GDkse5i7eyuvvvBZ7P3SBBMDNTvJyfq9uw4KLzNOIQkgZXr7A9Klk4QtAVTiwOrSVd9Hw5tf0EAAChDMRt2h53orMg0WEMmakjj/vLUerGr7H/uHD8d0+zVq8xN2uQ9rhS8vg8/36i+Kzpoe3jvDYsAAgCazfxGXacb2k8kCES6e5uKfZn2rQ/ZCOmNsn1sn85+0oFJ2qLbx/oYtXOtOnu39bgIYAW+LAAAFMXcxvwH/df8dnYjqBMZ6MxHku38NQ4PaErPksQEAffvzh8yGCkDE/+8pC2+bGPh9FMFNksn2fUDAKCGzGzo11Yw9LB9E5Ub7nLSSdWfozIByVU/9jjlnFynn/pYJShZjjqps0CSearAFwYAgCLk38jNdStiiKav5uN26u1J9qEKa9nsC0gefX77czAjJ8Uxpy2SlWOR61yBLwwAAEXItwEZfti+GQc1DwO1aGfb5t8SkNQgQ/KSFOi6V8WsTCzB2WJKDQkAoNGyv3nW2p2eqxub+T7k2K6S7VYgIJHhptTHPelmniIcRYbCaLIGAGi4ZC9cOG0dfAQ9OZ7/fZkZCYIRM+u52J72qzMkk+QZkpdkurCpIScJbuhFAgA4ANFPSsMyb9oNmpvtucHqzqYTc11JJRiwH5BkLyK96xzlPgfJ0Hx5e2L7CwIAQBnCn3D7P6aq4/AyZhOi6M6lFrMkQR1Mvmm2N70fMvdTkcyIO6ZuBABwMMKfCJvCG38D7avV0Ny0VJlGbLN9vJzPH8fHuc5BZsWkvY6PmZE82RkAAGoo/IksRaWSDfj2S7pC0DhZbubmApJ85yFt4t2rfvrGaQ9dWZX9LwYAAGUKf8LLOMtFr73imLmh3l2+MT5jJalljnoY9XD9shS2yvnOaYAGADg84U/81skelARDDrvrtmThWQhIpHZmdvEq0/HKdcs71CSBjIlrBwBAjUQ/KUWdeW6uMuTyx3G+A1yM2qVnSbJO972/PDLSP0WGbZYspgcAOCzxL1j9kn4Buc0hiL66Pz/PdZBSU1FmdkSm7KY9Ruk9kjWjFB6U9NWnM+tfDgAAyhL/AskW5J1+KzfXZY5ZI7NWOTNugoLS9Mcpq/CabnUvxyK1OBX4ggAAUIboJ2/O3xgLBIIur93MLdBvL14V3k5etn9zfZ34mPyHIGAr6LikFkdqUirwJQEAoGjRT3qT3XVqcg3f+O+VYY3Pb7NlS+7G/cIyJbLd78PXiY9FamN0RiXXcFb8+7NmbAAAqKHwJ5bDNxvDEJIFkIBAeo3kXadFtiX9SlSGA56/bRut1dCBlgRKKZq66XV9ch6DZD/+vNi/HQmUWFgPAHAAwp9YbTUlk7/m/SeCYQoDWYrgr/++uj9N355dD9+YGkryA4KFHxgk2a8EBp7Tzz3rRwI9CfhkmwunE9teXoKlJX1JAADNt/vLxbi7cdPVRanj56mw0oV0laELafgNt6+8cfpGarLwn8y+yZqpkKAgmFGTrAHal2G+KdAvMyOu87xPOe99GR95Pu31AQCgZnZ/uT1jZBVyQwzWaclXQ/EyCyD7mE+6qW+83jCY4ZI0MAmatvmBzKSdaF/fh0OdyVkb6IUi57kO6WJ7/y4+4yPX+O93+aZOAwBQcZu/+DI+3rg5rvRNNHzIQA9hTM2tyhvMxOmru2EndWBye3asXP84vYfgJCjAffj5Ybsyy2c+ThaI6HMb93LXy2wHJLOI/a0m8QEVU4ABAA23+YvtBe3khj6L2YDpoCTYZzAbZ+4kq+0II8csM2HkX5XiffJaufnnnVG0e05+QBTTjn759ufYLIxcjwp8WQAAKMrzf2a+7YyAl2DaaTB8Y/YGrjMKss1JsFjfrOALIf0+lromxcww1O557M9wxBXLyuci17kCXxgAAIrw/B/dcfTFzVhukPcJp8P6D8YzJU/H8VBjoutMpp3UWY8ov7aCwtj1tGe80+pmdiPZFGe51rF9SUbMtgEANNbzf7ZvhquEN9KXigpKNo8rqBHxnK5aTNrqbni0N3sg5/HH8bGaS53JOJi6W3Tn18dg6jbFysFxgdHqijoSAEBjBT98v369c4POuurtykDztDSCZm2PBaw9feMOilj7T0WuqwKGlPYel/QbcdLNjpHOrHHnWYEvDAAARQh+cLdmlASLuyXr0bFNCl2DGS7lBgBVkyWgkxlGUVOApehVsjwV+NIAAGBa8MP2tFO5+aUZatj28b2ZlYLrSrIjn85+Sn3dVCu6E65eC2hElgQA0Ej+TfD6eme4xsTwgP9QSk1JFS1zTNN1Y3qSSC+VCnxpAAAwraVuhq93iilN9b3wH5TnHFZQIsHdTY5rthi1I2tw6EcCAGgo6b/RCbnxmZvR4T8E7doPICjRtTfjfNdOpiN7UcM2BCQAgGZqhXYIzXtT3eY/+EGJ+aZjVSOZjQ8Grtf2assEJACARvMfQ4soZdjA9M707JtJ+I22CUxkRx5JrUjUPj7a/tIAAGCa7la6FZDITS9PDUQcadEet7JtnUkdjqlgYeHsDqMFn01f/dWlsBUA0DBB34vtDq19PfOmqJ1+Hw71LB7bAYRpnsFOqveXR6HXSHq73E6z9YcBAKCyls7uEIoOSAre8V/jH0pp3V5edmSg7jpHxq6PZFrCZtpIFmYxJkMCAGiYr2M7AYmQOpWmBCVZ2+zHCcuQEJAAABoprMi0rIBEfNer7dZ/5o1neFaSCJtpQ0ACAGgkLyQYKDMgEf+7qnePEr1uz7n5ug4vJHtEQAIAaCTXcoZEyL68iL4bdSAZniKuFwEJAOBghNVwrEsOSIQsRFfXepKVwa62L20vePiYjVkO39j/4gAAYFJoQHJVfkAiPKemAcmkmIAkLGskM29unWP7XxwAAEyK+ivcRjfQ+8vTWjZN80bFBCRhawxJQDJrm++iCwCAVeuI2o2/352XfjC6tXzNAhJpVHZ/cVLI9QgPSFjLBgDQQFF1G8uxnTqFqEXlqkoCBOk8W8S1CCtq9a4G9r80AACYFhmQFNDoK4m6FbauC1x9N6yGhNV+AQCN5EYEAF5BM0f2+VqzgMQrMEAIa1pn63MBAKBQq6vwIZIi//KPolcerlnX1iIzFuuwIRsyJACAJgqrU3i80aqSD+amV78F94oMSLY/G90UbcQMGwBAA7khq/3qG+3VQM3H5d785s5x7VrIFxWQ3Fxfq69b2SIbQSIAAKVwR6eRN9uyhwfCaiaqrqiA5K5ztJMtoqAVANBY/5EbX0RWQuo5yjwYN6KepcqKChLup92dfbkT1rABADRUXCGpBCq/dco7mLr1IBFFZZHckA660snW+hcGAIAi+I+R3VElIHHH5UwzlZqJdc26tIp1QVmk7c9kZWl9IQAASiK1G9GFpGXVkdxevAqd5lp1EijcGL4W0kJ/e4aNV/LwGQAAJZOAZLde4emG698Iy1jXxh3Vb7gmyJD01d2kY/RazJ32Tl3PcsJwDQCg0VrqP8MjvYpseAZgoAOWog8kavpx1cn1WUzMTo/2tq6FBIUz+18UAACK1NK1CXHDJWX0vwhbt6UulgYDto/vd9fzoV08AOAABD/E9QCRYOX7pNibYlRhbR2YDBiWo87GcI1ce2bXAAAOQPCDNzyNz5JcFVfc6j/UcobN07UxuDLydmAowY6y/yUBAKBowQ8y7XYV0vvi5V/q3lUxxa3+Q+0W1du4NldmZsDcbF0HyZR4Y5qhAQAOwvN/PCc+S6FrSd6bPwhpzlbHKb/PgUNf/ffyKPd1CFtMz/SUYgAAKur5P8u3P8fWcshf797I7BRXsT47th5U5AtI8l+XoGNuf2Obq4LrdgAAqJDNX+xr3y61HjfXZg/Cq+EaNtvcnMGDTK3eKGb1f561rX85AAAoy+Yvlk5Pt0OPv/mazZIsRtGN2eoizyJ7n852syOuQ+0IAOCgbP7Cf9ipZdgdougr78JcUOLuqV2pA130e3KS8fy3G6Gxbg0A4ODs/tIdn+60Lg/LCChDB7GuaZfWzSBtoNxR+n4hX8bHG9darus9M2sAAIdn95f+w0630LAbsKmF9+raNn7nmqTsRxK2iN6KRfQAAIcp/InFsLe3N4gUXi4N1DrUuW38ZkAy0EFG0vOWOpGX9Toy7PNfurICAA5T+BP+Q6J27p7/mm+j17kOIq5tfZ1IACdTp5Oc85fB8U4h67dfil9VGQCAiop+8rP0JUnQsEymAv9+kv0gmpIhEUmm//oPO9knGbr5WEDTOQAAaiL+BdIfI8mNWIKKDxkPokkBidSRqATn/DLQk6GvxdlPtr8IAADYFP8C/yHxwndyM05TQ/GoUQHJdKBuz473nrM77ulhGqkbWTjmu98CAFAz+1/0edRONHQTZEr6qTMlTQpIHgOzfecswzPLSU/NL5niCwBAK+kLl5NOogXwgunAvVSZkqYFJJJRypIpAgDggCV7of+gZ8Psa5j2HJT01W+dZNtuyiyb54BkoBbnZD4AAEgh+Yv9h8RDN3q1WqmPuPjH3u02LUOigxJDTeMAADgQ6d7wfThMlCXZyBY47dhtNi1DogOy6UD9av/DBQCgLtK/SdZf2bci8PbNWYIOFbE9KQK1HUAUYc7sGQAAksr2xvvJSaIi15eZEk8P4exmS5oakLBqLwAAiWV/89zpJq4peQpMpkGLdPViO96obT14KCogkcZyFfiQAQCounwbuH93nmjNm40b9WO2ZBw0EHNHb6wHD0UGJRX4kAEAqLr8G7m/PNVDMmlv1tKvw3N6au00M0MSnONA3Z1TSwIAwB5mNiSNwLLOlkmbYambJAvuAQBw4MxuUIZi0kwLPgQM2wAAsJf5jd5PToOCTgITzSMgAQBgn2I2fNdp6aGYpCsFN5We7jxmpg0AAHsUu4O509Z9Rg4xWyIN4Tx6kQAAkETxO7m5vlau01XegWRLpNfK2g/CPv/zxPaHCwBAXZS3s5lv7QcmWaYI14HUzXh+MHJ78cr2hwoAQN2Uv1PJmHz7ZaAzJqsUa+JUkQxFSZ2MTHkOa4sPAAASsbdz/0EtnI5/U+/VrsZECna1SVfN2tY/RAAA6s76AWifzn5SrtML+pikXB+n1CBEF6r21GLcpVgVAABzrB/AjrvOUVAE+xCc2Kw5kX3LLCFpcS9ByIcKXB8AABrI+gHEmvm+vD3xA4KHIZJpv7BW8+uH4EdqQuRnWYVYClRVBa4DAAANZ/0AUpE1c26upRvsiS4kdaXHie/bdBAEK9OHgEIyGw+Biy481b8PXrN+Qd67nHSVOz5Vf/Z/1Nu3fY4AABya/wNrnaX0sYDP9wAAAABJRU5ErkJggg==</t>
+        </is>
+      </c>
       <c r="N46" t="inlineStr">
         <is>
           <t>Protection &amp; Social Work</t>
@@ -4506,7 +4618,11 @@
           <t>SCI</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/7gAOQWRvYmUAZAAAAAAB/9sAxQAGBAQEBAQGBAQGCAYGBggKCAcHCAoMCgoKCgoMDAwMDA4ODAwMDhAQFRMMExQUFBQZGhwcHBofHx8fHx8fHx8fAQcGBgcGBwoICAoNDAwMDAwODg4ODBAMDREODhAUEBAQFBAQFBIVFRUVFRIXGhoaGhcdHx8fHR8fHx8fHx8fHx8CBwYGBwYHCggICg0MDAwMDA4ODg4MEAwNEQ4OEBQQEBAUEBAUEhUVFRUVEhcaGhoaFx0fHx8dHx8fHx8fHx8fH//dAAQANP/AABEIAK4DNwMAIgABEQECEQL/xAGiAAEAAgICAgMAAAAAAAAAAAAABgcFCAIEAQMJCgsBAQACAgICAwAAAAAAAAAAAAAEBQIGAwcBCAkKCxAAAgECAwICBgcKfwAAAAAAAAECAxEEBSEGEgcxEyJBUWFxFDI1cnOBswgWIyQlNGR0krEJChUXGBkaJicoKSozNjc4OTpCQ0RFRkdISUpSU1RVVldYWVpiY2VmZ2hpanV2d3h5eoKDhIWGh4iJipGTlJWWl5iZmqGio6SlpqeoqaqytLW2t7i5usHCw8TFxsfIycrR0tPU1dbX2Nna4eLj5OXm5+jp6vDx8vP09fb3+Pn6EQABAgIDBAYFEHsAAAAAAAABAAIDEQQFIQYSMUETImFxgZEUFUKx8QcICQoWFxgZMjQ1UWJyc6EaIyQlJicoKSozNjc4OTpDREVGR0hJSlJTVFVWV1hZWmNkZWZnaGlqdHV2d3h5eoKDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usHCw8TFxsfIycrR0tPU1dbX2Nna4eLj5OXm5+jp6vDy8/T19vf4+fr/2gAMAwAAARECEQA/ANVAAEQABEAARAZjJdlM6z208HR3KD8pFW8Kfkridm5axs91Oz47E4yfg7y3LMVSxuIxNXFVqFVVKdkqVPlbON4pzldNX0lbmW58aNTIMCYLpu3oWn6ytavqGn1heuZDLYZIy7sq2RxgG12gsTs5wdOvTp47PnKnCSUo4SPKzaun3EfHFNccVrrxpqxPMLhMHgabo4KhTw9NvecKUFBNtJXaSWui1PdxgpI1IiRzN5sxDEF2HV9VUSrWBsBgnIXzza9x3sn1wsXGpTp1acqVaEZwmnGcJJNSTVmmnxoi+0GwGWZnF1srUMDiVd2jHuFPlbKLitIcS1iufdNkqBjCjRILr5jiNdpLlpdBo1OhmHSIbXjNGWGaDhGgqJxeExOAxNTB4ym6Vak92cJcaffmuamtGj0l7YrB4PHQVPG4eliIRe8o1YKaT1V0pJq+phMXsHsxi1U3cNLDzqPe5JRnJOLvd7sW3BLmWtZLiLSHWrCBfsIOZaPXLT6TcZSGkmjxmOFsg+bHSxCYBBOloKpATXNuDPHUIOtk9dYtbz7gzSpzUbrdSk3uydm95vd4tOOxDq+Hr4WrKhiqc6NWNt6nUi4yV1dXTSa0dybCjwo4mxwOZj0lr1Nq2mVe69pEIsngOFpznCYOdNesAHKoaAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIv//Q1UAARADO7K7K4naPE7zvSwVJ9xq3P5u5C+jk79ktXzE8YkRsJpe4yAXNRqNGpcZsGC0ue4yAGvzAMZXQyjJsxzvFRwuX0nNtpTqNPkdNO/LTkk7LR9F8y7LFyDYDKsthCtmUY47FWu1NXowdmmlF6S4+OXOTSRmIQyPZbLnGLp4LCRblyzd5yaberblOVlotXZWXEQTaHhDx2PcsNk29g8M0r1HZV5Ozvqm1Fa6W10vfWxWOjUinEtggsZveDTPrgtvh0GqrnYbYtOIjUg4GABwGc0y7ydoKf5lnmUZSu6li6dFpKSp33ptN2TUI3k1dcaR2cNiKWLw1LF0G3SrQjUptq14yV09deJlEylKcnObcpSbcpN3bb422XvSoU8LRp4WjDkVOjFU4U9Xuxjoo8s3LS1tXcjUuiNorWWkl08wWS+GrSpK6i1xFjnI2shwwyQmXPJcThNglIb0uYAIivUAARD18nodSOonJYcn3OSci3lv7l7b27e9r6XPYQPhQqVKNTKK1KUoVIOvKM4tpxknSs01qmrHLR4WTxRDnKc7cOATUKs6bquoj6Te394WTbOUw5wbh0VPDoZxkeW59h1h8ypb+5vOnUi92dNyVm4v6x3TsrrQg+Q8I+JwdOGFzqnLFUoJRVeD7jJJPq280pviV7p813ZP8Fj8FmWHWKwFaFek7ctB3s2k7SXHF2aunqZRYEaiuBMxvThg01w0OsqBXUEsaQ6Yy8J4tGeDYc8TVZbRbCZlk/JsZg11KwMLy30+4lOCt1eNle13rG+iu7EYL8IDtNwe1a2Nhitn4wjTrzSrUJNRjSb45x9Ic+K1XMTWin0SsL7KRiAcTsAOetbru5YwuF9Aa5wnloW6iJ424yMzCM7BCcLl+Px+91Bw1bEblt/kVOU9297X3U7Xsxi8uzDAKDx2GrYfkl9zktOUN7dte28le11cunKsrwWS4KGAy+G5TjrKT6tOT45Sel27fWKysj316FDF0pYfF0oV6U7b1OpFSi7O6ummuNXMTWuXsZlZ73bJcrLiwYAvqQRFlaA2bA7esRlinoyxKhwZbarLsNlOf4vAYO6o05RcE3eynCM7X47Lesr6255iSzY4PaHDAQCNFafHguo8aJBfK+hvcwytE2mR1yAAyXGgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACL/9HVQkez2w+Z59ShjZThhsHO+7Wly8pWcovdgmuJxs7tdC5HC39jM1w2Z5BhqdGSVXCU4UK1K93HcW7GT0WklG/O5l9GRKdGiQIQdDGEyJwyV3c5V9ErGmGHSSZBhc1gN7fkETE8NgxC3SKxlPgwyRU4qtisVKaS3pRdOMW7atJwk0uhd9MzOZ5jluyGSxnCju0qVqWHoQ8lTabSb1txNyk+jxvjy56cXhMNj8NUweMpqrRqrdnCXNXf0+amtUU5jviubkzi5oMyJyW+Mq2BQ4UTUGHDhRXMLWuLb63FOdsp/XmqZzjPcyz3ELEZjV39y6pwS3YQUne0Uvdru7dlduxjySbT7F43IN7GUZdSMC52jUXV6adt1VFZJauya0fQukRsv4Lob2AwpXuKVktBdZU+DS4NJe2lh2SzmS4zJ3ozxjekLp2ZxFLE7O5bUoy3oxw1Om3ZrlqcVCa1S4pJopYsLgyzjklGvkVRTcqe9iKU3K8VBuEZQSfFq7q3Hd8XNi1lDL4N8NZM9DArm5KltgU8wnWCMwtG/gZgaNqnQAKRdhoAAiEC4VfKr6WI+wielUbf5rHMs/qUaTbpYJcgWrs5xb5I7NKzvyr5+7cmVcwupDSMDQSdES9eqG6qOyFVURjjbFcxrRmhweeCao0ZPKNos4yOS8E/ESjT3t6VCXLUpN7u9eL0Tagk5KztzTGHeynJsxzvExwuX0nNtpTqWfI6ad9Zys0lo+i+Zdl1EDC05JK9xzwLr2imkCMzUYvEQmTbyd9PMkrbyDaDA7Q4JYnCvcqxsq9Bu8qcvrYvmPm9O6WTMNs7stl2zlOTw962IqRSq4idr2Vrxil1WN1e2r57dkZk1yLkeSHI53s7JrtegmlGjQ9Sw0RZZa9MxP4e9ysngQwm1e0tLZvAxmo8kxWI3o4eDT3bxtecnzldacb+JWbKm2/p42G0td4yW9GcISw7XEqVrJJOUraqV+K7u7K5zUKA2PGvXmwCct7zFBugrCNVtBMSCMu5wYHSmGTmb6WhIZukY9UqVK1SVWrJznNuU5ybcpSbu229W2cQDYF1gSSZlAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABF//0tVCzuDrI+oOWyzavC1fG6U7qzjRXFxxTW89eNprdZX+SZdLNs2wuXJNqtUSnutKSgtZtOWl1FNlu53mFPIMjxGMoU0lhqahRpxjyqbahBWTjyqbV0uZxFdWMUkNgNwvInnTs0ytpuUojA6NWMbdEBrpGWO9m46Ddeu3RxeExM6tLDV6VadF7tWEJxlKDu1aSTbi7p8fOPcUvs/tBjdnscsXheWhK0a1FvlakedzbNcx8zoq6du5VmuCzrBQx+AnvU5aSi9JQkuOMlrZq/1qummQaVQ3UYg4WnHm70VslS15BrZpaQGRWzJZOc2zsIOPNXZqU6dWnKlVjGdOacZwkrxkmrNNPRogO1HB9W5OsXs5S36dTxkw28k4PzdFyaW6+ar6Pi00VgA4oFIiUd18w54OAqZWNWUas4WRx24LWubIPbnGR0sCoWpTqUakqVWLhODcZwkmpRknZpp6po92X47EZbjaOPwrtVoTU46tJ244uzTs1o1fVFt7RbK5btHCMsRejiaaap4imlfidlJPq0bu9tHzmrsr/Ntg8/y2U5UaPUyguq1KGsmm2knDq9+Ju10ueXEGnQY7ZOIaTYQTZprRKfc7T6tiZJBa6KxpvmvYMsJWzLRMiW94FYmQbR5dtDho1cNOMMRZurhZSXJINWTaWjcdVaS015j0WVKJwmLxOAxNPGYOo6Vak96E48affmuY09Gid5dwo02lHN8G00nephmneV9FuTasrcb3nr09IVJq57DOCL5u9Yx8NX9VXV0eOwMpxEOIJC+kbx2bZO9PBa5TsEZ8HE2Z6idSd+tyTzrcjfJOrW4/GPi16txdHQw2b8JznTdLI8O6bkta+Is5RumuVhFtXWjTba5jRHZQqQ8yvCLcJsCtY9f1XAZfmkNdZMBhv3GeKQwHPkpBtdtPQ2fwUqVOV8fXg1QgrXhe65LK6asnxJ8b057VRGQwuAzraHFTlh6dbG1m4qpVk3Kzs93fnJ2WkWld8zQnGRcG+Gwk4YnO6qxNSLusPT8YtL9WbSlJcTtZc53RZMMCrmEOdN5tIGE71ZiGetTpLayuppDYkKEWQWzawusY0YyXY3GyYE8SiWRbI5xnrp1qNPkWEnNxliZ2UUlxtRupS5ytpfS61tamUZPgMiwnULLouMG96cpScpTnuqLk78V91aKy6B26dOnSpxpUoxhTglGEIq0YpKySS0SORXUmmRKSZGxowAev3tbTVNRUaqhfNy8UgTe4Czew0Yhweah66+Iw+FoyxGKqwo0oW3qlSSjFXdlduy43Y9nGVlt3tX4KdfwSssr72Bp25LKKsqtRN8273oKytxJvXWyZhRqO6kRA0YMZ3oLnras4VVUYxX2uNjGztc74Qxqy6dSnVpwq0pKcJxUoTi7xlFq6aa0aItwhZH4KOV+ClhqcXiMHy1Sd7SdBKTkujZ62fEr21dnw4Oc7eOyyeVYid6+CtyPeesqL4rXk2916cVkt1EsnTp1oSo1YxnCpFxlCSTjJPRpp6Nc9Hk39DpGa06Y+uFi0wa9qy3dMZmYb14z52tcFQoO1meBqZZmOJy+pduhUlBSlFxcop8rKzvZNWa6DOqbCCHAEYDaurXsdDe5jhJzSQRvRFhCAA8rFAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEX//06U4LsvShjc2kldtYam7u6tac01xc2Fn0Djwo4/uxyqE+LexFWnbn8rTle3X1ZPp8wkexmC6g7M4KDUFOtB15uC6tyVuUW9E21FpPpW4iD8JGJp19pHRgpKWGoU6U72s5NyqaavS1Rc7UqYJyasHOwht9LQyoW709uq+5iFCEmmIIYdiJLzkhGfZLOsUWMps/tBjdnsasVhXv05WVeg3aNSK5nNs1fR8zoq6eLBaPY2I0tcJg4QtMgxolHiNiwnFr2mYIwgq8crzXBZ1goY/AT3qctJRekoSXHGS1s1f61XTTO2Uvs/tBjdncasVhXvU52Veg3aNSK5nNs1fR8zoptO3MqzXBZ1goY/AT3qctJRfVoSXHGS5jV/rVpZlFS6I6jOmLWHAfXFdkVHXkOtYd4+TY7Rlm4iObm5m9jEu4ACIrpdSvlGUYqtLEYrA4atVlbeqVKMJSdkkruUXzFYwuK4PdmMRBQpUauGad9+lUk5NWencRzVuyuSUHIyNFh7pe4ZxKjR6vodJ42wIb8NpYJ24bZTtUR8GxyDzsYzvqn+JGVwux2zGDqOpSy+nKTW73FcqsbXT6rUlJJ6cfGZkGTqTHeJGI7TlrlxQqoq6Ab5lGhA72WBx0JzkvXQoUMLSjh8LShRpRvu06cVGKu7uyVlxu57ADiw2qcAGgACQFgAsEkAPXXr0cLQq4rES3aVGEqlSVm7Rirt2V29FzBhQkNBJMgLSTgko7t1tF4I2WdRMJW3MdirKO5K06dPyVU4na9t1cT1unoVSZDPs4r57mlbMK10pvdpQbbUKa6rFavpu3NbfNMebBRKOKPCA1o2uz960F1dXlZurOmOeDwrZNsMYr0HDLe3YdIYllNms1lk2dYXG7+5S31Cu3vNcim7Tuo6uy5ZLXVLRl0PjKDLq2cxix+QYDFKcqjlQhGc5X3nOC3Ztt6t7yevNIdawxlIgzWnXj16v7i6USI9GJsF7EaJ282us0lBOEvL+o+dUsfCFoYykt6e9feqU+Vlpe6tFw5iT6dyIFj8KOFjPL8Djt+zo1pUty3VuSx3t699Lcita2t+hrXBLoL7+jMnimNIyHBKjukgCBWscASDi14wa00EmzfU0ABKVOgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACL/1IVg8NTwWDw+CpOThh6UKUHKzk4wSir2SV9CqNu3favHPsLtGmW8+Psl34qHbxW2rxy7C7RplLVZnSHE42HXhb/dg0Mq2E1tgEdgGcGPksAAC6WgIZbZvP8AE7P5jDE0pPkE3GOJpJXU6d9dLpbyu3F3WvQbMSDF7GxGlrhMHCuSBHiUaK2LCcWuaQQQr2wmLw2Pw1PGYOoqtGqt6E48TXf01xNPVc09xXHBpnFSjjqmSVZxVHEKVWlFxe860VG6TS4nCLbvpppq9bHNepMA0eKWYRhBzCu06prFtaUNlIAk61rwMAeMOhbMZhQAHCp6AAIgACIRPhJzFYXI4YCLW/jaiTi02+R0mptprRNS3VrzGSwrrhSxSnj8DgVCzo0ZVXO+j5LJR3bW0tyLjvrfmW1k0Fl/SWTxTOkLODVRdHHNHqqOQZFwDB2eQHeKzUIABsC6wQtng/xFOtsvh6dN3eHqVadRWeknOU7dHSaKmLO4MesDELvMn2nSINZidHnvTgdeFsdyDyysyBLLQng6Yd65OE7rAw/e5DtOqViWdwnPug4dd5cO06pWJ5q3duN/FYXWbyjuA4euQAE1a+gACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACL/9WIN316BWHCZThDaGnKMVGVTCwlNpJOT36iu+e7JLpIsLJcXLH5PgsbUqRq1K1CnKrOO7Z1HFb/AFXRNO6a5j0Izwn4OtXyzB42MpShhas4ygk2lyZRvNu9o604x6N0UNBdkVKDTvppz9iF2TdEzUyp3xGCchDijOsnpAkqtgAXy62QABFJOD6hVrbU4apTV40I1alR3StFwlC+r11mloWwVzwXYXfzDG47e0o0Y0t23HyWW8nfoci+JLGKOsnX1II5taB6/wBeuxrkoJhVWHc5IkR2lJnsKAAhLYEAARAAEQqvhGxSxG0tSiobvUWlTpN3vvXTqX4lbxktbXiv0C1CquEXC9R9palbe3upVKnVta27ZOnbjd/GO/M4+zJ1WS1IM+bTLPmPXLXLr7/VYL3BkzL7BumTvXyUYABdrrxC0uDahVo7OTqVI2jXxM6lN3TvFRjBvR6ctBrUq0uPY7CzwmzOX0aji5SpureN7WqydSK1S1Snr0SBWjpQAN7cOCBK2W4+Ff1i99smQXHMmSABpEqNcKeJ6zsHGpxKrUqUlLrqhJx76SfT6JASQ7eZjHMdo66ptOnhUsPFpNPlLuad+apSktNLLsyPHPQ2ZHR2A4ZT07VXV9SG0mtKREbgv70WzGUAZPRkgAJCq0AARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARf/9apODfHrE5FPBScd/B1ZJRV78jqcum+nJyWnOJDm2W0s4y3EZZXdo14WUtXuyWsJWTjezSdr6lZ7AZsstz6FCrJqjjVyCSu7KbfcN7qTu78qudvPUtcoacwwaSXCyZDgc3Yrsm56kQ6wqpsJ8nXjTBe042ykNAtMlQ9ehVwtephq8d2pSnKE46O0ouzWl1xo9ZOeErI40a0NoKUopYiUaFanrvOooycZrjVt2FmtLWXHd2gxcwIwjww8Y8OYca0KsqC+rqXEo7rb05U7207pOiEAByqGrK4L8PSjlGLxUY9xKmJ5HOV3rGEIyircWjnL3cmRGeDvCrD7MwqqV+pNapVa51nyO3xnckxrtLN9SIh30RpWLtSo4eRVXRWylOGHWb6y09GaAA4FZIAAiAAIhW/CjhpwzTB4x25HVw/I4rm71OTlK/Q7iKxZBB+FLCznhMvxqa3KVSpSkua5VEpK2lrWpu/ZEqr3XtJZmzHBKlumhZJVMeyZbeOGg8T4IlV2AC/XWa7GAwVfMsbRwGGV6teahHjsr8cnZN2S1b5iLnxdfDZDk1StGKVHA4e1OnKVk9yNoQ3nfV6JPXXnkK4M8mqvEVs8rwtThB0sO5RT3pyfLSi27qyW7e2t2r6NHu4Tc4qQWHyOk3GM4rEV3qlJXcYR0eqvFtprjSaKulHUqlMgjdLcPr+CW5VO3VNU8esHiT4shDBFssDDbiJJOaAFAalSpVqSq1ZOc5tylKTbcm3dtt6tnEAtFppJJmUAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEX//X1WhOdKcalOThODUoyi7NNappriZcuy+bPO8jw2NqSTrJOnXs03ySGjbSSSclaVraJlMEg2N2j7d/Mu5iVsHibRxNo7zW6pbklxPRvW19G9G7ESnUfJ4U2jLNtGaMYV5c5Wgq6mXsR0oUXKutsadZfoYDmEq1sZhMNj8LUwWMpqrRrR3ZxfxD6DXGnzGU5tBkGN2exzwmK5aEryo1kuVqR5/Ns+euZ0VZu56dSnVpxq0ZKdOaUoTi01KL1TTWjRjtoMgwe0OBeFxK3asLuhWS5anJ9/i+aub07NVdDpRoz5O3QcI3rNW4V9U7a1o99DlkzBwrM5BwwlpO9HFvRzCVSwO5muVY3JcbPAY+G5UhqmtYzi+KUXpdP9R63R0y+a4OAIMwcBXWsSG+E9zHtLXNJBBEiCMSt3YTxqmB9nu1qhnzAbCeNTwPs92tUM+a5SON8Tf7teu2Kq3jqJ1jwfOAgAOJTEAARAAEQw22GAp5hs3jqc7J0abxEJOKluuly7txWbScb85mZCMmPMN7XDCCDpLipEFtJgxILsD2OaezhJUGdzKsqxuc42GAwEN+pPVt6RhFccpPWyV/rFrZHsz/ACvwRs4xWW729GjPlHe73JJShd2jraSvpxnu2Zzx7P5tTx7i50mnTrwja8qcrXtfmppPmXta6ubG57nQi+HaS2bc2yxdUQYMOHTGwaWSxrYl5EIwiRk7SVp43FZbsrkrqRjClQw0N2hRvbklSzcYJ2bbk+N2fNb5rKgzLMcTm2OrZhi2nVrSvLdVkrJJJdBJJIy+1+1MtosVCOG5JTwVFLkdKdk3PW85KLavrZavTnXZHiPQaMYLS9+63Yd7A3r4atboq3bTooo9HPDPCkGgCTS4CV9LegLBmZ6AAmKgQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARf/Q1UAARTPYTa6llndGzOW7hqk3KjXk3alKVrxld2UG9bribbejurJtYoMl+ym3dfLFRyzNe4uBjeMatm6tJO27zeWguda9npxJFZTaCXkxYQt1ob3mjNW3XPXRto7W0SmGTBIQ4nNu+XZm9HFnYLBzXKsFnWCngMfDepy1jJaShJcUovmNX+sel0VZtFshmWz9RzaeJwlk1iYQaitUrTV3uO7SV3rzNbpW7TnTq041qUozpzSlCcWnGSaummtGjlcg0alxKMZC1uNp/WwrYq1qSi1uwOdlIgGViNEzLeiJgOH6grAbCeNUwPs72tUM+enC4TC4Km6OEpxo03Le5HDSEXaz3Y8UVzbK2t3xtnuOKK8RIjnjWnE6Zmp9DgmjUWDBcQTDhsYSMBvQBPRkgAMFzoAAiAAIgACKDcJ2VSqUcLnNGF+RXoV5LebUW7021rFRTck3prJLXmV4XhnGAwuaZXisDjaipUalPlqsnZU93llUd5QVotJ6tLTXQo8uqsi38EsOFh4I2j166+uuoYo9ObHbKUZszv5sg6zNEjnzQAE9a0gACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIgACIAAiAAIv/0dVAAEQABFlsj2mzbZ+UuoFROlN706FRb1OTta9rpp9Jq9le5YGTbf5JmlqWMfgn13zKsr0n1Z6VNEtFrvW1dlcqkEaPQ4Me0iTubhYdHe1bVbX1Oq2TGOv4Y5NvtboHCNAyzCr8tzQUnlef5xk28stxU6MZXvDSULu13uyUo35Va2uSzLuFGqmoZtgoyTbvUw7cWo205Sbd3fm7y/BrYtWxmWsk8Zlh0j8NbbQ7raBSJNjB0Fx3vLst30PXgKwAY7Is9we0GDljsHCrTpwqypNVVFS3oxjLyTKStaSMjoQnNcxxa4SIwhbBBiw48NsSG4Oa4TBGAhAeDzoYrNAerF4mlgsJXxtVSlDD0p1ZqKV3GEXJpXaV9NCHYvhRy+G71BwNare+9yacaVuK1t3kt+bzjlhQIsbjW0nSGvUOmVlQ6vlqTFDJiYEiSROVgaCVNjG5xtFlGRR7qFdRqOLlCjBb1SXHayXFe1k3ZX5pW+ZbebR5jF01XjhabSTjhluap3vvNymnzHZpW7MjpPg1W42xXSzG2nTWt067KGAW0OEXHm+JYBnNFp0SM5SzaTb/ABecYeeAwFJ4TDTbU5b16lSGqSdtIprqyV+de17xMAsoUGHBbesEgtSplOpNYRclpDy90pCwAAb0AJAIADkUZAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARAAEQABEAARf/Z</t>
+        </is>
+      </c>
       <c r="N47" t="inlineStr">
         <is>
           <t>Protection &amp; Social Work</t>
@@ -4590,7 +4706,11 @@
           <t>Mercy Corps</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQEAkACQAAD/2wBDAAgGBgcGBQgHBwcJCQgKDBQNDAsLDBkSEw8UHRofHh0aHBwgJC4nICIsIxwcKDcpLDAxNDQ0Hyc5PTgyPC4zNDL/2wBDAQkJCQwLDBgNDRgyIRwhMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjIyMjL/wAARCABoASUDASIAAhEBAxEB/8QAHwAAAQUBAQEBAQEAAAAAAAAAAAECAwQFBgcICQoL/8QAtRAAAgEDAwIEAwUFBAQAAAF9AQIDAAQRBRIhMUEGE1FhByJxFDKBkaEII0KxwRVS0fAkM2JyggkKFhcYGRolJicoKSo0NTY3ODk6Q0RFRkdISUpTVFVWV1hZWmNkZWZnaGlqc3R1dnd4eXqDhIWGh4iJipKTlJWWl5iZmqKjpKWmp6ipqrKztLW2t7i5usLDxMXGx8jJytLT1NXW19jZ2uHi4+Tl5ufo6erx8vP09fb3+Pn6/8QAHwEAAwEBAQEBAQEBAQAAAAAAAAECAwQFBgcICQoL/8QAtREAAgECBAQDBAcFBAQAAQJ3AAECAxEEBSExBhJBUQdhcRMiMoEIFEKRobHBCSMzUvAVYnLRChYkNOEl8RcYGRomJygpKjU2Nzg5OkNERUZHSElKU1RVVldYWVpjZGVmZ2hpanN0dXZ3eHl6goOEhYaHiImKkpOUlZaXmJmaoqOkpaanqKmqsrO0tba3uLm6wsPExcbHyMnK0tPU1dbX2Nna4uPk5ebn6Onq8vP09fb3+Pn6/9oADAMBAAIRAxEAPwD3+vP/ABjqd7rWqN4c0aZke2ia6upUPIKjKJ+e38x6V1PifW08P6Bc6g2C6LtiU/xOeAP6/QGub+GGlyRaPcazdkvd6jIXLt1KAn+ZyfyrObu+VHpYOCo0pYuS20j5v/gLU6PwvraeIPD1rfjHmMu2ZR/C44P+P0IrYry/wZef8I/481bw3IdtvPKzQA9mHI/NT+gr1CnCV1qZZhh1QrNR+F6r0f8AVgoqC8u7ewtJbq6lWKCJdzux4Arh7T4saRc6oLaS1ngt2batwxGPqw7D86bnGO7M6GDr14uVKLaW539FHUZFFUcwUUVm6nr+k6OudQv4IDjOxmyx+ijk0N23KhCU3yxV2aVFedal8W9OiYxaXYz3bk4DP+7Un26k/kKdZ3nxB8REOiW2jWrfxvF8+PZWyf5Vn7SOy1O/+y68Y89W0F/edvw3/A9DorM0bS7jTYHF1ql1fzPgs8xAA/3VHStOrRwTSjJqLuu4UVzVz4+8NWl1NbT6jtmhdo3XynOGBwR09aksPHHh3Ur6KztNQDzynaimNxk/UjFLnj3N3g8Qo8zpu3ozoaKKyNY8T6RoEkUepXYheUFkGxmyB9AabaW5jTpzqS5YK78jXorlf+FjeFf+gn/5Bf8A+Jrf/tO0/sn+1PN/0PyfP8zafuYznHXpSUk9maVMNWp254NX7pluiuV/4WN4V/6Cf/kF/wD4mj/hY3hX/oJ/+QX/APiaOePc0+oYr/n3L7mdVRXPaf438PapfRWVnf8AmXEpwieU4zxnqR7VZ1jxRo+gzRw6ld+Q8i7lHls2RnHYGjmja9zN4Wupqm4PmfSzubFFcr/wsbwr/wBBP/yC/wD8TUkXxB8LTOFGrRqT/fjdR+ZFHPHuW8DilvTl9zOmoqK2uYLyBZ7aaOaJvuvGwZT+IqWqOZpp2YUVV1DU7HSrc3F/dRW8X96RsZ9h6n6Vydx8VfDcEhVGu5wP4ooeP/HiKlyit2b0cJXr60oN/I7aiuPsfib4avZAjXMtsT08+PA/MZArqhdQPafao5BLDtLh4vnDD2x1/ChST2YquGrUXapFr1RNRXK/8LG8K/8AQT/8gv8A/E1taRrmna7bNcabcrPGjbGIBBB9weaFKL2YVMLXpx5pwaXmmaFFFczN8QfDFvPJDJqY3xsVbETkZHuBg03JLcmlQq1dKcW/RXOmornrXxvoN9v+yXUs+zG7y7aQ4z0z8vsaKXNHuU8LXi7OD+5nFfE+8l1XxBpfh22bncrMP9tzhc/Qc/jXqFnaxWNlBaQrtihjWNB7AYFeTaIf7c+Ml1dN8yW8srj6INi/0r1+op6tyPRzP91To4ZdI3fqzxf4lrLpPjq21K3O2R445lb/AGlJH/sor13S9Qi1XSrW/g/1c8YcD0z1H4HivOvjFaZttLvAPuu8RP1AI/kas/CPV/tGlXWlSNlrZ/MjB/uN1H4H/wBCqYvlqOPc6sVS+sZXSrreGj9L2/yD4vtdDRrARlhamY+bjoWx8uf/AB6vMvD+h3XiHV4bC2U/McyPjiNO7Gvo66tLe+tntrqGOaFxhkkXINU7PTdJ8PWkrWtvb2UAG+RxwMDuSaJ0uaV29CMFnP1bC+whH3tbP1L8UYhhSJc7UUKM+1c94i8b6P4dDRzTefdjpbw8sP8AePRfxrhPF/xNmuzJY6E7Q2/R7ro7/wC7/dHv1+leeQQXF9dJDDHJPcSthVUZZiaU69tIm+ByFzXtcU7Lt1+fb+tjrNc+JeuasWjtpBYW5/ggPzke79fyxT/Dnw81bxEy3l67Wlo/zebKCZJPoD/M/rXZeDvhvb6WI77WFS4vfvLCeUi/+KP6fzr0GiNJy1mGKzajhk6OAil5/wCXf1ZhaH4Q0Xw+oNnaKZwOZ5fmc/j2/DFaepX0em6Zc30xxHBE0h98DOKtV5r8WPEAgsYdDgf95PiSfB6IDwPxPP4e9ayahG6PHw1OrjsTGM223u/LqdJ4Au577wda3Vw5eWWSZ2Y98yNXTVg+C7X7H4N0qIjBMAkP/Avm/rW9Th8KMsY08RUcdrv8z5q8Sf8AI06v/wBfs3/oZqpYXb6fqNteRH54JVkX6g5q34k/5GnV/wDr9m/9DNUZLd44IZiPklztP0OD/SuB7n6NSSdGMX1S/I+nredLq1iuIjmOVA6n1BGRXhPxI1P+0fGV0qtmO1At1/D73/jxNei+B9fQ/Dv7VM2TpySI/PZBlf0IFeLfvtSv3Y/NNM7SMffkk/zrorTvFeZ83kmD9jiaspfY0/r5L8StXvX/ADSUf9gcf+iq8Fr3r/mko/7A4/8ARVRR6nXnv/Ln/EeC1uW/g7xDd20VxBpU8kMqh0cYwykZB61h161ovxQ0bTtDsLGa2vWkt7dImKouCVUA4+aogot+8z0MfXxNKKeHhzPqYfgzwnr2n+LtPurvTJ4oI3Yu7YwPlI9atfGH/kNad/17n/0Ku00D4gaX4i1RdPtLe6SVkL5lVQMD6E1xfxh/5DWnf9e5/wDQq2lGKpvlZ4mGr4itmcHiI8rSen3nC6Vo99rd4bTT4POnCF9u4DgY55PvT9V0HVNEdF1Kylt9/wB0sMq30I4rqPhOQPGD5IH+iP8AzWut+K+o2H/COx2Rmje7adXSMMCygA5J9B2/Gs1TThzHpVsxq08fHDKN4u3qcF4F8S3Gg69BH5h+xXMgjmjJ454DfUV7R4l1+Dw3ost/MNzD5Yo843ueg/r9BXzzpltJe6raW0QJklmVFx7mu9+L+oPJrFjp4J8uKHzSP9piR/Jf1qqc3GDOXMcBTxGPpLunzei/z2OG1jWr7Xb97y/naSRug/hQeijsKu6Z4P1/V4BPZabK8J+7I5CBvpuIz+FT+BtGi1zxXa21wu63TMsq/wB4L2/E4FfQiqqKFUBVAwABgAUqdLn1ZeZ5r9QcaFGKvb5JHzTquhapokipqNlLb7vuswyrfQjg1veAte1jTNXS2sYJ7y1kb99bIM4H94f3SPXp617dqWmWer2L2d9As0D9VP8AMHsaNP0yy0q2FvYWsVvEP4Y1xn3PqfrWioNSumedVz+FbDunVp3k/u9e/wDW55D8S/Cf9lX/APa9nHizum/eKBxHIf6Hr9c+1YPg7xNL4Y1pLglmtJcJcRjuvqPcdf07177qOn2+qafPY3aB4JlKsP6j3FfO3iLQrjw7rM2n3GTtOY5McSIehH+etRVi4S5kduUYyGNoPC19Wl96/wA0ewePPFkWleGVNjOrXF+uIHQ9EI5cfgePc14Wqs7hVBZmOABySafJPNMkSSSu6xLsjDHIUZJwPQZJrvPhf4Z/tLVTq9ymbazb92COHl7fl1+uKlt1ZHZRo0spwspN36+vZHongnw2vhzw/HDIo+1zfvLg/wC12X8Bx+dFdJRXYkkrI+GrVp1qjqT3Z4/8Jv3/AIn1O5b7xtz/AOPOD/SvYK8d+E7fZvFWoWj8Obdh+KuP8a9irOj8B6me/wC+PtZfkcT8VLfzvBjSY/1NxG/81/8AZq84+HOonTvGloC2EuQbdvfd0/8AHgK9V+IihvAmp57CMj/v4teEafcG01K1uVODDMkgP0INZVnaomevk0Pb5dUpPu1+CPpq4uIbS2kuLiRY4Y1LO7HAUDvXhfjXxvceJLlra3ZotMjb5I+hkP8Aeb+g7VpfEjxidUu20exk/wBCgb96yn/WuO30H8/wrz4DJwKVarf3UVkuVKlFYisveey7f8H8ia1tZ726itraJpZpWCoijkmvdvBfgq28M2gmmCy6lIv7yXHCD+6vt796o/DzwYNEsxqV9H/xMZ1+VWH+pQ9vqe/5etd1WlGlb3nuefnOautJ0KL91bvv/wAD8wooorc+dKWranb6NpdxqF022KFdx9WPYD3J4r55urq78T+JPNlObi9nVVA/hyQAB7AYFdP8SvFY1jUhpdnJmytG+ZgeJJO5+g6D8aPhZohv/ETajIuYLFcgnvI3A/IZP5Vy1Jc81FH2GXYdZfg5Yqp8TX/DL5s9oghW3t44UGEjQIo9gMVJRRXUfHt31Z81eJP+Rp1f/r9m/wDQzW1Npv2j4X2uoKuWtb+RWP8AsuF/qF/OsXxJ/wAjTq//AF+zf+hmvSvBemjV/hXf2OMtK8oT/eABX9QK4YR5pNH3+Lr+ww9Kp2cfutr+B53p2uyWPhzVtLUnF6Y8e20/N+YwK0/Aum/a7jVbxlylnp8zA/7TIVH6bvyrkyCCQRgivXPAum/ZPhvq16y4e8imIP8AsqhA/XdRTXNL0KzKccPQlKO82l99l+SPI696/wCaSj/sDj/0VXgte9f80lH/AGBx/wCiqqj1OTPf+XP+I8FrsrD4Za9qOn297DJZiK4jWVN0pBwRkZ+WuNr0LTPirc6ZpVpYrpUMi20KxBzKQW2jGentUQ5b+8ejj5YtRX1VJvrc2vBPgLWPD3iNL+9e1MIidCI5CTkj6Csv4w/8hrTv+vc/+hVs+Hfibc65r9ppr6ZFEs7FS4lJIwCemPasb4w/8hrTv+vc/wDoVbS5fZvlPDw31p5pB4pJSs9u2p57BBPMszwKx8mPzH29lyBn8yKiHzONzYBPJPau1+FsMdz4pngmQPFJZSI6noQSoIrD8VaBJ4c16exbJizvgc/xIen+B9xWHL7vMe/HFReJlh3ukmv68j1bwT4E0/RhFqrXS31zIm6KVRhEBHVfU471x3xct3j8UW05HyS2qgH3DNkfqPzrS+FvivY//CP3knysS1qzHoepT+o/Gup+IPhl/EWhBrZd17akyRD++P4l/Hj8RXRZSp+6fNRrVcJml8VK99L+T2/4PzPN/hjex2fjOFJCFFxE8Kk/3jgj+WPxr3avlpWltpwyl45Y2yD0ZWB/Q16RpXxeuoLZYtT09bmRRjzo5Nhb6jBGfpipo1FFWZ151ldbEVFWoq+lmj12ivDfE/xI1DX7VrO2hFlat98K+53HoTxx7CpfBvjPxKuo2+mQZ1JJDtEU5OVHc7+oA98itPbxvY8t5BiY0XUk0munl67f1ue215P8XtRspJrLT0jVr2LMjyd0U9F/Hr+A9a9I1vV4ND0e41G5PyQrkLnlm7KPqa+cNQv7jVNQnvrp9007l2P9B7dqVedlymvD+DdSt9Ye0fxYum6fcarqMFjarumncIo/qfYda+j9F0m30PSLfTrYfJCuC2OWbux+prhPhV4a+zWj67cp+9nBS3BHRO7fiePoPevSqKELK7Jz7He2q+wg/dj+f/A/zCiiitzwDxKWX/hE/i08r/JA1ySx7eXKOv4bv0r22vL/AIuaIXitdaiTPl/uJ8ehOVP55H4iuj+H3iNde8PRxyvm9tAIpQTyw/hb8R+oNYU/dk4nvZhH6zhKWLjulyy+X9fiiX4inHgTU/cRj/yItfP9e8fE6YReB7pSeZJI0H/fQP8ASvB6yxHxHscOK2Fk/wC8/wAkFekfDTwd9umXXL+PNvE3+jRsPvuP4voP5/SuR8LaBL4j16CxTIi+/M4/hQdT9ew9zX0TbW8NpbRW8EYjhiUIiDoAOlOjTu+Zk57mLow9hTfvS38l/wAElooorrPiwrz/AOIvjQaTavpGny/6fMuJXU/6lD/7Mf0HPpWh448bQ+G7Q21qyyanKvyL1EQ/vN/Qd68LnnluZ5J55GklkYs7sclie5rnrVbe6j6PJcqdVrEVl7q2Xf8A4H5iQxSXEyQxIzyyMFVVGSxPQV9EeEdAXw54fgsjgzt+8nYd3PX8uB+Fch8NvBTWgTXNSixMwzbRMOUB/jPue1emUUadveYs9zFVpfV6b91b+b/4AUUUV0Hzp5fqfwnuNQ1a8vRq0SC4neUKYSdu5icdfeuy8I+Hn8M6J/Z73C3B81pN6rt644x+FbpIAJJwB1JrktW+JHh7SpWiWeS8lXgrbKGAP+8SB+Waz5YQdz1HicdjoKgveS7JHO6l8JJLvU7q5g1SOGKaVpFjMJO0E5xnNd3Boy23hcaLE4AFobcSY7lcFsfU5rjF+MOml8Npd0E9Q6k/lXSaJ460HXZFht7ow3DdIbgbGP07H8DUw9nf3TfGRzOUI+3i7R8l+Nv1OJ/4U5c/9BmL/vwf/iq9B/sR/wDhDxofnjf9i+y+bt4zs25xWzSMyohZ2CqBkknAAq404x2OPEZlicRy+0lezutEeTf8Kcuf+gzF/wB+D/8AFUf8Kcuf+gzF/wB+D/8AFV1Gq/Ezw9psjRRyy3si8H7MoKj/AIESAfwzWZF8YNJaQCXTrxF/vKVb9MisnGij14YnOpx5knb0Qnh34Yz6Hr9pqT6pHMsDFighIJyCOufetLxp4Gl8V31tcR3yW4hjKFWjLZ5z6it3RfE+keIEzp94kkgGWib5XH/AT/OtetFCDjZbHl1cfjI4hVajtNK2qX5WOE8IfD6bwxrTX8moJcAwtHsWIr1IOc59q1fGXhCLxXZQoJhb3MLZSYru+U9VI/L8qTXPHmj+H9SawvRc+cqhj5cYIwenes7/AIWv4c9L3/vyP8aX7tLlNrZlWqxxSi3Lo7GBF8ILyGVJYtcjSRGDKywEEEdCPmr1G0WdLSJLqRJJ1UCR0XaGPcgdq5S3+J3hieQI11NDnvJCcfpmurtbu3vrdLi1njmhcZV42BB/GnBQXwmWYVcbUS+tJ6bXVv0OZ8S/D/SfEUjXPzWl6es0Q4b/AHl7/Xg1wtx8IdaSQi3vbKVOxYsh/LB/nXpfiLxVp3hhbdtQE2LgsE8pN33cZzz7isL/AIWv4c9L3/vyP8amcabeu51YLE5pCmvYpyj00ucvY/B/UXkBv9Rtoo+4hDO36gCvRvD3hbS/DVuY7GE+Y4/eTScu/wBT6ewrEj+Kfhl2AaW5TPdoTx+Wa6fS9Z07Wrcz6ddx3CDg7Tyv1HUfjThGmn7plj8RmNSNsQmo+lkct488Ma74oe3t7Ke0isYfnKyyMGd/UgKeAOn1NcnZfCPVvtsP226sxa7x5vlOxbb3xletexMwVSzEBQMkntXEat8UtC0+dobZZr51OC0IAT/vo9fwFKcIX5pF4HG490/YYaOi7L9TtYYY7eCOGJAkcahUUdAB0FPrzq2+L+kySBbmwu4VP8SlXx+orttJ1rTtctvtGnXSToPvbeCp9CDyK0jOMtmefiMFiaHvVYNef/BL9FFFUchW1Cwg1TT57G6XdDOhRh/Ue9eCpLqfw/8AFrhf9ZC2CDws8Z/of0P0r6Drk/HfhW38Q6Q04ZIry1QvHK3QqOSre38qyqwurrdHr5TjY0ZujW1hPR/5nD/EPxjZeINH02209yVdvPmU9YyAVCn35b9K87orQ0P+zxrdo2qOUslkDS4UtkDnGB69K5JSc3dn2mHw8MHQ5KabSu/M9m+HHhz+xPD63MyYvL0CR8jlU/hX8ufx9q7KuUPxH8KKmRqfHoIJP/iaytQ+Lei26EWVtc3cnbIEa/mef0rsUoRVrnxFXCY7F1pVJU3d+VvzPQK4Dxf8SLXSkkstIdLm++60o5ji/wDij7dPX0rz/wAQePtb19WhaYWtq3/LGDIyP9o9T/L2rG0jQ9R127Fvp9s8z/xMOFQepPQVjOs3pA9fB5FCkva4xqy6dPmypcXE97dPPPI808rZZmOSxNeo+BPh2Y2i1bXIcMMNBauOnozj+n51veEvh5Y+H9l3eFbvUByHI+SI/wCyPX3P6V2lVTo21kZZnnfPF0cLou/+QUUUV0HzIUUVU1S6NjpF7djrBA8o/wCAqT/SgcYuTUV1PKfiR4zmur2XRNPlKWsJ23DoeZW7r9B09zXCaZpV9rF2trp9s88x52qOg9SegH1qq7tJIzuxZmJJJ7mvdPhnpEWn+EoboIPPvCZZGxzjJCj6Y5/E1xRTqz1Pu8RUhlODSpq729X3f9eR53L8L/E0duZRbwOQM+Wkw3f4frXJS289tdNbyxSRzo20oykMD6Yr6jqmdKsG1H+0Gs4DebQvnFAWwPetZYddGeRQ4kqq/top9raf5nPeALrXptE2a5bSp5ePImm4eRf9odePU9a898feNptavZdOsZSmmxMVJU/68jufb0H416j40v303wfqdzGdriLYpHYsQuf1r51qa0nFKB0ZLh4YmrPGSilrouifVl/SdE1HXLr7Pp1q87jlscBR6kngVu3vw38TWVsZzZpMqjLLDIGYfh1P4Zr13wZosOieGLOFEAlljWWZscs7DJ/Lp+Fb9ONBW1McTxFVjWapRXKu/U+XIJ57K6SaCR4Z4myrKcMpr3bwH4t/4SbTGS52rqFtgSgcBx2YD+fvXCfFfRYdP1u31CBAi3qsZFA43rjJ/EEVlfDm/ex8a2QUnZcboXHqCOP1AqIN058p6GNp0sxwH1iK1Suvluiz8Uv+R1l/64R/yrE0DwvqXiV7hdOWJjAFL+Y+3rnH8jW38Uv+R1l/64R/yrW+Ed3bWtxqxuLiKEMkWDI4XPLetLlUqlmaxrzoZXGrT3UV+hw+taBqXh+5WDUrYxM4yhBDKw9iK6X4Z6/PpviSLT2kJtL07GQnhXx8rD37fj7Vp/FbXdN1IWFnZXEVzLCzvI8TBlXIAxkcZ4/SuY8CWUl74001Y1JEUvnOfRV5/wAB+NK3LUtEr2jxWXSniI2bT/DZnafGT/U6P/vTfySvNdK0u61rUorCyRXuJc7QzBRwCTyfYV6V8ZP9To/+9N/JK4vwJe22neMbG6vJkhgTzN0jnAGUYD9TTqJOpZmWVzlDK1OCu0pNet2Rax4N13Qrb7TfWRW3BwZEcOB9cHj8areHdcufD2swX1uzbVYCVAeHTuD/AJ616h428b6FP4avLCzu0u7i4XYqxgkLyOSeleNUppQl7rOnAVauLw7+tQtfTa116M9j+KmvSW2iWljayEC/yzsp6xjHH4kj8q8u0LRLrxBq0Wn2mwSOCSznAUDqTXoHxL0a6Hh7RLwIWW0hEM+B93Krgn2yCPxFec6Xql5o2oRX1jL5c8fQ4yCD1BHcU6r9/wB458pglgLUGubX776X/A7PUvhNrNpbGW0uYLwqMmNcox+meD+ddz8ONAfRPDYkuImju7tvMkVhhlHRVP4c/jXMaZ8YJAVTVdNVh3ktmwf++T/jXo+j63p+vWQu9PuBLHnDDoyH0I7Gtqap3vE8XM62Yqh7LEx0vuvy0NCiiitz58K5rx/fnT/BWoOpw8qCFf8AgRwf0zXS1wXxcdl8JW4HRrxAf++HP9Kio7RZ2ZdBVMXTi+6PFK7rQvhnd65oEGpJfxwPMSUikjJBUHAOQe+PSuKtoHurqG3iGZJXCKPcnAr6bsbSOwsLeziGI4I1jX6AYrmo01Ju59bneYVMJGCpO0n+SPHn+EevA/LdWDD13sP/AGWpYPhBq7MPP1CyjX/Z3Mf5CvZKK29hA8B5/jbbr7jz/S/hNo9owe/uJr1h/D/q0P4Dn9a7izsbXT7dbezt4oIV6JGoUVYorSMIx2R52IxlfEP97Jv8vu2CiiiqOYKKKKACqOs2zXuh6hap9+a2kjX6lSP61eooZUZOMlJdD5XIIJBGCK99+HOox3/gyzRWBktswyL6EHj9CK84+InhOXRdWk1G2jJ0+6csCo4jc9VPoM8j8u1c/oHiTUvDd4bjT5QA+BJE4yjj3H9etcUH7Oep91jKMc0walReu6/VM+kqb5iGQx713gbiueceuK8gl+MGpNblYtNtUmx98szD8v8A69cTPruqXOrNqj3swvWOfNRtpHsMdB7VtKvFbHh0OHcTO/tWo/ie6ePLR73wTqkSAlljEmB6KwY/oK+eq968B32uaxoTza4kbQuNsDMmHlXuWHTHpxzzXlfjTwnP4Z1V9qM1hMxMEvYD+6fcfrWdZcyU0ehkdRYepPBzaundW69z2zwxqMWq+GtPu4mB3QqrgfwsBhh+YNa1fO3hvxfqnhiR/sbrJBIcvBKCVJ9R6H6V0158XtUmtjHa2FvbyEY8wsXx7gcfrmtI1421ODE5BifbP2VnFvvt6knxf1KKfU7DT42DPbIzyY7F8YH5Ln8a5z4f2j3fjbTQoyI3MrH0Cgn+eB+Nc9cXE97dPPPI8s8rbmdjksTXs/w28JSaJZPqV9HsvbpQFQ9Y4+uD7nr+ArKN6lS57GJcMuy72Letml5t7/mcP8Uv+R1l/wCuEf8AKuTisp5rK4u403Q27IshH8O7OD9OMfiK6z4pf8jrL/1wj/lWn8KrGDUodesrlN8M0MaOPY7v1qXHmqNGtLEfVsthWtso/mkefWkcM15DHczGCF3CvKF3bB64yM19BeFvCmmeG7QmyJmlmUF7lyCXHbGOgrwjXdHn0LWbjTrj70TfK2Pvr2YfUV6Z8LvFf2m3/sG8k/fRAm2Zj95O6/Udvb6VVFpSszmzyFWthVVoy93druu5D8ZP9To/+9N/JK8ttrW4vJ1gtoZJpmztjjUsxxzwBXqXxk/1Oj/7038krk/hv/yPmnf9tP8A0W1Kor1LGmWVXSytVF0Un9zZlL4X192CjRb/ACfW3Yf0rtfBvw2vf7Qh1DW4hBBCwdLckFpCOmcdB+teu0VtGhFO54mI4gxFWDhFKN+vUjnWFoWS4EZif5WWTG1s8YOfXpXEat8KtEvnaSykmsZG52p86f8AfJ5/I1gfFbxHI15FoduXRItsszcjc3VQPYdfr9Kq6D8V76wtVttTtvtwQYWYPtfHvwQfrxRKpBy5ZFYTL8fToRxGGlZvp5dN9Gc14p8JXvhW7jjuXSaGYExTJwGx1BHY8j861/hZfy2vi9LVWPlXUTo69sgbgf0/U1Q8ZeMZvFlzAfs4t7e3B8tN24knGST+Ara+E+kS3OvyaoyEW9rGVDdi7DGPyz+lYxS9ouU93ESqLLZPF25rP7+n6Hs9FFFdp8EFcx4/0afW/Cc8FshkuImWaNB1YjqB74JoopSV1Y2w9SVKtGcd00eb/DXw7Pf+JVvp4WW2sSWJZcAyfwr9R1/Cvb6KKzopKJ6Od1pVMW1LpZL8wooorU8gKKKKACiiigAooooAKKKKAI57eG6geC4iSWJxhkcZDD3FcBq3wl0y7kaXTbuWyJ58th5iD6cgj8zRRUyhGW504fGV8M70ZW/rsYq/B2+34bVrcJ6iJifyzXSaH8LtH0uVZ7x31CZeQJAFjB/3e/4k0UVKpQXQ6qucY2rHllPTysjuAAAAAAB0AqG8srbULV7W8gSaBxhkcZBoorQ81Np3W555qvwhs5pGk0u/ktgefKlXeo+h4P55rLi+Dt+ZAJtVtlT1SNmP5HFFFZOjB9D1IZ3jYx5ef70jsvDvw+0bw/Itxta7u15E02PlP+yvQfqa6yiitFFRVkcFavVry56srs4rxN8O4PEmstqMmoyQMyKmxYgw4981c8I+C4vCcl28d69z9oCghowu3bn396KKnkjfmtqbSx+JlR9g5e7206B4t8EWfiuS3mkna2nhBXzEQNuX0P0P8zWDafCZLG7iurbXJ45omDowhHBH40UUOnFu7RVLMsVSp+yhP3e1l+qOh8WeD08WRWaTXrQG23HKR53Fse/HSsvw98NYPD+uW+ppqUkzQ7sI0QAOVI6596KKHCLd7akwzDEwo+wjL3ddNOu53VFFFWcZj6/4Y0vxJbiK/gy6j5JkOHT6H+h4rz67+Ds4kJs9WjZOwmiII/EE0UVEqcZbo7sNmWKwy5actO25Pp3weRZVbUtULoOsdumM/wDAj/hXpGnadaaVZR2djAsMEY+VV/mfU+9FFEYRjsTisfiMV/FldduhaoooqzjP/9k=</t>
+        </is>
+      </c>
       <c r="N48" t="inlineStr">
         <is>
           <t>Finance &amp; Accounting</t>
@@ -4742,7 +4862,11 @@
           <t>MRCS</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAnAAAABKCAYAAAA7bWlBAAAACXBIWXMAAA7EAAAOxAGVKw4bAAABfElEQVR4nO3OoQ3AQBAEseu/6U8Ni0aRDMx9d/cAAPiVPAAAwCYPAACwyQMAAGzyAAAAmzwAAMAmDwAAsMkDAABs8gAAAJs8AADAJg8AALDJAwAAbPIAAACbPAAAwCYPAACwyQMAAGzyAAAAmzwAAMAmDwAAsMkDAABs8gAAAJs8AADAJg8AALDJAwAAbPIAAACbPAAAwCYPAACwyQMAAGzyAAAAmzwAAMAmDwAAsMkDAABs8gAAAJs8AADAJg8AALDJAwAAbPIAAACbPAAAwCYPAACwyQMAAGzyAAAAmzwAAMAmDwAAsMkDAABs8gAAAJs8AADAJg8AALDJAwAAbPIAAACbPAAAwCYPAACwyQMAAGzyAAAAmzwAAMAmDwAAsMkDAABs8gAAAJs8AADAJg8AALDJAwAAbPIAAACbPAAAwCYPAACwyQMAAGzyAAAAmzwAAMAmDwAAsMkDAABs8gAAAJs8AADAJg8AALDJAwAAbPIAAACbPAAAwOAD/Hy2Hkw3IYQAAAAASUVORK5CYII=</t>
+        </is>
+      </c>
       <c r="N50" t="inlineStr">
         <is>
           <t>Logistics &amp; Supply Chain</t>
@@ -4830,7 +4954,11 @@
           <t>MRCS</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAnAAAABKCAYAAAA7bWlBAAAACXBIWXMAAA7EAAAOxAGVKw4bAAABfElEQVR4nO3OoQ3AQBAEseu/6U8Ni0aRDMx9d/cAAPiVPAAAwCYPAACwyQMAAGzyAAAAmzwAAMAmDwAAsMkDAABs8gAAAJs8AADAJg8AALDJAwAAbPIAAACbPAAAwCYPAACwyQMAAGzyAAAAmzwAAMAmDwAAsMkDAABs8gAAAJs8AADAJg8AALDJAwAAbPIAAACbPAAAwCYPAACwyQMAAGzyAAAAmzwAAMAmDwAAsMkDAABs8gAAAJs8AADAJg8AALDJAwAAbPIAAACbPAAAwCYPAACwyQMAAGzyAAAAmzwAAMAmDwAAsMkDAABs8gAAAJs8AADAJg8AALDJAwAAbPIAAACbPAAAwCYPAACwyQMAAGzyAAAAmzwAAMAmDwAAsMkDAABs8gAAAJs8AADAJg8AALDJAwAAbPIAAACbPAAAwCYPAACwyQMAAGzyAAAAmzwAAMAmDwAAsMkDAABs8gAAAJs8AADAJg8AALDJAwAAbPIAAACbPAAAwOAD/Hy2Hkw3IYQAAAAASUVORK5CYII=</t>
+        </is>
+      </c>
       <c r="N51" t="inlineStr">
         <is>
           <t>Administration &amp; Operations</t>

</xml_diff>

<commit_message>
chore: update jobs data [2026-06-17 10:18 UTC]
</commit_message>
<xml_diff>
--- a/mimu_jobs.xlsx
+++ b/mimu_jobs.xlsx
@@ -1399,7 +1399,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve">“Our vision for every child, life in all its fullness; Our prayer for every heart, the will to make it so” World Vision is a Christian, relief, development and advocacy organization working for/ with communities to create lasting change in the lives of children and families living in poverty. Inspired by our Christian values, we are dedicated to work with the world’s most vulnerable people regardless of religion, race, Vacancy Title Field Officer (Pool PNS), Myanmar Earthquake Recovery Program https://worldvision.wd1.myworkdayjobs.com/WorldVisionInternational/job/MandalayMyanmar/Field-Officer--Pool- WV has zero tolerance towards incidents of violence or abuse against children or adults, including sexual exploitation or abuse, committed either by employees or others affiliated with our work. WV is committed to continuous improvement of safeguarding efforts which emphasizes Protection from Sexual Exploitation and Abuse (PSEA) and other forms of violence or harm. We abhor any misuse of power, status, or trusted position for any sexual or other exploitative purposes. Thus, every staff of World Vision is required to adhere to the Code of Conduct and Safeguarding policy which includes World Vision does not tolerate harassment. In alignment with WV’s core value; “We Value People”, WV promotes the culture of dignity, respect and courtesy for everyone. WV is committed to preventing harassment and abuse in Applications received from the WV Careers Website are considered valid and will </t>
+          <t>“Our vision for every child, life in all its fullness; Our prayer for every heart, the will to make it so” World Vision is a Christian, relief, development and advocacy organization working for/ with communities to create lasting change in the lives of children and families living in poverty. Inspired by our Christian values, we are dedicated to work with the world’s most vulnerable people regardless of religion, race, Vacancy Title Field Officer (Pool PNS), Myanmar Earthquake Recovery Program https://worldvision.wd1.myworkdayjobs.com/WorldVisionInternational/job/MandalayMyanmar/Field-Officer--Pool- WV has zero tolerance towards incidents of violence or abuse against children or adults, including sexual exploitation or abuse, committed either by employees or others affiliated with our work. WV is committed to continuous improvement of safeguarding efforts which emphasizes Protection from Sexual Exploitation and Abuse (PSEA) and other forms of violence or harm. We abhor any misuse of power, status, or trusted position for any sexual or other exploitative purposes. Thus, every staff of World Vision is required to adhere to the Code of Conduct and Safeguarding policy which includes World Vision does not tolerate harassment. In alignment with WV’s core value; “We Value People”, WV promotes the culture of dignity, respect and courtesy for everyone. WV is committed to preventing harassment and abuse in Applications received from the WV Careers Website are considered valid and will</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2425,8 +2425,7 @@
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
-          <t>International Rescue Committee Who we are The International Rescue Committee (IRC) works in more than 40 countries and in 30 U.S. cities to help people affected by humanitarian crises to survive, recover and rebuild their lives. Watch our video 4 reasons to give to the IRC What is the IRC The International Rescue Committee responds to the world's worst humanitarian crises, including the conflict in Ukraine and the crisis in Afghanistan . We help to restore health , safety , education , economic wellbeing and power to people devastated by conflict and disaster. And we are proud to fight for a world where women and girls have an equal chance to succeed. Learn more about the IRC’s work from IRC Ambassadors including Rami Malek, Kingsley Ben-Adir, Morena Baccarin, Sepideh Moafi and Ebony Obsidian. To view this video please enable JavaScript, and consider upgrading to a
-      web browser that supports HTML5 video The IRC at a glance IRC President David Miliband Senior Staff Board &amp; Advisors</t>
+          <t>International Rescue Committee Who we are The International Rescue Committee (IRC) works in more than 40 countries and in 30 U.S. cities to help people affected by humanitarian crises to survive, recover and rebuild their lives. Watch our video 4 reasons to give to the IRC What is the IRC The International Rescue Committee responds to the world's worst humanitarian crises, including the conflict in Ukraine and the crisis in Afghanistan . We help to restore health , safety , education , economic wellbeing and power to people devastated by conflict and disaster. And we are proud to fight for a world where women and girls have an equal chance to succeed. Learn more about the IRC’s work from IRC Ambassadors including Rami Malek, Kingsley Ben-Adir, Morena Baccarin, Sepideh Moafi and Ebony Obsidian. To view this video please enable JavaScript, and consider upgrading to a web browser that supports HTML5 video The IRC at a glance IRC President David Miliband Senior Staff Board &amp; Advisors</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -3892,7 +3891,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sun Community Health is seeking Data Assistant to engage in TB team activities by: 1. Taking responsible for document and report preparation for TB team activities. 2. Assisting Medical Doctor (Team leader) and Medical Assistant for planning and implementing TB team activities in accordance with work plan and to achieve the targeted number of assigned projects. 3. Assisting Medical Doctor (Team Leader) and Medical Assistant to provide Tb services according to guidelines and in line with project objective. 4. Ensure to prepare adequate stock of all essential items as per team schedule. 5. Assisting Medical Doctor (Team Leader) and Medical Assistant for reporting and recording. 6. Conducting health education session and responsible for provision of counselling services for TB and related diseases. 7. Performing any other additional duties as required. Term of Agreement The Contractor will receive the basic daily service payment upon submission of a complete Daily Work Report to the respective Supervisor and payment will be made within 30 days after SCH receives and accepts the report. In addition, the Contractor may be eligible for a performance-based payment, which will be determined based on the verification of achievements against the Monthly or Quarterly Performance Indicator Report and the appraisal and approval of the respective Supervisor. Qualifications and Skills ➢ Any graduate and must have certificate of nurse aid training. ➢ Preferably relevant work experiences for </t>
+          <t>Sun Community Health is seeking Data Assistant to engage in TB team activities by: 1. Taking responsible for document and report preparation for TB team activities. 2. Assisting Medical Doctor (Team leader) and Medical Assistant for planning and implementing TB team activities in accordance with work plan and to achieve the targeted number of assigned projects. 3. Assisting Medical Doctor (Team Leader) and Medical Assistant to provide Tb services according to guidelines and in line with project objective. 4. Ensure to prepare adequate stock of all essential items as per team schedule. 5. Assisting Medical Doctor (Team Leader) and Medical Assistant for reporting and recording. 6. Conducting health education session and responsible for provision of counselling services for TB and related diseases. 7. Performing any other additional duties as required. Term of Agreement The Contractor will receive the basic daily service payment upon submission of a complete Daily Work Report to the respective Supervisor and payment will be made within 30 days after SCH receives and accepts the report. In addition, the Contractor may be eligible for a performance-based payment, which will be determined based on the verification of achievements against the Monthly or Quarterly Performance Indicator Report and the appraisal and approval of the respective Supervisor. Qualifications and Skills ➢ Any graduate and must have certificate of nurse aid training. ➢ Preferably relevant work experiences for</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -4068,7 +4067,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sun Community Health is seeking Team Leader to engage in TB Control activities by: 1. Co-operate with Sun Providers, health and local administrative authorities and SCH implementation team for planning, implementation, training, management and supervision of TB control activities. 2. Ensure to operate TB team activities in accordance with work plan and to achieve the targeted number of assigned projects. 3. Provide TB services according to guidelines and in line with project objective. 4. Supervise team members during field operation. 5. Take financial accountability and responsibility for team’s activities according to organization rules and regulations. 6. Provide project consumption of necessary stocks as per schedules in monthly basis and report to respective supervisor. 7. Analyze data regularly and take timely, corrective actions. 8. Review, check data and submit reports timely to respective units and supervisors by using standardized format. 9. Organize quarterly review meetings in respective project township and participate in the project review meetings if necessary. 10. Regular monitoring/supportive visit to all assigned Sun clinics in assigned area to distribute social franchising products, to deliver new updated forms, to collect MCRs, financial transaction of provider’s incentive payment, Clinic assistance fees and client’s incentive. 11. Assist Sun providers to meet social franchising and clinical practice minimum criteria 12. Conducting advocacy, area mapping, </t>
+          <t>Sun Community Health is seeking Team Leader to engage in TB Control activities by: 1. Co-operate with Sun Providers, health and local administrative authorities and SCH implementation team for planning, implementation, training, management and supervision of TB control activities. 2. Ensure to operate TB team activities in accordance with work plan and to achieve the targeted number of assigned projects. 3. Provide TB services according to guidelines and in line with project objective. 4. Supervise team members during field operation. 5. Take financial accountability and responsibility for team’s activities according to organization rules and regulations. 6. Provide project consumption of necessary stocks as per schedules in monthly basis and report to respective supervisor. 7. Analyze data regularly and take timely, corrective actions. 8. Review, check data and submit reports timely to respective units and supervisors by using standardized format. 9. Organize quarterly review meetings in respective project township and participate in the project review meetings if necessary. 10. Regular monitoring/supportive visit to all assigned Sun clinics in assigned area to distribute social franchising products, to deliver new updated forms, to collect MCRs, financial transaction of provider’s incentive payment, Clinic assistance fees and client’s incentive. 11. Assist Sun providers to meet social franchising and clinical practice minimum criteria 12. Conducting advocacy, area mapping,</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -4848,7 +4847,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Procurement 1. Carry out logistics and procurement processes under MRCS programmes in accordance with MRCS and donor standard procurement guidelines. 2. Maintain an updated local supplier database for frequently purchased items, monitor local market trends, and ensure all procured goods meet required quality standards and, where applicable, include proper certification. 3. Prepare and regularly update the procurement plan in coordination with the project and technical teams. 4. Collect quotations, prepare comparative bid analyses, and submit purchasing recommendations. Upon approval, procure goods and services following standard procedures. 5. Liaise with suppliers and service providers to ensure timely and quality delivery of goods and services in coordination with MRCS procurement and logistics teams. 6. Coordinate with internal stakeholders to ensure the timely delivery of supplies to distribution locations and communicate any delays or changes promptly. Transportation 7. Prepare and share weekly stock position and transportation status reports including logistics movement reports with relevant departments at headquarters. 8. Organize safe and efficient transportation of procured items to the affected people and areas, ensuring compliance with MRCS warehousing procedures before final distribution to affected people. 9. Plan and coordinate transport requirements, including MRCS-owned trucks and third-party trucking service providers and support the Senior Logistics Officer </t>
+          <t>Procurement 1. Carry out logistics and procurement processes under MRCS programmes in accordance with MRCS and donor standard procurement guidelines. 2. Maintain an updated local supplier database for frequently purchased items, monitor local market trends, and ensure all procured goods meet required quality standards and, where applicable, include proper certification. 3. Prepare and regularly update the procurement plan in coordination with the project and technical teams. 4. Collect quotations, prepare comparative bid analyses, and submit purchasing recommendations. Upon approval, procure goods and services following standard procedures. 5. Liaise with suppliers and service providers to ensure timely and quality delivery of goods and services in coordination with MRCS procurement and logistics teams. 6. Coordinate with internal stakeholders to ensure the timely delivery of supplies to distribution locations and communicate any delays or changes promptly. Transportation 7. Prepare and share weekly stock position and transportation status reports including logistics movement reports with relevant departments at headquarters. 8. Organize safe and efficient transportation of procured items to the affected people and areas, ensuring compliance with MRCS warehousing procedures before final distribution to affected people. 9. Plan and coordinate transport requirements, including MRCS-owned trucks and third-party trucking service providers and support the Senior Logistics Officer</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -4886,7 +4885,7 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t xml:space="preserve">terms of relief distribution, transport activity, local purchase of relief items, support to health and care activities, support to disaster management programmes (such as purchase of disaster preparedness stocks), carrying out custom clearance of the imported suppliers, dissemination of procedures and guidelines, training of staffs and volunteers. Since early 2013, the Logistics and Supply Chain Management Department has been supporting MRCS develop a common community- based approach to build community resilience. Technical assistance and support on strengthening disaster preparedness and response systems is also included in the operational plan. Logistics and Supply Chain Management Team is supporting to those programme as well as other projects and programme which MRCS is implementing in country with the bilateral supports of Partner National Societies (PNSs) in Myanmar. Purpose of the Position: The purpose of the Logistics Officer is to initiate and implement logistics activities, </t>
+          <t>terms of relief distribution, transport activity, local purchase of relief items, support to health and care activities, support to disaster management programmes (such as purchase of disaster preparedness stocks), carrying out custom clearance of the imported suppliers, dissemination of procedures and guidelines, training of staffs and volunteers. Since early 2013, the Logistics and Supply Chain Management Department has been supporting MRCS develop a common community- based approach to build community resilience. Technical assistance and support on strengthening disaster preparedness and response systems is also included in the operational plan. Logistics and Supply Chain Management Team is supporting to those programme as well as other projects and programme which MRCS is implementing in country with the bilateral supports of Partner National Societies (PNSs) in Myanmar. Purpose of the Position: The purpose of the Logistics Officer is to initiate and implement logistics activities,</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">

</xml_diff>